<commit_message>
Atualização automática: vencimentos_tmot (09/07/2026 23:47)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
@@ -20,16 +20,13 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -40,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -48,21 +45,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -433,57 +421,57 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>matricula</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>operador</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>pn</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>sn</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>nomenclatura</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>inspecao</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>tipo_vencimento</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>disponibilidade_valor</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>disponibilidade_texto</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>data_vencimento</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>vencido</t>
         </is>
@@ -527,7 +515,7 @@
         <v>-4402.8</v>
       </c>
       <c r="I2" t="inlineStr"/>
-      <c r="J2" s="2" t="n">
+      <c r="J2" s="1" t="n">
         <v>41388</v>
       </c>
       <c r="K2" t="b">
@@ -572,7 +560,7 @@
         <v>-4254.8</v>
       </c>
       <c r="I3" t="inlineStr"/>
-      <c r="J3" s="2" t="n">
+      <c r="J3" s="1" t="n">
         <v>39285</v>
       </c>
       <c r="K3" t="b">
@@ -617,7 +605,7 @@
         <v>-2354.2</v>
       </c>
       <c r="I4" t="inlineStr"/>
-      <c r="J4" s="2" t="n">
+      <c r="J4" s="1" t="n">
         <v>40669</v>
       </c>
       <c r="K4" t="b">
@@ -662,7 +650,7 @@
         <v>-896.8</v>
       </c>
       <c r="I5" t="inlineStr"/>
-      <c r="J5" s="2" t="n">
+      <c r="J5" s="1" t="n">
         <v>40669</v>
       </c>
       <c r="K5" t="b">
@@ -707,7 +695,7 @@
         <v>-854.1</v>
       </c>
       <c r="I6" t="inlineStr"/>
-      <c r="J6" s="2" t="n">
+      <c r="J6" s="1" t="n">
         <v>44884</v>
       </c>
       <c r="K6" t="b">
@@ -752,7 +740,7 @@
         <v>-413.2</v>
       </c>
       <c r="I7" t="inlineStr"/>
-      <c r="J7" s="2" t="n">
+      <c r="J7" s="1" t="n">
         <v>43855</v>
       </c>
       <c r="K7" t="b">
@@ -797,7 +785,7 @@
         <v>-391.8</v>
       </c>
       <c r="I8" t="inlineStr"/>
-      <c r="J8" s="2" t="n">
+      <c r="J8" s="1" t="n">
         <v>42769</v>
       </c>
       <c r="K8" t="b">
@@ -842,7 +830,7 @@
         <v>-371.5</v>
       </c>
       <c r="I9" t="inlineStr"/>
-      <c r="J9" s="2" t="n">
+      <c r="J9" s="1" t="n">
         <v>46014</v>
       </c>
       <c r="K9" t="b">
@@ -887,7 +875,7 @@
         <v>-368.8</v>
       </c>
       <c r="I10" t="inlineStr"/>
-      <c r="J10" s="2" t="n">
+      <c r="J10" s="1" t="n">
         <v>46014</v>
       </c>
       <c r="K10" t="b">
@@ -932,7 +920,7 @@
         <v>-359</v>
       </c>
       <c r="I11" t="inlineStr"/>
-      <c r="J11" s="2" t="n">
+      <c r="J11" s="1" t="n">
         <v>45804</v>
       </c>
       <c r="K11" t="b">
@@ -977,7 +965,7 @@
         <v>-359</v>
       </c>
       <c r="I12" t="inlineStr"/>
-      <c r="J12" s="2" t="n">
+      <c r="J12" s="1" t="n">
         <v>45804</v>
       </c>
       <c r="K12" t="b">
@@ -1022,7 +1010,7 @@
         <v>-351</v>
       </c>
       <c r="I13" t="inlineStr"/>
-      <c r="J13" s="2" t="n">
+      <c r="J13" s="1" t="n">
         <v>42821</v>
       </c>
       <c r="K13" t="b">
@@ -1067,7 +1055,7 @@
         <v>-351</v>
       </c>
       <c r="I14" t="inlineStr"/>
-      <c r="J14" s="2" t="n">
+      <c r="J14" s="1" t="n">
         <v>46014</v>
       </c>
       <c r="K14" t="b">
@@ -1112,7 +1100,7 @@
         <v>-351</v>
       </c>
       <c r="I15" t="inlineStr"/>
-      <c r="J15" s="2" t="n">
+      <c r="J15" s="1" t="n">
         <v>46014</v>
       </c>
       <c r="K15" t="b">
@@ -1157,7 +1145,7 @@
         <v>-351</v>
       </c>
       <c r="I16" t="inlineStr"/>
-      <c r="J16" s="2" t="n">
+      <c r="J16" s="1" t="n">
         <v>46014</v>
       </c>
       <c r="K16" t="b">
@@ -1202,7 +1190,7 @@
         <v>-345.8</v>
       </c>
       <c r="I17" t="inlineStr"/>
-      <c r="J17" s="2" t="n">
+      <c r="J17" s="1" t="n">
         <v>46017</v>
       </c>
       <c r="K17" t="b">
@@ -1247,7 +1235,7 @@
         <v>-345.8</v>
       </c>
       <c r="I18" t="inlineStr"/>
-      <c r="J18" s="2" t="n">
+      <c r="J18" s="1" t="n">
         <v>46017</v>
       </c>
       <c r="K18" t="b">
@@ -1292,7 +1280,7 @@
         <v>-264.2</v>
       </c>
       <c r="I19" t="inlineStr"/>
-      <c r="J19" s="2" t="n">
+      <c r="J19" s="1" t="n">
         <v>40979</v>
       </c>
       <c r="K19" t="b">
@@ -1337,7 +1325,7 @@
         <v>-206.4</v>
       </c>
       <c r="I20" t="inlineStr"/>
-      <c r="J20" s="2" t="n">
+      <c r="J20" s="1" t="n">
         <v>36669</v>
       </c>
       <c r="K20" t="b">
@@ -1382,7 +1370,7 @@
         <v>-131.6</v>
       </c>
       <c r="I21" t="inlineStr"/>
-      <c r="J21" s="2" t="n">
+      <c r="J21" s="1" t="n">
         <v>46111</v>
       </c>
       <c r="K21" t="b">
@@ -1427,7 +1415,7 @@
         <v>-131.6</v>
       </c>
       <c r="I22" t="inlineStr"/>
-      <c r="J22" s="2" t="n">
+      <c r="J22" s="1" t="n">
         <v>46111</v>
       </c>
       <c r="K22" t="b">
@@ -1472,7 +1460,7 @@
         <v>-131.6</v>
       </c>
       <c r="I23" t="inlineStr"/>
-      <c r="J23" s="2" t="n">
+      <c r="J23" s="1" t="n">
         <v>46111</v>
       </c>
       <c r="K23" t="b">
@@ -1517,7 +1505,7 @@
         <v>-131.6</v>
       </c>
       <c r="I24" t="inlineStr"/>
-      <c r="J24" s="2" t="n">
+      <c r="J24" s="1" t="n">
         <v>46111</v>
       </c>
       <c r="K24" t="b">
@@ -1562,7 +1550,7 @@
         <v>-131.6</v>
       </c>
       <c r="I25" t="inlineStr"/>
-      <c r="J25" s="2" t="n">
+      <c r="J25" s="1" t="n">
         <v>46111</v>
       </c>
       <c r="K25" t="b">
@@ -1607,7 +1595,7 @@
         <v>-105</v>
       </c>
       <c r="I26" t="inlineStr"/>
-      <c r="J26" s="2" t="n">
+      <c r="J26" s="1" t="n">
         <v>46161</v>
       </c>
       <c r="K26" t="b">
@@ -1652,7 +1640,7 @@
         <v>-79.8</v>
       </c>
       <c r="I27" t="inlineStr"/>
-      <c r="J27" s="2" t="n">
+      <c r="J27" s="1" t="n">
         <v>43340</v>
       </c>
       <c r="K27" t="b">
@@ -1697,7 +1685,7 @@
         <v>-12.3</v>
       </c>
       <c r="I28" t="inlineStr"/>
-      <c r="J28" s="2" t="n">
+      <c r="J28" s="1" t="n">
         <v>46048</v>
       </c>
       <c r="K28" t="b">
@@ -1742,7 +1730,7 @@
         <v>0</v>
       </c>
       <c r="I29" t="inlineStr"/>
-      <c r="J29" s="2" t="n">
+      <c r="J29" s="1" t="n">
         <v>46211</v>
       </c>
       <c r="K29" t="b">
@@ -1787,7 +1775,7 @@
         <v>3.6</v>
       </c>
       <c r="I30" t="inlineStr"/>
-      <c r="J30" s="2" t="n">
+      <c r="J30" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="K30" t="b">
@@ -1832,7 +1820,7 @@
         <v>6.2</v>
       </c>
       <c r="I31" t="inlineStr"/>
-      <c r="J31" s="2" t="n">
+      <c r="J31" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="K31" t="b">
@@ -1877,7 +1865,7 @@
         <v>7.5</v>
       </c>
       <c r="I32" t="inlineStr"/>
-      <c r="J32" s="2" t="n">
+      <c r="J32" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="K32" t="b">
@@ -1922,7 +1910,7 @@
         <v>10.7</v>
       </c>
       <c r="I33" t="inlineStr"/>
-      <c r="J33" s="2" t="n">
+      <c r="J33" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="K33" t="b">
@@ -1967,7 +1955,7 @@
         <v>20</v>
       </c>
       <c r="I34" t="inlineStr"/>
-      <c r="J34" s="2" t="n">
+      <c r="J34" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="K34" t="b">
@@ -2012,7 +2000,7 @@
         <v>30.8</v>
       </c>
       <c r="I35" t="inlineStr"/>
-      <c r="J35" s="2" t="n">
+      <c r="J35" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="K35" t="b">
@@ -2057,7 +2045,7 @@
         <v>37.1</v>
       </c>
       <c r="I36" t="inlineStr"/>
-      <c r="J36" s="2" t="n">
+      <c r="J36" s="1" t="n">
         <v>46256</v>
       </c>
       <c r="K36" t="b">
@@ -2102,7 +2090,7 @@
         <v>42.8</v>
       </c>
       <c r="I37" t="inlineStr"/>
-      <c r="J37" s="2" t="n">
+      <c r="J37" s="1" t="n">
         <v>46276</v>
       </c>
       <c r="K37" t="b">
@@ -2147,7 +2135,7 @@
         <v>45.2</v>
       </c>
       <c r="I38" t="inlineStr"/>
-      <c r="J38" s="2" t="n">
+      <c r="J38" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="K38" t="b">
@@ -2192,7 +2180,7 @@
         <v>46</v>
       </c>
       <c r="I39" t="inlineStr"/>
-      <c r="J39" s="2" t="n">
+      <c r="J39" s="1" t="n">
         <v>46251</v>
       </c>
       <c r="K39" t="b">
@@ -2237,7 +2225,7 @@
         <v>47.5</v>
       </c>
       <c r="I40" t="inlineStr"/>
-      <c r="J40" s="2" t="n">
+      <c r="J40" s="1" t="n">
         <v>46456</v>
       </c>
       <c r="K40" t="b">
@@ -2282,7 +2270,7 @@
         <v>57.2</v>
       </c>
       <c r="I41" t="inlineStr"/>
-      <c r="J41" s="2" t="n">
+      <c r="J41" s="1" t="n">
         <v>46246</v>
       </c>
       <c r="K41" t="b">
@@ -2327,7 +2315,7 @@
         <v>59.6</v>
       </c>
       <c r="I42" t="inlineStr"/>
-      <c r="J42" s="2" t="n">
+      <c r="J42" s="1" t="n">
         <v>46487</v>
       </c>
       <c r="K42" t="b">
@@ -2372,7 +2360,7 @@
         <v>75.40000000000001</v>
       </c>
       <c r="I43" t="inlineStr"/>
-      <c r="J43" s="2" t="n">
+      <c r="J43" s="1" t="n">
         <v>46283</v>
       </c>
       <c r="K43" t="b">
@@ -2417,7 +2405,7 @@
         <v>76.8</v>
       </c>
       <c r="I44" t="inlineStr"/>
-      <c r="J44" s="2" t="n">
+      <c r="J44" s="1" t="n">
         <v>46285</v>
       </c>
       <c r="K44" t="b">
@@ -2462,7 +2450,7 @@
         <v>83.2</v>
       </c>
       <c r="I45" t="inlineStr"/>
-      <c r="J45" s="2" t="n">
+      <c r="J45" s="1" t="n">
         <v>46547</v>
       </c>
       <c r="K45" t="b">
@@ -2507,7 +2495,7 @@
         <v>84.5</v>
       </c>
       <c r="I46" t="inlineStr"/>
-      <c r="J46" s="2" t="n">
+      <c r="J46" s="1" t="n">
         <v>46240</v>
       </c>
       <c r="K46" t="b">
@@ -2552,7 +2540,7 @@
         <v>85.8</v>
       </c>
       <c r="I47" t="inlineStr"/>
-      <c r="J47" s="2" t="n">
+      <c r="J47" s="1" t="n">
         <v>46266</v>
       </c>
       <c r="K47" t="b">
@@ -2597,7 +2585,7 @@
         <v>86.5</v>
       </c>
       <c r="I48" t="inlineStr"/>
-      <c r="J48" s="2" t="n">
+      <c r="J48" s="1" t="n">
         <v>46241</v>
       </c>
       <c r="K48" t="b">
@@ -2642,7 +2630,7 @@
         <v>91.7</v>
       </c>
       <c r="I49" t="inlineStr"/>
-      <c r="J49" s="2" t="n">
+      <c r="J49" s="1" t="n">
         <v>46243</v>
       </c>
       <c r="K49" t="b">
@@ -2687,7 +2675,7 @@
         <v>91.7</v>
       </c>
       <c r="I50" t="inlineStr"/>
-      <c r="J50" s="2" t="n">
+      <c r="J50" s="1" t="n">
         <v>46243</v>
       </c>
       <c r="K50" t="b">
@@ -2732,7 +2720,7 @@
         <v>91.7</v>
       </c>
       <c r="I51" t="inlineStr"/>
-      <c r="J51" s="2" t="n">
+      <c r="J51" s="1" t="n">
         <v>46250</v>
       </c>
       <c r="K51" t="b">
@@ -2777,7 +2765,7 @@
         <v>98.90000000000001</v>
       </c>
       <c r="I52" t="inlineStr"/>
-      <c r="J52" s="2" t="n">
+      <c r="J52" s="1" t="n">
         <v>46253</v>
       </c>
       <c r="K52" t="b">
@@ -2822,7 +2810,7 @@
         <v>105.5</v>
       </c>
       <c r="I53" t="inlineStr"/>
-      <c r="J53" s="2" t="n">
+      <c r="J53" s="1" t="n">
         <v>46280</v>
       </c>
       <c r="K53" t="b">
@@ -2867,7 +2855,7 @@
         <v>105.6</v>
       </c>
       <c r="I54" t="inlineStr"/>
-      <c r="J54" s="2" t="n">
+      <c r="J54" s="1" t="n">
         <v>46361</v>
       </c>
       <c r="K54" t="b">
@@ -2912,7 +2900,7 @@
         <v>105.7</v>
       </c>
       <c r="I55" t="inlineStr"/>
-      <c r="J55" s="2" t="n">
+      <c r="J55" s="1" t="n">
         <v>46362</v>
       </c>
       <c r="K55" t="b">
@@ -2957,7 +2945,7 @@
         <v>110.7</v>
       </c>
       <c r="I56" t="inlineStr"/>
-      <c r="J56" s="2" t="n">
+      <c r="J56" s="1" t="n">
         <v>46275</v>
       </c>
       <c r="K56" t="b">
@@ -3002,7 +2990,7 @@
         <v>113.2</v>
       </c>
       <c r="I57" t="inlineStr"/>
-      <c r="J57" s="2" t="n">
+      <c r="J57" s="1" t="n">
         <v>46377</v>
       </c>
       <c r="K57" t="b">
@@ -3047,7 +3035,7 @@
         <v>128.8</v>
       </c>
       <c r="I58" t="inlineStr"/>
-      <c r="J58" s="2" t="n">
+      <c r="J58" s="1" t="n">
         <v>46434</v>
       </c>
       <c r="K58" t="b">
@@ -3092,7 +3080,7 @@
         <v>128.8</v>
       </c>
       <c r="I59" t="inlineStr"/>
-      <c r="J59" s="2" t="n">
+      <c r="J59" s="1" t="n">
         <v>46434</v>
       </c>
       <c r="K59" t="b">
@@ -3137,7 +3125,7 @@
         <v>128.8</v>
       </c>
       <c r="I60" t="inlineStr"/>
-      <c r="J60" s="2" t="n">
+      <c r="J60" s="1" t="n">
         <v>46434</v>
       </c>
       <c r="K60" t="b">
@@ -3182,7 +3170,7 @@
         <v>128.8</v>
       </c>
       <c r="I61" t="inlineStr"/>
-      <c r="J61" s="2" t="n">
+      <c r="J61" s="1" t="n">
         <v>46434</v>
       </c>
       <c r="K61" t="b">
@@ -3227,7 +3215,7 @@
         <v>128.8</v>
       </c>
       <c r="I62" t="inlineStr"/>
-      <c r="J62" s="2" t="n">
+      <c r="J62" s="1" t="n">
         <v>46434</v>
       </c>
       <c r="K62" t="b">
@@ -3272,7 +3260,7 @@
         <v>135</v>
       </c>
       <c r="I63" t="inlineStr"/>
-      <c r="J63" s="2" t="n">
+      <c r="J63" s="1" t="n">
         <v>46280</v>
       </c>
       <c r="K63" t="b">
@@ -3317,7 +3305,7 @@
         <v>150.6</v>
       </c>
       <c r="I64" t="inlineStr"/>
-      <c r="J64" s="2" t="n">
+      <c r="J64" s="1" t="n">
         <v>46271</v>
       </c>
       <c r="K64" t="b">
@@ -3362,7 +3350,7 @@
         <v>174.2</v>
       </c>
       <c r="I65" t="inlineStr"/>
-      <c r="J65" s="2" t="n">
+      <c r="J65" s="1" t="n">
         <v>46363</v>
       </c>
       <c r="K65" t="b">
@@ -3407,7 +3395,7 @@
         <v>176.6</v>
       </c>
       <c r="I66" t="inlineStr"/>
-      <c r="J66" s="2" t="n">
+      <c r="J66" s="1" t="n">
         <v>46334</v>
       </c>
       <c r="K66" t="b">
@@ -3452,7 +3440,7 @@
         <v>177.4</v>
       </c>
       <c r="I67" t="inlineStr"/>
-      <c r="J67" s="2" t="n">
+      <c r="J67" s="1" t="n">
         <v>46407</v>
       </c>
       <c r="K67" t="b">
@@ -3497,7 +3485,7 @@
         <v>183.9</v>
       </c>
       <c r="I68" t="inlineStr"/>
-      <c r="J68" s="2" t="n">
+      <c r="J68" s="1" t="n">
         <v>46341</v>
       </c>
       <c r="K68" t="b">
@@ -3542,7 +3530,7 @@
         <v>191.7</v>
       </c>
       <c r="I69" t="inlineStr"/>
-      <c r="J69" s="2" t="n">
+      <c r="J69" s="1" t="n">
         <v>46300</v>
       </c>
       <c r="K69" t="b">
@@ -3587,7 +3575,7 @@
         <v>200</v>
       </c>
       <c r="I70" t="inlineStr"/>
-      <c r="J70" s="2" t="n">
+      <c r="J70" s="1" t="n">
         <v>46336</v>
       </c>
       <c r="K70" t="b">
@@ -3632,7 +3620,7 @@
         <v>201.1</v>
       </c>
       <c r="I71" t="inlineStr"/>
-      <c r="J71" s="2" t="n">
+      <c r="J71" s="1" t="n">
         <v>46319</v>
       </c>
       <c r="K71" t="b">
@@ -3677,7 +3665,7 @@
         <v>206.5</v>
       </c>
       <c r="I72" t="inlineStr"/>
-      <c r="J72" s="2" t="n">
+      <c r="J72" s="1" t="n">
         <v>46308</v>
       </c>
       <c r="K72" t="b">
@@ -3722,7 +3710,7 @@
         <v>207.5</v>
       </c>
       <c r="I73" t="inlineStr"/>
-      <c r="J73" s="2" t="n">
+      <c r="J73" s="1" t="n">
         <v>46390</v>
       </c>
       <c r="K73" t="b">
@@ -3767,7 +3755,7 @@
         <v>247</v>
       </c>
       <c r="I74" t="inlineStr"/>
-      <c r="J74" s="2" t="n">
+      <c r="J74" s="1" t="n">
         <v>46443</v>
       </c>
       <c r="K74" t="b">
@@ -3812,7 +3800,7 @@
         <v>285.3</v>
       </c>
       <c r="I75" t="inlineStr"/>
-      <c r="J75" s="2" t="n">
+      <c r="J75" s="1" t="n">
         <v>46304</v>
       </c>
       <c r="K75" t="b">
@@ -3857,7 +3845,7 @@
         <v>290.8</v>
       </c>
       <c r="I76" t="inlineStr"/>
-      <c r="J76" s="2" t="n">
+      <c r="J76" s="1" t="n">
         <v>46362</v>
       </c>
       <c r="K76" t="b">
@@ -3902,7 +3890,7 @@
         <v>295.2</v>
       </c>
       <c r="I77" t="inlineStr"/>
-      <c r="J77" s="2" t="n">
+      <c r="J77" s="1" t="n">
         <v>46463</v>
       </c>
       <c r="K77" t="b">
@@ -3947,7 +3935,7 @@
         <v>300.2</v>
       </c>
       <c r="I78" t="inlineStr"/>
-      <c r="J78" s="2" t="n">
+      <c r="J78" s="1" t="n">
         <v>46466</v>
       </c>
       <c r="K78" t="b">
@@ -3996,7 +3984,7 @@
           <t>-317m</t>
         </is>
       </c>
-      <c r="J79" s="2" t="n">
+      <c r="J79" s="1" t="n">
         <v>36557</v>
       </c>
       <c r="K79" t="b">
@@ -4045,7 +4033,7 @@
           <t>-164m</t>
         </is>
       </c>
-      <c r="J80" s="2" t="n">
+      <c r="J80" s="1" t="n">
         <v>41275</v>
       </c>
       <c r="K80" t="b">
@@ -4094,7 +4082,7 @@
           <t>-27m</t>
         </is>
       </c>
-      <c r="J81" s="2" t="n">
+      <c r="J81" s="1" t="n">
         <v>45380</v>
       </c>
       <c r="K81" t="b">
@@ -4143,7 +4131,7 @@
           <t>-25m</t>
         </is>
       </c>
-      <c r="J82" s="2" t="n">
+      <c r="J82" s="1" t="n">
         <v>45421</v>
       </c>
       <c r="K82" t="b">
@@ -4192,7 +4180,7 @@
           <t>-25m</t>
         </is>
       </c>
-      <c r="J83" s="2" t="n">
+      <c r="J83" s="1" t="n">
         <v>45428</v>
       </c>
       <c r="K83" t="b">
@@ -4241,7 +4229,7 @@
           <t>-23m</t>
         </is>
       </c>
-      <c r="J84" s="2" t="n">
+      <c r="J84" s="1" t="n">
         <v>45490</v>
       </c>
       <c r="K84" t="b">
@@ -4290,7 +4278,7 @@
           <t>-21m</t>
         </is>
       </c>
-      <c r="J85" s="2" t="n">
+      <c r="J85" s="1" t="n">
         <v>45566</v>
       </c>
       <c r="K85" t="b">
@@ -4339,7 +4327,7 @@
           <t>-7m</t>
         </is>
       </c>
-      <c r="J86" s="2" t="n">
+      <c r="J86" s="1" t="n">
         <v>45986</v>
       </c>
       <c r="K86" t="b">
@@ -4388,7 +4376,7 @@
           <t>-3m</t>
         </is>
       </c>
-      <c r="J87" s="2" t="n">
+      <c r="J87" s="1" t="n">
         <v>46106</v>
       </c>
       <c r="K87" t="b">
@@ -4437,7 +4425,7 @@
           <t>-2m</t>
         </is>
       </c>
-      <c r="J88" s="2" t="n">
+      <c r="J88" s="1" t="n">
         <v>46142</v>
       </c>
       <c r="K88" t="b">
@@ -4486,7 +4474,7 @@
           <t>2m</t>
         </is>
       </c>
-      <c r="J89" s="2" t="n">
+      <c r="J89" s="1" t="n">
         <v>46274</v>
       </c>
       <c r="K89" t="b">
@@ -4535,7 +4523,7 @@
           <t>2m</t>
         </is>
       </c>
-      <c r="J90" s="2" t="n">
+      <c r="J90" s="1" t="n">
         <v>46276</v>
       </c>
       <c r="K90" t="b">
@@ -4584,7 +4572,7 @@
           <t>2m</t>
         </is>
       </c>
-      <c r="J91" s="2" t="n">
+      <c r="J91" s="1" t="n">
         <v>46284</v>
       </c>
       <c r="K91" t="b">
@@ -4633,7 +4621,7 @@
           <t>3m</t>
         </is>
       </c>
-      <c r="J92" s="2" t="n">
+      <c r="J92" s="1" t="n">
         <v>46317</v>
       </c>
       <c r="K92" t="b">
@@ -4682,7 +4670,7 @@
           <t>3m</t>
         </is>
       </c>
-      <c r="J93" s="2" t="n">
+      <c r="J93" s="1" t="n">
         <v>46319</v>
       </c>
       <c r="K93" t="b">
@@ -4731,7 +4719,7 @@
           <t>4m</t>
         </is>
       </c>
-      <c r="J94" s="2" t="n">
+      <c r="J94" s="1" t="n">
         <v>46333</v>
       </c>
       <c r="K94" t="b">
@@ -4780,7 +4768,7 @@
           <t>4m</t>
         </is>
       </c>
-      <c r="J95" s="2" t="n">
+      <c r="J95" s="1" t="n">
         <v>46338</v>
       </c>
       <c r="K95" t="b">
@@ -4829,7 +4817,7 @@
           <t>4m</t>
         </is>
       </c>
-      <c r="J96" s="2" t="n">
+      <c r="J96" s="1" t="n">
         <v>46338</v>
       </c>
       <c r="K96" t="b">
@@ -4878,7 +4866,7 @@
           <t>4m</t>
         </is>
       </c>
-      <c r="J97" s="2" t="n">
+      <c r="J97" s="1" t="n">
         <v>46341</v>
       </c>
       <c r="K97" t="b">
@@ -4927,7 +4915,7 @@
           <t>4m</t>
         </is>
       </c>
-      <c r="J98" s="2" t="n">
+      <c r="J98" s="1" t="n">
         <v>46344</v>
       </c>
       <c r="K98" t="b">
@@ -4976,7 +4964,7 @@
           <t>4m</t>
         </is>
       </c>
-      <c r="J99" s="2" t="n">
+      <c r="J99" s="1" t="n">
         <v>46354</v>
       </c>
       <c r="K99" t="b">
@@ -5025,7 +5013,7 @@
           <t>4m</t>
         </is>
       </c>
-      <c r="J100" s="2" t="n">
+      <c r="J100" s="1" t="n">
         <v>46360</v>
       </c>
       <c r="K100" t="b">
@@ -5074,7 +5062,7 @@
           <t>4m</t>
         </is>
       </c>
-      <c r="J101" s="2" t="n">
+      <c r="J101" s="1" t="n">
         <v>46360</v>
       </c>
       <c r="K101" t="b">
@@ -5123,7 +5111,7 @@
           <t>5m</t>
         </is>
       </c>
-      <c r="J102" s="2" t="n">
+      <c r="J102" s="1" t="n">
         <v>46366</v>
       </c>
       <c r="K102" t="b">
@@ -5172,7 +5160,7 @@
           <t>5m</t>
         </is>
       </c>
-      <c r="J103" s="2" t="n">
+      <c r="J103" s="1" t="n">
         <v>46375</v>
       </c>
       <c r="K103" t="b">
@@ -5221,7 +5209,7 @@
           <t>5m</t>
         </is>
       </c>
-      <c r="J104" s="2" t="n">
+      <c r="J104" s="1" t="n">
         <v>46388</v>
       </c>
       <c r="K104" t="b">
@@ -5270,7 +5258,7 @@
           <t>6m</t>
         </is>
       </c>
-      <c r="J105" s="2" t="n">
+      <c r="J105" s="1" t="n">
         <v>46401</v>
       </c>
       <c r="K105" t="b">
@@ -5319,7 +5307,7 @@
           <t>6m</t>
         </is>
       </c>
-      <c r="J106" s="2" t="n">
+      <c r="J106" s="1" t="n">
         <v>46401</v>
       </c>
       <c r="K106" t="b">
@@ -5368,7 +5356,7 @@
           <t>6m</t>
         </is>
       </c>
-      <c r="J107" s="2" t="n">
+      <c r="J107" s="1" t="n">
         <v>46401</v>
       </c>
       <c r="K107" t="b">
@@ -5417,7 +5405,7 @@
           <t>6m</t>
         </is>
       </c>
-      <c r="J108" s="2" t="n">
+      <c r="J108" s="1" t="n">
         <v>46413</v>
       </c>
       <c r="K108" t="b">
@@ -5466,7 +5454,7 @@
           <t>7m</t>
         </is>
       </c>
-      <c r="J109" s="2" t="n">
+      <c r="J109" s="1" t="n">
         <v>46424</v>
       </c>
       <c r="K109" t="b">
@@ -5515,7 +5503,7 @@
           <t>7m</t>
         </is>
       </c>
-      <c r="J110" s="2" t="n">
+      <c r="J110" s="1" t="n">
         <v>46427</v>
       </c>
       <c r="K110" t="b">
@@ -5564,7 +5552,7 @@
           <t>7m</t>
         </is>
       </c>
-      <c r="J111" s="2" t="n">
+      <c r="J111" s="1" t="n">
         <v>46437</v>
       </c>
       <c r="K111" t="b">
@@ -5613,7 +5601,7 @@
           <t>7m</t>
         </is>
       </c>
-      <c r="J112" s="2" t="n">
+      <c r="J112" s="1" t="n">
         <v>46451</v>
       </c>
       <c r="K112" t="b">
@@ -5662,7 +5650,7 @@
           <t>8m</t>
         </is>
       </c>
-      <c r="J113" s="2" t="n">
+      <c r="J113" s="1" t="n">
         <v>46455</v>
       </c>
       <c r="K113" t="b">
@@ -5711,7 +5699,7 @@
           <t>8m</t>
         </is>
       </c>
-      <c r="J114" s="2" t="n">
+      <c r="J114" s="1" t="n">
         <v>46457</v>
       </c>
       <c r="K114" t="b">
@@ -5760,7 +5748,7 @@
           <t>8m</t>
         </is>
       </c>
-      <c r="J115" s="2" t="n">
+      <c r="J115" s="1" t="n">
         <v>46462</v>
       </c>
       <c r="K115" t="b">
@@ -5809,7 +5797,7 @@
           <t>8m</t>
         </is>
       </c>
-      <c r="J116" s="2" t="n">
+      <c r="J116" s="1" t="n">
         <v>46464</v>
       </c>
       <c r="K116" t="b">
@@ -5858,7 +5846,7 @@
           <t>8m</t>
         </is>
       </c>
-      <c r="J117" s="2" t="n">
+      <c r="J117" s="1" t="n">
         <v>46470</v>
       </c>
       <c r="K117" t="b">
@@ -5907,7 +5895,7 @@
           <t>9m</t>
         </is>
       </c>
-      <c r="J118" s="2" t="n">
+      <c r="J118" s="1" t="n">
         <v>46485</v>
       </c>
       <c r="K118" t="b">
@@ -5956,7 +5944,7 @@
           <t>9m</t>
         </is>
       </c>
-      <c r="J119" s="2" t="n">
+      <c r="J119" s="1" t="n">
         <v>46499</v>
       </c>
       <c r="K119" t="b">
@@ -6005,7 +5993,7 @@
           <t>9m</t>
         </is>
       </c>
-      <c r="J120" s="2" t="n">
+      <c r="J120" s="1" t="n">
         <v>46504</v>
       </c>
       <c r="K120" t="b">
@@ -6054,7 +6042,7 @@
           <t>9m</t>
         </is>
       </c>
-      <c r="J121" s="2" t="n">
+      <c r="J121" s="1" t="n">
         <v>46504</v>
       </c>
       <c r="K121" t="b">
@@ -6103,7 +6091,7 @@
           <t>9m</t>
         </is>
       </c>
-      <c r="J122" s="2" t="n">
+      <c r="J122" s="1" t="n">
         <v>46507</v>
       </c>
       <c r="K122" t="b">
@@ -6152,7 +6140,7 @@
           <t>9m</t>
         </is>
       </c>
-      <c r="J123" s="2" t="n">
+      <c r="J123" s="1" t="n">
         <v>46508</v>
       </c>
       <c r="K123" t="b">
@@ -6201,7 +6189,7 @@
           <t>9m</t>
         </is>
       </c>
-      <c r="J124" s="2" t="n">
+      <c r="J124" s="1" t="n">
         <v>46512</v>
       </c>
       <c r="K124" t="b">
@@ -6250,7 +6238,7 @@
           <t>9m</t>
         </is>
       </c>
-      <c r="J125" s="2" t="n">
+      <c r="J125" s="1" t="n">
         <v>46512</v>
       </c>
       <c r="K125" t="b">
@@ -6299,7 +6287,7 @@
           <t>10m</t>
         </is>
       </c>
-      <c r="J126" s="2" t="n">
+      <c r="J126" s="1" t="n">
         <v>46528</v>
       </c>
       <c r="K126" t="b">
@@ -6348,7 +6336,7 @@
           <t>10m</t>
         </is>
       </c>
-      <c r="J127" s="2" t="n">
+      <c r="J127" s="1" t="n">
         <v>46529</v>
       </c>
       <c r="K127" t="b">
@@ -6397,7 +6385,7 @@
           <t>10m</t>
         </is>
       </c>
-      <c r="J128" s="2" t="n">
+      <c r="J128" s="1" t="n">
         <v>46537</v>
       </c>
       <c r="K128" t="b">
@@ -6446,7 +6434,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J129" s="2" t="n">
+      <c r="J129" s="1" t="n">
         <v>46546</v>
       </c>
       <c r="K129" t="b">
@@ -6495,7 +6483,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J130" s="2" t="n">
+      <c r="J130" s="1" t="n">
         <v>46547</v>
       </c>
       <c r="K130" t="b">
@@ -6544,7 +6532,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J131" s="2" t="n">
+      <c r="J131" s="1" t="n">
         <v>46547</v>
       </c>
       <c r="K131" t="b">
@@ -6593,7 +6581,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J132" s="2" t="n">
+      <c r="J132" s="1" t="n">
         <v>46547</v>
       </c>
       <c r="K132" t="b">
@@ -6642,7 +6630,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J133" s="2" t="n">
+      <c r="J133" s="1" t="n">
         <v>46551</v>
       </c>
       <c r="K133" t="b">
@@ -6691,7 +6679,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J134" s="2" t="n">
+      <c r="J134" s="1" t="n">
         <v>46560</v>
       </c>
       <c r="K134" t="b">
@@ -6740,7 +6728,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J135" s="2" t="n">
+      <c r="J135" s="1" t="n">
         <v>46564</v>
       </c>
       <c r="K135" t="b">
@@ -6789,7 +6777,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J136" s="2" t="n">
+      <c r="J136" s="1" t="n">
         <v>46567</v>
       </c>
       <c r="K136" t="b">
@@ -6838,7 +6826,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J137" s="2" t="n">
+      <c r="J137" s="1" t="n">
         <v>46568</v>
       </c>
       <c r="K137" t="b">
@@ -6887,7 +6875,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J138" s="2" t="n">
+      <c r="J138" s="1" t="n">
         <v>46571</v>
       </c>
       <c r="K138" t="b">
@@ -6936,7 +6924,7 @@
           <t>-14d</t>
         </is>
       </c>
-      <c r="J139" s="2" t="n">
+      <c r="J139" s="1" t="n">
         <v>46197</v>
       </c>
       <c r="K139" t="b">
@@ -6985,7 +6973,7 @@
           <t>1d</t>
         </is>
       </c>
-      <c r="J140" s="2" t="n">
+      <c r="J140" s="1" t="n">
         <v>46212</v>
       </c>
       <c r="K140" t="b">
@@ -7034,7 +7022,7 @@
           <t>14d</t>
         </is>
       </c>
-      <c r="J141" s="2" t="n">
+      <c r="J141" s="1" t="n">
         <v>46225</v>
       </c>
       <c r="K141" t="b">
@@ -7083,7 +7071,7 @@
           <t>23d</t>
         </is>
       </c>
-      <c r="J142" s="2" t="n">
+      <c r="J142" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="K142" t="b">
@@ -7132,7 +7120,7 @@
           <t>24d</t>
         </is>
       </c>
-      <c r="J143" s="2" t="n">
+      <c r="J143" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="K143" t="b">
@@ -7181,7 +7169,7 @@
           <t>1me23d</t>
         </is>
       </c>
-      <c r="J144" s="2" t="n">
+      <c r="J144" s="1" t="n">
         <v>46263</v>
       </c>
       <c r="K144" t="b">
@@ -7230,7 +7218,7 @@
           <t>1me25d</t>
         </is>
       </c>
-      <c r="J145" s="2" t="n">
+      <c r="J145" s="1" t="n">
         <v>46266</v>
       </c>
       <c r="K145" t="b">
@@ -7275,7 +7263,7 @@
         <v>-1476</v>
       </c>
       <c r="I146" t="inlineStr"/>
-      <c r="J146" s="2" t="n">
+      <c r="J146" s="1" t="n">
         <v>43773</v>
       </c>
       <c r="K146" t="b">
@@ -7320,7 +7308,7 @@
         <v>-1469</v>
       </c>
       <c r="I147" t="inlineStr"/>
-      <c r="J147" s="2" t="n">
+      <c r="J147" s="1" t="n">
         <v>43773</v>
       </c>
       <c r="K147" t="b">
@@ -7365,7 +7353,7 @@
         <v>-1121</v>
       </c>
       <c r="I148" t="inlineStr"/>
-      <c r="J148" s="2" t="n">
+      <c r="J148" s="1" t="n">
         <v>45295</v>
       </c>
       <c r="K148" t="b">
@@ -7410,7 +7398,7 @@
         <v>-1018</v>
       </c>
       <c r="I149" t="inlineStr"/>
-      <c r="J149" s="2" t="n">
+      <c r="J149" s="1" t="n">
         <v>45617</v>
       </c>
       <c r="K149" t="b">
@@ -7455,7 +7443,7 @@
         <v>-950</v>
       </c>
       <c r="I150" t="inlineStr"/>
-      <c r="J150" s="2" t="n">
+      <c r="J150" s="1" t="n">
         <v>45677</v>
       </c>
       <c r="K150" t="b">
@@ -7500,7 +7488,7 @@
         <v>-943</v>
       </c>
       <c r="I151" t="inlineStr"/>
-      <c r="J151" s="2" t="n">
+      <c r="J151" s="1" t="n">
         <v>44944</v>
       </c>
       <c r="K151" t="b">
@@ -7545,7 +7533,7 @@
         <v>-252</v>
       </c>
       <c r="I152" t="inlineStr"/>
-      <c r="J152" s="2" t="n">
+      <c r="J152" s="1" t="n">
         <v>46092</v>
       </c>
       <c r="K152" t="b">
@@ -7590,7 +7578,7 @@
         <v>-196</v>
       </c>
       <c r="I153" t="inlineStr"/>
-      <c r="J153" s="2" t="n">
+      <c r="J153" s="1" t="n">
         <v>45988</v>
       </c>
       <c r="K153" t="b">
@@ -7635,7 +7623,7 @@
         <v>-196</v>
       </c>
       <c r="I154" t="inlineStr"/>
-      <c r="J154" s="2" t="n">
+      <c r="J154" s="1" t="n">
         <v>45988</v>
       </c>
       <c r="K154" t="b">
@@ -7680,7 +7668,7 @@
         <v>-47</v>
       </c>
       <c r="I155" t="inlineStr"/>
-      <c r="J155" s="2" t="n">
+      <c r="J155" s="1" t="n">
         <v>46176</v>
       </c>
       <c r="K155" t="b">
@@ -7725,7 +7713,7 @@
         <v>-47</v>
       </c>
       <c r="I156" t="inlineStr"/>
-      <c r="J156" s="2" t="n">
+      <c r="J156" s="1" t="n">
         <v>46176</v>
       </c>
       <c r="K156" t="b">
@@ -7770,7 +7758,7 @@
         <v>-33</v>
       </c>
       <c r="I157" t="inlineStr"/>
-      <c r="J157" s="2" t="n">
+      <c r="J157" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="K157" t="b">
@@ -7815,7 +7803,7 @@
         <v>-33</v>
       </c>
       <c r="I158" t="inlineStr"/>
-      <c r="J158" s="2" t="n">
+      <c r="J158" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="K158" t="b">
@@ -7860,7 +7848,7 @@
         <v>-6</v>
       </c>
       <c r="I159" t="inlineStr"/>
-      <c r="J159" s="2" t="n">
+      <c r="J159" s="1" t="n">
         <v>45967</v>
       </c>
       <c r="K159" t="b">
@@ -7905,7 +7893,7 @@
         <v>43</v>
       </c>
       <c r="I160" t="inlineStr"/>
-      <c r="J160" s="2" t="n">
+      <c r="J160" s="1" t="n">
         <v>46440</v>
       </c>
       <c r="K160" t="b">
@@ -7950,7 +7938,7 @@
         <v>43</v>
       </c>
       <c r="I161" t="inlineStr"/>
-      <c r="J161" s="2" t="n">
+      <c r="J161" s="1" t="n">
         <v>46440</v>
       </c>
       <c r="K161" t="b">
@@ -7995,7 +7983,7 @@
         <v>73</v>
       </c>
       <c r="I162" t="inlineStr"/>
-      <c r="J162" s="2" t="n">
+      <c r="J162" s="1" t="n">
         <v>46264</v>
       </c>
       <c r="K162" t="b">
@@ -8040,7 +8028,7 @@
         <v>73</v>
       </c>
       <c r="I163" t="inlineStr"/>
-      <c r="J163" s="2" t="n">
+      <c r="J163" s="1" t="n">
         <v>46264</v>
       </c>
       <c r="K163" t="b">
@@ -8085,7 +8073,7 @@
         <v>102</v>
       </c>
       <c r="I164" t="inlineStr"/>
-      <c r="J164" s="2" t="n">
+      <c r="J164" s="1" t="n">
         <v>46463</v>
       </c>
       <c r="K164" t="b">
@@ -8130,7 +8118,7 @@
         <v>118</v>
       </c>
       <c r="I165" t="inlineStr"/>
-      <c r="J165" s="2" t="n">
+      <c r="J165" s="1" t="n">
         <v>46337</v>
       </c>
       <c r="K165" t="b">
@@ -8175,7 +8163,7 @@
         <v>146</v>
       </c>
       <c r="I166" t="inlineStr"/>
-      <c r="J166" s="2" t="n">
+      <c r="J166" s="1" t="n">
         <v>46451</v>
       </c>
       <c r="K166" t="b">
@@ -8220,7 +8208,7 @@
         <v>152</v>
       </c>
       <c r="I167" t="inlineStr"/>
-      <c r="J167" s="2" t="n">
+      <c r="J167" s="1" t="n">
         <v>46245</v>
       </c>
       <c r="K167" t="b">
@@ -8265,7 +8253,7 @@
         <v>152</v>
       </c>
       <c r="I168" t="inlineStr"/>
-      <c r="J168" s="2" t="n">
+      <c r="J168" s="1" t="n">
         <v>46245</v>
       </c>
       <c r="K168" t="b">
@@ -8310,7 +8298,7 @@
         <v>163</v>
       </c>
       <c r="I169" t="inlineStr"/>
-      <c r="J169" s="2" t="n">
+      <c r="J169" s="1" t="n">
         <v>46324</v>
       </c>
       <c r="K169" t="b">
@@ -8355,7 +8343,7 @@
         <v>163</v>
       </c>
       <c r="I170" t="inlineStr"/>
-      <c r="J170" s="2" t="n">
+      <c r="J170" s="1" t="n">
         <v>46324</v>
       </c>
       <c r="K170" t="b">
@@ -8400,7 +8388,7 @@
         <v>164</v>
       </c>
       <c r="I171" t="inlineStr"/>
-      <c r="J171" s="2" t="n">
+      <c r="J171" s="1" t="n">
         <v>46426</v>
       </c>
       <c r="K171" t="b">
@@ -8445,7 +8433,7 @@
         <v>175</v>
       </c>
       <c r="I172" t="inlineStr"/>
-      <c r="J172" s="2" t="n">
+      <c r="J172" s="1" t="n">
         <v>46383</v>
       </c>
       <c r="K172" t="b">
@@ -8490,7 +8478,7 @@
         <v>186</v>
       </c>
       <c r="I173" t="inlineStr"/>
-      <c r="J173" s="2" t="n">
+      <c r="J173" s="1" t="n">
         <v>46392</v>
       </c>
       <c r="K173" t="b">
@@ -8535,7 +8523,7 @@
         <v>205</v>
       </c>
       <c r="I174" t="inlineStr"/>
-      <c r="J174" s="2" t="n">
+      <c r="J174" s="1" t="n">
         <v>46390</v>
       </c>
       <c r="K174" t="b">
@@ -8580,7 +8568,7 @@
         <v>207</v>
       </c>
       <c r="I175" t="inlineStr"/>
-      <c r="J175" s="2" t="n">
+      <c r="J175" s="1" t="n">
         <v>46392</v>
       </c>
       <c r="K175" t="b">
@@ -8625,7 +8613,7 @@
         <v>218</v>
       </c>
       <c r="I176" t="inlineStr"/>
-      <c r="J176" s="2" t="n">
+      <c r="J176" s="1" t="n">
         <v>46506</v>
       </c>
       <c r="K176" t="b">
@@ -8670,7 +8658,7 @@
         <v>246</v>
       </c>
       <c r="I177" t="inlineStr"/>
-      <c r="J177" s="2" t="n">
+      <c r="J177" s="1" t="n">
         <v>46478</v>
       </c>
       <c r="K177" t="b">
@@ -8715,7 +8703,7 @@
         <v>248</v>
       </c>
       <c r="I178" t="inlineStr"/>
-      <c r="J178" s="2" t="n">
+      <c r="J178" s="1" t="n">
         <v>46500</v>
       </c>
       <c r="K178" t="b">
@@ -8760,7 +8748,7 @@
         <v>276</v>
       </c>
       <c r="I179" t="inlineStr"/>
-      <c r="J179" s="2" t="n">
+      <c r="J179" s="1" t="n">
         <v>46430</v>
       </c>
       <c r="K179" t="b">
@@ -8805,7 +8793,7 @@
         <v>276</v>
       </c>
       <c r="I180" t="inlineStr"/>
-      <c r="J180" s="2" t="n">
+      <c r="J180" s="1" t="n">
         <v>46430</v>
       </c>
       <c r="K180" t="b">
@@ -8850,7 +8838,7 @@
         <v>290</v>
       </c>
       <c r="I181" t="inlineStr"/>
-      <c r="J181" s="2" t="n">
+      <c r="J181" s="1" t="n">
         <v>46467</v>
       </c>
       <c r="K181" t="b">
@@ -8895,7 +8883,7 @@
         <v>317</v>
       </c>
       <c r="I182" t="inlineStr"/>
-      <c r="J182" s="2" t="n">
+      <c r="J182" s="1" t="n">
         <v>46529</v>
       </c>
       <c r="K182" t="b">
@@ -8940,7 +8928,7 @@
         <v>420</v>
       </c>
       <c r="I183" t="inlineStr"/>
-      <c r="J183" s="2" t="n">
+      <c r="J183" s="1" t="n">
         <v>46566</v>
       </c>
       <c r="K183" t="b">
@@ -8985,7 +8973,7 @@
         <v>426</v>
       </c>
       <c r="I184" t="inlineStr"/>
-      <c r="J184" s="2" t="n">
+      <c r="J184" s="1" t="n">
         <v>46571</v>
       </c>
       <c r="K184" t="b">
@@ -9030,7 +9018,7 @@
         <v>721</v>
       </c>
       <c r="I185" t="inlineStr"/>
-      <c r="J185" s="2" t="n">
+      <c r="J185" s="1" t="n">
         <v>46325</v>
       </c>
       <c r="K185" t="b">
@@ -9075,7 +9063,7 @@
         <v>721</v>
       </c>
       <c r="I186" t="inlineStr"/>
-      <c r="J186" s="2" t="n">
+      <c r="J186" s="1" t="n">
         <v>46325</v>
       </c>
       <c r="K186" t="b">
@@ -9120,7 +9108,7 @@
         <v>850</v>
       </c>
       <c r="I187" t="inlineStr"/>
-      <c r="J187" s="2" t="n">
+      <c r="J187" s="1" t="n">
         <v>46345</v>
       </c>
       <c r="K187" t="b">
@@ -9165,7 +9153,7 @@
         <v>850</v>
       </c>
       <c r="I188" t="inlineStr"/>
-      <c r="J188" s="2" t="n">
+      <c r="J188" s="1" t="n">
         <v>46345</v>
       </c>
       <c r="K188" t="b">
@@ -9210,7 +9198,7 @@
         <v>1661</v>
       </c>
       <c r="I189" t="inlineStr"/>
-      <c r="J189" s="2" t="n">
+      <c r="J189" s="1" t="n">
         <v>46498</v>
       </c>
       <c r="K189" t="b">
@@ -9255,7 +9243,7 @@
         <v>1661</v>
       </c>
       <c r="I190" t="inlineStr"/>
-      <c r="J190" s="2" t="n">
+      <c r="J190" s="1" t="n">
         <v>46498</v>
       </c>
       <c r="K190" t="b">
@@ -9300,7 +9288,7 @@
         <v>488</v>
       </c>
       <c r="I191" t="inlineStr"/>
-      <c r="J191" s="2" t="n">
+      <c r="J191" s="1" t="n">
         <v>46190</v>
       </c>
       <c r="K191" t="b">
@@ -9345,7 +9333,7 @@
         <v>25565</v>
       </c>
       <c r="I192" t="inlineStr"/>
-      <c r="J192" s="2" t="n">
+      <c r="J192" s="1" t="n">
         <v>46190</v>
       </c>
       <c r="K192" t="b">
@@ -9390,7 +9378,7 @@
         <v>25567</v>
       </c>
       <c r="I193" t="inlineStr"/>
-      <c r="J193" s="2" t="n">
+      <c r="J193" s="1" t="n">
         <v>46190</v>
       </c>
       <c r="K193" t="b">
@@ -9435,7 +9423,7 @@
         <v>31293</v>
       </c>
       <c r="I194" t="inlineStr"/>
-      <c r="J194" s="2" t="n">
+      <c r="J194" s="1" t="n">
         <v>46190</v>
       </c>
       <c r="K194" t="b">

</xml_diff>

<commit_message>
Atualização automática: vencimentos_tmot (10/07/2026 10:10)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
@@ -20,13 +20,16 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +40,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,12 +48,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -421,57 +433,57 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>matricula</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>operador</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>pn</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>sn</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>nomenclatura</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>inspecao</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>tipo_vencimento</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>disponibilidade_valor</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>disponibilidade_texto</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>data_vencimento</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>vencido</t>
         </is>
@@ -515,7 +527,7 @@
         <v>-4402.8</v>
       </c>
       <c r="I2" t="inlineStr"/>
-      <c r="J2" s="1" t="n">
+      <c r="J2" s="2" t="n">
         <v>41388</v>
       </c>
       <c r="K2" t="b">
@@ -560,7 +572,7 @@
         <v>-4254.8</v>
       </c>
       <c r="I3" t="inlineStr"/>
-      <c r="J3" s="1" t="n">
+      <c r="J3" s="2" t="n">
         <v>39285</v>
       </c>
       <c r="K3" t="b">
@@ -605,7 +617,7 @@
         <v>-2354.2</v>
       </c>
       <c r="I4" t="inlineStr"/>
-      <c r="J4" s="1" t="n">
+      <c r="J4" s="2" t="n">
         <v>40669</v>
       </c>
       <c r="K4" t="b">
@@ -650,7 +662,7 @@
         <v>-896.8</v>
       </c>
       <c r="I5" t="inlineStr"/>
-      <c r="J5" s="1" t="n">
+      <c r="J5" s="2" t="n">
         <v>40669</v>
       </c>
       <c r="K5" t="b">
@@ -695,7 +707,7 @@
         <v>-854.1</v>
       </c>
       <c r="I6" t="inlineStr"/>
-      <c r="J6" s="1" t="n">
+      <c r="J6" s="2" t="n">
         <v>44884</v>
       </c>
       <c r="K6" t="b">
@@ -740,7 +752,7 @@
         <v>-413.2</v>
       </c>
       <c r="I7" t="inlineStr"/>
-      <c r="J7" s="1" t="n">
+      <c r="J7" s="2" t="n">
         <v>43855</v>
       </c>
       <c r="K7" t="b">
@@ -785,7 +797,7 @@
         <v>-391.8</v>
       </c>
       <c r="I8" t="inlineStr"/>
-      <c r="J8" s="1" t="n">
+      <c r="J8" s="2" t="n">
         <v>42769</v>
       </c>
       <c r="K8" t="b">
@@ -830,7 +842,7 @@
         <v>-371.5</v>
       </c>
       <c r="I9" t="inlineStr"/>
-      <c r="J9" s="1" t="n">
+      <c r="J9" s="2" t="n">
         <v>46014</v>
       </c>
       <c r="K9" t="b">
@@ -875,7 +887,7 @@
         <v>-368.8</v>
       </c>
       <c r="I10" t="inlineStr"/>
-      <c r="J10" s="1" t="n">
+      <c r="J10" s="2" t="n">
         <v>46014</v>
       </c>
       <c r="K10" t="b">
@@ -920,7 +932,7 @@
         <v>-359</v>
       </c>
       <c r="I11" t="inlineStr"/>
-      <c r="J11" s="1" t="n">
+      <c r="J11" s="2" t="n">
         <v>45804</v>
       </c>
       <c r="K11" t="b">
@@ -965,7 +977,7 @@
         <v>-359</v>
       </c>
       <c r="I12" t="inlineStr"/>
-      <c r="J12" s="1" t="n">
+      <c r="J12" s="2" t="n">
         <v>45804</v>
       </c>
       <c r="K12" t="b">
@@ -1010,7 +1022,7 @@
         <v>-351</v>
       </c>
       <c r="I13" t="inlineStr"/>
-      <c r="J13" s="1" t="n">
+      <c r="J13" s="2" t="n">
         <v>42821</v>
       </c>
       <c r="K13" t="b">
@@ -1055,7 +1067,7 @@
         <v>-351</v>
       </c>
       <c r="I14" t="inlineStr"/>
-      <c r="J14" s="1" t="n">
+      <c r="J14" s="2" t="n">
         <v>46014</v>
       </c>
       <c r="K14" t="b">
@@ -1100,7 +1112,7 @@
         <v>-351</v>
       </c>
       <c r="I15" t="inlineStr"/>
-      <c r="J15" s="1" t="n">
+      <c r="J15" s="2" t="n">
         <v>46014</v>
       </c>
       <c r="K15" t="b">
@@ -1145,7 +1157,7 @@
         <v>-351</v>
       </c>
       <c r="I16" t="inlineStr"/>
-      <c r="J16" s="1" t="n">
+      <c r="J16" s="2" t="n">
         <v>46014</v>
       </c>
       <c r="K16" t="b">
@@ -1190,7 +1202,7 @@
         <v>-345.8</v>
       </c>
       <c r="I17" t="inlineStr"/>
-      <c r="J17" s="1" t="n">
+      <c r="J17" s="2" t="n">
         <v>46017</v>
       </c>
       <c r="K17" t="b">
@@ -1235,7 +1247,7 @@
         <v>-345.8</v>
       </c>
       <c r="I18" t="inlineStr"/>
-      <c r="J18" s="1" t="n">
+      <c r="J18" s="2" t="n">
         <v>46017</v>
       </c>
       <c r="K18" t="b">
@@ -1280,7 +1292,7 @@
         <v>-264.2</v>
       </c>
       <c r="I19" t="inlineStr"/>
-      <c r="J19" s="1" t="n">
+      <c r="J19" s="2" t="n">
         <v>40979</v>
       </c>
       <c r="K19" t="b">
@@ -1325,7 +1337,7 @@
         <v>-206.4</v>
       </c>
       <c r="I20" t="inlineStr"/>
-      <c r="J20" s="1" t="n">
+      <c r="J20" s="2" t="n">
         <v>36669</v>
       </c>
       <c r="K20" t="b">
@@ -1370,7 +1382,7 @@
         <v>-131.6</v>
       </c>
       <c r="I21" t="inlineStr"/>
-      <c r="J21" s="1" t="n">
+      <c r="J21" s="2" t="n">
         <v>46111</v>
       </c>
       <c r="K21" t="b">
@@ -1415,7 +1427,7 @@
         <v>-131.6</v>
       </c>
       <c r="I22" t="inlineStr"/>
-      <c r="J22" s="1" t="n">
+      <c r="J22" s="2" t="n">
         <v>46111</v>
       </c>
       <c r="K22" t="b">
@@ -1460,7 +1472,7 @@
         <v>-131.6</v>
       </c>
       <c r="I23" t="inlineStr"/>
-      <c r="J23" s="1" t="n">
+      <c r="J23" s="2" t="n">
         <v>46111</v>
       </c>
       <c r="K23" t="b">
@@ -1505,7 +1517,7 @@
         <v>-131.6</v>
       </c>
       <c r="I24" t="inlineStr"/>
-      <c r="J24" s="1" t="n">
+      <c r="J24" s="2" t="n">
         <v>46111</v>
       </c>
       <c r="K24" t="b">
@@ -1550,7 +1562,7 @@
         <v>-131.6</v>
       </c>
       <c r="I25" t="inlineStr"/>
-      <c r="J25" s="1" t="n">
+      <c r="J25" s="2" t="n">
         <v>46111</v>
       </c>
       <c r="K25" t="b">
@@ -1595,7 +1607,7 @@
         <v>-105</v>
       </c>
       <c r="I26" t="inlineStr"/>
-      <c r="J26" s="1" t="n">
+      <c r="J26" s="2" t="n">
         <v>46161</v>
       </c>
       <c r="K26" t="b">
@@ -1640,7 +1652,7 @@
         <v>-79.8</v>
       </c>
       <c r="I27" t="inlineStr"/>
-      <c r="J27" s="1" t="n">
+      <c r="J27" s="2" t="n">
         <v>43340</v>
       </c>
       <c r="K27" t="b">
@@ -1685,7 +1697,7 @@
         <v>-12.3</v>
       </c>
       <c r="I28" t="inlineStr"/>
-      <c r="J28" s="1" t="n">
+      <c r="J28" s="2" t="n">
         <v>46048</v>
       </c>
       <c r="K28" t="b">
@@ -1730,7 +1742,7 @@
         <v>0</v>
       </c>
       <c r="I29" t="inlineStr"/>
-      <c r="J29" s="1" t="n">
+      <c r="J29" s="2" t="n">
         <v>46211</v>
       </c>
       <c r="K29" t="b">
@@ -1775,7 +1787,7 @@
         <v>3.6</v>
       </c>
       <c r="I30" t="inlineStr"/>
-      <c r="J30" s="1" t="n">
+      <c r="J30" s="2" t="n">
         <v>46234</v>
       </c>
       <c r="K30" t="b">
@@ -1820,7 +1832,7 @@
         <v>6.2</v>
       </c>
       <c r="I31" t="inlineStr"/>
-      <c r="J31" s="1" t="n">
+      <c r="J31" s="2" t="n">
         <v>46234</v>
       </c>
       <c r="K31" t="b">
@@ -1865,7 +1877,7 @@
         <v>7.5</v>
       </c>
       <c r="I32" t="inlineStr"/>
-      <c r="J32" s="1" t="n">
+      <c r="J32" s="2" t="n">
         <v>46234</v>
       </c>
       <c r="K32" t="b">
@@ -1910,7 +1922,7 @@
         <v>10.7</v>
       </c>
       <c r="I33" t="inlineStr"/>
-      <c r="J33" s="1" t="n">
+      <c r="J33" s="2" t="n">
         <v>46234</v>
       </c>
       <c r="K33" t="b">
@@ -1955,7 +1967,7 @@
         <v>20</v>
       </c>
       <c r="I34" t="inlineStr"/>
-      <c r="J34" s="1" t="n">
+      <c r="J34" s="2" t="n">
         <v>46234</v>
       </c>
       <c r="K34" t="b">
@@ -2000,7 +2012,7 @@
         <v>30.8</v>
       </c>
       <c r="I35" t="inlineStr"/>
-      <c r="J35" s="1" t="n">
+      <c r="J35" s="2" t="n">
         <v>46234</v>
       </c>
       <c r="K35" t="b">
@@ -2045,7 +2057,7 @@
         <v>37.1</v>
       </c>
       <c r="I36" t="inlineStr"/>
-      <c r="J36" s="1" t="n">
+      <c r="J36" s="2" t="n">
         <v>46256</v>
       </c>
       <c r="K36" t="b">
@@ -2090,7 +2102,7 @@
         <v>42.8</v>
       </c>
       <c r="I37" t="inlineStr"/>
-      <c r="J37" s="1" t="n">
+      <c r="J37" s="2" t="n">
         <v>46276</v>
       </c>
       <c r="K37" t="b">
@@ -2135,7 +2147,7 @@
         <v>45.2</v>
       </c>
       <c r="I38" t="inlineStr"/>
-      <c r="J38" s="1" t="n">
+      <c r="J38" s="2" t="n">
         <v>46234</v>
       </c>
       <c r="K38" t="b">
@@ -2180,7 +2192,7 @@
         <v>46</v>
       </c>
       <c r="I39" t="inlineStr"/>
-      <c r="J39" s="1" t="n">
+      <c r="J39" s="2" t="n">
         <v>46251</v>
       </c>
       <c r="K39" t="b">
@@ -2225,7 +2237,7 @@
         <v>47.5</v>
       </c>
       <c r="I40" t="inlineStr"/>
-      <c r="J40" s="1" t="n">
+      <c r="J40" s="2" t="n">
         <v>46456</v>
       </c>
       <c r="K40" t="b">
@@ -2270,7 +2282,7 @@
         <v>57.2</v>
       </c>
       <c r="I41" t="inlineStr"/>
-      <c r="J41" s="1" t="n">
+      <c r="J41" s="2" t="n">
         <v>46246</v>
       </c>
       <c r="K41" t="b">
@@ -2315,7 +2327,7 @@
         <v>59.6</v>
       </c>
       <c r="I42" t="inlineStr"/>
-      <c r="J42" s="1" t="n">
+      <c r="J42" s="2" t="n">
         <v>46487</v>
       </c>
       <c r="K42" t="b">
@@ -2360,7 +2372,7 @@
         <v>75.40000000000001</v>
       </c>
       <c r="I43" t="inlineStr"/>
-      <c r="J43" s="1" t="n">
+      <c r="J43" s="2" t="n">
         <v>46283</v>
       </c>
       <c r="K43" t="b">
@@ -2405,7 +2417,7 @@
         <v>76.8</v>
       </c>
       <c r="I44" t="inlineStr"/>
-      <c r="J44" s="1" t="n">
+      <c r="J44" s="2" t="n">
         <v>46285</v>
       </c>
       <c r="K44" t="b">
@@ -2450,7 +2462,7 @@
         <v>83.2</v>
       </c>
       <c r="I45" t="inlineStr"/>
-      <c r="J45" s="1" t="n">
+      <c r="J45" s="2" t="n">
         <v>46547</v>
       </c>
       <c r="K45" t="b">
@@ -2495,7 +2507,7 @@
         <v>84.5</v>
       </c>
       <c r="I46" t="inlineStr"/>
-      <c r="J46" s="1" t="n">
+      <c r="J46" s="2" t="n">
         <v>46240</v>
       </c>
       <c r="K46" t="b">
@@ -2540,7 +2552,7 @@
         <v>85.8</v>
       </c>
       <c r="I47" t="inlineStr"/>
-      <c r="J47" s="1" t="n">
+      <c r="J47" s="2" t="n">
         <v>46266</v>
       </c>
       <c r="K47" t="b">
@@ -2585,7 +2597,7 @@
         <v>86.5</v>
       </c>
       <c r="I48" t="inlineStr"/>
-      <c r="J48" s="1" t="n">
+      <c r="J48" s="2" t="n">
         <v>46241</v>
       </c>
       <c r="K48" t="b">
@@ -2630,7 +2642,7 @@
         <v>91.7</v>
       </c>
       <c r="I49" t="inlineStr"/>
-      <c r="J49" s="1" t="n">
+      <c r="J49" s="2" t="n">
         <v>46243</v>
       </c>
       <c r="K49" t="b">
@@ -2675,7 +2687,7 @@
         <v>91.7</v>
       </c>
       <c r="I50" t="inlineStr"/>
-      <c r="J50" s="1" t="n">
+      <c r="J50" s="2" t="n">
         <v>46243</v>
       </c>
       <c r="K50" t="b">
@@ -2720,7 +2732,7 @@
         <v>91.7</v>
       </c>
       <c r="I51" t="inlineStr"/>
-      <c r="J51" s="1" t="n">
+      <c r="J51" s="2" t="n">
         <v>46250</v>
       </c>
       <c r="K51" t="b">
@@ -2765,7 +2777,7 @@
         <v>98.90000000000001</v>
       </c>
       <c r="I52" t="inlineStr"/>
-      <c r="J52" s="1" t="n">
+      <c r="J52" s="2" t="n">
         <v>46253</v>
       </c>
       <c r="K52" t="b">
@@ -2810,7 +2822,7 @@
         <v>105.5</v>
       </c>
       <c r="I53" t="inlineStr"/>
-      <c r="J53" s="1" t="n">
+      <c r="J53" s="2" t="n">
         <v>46280</v>
       </c>
       <c r="K53" t="b">
@@ -2855,7 +2867,7 @@
         <v>105.6</v>
       </c>
       <c r="I54" t="inlineStr"/>
-      <c r="J54" s="1" t="n">
+      <c r="J54" s="2" t="n">
         <v>46361</v>
       </c>
       <c r="K54" t="b">
@@ -2900,7 +2912,7 @@
         <v>105.7</v>
       </c>
       <c r="I55" t="inlineStr"/>
-      <c r="J55" s="1" t="n">
+      <c r="J55" s="2" t="n">
         <v>46362</v>
       </c>
       <c r="K55" t="b">
@@ -2945,7 +2957,7 @@
         <v>110.7</v>
       </c>
       <c r="I56" t="inlineStr"/>
-      <c r="J56" s="1" t="n">
+      <c r="J56" s="2" t="n">
         <v>46275</v>
       </c>
       <c r="K56" t="b">
@@ -2990,7 +3002,7 @@
         <v>113.2</v>
       </c>
       <c r="I57" t="inlineStr"/>
-      <c r="J57" s="1" t="n">
+      <c r="J57" s="2" t="n">
         <v>46377</v>
       </c>
       <c r="K57" t="b">
@@ -3035,7 +3047,7 @@
         <v>128.8</v>
       </c>
       <c r="I58" t="inlineStr"/>
-      <c r="J58" s="1" t="n">
+      <c r="J58" s="2" t="n">
         <v>46434</v>
       </c>
       <c r="K58" t="b">
@@ -3080,7 +3092,7 @@
         <v>128.8</v>
       </c>
       <c r="I59" t="inlineStr"/>
-      <c r="J59" s="1" t="n">
+      <c r="J59" s="2" t="n">
         <v>46434</v>
       </c>
       <c r="K59" t="b">
@@ -3125,7 +3137,7 @@
         <v>128.8</v>
       </c>
       <c r="I60" t="inlineStr"/>
-      <c r="J60" s="1" t="n">
+      <c r="J60" s="2" t="n">
         <v>46434</v>
       </c>
       <c r="K60" t="b">
@@ -3170,7 +3182,7 @@
         <v>128.8</v>
       </c>
       <c r="I61" t="inlineStr"/>
-      <c r="J61" s="1" t="n">
+      <c r="J61" s="2" t="n">
         <v>46434</v>
       </c>
       <c r="K61" t="b">
@@ -3215,7 +3227,7 @@
         <v>128.8</v>
       </c>
       <c r="I62" t="inlineStr"/>
-      <c r="J62" s="1" t="n">
+      <c r="J62" s="2" t="n">
         <v>46434</v>
       </c>
       <c r="K62" t="b">
@@ -3260,7 +3272,7 @@
         <v>135</v>
       </c>
       <c r="I63" t="inlineStr"/>
-      <c r="J63" s="1" t="n">
+      <c r="J63" s="2" t="n">
         <v>46280</v>
       </c>
       <c r="K63" t="b">
@@ -3305,7 +3317,7 @@
         <v>150.6</v>
       </c>
       <c r="I64" t="inlineStr"/>
-      <c r="J64" s="1" t="n">
+      <c r="J64" s="2" t="n">
         <v>46271</v>
       </c>
       <c r="K64" t="b">
@@ -3350,7 +3362,7 @@
         <v>174.2</v>
       </c>
       <c r="I65" t="inlineStr"/>
-      <c r="J65" s="1" t="n">
+      <c r="J65" s="2" t="n">
         <v>46363</v>
       </c>
       <c r="K65" t="b">
@@ -3395,7 +3407,7 @@
         <v>176.6</v>
       </c>
       <c r="I66" t="inlineStr"/>
-      <c r="J66" s="1" t="n">
+      <c r="J66" s="2" t="n">
         <v>46334</v>
       </c>
       <c r="K66" t="b">
@@ -3440,7 +3452,7 @@
         <v>177.4</v>
       </c>
       <c r="I67" t="inlineStr"/>
-      <c r="J67" s="1" t="n">
+      <c r="J67" s="2" t="n">
         <v>46407</v>
       </c>
       <c r="K67" t="b">
@@ -3485,7 +3497,7 @@
         <v>183.9</v>
       </c>
       <c r="I68" t="inlineStr"/>
-      <c r="J68" s="1" t="n">
+      <c r="J68" s="2" t="n">
         <v>46341</v>
       </c>
       <c r="K68" t="b">
@@ -3530,7 +3542,7 @@
         <v>191.7</v>
       </c>
       <c r="I69" t="inlineStr"/>
-      <c r="J69" s="1" t="n">
+      <c r="J69" s="2" t="n">
         <v>46300</v>
       </c>
       <c r="K69" t="b">
@@ -3575,7 +3587,7 @@
         <v>200</v>
       </c>
       <c r="I70" t="inlineStr"/>
-      <c r="J70" s="1" t="n">
+      <c r="J70" s="2" t="n">
         <v>46336</v>
       </c>
       <c r="K70" t="b">
@@ -3620,7 +3632,7 @@
         <v>201.1</v>
       </c>
       <c r="I71" t="inlineStr"/>
-      <c r="J71" s="1" t="n">
+      <c r="J71" s="2" t="n">
         <v>46319</v>
       </c>
       <c r="K71" t="b">
@@ -3665,7 +3677,7 @@
         <v>206.5</v>
       </c>
       <c r="I72" t="inlineStr"/>
-      <c r="J72" s="1" t="n">
+      <c r="J72" s="2" t="n">
         <v>46308</v>
       </c>
       <c r="K72" t="b">
@@ -3710,7 +3722,7 @@
         <v>207.5</v>
       </c>
       <c r="I73" t="inlineStr"/>
-      <c r="J73" s="1" t="n">
+      <c r="J73" s="2" t="n">
         <v>46390</v>
       </c>
       <c r="K73" t="b">
@@ -3755,7 +3767,7 @@
         <v>247</v>
       </c>
       <c r="I74" t="inlineStr"/>
-      <c r="J74" s="1" t="n">
+      <c r="J74" s="2" t="n">
         <v>46443</v>
       </c>
       <c r="K74" t="b">
@@ -3800,7 +3812,7 @@
         <v>285.3</v>
       </c>
       <c r="I75" t="inlineStr"/>
-      <c r="J75" s="1" t="n">
+      <c r="J75" s="2" t="n">
         <v>46304</v>
       </c>
       <c r="K75" t="b">
@@ -3845,7 +3857,7 @@
         <v>290.8</v>
       </c>
       <c r="I76" t="inlineStr"/>
-      <c r="J76" s="1" t="n">
+      <c r="J76" s="2" t="n">
         <v>46362</v>
       </c>
       <c r="K76" t="b">
@@ -3890,7 +3902,7 @@
         <v>295.2</v>
       </c>
       <c r="I77" t="inlineStr"/>
-      <c r="J77" s="1" t="n">
+      <c r="J77" s="2" t="n">
         <v>46463</v>
       </c>
       <c r="K77" t="b">
@@ -3935,7 +3947,7 @@
         <v>300.2</v>
       </c>
       <c r="I78" t="inlineStr"/>
-      <c r="J78" s="1" t="n">
+      <c r="J78" s="2" t="n">
         <v>46466</v>
       </c>
       <c r="K78" t="b">
@@ -3984,7 +3996,7 @@
           <t>-317m</t>
         </is>
       </c>
-      <c r="J79" s="1" t="n">
+      <c r="J79" s="2" t="n">
         <v>36557</v>
       </c>
       <c r="K79" t="b">
@@ -4033,7 +4045,7 @@
           <t>-164m</t>
         </is>
       </c>
-      <c r="J80" s="1" t="n">
+      <c r="J80" s="2" t="n">
         <v>41275</v>
       </c>
       <c r="K80" t="b">
@@ -4082,7 +4094,7 @@
           <t>-27m</t>
         </is>
       </c>
-      <c r="J81" s="1" t="n">
+      <c r="J81" s="2" t="n">
         <v>45380</v>
       </c>
       <c r="K81" t="b">
@@ -4131,7 +4143,7 @@
           <t>-25m</t>
         </is>
       </c>
-      <c r="J82" s="1" t="n">
+      <c r="J82" s="2" t="n">
         <v>45421</v>
       </c>
       <c r="K82" t="b">
@@ -4180,7 +4192,7 @@
           <t>-25m</t>
         </is>
       </c>
-      <c r="J83" s="1" t="n">
+      <c r="J83" s="2" t="n">
         <v>45428</v>
       </c>
       <c r="K83" t="b">
@@ -4229,7 +4241,7 @@
           <t>-23m</t>
         </is>
       </c>
-      <c r="J84" s="1" t="n">
+      <c r="J84" s="2" t="n">
         <v>45490</v>
       </c>
       <c r="K84" t="b">
@@ -4278,7 +4290,7 @@
           <t>-21m</t>
         </is>
       </c>
-      <c r="J85" s="1" t="n">
+      <c r="J85" s="2" t="n">
         <v>45566</v>
       </c>
       <c r="K85" t="b">
@@ -4327,7 +4339,7 @@
           <t>-7m</t>
         </is>
       </c>
-      <c r="J86" s="1" t="n">
+      <c r="J86" s="2" t="n">
         <v>45986</v>
       </c>
       <c r="K86" t="b">
@@ -4376,7 +4388,7 @@
           <t>-3m</t>
         </is>
       </c>
-      <c r="J87" s="1" t="n">
+      <c r="J87" s="2" t="n">
         <v>46106</v>
       </c>
       <c r="K87" t="b">
@@ -4425,7 +4437,7 @@
           <t>-2m</t>
         </is>
       </c>
-      <c r="J88" s="1" t="n">
+      <c r="J88" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="K88" t="b">
@@ -4474,7 +4486,7 @@
           <t>2m</t>
         </is>
       </c>
-      <c r="J89" s="1" t="n">
+      <c r="J89" s="2" t="n">
         <v>46274</v>
       </c>
       <c r="K89" t="b">
@@ -4523,7 +4535,7 @@
           <t>2m</t>
         </is>
       </c>
-      <c r="J90" s="1" t="n">
+      <c r="J90" s="2" t="n">
         <v>46276</v>
       </c>
       <c r="K90" t="b">
@@ -4572,7 +4584,7 @@
           <t>2m</t>
         </is>
       </c>
-      <c r="J91" s="1" t="n">
+      <c r="J91" s="2" t="n">
         <v>46284</v>
       </c>
       <c r="K91" t="b">
@@ -4621,7 +4633,7 @@
           <t>3m</t>
         </is>
       </c>
-      <c r="J92" s="1" t="n">
+      <c r="J92" s="2" t="n">
         <v>46317</v>
       </c>
       <c r="K92" t="b">
@@ -4670,7 +4682,7 @@
           <t>3m</t>
         </is>
       </c>
-      <c r="J93" s="1" t="n">
+      <c r="J93" s="2" t="n">
         <v>46319</v>
       </c>
       <c r="K93" t="b">
@@ -4719,7 +4731,7 @@
           <t>4m</t>
         </is>
       </c>
-      <c r="J94" s="1" t="n">
+      <c r="J94" s="2" t="n">
         <v>46333</v>
       </c>
       <c r="K94" t="b">
@@ -4768,7 +4780,7 @@
           <t>4m</t>
         </is>
       </c>
-      <c r="J95" s="1" t="n">
+      <c r="J95" s="2" t="n">
         <v>46338</v>
       </c>
       <c r="K95" t="b">
@@ -4817,7 +4829,7 @@
           <t>4m</t>
         </is>
       </c>
-      <c r="J96" s="1" t="n">
+      <c r="J96" s="2" t="n">
         <v>46338</v>
       </c>
       <c r="K96" t="b">
@@ -4866,7 +4878,7 @@
           <t>4m</t>
         </is>
       </c>
-      <c r="J97" s="1" t="n">
+      <c r="J97" s="2" t="n">
         <v>46341</v>
       </c>
       <c r="K97" t="b">
@@ -4915,7 +4927,7 @@
           <t>4m</t>
         </is>
       </c>
-      <c r="J98" s="1" t="n">
+      <c r="J98" s="2" t="n">
         <v>46344</v>
       </c>
       <c r="K98" t="b">
@@ -4964,7 +4976,7 @@
           <t>4m</t>
         </is>
       </c>
-      <c r="J99" s="1" t="n">
+      <c r="J99" s="2" t="n">
         <v>46354</v>
       </c>
       <c r="K99" t="b">
@@ -5013,7 +5025,7 @@
           <t>4m</t>
         </is>
       </c>
-      <c r="J100" s="1" t="n">
+      <c r="J100" s="2" t="n">
         <v>46360</v>
       </c>
       <c r="K100" t="b">
@@ -5062,7 +5074,7 @@
           <t>4m</t>
         </is>
       </c>
-      <c r="J101" s="1" t="n">
+      <c r="J101" s="2" t="n">
         <v>46360</v>
       </c>
       <c r="K101" t="b">
@@ -5111,7 +5123,7 @@
           <t>5m</t>
         </is>
       </c>
-      <c r="J102" s="1" t="n">
+      <c r="J102" s="2" t="n">
         <v>46366</v>
       </c>
       <c r="K102" t="b">
@@ -5160,7 +5172,7 @@
           <t>5m</t>
         </is>
       </c>
-      <c r="J103" s="1" t="n">
+      <c r="J103" s="2" t="n">
         <v>46375</v>
       </c>
       <c r="K103" t="b">
@@ -5209,7 +5221,7 @@
           <t>5m</t>
         </is>
       </c>
-      <c r="J104" s="1" t="n">
+      <c r="J104" s="2" t="n">
         <v>46388</v>
       </c>
       <c r="K104" t="b">
@@ -5258,7 +5270,7 @@
           <t>6m</t>
         </is>
       </c>
-      <c r="J105" s="1" t="n">
+      <c r="J105" s="2" t="n">
         <v>46401</v>
       </c>
       <c r="K105" t="b">
@@ -5307,7 +5319,7 @@
           <t>6m</t>
         </is>
       </c>
-      <c r="J106" s="1" t="n">
+      <c r="J106" s="2" t="n">
         <v>46401</v>
       </c>
       <c r="K106" t="b">
@@ -5356,7 +5368,7 @@
           <t>6m</t>
         </is>
       </c>
-      <c r="J107" s="1" t="n">
+      <c r="J107" s="2" t="n">
         <v>46401</v>
       </c>
       <c r="K107" t="b">
@@ -5405,7 +5417,7 @@
           <t>6m</t>
         </is>
       </c>
-      <c r="J108" s="1" t="n">
+      <c r="J108" s="2" t="n">
         <v>46413</v>
       </c>
       <c r="K108" t="b">
@@ -5454,7 +5466,7 @@
           <t>7m</t>
         </is>
       </c>
-      <c r="J109" s="1" t="n">
+      <c r="J109" s="2" t="n">
         <v>46424</v>
       </c>
       <c r="K109" t="b">
@@ -5503,7 +5515,7 @@
           <t>7m</t>
         </is>
       </c>
-      <c r="J110" s="1" t="n">
+      <c r="J110" s="2" t="n">
         <v>46427</v>
       </c>
       <c r="K110" t="b">
@@ -5552,7 +5564,7 @@
           <t>7m</t>
         </is>
       </c>
-      <c r="J111" s="1" t="n">
+      <c r="J111" s="2" t="n">
         <v>46437</v>
       </c>
       <c r="K111" t="b">
@@ -5601,7 +5613,7 @@
           <t>7m</t>
         </is>
       </c>
-      <c r="J112" s="1" t="n">
+      <c r="J112" s="2" t="n">
         <v>46451</v>
       </c>
       <c r="K112" t="b">
@@ -5650,7 +5662,7 @@
           <t>8m</t>
         </is>
       </c>
-      <c r="J113" s="1" t="n">
+      <c r="J113" s="2" t="n">
         <v>46455</v>
       </c>
       <c r="K113" t="b">
@@ -5699,7 +5711,7 @@
           <t>8m</t>
         </is>
       </c>
-      <c r="J114" s="1" t="n">
+      <c r="J114" s="2" t="n">
         <v>46457</v>
       </c>
       <c r="K114" t="b">
@@ -5748,7 +5760,7 @@
           <t>8m</t>
         </is>
       </c>
-      <c r="J115" s="1" t="n">
+      <c r="J115" s="2" t="n">
         <v>46462</v>
       </c>
       <c r="K115" t="b">
@@ -5797,7 +5809,7 @@
           <t>8m</t>
         </is>
       </c>
-      <c r="J116" s="1" t="n">
+      <c r="J116" s="2" t="n">
         <v>46464</v>
       </c>
       <c r="K116" t="b">
@@ -5846,7 +5858,7 @@
           <t>8m</t>
         </is>
       </c>
-      <c r="J117" s="1" t="n">
+      <c r="J117" s="2" t="n">
         <v>46470</v>
       </c>
       <c r="K117" t="b">
@@ -5895,7 +5907,7 @@
           <t>9m</t>
         </is>
       </c>
-      <c r="J118" s="1" t="n">
+      <c r="J118" s="2" t="n">
         <v>46485</v>
       </c>
       <c r="K118" t="b">
@@ -5944,7 +5956,7 @@
           <t>9m</t>
         </is>
       </c>
-      <c r="J119" s="1" t="n">
+      <c r="J119" s="2" t="n">
         <v>46499</v>
       </c>
       <c r="K119" t="b">
@@ -5993,7 +6005,7 @@
           <t>9m</t>
         </is>
       </c>
-      <c r="J120" s="1" t="n">
+      <c r="J120" s="2" t="n">
         <v>46504</v>
       </c>
       <c r="K120" t="b">
@@ -6042,7 +6054,7 @@
           <t>9m</t>
         </is>
       </c>
-      <c r="J121" s="1" t="n">
+      <c r="J121" s="2" t="n">
         <v>46504</v>
       </c>
       <c r="K121" t="b">
@@ -6091,7 +6103,7 @@
           <t>9m</t>
         </is>
       </c>
-      <c r="J122" s="1" t="n">
+      <c r="J122" s="2" t="n">
         <v>46507</v>
       </c>
       <c r="K122" t="b">
@@ -6140,7 +6152,7 @@
           <t>9m</t>
         </is>
       </c>
-      <c r="J123" s="1" t="n">
+      <c r="J123" s="2" t="n">
         <v>46508</v>
       </c>
       <c r="K123" t="b">
@@ -6189,7 +6201,7 @@
           <t>9m</t>
         </is>
       </c>
-      <c r="J124" s="1" t="n">
+      <c r="J124" s="2" t="n">
         <v>46512</v>
       </c>
       <c r="K124" t="b">
@@ -6238,7 +6250,7 @@
           <t>9m</t>
         </is>
       </c>
-      <c r="J125" s="1" t="n">
+      <c r="J125" s="2" t="n">
         <v>46512</v>
       </c>
       <c r="K125" t="b">
@@ -6287,7 +6299,7 @@
           <t>10m</t>
         </is>
       </c>
-      <c r="J126" s="1" t="n">
+      <c r="J126" s="2" t="n">
         <v>46528</v>
       </c>
       <c r="K126" t="b">
@@ -6336,7 +6348,7 @@
           <t>10m</t>
         </is>
       </c>
-      <c r="J127" s="1" t="n">
+      <c r="J127" s="2" t="n">
         <v>46529</v>
       </c>
       <c r="K127" t="b">
@@ -6385,7 +6397,7 @@
           <t>10m</t>
         </is>
       </c>
-      <c r="J128" s="1" t="n">
+      <c r="J128" s="2" t="n">
         <v>46537</v>
       </c>
       <c r="K128" t="b">
@@ -6434,7 +6446,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J129" s="1" t="n">
+      <c r="J129" s="2" t="n">
         <v>46546</v>
       </c>
       <c r="K129" t="b">
@@ -6483,7 +6495,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J130" s="1" t="n">
+      <c r="J130" s="2" t="n">
         <v>46547</v>
       </c>
       <c r="K130" t="b">
@@ -6532,7 +6544,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J131" s="1" t="n">
+      <c r="J131" s="2" t="n">
         <v>46547</v>
       </c>
       <c r="K131" t="b">
@@ -6581,7 +6593,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J132" s="1" t="n">
+      <c r="J132" s="2" t="n">
         <v>46547</v>
       </c>
       <c r="K132" t="b">
@@ -6630,7 +6642,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J133" s="1" t="n">
+      <c r="J133" s="2" t="n">
         <v>46551</v>
       </c>
       <c r="K133" t="b">
@@ -6679,7 +6691,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J134" s="1" t="n">
+      <c r="J134" s="2" t="n">
         <v>46560</v>
       </c>
       <c r="K134" t="b">
@@ -6728,7 +6740,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J135" s="1" t="n">
+      <c r="J135" s="2" t="n">
         <v>46564</v>
       </c>
       <c r="K135" t="b">
@@ -6777,7 +6789,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J136" s="1" t="n">
+      <c r="J136" s="2" t="n">
         <v>46567</v>
       </c>
       <c r="K136" t="b">
@@ -6826,7 +6838,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J137" s="1" t="n">
+      <c r="J137" s="2" t="n">
         <v>46568</v>
       </c>
       <c r="K137" t="b">
@@ -6875,7 +6887,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J138" s="1" t="n">
+      <c r="J138" s="2" t="n">
         <v>46571</v>
       </c>
       <c r="K138" t="b">
@@ -6924,7 +6936,7 @@
           <t>-14d</t>
         </is>
       </c>
-      <c r="J139" s="1" t="n">
+      <c r="J139" s="2" t="n">
         <v>46197</v>
       </c>
       <c r="K139" t="b">
@@ -6973,7 +6985,7 @@
           <t>1d</t>
         </is>
       </c>
-      <c r="J140" s="1" t="n">
+      <c r="J140" s="2" t="n">
         <v>46212</v>
       </c>
       <c r="K140" t="b">
@@ -7022,7 +7034,7 @@
           <t>14d</t>
         </is>
       </c>
-      <c r="J141" s="1" t="n">
+      <c r="J141" s="2" t="n">
         <v>46225</v>
       </c>
       <c r="K141" t="b">
@@ -7071,7 +7083,7 @@
           <t>23d</t>
         </is>
       </c>
-      <c r="J142" s="1" t="n">
+      <c r="J142" s="2" t="n">
         <v>46234</v>
       </c>
       <c r="K142" t="b">
@@ -7120,7 +7132,7 @@
           <t>24d</t>
         </is>
       </c>
-      <c r="J143" s="1" t="n">
+      <c r="J143" s="2" t="n">
         <v>46234</v>
       </c>
       <c r="K143" t="b">
@@ -7169,7 +7181,7 @@
           <t>1me23d</t>
         </is>
       </c>
-      <c r="J144" s="1" t="n">
+      <c r="J144" s="2" t="n">
         <v>46263</v>
       </c>
       <c r="K144" t="b">
@@ -7218,7 +7230,7 @@
           <t>1me25d</t>
         </is>
       </c>
-      <c r="J145" s="1" t="n">
+      <c r="J145" s="2" t="n">
         <v>46266</v>
       </c>
       <c r="K145" t="b">
@@ -7263,7 +7275,7 @@
         <v>-1476</v>
       </c>
       <c r="I146" t="inlineStr"/>
-      <c r="J146" s="1" t="n">
+      <c r="J146" s="2" t="n">
         <v>43773</v>
       </c>
       <c r="K146" t="b">
@@ -7308,7 +7320,7 @@
         <v>-1469</v>
       </c>
       <c r="I147" t="inlineStr"/>
-      <c r="J147" s="1" t="n">
+      <c r="J147" s="2" t="n">
         <v>43773</v>
       </c>
       <c r="K147" t="b">
@@ -7353,7 +7365,7 @@
         <v>-1121</v>
       </c>
       <c r="I148" t="inlineStr"/>
-      <c r="J148" s="1" t="n">
+      <c r="J148" s="2" t="n">
         <v>45295</v>
       </c>
       <c r="K148" t="b">
@@ -7398,7 +7410,7 @@
         <v>-1018</v>
       </c>
       <c r="I149" t="inlineStr"/>
-      <c r="J149" s="1" t="n">
+      <c r="J149" s="2" t="n">
         <v>45617</v>
       </c>
       <c r="K149" t="b">
@@ -7443,7 +7455,7 @@
         <v>-950</v>
       </c>
       <c r="I150" t="inlineStr"/>
-      <c r="J150" s="1" t="n">
+      <c r="J150" s="2" t="n">
         <v>45677</v>
       </c>
       <c r="K150" t="b">
@@ -7488,7 +7500,7 @@
         <v>-943</v>
       </c>
       <c r="I151" t="inlineStr"/>
-      <c r="J151" s="1" t="n">
+      <c r="J151" s="2" t="n">
         <v>44944</v>
       </c>
       <c r="K151" t="b">
@@ -7533,7 +7545,7 @@
         <v>-252</v>
       </c>
       <c r="I152" t="inlineStr"/>
-      <c r="J152" s="1" t="n">
+      <c r="J152" s="2" t="n">
         <v>46092</v>
       </c>
       <c r="K152" t="b">
@@ -7578,7 +7590,7 @@
         <v>-196</v>
       </c>
       <c r="I153" t="inlineStr"/>
-      <c r="J153" s="1" t="n">
+      <c r="J153" s="2" t="n">
         <v>45988</v>
       </c>
       <c r="K153" t="b">
@@ -7623,7 +7635,7 @@
         <v>-196</v>
       </c>
       <c r="I154" t="inlineStr"/>
-      <c r="J154" s="1" t="n">
+      <c r="J154" s="2" t="n">
         <v>45988</v>
       </c>
       <c r="K154" t="b">
@@ -7668,7 +7680,7 @@
         <v>-47</v>
       </c>
       <c r="I155" t="inlineStr"/>
-      <c r="J155" s="1" t="n">
+      <c r="J155" s="2" t="n">
         <v>46176</v>
       </c>
       <c r="K155" t="b">
@@ -7713,7 +7725,7 @@
         <v>-47</v>
       </c>
       <c r="I156" t="inlineStr"/>
-      <c r="J156" s="1" t="n">
+      <c r="J156" s="2" t="n">
         <v>46176</v>
       </c>
       <c r="K156" t="b">
@@ -7758,7 +7770,7 @@
         <v>-33</v>
       </c>
       <c r="I157" t="inlineStr"/>
-      <c r="J157" s="1" t="n">
+      <c r="J157" s="2" t="n">
         <v>46199</v>
       </c>
       <c r="K157" t="b">
@@ -7803,7 +7815,7 @@
         <v>-33</v>
       </c>
       <c r="I158" t="inlineStr"/>
-      <c r="J158" s="1" t="n">
+      <c r="J158" s="2" t="n">
         <v>46199</v>
       </c>
       <c r="K158" t="b">
@@ -7848,7 +7860,7 @@
         <v>-6</v>
       </c>
       <c r="I159" t="inlineStr"/>
-      <c r="J159" s="1" t="n">
+      <c r="J159" s="2" t="n">
         <v>45967</v>
       </c>
       <c r="K159" t="b">
@@ -7893,7 +7905,7 @@
         <v>43</v>
       </c>
       <c r="I160" t="inlineStr"/>
-      <c r="J160" s="1" t="n">
+      <c r="J160" s="2" t="n">
         <v>46440</v>
       </c>
       <c r="K160" t="b">
@@ -7938,7 +7950,7 @@
         <v>43</v>
       </c>
       <c r="I161" t="inlineStr"/>
-      <c r="J161" s="1" t="n">
+      <c r="J161" s="2" t="n">
         <v>46440</v>
       </c>
       <c r="K161" t="b">
@@ -7983,7 +7995,7 @@
         <v>73</v>
       </c>
       <c r="I162" t="inlineStr"/>
-      <c r="J162" s="1" t="n">
+      <c r="J162" s="2" t="n">
         <v>46264</v>
       </c>
       <c r="K162" t="b">
@@ -8028,7 +8040,7 @@
         <v>73</v>
       </c>
       <c r="I163" t="inlineStr"/>
-      <c r="J163" s="1" t="n">
+      <c r="J163" s="2" t="n">
         <v>46264</v>
       </c>
       <c r="K163" t="b">
@@ -8073,7 +8085,7 @@
         <v>102</v>
       </c>
       <c r="I164" t="inlineStr"/>
-      <c r="J164" s="1" t="n">
+      <c r="J164" s="2" t="n">
         <v>46463</v>
       </c>
       <c r="K164" t="b">
@@ -8118,7 +8130,7 @@
         <v>118</v>
       </c>
       <c r="I165" t="inlineStr"/>
-      <c r="J165" s="1" t="n">
+      <c r="J165" s="2" t="n">
         <v>46337</v>
       </c>
       <c r="K165" t="b">
@@ -8163,7 +8175,7 @@
         <v>146</v>
       </c>
       <c r="I166" t="inlineStr"/>
-      <c r="J166" s="1" t="n">
+      <c r="J166" s="2" t="n">
         <v>46451</v>
       </c>
       <c r="K166" t="b">
@@ -8208,7 +8220,7 @@
         <v>152</v>
       </c>
       <c r="I167" t="inlineStr"/>
-      <c r="J167" s="1" t="n">
+      <c r="J167" s="2" t="n">
         <v>46245</v>
       </c>
       <c r="K167" t="b">
@@ -8253,7 +8265,7 @@
         <v>152</v>
       </c>
       <c r="I168" t="inlineStr"/>
-      <c r="J168" s="1" t="n">
+      <c r="J168" s="2" t="n">
         <v>46245</v>
       </c>
       <c r="K168" t="b">
@@ -8298,7 +8310,7 @@
         <v>163</v>
       </c>
       <c r="I169" t="inlineStr"/>
-      <c r="J169" s="1" t="n">
+      <c r="J169" s="2" t="n">
         <v>46324</v>
       </c>
       <c r="K169" t="b">
@@ -8343,7 +8355,7 @@
         <v>163</v>
       </c>
       <c r="I170" t="inlineStr"/>
-      <c r="J170" s="1" t="n">
+      <c r="J170" s="2" t="n">
         <v>46324</v>
       </c>
       <c r="K170" t="b">
@@ -8388,7 +8400,7 @@
         <v>164</v>
       </c>
       <c r="I171" t="inlineStr"/>
-      <c r="J171" s="1" t="n">
+      <c r="J171" s="2" t="n">
         <v>46426</v>
       </c>
       <c r="K171" t="b">
@@ -8433,7 +8445,7 @@
         <v>175</v>
       </c>
       <c r="I172" t="inlineStr"/>
-      <c r="J172" s="1" t="n">
+      <c r="J172" s="2" t="n">
         <v>46383</v>
       </c>
       <c r="K172" t="b">
@@ -8478,7 +8490,7 @@
         <v>186</v>
       </c>
       <c r="I173" t="inlineStr"/>
-      <c r="J173" s="1" t="n">
+      <c r="J173" s="2" t="n">
         <v>46392</v>
       </c>
       <c r="K173" t="b">
@@ -8523,7 +8535,7 @@
         <v>205</v>
       </c>
       <c r="I174" t="inlineStr"/>
-      <c r="J174" s="1" t="n">
+      <c r="J174" s="2" t="n">
         <v>46390</v>
       </c>
       <c r="K174" t="b">
@@ -8568,7 +8580,7 @@
         <v>207</v>
       </c>
       <c r="I175" t="inlineStr"/>
-      <c r="J175" s="1" t="n">
+      <c r="J175" s="2" t="n">
         <v>46392</v>
       </c>
       <c r="K175" t="b">
@@ -8613,7 +8625,7 @@
         <v>218</v>
       </c>
       <c r="I176" t="inlineStr"/>
-      <c r="J176" s="1" t="n">
+      <c r="J176" s="2" t="n">
         <v>46506</v>
       </c>
       <c r="K176" t="b">
@@ -8658,7 +8670,7 @@
         <v>246</v>
       </c>
       <c r="I177" t="inlineStr"/>
-      <c r="J177" s="1" t="n">
+      <c r="J177" s="2" t="n">
         <v>46478</v>
       </c>
       <c r="K177" t="b">
@@ -8703,7 +8715,7 @@
         <v>248</v>
       </c>
       <c r="I178" t="inlineStr"/>
-      <c r="J178" s="1" t="n">
+      <c r="J178" s="2" t="n">
         <v>46500</v>
       </c>
       <c r="K178" t="b">
@@ -8748,7 +8760,7 @@
         <v>276</v>
       </c>
       <c r="I179" t="inlineStr"/>
-      <c r="J179" s="1" t="n">
+      <c r="J179" s="2" t="n">
         <v>46430</v>
       </c>
       <c r="K179" t="b">
@@ -8793,7 +8805,7 @@
         <v>276</v>
       </c>
       <c r="I180" t="inlineStr"/>
-      <c r="J180" s="1" t="n">
+      <c r="J180" s="2" t="n">
         <v>46430</v>
       </c>
       <c r="K180" t="b">
@@ -8838,7 +8850,7 @@
         <v>290</v>
       </c>
       <c r="I181" t="inlineStr"/>
-      <c r="J181" s="1" t="n">
+      <c r="J181" s="2" t="n">
         <v>46467</v>
       </c>
       <c r="K181" t="b">
@@ -8883,7 +8895,7 @@
         <v>317</v>
       </c>
       <c r="I182" t="inlineStr"/>
-      <c r="J182" s="1" t="n">
+      <c r="J182" s="2" t="n">
         <v>46529</v>
       </c>
       <c r="K182" t="b">
@@ -8928,7 +8940,7 @@
         <v>420</v>
       </c>
       <c r="I183" t="inlineStr"/>
-      <c r="J183" s="1" t="n">
+      <c r="J183" s="2" t="n">
         <v>46566</v>
       </c>
       <c r="K183" t="b">
@@ -8973,7 +8985,7 @@
         <v>426</v>
       </c>
       <c r="I184" t="inlineStr"/>
-      <c r="J184" s="1" t="n">
+      <c r="J184" s="2" t="n">
         <v>46571</v>
       </c>
       <c r="K184" t="b">
@@ -9018,7 +9030,7 @@
         <v>721</v>
       </c>
       <c r="I185" t="inlineStr"/>
-      <c r="J185" s="1" t="n">
+      <c r="J185" s="2" t="n">
         <v>46325</v>
       </c>
       <c r="K185" t="b">
@@ -9063,7 +9075,7 @@
         <v>721</v>
       </c>
       <c r="I186" t="inlineStr"/>
-      <c r="J186" s="1" t="n">
+      <c r="J186" s="2" t="n">
         <v>46325</v>
       </c>
       <c r="K186" t="b">
@@ -9108,7 +9120,7 @@
         <v>850</v>
       </c>
       <c r="I187" t="inlineStr"/>
-      <c r="J187" s="1" t="n">
+      <c r="J187" s="2" t="n">
         <v>46345</v>
       </c>
       <c r="K187" t="b">
@@ -9153,7 +9165,7 @@
         <v>850</v>
       </c>
       <c r="I188" t="inlineStr"/>
-      <c r="J188" s="1" t="n">
+      <c r="J188" s="2" t="n">
         <v>46345</v>
       </c>
       <c r="K188" t="b">
@@ -9198,7 +9210,7 @@
         <v>1661</v>
       </c>
       <c r="I189" t="inlineStr"/>
-      <c r="J189" s="1" t="n">
+      <c r="J189" s="2" t="n">
         <v>46498</v>
       </c>
       <c r="K189" t="b">
@@ -9243,7 +9255,7 @@
         <v>1661</v>
       </c>
       <c r="I190" t="inlineStr"/>
-      <c r="J190" s="1" t="n">
+      <c r="J190" s="2" t="n">
         <v>46498</v>
       </c>
       <c r="K190" t="b">
@@ -9288,7 +9300,7 @@
         <v>488</v>
       </c>
       <c r="I191" t="inlineStr"/>
-      <c r="J191" s="1" t="n">
+      <c r="J191" s="2" t="n">
         <v>46190</v>
       </c>
       <c r="K191" t="b">
@@ -9333,7 +9345,7 @@
         <v>25565</v>
       </c>
       <c r="I192" t="inlineStr"/>
-      <c r="J192" s="1" t="n">
+      <c r="J192" s="2" t="n">
         <v>46190</v>
       </c>
       <c r="K192" t="b">
@@ -9378,7 +9390,7 @@
         <v>25567</v>
       </c>
       <c r="I193" t="inlineStr"/>
-      <c r="J193" s="1" t="n">
+      <c r="J193" s="2" t="n">
         <v>46190</v>
       </c>
       <c r="K193" t="b">
@@ -9423,7 +9435,7 @@
         <v>31293</v>
       </c>
       <c r="I194" t="inlineStr"/>
-      <c r="J194" s="1" t="n">
+      <c r="J194" s="2" t="n">
         <v>46190</v>
       </c>
       <c r="K194" t="b">

</xml_diff>

<commit_message>
Atualização automática: vencimentos_tmot (10/07/2026 17:31)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
@@ -20,16 +20,13 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -40,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -48,21 +45,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -433,57 +421,57 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>matricula</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>operador</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>pn</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>sn</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>nomenclatura</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>inspecao</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>tipo_vencimento</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>disponibilidade_valor</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>disponibilidade_texto</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>data_vencimento</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>vencido</t>
         </is>
@@ -527,7 +515,7 @@
         <v>-4402.8</v>
       </c>
       <c r="I2" t="inlineStr"/>
-      <c r="J2" s="2" t="n">
+      <c r="J2" s="1" t="n">
         <v>41388</v>
       </c>
       <c r="K2" t="b">
@@ -572,7 +560,7 @@
         <v>-4254.8</v>
       </c>
       <c r="I3" t="inlineStr"/>
-      <c r="J3" s="2" t="n">
+      <c r="J3" s="1" t="n">
         <v>39285</v>
       </c>
       <c r="K3" t="b">
@@ -617,7 +605,7 @@
         <v>-2354.2</v>
       </c>
       <c r="I4" t="inlineStr"/>
-      <c r="J4" s="2" t="n">
+      <c r="J4" s="1" t="n">
         <v>40669</v>
       </c>
       <c r="K4" t="b">
@@ -662,7 +650,7 @@
         <v>-896.8</v>
       </c>
       <c r="I5" t="inlineStr"/>
-      <c r="J5" s="2" t="n">
+      <c r="J5" s="1" t="n">
         <v>40669</v>
       </c>
       <c r="K5" t="b">
@@ -707,7 +695,7 @@
         <v>-854.1</v>
       </c>
       <c r="I6" t="inlineStr"/>
-      <c r="J6" s="2" t="n">
+      <c r="J6" s="1" t="n">
         <v>44884</v>
       </c>
       <c r="K6" t="b">
@@ -752,7 +740,7 @@
         <v>-413.2</v>
       </c>
       <c r="I7" t="inlineStr"/>
-      <c r="J7" s="2" t="n">
+      <c r="J7" s="1" t="n">
         <v>43855</v>
       </c>
       <c r="K7" t="b">
@@ -797,7 +785,7 @@
         <v>-391.8</v>
       </c>
       <c r="I8" t="inlineStr"/>
-      <c r="J8" s="2" t="n">
+      <c r="J8" s="1" t="n">
         <v>42769</v>
       </c>
       <c r="K8" t="b">
@@ -842,7 +830,7 @@
         <v>-371.5</v>
       </c>
       <c r="I9" t="inlineStr"/>
-      <c r="J9" s="2" t="n">
+      <c r="J9" s="1" t="n">
         <v>46014</v>
       </c>
       <c r="K9" t="b">
@@ -887,7 +875,7 @@
         <v>-368.8</v>
       </c>
       <c r="I10" t="inlineStr"/>
-      <c r="J10" s="2" t="n">
+      <c r="J10" s="1" t="n">
         <v>46014</v>
       </c>
       <c r="K10" t="b">
@@ -932,7 +920,7 @@
         <v>-359</v>
       </c>
       <c r="I11" t="inlineStr"/>
-      <c r="J11" s="2" t="n">
+      <c r="J11" s="1" t="n">
         <v>45804</v>
       </c>
       <c r="K11" t="b">
@@ -977,7 +965,7 @@
         <v>-359</v>
       </c>
       <c r="I12" t="inlineStr"/>
-      <c r="J12" s="2" t="n">
+      <c r="J12" s="1" t="n">
         <v>45804</v>
       </c>
       <c r="K12" t="b">
@@ -1022,7 +1010,7 @@
         <v>-351</v>
       </c>
       <c r="I13" t="inlineStr"/>
-      <c r="J13" s="2" t="n">
+      <c r="J13" s="1" t="n">
         <v>42821</v>
       </c>
       <c r="K13" t="b">
@@ -1067,7 +1055,7 @@
         <v>-351</v>
       </c>
       <c r="I14" t="inlineStr"/>
-      <c r="J14" s="2" t="n">
+      <c r="J14" s="1" t="n">
         <v>46014</v>
       </c>
       <c r="K14" t="b">
@@ -1112,7 +1100,7 @@
         <v>-351</v>
       </c>
       <c r="I15" t="inlineStr"/>
-      <c r="J15" s="2" t="n">
+      <c r="J15" s="1" t="n">
         <v>46014</v>
       </c>
       <c r="K15" t="b">
@@ -1157,7 +1145,7 @@
         <v>-351</v>
       </c>
       <c r="I16" t="inlineStr"/>
-      <c r="J16" s="2" t="n">
+      <c r="J16" s="1" t="n">
         <v>46014</v>
       </c>
       <c r="K16" t="b">
@@ -1202,7 +1190,7 @@
         <v>-345.8</v>
       </c>
       <c r="I17" t="inlineStr"/>
-      <c r="J17" s="2" t="n">
+      <c r="J17" s="1" t="n">
         <v>46017</v>
       </c>
       <c r="K17" t="b">
@@ -1247,7 +1235,7 @@
         <v>-345.8</v>
       </c>
       <c r="I18" t="inlineStr"/>
-      <c r="J18" s="2" t="n">
+      <c r="J18" s="1" t="n">
         <v>46017</v>
       </c>
       <c r="K18" t="b">
@@ -1292,7 +1280,7 @@
         <v>-264.2</v>
       </c>
       <c r="I19" t="inlineStr"/>
-      <c r="J19" s="2" t="n">
+      <c r="J19" s="1" t="n">
         <v>40979</v>
       </c>
       <c r="K19" t="b">
@@ -1337,7 +1325,7 @@
         <v>-206.4</v>
       </c>
       <c r="I20" t="inlineStr"/>
-      <c r="J20" s="2" t="n">
+      <c r="J20" s="1" t="n">
         <v>36669</v>
       </c>
       <c r="K20" t="b">
@@ -1382,7 +1370,7 @@
         <v>-131.6</v>
       </c>
       <c r="I21" t="inlineStr"/>
-      <c r="J21" s="2" t="n">
+      <c r="J21" s="1" t="n">
         <v>46111</v>
       </c>
       <c r="K21" t="b">
@@ -1427,7 +1415,7 @@
         <v>-131.6</v>
       </c>
       <c r="I22" t="inlineStr"/>
-      <c r="J22" s="2" t="n">
+      <c r="J22" s="1" t="n">
         <v>46111</v>
       </c>
       <c r="K22" t="b">
@@ -1472,7 +1460,7 @@
         <v>-131.6</v>
       </c>
       <c r="I23" t="inlineStr"/>
-      <c r="J23" s="2" t="n">
+      <c r="J23" s="1" t="n">
         <v>46111</v>
       </c>
       <c r="K23" t="b">
@@ -1517,7 +1505,7 @@
         <v>-131.6</v>
       </c>
       <c r="I24" t="inlineStr"/>
-      <c r="J24" s="2" t="n">
+      <c r="J24" s="1" t="n">
         <v>46111</v>
       </c>
       <c r="K24" t="b">
@@ -1562,7 +1550,7 @@
         <v>-131.6</v>
       </c>
       <c r="I25" t="inlineStr"/>
-      <c r="J25" s="2" t="n">
+      <c r="J25" s="1" t="n">
         <v>46111</v>
       </c>
       <c r="K25" t="b">
@@ -1607,7 +1595,7 @@
         <v>-105</v>
       </c>
       <c r="I26" t="inlineStr"/>
-      <c r="J26" s="2" t="n">
+      <c r="J26" s="1" t="n">
         <v>46161</v>
       </c>
       <c r="K26" t="b">
@@ -1652,7 +1640,7 @@
         <v>-79.8</v>
       </c>
       <c r="I27" t="inlineStr"/>
-      <c r="J27" s="2" t="n">
+      <c r="J27" s="1" t="n">
         <v>43340</v>
       </c>
       <c r="K27" t="b">
@@ -1697,7 +1685,7 @@
         <v>-12.3</v>
       </c>
       <c r="I28" t="inlineStr"/>
-      <c r="J28" s="2" t="n">
+      <c r="J28" s="1" t="n">
         <v>46048</v>
       </c>
       <c r="K28" t="b">
@@ -1742,7 +1730,7 @@
         <v>0</v>
       </c>
       <c r="I29" t="inlineStr"/>
-      <c r="J29" s="2" t="n">
+      <c r="J29" s="1" t="n">
         <v>46211</v>
       </c>
       <c r="K29" t="b">
@@ -1787,7 +1775,7 @@
         <v>3.6</v>
       </c>
       <c r="I30" t="inlineStr"/>
-      <c r="J30" s="2" t="n">
+      <c r="J30" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="K30" t="b">
@@ -1832,7 +1820,7 @@
         <v>6.2</v>
       </c>
       <c r="I31" t="inlineStr"/>
-      <c r="J31" s="2" t="n">
+      <c r="J31" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="K31" t="b">
@@ -1877,7 +1865,7 @@
         <v>7.5</v>
       </c>
       <c r="I32" t="inlineStr"/>
-      <c r="J32" s="2" t="n">
+      <c r="J32" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="K32" t="b">
@@ -1922,7 +1910,7 @@
         <v>10.7</v>
       </c>
       <c r="I33" t="inlineStr"/>
-      <c r="J33" s="2" t="n">
+      <c r="J33" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="K33" t="b">
@@ -1967,7 +1955,7 @@
         <v>20</v>
       </c>
       <c r="I34" t="inlineStr"/>
-      <c r="J34" s="2" t="n">
+      <c r="J34" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="K34" t="b">
@@ -2012,7 +2000,7 @@
         <v>30.8</v>
       </c>
       <c r="I35" t="inlineStr"/>
-      <c r="J35" s="2" t="n">
+      <c r="J35" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="K35" t="b">
@@ -2057,7 +2045,7 @@
         <v>37.1</v>
       </c>
       <c r="I36" t="inlineStr"/>
-      <c r="J36" s="2" t="n">
+      <c r="J36" s="1" t="n">
         <v>46256</v>
       </c>
       <c r="K36" t="b">
@@ -2102,7 +2090,7 @@
         <v>42.8</v>
       </c>
       <c r="I37" t="inlineStr"/>
-      <c r="J37" s="2" t="n">
+      <c r="J37" s="1" t="n">
         <v>46276</v>
       </c>
       <c r="K37" t="b">
@@ -2147,7 +2135,7 @@
         <v>45.2</v>
       </c>
       <c r="I38" t="inlineStr"/>
-      <c r="J38" s="2" t="n">
+      <c r="J38" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="K38" t="b">
@@ -2192,7 +2180,7 @@
         <v>46</v>
       </c>
       <c r="I39" t="inlineStr"/>
-      <c r="J39" s="2" t="n">
+      <c r="J39" s="1" t="n">
         <v>46251</v>
       </c>
       <c r="K39" t="b">
@@ -2237,7 +2225,7 @@
         <v>47.5</v>
       </c>
       <c r="I40" t="inlineStr"/>
-      <c r="J40" s="2" t="n">
+      <c r="J40" s="1" t="n">
         <v>46456</v>
       </c>
       <c r="K40" t="b">
@@ -2282,7 +2270,7 @@
         <v>57.2</v>
       </c>
       <c r="I41" t="inlineStr"/>
-      <c r="J41" s="2" t="n">
+      <c r="J41" s="1" t="n">
         <v>46246</v>
       </c>
       <c r="K41" t="b">
@@ -2327,7 +2315,7 @@
         <v>59.6</v>
       </c>
       <c r="I42" t="inlineStr"/>
-      <c r="J42" s="2" t="n">
+      <c r="J42" s="1" t="n">
         <v>46487</v>
       </c>
       <c r="K42" t="b">
@@ -2372,7 +2360,7 @@
         <v>75.40000000000001</v>
       </c>
       <c r="I43" t="inlineStr"/>
-      <c r="J43" s="2" t="n">
+      <c r="J43" s="1" t="n">
         <v>46283</v>
       </c>
       <c r="K43" t="b">
@@ -2417,7 +2405,7 @@
         <v>76.8</v>
       </c>
       <c r="I44" t="inlineStr"/>
-      <c r="J44" s="2" t="n">
+      <c r="J44" s="1" t="n">
         <v>46285</v>
       </c>
       <c r="K44" t="b">
@@ -2462,7 +2450,7 @@
         <v>83.2</v>
       </c>
       <c r="I45" t="inlineStr"/>
-      <c r="J45" s="2" t="n">
+      <c r="J45" s="1" t="n">
         <v>46547</v>
       </c>
       <c r="K45" t="b">
@@ -2507,7 +2495,7 @@
         <v>84.5</v>
       </c>
       <c r="I46" t="inlineStr"/>
-      <c r="J46" s="2" t="n">
+      <c r="J46" s="1" t="n">
         <v>46240</v>
       </c>
       <c r="K46" t="b">
@@ -2552,7 +2540,7 @@
         <v>85.8</v>
       </c>
       <c r="I47" t="inlineStr"/>
-      <c r="J47" s="2" t="n">
+      <c r="J47" s="1" t="n">
         <v>46266</v>
       </c>
       <c r="K47" t="b">
@@ -2597,7 +2585,7 @@
         <v>86.5</v>
       </c>
       <c r="I48" t="inlineStr"/>
-      <c r="J48" s="2" t="n">
+      <c r="J48" s="1" t="n">
         <v>46241</v>
       </c>
       <c r="K48" t="b">
@@ -2642,7 +2630,7 @@
         <v>91.7</v>
       </c>
       <c r="I49" t="inlineStr"/>
-      <c r="J49" s="2" t="n">
+      <c r="J49" s="1" t="n">
         <v>46243</v>
       </c>
       <c r="K49" t="b">
@@ -2687,7 +2675,7 @@
         <v>91.7</v>
       </c>
       <c r="I50" t="inlineStr"/>
-      <c r="J50" s="2" t="n">
+      <c r="J50" s="1" t="n">
         <v>46243</v>
       </c>
       <c r="K50" t="b">
@@ -2732,7 +2720,7 @@
         <v>91.7</v>
       </c>
       <c r="I51" t="inlineStr"/>
-      <c r="J51" s="2" t="n">
+      <c r="J51" s="1" t="n">
         <v>46250</v>
       </c>
       <c r="K51" t="b">
@@ -2777,7 +2765,7 @@
         <v>98.90000000000001</v>
       </c>
       <c r="I52" t="inlineStr"/>
-      <c r="J52" s="2" t="n">
+      <c r="J52" s="1" t="n">
         <v>46253</v>
       </c>
       <c r="K52" t="b">
@@ -2822,7 +2810,7 @@
         <v>105.5</v>
       </c>
       <c r="I53" t="inlineStr"/>
-      <c r="J53" s="2" t="n">
+      <c r="J53" s="1" t="n">
         <v>46280</v>
       </c>
       <c r="K53" t="b">
@@ -2867,7 +2855,7 @@
         <v>105.6</v>
       </c>
       <c r="I54" t="inlineStr"/>
-      <c r="J54" s="2" t="n">
+      <c r="J54" s="1" t="n">
         <v>46361</v>
       </c>
       <c r="K54" t="b">
@@ -2912,7 +2900,7 @@
         <v>105.7</v>
       </c>
       <c r="I55" t="inlineStr"/>
-      <c r="J55" s="2" t="n">
+      <c r="J55" s="1" t="n">
         <v>46362</v>
       </c>
       <c r="K55" t="b">
@@ -2957,7 +2945,7 @@
         <v>110.7</v>
       </c>
       <c r="I56" t="inlineStr"/>
-      <c r="J56" s="2" t="n">
+      <c r="J56" s="1" t="n">
         <v>46275</v>
       </c>
       <c r="K56" t="b">
@@ -3002,7 +2990,7 @@
         <v>113.2</v>
       </c>
       <c r="I57" t="inlineStr"/>
-      <c r="J57" s="2" t="n">
+      <c r="J57" s="1" t="n">
         <v>46377</v>
       </c>
       <c r="K57" t="b">
@@ -3047,7 +3035,7 @@
         <v>128.8</v>
       </c>
       <c r="I58" t="inlineStr"/>
-      <c r="J58" s="2" t="n">
+      <c r="J58" s="1" t="n">
         <v>46434</v>
       </c>
       <c r="K58" t="b">
@@ -3092,7 +3080,7 @@
         <v>128.8</v>
       </c>
       <c r="I59" t="inlineStr"/>
-      <c r="J59" s="2" t="n">
+      <c r="J59" s="1" t="n">
         <v>46434</v>
       </c>
       <c r="K59" t="b">
@@ -3137,7 +3125,7 @@
         <v>128.8</v>
       </c>
       <c r="I60" t="inlineStr"/>
-      <c r="J60" s="2" t="n">
+      <c r="J60" s="1" t="n">
         <v>46434</v>
       </c>
       <c r="K60" t="b">
@@ -3182,7 +3170,7 @@
         <v>128.8</v>
       </c>
       <c r="I61" t="inlineStr"/>
-      <c r="J61" s="2" t="n">
+      <c r="J61" s="1" t="n">
         <v>46434</v>
       </c>
       <c r="K61" t="b">
@@ -3227,7 +3215,7 @@
         <v>128.8</v>
       </c>
       <c r="I62" t="inlineStr"/>
-      <c r="J62" s="2" t="n">
+      <c r="J62" s="1" t="n">
         <v>46434</v>
       </c>
       <c r="K62" t="b">
@@ -3272,7 +3260,7 @@
         <v>135</v>
       </c>
       <c r="I63" t="inlineStr"/>
-      <c r="J63" s="2" t="n">
+      <c r="J63" s="1" t="n">
         <v>46280</v>
       </c>
       <c r="K63" t="b">
@@ -3317,7 +3305,7 @@
         <v>150.6</v>
       </c>
       <c r="I64" t="inlineStr"/>
-      <c r="J64" s="2" t="n">
+      <c r="J64" s="1" t="n">
         <v>46271</v>
       </c>
       <c r="K64" t="b">
@@ -3362,7 +3350,7 @@
         <v>174.2</v>
       </c>
       <c r="I65" t="inlineStr"/>
-      <c r="J65" s="2" t="n">
+      <c r="J65" s="1" t="n">
         <v>46363</v>
       </c>
       <c r="K65" t="b">
@@ -3407,7 +3395,7 @@
         <v>176.6</v>
       </c>
       <c r="I66" t="inlineStr"/>
-      <c r="J66" s="2" t="n">
+      <c r="J66" s="1" t="n">
         <v>46334</v>
       </c>
       <c r="K66" t="b">
@@ -3452,7 +3440,7 @@
         <v>177.4</v>
       </c>
       <c r="I67" t="inlineStr"/>
-      <c r="J67" s="2" t="n">
+      <c r="J67" s="1" t="n">
         <v>46407</v>
       </c>
       <c r="K67" t="b">
@@ -3497,7 +3485,7 @@
         <v>183.9</v>
       </c>
       <c r="I68" t="inlineStr"/>
-      <c r="J68" s="2" t="n">
+      <c r="J68" s="1" t="n">
         <v>46341</v>
       </c>
       <c r="K68" t="b">
@@ -3542,7 +3530,7 @@
         <v>191.7</v>
       </c>
       <c r="I69" t="inlineStr"/>
-      <c r="J69" s="2" t="n">
+      <c r="J69" s="1" t="n">
         <v>46300</v>
       </c>
       <c r="K69" t="b">
@@ -3587,7 +3575,7 @@
         <v>200</v>
       </c>
       <c r="I70" t="inlineStr"/>
-      <c r="J70" s="2" t="n">
+      <c r="J70" s="1" t="n">
         <v>46336</v>
       </c>
       <c r="K70" t="b">
@@ -3632,7 +3620,7 @@
         <v>201.1</v>
       </c>
       <c r="I71" t="inlineStr"/>
-      <c r="J71" s="2" t="n">
+      <c r="J71" s="1" t="n">
         <v>46319</v>
       </c>
       <c r="K71" t="b">
@@ -3677,7 +3665,7 @@
         <v>206.5</v>
       </c>
       <c r="I72" t="inlineStr"/>
-      <c r="J72" s="2" t="n">
+      <c r="J72" s="1" t="n">
         <v>46308</v>
       </c>
       <c r="K72" t="b">
@@ -3722,7 +3710,7 @@
         <v>207.5</v>
       </c>
       <c r="I73" t="inlineStr"/>
-      <c r="J73" s="2" t="n">
+      <c r="J73" s="1" t="n">
         <v>46390</v>
       </c>
       <c r="K73" t="b">
@@ -3767,7 +3755,7 @@
         <v>247</v>
       </c>
       <c r="I74" t="inlineStr"/>
-      <c r="J74" s="2" t="n">
+      <c r="J74" s="1" t="n">
         <v>46443</v>
       </c>
       <c r="K74" t="b">
@@ -3812,7 +3800,7 @@
         <v>285.3</v>
       </c>
       <c r="I75" t="inlineStr"/>
-      <c r="J75" s="2" t="n">
+      <c r="J75" s="1" t="n">
         <v>46304</v>
       </c>
       <c r="K75" t="b">
@@ -3857,7 +3845,7 @@
         <v>290.8</v>
       </c>
       <c r="I76" t="inlineStr"/>
-      <c r="J76" s="2" t="n">
+      <c r="J76" s="1" t="n">
         <v>46362</v>
       </c>
       <c r="K76" t="b">
@@ -3902,7 +3890,7 @@
         <v>295.2</v>
       </c>
       <c r="I77" t="inlineStr"/>
-      <c r="J77" s="2" t="n">
+      <c r="J77" s="1" t="n">
         <v>46463</v>
       </c>
       <c r="K77" t="b">
@@ -3947,7 +3935,7 @@
         <v>300.2</v>
       </c>
       <c r="I78" t="inlineStr"/>
-      <c r="J78" s="2" t="n">
+      <c r="J78" s="1" t="n">
         <v>46466</v>
       </c>
       <c r="K78" t="b">
@@ -3996,7 +3984,7 @@
           <t>-317m</t>
         </is>
       </c>
-      <c r="J79" s="2" t="n">
+      <c r="J79" s="1" t="n">
         <v>36557</v>
       </c>
       <c r="K79" t="b">
@@ -4045,7 +4033,7 @@
           <t>-164m</t>
         </is>
       </c>
-      <c r="J80" s="2" t="n">
+      <c r="J80" s="1" t="n">
         <v>41275</v>
       </c>
       <c r="K80" t="b">
@@ -4094,7 +4082,7 @@
           <t>-27m</t>
         </is>
       </c>
-      <c r="J81" s="2" t="n">
+      <c r="J81" s="1" t="n">
         <v>45380</v>
       </c>
       <c r="K81" t="b">
@@ -4143,7 +4131,7 @@
           <t>-25m</t>
         </is>
       </c>
-      <c r="J82" s="2" t="n">
+      <c r="J82" s="1" t="n">
         <v>45421</v>
       </c>
       <c r="K82" t="b">
@@ -4192,7 +4180,7 @@
           <t>-25m</t>
         </is>
       </c>
-      <c r="J83" s="2" t="n">
+      <c r="J83" s="1" t="n">
         <v>45428</v>
       </c>
       <c r="K83" t="b">
@@ -4241,7 +4229,7 @@
           <t>-23m</t>
         </is>
       </c>
-      <c r="J84" s="2" t="n">
+      <c r="J84" s="1" t="n">
         <v>45490</v>
       </c>
       <c r="K84" t="b">
@@ -4290,7 +4278,7 @@
           <t>-21m</t>
         </is>
       </c>
-      <c r="J85" s="2" t="n">
+      <c r="J85" s="1" t="n">
         <v>45566</v>
       </c>
       <c r="K85" t="b">
@@ -4339,7 +4327,7 @@
           <t>-7m</t>
         </is>
       </c>
-      <c r="J86" s="2" t="n">
+      <c r="J86" s="1" t="n">
         <v>45986</v>
       </c>
       <c r="K86" t="b">
@@ -4388,7 +4376,7 @@
           <t>-3m</t>
         </is>
       </c>
-      <c r="J87" s="2" t="n">
+      <c r="J87" s="1" t="n">
         <v>46106</v>
       </c>
       <c r="K87" t="b">
@@ -4437,7 +4425,7 @@
           <t>-2m</t>
         </is>
       </c>
-      <c r="J88" s="2" t="n">
+      <c r="J88" s="1" t="n">
         <v>46142</v>
       </c>
       <c r="K88" t="b">
@@ -4486,7 +4474,7 @@
           <t>2m</t>
         </is>
       </c>
-      <c r="J89" s="2" t="n">
+      <c r="J89" s="1" t="n">
         <v>46274</v>
       </c>
       <c r="K89" t="b">
@@ -4535,7 +4523,7 @@
           <t>2m</t>
         </is>
       </c>
-      <c r="J90" s="2" t="n">
+      <c r="J90" s="1" t="n">
         <v>46276</v>
       </c>
       <c r="K90" t="b">
@@ -4584,7 +4572,7 @@
           <t>2m</t>
         </is>
       </c>
-      <c r="J91" s="2" t="n">
+      <c r="J91" s="1" t="n">
         <v>46284</v>
       </c>
       <c r="K91" t="b">
@@ -4633,7 +4621,7 @@
           <t>3m</t>
         </is>
       </c>
-      <c r="J92" s="2" t="n">
+      <c r="J92" s="1" t="n">
         <v>46317</v>
       </c>
       <c r="K92" t="b">
@@ -4682,7 +4670,7 @@
           <t>3m</t>
         </is>
       </c>
-      <c r="J93" s="2" t="n">
+      <c r="J93" s="1" t="n">
         <v>46319</v>
       </c>
       <c r="K93" t="b">
@@ -4731,7 +4719,7 @@
           <t>4m</t>
         </is>
       </c>
-      <c r="J94" s="2" t="n">
+      <c r="J94" s="1" t="n">
         <v>46333</v>
       </c>
       <c r="K94" t="b">
@@ -4780,7 +4768,7 @@
           <t>4m</t>
         </is>
       </c>
-      <c r="J95" s="2" t="n">
+      <c r="J95" s="1" t="n">
         <v>46338</v>
       </c>
       <c r="K95" t="b">
@@ -4829,7 +4817,7 @@
           <t>4m</t>
         </is>
       </c>
-      <c r="J96" s="2" t="n">
+      <c r="J96" s="1" t="n">
         <v>46338</v>
       </c>
       <c r="K96" t="b">
@@ -4878,7 +4866,7 @@
           <t>4m</t>
         </is>
       </c>
-      <c r="J97" s="2" t="n">
+      <c r="J97" s="1" t="n">
         <v>46341</v>
       </c>
       <c r="K97" t="b">
@@ -4927,7 +4915,7 @@
           <t>4m</t>
         </is>
       </c>
-      <c r="J98" s="2" t="n">
+      <c r="J98" s="1" t="n">
         <v>46344</v>
       </c>
       <c r="K98" t="b">
@@ -4976,7 +4964,7 @@
           <t>4m</t>
         </is>
       </c>
-      <c r="J99" s="2" t="n">
+      <c r="J99" s="1" t="n">
         <v>46354</v>
       </c>
       <c r="K99" t="b">
@@ -5025,7 +5013,7 @@
           <t>4m</t>
         </is>
       </c>
-      <c r="J100" s="2" t="n">
+      <c r="J100" s="1" t="n">
         <v>46360</v>
       </c>
       <c r="K100" t="b">
@@ -5074,7 +5062,7 @@
           <t>4m</t>
         </is>
       </c>
-      <c r="J101" s="2" t="n">
+      <c r="J101" s="1" t="n">
         <v>46360</v>
       </c>
       <c r="K101" t="b">
@@ -5123,7 +5111,7 @@
           <t>5m</t>
         </is>
       </c>
-      <c r="J102" s="2" t="n">
+      <c r="J102" s="1" t="n">
         <v>46366</v>
       </c>
       <c r="K102" t="b">
@@ -5172,7 +5160,7 @@
           <t>5m</t>
         </is>
       </c>
-      <c r="J103" s="2" t="n">
+      <c r="J103" s="1" t="n">
         <v>46375</v>
       </c>
       <c r="K103" t="b">
@@ -5221,7 +5209,7 @@
           <t>5m</t>
         </is>
       </c>
-      <c r="J104" s="2" t="n">
+      <c r="J104" s="1" t="n">
         <v>46388</v>
       </c>
       <c r="K104" t="b">
@@ -5270,7 +5258,7 @@
           <t>6m</t>
         </is>
       </c>
-      <c r="J105" s="2" t="n">
+      <c r="J105" s="1" t="n">
         <v>46401</v>
       </c>
       <c r="K105" t="b">
@@ -5319,7 +5307,7 @@
           <t>6m</t>
         </is>
       </c>
-      <c r="J106" s="2" t="n">
+      <c r="J106" s="1" t="n">
         <v>46401</v>
       </c>
       <c r="K106" t="b">
@@ -5368,7 +5356,7 @@
           <t>6m</t>
         </is>
       </c>
-      <c r="J107" s="2" t="n">
+      <c r="J107" s="1" t="n">
         <v>46401</v>
       </c>
       <c r="K107" t="b">
@@ -5417,7 +5405,7 @@
           <t>6m</t>
         </is>
       </c>
-      <c r="J108" s="2" t="n">
+      <c r="J108" s="1" t="n">
         <v>46413</v>
       </c>
       <c r="K108" t="b">
@@ -5466,7 +5454,7 @@
           <t>7m</t>
         </is>
       </c>
-      <c r="J109" s="2" t="n">
+      <c r="J109" s="1" t="n">
         <v>46424</v>
       </c>
       <c r="K109" t="b">
@@ -5515,7 +5503,7 @@
           <t>7m</t>
         </is>
       </c>
-      <c r="J110" s="2" t="n">
+      <c r="J110" s="1" t="n">
         <v>46427</v>
       </c>
       <c r="K110" t="b">
@@ -5564,7 +5552,7 @@
           <t>7m</t>
         </is>
       </c>
-      <c r="J111" s="2" t="n">
+      <c r="J111" s="1" t="n">
         <v>46437</v>
       </c>
       <c r="K111" t="b">
@@ -5613,7 +5601,7 @@
           <t>7m</t>
         </is>
       </c>
-      <c r="J112" s="2" t="n">
+      <c r="J112" s="1" t="n">
         <v>46451</v>
       </c>
       <c r="K112" t="b">
@@ -5662,7 +5650,7 @@
           <t>8m</t>
         </is>
       </c>
-      <c r="J113" s="2" t="n">
+      <c r="J113" s="1" t="n">
         <v>46455</v>
       </c>
       <c r="K113" t="b">
@@ -5711,7 +5699,7 @@
           <t>8m</t>
         </is>
       </c>
-      <c r="J114" s="2" t="n">
+      <c r="J114" s="1" t="n">
         <v>46457</v>
       </c>
       <c r="K114" t="b">
@@ -5760,7 +5748,7 @@
           <t>8m</t>
         </is>
       </c>
-      <c r="J115" s="2" t="n">
+      <c r="J115" s="1" t="n">
         <v>46462</v>
       </c>
       <c r="K115" t="b">
@@ -5809,7 +5797,7 @@
           <t>8m</t>
         </is>
       </c>
-      <c r="J116" s="2" t="n">
+      <c r="J116" s="1" t="n">
         <v>46464</v>
       </c>
       <c r="K116" t="b">
@@ -5858,7 +5846,7 @@
           <t>8m</t>
         </is>
       </c>
-      <c r="J117" s="2" t="n">
+      <c r="J117" s="1" t="n">
         <v>46470</v>
       </c>
       <c r="K117" t="b">
@@ -5907,7 +5895,7 @@
           <t>9m</t>
         </is>
       </c>
-      <c r="J118" s="2" t="n">
+      <c r="J118" s="1" t="n">
         <v>46485</v>
       </c>
       <c r="K118" t="b">
@@ -5956,7 +5944,7 @@
           <t>9m</t>
         </is>
       </c>
-      <c r="J119" s="2" t="n">
+      <c r="J119" s="1" t="n">
         <v>46499</v>
       </c>
       <c r="K119" t="b">
@@ -6005,7 +5993,7 @@
           <t>9m</t>
         </is>
       </c>
-      <c r="J120" s="2" t="n">
+      <c r="J120" s="1" t="n">
         <v>46504</v>
       </c>
       <c r="K120" t="b">
@@ -6054,7 +6042,7 @@
           <t>9m</t>
         </is>
       </c>
-      <c r="J121" s="2" t="n">
+      <c r="J121" s="1" t="n">
         <v>46504</v>
       </c>
       <c r="K121" t="b">
@@ -6103,7 +6091,7 @@
           <t>9m</t>
         </is>
       </c>
-      <c r="J122" s="2" t="n">
+      <c r="J122" s="1" t="n">
         <v>46507</v>
       </c>
       <c r="K122" t="b">
@@ -6152,7 +6140,7 @@
           <t>9m</t>
         </is>
       </c>
-      <c r="J123" s="2" t="n">
+      <c r="J123" s="1" t="n">
         <v>46508</v>
       </c>
       <c r="K123" t="b">
@@ -6201,7 +6189,7 @@
           <t>9m</t>
         </is>
       </c>
-      <c r="J124" s="2" t="n">
+      <c r="J124" s="1" t="n">
         <v>46512</v>
       </c>
       <c r="K124" t="b">
@@ -6250,7 +6238,7 @@
           <t>9m</t>
         </is>
       </c>
-      <c r="J125" s="2" t="n">
+      <c r="J125" s="1" t="n">
         <v>46512</v>
       </c>
       <c r="K125" t="b">
@@ -6299,7 +6287,7 @@
           <t>10m</t>
         </is>
       </c>
-      <c r="J126" s="2" t="n">
+      <c r="J126" s="1" t="n">
         <v>46528</v>
       </c>
       <c r="K126" t="b">
@@ -6348,7 +6336,7 @@
           <t>10m</t>
         </is>
       </c>
-      <c r="J127" s="2" t="n">
+      <c r="J127" s="1" t="n">
         <v>46529</v>
       </c>
       <c r="K127" t="b">
@@ -6397,7 +6385,7 @@
           <t>10m</t>
         </is>
       </c>
-      <c r="J128" s="2" t="n">
+      <c r="J128" s="1" t="n">
         <v>46537</v>
       </c>
       <c r="K128" t="b">
@@ -6446,7 +6434,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J129" s="2" t="n">
+      <c r="J129" s="1" t="n">
         <v>46546</v>
       </c>
       <c r="K129" t="b">
@@ -6495,7 +6483,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J130" s="2" t="n">
+      <c r="J130" s="1" t="n">
         <v>46547</v>
       </c>
       <c r="K130" t="b">
@@ -6544,7 +6532,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J131" s="2" t="n">
+      <c r="J131" s="1" t="n">
         <v>46547</v>
       </c>
       <c r="K131" t="b">
@@ -6593,7 +6581,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J132" s="2" t="n">
+      <c r="J132" s="1" t="n">
         <v>46547</v>
       </c>
       <c r="K132" t="b">
@@ -6642,7 +6630,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J133" s="2" t="n">
+      <c r="J133" s="1" t="n">
         <v>46551</v>
       </c>
       <c r="K133" t="b">
@@ -6691,7 +6679,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J134" s="2" t="n">
+      <c r="J134" s="1" t="n">
         <v>46560</v>
       </c>
       <c r="K134" t="b">
@@ -6740,7 +6728,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J135" s="2" t="n">
+      <c r="J135" s="1" t="n">
         <v>46564</v>
       </c>
       <c r="K135" t="b">
@@ -6789,7 +6777,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J136" s="2" t="n">
+      <c r="J136" s="1" t="n">
         <v>46567</v>
       </c>
       <c r="K136" t="b">
@@ -6838,7 +6826,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J137" s="2" t="n">
+      <c r="J137" s="1" t="n">
         <v>46568</v>
       </c>
       <c r="K137" t="b">
@@ -6887,7 +6875,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J138" s="2" t="n">
+      <c r="J138" s="1" t="n">
         <v>46571</v>
       </c>
       <c r="K138" t="b">
@@ -6936,7 +6924,7 @@
           <t>-14d</t>
         </is>
       </c>
-      <c r="J139" s="2" t="n">
+      <c r="J139" s="1" t="n">
         <v>46197</v>
       </c>
       <c r="K139" t="b">
@@ -6985,7 +6973,7 @@
           <t>1d</t>
         </is>
       </c>
-      <c r="J140" s="2" t="n">
+      <c r="J140" s="1" t="n">
         <v>46212</v>
       </c>
       <c r="K140" t="b">
@@ -7034,7 +7022,7 @@
           <t>14d</t>
         </is>
       </c>
-      <c r="J141" s="2" t="n">
+      <c r="J141" s="1" t="n">
         <v>46225</v>
       </c>
       <c r="K141" t="b">
@@ -7083,7 +7071,7 @@
           <t>23d</t>
         </is>
       </c>
-      <c r="J142" s="2" t="n">
+      <c r="J142" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="K142" t="b">
@@ -7132,7 +7120,7 @@
           <t>24d</t>
         </is>
       </c>
-      <c r="J143" s="2" t="n">
+      <c r="J143" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="K143" t="b">
@@ -7181,7 +7169,7 @@
           <t>1me23d</t>
         </is>
       </c>
-      <c r="J144" s="2" t="n">
+      <c r="J144" s="1" t="n">
         <v>46263</v>
       </c>
       <c r="K144" t="b">
@@ -7230,7 +7218,7 @@
           <t>1me25d</t>
         </is>
       </c>
-      <c r="J145" s="2" t="n">
+      <c r="J145" s="1" t="n">
         <v>46266</v>
       </c>
       <c r="K145" t="b">
@@ -7275,7 +7263,7 @@
         <v>-1476</v>
       </c>
       <c r="I146" t="inlineStr"/>
-      <c r="J146" s="2" t="n">
+      <c r="J146" s="1" t="n">
         <v>43773</v>
       </c>
       <c r="K146" t="b">
@@ -7320,7 +7308,7 @@
         <v>-1469</v>
       </c>
       <c r="I147" t="inlineStr"/>
-      <c r="J147" s="2" t="n">
+      <c r="J147" s="1" t="n">
         <v>43773</v>
       </c>
       <c r="K147" t="b">
@@ -7365,7 +7353,7 @@
         <v>-1121</v>
       </c>
       <c r="I148" t="inlineStr"/>
-      <c r="J148" s="2" t="n">
+      <c r="J148" s="1" t="n">
         <v>45295</v>
       </c>
       <c r="K148" t="b">
@@ -7410,7 +7398,7 @@
         <v>-1018</v>
       </c>
       <c r="I149" t="inlineStr"/>
-      <c r="J149" s="2" t="n">
+      <c r="J149" s="1" t="n">
         <v>45617</v>
       </c>
       <c r="K149" t="b">
@@ -7455,7 +7443,7 @@
         <v>-950</v>
       </c>
       <c r="I150" t="inlineStr"/>
-      <c r="J150" s="2" t="n">
+      <c r="J150" s="1" t="n">
         <v>45677</v>
       </c>
       <c r="K150" t="b">
@@ -7500,7 +7488,7 @@
         <v>-943</v>
       </c>
       <c r="I151" t="inlineStr"/>
-      <c r="J151" s="2" t="n">
+      <c r="J151" s="1" t="n">
         <v>44944</v>
       </c>
       <c r="K151" t="b">
@@ -7545,7 +7533,7 @@
         <v>-252</v>
       </c>
       <c r="I152" t="inlineStr"/>
-      <c r="J152" s="2" t="n">
+      <c r="J152" s="1" t="n">
         <v>46092</v>
       </c>
       <c r="K152" t="b">
@@ -7590,7 +7578,7 @@
         <v>-196</v>
       </c>
       <c r="I153" t="inlineStr"/>
-      <c r="J153" s="2" t="n">
+      <c r="J153" s="1" t="n">
         <v>45988</v>
       </c>
       <c r="K153" t="b">
@@ -7635,7 +7623,7 @@
         <v>-196</v>
       </c>
       <c r="I154" t="inlineStr"/>
-      <c r="J154" s="2" t="n">
+      <c r="J154" s="1" t="n">
         <v>45988</v>
       </c>
       <c r="K154" t="b">
@@ -7680,7 +7668,7 @@
         <v>-47</v>
       </c>
       <c r="I155" t="inlineStr"/>
-      <c r="J155" s="2" t="n">
+      <c r="J155" s="1" t="n">
         <v>46176</v>
       </c>
       <c r="K155" t="b">
@@ -7725,7 +7713,7 @@
         <v>-47</v>
       </c>
       <c r="I156" t="inlineStr"/>
-      <c r="J156" s="2" t="n">
+      <c r="J156" s="1" t="n">
         <v>46176</v>
       </c>
       <c r="K156" t="b">
@@ -7770,7 +7758,7 @@
         <v>-33</v>
       </c>
       <c r="I157" t="inlineStr"/>
-      <c r="J157" s="2" t="n">
+      <c r="J157" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="K157" t="b">
@@ -7815,7 +7803,7 @@
         <v>-33</v>
       </c>
       <c r="I158" t="inlineStr"/>
-      <c r="J158" s="2" t="n">
+      <c r="J158" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="K158" t="b">
@@ -7860,7 +7848,7 @@
         <v>-6</v>
       </c>
       <c r="I159" t="inlineStr"/>
-      <c r="J159" s="2" t="n">
+      <c r="J159" s="1" t="n">
         <v>45967</v>
       </c>
       <c r="K159" t="b">
@@ -7905,7 +7893,7 @@
         <v>43</v>
       </c>
       <c r="I160" t="inlineStr"/>
-      <c r="J160" s="2" t="n">
+      <c r="J160" s="1" t="n">
         <v>46440</v>
       </c>
       <c r="K160" t="b">
@@ -7950,7 +7938,7 @@
         <v>43</v>
       </c>
       <c r="I161" t="inlineStr"/>
-      <c r="J161" s="2" t="n">
+      <c r="J161" s="1" t="n">
         <v>46440</v>
       </c>
       <c r="K161" t="b">
@@ -7995,7 +7983,7 @@
         <v>73</v>
       </c>
       <c r="I162" t="inlineStr"/>
-      <c r="J162" s="2" t="n">
+      <c r="J162" s="1" t="n">
         <v>46264</v>
       </c>
       <c r="K162" t="b">
@@ -8040,7 +8028,7 @@
         <v>73</v>
       </c>
       <c r="I163" t="inlineStr"/>
-      <c r="J163" s="2" t="n">
+      <c r="J163" s="1" t="n">
         <v>46264</v>
       </c>
       <c r="K163" t="b">
@@ -8085,7 +8073,7 @@
         <v>102</v>
       </c>
       <c r="I164" t="inlineStr"/>
-      <c r="J164" s="2" t="n">
+      <c r="J164" s="1" t="n">
         <v>46463</v>
       </c>
       <c r="K164" t="b">
@@ -8130,7 +8118,7 @@
         <v>118</v>
       </c>
       <c r="I165" t="inlineStr"/>
-      <c r="J165" s="2" t="n">
+      <c r="J165" s="1" t="n">
         <v>46337</v>
       </c>
       <c r="K165" t="b">
@@ -8175,7 +8163,7 @@
         <v>146</v>
       </c>
       <c r="I166" t="inlineStr"/>
-      <c r="J166" s="2" t="n">
+      <c r="J166" s="1" t="n">
         <v>46451</v>
       </c>
       <c r="K166" t="b">
@@ -8220,7 +8208,7 @@
         <v>152</v>
       </c>
       <c r="I167" t="inlineStr"/>
-      <c r="J167" s="2" t="n">
+      <c r="J167" s="1" t="n">
         <v>46245</v>
       </c>
       <c r="K167" t="b">
@@ -8265,7 +8253,7 @@
         <v>152</v>
       </c>
       <c r="I168" t="inlineStr"/>
-      <c r="J168" s="2" t="n">
+      <c r="J168" s="1" t="n">
         <v>46245</v>
       </c>
       <c r="K168" t="b">
@@ -8310,7 +8298,7 @@
         <v>163</v>
       </c>
       <c r="I169" t="inlineStr"/>
-      <c r="J169" s="2" t="n">
+      <c r="J169" s="1" t="n">
         <v>46324</v>
       </c>
       <c r="K169" t="b">
@@ -8355,7 +8343,7 @@
         <v>163</v>
       </c>
       <c r="I170" t="inlineStr"/>
-      <c r="J170" s="2" t="n">
+      <c r="J170" s="1" t="n">
         <v>46324</v>
       </c>
       <c r="K170" t="b">
@@ -8400,7 +8388,7 @@
         <v>164</v>
       </c>
       <c r="I171" t="inlineStr"/>
-      <c r="J171" s="2" t="n">
+      <c r="J171" s="1" t="n">
         <v>46426</v>
       </c>
       <c r="K171" t="b">
@@ -8445,7 +8433,7 @@
         <v>175</v>
       </c>
       <c r="I172" t="inlineStr"/>
-      <c r="J172" s="2" t="n">
+      <c r="J172" s="1" t="n">
         <v>46383</v>
       </c>
       <c r="K172" t="b">
@@ -8490,7 +8478,7 @@
         <v>186</v>
       </c>
       <c r="I173" t="inlineStr"/>
-      <c r="J173" s="2" t="n">
+      <c r="J173" s="1" t="n">
         <v>46392</v>
       </c>
       <c r="K173" t="b">
@@ -8535,7 +8523,7 @@
         <v>205</v>
       </c>
       <c r="I174" t="inlineStr"/>
-      <c r="J174" s="2" t="n">
+      <c r="J174" s="1" t="n">
         <v>46390</v>
       </c>
       <c r="K174" t="b">
@@ -8580,7 +8568,7 @@
         <v>207</v>
       </c>
       <c r="I175" t="inlineStr"/>
-      <c r="J175" s="2" t="n">
+      <c r="J175" s="1" t="n">
         <v>46392</v>
       </c>
       <c r="K175" t="b">
@@ -8625,7 +8613,7 @@
         <v>218</v>
       </c>
       <c r="I176" t="inlineStr"/>
-      <c r="J176" s="2" t="n">
+      <c r="J176" s="1" t="n">
         <v>46506</v>
       </c>
       <c r="K176" t="b">
@@ -8670,7 +8658,7 @@
         <v>246</v>
       </c>
       <c r="I177" t="inlineStr"/>
-      <c r="J177" s="2" t="n">
+      <c r="J177" s="1" t="n">
         <v>46478</v>
       </c>
       <c r="K177" t="b">
@@ -8715,7 +8703,7 @@
         <v>248</v>
       </c>
       <c r="I178" t="inlineStr"/>
-      <c r="J178" s="2" t="n">
+      <c r="J178" s="1" t="n">
         <v>46500</v>
       </c>
       <c r="K178" t="b">
@@ -8760,7 +8748,7 @@
         <v>276</v>
       </c>
       <c r="I179" t="inlineStr"/>
-      <c r="J179" s="2" t="n">
+      <c r="J179" s="1" t="n">
         <v>46430</v>
       </c>
       <c r="K179" t="b">
@@ -8805,7 +8793,7 @@
         <v>276</v>
       </c>
       <c r="I180" t="inlineStr"/>
-      <c r="J180" s="2" t="n">
+      <c r="J180" s="1" t="n">
         <v>46430</v>
       </c>
       <c r="K180" t="b">
@@ -8850,7 +8838,7 @@
         <v>290</v>
       </c>
       <c r="I181" t="inlineStr"/>
-      <c r="J181" s="2" t="n">
+      <c r="J181" s="1" t="n">
         <v>46467</v>
       </c>
       <c r="K181" t="b">
@@ -8895,7 +8883,7 @@
         <v>317</v>
       </c>
       <c r="I182" t="inlineStr"/>
-      <c r="J182" s="2" t="n">
+      <c r="J182" s="1" t="n">
         <v>46529</v>
       </c>
       <c r="K182" t="b">
@@ -8940,7 +8928,7 @@
         <v>420</v>
       </c>
       <c r="I183" t="inlineStr"/>
-      <c r="J183" s="2" t="n">
+      <c r="J183" s="1" t="n">
         <v>46566</v>
       </c>
       <c r="K183" t="b">
@@ -8985,7 +8973,7 @@
         <v>426</v>
       </c>
       <c r="I184" t="inlineStr"/>
-      <c r="J184" s="2" t="n">
+      <c r="J184" s="1" t="n">
         <v>46571</v>
       </c>
       <c r="K184" t="b">
@@ -9030,7 +9018,7 @@
         <v>721</v>
       </c>
       <c r="I185" t="inlineStr"/>
-      <c r="J185" s="2" t="n">
+      <c r="J185" s="1" t="n">
         <v>46325</v>
       </c>
       <c r="K185" t="b">
@@ -9075,7 +9063,7 @@
         <v>721</v>
       </c>
       <c r="I186" t="inlineStr"/>
-      <c r="J186" s="2" t="n">
+      <c r="J186" s="1" t="n">
         <v>46325</v>
       </c>
       <c r="K186" t="b">
@@ -9120,7 +9108,7 @@
         <v>850</v>
       </c>
       <c r="I187" t="inlineStr"/>
-      <c r="J187" s="2" t="n">
+      <c r="J187" s="1" t="n">
         <v>46345</v>
       </c>
       <c r="K187" t="b">
@@ -9165,7 +9153,7 @@
         <v>850</v>
       </c>
       <c r="I188" t="inlineStr"/>
-      <c r="J188" s="2" t="n">
+      <c r="J188" s="1" t="n">
         <v>46345</v>
       </c>
       <c r="K188" t="b">
@@ -9210,7 +9198,7 @@
         <v>1661</v>
       </c>
       <c r="I189" t="inlineStr"/>
-      <c r="J189" s="2" t="n">
+      <c r="J189" s="1" t="n">
         <v>46498</v>
       </c>
       <c r="K189" t="b">
@@ -9255,7 +9243,7 @@
         <v>1661</v>
       </c>
       <c r="I190" t="inlineStr"/>
-      <c r="J190" s="2" t="n">
+      <c r="J190" s="1" t="n">
         <v>46498</v>
       </c>
       <c r="K190" t="b">
@@ -9300,7 +9288,7 @@
         <v>488</v>
       </c>
       <c r="I191" t="inlineStr"/>
-      <c r="J191" s="2" t="n">
+      <c r="J191" s="1" t="n">
         <v>46190</v>
       </c>
       <c r="K191" t="b">
@@ -9345,7 +9333,7 @@
         <v>25565</v>
       </c>
       <c r="I192" t="inlineStr"/>
-      <c r="J192" s="2" t="n">
+      <c r="J192" s="1" t="n">
         <v>46190</v>
       </c>
       <c r="K192" t="b">
@@ -9390,7 +9378,7 @@
         <v>25567</v>
       </c>
       <c r="I193" t="inlineStr"/>
-      <c r="J193" s="2" t="n">
+      <c r="J193" s="1" t="n">
         <v>46190</v>
       </c>
       <c r="K193" t="b">
@@ -9435,7 +9423,7 @@
         <v>31293</v>
       </c>
       <c r="I194" t="inlineStr"/>
-      <c r="J194" s="2" t="n">
+      <c r="J194" s="1" t="n">
         <v>46190</v>
       </c>
       <c r="K194" t="b">

</xml_diff>

<commit_message>
Atualização automática: vencimentos_tmot (10/07/2026 16:00)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
@@ -20,13 +20,16 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +40,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,12 +48,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -421,57 +433,57 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>matricula</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>operador</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>pn</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>sn</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>nomenclatura</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>inspecao</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>tipo_vencimento</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>disponibilidade_valor</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>disponibilidade_texto</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>data_vencimento</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>vencido</t>
         </is>
@@ -515,7 +527,7 @@
         <v>-4402.8</v>
       </c>
       <c r="I2" t="inlineStr"/>
-      <c r="J2" s="1" t="n">
+      <c r="J2" s="2" t="n">
         <v>41388</v>
       </c>
       <c r="K2" t="b">
@@ -560,7 +572,7 @@
         <v>-4254.8</v>
       </c>
       <c r="I3" t="inlineStr"/>
-      <c r="J3" s="1" t="n">
+      <c r="J3" s="2" t="n">
         <v>39285</v>
       </c>
       <c r="K3" t="b">
@@ -605,7 +617,7 @@
         <v>-2354.2</v>
       </c>
       <c r="I4" t="inlineStr"/>
-      <c r="J4" s="1" t="n">
+      <c r="J4" s="2" t="n">
         <v>40669</v>
       </c>
       <c r="K4" t="b">
@@ -650,7 +662,7 @@
         <v>-896.8</v>
       </c>
       <c r="I5" t="inlineStr"/>
-      <c r="J5" s="1" t="n">
+      <c r="J5" s="2" t="n">
         <v>40669</v>
       </c>
       <c r="K5" t="b">
@@ -695,7 +707,7 @@
         <v>-854.1</v>
       </c>
       <c r="I6" t="inlineStr"/>
-      <c r="J6" s="1" t="n">
+      <c r="J6" s="2" t="n">
         <v>44884</v>
       </c>
       <c r="K6" t="b">
@@ -740,7 +752,7 @@
         <v>-413.2</v>
       </c>
       <c r="I7" t="inlineStr"/>
-      <c r="J7" s="1" t="n">
+      <c r="J7" s="2" t="n">
         <v>43855</v>
       </c>
       <c r="K7" t="b">
@@ -785,7 +797,7 @@
         <v>-391.8</v>
       </c>
       <c r="I8" t="inlineStr"/>
-      <c r="J8" s="1" t="n">
+      <c r="J8" s="2" t="n">
         <v>42769</v>
       </c>
       <c r="K8" t="b">
@@ -830,7 +842,7 @@
         <v>-371.5</v>
       </c>
       <c r="I9" t="inlineStr"/>
-      <c r="J9" s="1" t="n">
+      <c r="J9" s="2" t="n">
         <v>46014</v>
       </c>
       <c r="K9" t="b">
@@ -875,7 +887,7 @@
         <v>-368.8</v>
       </c>
       <c r="I10" t="inlineStr"/>
-      <c r="J10" s="1" t="n">
+      <c r="J10" s="2" t="n">
         <v>46014</v>
       </c>
       <c r="K10" t="b">
@@ -920,7 +932,7 @@
         <v>-359</v>
       </c>
       <c r="I11" t="inlineStr"/>
-      <c r="J11" s="1" t="n">
+      <c r="J11" s="2" t="n">
         <v>45804</v>
       </c>
       <c r="K11" t="b">
@@ -965,7 +977,7 @@
         <v>-359</v>
       </c>
       <c r="I12" t="inlineStr"/>
-      <c r="J12" s="1" t="n">
+      <c r="J12" s="2" t="n">
         <v>45804</v>
       </c>
       <c r="K12" t="b">
@@ -1010,7 +1022,7 @@
         <v>-351</v>
       </c>
       <c r="I13" t="inlineStr"/>
-      <c r="J13" s="1" t="n">
+      <c r="J13" s="2" t="n">
         <v>42821</v>
       </c>
       <c r="K13" t="b">
@@ -1055,7 +1067,7 @@
         <v>-351</v>
       </c>
       <c r="I14" t="inlineStr"/>
-      <c r="J14" s="1" t="n">
+      <c r="J14" s="2" t="n">
         <v>46014</v>
       </c>
       <c r="K14" t="b">
@@ -1100,7 +1112,7 @@
         <v>-351</v>
       </c>
       <c r="I15" t="inlineStr"/>
-      <c r="J15" s="1" t="n">
+      <c r="J15" s="2" t="n">
         <v>46014</v>
       </c>
       <c r="K15" t="b">
@@ -1145,7 +1157,7 @@
         <v>-351</v>
       </c>
       <c r="I16" t="inlineStr"/>
-      <c r="J16" s="1" t="n">
+      <c r="J16" s="2" t="n">
         <v>46014</v>
       </c>
       <c r="K16" t="b">
@@ -1190,7 +1202,7 @@
         <v>-345.8</v>
       </c>
       <c r="I17" t="inlineStr"/>
-      <c r="J17" s="1" t="n">
+      <c r="J17" s="2" t="n">
         <v>46017</v>
       </c>
       <c r="K17" t="b">
@@ -1235,7 +1247,7 @@
         <v>-345.8</v>
       </c>
       <c r="I18" t="inlineStr"/>
-      <c r="J18" s="1" t="n">
+      <c r="J18" s="2" t="n">
         <v>46017</v>
       </c>
       <c r="K18" t="b">
@@ -1280,7 +1292,7 @@
         <v>-264.2</v>
       </c>
       <c r="I19" t="inlineStr"/>
-      <c r="J19" s="1" t="n">
+      <c r="J19" s="2" t="n">
         <v>40979</v>
       </c>
       <c r="K19" t="b">
@@ -1325,7 +1337,7 @@
         <v>-206.4</v>
       </c>
       <c r="I20" t="inlineStr"/>
-      <c r="J20" s="1" t="n">
+      <c r="J20" s="2" t="n">
         <v>36669</v>
       </c>
       <c r="K20" t="b">
@@ -1370,7 +1382,7 @@
         <v>-131.6</v>
       </c>
       <c r="I21" t="inlineStr"/>
-      <c r="J21" s="1" t="n">
+      <c r="J21" s="2" t="n">
         <v>46111</v>
       </c>
       <c r="K21" t="b">
@@ -1415,7 +1427,7 @@
         <v>-131.6</v>
       </c>
       <c r="I22" t="inlineStr"/>
-      <c r="J22" s="1" t="n">
+      <c r="J22" s="2" t="n">
         <v>46111</v>
       </c>
       <c r="K22" t="b">
@@ -1460,7 +1472,7 @@
         <v>-131.6</v>
       </c>
       <c r="I23" t="inlineStr"/>
-      <c r="J23" s="1" t="n">
+      <c r="J23" s="2" t="n">
         <v>46111</v>
       </c>
       <c r="K23" t="b">
@@ -1505,7 +1517,7 @@
         <v>-131.6</v>
       </c>
       <c r="I24" t="inlineStr"/>
-      <c r="J24" s="1" t="n">
+      <c r="J24" s="2" t="n">
         <v>46111</v>
       </c>
       <c r="K24" t="b">
@@ -1550,7 +1562,7 @@
         <v>-131.6</v>
       </c>
       <c r="I25" t="inlineStr"/>
-      <c r="J25" s="1" t="n">
+      <c r="J25" s="2" t="n">
         <v>46111</v>
       </c>
       <c r="K25" t="b">
@@ -1595,7 +1607,7 @@
         <v>-105</v>
       </c>
       <c r="I26" t="inlineStr"/>
-      <c r="J26" s="1" t="n">
+      <c r="J26" s="2" t="n">
         <v>46161</v>
       </c>
       <c r="K26" t="b">
@@ -1640,7 +1652,7 @@
         <v>-79.8</v>
       </c>
       <c r="I27" t="inlineStr"/>
-      <c r="J27" s="1" t="n">
+      <c r="J27" s="2" t="n">
         <v>43340</v>
       </c>
       <c r="K27" t="b">
@@ -1685,7 +1697,7 @@
         <v>-12.3</v>
       </c>
       <c r="I28" t="inlineStr"/>
-      <c r="J28" s="1" t="n">
+      <c r="J28" s="2" t="n">
         <v>46048</v>
       </c>
       <c r="K28" t="b">
@@ -1730,7 +1742,7 @@
         <v>0</v>
       </c>
       <c r="I29" t="inlineStr"/>
-      <c r="J29" s="1" t="n">
+      <c r="J29" s="2" t="n">
         <v>46211</v>
       </c>
       <c r="K29" t="b">
@@ -1775,7 +1787,7 @@
         <v>3.6</v>
       </c>
       <c r="I30" t="inlineStr"/>
-      <c r="J30" s="1" t="n">
+      <c r="J30" s="2" t="n">
         <v>46234</v>
       </c>
       <c r="K30" t="b">
@@ -1820,7 +1832,7 @@
         <v>6.2</v>
       </c>
       <c r="I31" t="inlineStr"/>
-      <c r="J31" s="1" t="n">
+      <c r="J31" s="2" t="n">
         <v>46234</v>
       </c>
       <c r="K31" t="b">
@@ -1865,7 +1877,7 @@
         <v>7.5</v>
       </c>
       <c r="I32" t="inlineStr"/>
-      <c r="J32" s="1" t="n">
+      <c r="J32" s="2" t="n">
         <v>46234</v>
       </c>
       <c r="K32" t="b">
@@ -1910,7 +1922,7 @@
         <v>10.7</v>
       </c>
       <c r="I33" t="inlineStr"/>
-      <c r="J33" s="1" t="n">
+      <c r="J33" s="2" t="n">
         <v>46234</v>
       </c>
       <c r="K33" t="b">
@@ -1955,7 +1967,7 @@
         <v>20</v>
       </c>
       <c r="I34" t="inlineStr"/>
-      <c r="J34" s="1" t="n">
+      <c r="J34" s="2" t="n">
         <v>46234</v>
       </c>
       <c r="K34" t="b">
@@ -2000,7 +2012,7 @@
         <v>30.8</v>
       </c>
       <c r="I35" t="inlineStr"/>
-      <c r="J35" s="1" t="n">
+      <c r="J35" s="2" t="n">
         <v>46234</v>
       </c>
       <c r="K35" t="b">
@@ -2045,7 +2057,7 @@
         <v>37.1</v>
       </c>
       <c r="I36" t="inlineStr"/>
-      <c r="J36" s="1" t="n">
+      <c r="J36" s="2" t="n">
         <v>46256</v>
       </c>
       <c r="K36" t="b">
@@ -2090,7 +2102,7 @@
         <v>42.8</v>
       </c>
       <c r="I37" t="inlineStr"/>
-      <c r="J37" s="1" t="n">
+      <c r="J37" s="2" t="n">
         <v>46276</v>
       </c>
       <c r="K37" t="b">
@@ -2135,7 +2147,7 @@
         <v>45.2</v>
       </c>
       <c r="I38" t="inlineStr"/>
-      <c r="J38" s="1" t="n">
+      <c r="J38" s="2" t="n">
         <v>46234</v>
       </c>
       <c r="K38" t="b">
@@ -2180,7 +2192,7 @@
         <v>46</v>
       </c>
       <c r="I39" t="inlineStr"/>
-      <c r="J39" s="1" t="n">
+      <c r="J39" s="2" t="n">
         <v>46251</v>
       </c>
       <c r="K39" t="b">
@@ -2225,7 +2237,7 @@
         <v>47.5</v>
       </c>
       <c r="I40" t="inlineStr"/>
-      <c r="J40" s="1" t="n">
+      <c r="J40" s="2" t="n">
         <v>46456</v>
       </c>
       <c r="K40" t="b">
@@ -2270,7 +2282,7 @@
         <v>57.2</v>
       </c>
       <c r="I41" t="inlineStr"/>
-      <c r="J41" s="1" t="n">
+      <c r="J41" s="2" t="n">
         <v>46246</v>
       </c>
       <c r="K41" t="b">
@@ -2315,7 +2327,7 @@
         <v>59.6</v>
       </c>
       <c r="I42" t="inlineStr"/>
-      <c r="J42" s="1" t="n">
+      <c r="J42" s="2" t="n">
         <v>46487</v>
       </c>
       <c r="K42" t="b">
@@ -2360,7 +2372,7 @@
         <v>75.40000000000001</v>
       </c>
       <c r="I43" t="inlineStr"/>
-      <c r="J43" s="1" t="n">
+      <c r="J43" s="2" t="n">
         <v>46283</v>
       </c>
       <c r="K43" t="b">
@@ -2405,7 +2417,7 @@
         <v>76.8</v>
       </c>
       <c r="I44" t="inlineStr"/>
-      <c r="J44" s="1" t="n">
+      <c r="J44" s="2" t="n">
         <v>46285</v>
       </c>
       <c r="K44" t="b">
@@ -2450,7 +2462,7 @@
         <v>83.2</v>
       </c>
       <c r="I45" t="inlineStr"/>
-      <c r="J45" s="1" t="n">
+      <c r="J45" s="2" t="n">
         <v>46547</v>
       </c>
       <c r="K45" t="b">
@@ -2495,7 +2507,7 @@
         <v>84.5</v>
       </c>
       <c r="I46" t="inlineStr"/>
-      <c r="J46" s="1" t="n">
+      <c r="J46" s="2" t="n">
         <v>46240</v>
       </c>
       <c r="K46" t="b">
@@ -2540,7 +2552,7 @@
         <v>85.8</v>
       </c>
       <c r="I47" t="inlineStr"/>
-      <c r="J47" s="1" t="n">
+      <c r="J47" s="2" t="n">
         <v>46266</v>
       </c>
       <c r="K47" t="b">
@@ -2585,7 +2597,7 @@
         <v>86.5</v>
       </c>
       <c r="I48" t="inlineStr"/>
-      <c r="J48" s="1" t="n">
+      <c r="J48" s="2" t="n">
         <v>46241</v>
       </c>
       <c r="K48" t="b">
@@ -2630,7 +2642,7 @@
         <v>91.7</v>
       </c>
       <c r="I49" t="inlineStr"/>
-      <c r="J49" s="1" t="n">
+      <c r="J49" s="2" t="n">
         <v>46243</v>
       </c>
       <c r="K49" t="b">
@@ -2675,7 +2687,7 @@
         <v>91.7</v>
       </c>
       <c r="I50" t="inlineStr"/>
-      <c r="J50" s="1" t="n">
+      <c r="J50" s="2" t="n">
         <v>46243</v>
       </c>
       <c r="K50" t="b">
@@ -2720,7 +2732,7 @@
         <v>91.7</v>
       </c>
       <c r="I51" t="inlineStr"/>
-      <c r="J51" s="1" t="n">
+      <c r="J51" s="2" t="n">
         <v>46250</v>
       </c>
       <c r="K51" t="b">
@@ -2765,7 +2777,7 @@
         <v>98.90000000000001</v>
       </c>
       <c r="I52" t="inlineStr"/>
-      <c r="J52" s="1" t="n">
+      <c r="J52" s="2" t="n">
         <v>46253</v>
       </c>
       <c r="K52" t="b">
@@ -2810,7 +2822,7 @@
         <v>105.5</v>
       </c>
       <c r="I53" t="inlineStr"/>
-      <c r="J53" s="1" t="n">
+      <c r="J53" s="2" t="n">
         <v>46280</v>
       </c>
       <c r="K53" t="b">
@@ -2855,7 +2867,7 @@
         <v>105.6</v>
       </c>
       <c r="I54" t="inlineStr"/>
-      <c r="J54" s="1" t="n">
+      <c r="J54" s="2" t="n">
         <v>46361</v>
       </c>
       <c r="K54" t="b">
@@ -2900,7 +2912,7 @@
         <v>105.7</v>
       </c>
       <c r="I55" t="inlineStr"/>
-      <c r="J55" s="1" t="n">
+      <c r="J55" s="2" t="n">
         <v>46362</v>
       </c>
       <c r="K55" t="b">
@@ -2945,7 +2957,7 @@
         <v>110.7</v>
       </c>
       <c r="I56" t="inlineStr"/>
-      <c r="J56" s="1" t="n">
+      <c r="J56" s="2" t="n">
         <v>46275</v>
       </c>
       <c r="K56" t="b">
@@ -2990,7 +3002,7 @@
         <v>113.2</v>
       </c>
       <c r="I57" t="inlineStr"/>
-      <c r="J57" s="1" t="n">
+      <c r="J57" s="2" t="n">
         <v>46377</v>
       </c>
       <c r="K57" t="b">
@@ -3035,7 +3047,7 @@
         <v>128.8</v>
       </c>
       <c r="I58" t="inlineStr"/>
-      <c r="J58" s="1" t="n">
+      <c r="J58" s="2" t="n">
         <v>46434</v>
       </c>
       <c r="K58" t="b">
@@ -3080,7 +3092,7 @@
         <v>128.8</v>
       </c>
       <c r="I59" t="inlineStr"/>
-      <c r="J59" s="1" t="n">
+      <c r="J59" s="2" t="n">
         <v>46434</v>
       </c>
       <c r="K59" t="b">
@@ -3125,7 +3137,7 @@
         <v>128.8</v>
       </c>
       <c r="I60" t="inlineStr"/>
-      <c r="J60" s="1" t="n">
+      <c r="J60" s="2" t="n">
         <v>46434</v>
       </c>
       <c r="K60" t="b">
@@ -3170,7 +3182,7 @@
         <v>128.8</v>
       </c>
       <c r="I61" t="inlineStr"/>
-      <c r="J61" s="1" t="n">
+      <c r="J61" s="2" t="n">
         <v>46434</v>
       </c>
       <c r="K61" t="b">
@@ -3215,7 +3227,7 @@
         <v>128.8</v>
       </c>
       <c r="I62" t="inlineStr"/>
-      <c r="J62" s="1" t="n">
+      <c r="J62" s="2" t="n">
         <v>46434</v>
       </c>
       <c r="K62" t="b">
@@ -3260,7 +3272,7 @@
         <v>135</v>
       </c>
       <c r="I63" t="inlineStr"/>
-      <c r="J63" s="1" t="n">
+      <c r="J63" s="2" t="n">
         <v>46280</v>
       </c>
       <c r="K63" t="b">
@@ -3305,7 +3317,7 @@
         <v>150.6</v>
       </c>
       <c r="I64" t="inlineStr"/>
-      <c r="J64" s="1" t="n">
+      <c r="J64" s="2" t="n">
         <v>46271</v>
       </c>
       <c r="K64" t="b">
@@ -3350,7 +3362,7 @@
         <v>174.2</v>
       </c>
       <c r="I65" t="inlineStr"/>
-      <c r="J65" s="1" t="n">
+      <c r="J65" s="2" t="n">
         <v>46363</v>
       </c>
       <c r="K65" t="b">
@@ -3395,7 +3407,7 @@
         <v>176.6</v>
       </c>
       <c r="I66" t="inlineStr"/>
-      <c r="J66" s="1" t="n">
+      <c r="J66" s="2" t="n">
         <v>46334</v>
       </c>
       <c r="K66" t="b">
@@ -3440,7 +3452,7 @@
         <v>177.4</v>
       </c>
       <c r="I67" t="inlineStr"/>
-      <c r="J67" s="1" t="n">
+      <c r="J67" s="2" t="n">
         <v>46407</v>
       </c>
       <c r="K67" t="b">
@@ -3485,7 +3497,7 @@
         <v>183.9</v>
       </c>
       <c r="I68" t="inlineStr"/>
-      <c r="J68" s="1" t="n">
+      <c r="J68" s="2" t="n">
         <v>46341</v>
       </c>
       <c r="K68" t="b">
@@ -3530,7 +3542,7 @@
         <v>191.7</v>
       </c>
       <c r="I69" t="inlineStr"/>
-      <c r="J69" s="1" t="n">
+      <c r="J69" s="2" t="n">
         <v>46300</v>
       </c>
       <c r="K69" t="b">
@@ -3575,7 +3587,7 @@
         <v>200</v>
       </c>
       <c r="I70" t="inlineStr"/>
-      <c r="J70" s="1" t="n">
+      <c r="J70" s="2" t="n">
         <v>46336</v>
       </c>
       <c r="K70" t="b">
@@ -3620,7 +3632,7 @@
         <v>201.1</v>
       </c>
       <c r="I71" t="inlineStr"/>
-      <c r="J71" s="1" t="n">
+      <c r="J71" s="2" t="n">
         <v>46319</v>
       </c>
       <c r="K71" t="b">
@@ -3665,7 +3677,7 @@
         <v>206.5</v>
       </c>
       <c r="I72" t="inlineStr"/>
-      <c r="J72" s="1" t="n">
+      <c r="J72" s="2" t="n">
         <v>46308</v>
       </c>
       <c r="K72" t="b">
@@ -3710,7 +3722,7 @@
         <v>207.5</v>
       </c>
       <c r="I73" t="inlineStr"/>
-      <c r="J73" s="1" t="n">
+      <c r="J73" s="2" t="n">
         <v>46390</v>
       </c>
       <c r="K73" t="b">
@@ -3755,7 +3767,7 @@
         <v>247</v>
       </c>
       <c r="I74" t="inlineStr"/>
-      <c r="J74" s="1" t="n">
+      <c r="J74" s="2" t="n">
         <v>46443</v>
       </c>
       <c r="K74" t="b">
@@ -3800,7 +3812,7 @@
         <v>285.3</v>
       </c>
       <c r="I75" t="inlineStr"/>
-      <c r="J75" s="1" t="n">
+      <c r="J75" s="2" t="n">
         <v>46304</v>
       </c>
       <c r="K75" t="b">
@@ -3845,7 +3857,7 @@
         <v>290.8</v>
       </c>
       <c r="I76" t="inlineStr"/>
-      <c r="J76" s="1" t="n">
+      <c r="J76" s="2" t="n">
         <v>46362</v>
       </c>
       <c r="K76" t="b">
@@ -3890,7 +3902,7 @@
         <v>295.2</v>
       </c>
       <c r="I77" t="inlineStr"/>
-      <c r="J77" s="1" t="n">
+      <c r="J77" s="2" t="n">
         <v>46463</v>
       </c>
       <c r="K77" t="b">
@@ -3935,7 +3947,7 @@
         <v>300.2</v>
       </c>
       <c r="I78" t="inlineStr"/>
-      <c r="J78" s="1" t="n">
+      <c r="J78" s="2" t="n">
         <v>46466</v>
       </c>
       <c r="K78" t="b">
@@ -3984,7 +3996,7 @@
           <t>-317m</t>
         </is>
       </c>
-      <c r="J79" s="1" t="n">
+      <c r="J79" s="2" t="n">
         <v>36557</v>
       </c>
       <c r="K79" t="b">
@@ -4033,7 +4045,7 @@
           <t>-164m</t>
         </is>
       </c>
-      <c r="J80" s="1" t="n">
+      <c r="J80" s="2" t="n">
         <v>41275</v>
       </c>
       <c r="K80" t="b">
@@ -4082,7 +4094,7 @@
           <t>-27m</t>
         </is>
       </c>
-      <c r="J81" s="1" t="n">
+      <c r="J81" s="2" t="n">
         <v>45380</v>
       </c>
       <c r="K81" t="b">
@@ -4131,7 +4143,7 @@
           <t>-25m</t>
         </is>
       </c>
-      <c r="J82" s="1" t="n">
+      <c r="J82" s="2" t="n">
         <v>45421</v>
       </c>
       <c r="K82" t="b">
@@ -4180,7 +4192,7 @@
           <t>-25m</t>
         </is>
       </c>
-      <c r="J83" s="1" t="n">
+      <c r="J83" s="2" t="n">
         <v>45428</v>
       </c>
       <c r="K83" t="b">
@@ -4229,7 +4241,7 @@
           <t>-23m</t>
         </is>
       </c>
-      <c r="J84" s="1" t="n">
+      <c r="J84" s="2" t="n">
         <v>45490</v>
       </c>
       <c r="K84" t="b">
@@ -4278,7 +4290,7 @@
           <t>-21m</t>
         </is>
       </c>
-      <c r="J85" s="1" t="n">
+      <c r="J85" s="2" t="n">
         <v>45566</v>
       </c>
       <c r="K85" t="b">
@@ -4327,7 +4339,7 @@
           <t>-7m</t>
         </is>
       </c>
-      <c r="J86" s="1" t="n">
+      <c r="J86" s="2" t="n">
         <v>45986</v>
       </c>
       <c r="K86" t="b">
@@ -4376,7 +4388,7 @@
           <t>-3m</t>
         </is>
       </c>
-      <c r="J87" s="1" t="n">
+      <c r="J87" s="2" t="n">
         <v>46106</v>
       </c>
       <c r="K87" t="b">
@@ -4425,7 +4437,7 @@
           <t>-2m</t>
         </is>
       </c>
-      <c r="J88" s="1" t="n">
+      <c r="J88" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="K88" t="b">
@@ -4474,7 +4486,7 @@
           <t>2m</t>
         </is>
       </c>
-      <c r="J89" s="1" t="n">
+      <c r="J89" s="2" t="n">
         <v>46274</v>
       </c>
       <c r="K89" t="b">
@@ -4523,7 +4535,7 @@
           <t>2m</t>
         </is>
       </c>
-      <c r="J90" s="1" t="n">
+      <c r="J90" s="2" t="n">
         <v>46276</v>
       </c>
       <c r="K90" t="b">
@@ -4572,7 +4584,7 @@
           <t>2m</t>
         </is>
       </c>
-      <c r="J91" s="1" t="n">
+      <c r="J91" s="2" t="n">
         <v>46284</v>
       </c>
       <c r="K91" t="b">
@@ -4621,7 +4633,7 @@
           <t>3m</t>
         </is>
       </c>
-      <c r="J92" s="1" t="n">
+      <c r="J92" s="2" t="n">
         <v>46317</v>
       </c>
       <c r="K92" t="b">
@@ -4670,7 +4682,7 @@
           <t>3m</t>
         </is>
       </c>
-      <c r="J93" s="1" t="n">
+      <c r="J93" s="2" t="n">
         <v>46319</v>
       </c>
       <c r="K93" t="b">
@@ -4719,7 +4731,7 @@
           <t>4m</t>
         </is>
       </c>
-      <c r="J94" s="1" t="n">
+      <c r="J94" s="2" t="n">
         <v>46333</v>
       </c>
       <c r="K94" t="b">
@@ -4768,7 +4780,7 @@
           <t>4m</t>
         </is>
       </c>
-      <c r="J95" s="1" t="n">
+      <c r="J95" s="2" t="n">
         <v>46338</v>
       </c>
       <c r="K95" t="b">
@@ -4817,7 +4829,7 @@
           <t>4m</t>
         </is>
       </c>
-      <c r="J96" s="1" t="n">
+      <c r="J96" s="2" t="n">
         <v>46338</v>
       </c>
       <c r="K96" t="b">
@@ -4866,7 +4878,7 @@
           <t>4m</t>
         </is>
       </c>
-      <c r="J97" s="1" t="n">
+      <c r="J97" s="2" t="n">
         <v>46341</v>
       </c>
       <c r="K97" t="b">
@@ -4915,7 +4927,7 @@
           <t>4m</t>
         </is>
       </c>
-      <c r="J98" s="1" t="n">
+      <c r="J98" s="2" t="n">
         <v>46344</v>
       </c>
       <c r="K98" t="b">
@@ -4964,7 +4976,7 @@
           <t>4m</t>
         </is>
       </c>
-      <c r="J99" s="1" t="n">
+      <c r="J99" s="2" t="n">
         <v>46354</v>
       </c>
       <c r="K99" t="b">
@@ -5013,7 +5025,7 @@
           <t>4m</t>
         </is>
       </c>
-      <c r="J100" s="1" t="n">
+      <c r="J100" s="2" t="n">
         <v>46360</v>
       </c>
       <c r="K100" t="b">
@@ -5062,7 +5074,7 @@
           <t>4m</t>
         </is>
       </c>
-      <c r="J101" s="1" t="n">
+      <c r="J101" s="2" t="n">
         <v>46360</v>
       </c>
       <c r="K101" t="b">
@@ -5111,7 +5123,7 @@
           <t>5m</t>
         </is>
       </c>
-      <c r="J102" s="1" t="n">
+      <c r="J102" s="2" t="n">
         <v>46366</v>
       </c>
       <c r="K102" t="b">
@@ -5160,7 +5172,7 @@
           <t>5m</t>
         </is>
       </c>
-      <c r="J103" s="1" t="n">
+      <c r="J103" s="2" t="n">
         <v>46375</v>
       </c>
       <c r="K103" t="b">
@@ -5209,7 +5221,7 @@
           <t>5m</t>
         </is>
       </c>
-      <c r="J104" s="1" t="n">
+      <c r="J104" s="2" t="n">
         <v>46388</v>
       </c>
       <c r="K104" t="b">
@@ -5258,7 +5270,7 @@
           <t>6m</t>
         </is>
       </c>
-      <c r="J105" s="1" t="n">
+      <c r="J105" s="2" t="n">
         <v>46401</v>
       </c>
       <c r="K105" t="b">
@@ -5307,7 +5319,7 @@
           <t>6m</t>
         </is>
       </c>
-      <c r="J106" s="1" t="n">
+      <c r="J106" s="2" t="n">
         <v>46401</v>
       </c>
       <c r="K106" t="b">
@@ -5356,7 +5368,7 @@
           <t>6m</t>
         </is>
       </c>
-      <c r="J107" s="1" t="n">
+      <c r="J107" s="2" t="n">
         <v>46401</v>
       </c>
       <c r="K107" t="b">
@@ -5405,7 +5417,7 @@
           <t>6m</t>
         </is>
       </c>
-      <c r="J108" s="1" t="n">
+      <c r="J108" s="2" t="n">
         <v>46413</v>
       </c>
       <c r="K108" t="b">
@@ -5454,7 +5466,7 @@
           <t>7m</t>
         </is>
       </c>
-      <c r="J109" s="1" t="n">
+      <c r="J109" s="2" t="n">
         <v>46424</v>
       </c>
       <c r="K109" t="b">
@@ -5503,7 +5515,7 @@
           <t>7m</t>
         </is>
       </c>
-      <c r="J110" s="1" t="n">
+      <c r="J110" s="2" t="n">
         <v>46427</v>
       </c>
       <c r="K110" t="b">
@@ -5552,7 +5564,7 @@
           <t>7m</t>
         </is>
       </c>
-      <c r="J111" s="1" t="n">
+      <c r="J111" s="2" t="n">
         <v>46437</v>
       </c>
       <c r="K111" t="b">
@@ -5601,7 +5613,7 @@
           <t>7m</t>
         </is>
       </c>
-      <c r="J112" s="1" t="n">
+      <c r="J112" s="2" t="n">
         <v>46451</v>
       </c>
       <c r="K112" t="b">
@@ -5650,7 +5662,7 @@
           <t>8m</t>
         </is>
       </c>
-      <c r="J113" s="1" t="n">
+      <c r="J113" s="2" t="n">
         <v>46455</v>
       </c>
       <c r="K113" t="b">
@@ -5699,7 +5711,7 @@
           <t>8m</t>
         </is>
       </c>
-      <c r="J114" s="1" t="n">
+      <c r="J114" s="2" t="n">
         <v>46457</v>
       </c>
       <c r="K114" t="b">
@@ -5748,7 +5760,7 @@
           <t>8m</t>
         </is>
       </c>
-      <c r="J115" s="1" t="n">
+      <c r="J115" s="2" t="n">
         <v>46462</v>
       </c>
       <c r="K115" t="b">
@@ -5797,7 +5809,7 @@
           <t>8m</t>
         </is>
       </c>
-      <c r="J116" s="1" t="n">
+      <c r="J116" s="2" t="n">
         <v>46464</v>
       </c>
       <c r="K116" t="b">
@@ -5846,7 +5858,7 @@
           <t>8m</t>
         </is>
       </c>
-      <c r="J117" s="1" t="n">
+      <c r="J117" s="2" t="n">
         <v>46470</v>
       </c>
       <c r="K117" t="b">
@@ -5895,7 +5907,7 @@
           <t>9m</t>
         </is>
       </c>
-      <c r="J118" s="1" t="n">
+      <c r="J118" s="2" t="n">
         <v>46485</v>
       </c>
       <c r="K118" t="b">
@@ -5944,7 +5956,7 @@
           <t>9m</t>
         </is>
       </c>
-      <c r="J119" s="1" t="n">
+      <c r="J119" s="2" t="n">
         <v>46499</v>
       </c>
       <c r="K119" t="b">
@@ -5993,7 +6005,7 @@
           <t>9m</t>
         </is>
       </c>
-      <c r="J120" s="1" t="n">
+      <c r="J120" s="2" t="n">
         <v>46504</v>
       </c>
       <c r="K120" t="b">
@@ -6042,7 +6054,7 @@
           <t>9m</t>
         </is>
       </c>
-      <c r="J121" s="1" t="n">
+      <c r="J121" s="2" t="n">
         <v>46504</v>
       </c>
       <c r="K121" t="b">
@@ -6091,7 +6103,7 @@
           <t>9m</t>
         </is>
       </c>
-      <c r="J122" s="1" t="n">
+      <c r="J122" s="2" t="n">
         <v>46507</v>
       </c>
       <c r="K122" t="b">
@@ -6140,7 +6152,7 @@
           <t>9m</t>
         </is>
       </c>
-      <c r="J123" s="1" t="n">
+      <c r="J123" s="2" t="n">
         <v>46508</v>
       </c>
       <c r="K123" t="b">
@@ -6189,7 +6201,7 @@
           <t>9m</t>
         </is>
       </c>
-      <c r="J124" s="1" t="n">
+      <c r="J124" s="2" t="n">
         <v>46512</v>
       </c>
       <c r="K124" t="b">
@@ -6238,7 +6250,7 @@
           <t>9m</t>
         </is>
       </c>
-      <c r="J125" s="1" t="n">
+      <c r="J125" s="2" t="n">
         <v>46512</v>
       </c>
       <c r="K125" t="b">
@@ -6287,7 +6299,7 @@
           <t>10m</t>
         </is>
       </c>
-      <c r="J126" s="1" t="n">
+      <c r="J126" s="2" t="n">
         <v>46528</v>
       </c>
       <c r="K126" t="b">
@@ -6336,7 +6348,7 @@
           <t>10m</t>
         </is>
       </c>
-      <c r="J127" s="1" t="n">
+      <c r="J127" s="2" t="n">
         <v>46529</v>
       </c>
       <c r="K127" t="b">
@@ -6385,7 +6397,7 @@
           <t>10m</t>
         </is>
       </c>
-      <c r="J128" s="1" t="n">
+      <c r="J128" s="2" t="n">
         <v>46537</v>
       </c>
       <c r="K128" t="b">
@@ -6434,7 +6446,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J129" s="1" t="n">
+      <c r="J129" s="2" t="n">
         <v>46546</v>
       </c>
       <c r="K129" t="b">
@@ -6483,7 +6495,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J130" s="1" t="n">
+      <c r="J130" s="2" t="n">
         <v>46547</v>
       </c>
       <c r="K130" t="b">
@@ -6532,7 +6544,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J131" s="1" t="n">
+      <c r="J131" s="2" t="n">
         <v>46547</v>
       </c>
       <c r="K131" t="b">
@@ -6581,7 +6593,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J132" s="1" t="n">
+      <c r="J132" s="2" t="n">
         <v>46547</v>
       </c>
       <c r="K132" t="b">
@@ -6630,7 +6642,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J133" s="1" t="n">
+      <c r="J133" s="2" t="n">
         <v>46551</v>
       </c>
       <c r="K133" t="b">
@@ -6679,7 +6691,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J134" s="1" t="n">
+      <c r="J134" s="2" t="n">
         <v>46560</v>
       </c>
       <c r="K134" t="b">
@@ -6728,7 +6740,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J135" s="1" t="n">
+      <c r="J135" s="2" t="n">
         <v>46564</v>
       </c>
       <c r="K135" t="b">
@@ -6777,7 +6789,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J136" s="1" t="n">
+      <c r="J136" s="2" t="n">
         <v>46567</v>
       </c>
       <c r="K136" t="b">
@@ -6826,7 +6838,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J137" s="1" t="n">
+      <c r="J137" s="2" t="n">
         <v>46568</v>
       </c>
       <c r="K137" t="b">
@@ -6875,7 +6887,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J138" s="1" t="n">
+      <c r="J138" s="2" t="n">
         <v>46571</v>
       </c>
       <c r="K138" t="b">
@@ -6924,7 +6936,7 @@
           <t>-14d</t>
         </is>
       </c>
-      <c r="J139" s="1" t="n">
+      <c r="J139" s="2" t="n">
         <v>46197</v>
       </c>
       <c r="K139" t="b">
@@ -6973,7 +6985,7 @@
           <t>1d</t>
         </is>
       </c>
-      <c r="J140" s="1" t="n">
+      <c r="J140" s="2" t="n">
         <v>46212</v>
       </c>
       <c r="K140" t="b">
@@ -7022,7 +7034,7 @@
           <t>14d</t>
         </is>
       </c>
-      <c r="J141" s="1" t="n">
+      <c r="J141" s="2" t="n">
         <v>46225</v>
       </c>
       <c r="K141" t="b">
@@ -7071,7 +7083,7 @@
           <t>23d</t>
         </is>
       </c>
-      <c r="J142" s="1" t="n">
+      <c r="J142" s="2" t="n">
         <v>46234</v>
       </c>
       <c r="K142" t="b">
@@ -7120,7 +7132,7 @@
           <t>24d</t>
         </is>
       </c>
-      <c r="J143" s="1" t="n">
+      <c r="J143" s="2" t="n">
         <v>46234</v>
       </c>
       <c r="K143" t="b">
@@ -7169,7 +7181,7 @@
           <t>1me23d</t>
         </is>
       </c>
-      <c r="J144" s="1" t="n">
+      <c r="J144" s="2" t="n">
         <v>46263</v>
       </c>
       <c r="K144" t="b">
@@ -7218,7 +7230,7 @@
           <t>1me25d</t>
         </is>
       </c>
-      <c r="J145" s="1" t="n">
+      <c r="J145" s="2" t="n">
         <v>46266</v>
       </c>
       <c r="K145" t="b">
@@ -7263,7 +7275,7 @@
         <v>-1476</v>
       </c>
       <c r="I146" t="inlineStr"/>
-      <c r="J146" s="1" t="n">
+      <c r="J146" s="2" t="n">
         <v>43773</v>
       </c>
       <c r="K146" t="b">
@@ -7308,7 +7320,7 @@
         <v>-1469</v>
       </c>
       <c r="I147" t="inlineStr"/>
-      <c r="J147" s="1" t="n">
+      <c r="J147" s="2" t="n">
         <v>43773</v>
       </c>
       <c r="K147" t="b">
@@ -7353,7 +7365,7 @@
         <v>-1121</v>
       </c>
       <c r="I148" t="inlineStr"/>
-      <c r="J148" s="1" t="n">
+      <c r="J148" s="2" t="n">
         <v>45295</v>
       </c>
       <c r="K148" t="b">
@@ -7398,7 +7410,7 @@
         <v>-1018</v>
       </c>
       <c r="I149" t="inlineStr"/>
-      <c r="J149" s="1" t="n">
+      <c r="J149" s="2" t="n">
         <v>45617</v>
       </c>
       <c r="K149" t="b">
@@ -7443,7 +7455,7 @@
         <v>-950</v>
       </c>
       <c r="I150" t="inlineStr"/>
-      <c r="J150" s="1" t="n">
+      <c r="J150" s="2" t="n">
         <v>45677</v>
       </c>
       <c r="K150" t="b">
@@ -7488,7 +7500,7 @@
         <v>-943</v>
       </c>
       <c r="I151" t="inlineStr"/>
-      <c r="J151" s="1" t="n">
+      <c r="J151" s="2" t="n">
         <v>44944</v>
       </c>
       <c r="K151" t="b">
@@ -7533,7 +7545,7 @@
         <v>-252</v>
       </c>
       <c r="I152" t="inlineStr"/>
-      <c r="J152" s="1" t="n">
+      <c r="J152" s="2" t="n">
         <v>46092</v>
       </c>
       <c r="K152" t="b">
@@ -7578,7 +7590,7 @@
         <v>-196</v>
       </c>
       <c r="I153" t="inlineStr"/>
-      <c r="J153" s="1" t="n">
+      <c r="J153" s="2" t="n">
         <v>45988</v>
       </c>
       <c r="K153" t="b">
@@ -7623,7 +7635,7 @@
         <v>-196</v>
       </c>
       <c r="I154" t="inlineStr"/>
-      <c r="J154" s="1" t="n">
+      <c r="J154" s="2" t="n">
         <v>45988</v>
       </c>
       <c r="K154" t="b">
@@ -7668,7 +7680,7 @@
         <v>-47</v>
       </c>
       <c r="I155" t="inlineStr"/>
-      <c r="J155" s="1" t="n">
+      <c r="J155" s="2" t="n">
         <v>46176</v>
       </c>
       <c r="K155" t="b">
@@ -7713,7 +7725,7 @@
         <v>-47</v>
       </c>
       <c r="I156" t="inlineStr"/>
-      <c r="J156" s="1" t="n">
+      <c r="J156" s="2" t="n">
         <v>46176</v>
       </c>
       <c r="K156" t="b">
@@ -7758,7 +7770,7 @@
         <v>-33</v>
       </c>
       <c r="I157" t="inlineStr"/>
-      <c r="J157" s="1" t="n">
+      <c r="J157" s="2" t="n">
         <v>46199</v>
       </c>
       <c r="K157" t="b">
@@ -7803,7 +7815,7 @@
         <v>-33</v>
       </c>
       <c r="I158" t="inlineStr"/>
-      <c r="J158" s="1" t="n">
+      <c r="J158" s="2" t="n">
         <v>46199</v>
       </c>
       <c r="K158" t="b">
@@ -7848,7 +7860,7 @@
         <v>-6</v>
       </c>
       <c r="I159" t="inlineStr"/>
-      <c r="J159" s="1" t="n">
+      <c r="J159" s="2" t="n">
         <v>45967</v>
       </c>
       <c r="K159" t="b">
@@ -7893,7 +7905,7 @@
         <v>43</v>
       </c>
       <c r="I160" t="inlineStr"/>
-      <c r="J160" s="1" t="n">
+      <c r="J160" s="2" t="n">
         <v>46440</v>
       </c>
       <c r="K160" t="b">
@@ -7938,7 +7950,7 @@
         <v>43</v>
       </c>
       <c r="I161" t="inlineStr"/>
-      <c r="J161" s="1" t="n">
+      <c r="J161" s="2" t="n">
         <v>46440</v>
       </c>
       <c r="K161" t="b">
@@ -7983,7 +7995,7 @@
         <v>73</v>
       </c>
       <c r="I162" t="inlineStr"/>
-      <c r="J162" s="1" t="n">
+      <c r="J162" s="2" t="n">
         <v>46264</v>
       </c>
       <c r="K162" t="b">
@@ -8028,7 +8040,7 @@
         <v>73</v>
       </c>
       <c r="I163" t="inlineStr"/>
-      <c r="J163" s="1" t="n">
+      <c r="J163" s="2" t="n">
         <v>46264</v>
       </c>
       <c r="K163" t="b">
@@ -8073,7 +8085,7 @@
         <v>102</v>
       </c>
       <c r="I164" t="inlineStr"/>
-      <c r="J164" s="1" t="n">
+      <c r="J164" s="2" t="n">
         <v>46463</v>
       </c>
       <c r="K164" t="b">
@@ -8118,7 +8130,7 @@
         <v>118</v>
       </c>
       <c r="I165" t="inlineStr"/>
-      <c r="J165" s="1" t="n">
+      <c r="J165" s="2" t="n">
         <v>46337</v>
       </c>
       <c r="K165" t="b">
@@ -8163,7 +8175,7 @@
         <v>146</v>
       </c>
       <c r="I166" t="inlineStr"/>
-      <c r="J166" s="1" t="n">
+      <c r="J166" s="2" t="n">
         <v>46451</v>
       </c>
       <c r="K166" t="b">
@@ -8208,7 +8220,7 @@
         <v>152</v>
       </c>
       <c r="I167" t="inlineStr"/>
-      <c r="J167" s="1" t="n">
+      <c r="J167" s="2" t="n">
         <v>46245</v>
       </c>
       <c r="K167" t="b">
@@ -8253,7 +8265,7 @@
         <v>152</v>
       </c>
       <c r="I168" t="inlineStr"/>
-      <c r="J168" s="1" t="n">
+      <c r="J168" s="2" t="n">
         <v>46245</v>
       </c>
       <c r="K168" t="b">
@@ -8298,7 +8310,7 @@
         <v>163</v>
       </c>
       <c r="I169" t="inlineStr"/>
-      <c r="J169" s="1" t="n">
+      <c r="J169" s="2" t="n">
         <v>46324</v>
       </c>
       <c r="K169" t="b">
@@ -8343,7 +8355,7 @@
         <v>163</v>
       </c>
       <c r="I170" t="inlineStr"/>
-      <c r="J170" s="1" t="n">
+      <c r="J170" s="2" t="n">
         <v>46324</v>
       </c>
       <c r="K170" t="b">
@@ -8388,7 +8400,7 @@
         <v>164</v>
       </c>
       <c r="I171" t="inlineStr"/>
-      <c r="J171" s="1" t="n">
+      <c r="J171" s="2" t="n">
         <v>46426</v>
       </c>
       <c r="K171" t="b">
@@ -8433,7 +8445,7 @@
         <v>175</v>
       </c>
       <c r="I172" t="inlineStr"/>
-      <c r="J172" s="1" t="n">
+      <c r="J172" s="2" t="n">
         <v>46383</v>
       </c>
       <c r="K172" t="b">
@@ -8478,7 +8490,7 @@
         <v>186</v>
       </c>
       <c r="I173" t="inlineStr"/>
-      <c r="J173" s="1" t="n">
+      <c r="J173" s="2" t="n">
         <v>46392</v>
       </c>
       <c r="K173" t="b">
@@ -8523,7 +8535,7 @@
         <v>205</v>
       </c>
       <c r="I174" t="inlineStr"/>
-      <c r="J174" s="1" t="n">
+      <c r="J174" s="2" t="n">
         <v>46390</v>
       </c>
       <c r="K174" t="b">
@@ -8568,7 +8580,7 @@
         <v>207</v>
       </c>
       <c r="I175" t="inlineStr"/>
-      <c r="J175" s="1" t="n">
+      <c r="J175" s="2" t="n">
         <v>46392</v>
       </c>
       <c r="K175" t="b">
@@ -8613,7 +8625,7 @@
         <v>218</v>
       </c>
       <c r="I176" t="inlineStr"/>
-      <c r="J176" s="1" t="n">
+      <c r="J176" s="2" t="n">
         <v>46506</v>
       </c>
       <c r="K176" t="b">
@@ -8658,7 +8670,7 @@
         <v>246</v>
       </c>
       <c r="I177" t="inlineStr"/>
-      <c r="J177" s="1" t="n">
+      <c r="J177" s="2" t="n">
         <v>46478</v>
       </c>
       <c r="K177" t="b">
@@ -8703,7 +8715,7 @@
         <v>248</v>
       </c>
       <c r="I178" t="inlineStr"/>
-      <c r="J178" s="1" t="n">
+      <c r="J178" s="2" t="n">
         <v>46500</v>
       </c>
       <c r="K178" t="b">
@@ -8748,7 +8760,7 @@
         <v>276</v>
       </c>
       <c r="I179" t="inlineStr"/>
-      <c r="J179" s="1" t="n">
+      <c r="J179" s="2" t="n">
         <v>46430</v>
       </c>
       <c r="K179" t="b">
@@ -8793,7 +8805,7 @@
         <v>276</v>
       </c>
       <c r="I180" t="inlineStr"/>
-      <c r="J180" s="1" t="n">
+      <c r="J180" s="2" t="n">
         <v>46430</v>
       </c>
       <c r="K180" t="b">
@@ -8838,7 +8850,7 @@
         <v>290</v>
       </c>
       <c r="I181" t="inlineStr"/>
-      <c r="J181" s="1" t="n">
+      <c r="J181" s="2" t="n">
         <v>46467</v>
       </c>
       <c r="K181" t="b">
@@ -8883,7 +8895,7 @@
         <v>317</v>
       </c>
       <c r="I182" t="inlineStr"/>
-      <c r="J182" s="1" t="n">
+      <c r="J182" s="2" t="n">
         <v>46529</v>
       </c>
       <c r="K182" t="b">
@@ -8928,7 +8940,7 @@
         <v>420</v>
       </c>
       <c r="I183" t="inlineStr"/>
-      <c r="J183" s="1" t="n">
+      <c r="J183" s="2" t="n">
         <v>46566</v>
       </c>
       <c r="K183" t="b">
@@ -8973,7 +8985,7 @@
         <v>426</v>
       </c>
       <c r="I184" t="inlineStr"/>
-      <c r="J184" s="1" t="n">
+      <c r="J184" s="2" t="n">
         <v>46571</v>
       </c>
       <c r="K184" t="b">
@@ -9018,7 +9030,7 @@
         <v>721</v>
       </c>
       <c r="I185" t="inlineStr"/>
-      <c r="J185" s="1" t="n">
+      <c r="J185" s="2" t="n">
         <v>46325</v>
       </c>
       <c r="K185" t="b">
@@ -9063,7 +9075,7 @@
         <v>721</v>
       </c>
       <c r="I186" t="inlineStr"/>
-      <c r="J186" s="1" t="n">
+      <c r="J186" s="2" t="n">
         <v>46325</v>
       </c>
       <c r="K186" t="b">
@@ -9108,7 +9120,7 @@
         <v>850</v>
       </c>
       <c r="I187" t="inlineStr"/>
-      <c r="J187" s="1" t="n">
+      <c r="J187" s="2" t="n">
         <v>46345</v>
       </c>
       <c r="K187" t="b">
@@ -9153,7 +9165,7 @@
         <v>850</v>
       </c>
       <c r="I188" t="inlineStr"/>
-      <c r="J188" s="1" t="n">
+      <c r="J188" s="2" t="n">
         <v>46345</v>
       </c>
       <c r="K188" t="b">
@@ -9198,7 +9210,7 @@
         <v>1661</v>
       </c>
       <c r="I189" t="inlineStr"/>
-      <c r="J189" s="1" t="n">
+      <c r="J189" s="2" t="n">
         <v>46498</v>
       </c>
       <c r="K189" t="b">
@@ -9243,7 +9255,7 @@
         <v>1661</v>
       </c>
       <c r="I190" t="inlineStr"/>
-      <c r="J190" s="1" t="n">
+      <c r="J190" s="2" t="n">
         <v>46498</v>
       </c>
       <c r="K190" t="b">
@@ -9288,7 +9300,7 @@
         <v>488</v>
       </c>
       <c r="I191" t="inlineStr"/>
-      <c r="J191" s="1" t="n">
+      <c r="J191" s="2" t="n">
         <v>46190</v>
       </c>
       <c r="K191" t="b">
@@ -9333,7 +9345,7 @@
         <v>25565</v>
       </c>
       <c r="I192" t="inlineStr"/>
-      <c r="J192" s="1" t="n">
+      <c r="J192" s="2" t="n">
         <v>46190</v>
       </c>
       <c r="K192" t="b">
@@ -9378,7 +9390,7 @@
         <v>25567</v>
       </c>
       <c r="I193" t="inlineStr"/>
-      <c r="J193" s="1" t="n">
+      <c r="J193" s="2" t="n">
         <v>46190</v>
       </c>
       <c r="K193" t="b">
@@ -9423,7 +9435,7 @@
         <v>31293</v>
       </c>
       <c r="I194" t="inlineStr"/>
-      <c r="J194" s="1" t="n">
+      <c r="J194" s="2" t="n">
         <v>46190</v>
       </c>
       <c r="K194" t="b">

</xml_diff>

<commit_message>
Atualização automática: vencimentos_tmot (10/07/2026 22:38)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
@@ -20,16 +20,13 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -40,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -48,21 +45,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -433,57 +421,57 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>matricula</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>operador</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>pn</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>sn</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>nomenclatura</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>inspecao</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>tipo_vencimento</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>disponibilidade_valor</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>disponibilidade_texto</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>data_vencimento</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>vencido</t>
         </is>
@@ -527,7 +515,7 @@
         <v>-4402.8</v>
       </c>
       <c r="I2" t="inlineStr"/>
-      <c r="J2" s="2" t="n">
+      <c r="J2" s="1" t="n">
         <v>41388</v>
       </c>
       <c r="K2" t="b">
@@ -572,7 +560,7 @@
         <v>-4254.8</v>
       </c>
       <c r="I3" t="inlineStr"/>
-      <c r="J3" s="2" t="n">
+      <c r="J3" s="1" t="n">
         <v>39285</v>
       </c>
       <c r="K3" t="b">
@@ -617,7 +605,7 @@
         <v>-2354.2</v>
       </c>
       <c r="I4" t="inlineStr"/>
-      <c r="J4" s="2" t="n">
+      <c r="J4" s="1" t="n">
         <v>40669</v>
       </c>
       <c r="K4" t="b">
@@ -662,7 +650,7 @@
         <v>-896.8</v>
       </c>
       <c r="I5" t="inlineStr"/>
-      <c r="J5" s="2" t="n">
+      <c r="J5" s="1" t="n">
         <v>40669</v>
       </c>
       <c r="K5" t="b">
@@ -707,7 +695,7 @@
         <v>-854.1</v>
       </c>
       <c r="I6" t="inlineStr"/>
-      <c r="J6" s="2" t="n">
+      <c r="J6" s="1" t="n">
         <v>44884</v>
       </c>
       <c r="K6" t="b">
@@ -752,7 +740,7 @@
         <v>-413.2</v>
       </c>
       <c r="I7" t="inlineStr"/>
-      <c r="J7" s="2" t="n">
+      <c r="J7" s="1" t="n">
         <v>43855</v>
       </c>
       <c r="K7" t="b">
@@ -797,7 +785,7 @@
         <v>-391.8</v>
       </c>
       <c r="I8" t="inlineStr"/>
-      <c r="J8" s="2" t="n">
+      <c r="J8" s="1" t="n">
         <v>42769</v>
       </c>
       <c r="K8" t="b">
@@ -842,7 +830,7 @@
         <v>-371.5</v>
       </c>
       <c r="I9" t="inlineStr"/>
-      <c r="J9" s="2" t="n">
+      <c r="J9" s="1" t="n">
         <v>46014</v>
       </c>
       <c r="K9" t="b">
@@ -887,7 +875,7 @@
         <v>-368.8</v>
       </c>
       <c r="I10" t="inlineStr"/>
-      <c r="J10" s="2" t="n">
+      <c r="J10" s="1" t="n">
         <v>46014</v>
       </c>
       <c r="K10" t="b">
@@ -932,7 +920,7 @@
         <v>-359</v>
       </c>
       <c r="I11" t="inlineStr"/>
-      <c r="J11" s="2" t="n">
+      <c r="J11" s="1" t="n">
         <v>45804</v>
       </c>
       <c r="K11" t="b">
@@ -977,7 +965,7 @@
         <v>-359</v>
       </c>
       <c r="I12" t="inlineStr"/>
-      <c r="J12" s="2" t="n">
+      <c r="J12" s="1" t="n">
         <v>45804</v>
       </c>
       <c r="K12" t="b">
@@ -1022,7 +1010,7 @@
         <v>-351</v>
       </c>
       <c r="I13" t="inlineStr"/>
-      <c r="J13" s="2" t="n">
+      <c r="J13" s="1" t="n">
         <v>42821</v>
       </c>
       <c r="K13" t="b">
@@ -1067,7 +1055,7 @@
         <v>-351</v>
       </c>
       <c r="I14" t="inlineStr"/>
-      <c r="J14" s="2" t="n">
+      <c r="J14" s="1" t="n">
         <v>46014</v>
       </c>
       <c r="K14" t="b">
@@ -1112,7 +1100,7 @@
         <v>-351</v>
       </c>
       <c r="I15" t="inlineStr"/>
-      <c r="J15" s="2" t="n">
+      <c r="J15" s="1" t="n">
         <v>46014</v>
       </c>
       <c r="K15" t="b">
@@ -1157,7 +1145,7 @@
         <v>-351</v>
       </c>
       <c r="I16" t="inlineStr"/>
-      <c r="J16" s="2" t="n">
+      <c r="J16" s="1" t="n">
         <v>46014</v>
       </c>
       <c r="K16" t="b">
@@ -1202,7 +1190,7 @@
         <v>-345.8</v>
       </c>
       <c r="I17" t="inlineStr"/>
-      <c r="J17" s="2" t="n">
+      <c r="J17" s="1" t="n">
         <v>46017</v>
       </c>
       <c r="K17" t="b">
@@ -1247,7 +1235,7 @@
         <v>-345.8</v>
       </c>
       <c r="I18" t="inlineStr"/>
-      <c r="J18" s="2" t="n">
+      <c r="J18" s="1" t="n">
         <v>46017</v>
       </c>
       <c r="K18" t="b">
@@ -1292,7 +1280,7 @@
         <v>-264.2</v>
       </c>
       <c r="I19" t="inlineStr"/>
-      <c r="J19" s="2" t="n">
+      <c r="J19" s="1" t="n">
         <v>40979</v>
       </c>
       <c r="K19" t="b">
@@ -1337,7 +1325,7 @@
         <v>-206.4</v>
       </c>
       <c r="I20" t="inlineStr"/>
-      <c r="J20" s="2" t="n">
+      <c r="J20" s="1" t="n">
         <v>36669</v>
       </c>
       <c r="K20" t="b">
@@ -1382,7 +1370,7 @@
         <v>-131.6</v>
       </c>
       <c r="I21" t="inlineStr"/>
-      <c r="J21" s="2" t="n">
+      <c r="J21" s="1" t="n">
         <v>46111</v>
       </c>
       <c r="K21" t="b">
@@ -1427,7 +1415,7 @@
         <v>-131.6</v>
       </c>
       <c r="I22" t="inlineStr"/>
-      <c r="J22" s="2" t="n">
+      <c r="J22" s="1" t="n">
         <v>46111</v>
       </c>
       <c r="K22" t="b">
@@ -1472,7 +1460,7 @@
         <v>-131.6</v>
       </c>
       <c r="I23" t="inlineStr"/>
-      <c r="J23" s="2" t="n">
+      <c r="J23" s="1" t="n">
         <v>46111</v>
       </c>
       <c r="K23" t="b">
@@ -1517,7 +1505,7 @@
         <v>-131.6</v>
       </c>
       <c r="I24" t="inlineStr"/>
-      <c r="J24" s="2" t="n">
+      <c r="J24" s="1" t="n">
         <v>46111</v>
       </c>
       <c r="K24" t="b">
@@ -1562,7 +1550,7 @@
         <v>-131.6</v>
       </c>
       <c r="I25" t="inlineStr"/>
-      <c r="J25" s="2" t="n">
+      <c r="J25" s="1" t="n">
         <v>46111</v>
       </c>
       <c r="K25" t="b">
@@ -1607,7 +1595,7 @@
         <v>-105</v>
       </c>
       <c r="I26" t="inlineStr"/>
-      <c r="J26" s="2" t="n">
+      <c r="J26" s="1" t="n">
         <v>46161</v>
       </c>
       <c r="K26" t="b">
@@ -1652,7 +1640,7 @@
         <v>-79.8</v>
       </c>
       <c r="I27" t="inlineStr"/>
-      <c r="J27" s="2" t="n">
+      <c r="J27" s="1" t="n">
         <v>43340</v>
       </c>
       <c r="K27" t="b">
@@ -1697,7 +1685,7 @@
         <v>-12.3</v>
       </c>
       <c r="I28" t="inlineStr"/>
-      <c r="J28" s="2" t="n">
+      <c r="J28" s="1" t="n">
         <v>46048</v>
       </c>
       <c r="K28" t="b">
@@ -1742,7 +1730,7 @@
         <v>0</v>
       </c>
       <c r="I29" t="inlineStr"/>
-      <c r="J29" s="2" t="n">
+      <c r="J29" s="1" t="n">
         <v>46211</v>
       </c>
       <c r="K29" t="b">
@@ -1787,7 +1775,7 @@
         <v>3.6</v>
       </c>
       <c r="I30" t="inlineStr"/>
-      <c r="J30" s="2" t="n">
+      <c r="J30" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="K30" t="b">
@@ -1832,7 +1820,7 @@
         <v>6.2</v>
       </c>
       <c r="I31" t="inlineStr"/>
-      <c r="J31" s="2" t="n">
+      <c r="J31" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="K31" t="b">
@@ -1877,7 +1865,7 @@
         <v>7.5</v>
       </c>
       <c r="I32" t="inlineStr"/>
-      <c r="J32" s="2" t="n">
+      <c r="J32" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="K32" t="b">
@@ -1922,7 +1910,7 @@
         <v>10.7</v>
       </c>
       <c r="I33" t="inlineStr"/>
-      <c r="J33" s="2" t="n">
+      <c r="J33" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="K33" t="b">
@@ -1967,7 +1955,7 @@
         <v>20</v>
       </c>
       <c r="I34" t="inlineStr"/>
-      <c r="J34" s="2" t="n">
+      <c r="J34" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="K34" t="b">
@@ -2012,7 +2000,7 @@
         <v>30.8</v>
       </c>
       <c r="I35" t="inlineStr"/>
-      <c r="J35" s="2" t="n">
+      <c r="J35" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="K35" t="b">
@@ -2057,7 +2045,7 @@
         <v>37.1</v>
       </c>
       <c r="I36" t="inlineStr"/>
-      <c r="J36" s="2" t="n">
+      <c r="J36" s="1" t="n">
         <v>46256</v>
       </c>
       <c r="K36" t="b">
@@ -2102,7 +2090,7 @@
         <v>42.8</v>
       </c>
       <c r="I37" t="inlineStr"/>
-      <c r="J37" s="2" t="n">
+      <c r="J37" s="1" t="n">
         <v>46276</v>
       </c>
       <c r="K37" t="b">
@@ -2147,7 +2135,7 @@
         <v>45.2</v>
       </c>
       <c r="I38" t="inlineStr"/>
-      <c r="J38" s="2" t="n">
+      <c r="J38" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="K38" t="b">
@@ -2192,7 +2180,7 @@
         <v>46</v>
       </c>
       <c r="I39" t="inlineStr"/>
-      <c r="J39" s="2" t="n">
+      <c r="J39" s="1" t="n">
         <v>46251</v>
       </c>
       <c r="K39" t="b">
@@ -2237,7 +2225,7 @@
         <v>47.5</v>
       </c>
       <c r="I40" t="inlineStr"/>
-      <c r="J40" s="2" t="n">
+      <c r="J40" s="1" t="n">
         <v>46456</v>
       </c>
       <c r="K40" t="b">
@@ -2282,7 +2270,7 @@
         <v>57.2</v>
       </c>
       <c r="I41" t="inlineStr"/>
-      <c r="J41" s="2" t="n">
+      <c r="J41" s="1" t="n">
         <v>46246</v>
       </c>
       <c r="K41" t="b">
@@ -2327,7 +2315,7 @@
         <v>59.6</v>
       </c>
       <c r="I42" t="inlineStr"/>
-      <c r="J42" s="2" t="n">
+      <c r="J42" s="1" t="n">
         <v>46487</v>
       </c>
       <c r="K42" t="b">
@@ -2372,7 +2360,7 @@
         <v>75.40000000000001</v>
       </c>
       <c r="I43" t="inlineStr"/>
-      <c r="J43" s="2" t="n">
+      <c r="J43" s="1" t="n">
         <v>46283</v>
       </c>
       <c r="K43" t="b">
@@ -2417,7 +2405,7 @@
         <v>76.8</v>
       </c>
       <c r="I44" t="inlineStr"/>
-      <c r="J44" s="2" t="n">
+      <c r="J44" s="1" t="n">
         <v>46285</v>
       </c>
       <c r="K44" t="b">
@@ -2462,7 +2450,7 @@
         <v>83.2</v>
       </c>
       <c r="I45" t="inlineStr"/>
-      <c r="J45" s="2" t="n">
+      <c r="J45" s="1" t="n">
         <v>46547</v>
       </c>
       <c r="K45" t="b">
@@ -2507,7 +2495,7 @@
         <v>84.5</v>
       </c>
       <c r="I46" t="inlineStr"/>
-      <c r="J46" s="2" t="n">
+      <c r="J46" s="1" t="n">
         <v>46240</v>
       </c>
       <c r="K46" t="b">
@@ -2552,7 +2540,7 @@
         <v>85.8</v>
       </c>
       <c r="I47" t="inlineStr"/>
-      <c r="J47" s="2" t="n">
+      <c r="J47" s="1" t="n">
         <v>46266</v>
       </c>
       <c r="K47" t="b">
@@ -2597,7 +2585,7 @@
         <v>86.5</v>
       </c>
       <c r="I48" t="inlineStr"/>
-      <c r="J48" s="2" t="n">
+      <c r="J48" s="1" t="n">
         <v>46241</v>
       </c>
       <c r="K48" t="b">
@@ -2642,7 +2630,7 @@
         <v>91.7</v>
       </c>
       <c r="I49" t="inlineStr"/>
-      <c r="J49" s="2" t="n">
+      <c r="J49" s="1" t="n">
         <v>46243</v>
       </c>
       <c r="K49" t="b">
@@ -2687,7 +2675,7 @@
         <v>91.7</v>
       </c>
       <c r="I50" t="inlineStr"/>
-      <c r="J50" s="2" t="n">
+      <c r="J50" s="1" t="n">
         <v>46243</v>
       </c>
       <c r="K50" t="b">
@@ -2732,7 +2720,7 @@
         <v>91.7</v>
       </c>
       <c r="I51" t="inlineStr"/>
-      <c r="J51" s="2" t="n">
+      <c r="J51" s="1" t="n">
         <v>46250</v>
       </c>
       <c r="K51" t="b">
@@ -2777,7 +2765,7 @@
         <v>98.90000000000001</v>
       </c>
       <c r="I52" t="inlineStr"/>
-      <c r="J52" s="2" t="n">
+      <c r="J52" s="1" t="n">
         <v>46253</v>
       </c>
       <c r="K52" t="b">
@@ -2822,7 +2810,7 @@
         <v>105.5</v>
       </c>
       <c r="I53" t="inlineStr"/>
-      <c r="J53" s="2" t="n">
+      <c r="J53" s="1" t="n">
         <v>46280</v>
       </c>
       <c r="K53" t="b">
@@ -2867,7 +2855,7 @@
         <v>105.6</v>
       </c>
       <c r="I54" t="inlineStr"/>
-      <c r="J54" s="2" t="n">
+      <c r="J54" s="1" t="n">
         <v>46361</v>
       </c>
       <c r="K54" t="b">
@@ -2912,7 +2900,7 @@
         <v>105.7</v>
       </c>
       <c r="I55" t="inlineStr"/>
-      <c r="J55" s="2" t="n">
+      <c r="J55" s="1" t="n">
         <v>46362</v>
       </c>
       <c r="K55" t="b">
@@ -2957,7 +2945,7 @@
         <v>110.7</v>
       </c>
       <c r="I56" t="inlineStr"/>
-      <c r="J56" s="2" t="n">
+      <c r="J56" s="1" t="n">
         <v>46275</v>
       </c>
       <c r="K56" t="b">
@@ -3002,7 +2990,7 @@
         <v>113.2</v>
       </c>
       <c r="I57" t="inlineStr"/>
-      <c r="J57" s="2" t="n">
+      <c r="J57" s="1" t="n">
         <v>46377</v>
       </c>
       <c r="K57" t="b">
@@ -3047,7 +3035,7 @@
         <v>128.8</v>
       </c>
       <c r="I58" t="inlineStr"/>
-      <c r="J58" s="2" t="n">
+      <c r="J58" s="1" t="n">
         <v>46434</v>
       </c>
       <c r="K58" t="b">
@@ -3092,7 +3080,7 @@
         <v>128.8</v>
       </c>
       <c r="I59" t="inlineStr"/>
-      <c r="J59" s="2" t="n">
+      <c r="J59" s="1" t="n">
         <v>46434</v>
       </c>
       <c r="K59" t="b">
@@ -3137,7 +3125,7 @@
         <v>128.8</v>
       </c>
       <c r="I60" t="inlineStr"/>
-      <c r="J60" s="2" t="n">
+      <c r="J60" s="1" t="n">
         <v>46434</v>
       </c>
       <c r="K60" t="b">
@@ -3182,7 +3170,7 @@
         <v>128.8</v>
       </c>
       <c r="I61" t="inlineStr"/>
-      <c r="J61" s="2" t="n">
+      <c r="J61" s="1" t="n">
         <v>46434</v>
       </c>
       <c r="K61" t="b">
@@ -3227,7 +3215,7 @@
         <v>128.8</v>
       </c>
       <c r="I62" t="inlineStr"/>
-      <c r="J62" s="2" t="n">
+      <c r="J62" s="1" t="n">
         <v>46434</v>
       </c>
       <c r="K62" t="b">
@@ -3272,7 +3260,7 @@
         <v>135</v>
       </c>
       <c r="I63" t="inlineStr"/>
-      <c r="J63" s="2" t="n">
+      <c r="J63" s="1" t="n">
         <v>46280</v>
       </c>
       <c r="K63" t="b">
@@ -3317,7 +3305,7 @@
         <v>150.6</v>
       </c>
       <c r="I64" t="inlineStr"/>
-      <c r="J64" s="2" t="n">
+      <c r="J64" s="1" t="n">
         <v>46271</v>
       </c>
       <c r="K64" t="b">
@@ -3362,7 +3350,7 @@
         <v>174.2</v>
       </c>
       <c r="I65" t="inlineStr"/>
-      <c r="J65" s="2" t="n">
+      <c r="J65" s="1" t="n">
         <v>46363</v>
       </c>
       <c r="K65" t="b">
@@ -3407,7 +3395,7 @@
         <v>176.6</v>
       </c>
       <c r="I66" t="inlineStr"/>
-      <c r="J66" s="2" t="n">
+      <c r="J66" s="1" t="n">
         <v>46334</v>
       </c>
       <c r="K66" t="b">
@@ -3452,7 +3440,7 @@
         <v>177.4</v>
       </c>
       <c r="I67" t="inlineStr"/>
-      <c r="J67" s="2" t="n">
+      <c r="J67" s="1" t="n">
         <v>46407</v>
       </c>
       <c r="K67" t="b">
@@ -3497,7 +3485,7 @@
         <v>183.9</v>
       </c>
       <c r="I68" t="inlineStr"/>
-      <c r="J68" s="2" t="n">
+      <c r="J68" s="1" t="n">
         <v>46341</v>
       </c>
       <c r="K68" t="b">
@@ -3542,7 +3530,7 @@
         <v>191.7</v>
       </c>
       <c r="I69" t="inlineStr"/>
-      <c r="J69" s="2" t="n">
+      <c r="J69" s="1" t="n">
         <v>46300</v>
       </c>
       <c r="K69" t="b">
@@ -3587,7 +3575,7 @@
         <v>200</v>
       </c>
       <c r="I70" t="inlineStr"/>
-      <c r="J70" s="2" t="n">
+      <c r="J70" s="1" t="n">
         <v>46336</v>
       </c>
       <c r="K70" t="b">
@@ -3632,7 +3620,7 @@
         <v>201.1</v>
       </c>
       <c r="I71" t="inlineStr"/>
-      <c r="J71" s="2" t="n">
+      <c r="J71" s="1" t="n">
         <v>46319</v>
       </c>
       <c r="K71" t="b">
@@ -3677,7 +3665,7 @@
         <v>206.5</v>
       </c>
       <c r="I72" t="inlineStr"/>
-      <c r="J72" s="2" t="n">
+      <c r="J72" s="1" t="n">
         <v>46308</v>
       </c>
       <c r="K72" t="b">
@@ -3722,7 +3710,7 @@
         <v>207.5</v>
       </c>
       <c r="I73" t="inlineStr"/>
-      <c r="J73" s="2" t="n">
+      <c r="J73" s="1" t="n">
         <v>46390</v>
       </c>
       <c r="K73" t="b">
@@ -3767,7 +3755,7 @@
         <v>247</v>
       </c>
       <c r="I74" t="inlineStr"/>
-      <c r="J74" s="2" t="n">
+      <c r="J74" s="1" t="n">
         <v>46443</v>
       </c>
       <c r="K74" t="b">
@@ -3812,7 +3800,7 @@
         <v>285.3</v>
       </c>
       <c r="I75" t="inlineStr"/>
-      <c r="J75" s="2" t="n">
+      <c r="J75" s="1" t="n">
         <v>46304</v>
       </c>
       <c r="K75" t="b">
@@ -3857,7 +3845,7 @@
         <v>290.8</v>
       </c>
       <c r="I76" t="inlineStr"/>
-      <c r="J76" s="2" t="n">
+      <c r="J76" s="1" t="n">
         <v>46362</v>
       </c>
       <c r="K76" t="b">
@@ -3902,7 +3890,7 @@
         <v>295.2</v>
       </c>
       <c r="I77" t="inlineStr"/>
-      <c r="J77" s="2" t="n">
+      <c r="J77" s="1" t="n">
         <v>46463</v>
       </c>
       <c r="K77" t="b">
@@ -3947,7 +3935,7 @@
         <v>300.2</v>
       </c>
       <c r="I78" t="inlineStr"/>
-      <c r="J78" s="2" t="n">
+      <c r="J78" s="1" t="n">
         <v>46466</v>
       </c>
       <c r="K78" t="b">
@@ -3996,7 +3984,7 @@
           <t>-317m</t>
         </is>
       </c>
-      <c r="J79" s="2" t="n">
+      <c r="J79" s="1" t="n">
         <v>36557</v>
       </c>
       <c r="K79" t="b">
@@ -4045,7 +4033,7 @@
           <t>-164m</t>
         </is>
       </c>
-      <c r="J80" s="2" t="n">
+      <c r="J80" s="1" t="n">
         <v>41275</v>
       </c>
       <c r="K80" t="b">
@@ -4094,7 +4082,7 @@
           <t>-27m</t>
         </is>
       </c>
-      <c r="J81" s="2" t="n">
+      <c r="J81" s="1" t="n">
         <v>45380</v>
       </c>
       <c r="K81" t="b">
@@ -4143,7 +4131,7 @@
           <t>-25m</t>
         </is>
       </c>
-      <c r="J82" s="2" t="n">
+      <c r="J82" s="1" t="n">
         <v>45421</v>
       </c>
       <c r="K82" t="b">
@@ -4192,7 +4180,7 @@
           <t>-25m</t>
         </is>
       </c>
-      <c r="J83" s="2" t="n">
+      <c r="J83" s="1" t="n">
         <v>45428</v>
       </c>
       <c r="K83" t="b">
@@ -4241,7 +4229,7 @@
           <t>-23m</t>
         </is>
       </c>
-      <c r="J84" s="2" t="n">
+      <c r="J84" s="1" t="n">
         <v>45490</v>
       </c>
       <c r="K84" t="b">
@@ -4290,7 +4278,7 @@
           <t>-21m</t>
         </is>
       </c>
-      <c r="J85" s="2" t="n">
+      <c r="J85" s="1" t="n">
         <v>45566</v>
       </c>
       <c r="K85" t="b">
@@ -4339,7 +4327,7 @@
           <t>-7m</t>
         </is>
       </c>
-      <c r="J86" s="2" t="n">
+      <c r="J86" s="1" t="n">
         <v>45986</v>
       </c>
       <c r="K86" t="b">
@@ -4388,7 +4376,7 @@
           <t>-3m</t>
         </is>
       </c>
-      <c r="J87" s="2" t="n">
+      <c r="J87" s="1" t="n">
         <v>46106</v>
       </c>
       <c r="K87" t="b">
@@ -4437,7 +4425,7 @@
           <t>-2m</t>
         </is>
       </c>
-      <c r="J88" s="2" t="n">
+      <c r="J88" s="1" t="n">
         <v>46142</v>
       </c>
       <c r="K88" t="b">
@@ -4486,7 +4474,7 @@
           <t>2m</t>
         </is>
       </c>
-      <c r="J89" s="2" t="n">
+      <c r="J89" s="1" t="n">
         <v>46274</v>
       </c>
       <c r="K89" t="b">
@@ -4535,7 +4523,7 @@
           <t>2m</t>
         </is>
       </c>
-      <c r="J90" s="2" t="n">
+      <c r="J90" s="1" t="n">
         <v>46276</v>
       </c>
       <c r="K90" t="b">
@@ -4584,7 +4572,7 @@
           <t>2m</t>
         </is>
       </c>
-      <c r="J91" s="2" t="n">
+      <c r="J91" s="1" t="n">
         <v>46284</v>
       </c>
       <c r="K91" t="b">
@@ -4633,7 +4621,7 @@
           <t>3m</t>
         </is>
       </c>
-      <c r="J92" s="2" t="n">
+      <c r="J92" s="1" t="n">
         <v>46317</v>
       </c>
       <c r="K92" t="b">
@@ -4682,7 +4670,7 @@
           <t>3m</t>
         </is>
       </c>
-      <c r="J93" s="2" t="n">
+      <c r="J93" s="1" t="n">
         <v>46319</v>
       </c>
       <c r="K93" t="b">
@@ -4731,7 +4719,7 @@
           <t>4m</t>
         </is>
       </c>
-      <c r="J94" s="2" t="n">
+      <c r="J94" s="1" t="n">
         <v>46333</v>
       </c>
       <c r="K94" t="b">
@@ -4780,7 +4768,7 @@
           <t>4m</t>
         </is>
       </c>
-      <c r="J95" s="2" t="n">
+      <c r="J95" s="1" t="n">
         <v>46338</v>
       </c>
       <c r="K95" t="b">
@@ -4829,7 +4817,7 @@
           <t>4m</t>
         </is>
       </c>
-      <c r="J96" s="2" t="n">
+      <c r="J96" s="1" t="n">
         <v>46338</v>
       </c>
       <c r="K96" t="b">
@@ -4878,7 +4866,7 @@
           <t>4m</t>
         </is>
       </c>
-      <c r="J97" s="2" t="n">
+      <c r="J97" s="1" t="n">
         <v>46341</v>
       </c>
       <c r="K97" t="b">
@@ -4927,7 +4915,7 @@
           <t>4m</t>
         </is>
       </c>
-      <c r="J98" s="2" t="n">
+      <c r="J98" s="1" t="n">
         <v>46344</v>
       </c>
       <c r="K98" t="b">
@@ -4976,7 +4964,7 @@
           <t>4m</t>
         </is>
       </c>
-      <c r="J99" s="2" t="n">
+      <c r="J99" s="1" t="n">
         <v>46354</v>
       </c>
       <c r="K99" t="b">
@@ -5025,7 +5013,7 @@
           <t>4m</t>
         </is>
       </c>
-      <c r="J100" s="2" t="n">
+      <c r="J100" s="1" t="n">
         <v>46360</v>
       </c>
       <c r="K100" t="b">
@@ -5074,7 +5062,7 @@
           <t>4m</t>
         </is>
       </c>
-      <c r="J101" s="2" t="n">
+      <c r="J101" s="1" t="n">
         <v>46360</v>
       </c>
       <c r="K101" t="b">
@@ -5123,7 +5111,7 @@
           <t>5m</t>
         </is>
       </c>
-      <c r="J102" s="2" t="n">
+      <c r="J102" s="1" t="n">
         <v>46366</v>
       </c>
       <c r="K102" t="b">
@@ -5172,7 +5160,7 @@
           <t>5m</t>
         </is>
       </c>
-      <c r="J103" s="2" t="n">
+      <c r="J103" s="1" t="n">
         <v>46375</v>
       </c>
       <c r="K103" t="b">
@@ -5221,7 +5209,7 @@
           <t>5m</t>
         </is>
       </c>
-      <c r="J104" s="2" t="n">
+      <c r="J104" s="1" t="n">
         <v>46388</v>
       </c>
       <c r="K104" t="b">
@@ -5270,7 +5258,7 @@
           <t>6m</t>
         </is>
       </c>
-      <c r="J105" s="2" t="n">
+      <c r="J105" s="1" t="n">
         <v>46401</v>
       </c>
       <c r="K105" t="b">
@@ -5319,7 +5307,7 @@
           <t>6m</t>
         </is>
       </c>
-      <c r="J106" s="2" t="n">
+      <c r="J106" s="1" t="n">
         <v>46401</v>
       </c>
       <c r="K106" t="b">
@@ -5368,7 +5356,7 @@
           <t>6m</t>
         </is>
       </c>
-      <c r="J107" s="2" t="n">
+      <c r="J107" s="1" t="n">
         <v>46401</v>
       </c>
       <c r="K107" t="b">
@@ -5417,7 +5405,7 @@
           <t>6m</t>
         </is>
       </c>
-      <c r="J108" s="2" t="n">
+      <c r="J108" s="1" t="n">
         <v>46413</v>
       </c>
       <c r="K108" t="b">
@@ -5466,7 +5454,7 @@
           <t>7m</t>
         </is>
       </c>
-      <c r="J109" s="2" t="n">
+      <c r="J109" s="1" t="n">
         <v>46424</v>
       </c>
       <c r="K109" t="b">
@@ -5515,7 +5503,7 @@
           <t>7m</t>
         </is>
       </c>
-      <c r="J110" s="2" t="n">
+      <c r="J110" s="1" t="n">
         <v>46427</v>
       </c>
       <c r="K110" t="b">
@@ -5564,7 +5552,7 @@
           <t>7m</t>
         </is>
       </c>
-      <c r="J111" s="2" t="n">
+      <c r="J111" s="1" t="n">
         <v>46437</v>
       </c>
       <c r="K111" t="b">
@@ -5613,7 +5601,7 @@
           <t>7m</t>
         </is>
       </c>
-      <c r="J112" s="2" t="n">
+      <c r="J112" s="1" t="n">
         <v>46451</v>
       </c>
       <c r="K112" t="b">
@@ -5662,7 +5650,7 @@
           <t>8m</t>
         </is>
       </c>
-      <c r="J113" s="2" t="n">
+      <c r="J113" s="1" t="n">
         <v>46455</v>
       </c>
       <c r="K113" t="b">
@@ -5711,7 +5699,7 @@
           <t>8m</t>
         </is>
       </c>
-      <c r="J114" s="2" t="n">
+      <c r="J114" s="1" t="n">
         <v>46457</v>
       </c>
       <c r="K114" t="b">
@@ -5760,7 +5748,7 @@
           <t>8m</t>
         </is>
       </c>
-      <c r="J115" s="2" t="n">
+      <c r="J115" s="1" t="n">
         <v>46462</v>
       </c>
       <c r="K115" t="b">
@@ -5809,7 +5797,7 @@
           <t>8m</t>
         </is>
       </c>
-      <c r="J116" s="2" t="n">
+      <c r="J116" s="1" t="n">
         <v>46464</v>
       </c>
       <c r="K116" t="b">
@@ -5858,7 +5846,7 @@
           <t>8m</t>
         </is>
       </c>
-      <c r="J117" s="2" t="n">
+      <c r="J117" s="1" t="n">
         <v>46470</v>
       </c>
       <c r="K117" t="b">
@@ -5907,7 +5895,7 @@
           <t>9m</t>
         </is>
       </c>
-      <c r="J118" s="2" t="n">
+      <c r="J118" s="1" t="n">
         <v>46485</v>
       </c>
       <c r="K118" t="b">
@@ -5956,7 +5944,7 @@
           <t>9m</t>
         </is>
       </c>
-      <c r="J119" s="2" t="n">
+      <c r="J119" s="1" t="n">
         <v>46499</v>
       </c>
       <c r="K119" t="b">
@@ -6005,7 +5993,7 @@
           <t>9m</t>
         </is>
       </c>
-      <c r="J120" s="2" t="n">
+      <c r="J120" s="1" t="n">
         <v>46504</v>
       </c>
       <c r="K120" t="b">
@@ -6054,7 +6042,7 @@
           <t>9m</t>
         </is>
       </c>
-      <c r="J121" s="2" t="n">
+      <c r="J121" s="1" t="n">
         <v>46504</v>
       </c>
       <c r="K121" t="b">
@@ -6103,7 +6091,7 @@
           <t>9m</t>
         </is>
       </c>
-      <c r="J122" s="2" t="n">
+      <c r="J122" s="1" t="n">
         <v>46507</v>
       </c>
       <c r="K122" t="b">
@@ -6152,7 +6140,7 @@
           <t>9m</t>
         </is>
       </c>
-      <c r="J123" s="2" t="n">
+      <c r="J123" s="1" t="n">
         <v>46508</v>
       </c>
       <c r="K123" t="b">
@@ -6201,7 +6189,7 @@
           <t>9m</t>
         </is>
       </c>
-      <c r="J124" s="2" t="n">
+      <c r="J124" s="1" t="n">
         <v>46512</v>
       </c>
       <c r="K124" t="b">
@@ -6250,7 +6238,7 @@
           <t>9m</t>
         </is>
       </c>
-      <c r="J125" s="2" t="n">
+      <c r="J125" s="1" t="n">
         <v>46512</v>
       </c>
       <c r="K125" t="b">
@@ -6299,7 +6287,7 @@
           <t>10m</t>
         </is>
       </c>
-      <c r="J126" s="2" t="n">
+      <c r="J126" s="1" t="n">
         <v>46528</v>
       </c>
       <c r="K126" t="b">
@@ -6348,7 +6336,7 @@
           <t>10m</t>
         </is>
       </c>
-      <c r="J127" s="2" t="n">
+      <c r="J127" s="1" t="n">
         <v>46529</v>
       </c>
       <c r="K127" t="b">
@@ -6397,7 +6385,7 @@
           <t>10m</t>
         </is>
       </c>
-      <c r="J128" s="2" t="n">
+      <c r="J128" s="1" t="n">
         <v>46537</v>
       </c>
       <c r="K128" t="b">
@@ -6446,7 +6434,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J129" s="2" t="n">
+      <c r="J129" s="1" t="n">
         <v>46546</v>
       </c>
       <c r="K129" t="b">
@@ -6495,7 +6483,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J130" s="2" t="n">
+      <c r="J130" s="1" t="n">
         <v>46547</v>
       </c>
       <c r="K130" t="b">
@@ -6544,7 +6532,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J131" s="2" t="n">
+      <c r="J131" s="1" t="n">
         <v>46547</v>
       </c>
       <c r="K131" t="b">
@@ -6593,7 +6581,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J132" s="2" t="n">
+      <c r="J132" s="1" t="n">
         <v>46547</v>
       </c>
       <c r="K132" t="b">
@@ -6642,7 +6630,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J133" s="2" t="n">
+      <c r="J133" s="1" t="n">
         <v>46551</v>
       </c>
       <c r="K133" t="b">
@@ -6691,7 +6679,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J134" s="2" t="n">
+      <c r="J134" s="1" t="n">
         <v>46560</v>
       </c>
       <c r="K134" t="b">
@@ -6740,7 +6728,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J135" s="2" t="n">
+      <c r="J135" s="1" t="n">
         <v>46564</v>
       </c>
       <c r="K135" t="b">
@@ -6789,7 +6777,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J136" s="2" t="n">
+      <c r="J136" s="1" t="n">
         <v>46567</v>
       </c>
       <c r="K136" t="b">
@@ -6838,7 +6826,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J137" s="2" t="n">
+      <c r="J137" s="1" t="n">
         <v>46568</v>
       </c>
       <c r="K137" t="b">
@@ -6887,7 +6875,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J138" s="2" t="n">
+      <c r="J138" s="1" t="n">
         <v>46571</v>
       </c>
       <c r="K138" t="b">
@@ -6936,7 +6924,7 @@
           <t>-14d</t>
         </is>
       </c>
-      <c r="J139" s="2" t="n">
+      <c r="J139" s="1" t="n">
         <v>46197</v>
       </c>
       <c r="K139" t="b">
@@ -6985,7 +6973,7 @@
           <t>1d</t>
         </is>
       </c>
-      <c r="J140" s="2" t="n">
+      <c r="J140" s="1" t="n">
         <v>46212</v>
       </c>
       <c r="K140" t="b">
@@ -7034,7 +7022,7 @@
           <t>14d</t>
         </is>
       </c>
-      <c r="J141" s="2" t="n">
+      <c r="J141" s="1" t="n">
         <v>46225</v>
       </c>
       <c r="K141" t="b">
@@ -7083,7 +7071,7 @@
           <t>23d</t>
         </is>
       </c>
-      <c r="J142" s="2" t="n">
+      <c r="J142" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="K142" t="b">
@@ -7132,7 +7120,7 @@
           <t>24d</t>
         </is>
       </c>
-      <c r="J143" s="2" t="n">
+      <c r="J143" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="K143" t="b">
@@ -7181,7 +7169,7 @@
           <t>1me23d</t>
         </is>
       </c>
-      <c r="J144" s="2" t="n">
+      <c r="J144" s="1" t="n">
         <v>46263</v>
       </c>
       <c r="K144" t="b">
@@ -7230,7 +7218,7 @@
           <t>1me25d</t>
         </is>
       </c>
-      <c r="J145" s="2" t="n">
+      <c r="J145" s="1" t="n">
         <v>46266</v>
       </c>
       <c r="K145" t="b">
@@ -7275,7 +7263,7 @@
         <v>-1476</v>
       </c>
       <c r="I146" t="inlineStr"/>
-      <c r="J146" s="2" t="n">
+      <c r="J146" s="1" t="n">
         <v>43773</v>
       </c>
       <c r="K146" t="b">
@@ -7320,7 +7308,7 @@
         <v>-1469</v>
       </c>
       <c r="I147" t="inlineStr"/>
-      <c r="J147" s="2" t="n">
+      <c r="J147" s="1" t="n">
         <v>43773</v>
       </c>
       <c r="K147" t="b">
@@ -7365,7 +7353,7 @@
         <v>-1121</v>
       </c>
       <c r="I148" t="inlineStr"/>
-      <c r="J148" s="2" t="n">
+      <c r="J148" s="1" t="n">
         <v>45295</v>
       </c>
       <c r="K148" t="b">
@@ -7410,7 +7398,7 @@
         <v>-1018</v>
       </c>
       <c r="I149" t="inlineStr"/>
-      <c r="J149" s="2" t="n">
+      <c r="J149" s="1" t="n">
         <v>45617</v>
       </c>
       <c r="K149" t="b">
@@ -7455,7 +7443,7 @@
         <v>-950</v>
       </c>
       <c r="I150" t="inlineStr"/>
-      <c r="J150" s="2" t="n">
+      <c r="J150" s="1" t="n">
         <v>45677</v>
       </c>
       <c r="K150" t="b">
@@ -7500,7 +7488,7 @@
         <v>-943</v>
       </c>
       <c r="I151" t="inlineStr"/>
-      <c r="J151" s="2" t="n">
+      <c r="J151" s="1" t="n">
         <v>44944</v>
       </c>
       <c r="K151" t="b">
@@ -7545,7 +7533,7 @@
         <v>-252</v>
       </c>
       <c r="I152" t="inlineStr"/>
-      <c r="J152" s="2" t="n">
+      <c r="J152" s="1" t="n">
         <v>46092</v>
       </c>
       <c r="K152" t="b">
@@ -7590,7 +7578,7 @@
         <v>-196</v>
       </c>
       <c r="I153" t="inlineStr"/>
-      <c r="J153" s="2" t="n">
+      <c r="J153" s="1" t="n">
         <v>45988</v>
       </c>
       <c r="K153" t="b">
@@ -7635,7 +7623,7 @@
         <v>-196</v>
       </c>
       <c r="I154" t="inlineStr"/>
-      <c r="J154" s="2" t="n">
+      <c r="J154" s="1" t="n">
         <v>45988</v>
       </c>
       <c r="K154" t="b">
@@ -7680,7 +7668,7 @@
         <v>-47</v>
       </c>
       <c r="I155" t="inlineStr"/>
-      <c r="J155" s="2" t="n">
+      <c r="J155" s="1" t="n">
         <v>46176</v>
       </c>
       <c r="K155" t="b">
@@ -7725,7 +7713,7 @@
         <v>-47</v>
       </c>
       <c r="I156" t="inlineStr"/>
-      <c r="J156" s="2" t="n">
+      <c r="J156" s="1" t="n">
         <v>46176</v>
       </c>
       <c r="K156" t="b">
@@ -7770,7 +7758,7 @@
         <v>-33</v>
       </c>
       <c r="I157" t="inlineStr"/>
-      <c r="J157" s="2" t="n">
+      <c r="J157" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="K157" t="b">
@@ -7815,7 +7803,7 @@
         <v>-33</v>
       </c>
       <c r="I158" t="inlineStr"/>
-      <c r="J158" s="2" t="n">
+      <c r="J158" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="K158" t="b">
@@ -7860,7 +7848,7 @@
         <v>-6</v>
       </c>
       <c r="I159" t="inlineStr"/>
-      <c r="J159" s="2" t="n">
+      <c r="J159" s="1" t="n">
         <v>45967</v>
       </c>
       <c r="K159" t="b">
@@ -7905,7 +7893,7 @@
         <v>43</v>
       </c>
       <c r="I160" t="inlineStr"/>
-      <c r="J160" s="2" t="n">
+      <c r="J160" s="1" t="n">
         <v>46440</v>
       </c>
       <c r="K160" t="b">
@@ -7950,7 +7938,7 @@
         <v>43</v>
       </c>
       <c r="I161" t="inlineStr"/>
-      <c r="J161" s="2" t="n">
+      <c r="J161" s="1" t="n">
         <v>46440</v>
       </c>
       <c r="K161" t="b">
@@ -7995,7 +7983,7 @@
         <v>73</v>
       </c>
       <c r="I162" t="inlineStr"/>
-      <c r="J162" s="2" t="n">
+      <c r="J162" s="1" t="n">
         <v>46264</v>
       </c>
       <c r="K162" t="b">
@@ -8040,7 +8028,7 @@
         <v>73</v>
       </c>
       <c r="I163" t="inlineStr"/>
-      <c r="J163" s="2" t="n">
+      <c r="J163" s="1" t="n">
         <v>46264</v>
       </c>
       <c r="K163" t="b">
@@ -8085,7 +8073,7 @@
         <v>102</v>
       </c>
       <c r="I164" t="inlineStr"/>
-      <c r="J164" s="2" t="n">
+      <c r="J164" s="1" t="n">
         <v>46463</v>
       </c>
       <c r="K164" t="b">
@@ -8130,7 +8118,7 @@
         <v>118</v>
       </c>
       <c r="I165" t="inlineStr"/>
-      <c r="J165" s="2" t="n">
+      <c r="J165" s="1" t="n">
         <v>46337</v>
       </c>
       <c r="K165" t="b">
@@ -8175,7 +8163,7 @@
         <v>146</v>
       </c>
       <c r="I166" t="inlineStr"/>
-      <c r="J166" s="2" t="n">
+      <c r="J166" s="1" t="n">
         <v>46451</v>
       </c>
       <c r="K166" t="b">
@@ -8220,7 +8208,7 @@
         <v>152</v>
       </c>
       <c r="I167" t="inlineStr"/>
-      <c r="J167" s="2" t="n">
+      <c r="J167" s="1" t="n">
         <v>46245</v>
       </c>
       <c r="K167" t="b">
@@ -8265,7 +8253,7 @@
         <v>152</v>
       </c>
       <c r="I168" t="inlineStr"/>
-      <c r="J168" s="2" t="n">
+      <c r="J168" s="1" t="n">
         <v>46245</v>
       </c>
       <c r="K168" t="b">
@@ -8310,7 +8298,7 @@
         <v>163</v>
       </c>
       <c r="I169" t="inlineStr"/>
-      <c r="J169" s="2" t="n">
+      <c r="J169" s="1" t="n">
         <v>46324</v>
       </c>
       <c r="K169" t="b">
@@ -8355,7 +8343,7 @@
         <v>163</v>
       </c>
       <c r="I170" t="inlineStr"/>
-      <c r="J170" s="2" t="n">
+      <c r="J170" s="1" t="n">
         <v>46324</v>
       </c>
       <c r="K170" t="b">
@@ -8400,7 +8388,7 @@
         <v>164</v>
       </c>
       <c r="I171" t="inlineStr"/>
-      <c r="J171" s="2" t="n">
+      <c r="J171" s="1" t="n">
         <v>46426</v>
       </c>
       <c r="K171" t="b">
@@ -8445,7 +8433,7 @@
         <v>175</v>
       </c>
       <c r="I172" t="inlineStr"/>
-      <c r="J172" s="2" t="n">
+      <c r="J172" s="1" t="n">
         <v>46383</v>
       </c>
       <c r="K172" t="b">
@@ -8490,7 +8478,7 @@
         <v>186</v>
       </c>
       <c r="I173" t="inlineStr"/>
-      <c r="J173" s="2" t="n">
+      <c r="J173" s="1" t="n">
         <v>46392</v>
       </c>
       <c r="K173" t="b">
@@ -8535,7 +8523,7 @@
         <v>205</v>
       </c>
       <c r="I174" t="inlineStr"/>
-      <c r="J174" s="2" t="n">
+      <c r="J174" s="1" t="n">
         <v>46390</v>
       </c>
       <c r="K174" t="b">
@@ -8580,7 +8568,7 @@
         <v>207</v>
       </c>
       <c r="I175" t="inlineStr"/>
-      <c r="J175" s="2" t="n">
+      <c r="J175" s="1" t="n">
         <v>46392</v>
       </c>
       <c r="K175" t="b">
@@ -8625,7 +8613,7 @@
         <v>218</v>
       </c>
       <c r="I176" t="inlineStr"/>
-      <c r="J176" s="2" t="n">
+      <c r="J176" s="1" t="n">
         <v>46506</v>
       </c>
       <c r="K176" t="b">
@@ -8670,7 +8658,7 @@
         <v>246</v>
       </c>
       <c r="I177" t="inlineStr"/>
-      <c r="J177" s="2" t="n">
+      <c r="J177" s="1" t="n">
         <v>46478</v>
       </c>
       <c r="K177" t="b">
@@ -8715,7 +8703,7 @@
         <v>248</v>
       </c>
       <c r="I178" t="inlineStr"/>
-      <c r="J178" s="2" t="n">
+      <c r="J178" s="1" t="n">
         <v>46500</v>
       </c>
       <c r="K178" t="b">
@@ -8760,7 +8748,7 @@
         <v>276</v>
       </c>
       <c r="I179" t="inlineStr"/>
-      <c r="J179" s="2" t="n">
+      <c r="J179" s="1" t="n">
         <v>46430</v>
       </c>
       <c r="K179" t="b">
@@ -8805,7 +8793,7 @@
         <v>276</v>
       </c>
       <c r="I180" t="inlineStr"/>
-      <c r="J180" s="2" t="n">
+      <c r="J180" s="1" t="n">
         <v>46430</v>
       </c>
       <c r="K180" t="b">
@@ -8850,7 +8838,7 @@
         <v>290</v>
       </c>
       <c r="I181" t="inlineStr"/>
-      <c r="J181" s="2" t="n">
+      <c r="J181" s="1" t="n">
         <v>46467</v>
       </c>
       <c r="K181" t="b">
@@ -8895,7 +8883,7 @@
         <v>317</v>
       </c>
       <c r="I182" t="inlineStr"/>
-      <c r="J182" s="2" t="n">
+      <c r="J182" s="1" t="n">
         <v>46529</v>
       </c>
       <c r="K182" t="b">
@@ -8940,7 +8928,7 @@
         <v>420</v>
       </c>
       <c r="I183" t="inlineStr"/>
-      <c r="J183" s="2" t="n">
+      <c r="J183" s="1" t="n">
         <v>46566</v>
       </c>
       <c r="K183" t="b">
@@ -8985,7 +8973,7 @@
         <v>426</v>
       </c>
       <c r="I184" t="inlineStr"/>
-      <c r="J184" s="2" t="n">
+      <c r="J184" s="1" t="n">
         <v>46571</v>
       </c>
       <c r="K184" t="b">
@@ -9030,7 +9018,7 @@
         <v>721</v>
       </c>
       <c r="I185" t="inlineStr"/>
-      <c r="J185" s="2" t="n">
+      <c r="J185" s="1" t="n">
         <v>46325</v>
       </c>
       <c r="K185" t="b">
@@ -9075,7 +9063,7 @@
         <v>721</v>
       </c>
       <c r="I186" t="inlineStr"/>
-      <c r="J186" s="2" t="n">
+      <c r="J186" s="1" t="n">
         <v>46325</v>
       </c>
       <c r="K186" t="b">
@@ -9120,7 +9108,7 @@
         <v>850</v>
       </c>
       <c r="I187" t="inlineStr"/>
-      <c r="J187" s="2" t="n">
+      <c r="J187" s="1" t="n">
         <v>46345</v>
       </c>
       <c r="K187" t="b">
@@ -9165,7 +9153,7 @@
         <v>850</v>
       </c>
       <c r="I188" t="inlineStr"/>
-      <c r="J188" s="2" t="n">
+      <c r="J188" s="1" t="n">
         <v>46345</v>
       </c>
       <c r="K188" t="b">
@@ -9210,7 +9198,7 @@
         <v>1661</v>
       </c>
       <c r="I189" t="inlineStr"/>
-      <c r="J189" s="2" t="n">
+      <c r="J189" s="1" t="n">
         <v>46498</v>
       </c>
       <c r="K189" t="b">
@@ -9255,7 +9243,7 @@
         <v>1661</v>
       </c>
       <c r="I190" t="inlineStr"/>
-      <c r="J190" s="2" t="n">
+      <c r="J190" s="1" t="n">
         <v>46498</v>
       </c>
       <c r="K190" t="b">
@@ -9300,7 +9288,7 @@
         <v>488</v>
       </c>
       <c r="I191" t="inlineStr"/>
-      <c r="J191" s="2" t="n">
+      <c r="J191" s="1" t="n">
         <v>46190</v>
       </c>
       <c r="K191" t="b">
@@ -9345,7 +9333,7 @@
         <v>25565</v>
       </c>
       <c r="I192" t="inlineStr"/>
-      <c r="J192" s="2" t="n">
+      <c r="J192" s="1" t="n">
         <v>46190</v>
       </c>
       <c r="K192" t="b">
@@ -9390,7 +9378,7 @@
         <v>25567</v>
       </c>
       <c r="I193" t="inlineStr"/>
-      <c r="J193" s="2" t="n">
+      <c r="J193" s="1" t="n">
         <v>46190</v>
       </c>
       <c r="K193" t="b">
@@ -9435,7 +9423,7 @@
         <v>31293</v>
       </c>
       <c r="I194" t="inlineStr"/>
-      <c r="J194" s="2" t="n">
+      <c r="J194" s="1" t="n">
         <v>46190</v>
       </c>
       <c r="K194" t="b">

</xml_diff>

<commit_message>
Atualização automática: vencimentos_tmot (10/07/2026 20:00)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
@@ -20,13 +20,16 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +40,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,12 +48,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -421,57 +433,57 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>matricula</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>operador</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>pn</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>sn</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>nomenclatura</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>inspecao</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>tipo_vencimento</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>disponibilidade_valor</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>disponibilidade_texto</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>data_vencimento</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>vencido</t>
         </is>
@@ -515,7 +527,7 @@
         <v>-4402.8</v>
       </c>
       <c r="I2" t="inlineStr"/>
-      <c r="J2" s="1" t="n">
+      <c r="J2" s="2" t="n">
         <v>41388</v>
       </c>
       <c r="K2" t="b">
@@ -560,7 +572,7 @@
         <v>-4254.8</v>
       </c>
       <c r="I3" t="inlineStr"/>
-      <c r="J3" s="1" t="n">
+      <c r="J3" s="2" t="n">
         <v>39285</v>
       </c>
       <c r="K3" t="b">
@@ -605,7 +617,7 @@
         <v>-2354.2</v>
       </c>
       <c r="I4" t="inlineStr"/>
-      <c r="J4" s="1" t="n">
+      <c r="J4" s="2" t="n">
         <v>40669</v>
       </c>
       <c r="K4" t="b">
@@ -650,7 +662,7 @@
         <v>-896.8</v>
       </c>
       <c r="I5" t="inlineStr"/>
-      <c r="J5" s="1" t="n">
+      <c r="J5" s="2" t="n">
         <v>40669</v>
       </c>
       <c r="K5" t="b">
@@ -695,7 +707,7 @@
         <v>-854.1</v>
       </c>
       <c r="I6" t="inlineStr"/>
-      <c r="J6" s="1" t="n">
+      <c r="J6" s="2" t="n">
         <v>44884</v>
       </c>
       <c r="K6" t="b">
@@ -740,7 +752,7 @@
         <v>-413.2</v>
       </c>
       <c r="I7" t="inlineStr"/>
-      <c r="J7" s="1" t="n">
+      <c r="J7" s="2" t="n">
         <v>43855</v>
       </c>
       <c r="K7" t="b">
@@ -785,7 +797,7 @@
         <v>-391.8</v>
       </c>
       <c r="I8" t="inlineStr"/>
-      <c r="J8" s="1" t="n">
+      <c r="J8" s="2" t="n">
         <v>42769</v>
       </c>
       <c r="K8" t="b">
@@ -830,7 +842,7 @@
         <v>-371.5</v>
       </c>
       <c r="I9" t="inlineStr"/>
-      <c r="J9" s="1" t="n">
+      <c r="J9" s="2" t="n">
         <v>46014</v>
       </c>
       <c r="K9" t="b">
@@ -875,7 +887,7 @@
         <v>-368.8</v>
       </c>
       <c r="I10" t="inlineStr"/>
-      <c r="J10" s="1" t="n">
+      <c r="J10" s="2" t="n">
         <v>46014</v>
       </c>
       <c r="K10" t="b">
@@ -920,7 +932,7 @@
         <v>-359</v>
       </c>
       <c r="I11" t="inlineStr"/>
-      <c r="J11" s="1" t="n">
+      <c r="J11" s="2" t="n">
         <v>45804</v>
       </c>
       <c r="K11" t="b">
@@ -965,7 +977,7 @@
         <v>-359</v>
       </c>
       <c r="I12" t="inlineStr"/>
-      <c r="J12" s="1" t="n">
+      <c r="J12" s="2" t="n">
         <v>45804</v>
       </c>
       <c r="K12" t="b">
@@ -1010,7 +1022,7 @@
         <v>-351</v>
       </c>
       <c r="I13" t="inlineStr"/>
-      <c r="J13" s="1" t="n">
+      <c r="J13" s="2" t="n">
         <v>42821</v>
       </c>
       <c r="K13" t="b">
@@ -1055,7 +1067,7 @@
         <v>-351</v>
       </c>
       <c r="I14" t="inlineStr"/>
-      <c r="J14" s="1" t="n">
+      <c r="J14" s="2" t="n">
         <v>46014</v>
       </c>
       <c r="K14" t="b">
@@ -1100,7 +1112,7 @@
         <v>-351</v>
       </c>
       <c r="I15" t="inlineStr"/>
-      <c r="J15" s="1" t="n">
+      <c r="J15" s="2" t="n">
         <v>46014</v>
       </c>
       <c r="K15" t="b">
@@ -1145,7 +1157,7 @@
         <v>-351</v>
       </c>
       <c r="I16" t="inlineStr"/>
-      <c r="J16" s="1" t="n">
+      <c r="J16" s="2" t="n">
         <v>46014</v>
       </c>
       <c r="K16" t="b">
@@ -1190,7 +1202,7 @@
         <v>-345.8</v>
       </c>
       <c r="I17" t="inlineStr"/>
-      <c r="J17" s="1" t="n">
+      <c r="J17" s="2" t="n">
         <v>46017</v>
       </c>
       <c r="K17" t="b">
@@ -1235,7 +1247,7 @@
         <v>-345.8</v>
       </c>
       <c r="I18" t="inlineStr"/>
-      <c r="J18" s="1" t="n">
+      <c r="J18" s="2" t="n">
         <v>46017</v>
       </c>
       <c r="K18" t="b">
@@ -1280,7 +1292,7 @@
         <v>-264.2</v>
       </c>
       <c r="I19" t="inlineStr"/>
-      <c r="J19" s="1" t="n">
+      <c r="J19" s="2" t="n">
         <v>40979</v>
       </c>
       <c r="K19" t="b">
@@ -1325,7 +1337,7 @@
         <v>-206.4</v>
       </c>
       <c r="I20" t="inlineStr"/>
-      <c r="J20" s="1" t="n">
+      <c r="J20" s="2" t="n">
         <v>36669</v>
       </c>
       <c r="K20" t="b">
@@ -1370,7 +1382,7 @@
         <v>-131.6</v>
       </c>
       <c r="I21" t="inlineStr"/>
-      <c r="J21" s="1" t="n">
+      <c r="J21" s="2" t="n">
         <v>46111</v>
       </c>
       <c r="K21" t="b">
@@ -1415,7 +1427,7 @@
         <v>-131.6</v>
       </c>
       <c r="I22" t="inlineStr"/>
-      <c r="J22" s="1" t="n">
+      <c r="J22" s="2" t="n">
         <v>46111</v>
       </c>
       <c r="K22" t="b">
@@ -1460,7 +1472,7 @@
         <v>-131.6</v>
       </c>
       <c r="I23" t="inlineStr"/>
-      <c r="J23" s="1" t="n">
+      <c r="J23" s="2" t="n">
         <v>46111</v>
       </c>
       <c r="K23" t="b">
@@ -1505,7 +1517,7 @@
         <v>-131.6</v>
       </c>
       <c r="I24" t="inlineStr"/>
-      <c r="J24" s="1" t="n">
+      <c r="J24" s="2" t="n">
         <v>46111</v>
       </c>
       <c r="K24" t="b">
@@ -1550,7 +1562,7 @@
         <v>-131.6</v>
       </c>
       <c r="I25" t="inlineStr"/>
-      <c r="J25" s="1" t="n">
+      <c r="J25" s="2" t="n">
         <v>46111</v>
       </c>
       <c r="K25" t="b">
@@ -1595,7 +1607,7 @@
         <v>-105</v>
       </c>
       <c r="I26" t="inlineStr"/>
-      <c r="J26" s="1" t="n">
+      <c r="J26" s="2" t="n">
         <v>46161</v>
       </c>
       <c r="K26" t="b">
@@ -1640,7 +1652,7 @@
         <v>-79.8</v>
       </c>
       <c r="I27" t="inlineStr"/>
-      <c r="J27" s="1" t="n">
+      <c r="J27" s="2" t="n">
         <v>43340</v>
       </c>
       <c r="K27" t="b">
@@ -1685,7 +1697,7 @@
         <v>-12.3</v>
       </c>
       <c r="I28" t="inlineStr"/>
-      <c r="J28" s="1" t="n">
+      <c r="J28" s="2" t="n">
         <v>46048</v>
       </c>
       <c r="K28" t="b">
@@ -1730,7 +1742,7 @@
         <v>0</v>
       </c>
       <c r="I29" t="inlineStr"/>
-      <c r="J29" s="1" t="n">
+      <c r="J29" s="2" t="n">
         <v>46211</v>
       </c>
       <c r="K29" t="b">
@@ -1775,7 +1787,7 @@
         <v>3.6</v>
       </c>
       <c r="I30" t="inlineStr"/>
-      <c r="J30" s="1" t="n">
+      <c r="J30" s="2" t="n">
         <v>46234</v>
       </c>
       <c r="K30" t="b">
@@ -1820,7 +1832,7 @@
         <v>6.2</v>
       </c>
       <c r="I31" t="inlineStr"/>
-      <c r="J31" s="1" t="n">
+      <c r="J31" s="2" t="n">
         <v>46234</v>
       </c>
       <c r="K31" t="b">
@@ -1865,7 +1877,7 @@
         <v>7.5</v>
       </c>
       <c r="I32" t="inlineStr"/>
-      <c r="J32" s="1" t="n">
+      <c r="J32" s="2" t="n">
         <v>46234</v>
       </c>
       <c r="K32" t="b">
@@ -1910,7 +1922,7 @@
         <v>10.7</v>
       </c>
       <c r="I33" t="inlineStr"/>
-      <c r="J33" s="1" t="n">
+      <c r="J33" s="2" t="n">
         <v>46234</v>
       </c>
       <c r="K33" t="b">
@@ -1955,7 +1967,7 @@
         <v>20</v>
       </c>
       <c r="I34" t="inlineStr"/>
-      <c r="J34" s="1" t="n">
+      <c r="J34" s="2" t="n">
         <v>46234</v>
       </c>
       <c r="K34" t="b">
@@ -2000,7 +2012,7 @@
         <v>30.8</v>
       </c>
       <c r="I35" t="inlineStr"/>
-      <c r="J35" s="1" t="n">
+      <c r="J35" s="2" t="n">
         <v>46234</v>
       </c>
       <c r="K35" t="b">
@@ -2045,7 +2057,7 @@
         <v>37.1</v>
       </c>
       <c r="I36" t="inlineStr"/>
-      <c r="J36" s="1" t="n">
+      <c r="J36" s="2" t="n">
         <v>46256</v>
       </c>
       <c r="K36" t="b">
@@ -2090,7 +2102,7 @@
         <v>42.8</v>
       </c>
       <c r="I37" t="inlineStr"/>
-      <c r="J37" s="1" t="n">
+      <c r="J37" s="2" t="n">
         <v>46276</v>
       </c>
       <c r="K37" t="b">
@@ -2135,7 +2147,7 @@
         <v>45.2</v>
       </c>
       <c r="I38" t="inlineStr"/>
-      <c r="J38" s="1" t="n">
+      <c r="J38" s="2" t="n">
         <v>46234</v>
       </c>
       <c r="K38" t="b">
@@ -2180,7 +2192,7 @@
         <v>46</v>
       </c>
       <c r="I39" t="inlineStr"/>
-      <c r="J39" s="1" t="n">
+      <c r="J39" s="2" t="n">
         <v>46251</v>
       </c>
       <c r="K39" t="b">
@@ -2225,7 +2237,7 @@
         <v>47.5</v>
       </c>
       <c r="I40" t="inlineStr"/>
-      <c r="J40" s="1" t="n">
+      <c r="J40" s="2" t="n">
         <v>46456</v>
       </c>
       <c r="K40" t="b">
@@ -2270,7 +2282,7 @@
         <v>57.2</v>
       </c>
       <c r="I41" t="inlineStr"/>
-      <c r="J41" s="1" t="n">
+      <c r="J41" s="2" t="n">
         <v>46246</v>
       </c>
       <c r="K41" t="b">
@@ -2315,7 +2327,7 @@
         <v>59.6</v>
       </c>
       <c r="I42" t="inlineStr"/>
-      <c r="J42" s="1" t="n">
+      <c r="J42" s="2" t="n">
         <v>46487</v>
       </c>
       <c r="K42" t="b">
@@ -2360,7 +2372,7 @@
         <v>75.40000000000001</v>
       </c>
       <c r="I43" t="inlineStr"/>
-      <c r="J43" s="1" t="n">
+      <c r="J43" s="2" t="n">
         <v>46283</v>
       </c>
       <c r="K43" t="b">
@@ -2405,7 +2417,7 @@
         <v>76.8</v>
       </c>
       <c r="I44" t="inlineStr"/>
-      <c r="J44" s="1" t="n">
+      <c r="J44" s="2" t="n">
         <v>46285</v>
       </c>
       <c r="K44" t="b">
@@ -2450,7 +2462,7 @@
         <v>83.2</v>
       </c>
       <c r="I45" t="inlineStr"/>
-      <c r="J45" s="1" t="n">
+      <c r="J45" s="2" t="n">
         <v>46547</v>
       </c>
       <c r="K45" t="b">
@@ -2495,7 +2507,7 @@
         <v>84.5</v>
       </c>
       <c r="I46" t="inlineStr"/>
-      <c r="J46" s="1" t="n">
+      <c r="J46" s="2" t="n">
         <v>46240</v>
       </c>
       <c r="K46" t="b">
@@ -2540,7 +2552,7 @@
         <v>85.8</v>
       </c>
       <c r="I47" t="inlineStr"/>
-      <c r="J47" s="1" t="n">
+      <c r="J47" s="2" t="n">
         <v>46266</v>
       </c>
       <c r="K47" t="b">
@@ -2585,7 +2597,7 @@
         <v>86.5</v>
       </c>
       <c r="I48" t="inlineStr"/>
-      <c r="J48" s="1" t="n">
+      <c r="J48" s="2" t="n">
         <v>46241</v>
       </c>
       <c r="K48" t="b">
@@ -2630,7 +2642,7 @@
         <v>91.7</v>
       </c>
       <c r="I49" t="inlineStr"/>
-      <c r="J49" s="1" t="n">
+      <c r="J49" s="2" t="n">
         <v>46243</v>
       </c>
       <c r="K49" t="b">
@@ -2675,7 +2687,7 @@
         <v>91.7</v>
       </c>
       <c r="I50" t="inlineStr"/>
-      <c r="J50" s="1" t="n">
+      <c r="J50" s="2" t="n">
         <v>46243</v>
       </c>
       <c r="K50" t="b">
@@ -2720,7 +2732,7 @@
         <v>91.7</v>
       </c>
       <c r="I51" t="inlineStr"/>
-      <c r="J51" s="1" t="n">
+      <c r="J51" s="2" t="n">
         <v>46250</v>
       </c>
       <c r="K51" t="b">
@@ -2765,7 +2777,7 @@
         <v>98.90000000000001</v>
       </c>
       <c r="I52" t="inlineStr"/>
-      <c r="J52" s="1" t="n">
+      <c r="J52" s="2" t="n">
         <v>46253</v>
       </c>
       <c r="K52" t="b">
@@ -2810,7 +2822,7 @@
         <v>105.5</v>
       </c>
       <c r="I53" t="inlineStr"/>
-      <c r="J53" s="1" t="n">
+      <c r="J53" s="2" t="n">
         <v>46280</v>
       </c>
       <c r="K53" t="b">
@@ -2855,7 +2867,7 @@
         <v>105.6</v>
       </c>
       <c r="I54" t="inlineStr"/>
-      <c r="J54" s="1" t="n">
+      <c r="J54" s="2" t="n">
         <v>46361</v>
       </c>
       <c r="K54" t="b">
@@ -2900,7 +2912,7 @@
         <v>105.7</v>
       </c>
       <c r="I55" t="inlineStr"/>
-      <c r="J55" s="1" t="n">
+      <c r="J55" s="2" t="n">
         <v>46362</v>
       </c>
       <c r="K55" t="b">
@@ -2945,7 +2957,7 @@
         <v>110.7</v>
       </c>
       <c r="I56" t="inlineStr"/>
-      <c r="J56" s="1" t="n">
+      <c r="J56" s="2" t="n">
         <v>46275</v>
       </c>
       <c r="K56" t="b">
@@ -2990,7 +3002,7 @@
         <v>113.2</v>
       </c>
       <c r="I57" t="inlineStr"/>
-      <c r="J57" s="1" t="n">
+      <c r="J57" s="2" t="n">
         <v>46377</v>
       </c>
       <c r="K57" t="b">
@@ -3035,7 +3047,7 @@
         <v>128.8</v>
       </c>
       <c r="I58" t="inlineStr"/>
-      <c r="J58" s="1" t="n">
+      <c r="J58" s="2" t="n">
         <v>46434</v>
       </c>
       <c r="K58" t="b">
@@ -3080,7 +3092,7 @@
         <v>128.8</v>
       </c>
       <c r="I59" t="inlineStr"/>
-      <c r="J59" s="1" t="n">
+      <c r="J59" s="2" t="n">
         <v>46434</v>
       </c>
       <c r="K59" t="b">
@@ -3125,7 +3137,7 @@
         <v>128.8</v>
       </c>
       <c r="I60" t="inlineStr"/>
-      <c r="J60" s="1" t="n">
+      <c r="J60" s="2" t="n">
         <v>46434</v>
       </c>
       <c r="K60" t="b">
@@ -3170,7 +3182,7 @@
         <v>128.8</v>
       </c>
       <c r="I61" t="inlineStr"/>
-      <c r="J61" s="1" t="n">
+      <c r="J61" s="2" t="n">
         <v>46434</v>
       </c>
       <c r="K61" t="b">
@@ -3215,7 +3227,7 @@
         <v>128.8</v>
       </c>
       <c r="I62" t="inlineStr"/>
-      <c r="J62" s="1" t="n">
+      <c r="J62" s="2" t="n">
         <v>46434</v>
       </c>
       <c r="K62" t="b">
@@ -3260,7 +3272,7 @@
         <v>135</v>
       </c>
       <c r="I63" t="inlineStr"/>
-      <c r="J63" s="1" t="n">
+      <c r="J63" s="2" t="n">
         <v>46280</v>
       </c>
       <c r="K63" t="b">
@@ -3305,7 +3317,7 @@
         <v>150.6</v>
       </c>
       <c r="I64" t="inlineStr"/>
-      <c r="J64" s="1" t="n">
+      <c r="J64" s="2" t="n">
         <v>46271</v>
       </c>
       <c r="K64" t="b">
@@ -3350,7 +3362,7 @@
         <v>174.2</v>
       </c>
       <c r="I65" t="inlineStr"/>
-      <c r="J65" s="1" t="n">
+      <c r="J65" s="2" t="n">
         <v>46363</v>
       </c>
       <c r="K65" t="b">
@@ -3395,7 +3407,7 @@
         <v>176.6</v>
       </c>
       <c r="I66" t="inlineStr"/>
-      <c r="J66" s="1" t="n">
+      <c r="J66" s="2" t="n">
         <v>46334</v>
       </c>
       <c r="K66" t="b">
@@ -3440,7 +3452,7 @@
         <v>177.4</v>
       </c>
       <c r="I67" t="inlineStr"/>
-      <c r="J67" s="1" t="n">
+      <c r="J67" s="2" t="n">
         <v>46407</v>
       </c>
       <c r="K67" t="b">
@@ -3485,7 +3497,7 @@
         <v>183.9</v>
       </c>
       <c r="I68" t="inlineStr"/>
-      <c r="J68" s="1" t="n">
+      <c r="J68" s="2" t="n">
         <v>46341</v>
       </c>
       <c r="K68" t="b">
@@ -3530,7 +3542,7 @@
         <v>191.7</v>
       </c>
       <c r="I69" t="inlineStr"/>
-      <c r="J69" s="1" t="n">
+      <c r="J69" s="2" t="n">
         <v>46300</v>
       </c>
       <c r="K69" t="b">
@@ -3575,7 +3587,7 @@
         <v>200</v>
       </c>
       <c r="I70" t="inlineStr"/>
-      <c r="J70" s="1" t="n">
+      <c r="J70" s="2" t="n">
         <v>46336</v>
       </c>
       <c r="K70" t="b">
@@ -3620,7 +3632,7 @@
         <v>201.1</v>
       </c>
       <c r="I71" t="inlineStr"/>
-      <c r="J71" s="1" t="n">
+      <c r="J71" s="2" t="n">
         <v>46319</v>
       </c>
       <c r="K71" t="b">
@@ -3665,7 +3677,7 @@
         <v>206.5</v>
       </c>
       <c r="I72" t="inlineStr"/>
-      <c r="J72" s="1" t="n">
+      <c r="J72" s="2" t="n">
         <v>46308</v>
       </c>
       <c r="K72" t="b">
@@ -3710,7 +3722,7 @@
         <v>207.5</v>
       </c>
       <c r="I73" t="inlineStr"/>
-      <c r="J73" s="1" t="n">
+      <c r="J73" s="2" t="n">
         <v>46390</v>
       </c>
       <c r="K73" t="b">
@@ -3755,7 +3767,7 @@
         <v>247</v>
       </c>
       <c r="I74" t="inlineStr"/>
-      <c r="J74" s="1" t="n">
+      <c r="J74" s="2" t="n">
         <v>46443</v>
       </c>
       <c r="K74" t="b">
@@ -3800,7 +3812,7 @@
         <v>285.3</v>
       </c>
       <c r="I75" t="inlineStr"/>
-      <c r="J75" s="1" t="n">
+      <c r="J75" s="2" t="n">
         <v>46304</v>
       </c>
       <c r="K75" t="b">
@@ -3845,7 +3857,7 @@
         <v>290.8</v>
       </c>
       <c r="I76" t="inlineStr"/>
-      <c r="J76" s="1" t="n">
+      <c r="J76" s="2" t="n">
         <v>46362</v>
       </c>
       <c r="K76" t="b">
@@ -3890,7 +3902,7 @@
         <v>295.2</v>
       </c>
       <c r="I77" t="inlineStr"/>
-      <c r="J77" s="1" t="n">
+      <c r="J77" s="2" t="n">
         <v>46463</v>
       </c>
       <c r="K77" t="b">
@@ -3935,7 +3947,7 @@
         <v>300.2</v>
       </c>
       <c r="I78" t="inlineStr"/>
-      <c r="J78" s="1" t="n">
+      <c r="J78" s="2" t="n">
         <v>46466</v>
       </c>
       <c r="K78" t="b">
@@ -3984,7 +3996,7 @@
           <t>-317m</t>
         </is>
       </c>
-      <c r="J79" s="1" t="n">
+      <c r="J79" s="2" t="n">
         <v>36557</v>
       </c>
       <c r="K79" t="b">
@@ -4033,7 +4045,7 @@
           <t>-164m</t>
         </is>
       </c>
-      <c r="J80" s="1" t="n">
+      <c r="J80" s="2" t="n">
         <v>41275</v>
       </c>
       <c r="K80" t="b">
@@ -4082,7 +4094,7 @@
           <t>-27m</t>
         </is>
       </c>
-      <c r="J81" s="1" t="n">
+      <c r="J81" s="2" t="n">
         <v>45380</v>
       </c>
       <c r="K81" t="b">
@@ -4131,7 +4143,7 @@
           <t>-25m</t>
         </is>
       </c>
-      <c r="J82" s="1" t="n">
+      <c r="J82" s="2" t="n">
         <v>45421</v>
       </c>
       <c r="K82" t="b">
@@ -4180,7 +4192,7 @@
           <t>-25m</t>
         </is>
       </c>
-      <c r="J83" s="1" t="n">
+      <c r="J83" s="2" t="n">
         <v>45428</v>
       </c>
       <c r="K83" t="b">
@@ -4229,7 +4241,7 @@
           <t>-23m</t>
         </is>
       </c>
-      <c r="J84" s="1" t="n">
+      <c r="J84" s="2" t="n">
         <v>45490</v>
       </c>
       <c r="K84" t="b">
@@ -4278,7 +4290,7 @@
           <t>-21m</t>
         </is>
       </c>
-      <c r="J85" s="1" t="n">
+      <c r="J85" s="2" t="n">
         <v>45566</v>
       </c>
       <c r="K85" t="b">
@@ -4327,7 +4339,7 @@
           <t>-7m</t>
         </is>
       </c>
-      <c r="J86" s="1" t="n">
+      <c r="J86" s="2" t="n">
         <v>45986</v>
       </c>
       <c r="K86" t="b">
@@ -4376,7 +4388,7 @@
           <t>-3m</t>
         </is>
       </c>
-      <c r="J87" s="1" t="n">
+      <c r="J87" s="2" t="n">
         <v>46106</v>
       </c>
       <c r="K87" t="b">
@@ -4425,7 +4437,7 @@
           <t>-2m</t>
         </is>
       </c>
-      <c r="J88" s="1" t="n">
+      <c r="J88" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="K88" t="b">
@@ -4474,7 +4486,7 @@
           <t>2m</t>
         </is>
       </c>
-      <c r="J89" s="1" t="n">
+      <c r="J89" s="2" t="n">
         <v>46274</v>
       </c>
       <c r="K89" t="b">
@@ -4523,7 +4535,7 @@
           <t>2m</t>
         </is>
       </c>
-      <c r="J90" s="1" t="n">
+      <c r="J90" s="2" t="n">
         <v>46276</v>
       </c>
       <c r="K90" t="b">
@@ -4572,7 +4584,7 @@
           <t>2m</t>
         </is>
       </c>
-      <c r="J91" s="1" t="n">
+      <c r="J91" s="2" t="n">
         <v>46284</v>
       </c>
       <c r="K91" t="b">
@@ -4621,7 +4633,7 @@
           <t>3m</t>
         </is>
       </c>
-      <c r="J92" s="1" t="n">
+      <c r="J92" s="2" t="n">
         <v>46317</v>
       </c>
       <c r="K92" t="b">
@@ -4670,7 +4682,7 @@
           <t>3m</t>
         </is>
       </c>
-      <c r="J93" s="1" t="n">
+      <c r="J93" s="2" t="n">
         <v>46319</v>
       </c>
       <c r="K93" t="b">
@@ -4719,7 +4731,7 @@
           <t>4m</t>
         </is>
       </c>
-      <c r="J94" s="1" t="n">
+      <c r="J94" s="2" t="n">
         <v>46333</v>
       </c>
       <c r="K94" t="b">
@@ -4768,7 +4780,7 @@
           <t>4m</t>
         </is>
       </c>
-      <c r="J95" s="1" t="n">
+      <c r="J95" s="2" t="n">
         <v>46338</v>
       </c>
       <c r="K95" t="b">
@@ -4817,7 +4829,7 @@
           <t>4m</t>
         </is>
       </c>
-      <c r="J96" s="1" t="n">
+      <c r="J96" s="2" t="n">
         <v>46338</v>
       </c>
       <c r="K96" t="b">
@@ -4866,7 +4878,7 @@
           <t>4m</t>
         </is>
       </c>
-      <c r="J97" s="1" t="n">
+      <c r="J97" s="2" t="n">
         <v>46341</v>
       </c>
       <c r="K97" t="b">
@@ -4915,7 +4927,7 @@
           <t>4m</t>
         </is>
       </c>
-      <c r="J98" s="1" t="n">
+      <c r="J98" s="2" t="n">
         <v>46344</v>
       </c>
       <c r="K98" t="b">
@@ -4964,7 +4976,7 @@
           <t>4m</t>
         </is>
       </c>
-      <c r="J99" s="1" t="n">
+      <c r="J99" s="2" t="n">
         <v>46354</v>
       </c>
       <c r="K99" t="b">
@@ -5013,7 +5025,7 @@
           <t>4m</t>
         </is>
       </c>
-      <c r="J100" s="1" t="n">
+      <c r="J100" s="2" t="n">
         <v>46360</v>
       </c>
       <c r="K100" t="b">
@@ -5062,7 +5074,7 @@
           <t>4m</t>
         </is>
       </c>
-      <c r="J101" s="1" t="n">
+      <c r="J101" s="2" t="n">
         <v>46360</v>
       </c>
       <c r="K101" t="b">
@@ -5111,7 +5123,7 @@
           <t>5m</t>
         </is>
       </c>
-      <c r="J102" s="1" t="n">
+      <c r="J102" s="2" t="n">
         <v>46366</v>
       </c>
       <c r="K102" t="b">
@@ -5160,7 +5172,7 @@
           <t>5m</t>
         </is>
       </c>
-      <c r="J103" s="1" t="n">
+      <c r="J103" s="2" t="n">
         <v>46375</v>
       </c>
       <c r="K103" t="b">
@@ -5209,7 +5221,7 @@
           <t>5m</t>
         </is>
       </c>
-      <c r="J104" s="1" t="n">
+      <c r="J104" s="2" t="n">
         <v>46388</v>
       </c>
       <c r="K104" t="b">
@@ -5258,7 +5270,7 @@
           <t>6m</t>
         </is>
       </c>
-      <c r="J105" s="1" t="n">
+      <c r="J105" s="2" t="n">
         <v>46401</v>
       </c>
       <c r="K105" t="b">
@@ -5307,7 +5319,7 @@
           <t>6m</t>
         </is>
       </c>
-      <c r="J106" s="1" t="n">
+      <c r="J106" s="2" t="n">
         <v>46401</v>
       </c>
       <c r="K106" t="b">
@@ -5356,7 +5368,7 @@
           <t>6m</t>
         </is>
       </c>
-      <c r="J107" s="1" t="n">
+      <c r="J107" s="2" t="n">
         <v>46401</v>
       </c>
       <c r="K107" t="b">
@@ -5405,7 +5417,7 @@
           <t>6m</t>
         </is>
       </c>
-      <c r="J108" s="1" t="n">
+      <c r="J108" s="2" t="n">
         <v>46413</v>
       </c>
       <c r="K108" t="b">
@@ -5454,7 +5466,7 @@
           <t>7m</t>
         </is>
       </c>
-      <c r="J109" s="1" t="n">
+      <c r="J109" s="2" t="n">
         <v>46424</v>
       </c>
       <c r="K109" t="b">
@@ -5503,7 +5515,7 @@
           <t>7m</t>
         </is>
       </c>
-      <c r="J110" s="1" t="n">
+      <c r="J110" s="2" t="n">
         <v>46427</v>
       </c>
       <c r="K110" t="b">
@@ -5552,7 +5564,7 @@
           <t>7m</t>
         </is>
       </c>
-      <c r="J111" s="1" t="n">
+      <c r="J111" s="2" t="n">
         <v>46437</v>
       </c>
       <c r="K111" t="b">
@@ -5601,7 +5613,7 @@
           <t>7m</t>
         </is>
       </c>
-      <c r="J112" s="1" t="n">
+      <c r="J112" s="2" t="n">
         <v>46451</v>
       </c>
       <c r="K112" t="b">
@@ -5650,7 +5662,7 @@
           <t>8m</t>
         </is>
       </c>
-      <c r="J113" s="1" t="n">
+      <c r="J113" s="2" t="n">
         <v>46455</v>
       </c>
       <c r="K113" t="b">
@@ -5699,7 +5711,7 @@
           <t>8m</t>
         </is>
       </c>
-      <c r="J114" s="1" t="n">
+      <c r="J114" s="2" t="n">
         <v>46457</v>
       </c>
       <c r="K114" t="b">
@@ -5748,7 +5760,7 @@
           <t>8m</t>
         </is>
       </c>
-      <c r="J115" s="1" t="n">
+      <c r="J115" s="2" t="n">
         <v>46462</v>
       </c>
       <c r="K115" t="b">
@@ -5797,7 +5809,7 @@
           <t>8m</t>
         </is>
       </c>
-      <c r="J116" s="1" t="n">
+      <c r="J116" s="2" t="n">
         <v>46464</v>
       </c>
       <c r="K116" t="b">
@@ -5846,7 +5858,7 @@
           <t>8m</t>
         </is>
       </c>
-      <c r="J117" s="1" t="n">
+      <c r="J117" s="2" t="n">
         <v>46470</v>
       </c>
       <c r="K117" t="b">
@@ -5895,7 +5907,7 @@
           <t>9m</t>
         </is>
       </c>
-      <c r="J118" s="1" t="n">
+      <c r="J118" s="2" t="n">
         <v>46485</v>
       </c>
       <c r="K118" t="b">
@@ -5944,7 +5956,7 @@
           <t>9m</t>
         </is>
       </c>
-      <c r="J119" s="1" t="n">
+      <c r="J119" s="2" t="n">
         <v>46499</v>
       </c>
       <c r="K119" t="b">
@@ -5993,7 +6005,7 @@
           <t>9m</t>
         </is>
       </c>
-      <c r="J120" s="1" t="n">
+      <c r="J120" s="2" t="n">
         <v>46504</v>
       </c>
       <c r="K120" t="b">
@@ -6042,7 +6054,7 @@
           <t>9m</t>
         </is>
       </c>
-      <c r="J121" s="1" t="n">
+      <c r="J121" s="2" t="n">
         <v>46504</v>
       </c>
       <c r="K121" t="b">
@@ -6091,7 +6103,7 @@
           <t>9m</t>
         </is>
       </c>
-      <c r="J122" s="1" t="n">
+      <c r="J122" s="2" t="n">
         <v>46507</v>
       </c>
       <c r="K122" t="b">
@@ -6140,7 +6152,7 @@
           <t>9m</t>
         </is>
       </c>
-      <c r="J123" s="1" t="n">
+      <c r="J123" s="2" t="n">
         <v>46508</v>
       </c>
       <c r="K123" t="b">
@@ -6189,7 +6201,7 @@
           <t>9m</t>
         </is>
       </c>
-      <c r="J124" s="1" t="n">
+      <c r="J124" s="2" t="n">
         <v>46512</v>
       </c>
       <c r="K124" t="b">
@@ -6238,7 +6250,7 @@
           <t>9m</t>
         </is>
       </c>
-      <c r="J125" s="1" t="n">
+      <c r="J125" s="2" t="n">
         <v>46512</v>
       </c>
       <c r="K125" t="b">
@@ -6287,7 +6299,7 @@
           <t>10m</t>
         </is>
       </c>
-      <c r="J126" s="1" t="n">
+      <c r="J126" s="2" t="n">
         <v>46528</v>
       </c>
       <c r="K126" t="b">
@@ -6336,7 +6348,7 @@
           <t>10m</t>
         </is>
       </c>
-      <c r="J127" s="1" t="n">
+      <c r="J127" s="2" t="n">
         <v>46529</v>
       </c>
       <c r="K127" t="b">
@@ -6385,7 +6397,7 @@
           <t>10m</t>
         </is>
       </c>
-      <c r="J128" s="1" t="n">
+      <c r="J128" s="2" t="n">
         <v>46537</v>
       </c>
       <c r="K128" t="b">
@@ -6434,7 +6446,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J129" s="1" t="n">
+      <c r="J129" s="2" t="n">
         <v>46546</v>
       </c>
       <c r="K129" t="b">
@@ -6483,7 +6495,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J130" s="1" t="n">
+      <c r="J130" s="2" t="n">
         <v>46547</v>
       </c>
       <c r="K130" t="b">
@@ -6532,7 +6544,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J131" s="1" t="n">
+      <c r="J131" s="2" t="n">
         <v>46547</v>
       </c>
       <c r="K131" t="b">
@@ -6581,7 +6593,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J132" s="1" t="n">
+      <c r="J132" s="2" t="n">
         <v>46547</v>
       </c>
       <c r="K132" t="b">
@@ -6630,7 +6642,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J133" s="1" t="n">
+      <c r="J133" s="2" t="n">
         <v>46551</v>
       </c>
       <c r="K133" t="b">
@@ -6679,7 +6691,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J134" s="1" t="n">
+      <c r="J134" s="2" t="n">
         <v>46560</v>
       </c>
       <c r="K134" t="b">
@@ -6728,7 +6740,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J135" s="1" t="n">
+      <c r="J135" s="2" t="n">
         <v>46564</v>
       </c>
       <c r="K135" t="b">
@@ -6777,7 +6789,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J136" s="1" t="n">
+      <c r="J136" s="2" t="n">
         <v>46567</v>
       </c>
       <c r="K136" t="b">
@@ -6826,7 +6838,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J137" s="1" t="n">
+      <c r="J137" s="2" t="n">
         <v>46568</v>
       </c>
       <c r="K137" t="b">
@@ -6875,7 +6887,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J138" s="1" t="n">
+      <c r="J138" s="2" t="n">
         <v>46571</v>
       </c>
       <c r="K138" t="b">
@@ -6924,7 +6936,7 @@
           <t>-14d</t>
         </is>
       </c>
-      <c r="J139" s="1" t="n">
+      <c r="J139" s="2" t="n">
         <v>46197</v>
       </c>
       <c r="K139" t="b">
@@ -6973,7 +6985,7 @@
           <t>1d</t>
         </is>
       </c>
-      <c r="J140" s="1" t="n">
+      <c r="J140" s="2" t="n">
         <v>46212</v>
       </c>
       <c r="K140" t="b">
@@ -7022,7 +7034,7 @@
           <t>14d</t>
         </is>
       </c>
-      <c r="J141" s="1" t="n">
+      <c r="J141" s="2" t="n">
         <v>46225</v>
       </c>
       <c r="K141" t="b">
@@ -7071,7 +7083,7 @@
           <t>23d</t>
         </is>
       </c>
-      <c r="J142" s="1" t="n">
+      <c r="J142" s="2" t="n">
         <v>46234</v>
       </c>
       <c r="K142" t="b">
@@ -7120,7 +7132,7 @@
           <t>24d</t>
         </is>
       </c>
-      <c r="J143" s="1" t="n">
+      <c r="J143" s="2" t="n">
         <v>46234</v>
       </c>
       <c r="K143" t="b">
@@ -7169,7 +7181,7 @@
           <t>1me23d</t>
         </is>
       </c>
-      <c r="J144" s="1" t="n">
+      <c r="J144" s="2" t="n">
         <v>46263</v>
       </c>
       <c r="K144" t="b">
@@ -7218,7 +7230,7 @@
           <t>1me25d</t>
         </is>
       </c>
-      <c r="J145" s="1" t="n">
+      <c r="J145" s="2" t="n">
         <v>46266</v>
       </c>
       <c r="K145" t="b">
@@ -7263,7 +7275,7 @@
         <v>-1476</v>
       </c>
       <c r="I146" t="inlineStr"/>
-      <c r="J146" s="1" t="n">
+      <c r="J146" s="2" t="n">
         <v>43773</v>
       </c>
       <c r="K146" t="b">
@@ -7308,7 +7320,7 @@
         <v>-1469</v>
       </c>
       <c r="I147" t="inlineStr"/>
-      <c r="J147" s="1" t="n">
+      <c r="J147" s="2" t="n">
         <v>43773</v>
       </c>
       <c r="K147" t="b">
@@ -7353,7 +7365,7 @@
         <v>-1121</v>
       </c>
       <c r="I148" t="inlineStr"/>
-      <c r="J148" s="1" t="n">
+      <c r="J148" s="2" t="n">
         <v>45295</v>
       </c>
       <c r="K148" t="b">
@@ -7398,7 +7410,7 @@
         <v>-1018</v>
       </c>
       <c r="I149" t="inlineStr"/>
-      <c r="J149" s="1" t="n">
+      <c r="J149" s="2" t="n">
         <v>45617</v>
       </c>
       <c r="K149" t="b">
@@ -7443,7 +7455,7 @@
         <v>-950</v>
       </c>
       <c r="I150" t="inlineStr"/>
-      <c r="J150" s="1" t="n">
+      <c r="J150" s="2" t="n">
         <v>45677</v>
       </c>
       <c r="K150" t="b">
@@ -7488,7 +7500,7 @@
         <v>-943</v>
       </c>
       <c r="I151" t="inlineStr"/>
-      <c r="J151" s="1" t="n">
+      <c r="J151" s="2" t="n">
         <v>44944</v>
       </c>
       <c r="K151" t="b">
@@ -7533,7 +7545,7 @@
         <v>-252</v>
       </c>
       <c r="I152" t="inlineStr"/>
-      <c r="J152" s="1" t="n">
+      <c r="J152" s="2" t="n">
         <v>46092</v>
       </c>
       <c r="K152" t="b">
@@ -7578,7 +7590,7 @@
         <v>-196</v>
       </c>
       <c r="I153" t="inlineStr"/>
-      <c r="J153" s="1" t="n">
+      <c r="J153" s="2" t="n">
         <v>45988</v>
       </c>
       <c r="K153" t="b">
@@ -7623,7 +7635,7 @@
         <v>-196</v>
       </c>
       <c r="I154" t="inlineStr"/>
-      <c r="J154" s="1" t="n">
+      <c r="J154" s="2" t="n">
         <v>45988</v>
       </c>
       <c r="K154" t="b">
@@ -7668,7 +7680,7 @@
         <v>-47</v>
       </c>
       <c r="I155" t="inlineStr"/>
-      <c r="J155" s="1" t="n">
+      <c r="J155" s="2" t="n">
         <v>46176</v>
       </c>
       <c r="K155" t="b">
@@ -7713,7 +7725,7 @@
         <v>-47</v>
       </c>
       <c r="I156" t="inlineStr"/>
-      <c r="J156" s="1" t="n">
+      <c r="J156" s="2" t="n">
         <v>46176</v>
       </c>
       <c r="K156" t="b">
@@ -7758,7 +7770,7 @@
         <v>-33</v>
       </c>
       <c r="I157" t="inlineStr"/>
-      <c r="J157" s="1" t="n">
+      <c r="J157" s="2" t="n">
         <v>46199</v>
       </c>
       <c r="K157" t="b">
@@ -7803,7 +7815,7 @@
         <v>-33</v>
       </c>
       <c r="I158" t="inlineStr"/>
-      <c r="J158" s="1" t="n">
+      <c r="J158" s="2" t="n">
         <v>46199</v>
       </c>
       <c r="K158" t="b">
@@ -7848,7 +7860,7 @@
         <v>-6</v>
       </c>
       <c r="I159" t="inlineStr"/>
-      <c r="J159" s="1" t="n">
+      <c r="J159" s="2" t="n">
         <v>45967</v>
       </c>
       <c r="K159" t="b">
@@ -7893,7 +7905,7 @@
         <v>43</v>
       </c>
       <c r="I160" t="inlineStr"/>
-      <c r="J160" s="1" t="n">
+      <c r="J160" s="2" t="n">
         <v>46440</v>
       </c>
       <c r="K160" t="b">
@@ -7938,7 +7950,7 @@
         <v>43</v>
       </c>
       <c r="I161" t="inlineStr"/>
-      <c r="J161" s="1" t="n">
+      <c r="J161" s="2" t="n">
         <v>46440</v>
       </c>
       <c r="K161" t="b">
@@ -7983,7 +7995,7 @@
         <v>73</v>
       </c>
       <c r="I162" t="inlineStr"/>
-      <c r="J162" s="1" t="n">
+      <c r="J162" s="2" t="n">
         <v>46264</v>
       </c>
       <c r="K162" t="b">
@@ -8028,7 +8040,7 @@
         <v>73</v>
       </c>
       <c r="I163" t="inlineStr"/>
-      <c r="J163" s="1" t="n">
+      <c r="J163" s="2" t="n">
         <v>46264</v>
       </c>
       <c r="K163" t="b">
@@ -8073,7 +8085,7 @@
         <v>102</v>
       </c>
       <c r="I164" t="inlineStr"/>
-      <c r="J164" s="1" t="n">
+      <c r="J164" s="2" t="n">
         <v>46463</v>
       </c>
       <c r="K164" t="b">
@@ -8118,7 +8130,7 @@
         <v>118</v>
       </c>
       <c r="I165" t="inlineStr"/>
-      <c r="J165" s="1" t="n">
+      <c r="J165" s="2" t="n">
         <v>46337</v>
       </c>
       <c r="K165" t="b">
@@ -8163,7 +8175,7 @@
         <v>146</v>
       </c>
       <c r="I166" t="inlineStr"/>
-      <c r="J166" s="1" t="n">
+      <c r="J166" s="2" t="n">
         <v>46451</v>
       </c>
       <c r="K166" t="b">
@@ -8208,7 +8220,7 @@
         <v>152</v>
       </c>
       <c r="I167" t="inlineStr"/>
-      <c r="J167" s="1" t="n">
+      <c r="J167" s="2" t="n">
         <v>46245</v>
       </c>
       <c r="K167" t="b">
@@ -8253,7 +8265,7 @@
         <v>152</v>
       </c>
       <c r="I168" t="inlineStr"/>
-      <c r="J168" s="1" t="n">
+      <c r="J168" s="2" t="n">
         <v>46245</v>
       </c>
       <c r="K168" t="b">
@@ -8298,7 +8310,7 @@
         <v>163</v>
       </c>
       <c r="I169" t="inlineStr"/>
-      <c r="J169" s="1" t="n">
+      <c r="J169" s="2" t="n">
         <v>46324</v>
       </c>
       <c r="K169" t="b">
@@ -8343,7 +8355,7 @@
         <v>163</v>
       </c>
       <c r="I170" t="inlineStr"/>
-      <c r="J170" s="1" t="n">
+      <c r="J170" s="2" t="n">
         <v>46324</v>
       </c>
       <c r="K170" t="b">
@@ -8388,7 +8400,7 @@
         <v>164</v>
       </c>
       <c r="I171" t="inlineStr"/>
-      <c r="J171" s="1" t="n">
+      <c r="J171" s="2" t="n">
         <v>46426</v>
       </c>
       <c r="K171" t="b">
@@ -8433,7 +8445,7 @@
         <v>175</v>
       </c>
       <c r="I172" t="inlineStr"/>
-      <c r="J172" s="1" t="n">
+      <c r="J172" s="2" t="n">
         <v>46383</v>
       </c>
       <c r="K172" t="b">
@@ -8478,7 +8490,7 @@
         <v>186</v>
       </c>
       <c r="I173" t="inlineStr"/>
-      <c r="J173" s="1" t="n">
+      <c r="J173" s="2" t="n">
         <v>46392</v>
       </c>
       <c r="K173" t="b">
@@ -8523,7 +8535,7 @@
         <v>205</v>
       </c>
       <c r="I174" t="inlineStr"/>
-      <c r="J174" s="1" t="n">
+      <c r="J174" s="2" t="n">
         <v>46390</v>
       </c>
       <c r="K174" t="b">
@@ -8568,7 +8580,7 @@
         <v>207</v>
       </c>
       <c r="I175" t="inlineStr"/>
-      <c r="J175" s="1" t="n">
+      <c r="J175" s="2" t="n">
         <v>46392</v>
       </c>
       <c r="K175" t="b">
@@ -8613,7 +8625,7 @@
         <v>218</v>
       </c>
       <c r="I176" t="inlineStr"/>
-      <c r="J176" s="1" t="n">
+      <c r="J176" s="2" t="n">
         <v>46506</v>
       </c>
       <c r="K176" t="b">
@@ -8658,7 +8670,7 @@
         <v>246</v>
       </c>
       <c r="I177" t="inlineStr"/>
-      <c r="J177" s="1" t="n">
+      <c r="J177" s="2" t="n">
         <v>46478</v>
       </c>
       <c r="K177" t="b">
@@ -8703,7 +8715,7 @@
         <v>248</v>
       </c>
       <c r="I178" t="inlineStr"/>
-      <c r="J178" s="1" t="n">
+      <c r="J178" s="2" t="n">
         <v>46500</v>
       </c>
       <c r="K178" t="b">
@@ -8748,7 +8760,7 @@
         <v>276</v>
       </c>
       <c r="I179" t="inlineStr"/>
-      <c r="J179" s="1" t="n">
+      <c r="J179" s="2" t="n">
         <v>46430</v>
       </c>
       <c r="K179" t="b">
@@ -8793,7 +8805,7 @@
         <v>276</v>
       </c>
       <c r="I180" t="inlineStr"/>
-      <c r="J180" s="1" t="n">
+      <c r="J180" s="2" t="n">
         <v>46430</v>
       </c>
       <c r="K180" t="b">
@@ -8838,7 +8850,7 @@
         <v>290</v>
       </c>
       <c r="I181" t="inlineStr"/>
-      <c r="J181" s="1" t="n">
+      <c r="J181" s="2" t="n">
         <v>46467</v>
       </c>
       <c r="K181" t="b">
@@ -8883,7 +8895,7 @@
         <v>317</v>
       </c>
       <c r="I182" t="inlineStr"/>
-      <c r="J182" s="1" t="n">
+      <c r="J182" s="2" t="n">
         <v>46529</v>
       </c>
       <c r="K182" t="b">
@@ -8928,7 +8940,7 @@
         <v>420</v>
       </c>
       <c r="I183" t="inlineStr"/>
-      <c r="J183" s="1" t="n">
+      <c r="J183" s="2" t="n">
         <v>46566</v>
       </c>
       <c r="K183" t="b">
@@ -8973,7 +8985,7 @@
         <v>426</v>
       </c>
       <c r="I184" t="inlineStr"/>
-      <c r="J184" s="1" t="n">
+      <c r="J184" s="2" t="n">
         <v>46571</v>
       </c>
       <c r="K184" t="b">
@@ -9018,7 +9030,7 @@
         <v>721</v>
       </c>
       <c r="I185" t="inlineStr"/>
-      <c r="J185" s="1" t="n">
+      <c r="J185" s="2" t="n">
         <v>46325</v>
       </c>
       <c r="K185" t="b">
@@ -9063,7 +9075,7 @@
         <v>721</v>
       </c>
       <c r="I186" t="inlineStr"/>
-      <c r="J186" s="1" t="n">
+      <c r="J186" s="2" t="n">
         <v>46325</v>
       </c>
       <c r="K186" t="b">
@@ -9108,7 +9120,7 @@
         <v>850</v>
       </c>
       <c r="I187" t="inlineStr"/>
-      <c r="J187" s="1" t="n">
+      <c r="J187" s="2" t="n">
         <v>46345</v>
       </c>
       <c r="K187" t="b">
@@ -9153,7 +9165,7 @@
         <v>850</v>
       </c>
       <c r="I188" t="inlineStr"/>
-      <c r="J188" s="1" t="n">
+      <c r="J188" s="2" t="n">
         <v>46345</v>
       </c>
       <c r="K188" t="b">
@@ -9198,7 +9210,7 @@
         <v>1661</v>
       </c>
       <c r="I189" t="inlineStr"/>
-      <c r="J189" s="1" t="n">
+      <c r="J189" s="2" t="n">
         <v>46498</v>
       </c>
       <c r="K189" t="b">
@@ -9243,7 +9255,7 @@
         <v>1661</v>
       </c>
       <c r="I190" t="inlineStr"/>
-      <c r="J190" s="1" t="n">
+      <c r="J190" s="2" t="n">
         <v>46498</v>
       </c>
       <c r="K190" t="b">
@@ -9288,7 +9300,7 @@
         <v>488</v>
       </c>
       <c r="I191" t="inlineStr"/>
-      <c r="J191" s="1" t="n">
+      <c r="J191" s="2" t="n">
         <v>46190</v>
       </c>
       <c r="K191" t="b">
@@ -9333,7 +9345,7 @@
         <v>25565</v>
       </c>
       <c r="I192" t="inlineStr"/>
-      <c r="J192" s="1" t="n">
+      <c r="J192" s="2" t="n">
         <v>46190</v>
       </c>
       <c r="K192" t="b">
@@ -9378,7 +9390,7 @@
         <v>25567</v>
       </c>
       <c r="I193" t="inlineStr"/>
-      <c r="J193" s="1" t="n">
+      <c r="J193" s="2" t="n">
         <v>46190</v>
       </c>
       <c r="K193" t="b">
@@ -9423,7 +9435,7 @@
         <v>31293</v>
       </c>
       <c r="I194" t="inlineStr"/>
-      <c r="J194" s="1" t="n">
+      <c r="J194" s="2" t="n">
         <v>46190</v>
       </c>
       <c r="K194" t="b">

</xml_diff>

<commit_message>
Atualização automática: vencimentos_tmot (11/07/2026 07:20)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
@@ -20,16 +20,13 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -40,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -48,21 +45,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -433,57 +421,57 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>matricula</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>operador</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>pn</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>sn</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>nomenclatura</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>inspecao</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>tipo_vencimento</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>disponibilidade_valor</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>disponibilidade_texto</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>data_vencimento</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>vencido</t>
         </is>
@@ -527,7 +515,7 @@
         <v>-4402.8</v>
       </c>
       <c r="I2" t="inlineStr"/>
-      <c r="J2" s="2" t="n">
+      <c r="J2" s="1" t="n">
         <v>41388</v>
       </c>
       <c r="K2" t="b">
@@ -572,7 +560,7 @@
         <v>-4254.8</v>
       </c>
       <c r="I3" t="inlineStr"/>
-      <c r="J3" s="2" t="n">
+      <c r="J3" s="1" t="n">
         <v>39285</v>
       </c>
       <c r="K3" t="b">
@@ -617,7 +605,7 @@
         <v>-2354.2</v>
       </c>
       <c r="I4" t="inlineStr"/>
-      <c r="J4" s="2" t="n">
+      <c r="J4" s="1" t="n">
         <v>40669</v>
       </c>
       <c r="K4" t="b">
@@ -662,7 +650,7 @@
         <v>-896.8</v>
       </c>
       <c r="I5" t="inlineStr"/>
-      <c r="J5" s="2" t="n">
+      <c r="J5" s="1" t="n">
         <v>40669</v>
       </c>
       <c r="K5" t="b">
@@ -707,7 +695,7 @@
         <v>-854.1</v>
       </c>
       <c r="I6" t="inlineStr"/>
-      <c r="J6" s="2" t="n">
+      <c r="J6" s="1" t="n">
         <v>44884</v>
       </c>
       <c r="K6" t="b">
@@ -752,7 +740,7 @@
         <v>-413.2</v>
       </c>
       <c r="I7" t="inlineStr"/>
-      <c r="J7" s="2" t="n">
+      <c r="J7" s="1" t="n">
         <v>43855</v>
       </c>
       <c r="K7" t="b">
@@ -797,7 +785,7 @@
         <v>-391.8</v>
       </c>
       <c r="I8" t="inlineStr"/>
-      <c r="J8" s="2" t="n">
+      <c r="J8" s="1" t="n">
         <v>42769</v>
       </c>
       <c r="K8" t="b">
@@ -842,7 +830,7 @@
         <v>-371.5</v>
       </c>
       <c r="I9" t="inlineStr"/>
-      <c r="J9" s="2" t="n">
+      <c r="J9" s="1" t="n">
         <v>46014</v>
       </c>
       <c r="K9" t="b">
@@ -887,7 +875,7 @@
         <v>-368.8</v>
       </c>
       <c r="I10" t="inlineStr"/>
-      <c r="J10" s="2" t="n">
+      <c r="J10" s="1" t="n">
         <v>46014</v>
       </c>
       <c r="K10" t="b">
@@ -932,7 +920,7 @@
         <v>-359</v>
       </c>
       <c r="I11" t="inlineStr"/>
-      <c r="J11" s="2" t="n">
+      <c r="J11" s="1" t="n">
         <v>45804</v>
       </c>
       <c r="K11" t="b">
@@ -977,7 +965,7 @@
         <v>-359</v>
       </c>
       <c r="I12" t="inlineStr"/>
-      <c r="J12" s="2" t="n">
+      <c r="J12" s="1" t="n">
         <v>45804</v>
       </c>
       <c r="K12" t="b">
@@ -1022,7 +1010,7 @@
         <v>-351</v>
       </c>
       <c r="I13" t="inlineStr"/>
-      <c r="J13" s="2" t="n">
+      <c r="J13" s="1" t="n">
         <v>42821</v>
       </c>
       <c r="K13" t="b">
@@ -1067,7 +1055,7 @@
         <v>-351</v>
       </c>
       <c r="I14" t="inlineStr"/>
-      <c r="J14" s="2" t="n">
+      <c r="J14" s="1" t="n">
         <v>46014</v>
       </c>
       <c r="K14" t="b">
@@ -1112,7 +1100,7 @@
         <v>-351</v>
       </c>
       <c r="I15" t="inlineStr"/>
-      <c r="J15" s="2" t="n">
+      <c r="J15" s="1" t="n">
         <v>46014</v>
       </c>
       <c r="K15" t="b">
@@ -1157,7 +1145,7 @@
         <v>-351</v>
       </c>
       <c r="I16" t="inlineStr"/>
-      <c r="J16" s="2" t="n">
+      <c r="J16" s="1" t="n">
         <v>46014</v>
       </c>
       <c r="K16" t="b">
@@ -1202,7 +1190,7 @@
         <v>-345.8</v>
       </c>
       <c r="I17" t="inlineStr"/>
-      <c r="J17" s="2" t="n">
+      <c r="J17" s="1" t="n">
         <v>46017</v>
       </c>
       <c r="K17" t="b">
@@ -1247,7 +1235,7 @@
         <v>-345.8</v>
       </c>
       <c r="I18" t="inlineStr"/>
-      <c r="J18" s="2" t="n">
+      <c r="J18" s="1" t="n">
         <v>46017</v>
       </c>
       <c r="K18" t="b">
@@ -1292,7 +1280,7 @@
         <v>-264.2</v>
       </c>
       <c r="I19" t="inlineStr"/>
-      <c r="J19" s="2" t="n">
+      <c r="J19" s="1" t="n">
         <v>40979</v>
       </c>
       <c r="K19" t="b">
@@ -1337,7 +1325,7 @@
         <v>-206.4</v>
       </c>
       <c r="I20" t="inlineStr"/>
-      <c r="J20" s="2" t="n">
+      <c r="J20" s="1" t="n">
         <v>36669</v>
       </c>
       <c r="K20" t="b">
@@ -1382,7 +1370,7 @@
         <v>-131.6</v>
       </c>
       <c r="I21" t="inlineStr"/>
-      <c r="J21" s="2" t="n">
+      <c r="J21" s="1" t="n">
         <v>46111</v>
       </c>
       <c r="K21" t="b">
@@ -1427,7 +1415,7 @@
         <v>-131.6</v>
       </c>
       <c r="I22" t="inlineStr"/>
-      <c r="J22" s="2" t="n">
+      <c r="J22" s="1" t="n">
         <v>46111</v>
       </c>
       <c r="K22" t="b">
@@ -1472,7 +1460,7 @@
         <v>-131.6</v>
       </c>
       <c r="I23" t="inlineStr"/>
-      <c r="J23" s="2" t="n">
+      <c r="J23" s="1" t="n">
         <v>46111</v>
       </c>
       <c r="K23" t="b">
@@ -1517,7 +1505,7 @@
         <v>-131.6</v>
       </c>
       <c r="I24" t="inlineStr"/>
-      <c r="J24" s="2" t="n">
+      <c r="J24" s="1" t="n">
         <v>46111</v>
       </c>
       <c r="K24" t="b">
@@ -1562,7 +1550,7 @@
         <v>-131.6</v>
       </c>
       <c r="I25" t="inlineStr"/>
-      <c r="J25" s="2" t="n">
+      <c r="J25" s="1" t="n">
         <v>46111</v>
       </c>
       <c r="K25" t="b">
@@ -1607,7 +1595,7 @@
         <v>-105</v>
       </c>
       <c r="I26" t="inlineStr"/>
-      <c r="J26" s="2" t="n">
+      <c r="J26" s="1" t="n">
         <v>46161</v>
       </c>
       <c r="K26" t="b">
@@ -1652,7 +1640,7 @@
         <v>-79.8</v>
       </c>
       <c r="I27" t="inlineStr"/>
-      <c r="J27" s="2" t="n">
+      <c r="J27" s="1" t="n">
         <v>43340</v>
       </c>
       <c r="K27" t="b">
@@ -1697,7 +1685,7 @@
         <v>-12.3</v>
       </c>
       <c r="I28" t="inlineStr"/>
-      <c r="J28" s="2" t="n">
+      <c r="J28" s="1" t="n">
         <v>46048</v>
       </c>
       <c r="K28" t="b">
@@ -1742,7 +1730,7 @@
         <v>0</v>
       </c>
       <c r="I29" t="inlineStr"/>
-      <c r="J29" s="2" t="n">
+      <c r="J29" s="1" t="n">
         <v>46211</v>
       </c>
       <c r="K29" t="b">
@@ -1787,7 +1775,7 @@
         <v>3.6</v>
       </c>
       <c r="I30" t="inlineStr"/>
-      <c r="J30" s="2" t="n">
+      <c r="J30" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="K30" t="b">
@@ -1832,7 +1820,7 @@
         <v>6.2</v>
       </c>
       <c r="I31" t="inlineStr"/>
-      <c r="J31" s="2" t="n">
+      <c r="J31" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="K31" t="b">
@@ -1877,7 +1865,7 @@
         <v>7.5</v>
       </c>
       <c r="I32" t="inlineStr"/>
-      <c r="J32" s="2" t="n">
+      <c r="J32" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="K32" t="b">
@@ -1922,7 +1910,7 @@
         <v>10.7</v>
       </c>
       <c r="I33" t="inlineStr"/>
-      <c r="J33" s="2" t="n">
+      <c r="J33" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="K33" t="b">
@@ -1967,7 +1955,7 @@
         <v>20</v>
       </c>
       <c r="I34" t="inlineStr"/>
-      <c r="J34" s="2" t="n">
+      <c r="J34" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="K34" t="b">
@@ -2012,7 +2000,7 @@
         <v>30.8</v>
       </c>
       <c r="I35" t="inlineStr"/>
-      <c r="J35" s="2" t="n">
+      <c r="J35" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="K35" t="b">
@@ -2057,7 +2045,7 @@
         <v>37.1</v>
       </c>
       <c r="I36" t="inlineStr"/>
-      <c r="J36" s="2" t="n">
+      <c r="J36" s="1" t="n">
         <v>46256</v>
       </c>
       <c r="K36" t="b">
@@ -2102,7 +2090,7 @@
         <v>42.8</v>
       </c>
       <c r="I37" t="inlineStr"/>
-      <c r="J37" s="2" t="n">
+      <c r="J37" s="1" t="n">
         <v>46276</v>
       </c>
       <c r="K37" t="b">
@@ -2147,7 +2135,7 @@
         <v>45.2</v>
       </c>
       <c r="I38" t="inlineStr"/>
-      <c r="J38" s="2" t="n">
+      <c r="J38" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="K38" t="b">
@@ -2192,7 +2180,7 @@
         <v>46</v>
       </c>
       <c r="I39" t="inlineStr"/>
-      <c r="J39" s="2" t="n">
+      <c r="J39" s="1" t="n">
         <v>46251</v>
       </c>
       <c r="K39" t="b">
@@ -2237,7 +2225,7 @@
         <v>47.5</v>
       </c>
       <c r="I40" t="inlineStr"/>
-      <c r="J40" s="2" t="n">
+      <c r="J40" s="1" t="n">
         <v>46456</v>
       </c>
       <c r="K40" t="b">
@@ -2282,7 +2270,7 @@
         <v>57.2</v>
       </c>
       <c r="I41" t="inlineStr"/>
-      <c r="J41" s="2" t="n">
+      <c r="J41" s="1" t="n">
         <v>46246</v>
       </c>
       <c r="K41" t="b">
@@ -2327,7 +2315,7 @@
         <v>59.6</v>
       </c>
       <c r="I42" t="inlineStr"/>
-      <c r="J42" s="2" t="n">
+      <c r="J42" s="1" t="n">
         <v>46487</v>
       </c>
       <c r="K42" t="b">
@@ -2372,7 +2360,7 @@
         <v>75.40000000000001</v>
       </c>
       <c r="I43" t="inlineStr"/>
-      <c r="J43" s="2" t="n">
+      <c r="J43" s="1" t="n">
         <v>46283</v>
       </c>
       <c r="K43" t="b">
@@ -2417,7 +2405,7 @@
         <v>76.8</v>
       </c>
       <c r="I44" t="inlineStr"/>
-      <c r="J44" s="2" t="n">
+      <c r="J44" s="1" t="n">
         <v>46285</v>
       </c>
       <c r="K44" t="b">
@@ -2462,7 +2450,7 @@
         <v>83.2</v>
       </c>
       <c r="I45" t="inlineStr"/>
-      <c r="J45" s="2" t="n">
+      <c r="J45" s="1" t="n">
         <v>46547</v>
       </c>
       <c r="K45" t="b">
@@ -2507,7 +2495,7 @@
         <v>84.5</v>
       </c>
       <c r="I46" t="inlineStr"/>
-      <c r="J46" s="2" t="n">
+      <c r="J46" s="1" t="n">
         <v>46240</v>
       </c>
       <c r="K46" t="b">
@@ -2552,7 +2540,7 @@
         <v>85.8</v>
       </c>
       <c r="I47" t="inlineStr"/>
-      <c r="J47" s="2" t="n">
+      <c r="J47" s="1" t="n">
         <v>46266</v>
       </c>
       <c r="K47" t="b">
@@ -2597,7 +2585,7 @@
         <v>86.5</v>
       </c>
       <c r="I48" t="inlineStr"/>
-      <c r="J48" s="2" t="n">
+      <c r="J48" s="1" t="n">
         <v>46241</v>
       </c>
       <c r="K48" t="b">
@@ -2642,7 +2630,7 @@
         <v>91.7</v>
       </c>
       <c r="I49" t="inlineStr"/>
-      <c r="J49" s="2" t="n">
+      <c r="J49" s="1" t="n">
         <v>46243</v>
       </c>
       <c r="K49" t="b">
@@ -2687,7 +2675,7 @@
         <v>91.7</v>
       </c>
       <c r="I50" t="inlineStr"/>
-      <c r="J50" s="2" t="n">
+      <c r="J50" s="1" t="n">
         <v>46243</v>
       </c>
       <c r="K50" t="b">
@@ -2732,7 +2720,7 @@
         <v>91.7</v>
       </c>
       <c r="I51" t="inlineStr"/>
-      <c r="J51" s="2" t="n">
+      <c r="J51" s="1" t="n">
         <v>46250</v>
       </c>
       <c r="K51" t="b">
@@ -2777,7 +2765,7 @@
         <v>98.90000000000001</v>
       </c>
       <c r="I52" t="inlineStr"/>
-      <c r="J52" s="2" t="n">
+      <c r="J52" s="1" t="n">
         <v>46253</v>
       </c>
       <c r="K52" t="b">
@@ -2822,7 +2810,7 @@
         <v>105.5</v>
       </c>
       <c r="I53" t="inlineStr"/>
-      <c r="J53" s="2" t="n">
+      <c r="J53" s="1" t="n">
         <v>46280</v>
       </c>
       <c r="K53" t="b">
@@ -2867,7 +2855,7 @@
         <v>105.6</v>
       </c>
       <c r="I54" t="inlineStr"/>
-      <c r="J54" s="2" t="n">
+      <c r="J54" s="1" t="n">
         <v>46361</v>
       </c>
       <c r="K54" t="b">
@@ -2912,7 +2900,7 @@
         <v>105.7</v>
       </c>
       <c r="I55" t="inlineStr"/>
-      <c r="J55" s="2" t="n">
+      <c r="J55" s="1" t="n">
         <v>46362</v>
       </c>
       <c r="K55" t="b">
@@ -2957,7 +2945,7 @@
         <v>110.7</v>
       </c>
       <c r="I56" t="inlineStr"/>
-      <c r="J56" s="2" t="n">
+      <c r="J56" s="1" t="n">
         <v>46275</v>
       </c>
       <c r="K56" t="b">
@@ -3002,7 +2990,7 @@
         <v>113.2</v>
       </c>
       <c r="I57" t="inlineStr"/>
-      <c r="J57" s="2" t="n">
+      <c r="J57" s="1" t="n">
         <v>46377</v>
       </c>
       <c r="K57" t="b">
@@ -3047,7 +3035,7 @@
         <v>128.8</v>
       </c>
       <c r="I58" t="inlineStr"/>
-      <c r="J58" s="2" t="n">
+      <c r="J58" s="1" t="n">
         <v>46434</v>
       </c>
       <c r="K58" t="b">
@@ -3092,7 +3080,7 @@
         <v>128.8</v>
       </c>
       <c r="I59" t="inlineStr"/>
-      <c r="J59" s="2" t="n">
+      <c r="J59" s="1" t="n">
         <v>46434</v>
       </c>
       <c r="K59" t="b">
@@ -3137,7 +3125,7 @@
         <v>128.8</v>
       </c>
       <c r="I60" t="inlineStr"/>
-      <c r="J60" s="2" t="n">
+      <c r="J60" s="1" t="n">
         <v>46434</v>
       </c>
       <c r="K60" t="b">
@@ -3182,7 +3170,7 @@
         <v>128.8</v>
       </c>
       <c r="I61" t="inlineStr"/>
-      <c r="J61" s="2" t="n">
+      <c r="J61" s="1" t="n">
         <v>46434</v>
       </c>
       <c r="K61" t="b">
@@ -3227,7 +3215,7 @@
         <v>128.8</v>
       </c>
       <c r="I62" t="inlineStr"/>
-      <c r="J62" s="2" t="n">
+      <c r="J62" s="1" t="n">
         <v>46434</v>
       </c>
       <c r="K62" t="b">
@@ -3272,7 +3260,7 @@
         <v>135</v>
       </c>
       <c r="I63" t="inlineStr"/>
-      <c r="J63" s="2" t="n">
+      <c r="J63" s="1" t="n">
         <v>46280</v>
       </c>
       <c r="K63" t="b">
@@ -3317,7 +3305,7 @@
         <v>150.6</v>
       </c>
       <c r="I64" t="inlineStr"/>
-      <c r="J64" s="2" t="n">
+      <c r="J64" s="1" t="n">
         <v>46271</v>
       </c>
       <c r="K64" t="b">
@@ -3362,7 +3350,7 @@
         <v>174.2</v>
       </c>
       <c r="I65" t="inlineStr"/>
-      <c r="J65" s="2" t="n">
+      <c r="J65" s="1" t="n">
         <v>46363</v>
       </c>
       <c r="K65" t="b">
@@ -3407,7 +3395,7 @@
         <v>176.6</v>
       </c>
       <c r="I66" t="inlineStr"/>
-      <c r="J66" s="2" t="n">
+      <c r="J66" s="1" t="n">
         <v>46334</v>
       </c>
       <c r="K66" t="b">
@@ -3452,7 +3440,7 @@
         <v>177.4</v>
       </c>
       <c r="I67" t="inlineStr"/>
-      <c r="J67" s="2" t="n">
+      <c r="J67" s="1" t="n">
         <v>46407</v>
       </c>
       <c r="K67" t="b">
@@ -3497,7 +3485,7 @@
         <v>183.9</v>
       </c>
       <c r="I68" t="inlineStr"/>
-      <c r="J68" s="2" t="n">
+      <c r="J68" s="1" t="n">
         <v>46341</v>
       </c>
       <c r="K68" t="b">
@@ -3542,7 +3530,7 @@
         <v>191.7</v>
       </c>
       <c r="I69" t="inlineStr"/>
-      <c r="J69" s="2" t="n">
+      <c r="J69" s="1" t="n">
         <v>46300</v>
       </c>
       <c r="K69" t="b">
@@ -3587,7 +3575,7 @@
         <v>200</v>
       </c>
       <c r="I70" t="inlineStr"/>
-      <c r="J70" s="2" t="n">
+      <c r="J70" s="1" t="n">
         <v>46336</v>
       </c>
       <c r="K70" t="b">
@@ -3632,7 +3620,7 @@
         <v>201.1</v>
       </c>
       <c r="I71" t="inlineStr"/>
-      <c r="J71" s="2" t="n">
+      <c r="J71" s="1" t="n">
         <v>46319</v>
       </c>
       <c r="K71" t="b">
@@ -3677,7 +3665,7 @@
         <v>206.5</v>
       </c>
       <c r="I72" t="inlineStr"/>
-      <c r="J72" s="2" t="n">
+      <c r="J72" s="1" t="n">
         <v>46308</v>
       </c>
       <c r="K72" t="b">
@@ -3722,7 +3710,7 @@
         <v>207.5</v>
       </c>
       <c r="I73" t="inlineStr"/>
-      <c r="J73" s="2" t="n">
+      <c r="J73" s="1" t="n">
         <v>46390</v>
       </c>
       <c r="K73" t="b">
@@ -3767,7 +3755,7 @@
         <v>247</v>
       </c>
       <c r="I74" t="inlineStr"/>
-      <c r="J74" s="2" t="n">
+      <c r="J74" s="1" t="n">
         <v>46443</v>
       </c>
       <c r="K74" t="b">
@@ -3812,7 +3800,7 @@
         <v>285.3</v>
       </c>
       <c r="I75" t="inlineStr"/>
-      <c r="J75" s="2" t="n">
+      <c r="J75" s="1" t="n">
         <v>46304</v>
       </c>
       <c r="K75" t="b">
@@ -3857,7 +3845,7 @@
         <v>290.8</v>
       </c>
       <c r="I76" t="inlineStr"/>
-      <c r="J76" s="2" t="n">
+      <c r="J76" s="1" t="n">
         <v>46362</v>
       </c>
       <c r="K76" t="b">
@@ -3902,7 +3890,7 @@
         <v>295.2</v>
       </c>
       <c r="I77" t="inlineStr"/>
-      <c r="J77" s="2" t="n">
+      <c r="J77" s="1" t="n">
         <v>46463</v>
       </c>
       <c r="K77" t="b">
@@ -3947,7 +3935,7 @@
         <v>300.2</v>
       </c>
       <c r="I78" t="inlineStr"/>
-      <c r="J78" s="2" t="n">
+      <c r="J78" s="1" t="n">
         <v>46466</v>
       </c>
       <c r="K78" t="b">
@@ -3996,7 +3984,7 @@
           <t>-317m</t>
         </is>
       </c>
-      <c r="J79" s="2" t="n">
+      <c r="J79" s="1" t="n">
         <v>36557</v>
       </c>
       <c r="K79" t="b">
@@ -4045,7 +4033,7 @@
           <t>-164m</t>
         </is>
       </c>
-      <c r="J80" s="2" t="n">
+      <c r="J80" s="1" t="n">
         <v>41275</v>
       </c>
       <c r="K80" t="b">
@@ -4094,7 +4082,7 @@
           <t>-27m</t>
         </is>
       </c>
-      <c r="J81" s="2" t="n">
+      <c r="J81" s="1" t="n">
         <v>45380</v>
       </c>
       <c r="K81" t="b">
@@ -4143,7 +4131,7 @@
           <t>-25m</t>
         </is>
       </c>
-      <c r="J82" s="2" t="n">
+      <c r="J82" s="1" t="n">
         <v>45421</v>
       </c>
       <c r="K82" t="b">
@@ -4192,7 +4180,7 @@
           <t>-25m</t>
         </is>
       </c>
-      <c r="J83" s="2" t="n">
+      <c r="J83" s="1" t="n">
         <v>45428</v>
       </c>
       <c r="K83" t="b">
@@ -4241,7 +4229,7 @@
           <t>-23m</t>
         </is>
       </c>
-      <c r="J84" s="2" t="n">
+      <c r="J84" s="1" t="n">
         <v>45490</v>
       </c>
       <c r="K84" t="b">
@@ -4290,7 +4278,7 @@
           <t>-21m</t>
         </is>
       </c>
-      <c r="J85" s="2" t="n">
+      <c r="J85" s="1" t="n">
         <v>45566</v>
       </c>
       <c r="K85" t="b">
@@ -4339,7 +4327,7 @@
           <t>-7m</t>
         </is>
       </c>
-      <c r="J86" s="2" t="n">
+      <c r="J86" s="1" t="n">
         <v>45986</v>
       </c>
       <c r="K86" t="b">
@@ -4388,7 +4376,7 @@
           <t>-3m</t>
         </is>
       </c>
-      <c r="J87" s="2" t="n">
+      <c r="J87" s="1" t="n">
         <v>46106</v>
       </c>
       <c r="K87" t="b">
@@ -4437,7 +4425,7 @@
           <t>-2m</t>
         </is>
       </c>
-      <c r="J88" s="2" t="n">
+      <c r="J88" s="1" t="n">
         <v>46142</v>
       </c>
       <c r="K88" t="b">
@@ -4486,7 +4474,7 @@
           <t>2m</t>
         </is>
       </c>
-      <c r="J89" s="2" t="n">
+      <c r="J89" s="1" t="n">
         <v>46274</v>
       </c>
       <c r="K89" t="b">
@@ -4535,7 +4523,7 @@
           <t>2m</t>
         </is>
       </c>
-      <c r="J90" s="2" t="n">
+      <c r="J90" s="1" t="n">
         <v>46276</v>
       </c>
       <c r="K90" t="b">
@@ -4584,7 +4572,7 @@
           <t>2m</t>
         </is>
       </c>
-      <c r="J91" s="2" t="n">
+      <c r="J91" s="1" t="n">
         <v>46284</v>
       </c>
       <c r="K91" t="b">
@@ -4633,7 +4621,7 @@
           <t>3m</t>
         </is>
       </c>
-      <c r="J92" s="2" t="n">
+      <c r="J92" s="1" t="n">
         <v>46317</v>
       </c>
       <c r="K92" t="b">
@@ -4682,7 +4670,7 @@
           <t>3m</t>
         </is>
       </c>
-      <c r="J93" s="2" t="n">
+      <c r="J93" s="1" t="n">
         <v>46319</v>
       </c>
       <c r="K93" t="b">
@@ -4731,7 +4719,7 @@
           <t>4m</t>
         </is>
       </c>
-      <c r="J94" s="2" t="n">
+      <c r="J94" s="1" t="n">
         <v>46333</v>
       </c>
       <c r="K94" t="b">
@@ -4780,7 +4768,7 @@
           <t>4m</t>
         </is>
       </c>
-      <c r="J95" s="2" t="n">
+      <c r="J95" s="1" t="n">
         <v>46338</v>
       </c>
       <c r="K95" t="b">
@@ -4829,7 +4817,7 @@
           <t>4m</t>
         </is>
       </c>
-      <c r="J96" s="2" t="n">
+      <c r="J96" s="1" t="n">
         <v>46338</v>
       </c>
       <c r="K96" t="b">
@@ -4878,7 +4866,7 @@
           <t>4m</t>
         </is>
       </c>
-      <c r="J97" s="2" t="n">
+      <c r="J97" s="1" t="n">
         <v>46341</v>
       </c>
       <c r="K97" t="b">
@@ -4927,7 +4915,7 @@
           <t>4m</t>
         </is>
       </c>
-      <c r="J98" s="2" t="n">
+      <c r="J98" s="1" t="n">
         <v>46344</v>
       </c>
       <c r="K98" t="b">
@@ -4976,7 +4964,7 @@
           <t>4m</t>
         </is>
       </c>
-      <c r="J99" s="2" t="n">
+      <c r="J99" s="1" t="n">
         <v>46354</v>
       </c>
       <c r="K99" t="b">
@@ -5025,7 +5013,7 @@
           <t>4m</t>
         </is>
       </c>
-      <c r="J100" s="2" t="n">
+      <c r="J100" s="1" t="n">
         <v>46360</v>
       </c>
       <c r="K100" t="b">
@@ -5074,7 +5062,7 @@
           <t>4m</t>
         </is>
       </c>
-      <c r="J101" s="2" t="n">
+      <c r="J101" s="1" t="n">
         <v>46360</v>
       </c>
       <c r="K101" t="b">
@@ -5123,7 +5111,7 @@
           <t>5m</t>
         </is>
       </c>
-      <c r="J102" s="2" t="n">
+      <c r="J102" s="1" t="n">
         <v>46366</v>
       </c>
       <c r="K102" t="b">
@@ -5172,7 +5160,7 @@
           <t>5m</t>
         </is>
       </c>
-      <c r="J103" s="2" t="n">
+      <c r="J103" s="1" t="n">
         <v>46375</v>
       </c>
       <c r="K103" t="b">
@@ -5221,7 +5209,7 @@
           <t>5m</t>
         </is>
       </c>
-      <c r="J104" s="2" t="n">
+      <c r="J104" s="1" t="n">
         <v>46388</v>
       </c>
       <c r="K104" t="b">
@@ -5270,7 +5258,7 @@
           <t>6m</t>
         </is>
       </c>
-      <c r="J105" s="2" t="n">
+      <c r="J105" s="1" t="n">
         <v>46401</v>
       </c>
       <c r="K105" t="b">
@@ -5319,7 +5307,7 @@
           <t>6m</t>
         </is>
       </c>
-      <c r="J106" s="2" t="n">
+      <c r="J106" s="1" t="n">
         <v>46401</v>
       </c>
       <c r="K106" t="b">
@@ -5368,7 +5356,7 @@
           <t>6m</t>
         </is>
       </c>
-      <c r="J107" s="2" t="n">
+      <c r="J107" s="1" t="n">
         <v>46401</v>
       </c>
       <c r="K107" t="b">
@@ -5417,7 +5405,7 @@
           <t>6m</t>
         </is>
       </c>
-      <c r="J108" s="2" t="n">
+      <c r="J108" s="1" t="n">
         <v>46413</v>
       </c>
       <c r="K108" t="b">
@@ -5466,7 +5454,7 @@
           <t>7m</t>
         </is>
       </c>
-      <c r="J109" s="2" t="n">
+      <c r="J109" s="1" t="n">
         <v>46424</v>
       </c>
       <c r="K109" t="b">
@@ -5515,7 +5503,7 @@
           <t>7m</t>
         </is>
       </c>
-      <c r="J110" s="2" t="n">
+      <c r="J110" s="1" t="n">
         <v>46427</v>
       </c>
       <c r="K110" t="b">
@@ -5564,7 +5552,7 @@
           <t>7m</t>
         </is>
       </c>
-      <c r="J111" s="2" t="n">
+      <c r="J111" s="1" t="n">
         <v>46437</v>
       </c>
       <c r="K111" t="b">
@@ -5613,7 +5601,7 @@
           <t>7m</t>
         </is>
       </c>
-      <c r="J112" s="2" t="n">
+      <c r="J112" s="1" t="n">
         <v>46451</v>
       </c>
       <c r="K112" t="b">
@@ -5662,7 +5650,7 @@
           <t>8m</t>
         </is>
       </c>
-      <c r="J113" s="2" t="n">
+      <c r="J113" s="1" t="n">
         <v>46455</v>
       </c>
       <c r="K113" t="b">
@@ -5711,7 +5699,7 @@
           <t>8m</t>
         </is>
       </c>
-      <c r="J114" s="2" t="n">
+      <c r="J114" s="1" t="n">
         <v>46457</v>
       </c>
       <c r="K114" t="b">
@@ -5760,7 +5748,7 @@
           <t>8m</t>
         </is>
       </c>
-      <c r="J115" s="2" t="n">
+      <c r="J115" s="1" t="n">
         <v>46462</v>
       </c>
       <c r="K115" t="b">
@@ -5809,7 +5797,7 @@
           <t>8m</t>
         </is>
       </c>
-      <c r="J116" s="2" t="n">
+      <c r="J116" s="1" t="n">
         <v>46464</v>
       </c>
       <c r="K116" t="b">
@@ -5858,7 +5846,7 @@
           <t>8m</t>
         </is>
       </c>
-      <c r="J117" s="2" t="n">
+      <c r="J117" s="1" t="n">
         <v>46470</v>
       </c>
       <c r="K117" t="b">
@@ -5907,7 +5895,7 @@
           <t>9m</t>
         </is>
       </c>
-      <c r="J118" s="2" t="n">
+      <c r="J118" s="1" t="n">
         <v>46485</v>
       </c>
       <c r="K118" t="b">
@@ -5956,7 +5944,7 @@
           <t>9m</t>
         </is>
       </c>
-      <c r="J119" s="2" t="n">
+      <c r="J119" s="1" t="n">
         <v>46499</v>
       </c>
       <c r="K119" t="b">
@@ -6005,7 +5993,7 @@
           <t>9m</t>
         </is>
       </c>
-      <c r="J120" s="2" t="n">
+      <c r="J120" s="1" t="n">
         <v>46504</v>
       </c>
       <c r="K120" t="b">
@@ -6054,7 +6042,7 @@
           <t>9m</t>
         </is>
       </c>
-      <c r="J121" s="2" t="n">
+      <c r="J121" s="1" t="n">
         <v>46504</v>
       </c>
       <c r="K121" t="b">
@@ -6103,7 +6091,7 @@
           <t>9m</t>
         </is>
       </c>
-      <c r="J122" s="2" t="n">
+      <c r="J122" s="1" t="n">
         <v>46507</v>
       </c>
       <c r="K122" t="b">
@@ -6152,7 +6140,7 @@
           <t>9m</t>
         </is>
       </c>
-      <c r="J123" s="2" t="n">
+      <c r="J123" s="1" t="n">
         <v>46508</v>
       </c>
       <c r="K123" t="b">
@@ -6201,7 +6189,7 @@
           <t>9m</t>
         </is>
       </c>
-      <c r="J124" s="2" t="n">
+      <c r="J124" s="1" t="n">
         <v>46512</v>
       </c>
       <c r="K124" t="b">
@@ -6250,7 +6238,7 @@
           <t>9m</t>
         </is>
       </c>
-      <c r="J125" s="2" t="n">
+      <c r="J125" s="1" t="n">
         <v>46512</v>
       </c>
       <c r="K125" t="b">
@@ -6299,7 +6287,7 @@
           <t>10m</t>
         </is>
       </c>
-      <c r="J126" s="2" t="n">
+      <c r="J126" s="1" t="n">
         <v>46528</v>
       </c>
       <c r="K126" t="b">
@@ -6348,7 +6336,7 @@
           <t>10m</t>
         </is>
       </c>
-      <c r="J127" s="2" t="n">
+      <c r="J127" s="1" t="n">
         <v>46529</v>
       </c>
       <c r="K127" t="b">
@@ -6397,7 +6385,7 @@
           <t>10m</t>
         </is>
       </c>
-      <c r="J128" s="2" t="n">
+      <c r="J128" s="1" t="n">
         <v>46537</v>
       </c>
       <c r="K128" t="b">
@@ -6446,7 +6434,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J129" s="2" t="n">
+      <c r="J129" s="1" t="n">
         <v>46546</v>
       </c>
       <c r="K129" t="b">
@@ -6495,7 +6483,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J130" s="2" t="n">
+      <c r="J130" s="1" t="n">
         <v>46547</v>
       </c>
       <c r="K130" t="b">
@@ -6544,7 +6532,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J131" s="2" t="n">
+      <c r="J131" s="1" t="n">
         <v>46547</v>
       </c>
       <c r="K131" t="b">
@@ -6593,7 +6581,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J132" s="2" t="n">
+      <c r="J132" s="1" t="n">
         <v>46547</v>
       </c>
       <c r="K132" t="b">
@@ -6642,7 +6630,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J133" s="2" t="n">
+      <c r="J133" s="1" t="n">
         <v>46551</v>
       </c>
       <c r="K133" t="b">
@@ -6691,7 +6679,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J134" s="2" t="n">
+      <c r="J134" s="1" t="n">
         <v>46560</v>
       </c>
       <c r="K134" t="b">
@@ -6740,7 +6728,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J135" s="2" t="n">
+      <c r="J135" s="1" t="n">
         <v>46564</v>
       </c>
       <c r="K135" t="b">
@@ -6789,7 +6777,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J136" s="2" t="n">
+      <c r="J136" s="1" t="n">
         <v>46567</v>
       </c>
       <c r="K136" t="b">
@@ -6838,7 +6826,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J137" s="2" t="n">
+      <c r="J137" s="1" t="n">
         <v>46568</v>
       </c>
       <c r="K137" t="b">
@@ -6887,7 +6875,7 @@
           <t>11m</t>
         </is>
       </c>
-      <c r="J138" s="2" t="n">
+      <c r="J138" s="1" t="n">
         <v>46571</v>
       </c>
       <c r="K138" t="b">
@@ -6936,7 +6924,7 @@
           <t>-14d</t>
         </is>
       </c>
-      <c r="J139" s="2" t="n">
+      <c r="J139" s="1" t="n">
         <v>46197</v>
       </c>
       <c r="K139" t="b">
@@ -6985,7 +6973,7 @@
           <t>1d</t>
         </is>
       </c>
-      <c r="J140" s="2" t="n">
+      <c r="J140" s="1" t="n">
         <v>46212</v>
       </c>
       <c r="K140" t="b">
@@ -7034,7 +7022,7 @@
           <t>14d</t>
         </is>
       </c>
-      <c r="J141" s="2" t="n">
+      <c r="J141" s="1" t="n">
         <v>46225</v>
       </c>
       <c r="K141" t="b">
@@ -7083,7 +7071,7 @@
           <t>23d</t>
         </is>
       </c>
-      <c r="J142" s="2" t="n">
+      <c r="J142" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="K142" t="b">
@@ -7132,7 +7120,7 @@
           <t>24d</t>
         </is>
       </c>
-      <c r="J143" s="2" t="n">
+      <c r="J143" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="K143" t="b">
@@ -7181,7 +7169,7 @@
           <t>1me23d</t>
         </is>
       </c>
-      <c r="J144" s="2" t="n">
+      <c r="J144" s="1" t="n">
         <v>46263</v>
       </c>
       <c r="K144" t="b">
@@ -7230,7 +7218,7 @@
           <t>1me25d</t>
         </is>
       </c>
-      <c r="J145" s="2" t="n">
+      <c r="J145" s="1" t="n">
         <v>46266</v>
       </c>
       <c r="K145" t="b">
@@ -7275,7 +7263,7 @@
         <v>-1476</v>
       </c>
       <c r="I146" t="inlineStr"/>
-      <c r="J146" s="2" t="n">
+      <c r="J146" s="1" t="n">
         <v>43773</v>
       </c>
       <c r="K146" t="b">
@@ -7320,7 +7308,7 @@
         <v>-1469</v>
       </c>
       <c r="I147" t="inlineStr"/>
-      <c r="J147" s="2" t="n">
+      <c r="J147" s="1" t="n">
         <v>43773</v>
       </c>
       <c r="K147" t="b">
@@ -7365,7 +7353,7 @@
         <v>-1121</v>
       </c>
       <c r="I148" t="inlineStr"/>
-      <c r="J148" s="2" t="n">
+      <c r="J148" s="1" t="n">
         <v>45295</v>
       </c>
       <c r="K148" t="b">
@@ -7410,7 +7398,7 @@
         <v>-1018</v>
       </c>
       <c r="I149" t="inlineStr"/>
-      <c r="J149" s="2" t="n">
+      <c r="J149" s="1" t="n">
         <v>45617</v>
       </c>
       <c r="K149" t="b">
@@ -7455,7 +7443,7 @@
         <v>-950</v>
       </c>
       <c r="I150" t="inlineStr"/>
-      <c r="J150" s="2" t="n">
+      <c r="J150" s="1" t="n">
         <v>45677</v>
       </c>
       <c r="K150" t="b">
@@ -7500,7 +7488,7 @@
         <v>-943</v>
       </c>
       <c r="I151" t="inlineStr"/>
-      <c r="J151" s="2" t="n">
+      <c r="J151" s="1" t="n">
         <v>44944</v>
       </c>
       <c r="K151" t="b">
@@ -7545,7 +7533,7 @@
         <v>-252</v>
       </c>
       <c r="I152" t="inlineStr"/>
-      <c r="J152" s="2" t="n">
+      <c r="J152" s="1" t="n">
         <v>46092</v>
       </c>
       <c r="K152" t="b">
@@ -7590,7 +7578,7 @@
         <v>-196</v>
       </c>
       <c r="I153" t="inlineStr"/>
-      <c r="J153" s="2" t="n">
+      <c r="J153" s="1" t="n">
         <v>45988</v>
       </c>
       <c r="K153" t="b">
@@ -7635,7 +7623,7 @@
         <v>-196</v>
       </c>
       <c r="I154" t="inlineStr"/>
-      <c r="J154" s="2" t="n">
+      <c r="J154" s="1" t="n">
         <v>45988</v>
       </c>
       <c r="K154" t="b">
@@ -7680,7 +7668,7 @@
         <v>-47</v>
       </c>
       <c r="I155" t="inlineStr"/>
-      <c r="J155" s="2" t="n">
+      <c r="J155" s="1" t="n">
         <v>46176</v>
       </c>
       <c r="K155" t="b">
@@ -7725,7 +7713,7 @@
         <v>-47</v>
       </c>
       <c r="I156" t="inlineStr"/>
-      <c r="J156" s="2" t="n">
+      <c r="J156" s="1" t="n">
         <v>46176</v>
       </c>
       <c r="K156" t="b">
@@ -7770,7 +7758,7 @@
         <v>-33</v>
       </c>
       <c r="I157" t="inlineStr"/>
-      <c r="J157" s="2" t="n">
+      <c r="J157" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="K157" t="b">
@@ -7815,7 +7803,7 @@
         <v>-33</v>
       </c>
       <c r="I158" t="inlineStr"/>
-      <c r="J158" s="2" t="n">
+      <c r="J158" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="K158" t="b">
@@ -7860,7 +7848,7 @@
         <v>-6</v>
       </c>
       <c r="I159" t="inlineStr"/>
-      <c r="J159" s="2" t="n">
+      <c r="J159" s="1" t="n">
         <v>45967</v>
       </c>
       <c r="K159" t="b">
@@ -7905,7 +7893,7 @@
         <v>43</v>
       </c>
       <c r="I160" t="inlineStr"/>
-      <c r="J160" s="2" t="n">
+      <c r="J160" s="1" t="n">
         <v>46440</v>
       </c>
       <c r="K160" t="b">
@@ -7950,7 +7938,7 @@
         <v>43</v>
       </c>
       <c r="I161" t="inlineStr"/>
-      <c r="J161" s="2" t="n">
+      <c r="J161" s="1" t="n">
         <v>46440</v>
       </c>
       <c r="K161" t="b">
@@ -7995,7 +7983,7 @@
         <v>73</v>
       </c>
       <c r="I162" t="inlineStr"/>
-      <c r="J162" s="2" t="n">
+      <c r="J162" s="1" t="n">
         <v>46264</v>
       </c>
       <c r="K162" t="b">
@@ -8040,7 +8028,7 @@
         <v>73</v>
       </c>
       <c r="I163" t="inlineStr"/>
-      <c r="J163" s="2" t="n">
+      <c r="J163" s="1" t="n">
         <v>46264</v>
       </c>
       <c r="K163" t="b">
@@ -8085,7 +8073,7 @@
         <v>102</v>
       </c>
       <c r="I164" t="inlineStr"/>
-      <c r="J164" s="2" t="n">
+      <c r="J164" s="1" t="n">
         <v>46463</v>
       </c>
       <c r="K164" t="b">
@@ -8130,7 +8118,7 @@
         <v>118</v>
       </c>
       <c r="I165" t="inlineStr"/>
-      <c r="J165" s="2" t="n">
+      <c r="J165" s="1" t="n">
         <v>46337</v>
       </c>
       <c r="K165" t="b">
@@ -8175,7 +8163,7 @@
         <v>146</v>
       </c>
       <c r="I166" t="inlineStr"/>
-      <c r="J166" s="2" t="n">
+      <c r="J166" s="1" t="n">
         <v>46451</v>
       </c>
       <c r="K166" t="b">
@@ -8220,7 +8208,7 @@
         <v>152</v>
       </c>
       <c r="I167" t="inlineStr"/>
-      <c r="J167" s="2" t="n">
+      <c r="J167" s="1" t="n">
         <v>46245</v>
       </c>
       <c r="K167" t="b">
@@ -8265,7 +8253,7 @@
         <v>152</v>
       </c>
       <c r="I168" t="inlineStr"/>
-      <c r="J168" s="2" t="n">
+      <c r="J168" s="1" t="n">
         <v>46245</v>
       </c>
       <c r="K168" t="b">
@@ -8310,7 +8298,7 @@
         <v>163</v>
       </c>
       <c r="I169" t="inlineStr"/>
-      <c r="J169" s="2" t="n">
+      <c r="J169" s="1" t="n">
         <v>46324</v>
       </c>
       <c r="K169" t="b">
@@ -8355,7 +8343,7 @@
         <v>163</v>
       </c>
       <c r="I170" t="inlineStr"/>
-      <c r="J170" s="2" t="n">
+      <c r="J170" s="1" t="n">
         <v>46324</v>
       </c>
       <c r="K170" t="b">
@@ -8400,7 +8388,7 @@
         <v>164</v>
       </c>
       <c r="I171" t="inlineStr"/>
-      <c r="J171" s="2" t="n">
+      <c r="J171" s="1" t="n">
         <v>46426</v>
       </c>
       <c r="K171" t="b">
@@ -8445,7 +8433,7 @@
         <v>175</v>
       </c>
       <c r="I172" t="inlineStr"/>
-      <c r="J172" s="2" t="n">
+      <c r="J172" s="1" t="n">
         <v>46383</v>
       </c>
       <c r="K172" t="b">
@@ -8490,7 +8478,7 @@
         <v>186</v>
       </c>
       <c r="I173" t="inlineStr"/>
-      <c r="J173" s="2" t="n">
+      <c r="J173" s="1" t="n">
         <v>46392</v>
       </c>
       <c r="K173" t="b">
@@ -8535,7 +8523,7 @@
         <v>205</v>
       </c>
       <c r="I174" t="inlineStr"/>
-      <c r="J174" s="2" t="n">
+      <c r="J174" s="1" t="n">
         <v>46390</v>
       </c>
       <c r="K174" t="b">
@@ -8580,7 +8568,7 @@
         <v>207</v>
       </c>
       <c r="I175" t="inlineStr"/>
-      <c r="J175" s="2" t="n">
+      <c r="J175" s="1" t="n">
         <v>46392</v>
       </c>
       <c r="K175" t="b">
@@ -8625,7 +8613,7 @@
         <v>218</v>
       </c>
       <c r="I176" t="inlineStr"/>
-      <c r="J176" s="2" t="n">
+      <c r="J176" s="1" t="n">
         <v>46506</v>
       </c>
       <c r="K176" t="b">
@@ -8670,7 +8658,7 @@
         <v>246</v>
       </c>
       <c r="I177" t="inlineStr"/>
-      <c r="J177" s="2" t="n">
+      <c r="J177" s="1" t="n">
         <v>46478</v>
       </c>
       <c r="K177" t="b">
@@ -8715,7 +8703,7 @@
         <v>248</v>
       </c>
       <c r="I178" t="inlineStr"/>
-      <c r="J178" s="2" t="n">
+      <c r="J178" s="1" t="n">
         <v>46500</v>
       </c>
       <c r="K178" t="b">
@@ -8760,7 +8748,7 @@
         <v>276</v>
       </c>
       <c r="I179" t="inlineStr"/>
-      <c r="J179" s="2" t="n">
+      <c r="J179" s="1" t="n">
         <v>46430</v>
       </c>
       <c r="K179" t="b">
@@ -8805,7 +8793,7 @@
         <v>276</v>
       </c>
       <c r="I180" t="inlineStr"/>
-      <c r="J180" s="2" t="n">
+      <c r="J180" s="1" t="n">
         <v>46430</v>
       </c>
       <c r="K180" t="b">
@@ -8850,7 +8838,7 @@
         <v>290</v>
       </c>
       <c r="I181" t="inlineStr"/>
-      <c r="J181" s="2" t="n">
+      <c r="J181" s="1" t="n">
         <v>46467</v>
       </c>
       <c r="K181" t="b">
@@ -8895,7 +8883,7 @@
         <v>317</v>
       </c>
       <c r="I182" t="inlineStr"/>
-      <c r="J182" s="2" t="n">
+      <c r="J182" s="1" t="n">
         <v>46529</v>
       </c>
       <c r="K182" t="b">
@@ -8940,7 +8928,7 @@
         <v>420</v>
       </c>
       <c r="I183" t="inlineStr"/>
-      <c r="J183" s="2" t="n">
+      <c r="J183" s="1" t="n">
         <v>46566</v>
       </c>
       <c r="K183" t="b">
@@ -8985,7 +8973,7 @@
         <v>426</v>
       </c>
       <c r="I184" t="inlineStr"/>
-      <c r="J184" s="2" t="n">
+      <c r="J184" s="1" t="n">
         <v>46571</v>
       </c>
       <c r="K184" t="b">
@@ -9030,7 +9018,7 @@
         <v>721</v>
       </c>
       <c r="I185" t="inlineStr"/>
-      <c r="J185" s="2" t="n">
+      <c r="J185" s="1" t="n">
         <v>46325</v>
       </c>
       <c r="K185" t="b">
@@ -9075,7 +9063,7 @@
         <v>721</v>
       </c>
       <c r="I186" t="inlineStr"/>
-      <c r="J186" s="2" t="n">
+      <c r="J186" s="1" t="n">
         <v>46325</v>
       </c>
       <c r="K186" t="b">
@@ -9120,7 +9108,7 @@
         <v>850</v>
       </c>
       <c r="I187" t="inlineStr"/>
-      <c r="J187" s="2" t="n">
+      <c r="J187" s="1" t="n">
         <v>46345</v>
       </c>
       <c r="K187" t="b">
@@ -9165,7 +9153,7 @@
         <v>850</v>
       </c>
       <c r="I188" t="inlineStr"/>
-      <c r="J188" s="2" t="n">
+      <c r="J188" s="1" t="n">
         <v>46345</v>
       </c>
       <c r="K188" t="b">
@@ -9210,7 +9198,7 @@
         <v>1661</v>
       </c>
       <c r="I189" t="inlineStr"/>
-      <c r="J189" s="2" t="n">
+      <c r="J189" s="1" t="n">
         <v>46498</v>
       </c>
       <c r="K189" t="b">
@@ -9255,7 +9243,7 @@
         <v>1661</v>
       </c>
       <c r="I190" t="inlineStr"/>
-      <c r="J190" s="2" t="n">
+      <c r="J190" s="1" t="n">
         <v>46498</v>
       </c>
       <c r="K190" t="b">
@@ -9300,7 +9288,7 @@
         <v>488</v>
       </c>
       <c r="I191" t="inlineStr"/>
-      <c r="J191" s="2" t="n">
+      <c r="J191" s="1" t="n">
         <v>46190</v>
       </c>
       <c r="K191" t="b">
@@ -9345,7 +9333,7 @@
         <v>25565</v>
       </c>
       <c r="I192" t="inlineStr"/>
-      <c r="J192" s="2" t="n">
+      <c r="J192" s="1" t="n">
         <v>46190</v>
       </c>
       <c r="K192" t="b">
@@ -9390,7 +9378,7 @@
         <v>25567</v>
       </c>
       <c r="I193" t="inlineStr"/>
-      <c r="J193" s="2" t="n">
+      <c r="J193" s="1" t="n">
         <v>46190</v>
       </c>
       <c r="K193" t="b">
@@ -9435,7 +9423,7 @@
         <v>31293</v>
       </c>
       <c r="I194" t="inlineStr"/>
-      <c r="J194" s="2" t="n">
+      <c r="J194" s="1" t="n">
         <v>46190</v>
       </c>
       <c r="K194" t="b">

</xml_diff>

<commit_message>
Atualização automática: vencimentos_tmot (22/07/2026 12:02)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
@@ -1040,8 +1040,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1057,7 +1065,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1065,12 +1073,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1370,37 +1396,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1429,7 +1455,7 @@
       <c r="H2">
         <v>-4402.8</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>41388</v>
       </c>
       <c r="K2" t="b">
@@ -1461,7 +1487,7 @@
       <c r="H3">
         <v>-4254.8</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>39285</v>
       </c>
       <c r="K3" t="b">
@@ -1493,7 +1519,7 @@
       <c r="H4">
         <v>-2354.2</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>40669</v>
       </c>
       <c r="K4" t="b">
@@ -1525,7 +1551,7 @@
       <c r="H5">
         <v>-896.8</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>40669</v>
       </c>
       <c r="K5" t="b">
@@ -1557,7 +1583,7 @@
       <c r="H6">
         <v>-854.1</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>44884</v>
       </c>
       <c r="K6" t="b">
@@ -1589,7 +1615,7 @@
       <c r="H7">
         <v>-413.2</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>43855</v>
       </c>
       <c r="K7" t="b">
@@ -1621,7 +1647,7 @@
       <c r="H8">
         <v>-391.8</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>42769</v>
       </c>
       <c r="K8" t="b">
@@ -1653,7 +1679,7 @@
       <c r="H9">
         <v>-371.5</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>46014</v>
       </c>
       <c r="K9" t="b">
@@ -1685,7 +1711,7 @@
       <c r="H10">
         <v>-368.8</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>46014</v>
       </c>
       <c r="K10" t="b">
@@ -1717,7 +1743,7 @@
       <c r="H11">
         <v>-359</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>45804</v>
       </c>
       <c r="K11" t="b">
@@ -1749,7 +1775,7 @@
       <c r="H12">
         <v>-359</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>45804</v>
       </c>
       <c r="K12" t="b">
@@ -1781,7 +1807,7 @@
       <c r="H13">
         <v>-351</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>42821</v>
       </c>
       <c r="K13" t="b">
@@ -1813,7 +1839,7 @@
       <c r="H14">
         <v>-351</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>46014</v>
       </c>
       <c r="K14" t="b">
@@ -1845,7 +1871,7 @@
       <c r="H15">
         <v>-351</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>46014</v>
       </c>
       <c r="K15" t="b">
@@ -1877,7 +1903,7 @@
       <c r="H16">
         <v>-351</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="2">
         <v>46014</v>
       </c>
       <c r="K16" t="b">
@@ -1909,7 +1935,7 @@
       <c r="H17">
         <v>-345.8</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="2">
         <v>46017</v>
       </c>
       <c r="K17" t="b">
@@ -1941,7 +1967,7 @@
       <c r="H18">
         <v>-345.8</v>
       </c>
-      <c r="J18" s="1">
+      <c r="J18" s="2">
         <v>46017</v>
       </c>
       <c r="K18" t="b">
@@ -1973,7 +1999,7 @@
       <c r="H19">
         <v>-264.2</v>
       </c>
-      <c r="J19" s="1">
+      <c r="J19" s="2">
         <v>40979</v>
       </c>
       <c r="K19" t="b">
@@ -2005,7 +2031,7 @@
       <c r="H20">
         <v>-206.4</v>
       </c>
-      <c r="J20" s="1">
+      <c r="J20" s="2">
         <v>36669</v>
       </c>
       <c r="K20" t="b">
@@ -2037,7 +2063,7 @@
       <c r="H21">
         <v>-131.6</v>
       </c>
-      <c r="J21" s="1">
+      <c r="J21" s="2">
         <v>46111</v>
       </c>
       <c r="K21" t="b">
@@ -2069,7 +2095,7 @@
       <c r="H22">
         <v>-131.6</v>
       </c>
-      <c r="J22" s="1">
+      <c r="J22" s="2">
         <v>46111</v>
       </c>
       <c r="K22" t="b">
@@ -2101,7 +2127,7 @@
       <c r="H23">
         <v>-131.6</v>
       </c>
-      <c r="J23" s="1">
+      <c r="J23" s="2">
         <v>46111</v>
       </c>
       <c r="K23" t="b">
@@ -2133,7 +2159,7 @@
       <c r="H24">
         <v>-131.6</v>
       </c>
-      <c r="J24" s="1">
+      <c r="J24" s="2">
         <v>46111</v>
       </c>
       <c r="K24" t="b">
@@ -2165,7 +2191,7 @@
       <c r="H25">
         <v>-131.6</v>
       </c>
-      <c r="J25" s="1">
+      <c r="J25" s="2">
         <v>46111</v>
       </c>
       <c r="K25" t="b">
@@ -2197,7 +2223,7 @@
       <c r="H26">
         <v>-105</v>
       </c>
-      <c r="J26" s="1">
+      <c r="J26" s="2">
         <v>46161</v>
       </c>
       <c r="K26" t="b">
@@ -2229,7 +2255,7 @@
       <c r="H27">
         <v>-79.8</v>
       </c>
-      <c r="J27" s="1">
+      <c r="J27" s="2">
         <v>43340</v>
       </c>
       <c r="K27" t="b">
@@ -2261,7 +2287,7 @@
       <c r="H28">
         <v>-12.3</v>
       </c>
-      <c r="J28" s="1">
+      <c r="J28" s="2">
         <v>46048</v>
       </c>
       <c r="K28" t="b">
@@ -2293,7 +2319,7 @@
       <c r="H29">
         <v>0</v>
       </c>
-      <c r="J29" s="1">
+      <c r="J29" s="2">
         <v>46211</v>
       </c>
       <c r="K29" t="b">
@@ -2325,7 +2351,7 @@
       <c r="H30">
         <v>3.6</v>
       </c>
-      <c r="J30" s="1">
+      <c r="J30" s="2">
         <v>46234</v>
       </c>
       <c r="K30" t="b">
@@ -2357,7 +2383,7 @@
       <c r="H31">
         <v>6.2</v>
       </c>
-      <c r="J31" s="1">
+      <c r="J31" s="2">
         <v>46234</v>
       </c>
       <c r="K31" t="b">
@@ -2389,7 +2415,7 @@
       <c r="H32">
         <v>7.5</v>
       </c>
-      <c r="J32" s="1">
+      <c r="J32" s="2">
         <v>46234</v>
       </c>
       <c r="K32" t="b">
@@ -2421,7 +2447,7 @@
       <c r="H33">
         <v>10.7</v>
       </c>
-      <c r="J33" s="1">
+      <c r="J33" s="2">
         <v>46234</v>
       </c>
       <c r="K33" t="b">
@@ -2453,7 +2479,7 @@
       <c r="H34">
         <v>20</v>
       </c>
-      <c r="J34" s="1">
+      <c r="J34" s="2">
         <v>46234</v>
       </c>
       <c r="K34" t="b">
@@ -2485,7 +2511,7 @@
       <c r="H35">
         <v>30.8</v>
       </c>
-      <c r="J35" s="1">
+      <c r="J35" s="2">
         <v>46234</v>
       </c>
       <c r="K35" t="b">
@@ -2517,7 +2543,7 @@
       <c r="H36">
         <v>37.1</v>
       </c>
-      <c r="J36" s="1">
+      <c r="J36" s="2">
         <v>46256</v>
       </c>
       <c r="K36" t="b">
@@ -2549,7 +2575,7 @@
       <c r="H37">
         <v>42.8</v>
       </c>
-      <c r="J37" s="1">
+      <c r="J37" s="2">
         <v>46276</v>
       </c>
       <c r="K37" t="b">
@@ -2581,7 +2607,7 @@
       <c r="H38">
         <v>45.2</v>
       </c>
-      <c r="J38" s="1">
+      <c r="J38" s="2">
         <v>46234</v>
       </c>
       <c r="K38" t="b">
@@ -2613,7 +2639,7 @@
       <c r="H39">
         <v>46</v>
       </c>
-      <c r="J39" s="1">
+      <c r="J39" s="2">
         <v>46251</v>
       </c>
       <c r="K39" t="b">
@@ -2645,7 +2671,7 @@
       <c r="H40">
         <v>47.5</v>
       </c>
-      <c r="J40" s="1">
+      <c r="J40" s="2">
         <v>46456</v>
       </c>
       <c r="K40" t="b">
@@ -2677,7 +2703,7 @@
       <c r="H41">
         <v>57.2</v>
       </c>
-      <c r="J41" s="1">
+      <c r="J41" s="2">
         <v>46246</v>
       </c>
       <c r="K41" t="b">
@@ -2709,7 +2735,7 @@
       <c r="H42">
         <v>59.6</v>
       </c>
-      <c r="J42" s="1">
+      <c r="J42" s="2">
         <v>46487</v>
       </c>
       <c r="K42" t="b">
@@ -2741,7 +2767,7 @@
       <c r="H43">
         <v>75.40000000000001</v>
       </c>
-      <c r="J43" s="1">
+      <c r="J43" s="2">
         <v>46283</v>
       </c>
       <c r="K43" t="b">
@@ -2773,7 +2799,7 @@
       <c r="H44">
         <v>76.8</v>
       </c>
-      <c r="J44" s="1">
+      <c r="J44" s="2">
         <v>46285</v>
       </c>
       <c r="K44" t="b">
@@ -2805,7 +2831,7 @@
       <c r="H45">
         <v>83.2</v>
       </c>
-      <c r="J45" s="1">
+      <c r="J45" s="2">
         <v>46547</v>
       </c>
       <c r="K45" t="b">
@@ -2837,7 +2863,7 @@
       <c r="H46">
         <v>84.5</v>
       </c>
-      <c r="J46" s="1">
+      <c r="J46" s="2">
         <v>46240</v>
       </c>
       <c r="K46" t="b">
@@ -2869,7 +2895,7 @@
       <c r="H47">
         <v>85.8</v>
       </c>
-      <c r="J47" s="1">
+      <c r="J47" s="2">
         <v>46266</v>
       </c>
       <c r="K47" t="b">
@@ -2901,7 +2927,7 @@
       <c r="H48">
         <v>86.5</v>
       </c>
-      <c r="J48" s="1">
+      <c r="J48" s="2">
         <v>46241</v>
       </c>
       <c r="K48" t="b">
@@ -2933,7 +2959,7 @@
       <c r="H49">
         <v>91.7</v>
       </c>
-      <c r="J49" s="1">
+      <c r="J49" s="2">
         <v>46243</v>
       </c>
       <c r="K49" t="b">
@@ -2965,7 +2991,7 @@
       <c r="H50">
         <v>91.7</v>
       </c>
-      <c r="J50" s="1">
+      <c r="J50" s="2">
         <v>46243</v>
       </c>
       <c r="K50" t="b">
@@ -2997,7 +3023,7 @@
       <c r="H51">
         <v>91.7</v>
       </c>
-      <c r="J51" s="1">
+      <c r="J51" s="2">
         <v>46250</v>
       </c>
       <c r="K51" t="b">
@@ -3029,7 +3055,7 @@
       <c r="H52">
         <v>98.90000000000001</v>
       </c>
-      <c r="J52" s="1">
+      <c r="J52" s="2">
         <v>46253</v>
       </c>
       <c r="K52" t="b">
@@ -3061,7 +3087,7 @@
       <c r="H53">
         <v>105.5</v>
       </c>
-      <c r="J53" s="1">
+      <c r="J53" s="2">
         <v>46280</v>
       </c>
       <c r="K53" t="b">
@@ -3093,7 +3119,7 @@
       <c r="H54">
         <v>105.6</v>
       </c>
-      <c r="J54" s="1">
+      <c r="J54" s="2">
         <v>46361</v>
       </c>
       <c r="K54" t="b">
@@ -3125,7 +3151,7 @@
       <c r="H55">
         <v>105.7</v>
       </c>
-      <c r="J55" s="1">
+      <c r="J55" s="2">
         <v>46362</v>
       </c>
       <c r="K55" t="b">
@@ -3157,7 +3183,7 @@
       <c r="H56">
         <v>110.7</v>
       </c>
-      <c r="J56" s="1">
+      <c r="J56" s="2">
         <v>46275</v>
       </c>
       <c r="K56" t="b">
@@ -3189,7 +3215,7 @@
       <c r="H57">
         <v>113.2</v>
       </c>
-      <c r="J57" s="1">
+      <c r="J57" s="2">
         <v>46377</v>
       </c>
       <c r="K57" t="b">
@@ -3221,7 +3247,7 @@
       <c r="H58">
         <v>128.8</v>
       </c>
-      <c r="J58" s="1">
+      <c r="J58" s="2">
         <v>46434</v>
       </c>
       <c r="K58" t="b">
@@ -3253,7 +3279,7 @@
       <c r="H59">
         <v>128.8</v>
       </c>
-      <c r="J59" s="1">
+      <c r="J59" s="2">
         <v>46434</v>
       </c>
       <c r="K59" t="b">
@@ -3285,7 +3311,7 @@
       <c r="H60">
         <v>128.8</v>
       </c>
-      <c r="J60" s="1">
+      <c r="J60" s="2">
         <v>46434</v>
       </c>
       <c r="K60" t="b">
@@ -3317,7 +3343,7 @@
       <c r="H61">
         <v>128.8</v>
       </c>
-      <c r="J61" s="1">
+      <c r="J61" s="2">
         <v>46434</v>
       </c>
       <c r="K61" t="b">
@@ -3349,7 +3375,7 @@
       <c r="H62">
         <v>128.8</v>
       </c>
-      <c r="J62" s="1">
+      <c r="J62" s="2">
         <v>46434</v>
       </c>
       <c r="K62" t="b">
@@ -3381,7 +3407,7 @@
       <c r="H63">
         <v>135</v>
       </c>
-      <c r="J63" s="1">
+      <c r="J63" s="2">
         <v>46280</v>
       </c>
       <c r="K63" t="b">
@@ -3413,7 +3439,7 @@
       <c r="H64">
         <v>150.6</v>
       </c>
-      <c r="J64" s="1">
+      <c r="J64" s="2">
         <v>46271</v>
       </c>
       <c r="K64" t="b">
@@ -3445,7 +3471,7 @@
       <c r="H65">
         <v>174.2</v>
       </c>
-      <c r="J65" s="1">
+      <c r="J65" s="2">
         <v>46363</v>
       </c>
       <c r="K65" t="b">
@@ -3477,7 +3503,7 @@
       <c r="H66">
         <v>176.6</v>
       </c>
-      <c r="J66" s="1">
+      <c r="J66" s="2">
         <v>46334</v>
       </c>
       <c r="K66" t="b">
@@ -3509,7 +3535,7 @@
       <c r="H67">
         <v>177.4</v>
       </c>
-      <c r="J67" s="1">
+      <c r="J67" s="2">
         <v>46407</v>
       </c>
       <c r="K67" t="b">
@@ -3541,7 +3567,7 @@
       <c r="H68">
         <v>183.9</v>
       </c>
-      <c r="J68" s="1">
+      <c r="J68" s="2">
         <v>46341</v>
       </c>
       <c r="K68" t="b">
@@ -3573,7 +3599,7 @@
       <c r="H69">
         <v>191.7</v>
       </c>
-      <c r="J69" s="1">
+      <c r="J69" s="2">
         <v>46300</v>
       </c>
       <c r="K69" t="b">
@@ -3605,7 +3631,7 @@
       <c r="H70">
         <v>200</v>
       </c>
-      <c r="J70" s="1">
+      <c r="J70" s="2">
         <v>46336</v>
       </c>
       <c r="K70" t="b">
@@ -3637,7 +3663,7 @@
       <c r="H71">
         <v>201.1</v>
       </c>
-      <c r="J71" s="1">
+      <c r="J71" s="2">
         <v>46319</v>
       </c>
       <c r="K71" t="b">
@@ -3669,7 +3695,7 @@
       <c r="H72">
         <v>206.5</v>
       </c>
-      <c r="J72" s="1">
+      <c r="J72" s="2">
         <v>46308</v>
       </c>
       <c r="K72" t="b">
@@ -3701,7 +3727,7 @@
       <c r="H73">
         <v>207.5</v>
       </c>
-      <c r="J73" s="1">
+      <c r="J73" s="2">
         <v>46390</v>
       </c>
       <c r="K73" t="b">
@@ -3733,7 +3759,7 @@
       <c r="H74">
         <v>247</v>
       </c>
-      <c r="J74" s="1">
+      <c r="J74" s="2">
         <v>46443</v>
       </c>
       <c r="K74" t="b">
@@ -3765,7 +3791,7 @@
       <c r="H75">
         <v>285.3</v>
       </c>
-      <c r="J75" s="1">
+      <c r="J75" s="2">
         <v>46304</v>
       </c>
       <c r="K75" t="b">
@@ -3797,7 +3823,7 @@
       <c r="H76">
         <v>290.8</v>
       </c>
-      <c r="J76" s="1">
+      <c r="J76" s="2">
         <v>46362</v>
       </c>
       <c r="K76" t="b">
@@ -3829,7 +3855,7 @@
       <c r="H77">
         <v>295.2</v>
       </c>
-      <c r="J77" s="1">
+      <c r="J77" s="2">
         <v>46463</v>
       </c>
       <c r="K77" t="b">
@@ -3861,7 +3887,7 @@
       <c r="H78">
         <v>300.2</v>
       </c>
-      <c r="J78" s="1">
+      <c r="J78" s="2">
         <v>46466</v>
       </c>
       <c r="K78" t="b">
@@ -3896,7 +3922,7 @@
       <c r="I79" t="s">
         <v>313</v>
       </c>
-      <c r="J79" s="1">
+      <c r="J79" s="2">
         <v>36557</v>
       </c>
       <c r="K79" t="b">
@@ -3931,7 +3957,7 @@
       <c r="I80" t="s">
         <v>314</v>
       </c>
-      <c r="J80" s="1">
+      <c r="J80" s="2">
         <v>41275</v>
       </c>
       <c r="K80" t="b">
@@ -3966,7 +3992,7 @@
       <c r="I81" t="s">
         <v>315</v>
       </c>
-      <c r="J81" s="1">
+      <c r="J81" s="2">
         <v>45380</v>
       </c>
       <c r="K81" t="b">
@@ -4001,7 +4027,7 @@
       <c r="I82" t="s">
         <v>316</v>
       </c>
-      <c r="J82" s="1">
+      <c r="J82" s="2">
         <v>45421</v>
       </c>
       <c r="K82" t="b">
@@ -4036,7 +4062,7 @@
       <c r="I83" t="s">
         <v>316</v>
       </c>
-      <c r="J83" s="1">
+      <c r="J83" s="2">
         <v>45428</v>
       </c>
       <c r="K83" t="b">
@@ -4071,7 +4097,7 @@
       <c r="I84" t="s">
         <v>317</v>
       </c>
-      <c r="J84" s="1">
+      <c r="J84" s="2">
         <v>45490</v>
       </c>
       <c r="K84" t="b">
@@ -4106,7 +4132,7 @@
       <c r="I85" t="s">
         <v>318</v>
       </c>
-      <c r="J85" s="1">
+      <c r="J85" s="2">
         <v>45566</v>
       </c>
       <c r="K85" t="b">
@@ -4141,7 +4167,7 @@
       <c r="I86" t="s">
         <v>319</v>
       </c>
-      <c r="J86" s="1">
+      <c r="J86" s="2">
         <v>45986</v>
       </c>
       <c r="K86" t="b">
@@ -4176,7 +4202,7 @@
       <c r="I87" t="s">
         <v>320</v>
       </c>
-      <c r="J87" s="1">
+      <c r="J87" s="2">
         <v>46106</v>
       </c>
       <c r="K87" t="b">
@@ -4211,7 +4237,7 @@
       <c r="I88" t="s">
         <v>321</v>
       </c>
-      <c r="J88" s="1">
+      <c r="J88" s="2">
         <v>46142</v>
       </c>
       <c r="K88" t="b">
@@ -4246,7 +4272,7 @@
       <c r="I89" t="s">
         <v>322</v>
       </c>
-      <c r="J89" s="1">
+      <c r="J89" s="2">
         <v>46274</v>
       </c>
       <c r="K89" t="b">
@@ -4281,7 +4307,7 @@
       <c r="I90" t="s">
         <v>322</v>
       </c>
-      <c r="J90" s="1">
+      <c r="J90" s="2">
         <v>46276</v>
       </c>
       <c r="K90" t="b">
@@ -4316,7 +4342,7 @@
       <c r="I91" t="s">
         <v>322</v>
       </c>
-      <c r="J91" s="1">
+      <c r="J91" s="2">
         <v>46284</v>
       </c>
       <c r="K91" t="b">
@@ -4351,7 +4377,7 @@
       <c r="I92" t="s">
         <v>323</v>
       </c>
-      <c r="J92" s="1">
+      <c r="J92" s="2">
         <v>46317</v>
       </c>
       <c r="K92" t="b">
@@ -4386,7 +4412,7 @@
       <c r="I93" t="s">
         <v>323</v>
       </c>
-      <c r="J93" s="1">
+      <c r="J93" s="2">
         <v>46319</v>
       </c>
       <c r="K93" t="b">
@@ -4421,7 +4447,7 @@
       <c r="I94" t="s">
         <v>324</v>
       </c>
-      <c r="J94" s="1">
+      <c r="J94" s="2">
         <v>46333</v>
       </c>
       <c r="K94" t="b">
@@ -4456,7 +4482,7 @@
       <c r="I95" t="s">
         <v>324</v>
       </c>
-      <c r="J95" s="1">
+      <c r="J95" s="2">
         <v>46338</v>
       </c>
       <c r="K95" t="b">
@@ -4491,7 +4517,7 @@
       <c r="I96" t="s">
         <v>324</v>
       </c>
-      <c r="J96" s="1">
+      <c r="J96" s="2">
         <v>46338</v>
       </c>
       <c r="K96" t="b">
@@ -4526,7 +4552,7 @@
       <c r="I97" t="s">
         <v>324</v>
       </c>
-      <c r="J97" s="1">
+      <c r="J97" s="2">
         <v>46341</v>
       </c>
       <c r="K97" t="b">
@@ -4561,7 +4587,7 @@
       <c r="I98" t="s">
         <v>324</v>
       </c>
-      <c r="J98" s="1">
+      <c r="J98" s="2">
         <v>46344</v>
       </c>
       <c r="K98" t="b">
@@ -4596,7 +4622,7 @@
       <c r="I99" t="s">
         <v>324</v>
       </c>
-      <c r="J99" s="1">
+      <c r="J99" s="2">
         <v>46354</v>
       </c>
       <c r="K99" t="b">
@@ -4631,7 +4657,7 @@
       <c r="I100" t="s">
         <v>324</v>
       </c>
-      <c r="J100" s="1">
+      <c r="J100" s="2">
         <v>46360</v>
       </c>
       <c r="K100" t="b">
@@ -4666,7 +4692,7 @@
       <c r="I101" t="s">
         <v>324</v>
       </c>
-      <c r="J101" s="1">
+      <c r="J101" s="2">
         <v>46360</v>
       </c>
       <c r="K101" t="b">
@@ -4701,7 +4727,7 @@
       <c r="I102" t="s">
         <v>325</v>
       </c>
-      <c r="J102" s="1">
+      <c r="J102" s="2">
         <v>46366</v>
       </c>
       <c r="K102" t="b">
@@ -4736,7 +4762,7 @@
       <c r="I103" t="s">
         <v>325</v>
       </c>
-      <c r="J103" s="1">
+      <c r="J103" s="2">
         <v>46375</v>
       </c>
       <c r="K103" t="b">
@@ -4771,7 +4797,7 @@
       <c r="I104" t="s">
         <v>325</v>
       </c>
-      <c r="J104" s="1">
+      <c r="J104" s="2">
         <v>46388</v>
       </c>
       <c r="K104" t="b">
@@ -4806,7 +4832,7 @@
       <c r="I105" t="s">
         <v>326</v>
       </c>
-      <c r="J105" s="1">
+      <c r="J105" s="2">
         <v>46401</v>
       </c>
       <c r="K105" t="b">
@@ -4841,7 +4867,7 @@
       <c r="I106" t="s">
         <v>326</v>
       </c>
-      <c r="J106" s="1">
+      <c r="J106" s="2">
         <v>46401</v>
       </c>
       <c r="K106" t="b">
@@ -4876,7 +4902,7 @@
       <c r="I107" t="s">
         <v>326</v>
       </c>
-      <c r="J107" s="1">
+      <c r="J107" s="2">
         <v>46401</v>
       </c>
       <c r="K107" t="b">
@@ -4911,7 +4937,7 @@
       <c r="I108" t="s">
         <v>326</v>
       </c>
-      <c r="J108" s="1">
+      <c r="J108" s="2">
         <v>46413</v>
       </c>
       <c r="K108" t="b">
@@ -4946,7 +4972,7 @@
       <c r="I109" t="s">
         <v>327</v>
       </c>
-      <c r="J109" s="1">
+      <c r="J109" s="2">
         <v>46424</v>
       </c>
       <c r="K109" t="b">
@@ -4981,7 +5007,7 @@
       <c r="I110" t="s">
         <v>327</v>
       </c>
-      <c r="J110" s="1">
+      <c r="J110" s="2">
         <v>46427</v>
       </c>
       <c r="K110" t="b">
@@ -5016,7 +5042,7 @@
       <c r="I111" t="s">
         <v>327</v>
       </c>
-      <c r="J111" s="1">
+      <c r="J111" s="2">
         <v>46437</v>
       </c>
       <c r="K111" t="b">
@@ -5051,7 +5077,7 @@
       <c r="I112" t="s">
         <v>327</v>
       </c>
-      <c r="J112" s="1">
+      <c r="J112" s="2">
         <v>46451</v>
       </c>
       <c r="K112" t="b">
@@ -5086,7 +5112,7 @@
       <c r="I113" t="s">
         <v>328</v>
       </c>
-      <c r="J113" s="1">
+      <c r="J113" s="2">
         <v>46455</v>
       </c>
       <c r="K113" t="b">
@@ -5121,7 +5147,7 @@
       <c r="I114" t="s">
         <v>328</v>
       </c>
-      <c r="J114" s="1">
+      <c r="J114" s="2">
         <v>46457</v>
       </c>
       <c r="K114" t="b">
@@ -5156,7 +5182,7 @@
       <c r="I115" t="s">
         <v>328</v>
       </c>
-      <c r="J115" s="1">
+      <c r="J115" s="2">
         <v>46462</v>
       </c>
       <c r="K115" t="b">
@@ -5191,7 +5217,7 @@
       <c r="I116" t="s">
         <v>328</v>
       </c>
-      <c r="J116" s="1">
+      <c r="J116" s="2">
         <v>46464</v>
       </c>
       <c r="K116" t="b">
@@ -5226,7 +5252,7 @@
       <c r="I117" t="s">
         <v>328</v>
       </c>
-      <c r="J117" s="1">
+      <c r="J117" s="2">
         <v>46470</v>
       </c>
       <c r="K117" t="b">
@@ -5261,7 +5287,7 @@
       <c r="I118" t="s">
         <v>329</v>
       </c>
-      <c r="J118" s="1">
+      <c r="J118" s="2">
         <v>46485</v>
       </c>
       <c r="K118" t="b">
@@ -5296,7 +5322,7 @@
       <c r="I119" t="s">
         <v>329</v>
       </c>
-      <c r="J119" s="1">
+      <c r="J119" s="2">
         <v>46499</v>
       </c>
       <c r="K119" t="b">
@@ -5331,7 +5357,7 @@
       <c r="I120" t="s">
         <v>329</v>
       </c>
-      <c r="J120" s="1">
+      <c r="J120" s="2">
         <v>46504</v>
       </c>
       <c r="K120" t="b">
@@ -5366,7 +5392,7 @@
       <c r="I121" t="s">
         <v>329</v>
       </c>
-      <c r="J121" s="1">
+      <c r="J121" s="2">
         <v>46504</v>
       </c>
       <c r="K121" t="b">
@@ -5401,7 +5427,7 @@
       <c r="I122" t="s">
         <v>329</v>
       </c>
-      <c r="J122" s="1">
+      <c r="J122" s="2">
         <v>46507</v>
       </c>
       <c r="K122" t="b">
@@ -5436,7 +5462,7 @@
       <c r="I123" t="s">
         <v>329</v>
       </c>
-      <c r="J123" s="1">
+      <c r="J123" s="2">
         <v>46508</v>
       </c>
       <c r="K123" t="b">
@@ -5471,7 +5497,7 @@
       <c r="I124" t="s">
         <v>329</v>
       </c>
-      <c r="J124" s="1">
+      <c r="J124" s="2">
         <v>46512</v>
       </c>
       <c r="K124" t="b">
@@ -5506,7 +5532,7 @@
       <c r="I125" t="s">
         <v>329</v>
       </c>
-      <c r="J125" s="1">
+      <c r="J125" s="2">
         <v>46512</v>
       </c>
       <c r="K125" t="b">
@@ -5541,7 +5567,7 @@
       <c r="I126" t="s">
         <v>330</v>
       </c>
-      <c r="J126" s="1">
+      <c r="J126" s="2">
         <v>46528</v>
       </c>
       <c r="K126" t="b">
@@ -5576,7 +5602,7 @@
       <c r="I127" t="s">
         <v>330</v>
       </c>
-      <c r="J127" s="1">
+      <c r="J127" s="2">
         <v>46529</v>
       </c>
       <c r="K127" t="b">
@@ -5611,7 +5637,7 @@
       <c r="I128" t="s">
         <v>330</v>
       </c>
-      <c r="J128" s="1">
+      <c r="J128" s="2">
         <v>46537</v>
       </c>
       <c r="K128" t="b">
@@ -5646,7 +5672,7 @@
       <c r="I129" t="s">
         <v>331</v>
       </c>
-      <c r="J129" s="1">
+      <c r="J129" s="2">
         <v>46546</v>
       </c>
       <c r="K129" t="b">
@@ -5681,7 +5707,7 @@
       <c r="I130" t="s">
         <v>331</v>
       </c>
-      <c r="J130" s="1">
+      <c r="J130" s="2">
         <v>46547</v>
       </c>
       <c r="K130" t="b">
@@ -5716,7 +5742,7 @@
       <c r="I131" t="s">
         <v>331</v>
       </c>
-      <c r="J131" s="1">
+      <c r="J131" s="2">
         <v>46547</v>
       </c>
       <c r="K131" t="b">
@@ -5751,7 +5777,7 @@
       <c r="I132" t="s">
         <v>331</v>
       </c>
-      <c r="J132" s="1">
+      <c r="J132" s="2">
         <v>46547</v>
       </c>
       <c r="K132" t="b">
@@ -5786,7 +5812,7 @@
       <c r="I133" t="s">
         <v>331</v>
       </c>
-      <c r="J133" s="1">
+      <c r="J133" s="2">
         <v>46551</v>
       </c>
       <c r="K133" t="b">
@@ -5821,7 +5847,7 @@
       <c r="I134" t="s">
         <v>331</v>
       </c>
-      <c r="J134" s="1">
+      <c r="J134" s="2">
         <v>46560</v>
       </c>
       <c r="K134" t="b">
@@ -5856,7 +5882,7 @@
       <c r="I135" t="s">
         <v>331</v>
       </c>
-      <c r="J135" s="1">
+      <c r="J135" s="2">
         <v>46564</v>
       </c>
       <c r="K135" t="b">
@@ -5891,7 +5917,7 @@
       <c r="I136" t="s">
         <v>331</v>
       </c>
-      <c r="J136" s="1">
+      <c r="J136" s="2">
         <v>46567</v>
       </c>
       <c r="K136" t="b">
@@ -5926,7 +5952,7 @@
       <c r="I137" t="s">
         <v>331</v>
       </c>
-      <c r="J137" s="1">
+      <c r="J137" s="2">
         <v>46568</v>
       </c>
       <c r="K137" t="b">
@@ -5961,7 +5987,7 @@
       <c r="I138" t="s">
         <v>331</v>
       </c>
-      <c r="J138" s="1">
+      <c r="J138" s="2">
         <v>46571</v>
       </c>
       <c r="K138" t="b">
@@ -5996,7 +6022,7 @@
       <c r="I139" t="s">
         <v>332</v>
       </c>
-      <c r="J139" s="1">
+      <c r="J139" s="2">
         <v>46197</v>
       </c>
       <c r="K139" t="b">
@@ -6031,7 +6057,7 @@
       <c r="I140" t="s">
         <v>333</v>
       </c>
-      <c r="J140" s="1">
+      <c r="J140" s="2">
         <v>46212</v>
       </c>
       <c r="K140" t="b">
@@ -6066,7 +6092,7 @@
       <c r="I141" t="s">
         <v>334</v>
       </c>
-      <c r="J141" s="1">
+      <c r="J141" s="2">
         <v>46225</v>
       </c>
       <c r="K141" t="b">
@@ -6101,7 +6127,7 @@
       <c r="I142" t="s">
         <v>335</v>
       </c>
-      <c r="J142" s="1">
+      <c r="J142" s="2">
         <v>46234</v>
       </c>
       <c r="K142" t="b">
@@ -6136,7 +6162,7 @@
       <c r="I143" t="s">
         <v>336</v>
       </c>
-      <c r="J143" s="1">
+      <c r="J143" s="2">
         <v>46234</v>
       </c>
       <c r="K143" t="b">
@@ -6171,7 +6197,7 @@
       <c r="I144" t="s">
         <v>337</v>
       </c>
-      <c r="J144" s="1">
+      <c r="J144" s="2">
         <v>46263</v>
       </c>
       <c r="K144" t="b">
@@ -6206,7 +6232,7 @@
       <c r="I145" t="s">
         <v>338</v>
       </c>
-      <c r="J145" s="1">
+      <c r="J145" s="2">
         <v>46266</v>
       </c>
       <c r="K145" t="b">
@@ -6238,7 +6264,7 @@
       <c r="H146">
         <v>-1476</v>
       </c>
-      <c r="J146" s="1">
+      <c r="J146" s="2">
         <v>43773</v>
       </c>
       <c r="K146" t="b">
@@ -6270,7 +6296,7 @@
       <c r="H147">
         <v>-1469</v>
       </c>
-      <c r="J147" s="1">
+      <c r="J147" s="2">
         <v>43773</v>
       </c>
       <c r="K147" t="b">
@@ -6302,7 +6328,7 @@
       <c r="H148">
         <v>-1121</v>
       </c>
-      <c r="J148" s="1">
+      <c r="J148" s="2">
         <v>45295</v>
       </c>
       <c r="K148" t="b">
@@ -6334,7 +6360,7 @@
       <c r="H149">
         <v>-1018</v>
       </c>
-      <c r="J149" s="1">
+      <c r="J149" s="2">
         <v>45617</v>
       </c>
       <c r="K149" t="b">
@@ -6366,7 +6392,7 @@
       <c r="H150">
         <v>-950</v>
       </c>
-      <c r="J150" s="1">
+      <c r="J150" s="2">
         <v>45677</v>
       </c>
       <c r="K150" t="b">
@@ -6398,7 +6424,7 @@
       <c r="H151">
         <v>-943</v>
       </c>
-      <c r="J151" s="1">
+      <c r="J151" s="2">
         <v>44944</v>
       </c>
       <c r="K151" t="b">
@@ -6430,7 +6456,7 @@
       <c r="H152">
         <v>-252</v>
       </c>
-      <c r="J152" s="1">
+      <c r="J152" s="2">
         <v>46092</v>
       </c>
       <c r="K152" t="b">
@@ -6462,7 +6488,7 @@
       <c r="H153">
         <v>-196</v>
       </c>
-      <c r="J153" s="1">
+      <c r="J153" s="2">
         <v>45988</v>
       </c>
       <c r="K153" t="b">
@@ -6494,7 +6520,7 @@
       <c r="H154">
         <v>-196</v>
       </c>
-      <c r="J154" s="1">
+      <c r="J154" s="2">
         <v>45988</v>
       </c>
       <c r="K154" t="b">
@@ -6526,7 +6552,7 @@
       <c r="H155">
         <v>-47</v>
       </c>
-      <c r="J155" s="1">
+      <c r="J155" s="2">
         <v>46176</v>
       </c>
       <c r="K155" t="b">
@@ -6558,7 +6584,7 @@
       <c r="H156">
         <v>-47</v>
       </c>
-      <c r="J156" s="1">
+      <c r="J156" s="2">
         <v>46176</v>
       </c>
       <c r="K156" t="b">
@@ -6590,7 +6616,7 @@
       <c r="H157">
         <v>-33</v>
       </c>
-      <c r="J157" s="1">
+      <c r="J157" s="2">
         <v>46199</v>
       </c>
       <c r="K157" t="b">
@@ -6622,7 +6648,7 @@
       <c r="H158">
         <v>-33</v>
       </c>
-      <c r="J158" s="1">
+      <c r="J158" s="2">
         <v>46199</v>
       </c>
       <c r="K158" t="b">
@@ -6654,7 +6680,7 @@
       <c r="H159">
         <v>-6</v>
       </c>
-      <c r="J159" s="1">
+      <c r="J159" s="2">
         <v>45967</v>
       </c>
       <c r="K159" t="b">
@@ -6686,7 +6712,7 @@
       <c r="H160">
         <v>43</v>
       </c>
-      <c r="J160" s="1">
+      <c r="J160" s="2">
         <v>46440</v>
       </c>
       <c r="K160" t="b">
@@ -6718,7 +6744,7 @@
       <c r="H161">
         <v>43</v>
       </c>
-      <c r="J161" s="1">
+      <c r="J161" s="2">
         <v>46440</v>
       </c>
       <c r="K161" t="b">
@@ -6750,7 +6776,7 @@
       <c r="H162">
         <v>73</v>
       </c>
-      <c r="J162" s="1">
+      <c r="J162" s="2">
         <v>46264</v>
       </c>
       <c r="K162" t="b">
@@ -6782,7 +6808,7 @@
       <c r="H163">
         <v>73</v>
       </c>
-      <c r="J163" s="1">
+      <c r="J163" s="2">
         <v>46264</v>
       </c>
       <c r="K163" t="b">
@@ -6814,7 +6840,7 @@
       <c r="H164">
         <v>102</v>
       </c>
-      <c r="J164" s="1">
+      <c r="J164" s="2">
         <v>46463</v>
       </c>
       <c r="K164" t="b">
@@ -6846,7 +6872,7 @@
       <c r="H165">
         <v>118</v>
       </c>
-      <c r="J165" s="1">
+      <c r="J165" s="2">
         <v>46337</v>
       </c>
       <c r="K165" t="b">
@@ -6878,7 +6904,7 @@
       <c r="H166">
         <v>146</v>
       </c>
-      <c r="J166" s="1">
+      <c r="J166" s="2">
         <v>46451</v>
       </c>
       <c r="K166" t="b">
@@ -6910,7 +6936,7 @@
       <c r="H167">
         <v>152</v>
       </c>
-      <c r="J167" s="1">
+      <c r="J167" s="2">
         <v>46245</v>
       </c>
       <c r="K167" t="b">
@@ -6942,7 +6968,7 @@
       <c r="H168">
         <v>152</v>
       </c>
-      <c r="J168" s="1">
+      <c r="J168" s="2">
         <v>46245</v>
       </c>
       <c r="K168" t="b">
@@ -6974,7 +7000,7 @@
       <c r="H169">
         <v>163</v>
       </c>
-      <c r="J169" s="1">
+      <c r="J169" s="2">
         <v>46324</v>
       </c>
       <c r="K169" t="b">
@@ -7006,7 +7032,7 @@
       <c r="H170">
         <v>163</v>
       </c>
-      <c r="J170" s="1">
+      <c r="J170" s="2">
         <v>46324</v>
       </c>
       <c r="K170" t="b">
@@ -7038,7 +7064,7 @@
       <c r="H171">
         <v>164</v>
       </c>
-      <c r="J171" s="1">
+      <c r="J171" s="2">
         <v>46426</v>
       </c>
       <c r="K171" t="b">
@@ -7070,7 +7096,7 @@
       <c r="H172">
         <v>175</v>
       </c>
-      <c r="J172" s="1">
+      <c r="J172" s="2">
         <v>46383</v>
       </c>
       <c r="K172" t="b">
@@ -7102,7 +7128,7 @@
       <c r="H173">
         <v>186</v>
       </c>
-      <c r="J173" s="1">
+      <c r="J173" s="2">
         <v>46392</v>
       </c>
       <c r="K173" t="b">
@@ -7134,7 +7160,7 @@
       <c r="H174">
         <v>205</v>
       </c>
-      <c r="J174" s="1">
+      <c r="J174" s="2">
         <v>46390</v>
       </c>
       <c r="K174" t="b">
@@ -7166,7 +7192,7 @@
       <c r="H175">
         <v>207</v>
       </c>
-      <c r="J175" s="1">
+      <c r="J175" s="2">
         <v>46392</v>
       </c>
       <c r="K175" t="b">
@@ -7198,7 +7224,7 @@
       <c r="H176">
         <v>218</v>
       </c>
-      <c r="J176" s="1">
+      <c r="J176" s="2">
         <v>46506</v>
       </c>
       <c r="K176" t="b">
@@ -7230,7 +7256,7 @@
       <c r="H177">
         <v>246</v>
       </c>
-      <c r="J177" s="1">
+      <c r="J177" s="2">
         <v>46478</v>
       </c>
       <c r="K177" t="b">
@@ -7262,7 +7288,7 @@
       <c r="H178">
         <v>248</v>
       </c>
-      <c r="J178" s="1">
+      <c r="J178" s="2">
         <v>46500</v>
       </c>
       <c r="K178" t="b">
@@ -7294,7 +7320,7 @@
       <c r="H179">
         <v>276</v>
       </c>
-      <c r="J179" s="1">
+      <c r="J179" s="2">
         <v>46430</v>
       </c>
       <c r="K179" t="b">
@@ -7326,7 +7352,7 @@
       <c r="H180">
         <v>276</v>
       </c>
-      <c r="J180" s="1">
+      <c r="J180" s="2">
         <v>46430</v>
       </c>
       <c r="K180" t="b">
@@ -7358,7 +7384,7 @@
       <c r="H181">
         <v>290</v>
       </c>
-      <c r="J181" s="1">
+      <c r="J181" s="2">
         <v>46467</v>
       </c>
       <c r="K181" t="b">
@@ -7390,7 +7416,7 @@
       <c r="H182">
         <v>317</v>
       </c>
-      <c r="J182" s="1">
+      <c r="J182" s="2">
         <v>46529</v>
       </c>
       <c r="K182" t="b">
@@ -7422,7 +7448,7 @@
       <c r="H183">
         <v>420</v>
       </c>
-      <c r="J183" s="1">
+      <c r="J183" s="2">
         <v>46566</v>
       </c>
       <c r="K183" t="b">
@@ -7454,7 +7480,7 @@
       <c r="H184">
         <v>426</v>
       </c>
-      <c r="J184" s="1">
+      <c r="J184" s="2">
         <v>46571</v>
       </c>
       <c r="K184" t="b">
@@ -7486,7 +7512,7 @@
       <c r="H185">
         <v>721</v>
       </c>
-      <c r="J185" s="1">
+      <c r="J185" s="2">
         <v>46325</v>
       </c>
       <c r="K185" t="b">
@@ -7518,7 +7544,7 @@
       <c r="H186">
         <v>721</v>
       </c>
-      <c r="J186" s="1">
+      <c r="J186" s="2">
         <v>46325</v>
       </c>
       <c r="K186" t="b">
@@ -7550,7 +7576,7 @@
       <c r="H187">
         <v>850</v>
       </c>
-      <c r="J187" s="1">
+      <c r="J187" s="2">
         <v>46345</v>
       </c>
       <c r="K187" t="b">
@@ -7582,7 +7608,7 @@
       <c r="H188">
         <v>850</v>
       </c>
-      <c r="J188" s="1">
+      <c r="J188" s="2">
         <v>46345</v>
       </c>
       <c r="K188" t="b">
@@ -7614,7 +7640,7 @@
       <c r="H189">
         <v>1661</v>
       </c>
-      <c r="J189" s="1">
+      <c r="J189" s="2">
         <v>46498</v>
       </c>
       <c r="K189" t="b">
@@ -7646,7 +7672,7 @@
       <c r="H190">
         <v>1661</v>
       </c>
-      <c r="J190" s="1">
+      <c r="J190" s="2">
         <v>46498</v>
       </c>
       <c r="K190" t="b">
@@ -7678,7 +7704,7 @@
       <c r="H191">
         <v>488</v>
       </c>
-      <c r="J191" s="1">
+      <c r="J191" s="2">
         <v>46190</v>
       </c>
       <c r="K191" t="b">
@@ -7710,7 +7736,7 @@
       <c r="H192">
         <v>25565</v>
       </c>
-      <c r="J192" s="1">
+      <c r="J192" s="2">
         <v>46190</v>
       </c>
       <c r="K192" t="b">
@@ -7742,7 +7768,7 @@
       <c r="H193">
         <v>25567</v>
       </c>
-      <c r="J193" s="1">
+      <c r="J193" s="2">
         <v>46190</v>
       </c>
       <c r="K193" t="b">
@@ -7774,7 +7800,7 @@
       <c r="H194">
         <v>31293</v>
       </c>
-      <c r="J194" s="1">
+      <c r="J194" s="2">
         <v>46190</v>
       </c>
       <c r="K194" t="b">

</xml_diff>

<commit_message>
Atualização automática: vencimentos_tmot (22/07/2026 16:09)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
@@ -1040,16 +1040,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1065,7 +1057,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1073,30 +1065,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1396,37 +1370,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1455,7 +1429,7 @@
       <c r="H2">
         <v>-4402.8</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>41388</v>
       </c>
       <c r="K2" t="b">
@@ -1487,7 +1461,7 @@
       <c r="H3">
         <v>-4254.8</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>39285</v>
       </c>
       <c r="K3" t="b">
@@ -1519,7 +1493,7 @@
       <c r="H4">
         <v>-2354.2</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>40669</v>
       </c>
       <c r="K4" t="b">
@@ -1551,7 +1525,7 @@
       <c r="H5">
         <v>-896.8</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>40669</v>
       </c>
       <c r="K5" t="b">
@@ -1583,7 +1557,7 @@
       <c r="H6">
         <v>-854.1</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>44884</v>
       </c>
       <c r="K6" t="b">
@@ -1615,7 +1589,7 @@
       <c r="H7">
         <v>-413.2</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>43855</v>
       </c>
       <c r="K7" t="b">
@@ -1647,7 +1621,7 @@
       <c r="H8">
         <v>-391.8</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>42769</v>
       </c>
       <c r="K8" t="b">
@@ -1679,7 +1653,7 @@
       <c r="H9">
         <v>-371.5</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>46014</v>
       </c>
       <c r="K9" t="b">
@@ -1711,7 +1685,7 @@
       <c r="H10">
         <v>-368.8</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>46014</v>
       </c>
       <c r="K10" t="b">
@@ -1743,7 +1717,7 @@
       <c r="H11">
         <v>-359</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>45804</v>
       </c>
       <c r="K11" t="b">
@@ -1775,7 +1749,7 @@
       <c r="H12">
         <v>-359</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>45804</v>
       </c>
       <c r="K12" t="b">
@@ -1807,7 +1781,7 @@
       <c r="H13">
         <v>-351</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>42821</v>
       </c>
       <c r="K13" t="b">
@@ -1839,7 +1813,7 @@
       <c r="H14">
         <v>-351</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>46014</v>
       </c>
       <c r="K14" t="b">
@@ -1871,7 +1845,7 @@
       <c r="H15">
         <v>-351</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <v>46014</v>
       </c>
       <c r="K15" t="b">
@@ -1903,7 +1877,7 @@
       <c r="H16">
         <v>-351</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <v>46014</v>
       </c>
       <c r="K16" t="b">
@@ -1935,7 +1909,7 @@
       <c r="H17">
         <v>-345.8</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="1">
         <v>46017</v>
       </c>
       <c r="K17" t="b">
@@ -1967,7 +1941,7 @@
       <c r="H18">
         <v>-345.8</v>
       </c>
-      <c r="J18" s="2">
+      <c r="J18" s="1">
         <v>46017</v>
       </c>
       <c r="K18" t="b">
@@ -1999,7 +1973,7 @@
       <c r="H19">
         <v>-264.2</v>
       </c>
-      <c r="J19" s="2">
+      <c r="J19" s="1">
         <v>40979</v>
       </c>
       <c r="K19" t="b">
@@ -2031,7 +2005,7 @@
       <c r="H20">
         <v>-206.4</v>
       </c>
-      <c r="J20" s="2">
+      <c r="J20" s="1">
         <v>36669</v>
       </c>
       <c r="K20" t="b">
@@ -2063,7 +2037,7 @@
       <c r="H21">
         <v>-131.6</v>
       </c>
-      <c r="J21" s="2">
+      <c r="J21" s="1">
         <v>46111</v>
       </c>
       <c r="K21" t="b">
@@ -2095,7 +2069,7 @@
       <c r="H22">
         <v>-131.6</v>
       </c>
-      <c r="J22" s="2">
+      <c r="J22" s="1">
         <v>46111</v>
       </c>
       <c r="K22" t="b">
@@ -2127,7 +2101,7 @@
       <c r="H23">
         <v>-131.6</v>
       </c>
-      <c r="J23" s="2">
+      <c r="J23" s="1">
         <v>46111</v>
       </c>
       <c r="K23" t="b">
@@ -2159,7 +2133,7 @@
       <c r="H24">
         <v>-131.6</v>
       </c>
-      <c r="J24" s="2">
+      <c r="J24" s="1">
         <v>46111</v>
       </c>
       <c r="K24" t="b">
@@ -2191,7 +2165,7 @@
       <c r="H25">
         <v>-131.6</v>
       </c>
-      <c r="J25" s="2">
+      <c r="J25" s="1">
         <v>46111</v>
       </c>
       <c r="K25" t="b">
@@ -2223,7 +2197,7 @@
       <c r="H26">
         <v>-105</v>
       </c>
-      <c r="J26" s="2">
+      <c r="J26" s="1">
         <v>46161</v>
       </c>
       <c r="K26" t="b">
@@ -2255,7 +2229,7 @@
       <c r="H27">
         <v>-79.8</v>
       </c>
-      <c r="J27" s="2">
+      <c r="J27" s="1">
         <v>43340</v>
       </c>
       <c r="K27" t="b">
@@ -2287,7 +2261,7 @@
       <c r="H28">
         <v>-12.3</v>
       </c>
-      <c r="J28" s="2">
+      <c r="J28" s="1">
         <v>46048</v>
       </c>
       <c r="K28" t="b">
@@ -2319,7 +2293,7 @@
       <c r="H29">
         <v>0</v>
       </c>
-      <c r="J29" s="2">
+      <c r="J29" s="1">
         <v>46211</v>
       </c>
       <c r="K29" t="b">
@@ -2351,7 +2325,7 @@
       <c r="H30">
         <v>3.6</v>
       </c>
-      <c r="J30" s="2">
+      <c r="J30" s="1">
         <v>46234</v>
       </c>
       <c r="K30" t="b">
@@ -2383,7 +2357,7 @@
       <c r="H31">
         <v>6.2</v>
       </c>
-      <c r="J31" s="2">
+      <c r="J31" s="1">
         <v>46234</v>
       </c>
       <c r="K31" t="b">
@@ -2415,7 +2389,7 @@
       <c r="H32">
         <v>7.5</v>
       </c>
-      <c r="J32" s="2">
+      <c r="J32" s="1">
         <v>46234</v>
       </c>
       <c r="K32" t="b">
@@ -2447,7 +2421,7 @@
       <c r="H33">
         <v>10.7</v>
       </c>
-      <c r="J33" s="2">
+      <c r="J33" s="1">
         <v>46234</v>
       </c>
       <c r="K33" t="b">
@@ -2479,7 +2453,7 @@
       <c r="H34">
         <v>20</v>
       </c>
-      <c r="J34" s="2">
+      <c r="J34" s="1">
         <v>46234</v>
       </c>
       <c r="K34" t="b">
@@ -2511,7 +2485,7 @@
       <c r="H35">
         <v>30.8</v>
       </c>
-      <c r="J35" s="2">
+      <c r="J35" s="1">
         <v>46234</v>
       </c>
       <c r="K35" t="b">
@@ -2543,7 +2517,7 @@
       <c r="H36">
         <v>37.1</v>
       </c>
-      <c r="J36" s="2">
+      <c r="J36" s="1">
         <v>46256</v>
       </c>
       <c r="K36" t="b">
@@ -2575,7 +2549,7 @@
       <c r="H37">
         <v>42.8</v>
       </c>
-      <c r="J37" s="2">
+      <c r="J37" s="1">
         <v>46276</v>
       </c>
       <c r="K37" t="b">
@@ -2607,7 +2581,7 @@
       <c r="H38">
         <v>45.2</v>
       </c>
-      <c r="J38" s="2">
+      <c r="J38" s="1">
         <v>46234</v>
       </c>
       <c r="K38" t="b">
@@ -2639,7 +2613,7 @@
       <c r="H39">
         <v>46</v>
       </c>
-      <c r="J39" s="2">
+      <c r="J39" s="1">
         <v>46251</v>
       </c>
       <c r="K39" t="b">
@@ -2671,7 +2645,7 @@
       <c r="H40">
         <v>47.5</v>
       </c>
-      <c r="J40" s="2">
+      <c r="J40" s="1">
         <v>46456</v>
       </c>
       <c r="K40" t="b">
@@ -2703,7 +2677,7 @@
       <c r="H41">
         <v>57.2</v>
       </c>
-      <c r="J41" s="2">
+      <c r="J41" s="1">
         <v>46246</v>
       </c>
       <c r="K41" t="b">
@@ -2735,7 +2709,7 @@
       <c r="H42">
         <v>59.6</v>
       </c>
-      <c r="J42" s="2">
+      <c r="J42" s="1">
         <v>46487</v>
       </c>
       <c r="K42" t="b">
@@ -2767,7 +2741,7 @@
       <c r="H43">
         <v>75.40000000000001</v>
       </c>
-      <c r="J43" s="2">
+      <c r="J43" s="1">
         <v>46283</v>
       </c>
       <c r="K43" t="b">
@@ -2799,7 +2773,7 @@
       <c r="H44">
         <v>76.8</v>
       </c>
-      <c r="J44" s="2">
+      <c r="J44" s="1">
         <v>46285</v>
       </c>
       <c r="K44" t="b">
@@ -2831,7 +2805,7 @@
       <c r="H45">
         <v>83.2</v>
       </c>
-      <c r="J45" s="2">
+      <c r="J45" s="1">
         <v>46547</v>
       </c>
       <c r="K45" t="b">
@@ -2863,7 +2837,7 @@
       <c r="H46">
         <v>84.5</v>
       </c>
-      <c r="J46" s="2">
+      <c r="J46" s="1">
         <v>46240</v>
       </c>
       <c r="K46" t="b">
@@ -2895,7 +2869,7 @@
       <c r="H47">
         <v>85.8</v>
       </c>
-      <c r="J47" s="2">
+      <c r="J47" s="1">
         <v>46266</v>
       </c>
       <c r="K47" t="b">
@@ -2927,7 +2901,7 @@
       <c r="H48">
         <v>86.5</v>
       </c>
-      <c r="J48" s="2">
+      <c r="J48" s="1">
         <v>46241</v>
       </c>
       <c r="K48" t="b">
@@ -2959,7 +2933,7 @@
       <c r="H49">
         <v>91.7</v>
       </c>
-      <c r="J49" s="2">
+      <c r="J49" s="1">
         <v>46243</v>
       </c>
       <c r="K49" t="b">
@@ -2991,7 +2965,7 @@
       <c r="H50">
         <v>91.7</v>
       </c>
-      <c r="J50" s="2">
+      <c r="J50" s="1">
         <v>46243</v>
       </c>
       <c r="K50" t="b">
@@ -3023,7 +2997,7 @@
       <c r="H51">
         <v>91.7</v>
       </c>
-      <c r="J51" s="2">
+      <c r="J51" s="1">
         <v>46250</v>
       </c>
       <c r="K51" t="b">
@@ -3055,7 +3029,7 @@
       <c r="H52">
         <v>98.90000000000001</v>
       </c>
-      <c r="J52" s="2">
+      <c r="J52" s="1">
         <v>46253</v>
       </c>
       <c r="K52" t="b">
@@ -3087,7 +3061,7 @@
       <c r="H53">
         <v>105.5</v>
       </c>
-      <c r="J53" s="2">
+      <c r="J53" s="1">
         <v>46280</v>
       </c>
       <c r="K53" t="b">
@@ -3119,7 +3093,7 @@
       <c r="H54">
         <v>105.6</v>
       </c>
-      <c r="J54" s="2">
+      <c r="J54" s="1">
         <v>46361</v>
       </c>
       <c r="K54" t="b">
@@ -3151,7 +3125,7 @@
       <c r="H55">
         <v>105.7</v>
       </c>
-      <c r="J55" s="2">
+      <c r="J55" s="1">
         <v>46362</v>
       </c>
       <c r="K55" t="b">
@@ -3183,7 +3157,7 @@
       <c r="H56">
         <v>110.7</v>
       </c>
-      <c r="J56" s="2">
+      <c r="J56" s="1">
         <v>46275</v>
       </c>
       <c r="K56" t="b">
@@ -3215,7 +3189,7 @@
       <c r="H57">
         <v>113.2</v>
       </c>
-      <c r="J57" s="2">
+      <c r="J57" s="1">
         <v>46377</v>
       </c>
       <c r="K57" t="b">
@@ -3247,7 +3221,7 @@
       <c r="H58">
         <v>128.8</v>
       </c>
-      <c r="J58" s="2">
+      <c r="J58" s="1">
         <v>46434</v>
       </c>
       <c r="K58" t="b">
@@ -3279,7 +3253,7 @@
       <c r="H59">
         <v>128.8</v>
       </c>
-      <c r="J59" s="2">
+      <c r="J59" s="1">
         <v>46434</v>
       </c>
       <c r="K59" t="b">
@@ -3311,7 +3285,7 @@
       <c r="H60">
         <v>128.8</v>
       </c>
-      <c r="J60" s="2">
+      <c r="J60" s="1">
         <v>46434</v>
       </c>
       <c r="K60" t="b">
@@ -3343,7 +3317,7 @@
       <c r="H61">
         <v>128.8</v>
       </c>
-      <c r="J61" s="2">
+      <c r="J61" s="1">
         <v>46434</v>
       </c>
       <c r="K61" t="b">
@@ -3375,7 +3349,7 @@
       <c r="H62">
         <v>128.8</v>
       </c>
-      <c r="J62" s="2">
+      <c r="J62" s="1">
         <v>46434</v>
       </c>
       <c r="K62" t="b">
@@ -3407,7 +3381,7 @@
       <c r="H63">
         <v>135</v>
       </c>
-      <c r="J63" s="2">
+      <c r="J63" s="1">
         <v>46280</v>
       </c>
       <c r="K63" t="b">
@@ -3439,7 +3413,7 @@
       <c r="H64">
         <v>150.6</v>
       </c>
-      <c r="J64" s="2">
+      <c r="J64" s="1">
         <v>46271</v>
       </c>
       <c r="K64" t="b">
@@ -3471,7 +3445,7 @@
       <c r="H65">
         <v>174.2</v>
       </c>
-      <c r="J65" s="2">
+      <c r="J65" s="1">
         <v>46363</v>
       </c>
       <c r="K65" t="b">
@@ -3503,7 +3477,7 @@
       <c r="H66">
         <v>176.6</v>
       </c>
-      <c r="J66" s="2">
+      <c r="J66" s="1">
         <v>46334</v>
       </c>
       <c r="K66" t="b">
@@ -3535,7 +3509,7 @@
       <c r="H67">
         <v>177.4</v>
       </c>
-      <c r="J67" s="2">
+      <c r="J67" s="1">
         <v>46407</v>
       </c>
       <c r="K67" t="b">
@@ -3567,7 +3541,7 @@
       <c r="H68">
         <v>183.9</v>
       </c>
-      <c r="J68" s="2">
+      <c r="J68" s="1">
         <v>46341</v>
       </c>
       <c r="K68" t="b">
@@ -3599,7 +3573,7 @@
       <c r="H69">
         <v>191.7</v>
       </c>
-      <c r="J69" s="2">
+      <c r="J69" s="1">
         <v>46300</v>
       </c>
       <c r="K69" t="b">
@@ -3631,7 +3605,7 @@
       <c r="H70">
         <v>200</v>
       </c>
-      <c r="J70" s="2">
+      <c r="J70" s="1">
         <v>46336</v>
       </c>
       <c r="K70" t="b">
@@ -3663,7 +3637,7 @@
       <c r="H71">
         <v>201.1</v>
       </c>
-      <c r="J71" s="2">
+      <c r="J71" s="1">
         <v>46319</v>
       </c>
       <c r="K71" t="b">
@@ -3695,7 +3669,7 @@
       <c r="H72">
         <v>206.5</v>
       </c>
-      <c r="J72" s="2">
+      <c r="J72" s="1">
         <v>46308</v>
       </c>
       <c r="K72" t="b">
@@ -3727,7 +3701,7 @@
       <c r="H73">
         <v>207.5</v>
       </c>
-      <c r="J73" s="2">
+      <c r="J73" s="1">
         <v>46390</v>
       </c>
       <c r="K73" t="b">
@@ -3759,7 +3733,7 @@
       <c r="H74">
         <v>247</v>
       </c>
-      <c r="J74" s="2">
+      <c r="J74" s="1">
         <v>46443</v>
       </c>
       <c r="K74" t="b">
@@ -3791,7 +3765,7 @@
       <c r="H75">
         <v>285.3</v>
       </c>
-      <c r="J75" s="2">
+      <c r="J75" s="1">
         <v>46304</v>
       </c>
       <c r="K75" t="b">
@@ -3823,7 +3797,7 @@
       <c r="H76">
         <v>290.8</v>
       </c>
-      <c r="J76" s="2">
+      <c r="J76" s="1">
         <v>46362</v>
       </c>
       <c r="K76" t="b">
@@ -3855,7 +3829,7 @@
       <c r="H77">
         <v>295.2</v>
       </c>
-      <c r="J77" s="2">
+      <c r="J77" s="1">
         <v>46463</v>
       </c>
       <c r="K77" t="b">
@@ -3887,7 +3861,7 @@
       <c r="H78">
         <v>300.2</v>
       </c>
-      <c r="J78" s="2">
+      <c r="J78" s="1">
         <v>46466</v>
       </c>
       <c r="K78" t="b">
@@ -3922,7 +3896,7 @@
       <c r="I79" t="s">
         <v>313</v>
       </c>
-      <c r="J79" s="2">
+      <c r="J79" s="1">
         <v>36557</v>
       </c>
       <c r="K79" t="b">
@@ -3957,7 +3931,7 @@
       <c r="I80" t="s">
         <v>314</v>
       </c>
-      <c r="J80" s="2">
+      <c r="J80" s="1">
         <v>41275</v>
       </c>
       <c r="K80" t="b">
@@ -3992,7 +3966,7 @@
       <c r="I81" t="s">
         <v>315</v>
       </c>
-      <c r="J81" s="2">
+      <c r="J81" s="1">
         <v>45380</v>
       </c>
       <c r="K81" t="b">
@@ -4027,7 +4001,7 @@
       <c r="I82" t="s">
         <v>316</v>
       </c>
-      <c r="J82" s="2">
+      <c r="J82" s="1">
         <v>45421</v>
       </c>
       <c r="K82" t="b">
@@ -4062,7 +4036,7 @@
       <c r="I83" t="s">
         <v>316</v>
       </c>
-      <c r="J83" s="2">
+      <c r="J83" s="1">
         <v>45428</v>
       </c>
       <c r="K83" t="b">
@@ -4097,7 +4071,7 @@
       <c r="I84" t="s">
         <v>317</v>
       </c>
-      <c r="J84" s="2">
+      <c r="J84" s="1">
         <v>45490</v>
       </c>
       <c r="K84" t="b">
@@ -4132,7 +4106,7 @@
       <c r="I85" t="s">
         <v>318</v>
       </c>
-      <c r="J85" s="2">
+      <c r="J85" s="1">
         <v>45566</v>
       </c>
       <c r="K85" t="b">
@@ -4167,7 +4141,7 @@
       <c r="I86" t="s">
         <v>319</v>
       </c>
-      <c r="J86" s="2">
+      <c r="J86" s="1">
         <v>45986</v>
       </c>
       <c r="K86" t="b">
@@ -4202,7 +4176,7 @@
       <c r="I87" t="s">
         <v>320</v>
       </c>
-      <c r="J87" s="2">
+      <c r="J87" s="1">
         <v>46106</v>
       </c>
       <c r="K87" t="b">
@@ -4237,7 +4211,7 @@
       <c r="I88" t="s">
         <v>321</v>
       </c>
-      <c r="J88" s="2">
+      <c r="J88" s="1">
         <v>46142</v>
       </c>
       <c r="K88" t="b">
@@ -4272,7 +4246,7 @@
       <c r="I89" t="s">
         <v>322</v>
       </c>
-      <c r="J89" s="2">
+      <c r="J89" s="1">
         <v>46274</v>
       </c>
       <c r="K89" t="b">
@@ -4307,7 +4281,7 @@
       <c r="I90" t="s">
         <v>322</v>
       </c>
-      <c r="J90" s="2">
+      <c r="J90" s="1">
         <v>46276</v>
       </c>
       <c r="K90" t="b">
@@ -4342,7 +4316,7 @@
       <c r="I91" t="s">
         <v>322</v>
       </c>
-      <c r="J91" s="2">
+      <c r="J91" s="1">
         <v>46284</v>
       </c>
       <c r="K91" t="b">
@@ -4377,7 +4351,7 @@
       <c r="I92" t="s">
         <v>323</v>
       </c>
-      <c r="J92" s="2">
+      <c r="J92" s="1">
         <v>46317</v>
       </c>
       <c r="K92" t="b">
@@ -4412,7 +4386,7 @@
       <c r="I93" t="s">
         <v>323</v>
       </c>
-      <c r="J93" s="2">
+      <c r="J93" s="1">
         <v>46319</v>
       </c>
       <c r="K93" t="b">
@@ -4447,7 +4421,7 @@
       <c r="I94" t="s">
         <v>324</v>
       </c>
-      <c r="J94" s="2">
+      <c r="J94" s="1">
         <v>46333</v>
       </c>
       <c r="K94" t="b">
@@ -4482,7 +4456,7 @@
       <c r="I95" t="s">
         <v>324</v>
       </c>
-      <c r="J95" s="2">
+      <c r="J95" s="1">
         <v>46338</v>
       </c>
       <c r="K95" t="b">
@@ -4517,7 +4491,7 @@
       <c r="I96" t="s">
         <v>324</v>
       </c>
-      <c r="J96" s="2">
+      <c r="J96" s="1">
         <v>46338</v>
       </c>
       <c r="K96" t="b">
@@ -4552,7 +4526,7 @@
       <c r="I97" t="s">
         <v>324</v>
       </c>
-      <c r="J97" s="2">
+      <c r="J97" s="1">
         <v>46341</v>
       </c>
       <c r="K97" t="b">
@@ -4587,7 +4561,7 @@
       <c r="I98" t="s">
         <v>324</v>
       </c>
-      <c r="J98" s="2">
+      <c r="J98" s="1">
         <v>46344</v>
       </c>
       <c r="K98" t="b">
@@ -4622,7 +4596,7 @@
       <c r="I99" t="s">
         <v>324</v>
       </c>
-      <c r="J99" s="2">
+      <c r="J99" s="1">
         <v>46354</v>
       </c>
       <c r="K99" t="b">
@@ -4657,7 +4631,7 @@
       <c r="I100" t="s">
         <v>324</v>
       </c>
-      <c r="J100" s="2">
+      <c r="J100" s="1">
         <v>46360</v>
       </c>
       <c r="K100" t="b">
@@ -4692,7 +4666,7 @@
       <c r="I101" t="s">
         <v>324</v>
       </c>
-      <c r="J101" s="2">
+      <c r="J101" s="1">
         <v>46360</v>
       </c>
       <c r="K101" t="b">
@@ -4727,7 +4701,7 @@
       <c r="I102" t="s">
         <v>325</v>
       </c>
-      <c r="J102" s="2">
+      <c r="J102" s="1">
         <v>46366</v>
       </c>
       <c r="K102" t="b">
@@ -4762,7 +4736,7 @@
       <c r="I103" t="s">
         <v>325</v>
       </c>
-      <c r="J103" s="2">
+      <c r="J103" s="1">
         <v>46375</v>
       </c>
       <c r="K103" t="b">
@@ -4797,7 +4771,7 @@
       <c r="I104" t="s">
         <v>325</v>
       </c>
-      <c r="J104" s="2">
+      <c r="J104" s="1">
         <v>46388</v>
       </c>
       <c r="K104" t="b">
@@ -4832,7 +4806,7 @@
       <c r="I105" t="s">
         <v>326</v>
       </c>
-      <c r="J105" s="2">
+      <c r="J105" s="1">
         <v>46401</v>
       </c>
       <c r="K105" t="b">
@@ -4867,7 +4841,7 @@
       <c r="I106" t="s">
         <v>326</v>
       </c>
-      <c r="J106" s="2">
+      <c r="J106" s="1">
         <v>46401</v>
       </c>
       <c r="K106" t="b">
@@ -4902,7 +4876,7 @@
       <c r="I107" t="s">
         <v>326</v>
       </c>
-      <c r="J107" s="2">
+      <c r="J107" s="1">
         <v>46401</v>
       </c>
       <c r="K107" t="b">
@@ -4937,7 +4911,7 @@
       <c r="I108" t="s">
         <v>326</v>
       </c>
-      <c r="J108" s="2">
+      <c r="J108" s="1">
         <v>46413</v>
       </c>
       <c r="K108" t="b">
@@ -4972,7 +4946,7 @@
       <c r="I109" t="s">
         <v>327</v>
       </c>
-      <c r="J109" s="2">
+      <c r="J109" s="1">
         <v>46424</v>
       </c>
       <c r="K109" t="b">
@@ -5007,7 +4981,7 @@
       <c r="I110" t="s">
         <v>327</v>
       </c>
-      <c r="J110" s="2">
+      <c r="J110" s="1">
         <v>46427</v>
       </c>
       <c r="K110" t="b">
@@ -5042,7 +5016,7 @@
       <c r="I111" t="s">
         <v>327</v>
       </c>
-      <c r="J111" s="2">
+      <c r="J111" s="1">
         <v>46437</v>
       </c>
       <c r="K111" t="b">
@@ -5077,7 +5051,7 @@
       <c r="I112" t="s">
         <v>327</v>
       </c>
-      <c r="J112" s="2">
+      <c r="J112" s="1">
         <v>46451</v>
       </c>
       <c r="K112" t="b">
@@ -5112,7 +5086,7 @@
       <c r="I113" t="s">
         <v>328</v>
       </c>
-      <c r="J113" s="2">
+      <c r="J113" s="1">
         <v>46455</v>
       </c>
       <c r="K113" t="b">
@@ -5147,7 +5121,7 @@
       <c r="I114" t="s">
         <v>328</v>
       </c>
-      <c r="J114" s="2">
+      <c r="J114" s="1">
         <v>46457</v>
       </c>
       <c r="K114" t="b">
@@ -5182,7 +5156,7 @@
       <c r="I115" t="s">
         <v>328</v>
       </c>
-      <c r="J115" s="2">
+      <c r="J115" s="1">
         <v>46462</v>
       </c>
       <c r="K115" t="b">
@@ -5217,7 +5191,7 @@
       <c r="I116" t="s">
         <v>328</v>
       </c>
-      <c r="J116" s="2">
+      <c r="J116" s="1">
         <v>46464</v>
       </c>
       <c r="K116" t="b">
@@ -5252,7 +5226,7 @@
       <c r="I117" t="s">
         <v>328</v>
       </c>
-      <c r="J117" s="2">
+      <c r="J117" s="1">
         <v>46470</v>
       </c>
       <c r="K117" t="b">
@@ -5287,7 +5261,7 @@
       <c r="I118" t="s">
         <v>329</v>
       </c>
-      <c r="J118" s="2">
+      <c r="J118" s="1">
         <v>46485</v>
       </c>
       <c r="K118" t="b">
@@ -5322,7 +5296,7 @@
       <c r="I119" t="s">
         <v>329</v>
       </c>
-      <c r="J119" s="2">
+      <c r="J119" s="1">
         <v>46499</v>
       </c>
       <c r="K119" t="b">
@@ -5357,7 +5331,7 @@
       <c r="I120" t="s">
         <v>329</v>
       </c>
-      <c r="J120" s="2">
+      <c r="J120" s="1">
         <v>46504</v>
       </c>
       <c r="K120" t="b">
@@ -5392,7 +5366,7 @@
       <c r="I121" t="s">
         <v>329</v>
       </c>
-      <c r="J121" s="2">
+      <c r="J121" s="1">
         <v>46504</v>
       </c>
       <c r="K121" t="b">
@@ -5427,7 +5401,7 @@
       <c r="I122" t="s">
         <v>329</v>
       </c>
-      <c r="J122" s="2">
+      <c r="J122" s="1">
         <v>46507</v>
       </c>
       <c r="K122" t="b">
@@ -5462,7 +5436,7 @@
       <c r="I123" t="s">
         <v>329</v>
       </c>
-      <c r="J123" s="2">
+      <c r="J123" s="1">
         <v>46508</v>
       </c>
       <c r="K123" t="b">
@@ -5497,7 +5471,7 @@
       <c r="I124" t="s">
         <v>329</v>
       </c>
-      <c r="J124" s="2">
+      <c r="J124" s="1">
         <v>46512</v>
       </c>
       <c r="K124" t="b">
@@ -5532,7 +5506,7 @@
       <c r="I125" t="s">
         <v>329</v>
       </c>
-      <c r="J125" s="2">
+      <c r="J125" s="1">
         <v>46512</v>
       </c>
       <c r="K125" t="b">
@@ -5567,7 +5541,7 @@
       <c r="I126" t="s">
         <v>330</v>
       </c>
-      <c r="J126" s="2">
+      <c r="J126" s="1">
         <v>46528</v>
       </c>
       <c r="K126" t="b">
@@ -5602,7 +5576,7 @@
       <c r="I127" t="s">
         <v>330</v>
       </c>
-      <c r="J127" s="2">
+      <c r="J127" s="1">
         <v>46529</v>
       </c>
       <c r="K127" t="b">
@@ -5637,7 +5611,7 @@
       <c r="I128" t="s">
         <v>330</v>
       </c>
-      <c r="J128" s="2">
+      <c r="J128" s="1">
         <v>46537</v>
       </c>
       <c r="K128" t="b">
@@ -5672,7 +5646,7 @@
       <c r="I129" t="s">
         <v>331</v>
       </c>
-      <c r="J129" s="2">
+      <c r="J129" s="1">
         <v>46546</v>
       </c>
       <c r="K129" t="b">
@@ -5707,7 +5681,7 @@
       <c r="I130" t="s">
         <v>331</v>
       </c>
-      <c r="J130" s="2">
+      <c r="J130" s="1">
         <v>46547</v>
       </c>
       <c r="K130" t="b">
@@ -5742,7 +5716,7 @@
       <c r="I131" t="s">
         <v>331</v>
       </c>
-      <c r="J131" s="2">
+      <c r="J131" s="1">
         <v>46547</v>
       </c>
       <c r="K131" t="b">
@@ -5777,7 +5751,7 @@
       <c r="I132" t="s">
         <v>331</v>
       </c>
-      <c r="J132" s="2">
+      <c r="J132" s="1">
         <v>46547</v>
       </c>
       <c r="K132" t="b">
@@ -5812,7 +5786,7 @@
       <c r="I133" t="s">
         <v>331</v>
       </c>
-      <c r="J133" s="2">
+      <c r="J133" s="1">
         <v>46551</v>
       </c>
       <c r="K133" t="b">
@@ -5847,7 +5821,7 @@
       <c r="I134" t="s">
         <v>331</v>
       </c>
-      <c r="J134" s="2">
+      <c r="J134" s="1">
         <v>46560</v>
       </c>
       <c r="K134" t="b">
@@ -5882,7 +5856,7 @@
       <c r="I135" t="s">
         <v>331</v>
       </c>
-      <c r="J135" s="2">
+      <c r="J135" s="1">
         <v>46564</v>
       </c>
       <c r="K135" t="b">
@@ -5917,7 +5891,7 @@
       <c r="I136" t="s">
         <v>331</v>
       </c>
-      <c r="J136" s="2">
+      <c r="J136" s="1">
         <v>46567</v>
       </c>
       <c r="K136" t="b">
@@ -5952,7 +5926,7 @@
       <c r="I137" t="s">
         <v>331</v>
       </c>
-      <c r="J137" s="2">
+      <c r="J137" s="1">
         <v>46568</v>
       </c>
       <c r="K137" t="b">
@@ -5987,7 +5961,7 @@
       <c r="I138" t="s">
         <v>331</v>
       </c>
-      <c r="J138" s="2">
+      <c r="J138" s="1">
         <v>46571</v>
       </c>
       <c r="K138" t="b">
@@ -6022,7 +5996,7 @@
       <c r="I139" t="s">
         <v>332</v>
       </c>
-      <c r="J139" s="2">
+      <c r="J139" s="1">
         <v>46197</v>
       </c>
       <c r="K139" t="b">
@@ -6057,7 +6031,7 @@
       <c r="I140" t="s">
         <v>333</v>
       </c>
-      <c r="J140" s="2">
+      <c r="J140" s="1">
         <v>46212</v>
       </c>
       <c r="K140" t="b">
@@ -6092,7 +6066,7 @@
       <c r="I141" t="s">
         <v>334</v>
       </c>
-      <c r="J141" s="2">
+      <c r="J141" s="1">
         <v>46225</v>
       </c>
       <c r="K141" t="b">
@@ -6127,7 +6101,7 @@
       <c r="I142" t="s">
         <v>335</v>
       </c>
-      <c r="J142" s="2">
+      <c r="J142" s="1">
         <v>46234</v>
       </c>
       <c r="K142" t="b">
@@ -6162,7 +6136,7 @@
       <c r="I143" t="s">
         <v>336</v>
       </c>
-      <c r="J143" s="2">
+      <c r="J143" s="1">
         <v>46234</v>
       </c>
       <c r="K143" t="b">
@@ -6197,7 +6171,7 @@
       <c r="I144" t="s">
         <v>337</v>
       </c>
-      <c r="J144" s="2">
+      <c r="J144" s="1">
         <v>46263</v>
       </c>
       <c r="K144" t="b">
@@ -6232,7 +6206,7 @@
       <c r="I145" t="s">
         <v>338</v>
       </c>
-      <c r="J145" s="2">
+      <c r="J145" s="1">
         <v>46266</v>
       </c>
       <c r="K145" t="b">
@@ -6264,7 +6238,7 @@
       <c r="H146">
         <v>-1476</v>
       </c>
-      <c r="J146" s="2">
+      <c r="J146" s="1">
         <v>43773</v>
       </c>
       <c r="K146" t="b">
@@ -6296,7 +6270,7 @@
       <c r="H147">
         <v>-1469</v>
       </c>
-      <c r="J147" s="2">
+      <c r="J147" s="1">
         <v>43773</v>
       </c>
       <c r="K147" t="b">
@@ -6328,7 +6302,7 @@
       <c r="H148">
         <v>-1121</v>
       </c>
-      <c r="J148" s="2">
+      <c r="J148" s="1">
         <v>45295</v>
       </c>
       <c r="K148" t="b">
@@ -6360,7 +6334,7 @@
       <c r="H149">
         <v>-1018</v>
       </c>
-      <c r="J149" s="2">
+      <c r="J149" s="1">
         <v>45617</v>
       </c>
       <c r="K149" t="b">
@@ -6392,7 +6366,7 @@
       <c r="H150">
         <v>-950</v>
       </c>
-      <c r="J150" s="2">
+      <c r="J150" s="1">
         <v>45677</v>
       </c>
       <c r="K150" t="b">
@@ -6424,7 +6398,7 @@
       <c r="H151">
         <v>-943</v>
       </c>
-      <c r="J151" s="2">
+      <c r="J151" s="1">
         <v>44944</v>
       </c>
       <c r="K151" t="b">
@@ -6456,7 +6430,7 @@
       <c r="H152">
         <v>-252</v>
       </c>
-      <c r="J152" s="2">
+      <c r="J152" s="1">
         <v>46092</v>
       </c>
       <c r="K152" t="b">
@@ -6488,7 +6462,7 @@
       <c r="H153">
         <v>-196</v>
       </c>
-      <c r="J153" s="2">
+      <c r="J153" s="1">
         <v>45988</v>
       </c>
       <c r="K153" t="b">
@@ -6520,7 +6494,7 @@
       <c r="H154">
         <v>-196</v>
       </c>
-      <c r="J154" s="2">
+      <c r="J154" s="1">
         <v>45988</v>
       </c>
       <c r="K154" t="b">
@@ -6552,7 +6526,7 @@
       <c r="H155">
         <v>-47</v>
       </c>
-      <c r="J155" s="2">
+      <c r="J155" s="1">
         <v>46176</v>
       </c>
       <c r="K155" t="b">
@@ -6584,7 +6558,7 @@
       <c r="H156">
         <v>-47</v>
       </c>
-      <c r="J156" s="2">
+      <c r="J156" s="1">
         <v>46176</v>
       </c>
       <c r="K156" t="b">
@@ -6616,7 +6590,7 @@
       <c r="H157">
         <v>-33</v>
       </c>
-      <c r="J157" s="2">
+      <c r="J157" s="1">
         <v>46199</v>
       </c>
       <c r="K157" t="b">
@@ -6648,7 +6622,7 @@
       <c r="H158">
         <v>-33</v>
       </c>
-      <c r="J158" s="2">
+      <c r="J158" s="1">
         <v>46199</v>
       </c>
       <c r="K158" t="b">
@@ -6680,7 +6654,7 @@
       <c r="H159">
         <v>-6</v>
       </c>
-      <c r="J159" s="2">
+      <c r="J159" s="1">
         <v>45967</v>
       </c>
       <c r="K159" t="b">
@@ -6712,7 +6686,7 @@
       <c r="H160">
         <v>43</v>
       </c>
-      <c r="J160" s="2">
+      <c r="J160" s="1">
         <v>46440</v>
       </c>
       <c r="K160" t="b">
@@ -6744,7 +6718,7 @@
       <c r="H161">
         <v>43</v>
       </c>
-      <c r="J161" s="2">
+      <c r="J161" s="1">
         <v>46440</v>
       </c>
       <c r="K161" t="b">
@@ -6776,7 +6750,7 @@
       <c r="H162">
         <v>73</v>
       </c>
-      <c r="J162" s="2">
+      <c r="J162" s="1">
         <v>46264</v>
       </c>
       <c r="K162" t="b">
@@ -6808,7 +6782,7 @@
       <c r="H163">
         <v>73</v>
       </c>
-      <c r="J163" s="2">
+      <c r="J163" s="1">
         <v>46264</v>
       </c>
       <c r="K163" t="b">
@@ -6840,7 +6814,7 @@
       <c r="H164">
         <v>102</v>
       </c>
-      <c r="J164" s="2">
+      <c r="J164" s="1">
         <v>46463</v>
       </c>
       <c r="K164" t="b">
@@ -6872,7 +6846,7 @@
       <c r="H165">
         <v>118</v>
       </c>
-      <c r="J165" s="2">
+      <c r="J165" s="1">
         <v>46337</v>
       </c>
       <c r="K165" t="b">
@@ -6904,7 +6878,7 @@
       <c r="H166">
         <v>146</v>
       </c>
-      <c r="J166" s="2">
+      <c r="J166" s="1">
         <v>46451</v>
       </c>
       <c r="K166" t="b">
@@ -6936,7 +6910,7 @@
       <c r="H167">
         <v>152</v>
       </c>
-      <c r="J167" s="2">
+      <c r="J167" s="1">
         <v>46245</v>
       </c>
       <c r="K167" t="b">
@@ -6968,7 +6942,7 @@
       <c r="H168">
         <v>152</v>
       </c>
-      <c r="J168" s="2">
+      <c r="J168" s="1">
         <v>46245</v>
       </c>
       <c r="K168" t="b">
@@ -7000,7 +6974,7 @@
       <c r="H169">
         <v>163</v>
       </c>
-      <c r="J169" s="2">
+      <c r="J169" s="1">
         <v>46324</v>
       </c>
       <c r="K169" t="b">
@@ -7032,7 +7006,7 @@
       <c r="H170">
         <v>163</v>
       </c>
-      <c r="J170" s="2">
+      <c r="J170" s="1">
         <v>46324</v>
       </c>
       <c r="K170" t="b">
@@ -7064,7 +7038,7 @@
       <c r="H171">
         <v>164</v>
       </c>
-      <c r="J171" s="2">
+      <c r="J171" s="1">
         <v>46426</v>
       </c>
       <c r="K171" t="b">
@@ -7096,7 +7070,7 @@
       <c r="H172">
         <v>175</v>
       </c>
-      <c r="J172" s="2">
+      <c r="J172" s="1">
         <v>46383</v>
       </c>
       <c r="K172" t="b">
@@ -7128,7 +7102,7 @@
       <c r="H173">
         <v>186</v>
       </c>
-      <c r="J173" s="2">
+      <c r="J173" s="1">
         <v>46392</v>
       </c>
       <c r="K173" t="b">
@@ -7160,7 +7134,7 @@
       <c r="H174">
         <v>205</v>
       </c>
-      <c r="J174" s="2">
+      <c r="J174" s="1">
         <v>46390</v>
       </c>
       <c r="K174" t="b">
@@ -7192,7 +7166,7 @@
       <c r="H175">
         <v>207</v>
       </c>
-      <c r="J175" s="2">
+      <c r="J175" s="1">
         <v>46392</v>
       </c>
       <c r="K175" t="b">
@@ -7224,7 +7198,7 @@
       <c r="H176">
         <v>218</v>
       </c>
-      <c r="J176" s="2">
+      <c r="J176" s="1">
         <v>46506</v>
       </c>
       <c r="K176" t="b">
@@ -7256,7 +7230,7 @@
       <c r="H177">
         <v>246</v>
       </c>
-      <c r="J177" s="2">
+      <c r="J177" s="1">
         <v>46478</v>
       </c>
       <c r="K177" t="b">
@@ -7288,7 +7262,7 @@
       <c r="H178">
         <v>248</v>
       </c>
-      <c r="J178" s="2">
+      <c r="J178" s="1">
         <v>46500</v>
       </c>
       <c r="K178" t="b">
@@ -7320,7 +7294,7 @@
       <c r="H179">
         <v>276</v>
       </c>
-      <c r="J179" s="2">
+      <c r="J179" s="1">
         <v>46430</v>
       </c>
       <c r="K179" t="b">
@@ -7352,7 +7326,7 @@
       <c r="H180">
         <v>276</v>
       </c>
-      <c r="J180" s="2">
+      <c r="J180" s="1">
         <v>46430</v>
       </c>
       <c r="K180" t="b">
@@ -7384,7 +7358,7 @@
       <c r="H181">
         <v>290</v>
       </c>
-      <c r="J181" s="2">
+      <c r="J181" s="1">
         <v>46467</v>
       </c>
       <c r="K181" t="b">
@@ -7416,7 +7390,7 @@
       <c r="H182">
         <v>317</v>
       </c>
-      <c r="J182" s="2">
+      <c r="J182" s="1">
         <v>46529</v>
       </c>
       <c r="K182" t="b">
@@ -7448,7 +7422,7 @@
       <c r="H183">
         <v>420</v>
       </c>
-      <c r="J183" s="2">
+      <c r="J183" s="1">
         <v>46566</v>
       </c>
       <c r="K183" t="b">
@@ -7480,7 +7454,7 @@
       <c r="H184">
         <v>426</v>
       </c>
-      <c r="J184" s="2">
+      <c r="J184" s="1">
         <v>46571</v>
       </c>
       <c r="K184" t="b">
@@ -7512,7 +7486,7 @@
       <c r="H185">
         <v>721</v>
       </c>
-      <c r="J185" s="2">
+      <c r="J185" s="1">
         <v>46325</v>
       </c>
       <c r="K185" t="b">
@@ -7544,7 +7518,7 @@
       <c r="H186">
         <v>721</v>
       </c>
-      <c r="J186" s="2">
+      <c r="J186" s="1">
         <v>46325</v>
       </c>
       <c r="K186" t="b">
@@ -7576,7 +7550,7 @@
       <c r="H187">
         <v>850</v>
       </c>
-      <c r="J187" s="2">
+      <c r="J187" s="1">
         <v>46345</v>
       </c>
       <c r="K187" t="b">
@@ -7608,7 +7582,7 @@
       <c r="H188">
         <v>850</v>
       </c>
-      <c r="J188" s="2">
+      <c r="J188" s="1">
         <v>46345</v>
       </c>
       <c r="K188" t="b">
@@ -7640,7 +7614,7 @@
       <c r="H189">
         <v>1661</v>
       </c>
-      <c r="J189" s="2">
+      <c r="J189" s="1">
         <v>46498</v>
       </c>
       <c r="K189" t="b">
@@ -7672,7 +7646,7 @@
       <c r="H190">
         <v>1661</v>
       </c>
-      <c r="J190" s="2">
+      <c r="J190" s="1">
         <v>46498</v>
       </c>
       <c r="K190" t="b">
@@ -7704,7 +7678,7 @@
       <c r="H191">
         <v>488</v>
       </c>
-      <c r="J191" s="2">
+      <c r="J191" s="1">
         <v>46190</v>
       </c>
       <c r="K191" t="b">
@@ -7736,7 +7710,7 @@
       <c r="H192">
         <v>25565</v>
       </c>
-      <c r="J192" s="2">
+      <c r="J192" s="1">
         <v>46190</v>
       </c>
       <c r="K192" t="b">
@@ -7768,7 +7742,7 @@
       <c r="H193">
         <v>25567</v>
       </c>
-      <c r="J193" s="2">
+      <c r="J193" s="1">
         <v>46190</v>
       </c>
       <c r="K193" t="b">
@@ -7800,7 +7774,7 @@
       <c r="H194">
         <v>31293</v>
       </c>
-      <c r="J194" s="2">
+      <c r="J194" s="1">
         <v>46190</v>
       </c>
       <c r="K194" t="b">

</xml_diff>

<commit_message>
Atualização automática: vencimentos_tmot (23/07/2026 11:41)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
@@ -1040,8 +1040,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1057,7 +1065,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1065,12 +1073,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1370,37 +1396,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1429,7 +1455,7 @@
       <c r="H2">
         <v>-4402.8</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>41388</v>
       </c>
       <c r="K2" t="b">
@@ -1461,7 +1487,7 @@
       <c r="H3">
         <v>-4254.8</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>39285</v>
       </c>
       <c r="K3" t="b">
@@ -1493,7 +1519,7 @@
       <c r="H4">
         <v>-2354.2</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>40669</v>
       </c>
       <c r="K4" t="b">
@@ -1525,7 +1551,7 @@
       <c r="H5">
         <v>-896.8</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>40669</v>
       </c>
       <c r="K5" t="b">
@@ -1557,7 +1583,7 @@
       <c r="H6">
         <v>-854.1</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>44884</v>
       </c>
       <c r="K6" t="b">
@@ -1589,7 +1615,7 @@
       <c r="H7">
         <v>-413.2</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>43855</v>
       </c>
       <c r="K7" t="b">
@@ -1621,7 +1647,7 @@
       <c r="H8">
         <v>-391.8</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>42769</v>
       </c>
       <c r="K8" t="b">
@@ -1653,7 +1679,7 @@
       <c r="H9">
         <v>-371.5</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>46014</v>
       </c>
       <c r="K9" t="b">
@@ -1685,7 +1711,7 @@
       <c r="H10">
         <v>-368.8</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>46014</v>
       </c>
       <c r="K10" t="b">
@@ -1717,7 +1743,7 @@
       <c r="H11">
         <v>-359</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>45804</v>
       </c>
       <c r="K11" t="b">
@@ -1749,7 +1775,7 @@
       <c r="H12">
         <v>-359</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>45804</v>
       </c>
       <c r="K12" t="b">
@@ -1781,7 +1807,7 @@
       <c r="H13">
         <v>-351</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>42821</v>
       </c>
       <c r="K13" t="b">
@@ -1813,7 +1839,7 @@
       <c r="H14">
         <v>-351</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>46014</v>
       </c>
       <c r="K14" t="b">
@@ -1845,7 +1871,7 @@
       <c r="H15">
         <v>-351</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>46014</v>
       </c>
       <c r="K15" t="b">
@@ -1877,7 +1903,7 @@
       <c r="H16">
         <v>-351</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="2">
         <v>46014</v>
       </c>
       <c r="K16" t="b">
@@ -1909,7 +1935,7 @@
       <c r="H17">
         <v>-345.8</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="2">
         <v>46017</v>
       </c>
       <c r="K17" t="b">
@@ -1941,7 +1967,7 @@
       <c r="H18">
         <v>-345.8</v>
       </c>
-      <c r="J18" s="1">
+      <c r="J18" s="2">
         <v>46017</v>
       </c>
       <c r="K18" t="b">
@@ -1973,7 +1999,7 @@
       <c r="H19">
         <v>-264.2</v>
       </c>
-      <c r="J19" s="1">
+      <c r="J19" s="2">
         <v>40979</v>
       </c>
       <c r="K19" t="b">
@@ -2005,7 +2031,7 @@
       <c r="H20">
         <v>-206.4</v>
       </c>
-      <c r="J20" s="1">
+      <c r="J20" s="2">
         <v>36669</v>
       </c>
       <c r="K20" t="b">
@@ -2037,7 +2063,7 @@
       <c r="H21">
         <v>-131.6</v>
       </c>
-      <c r="J21" s="1">
+      <c r="J21" s="2">
         <v>46111</v>
       </c>
       <c r="K21" t="b">
@@ -2069,7 +2095,7 @@
       <c r="H22">
         <v>-131.6</v>
       </c>
-      <c r="J22" s="1">
+      <c r="J22" s="2">
         <v>46111</v>
       </c>
       <c r="K22" t="b">
@@ -2101,7 +2127,7 @@
       <c r="H23">
         <v>-131.6</v>
       </c>
-      <c r="J23" s="1">
+      <c r="J23" s="2">
         <v>46111</v>
       </c>
       <c r="K23" t="b">
@@ -2133,7 +2159,7 @@
       <c r="H24">
         <v>-131.6</v>
       </c>
-      <c r="J24" s="1">
+      <c r="J24" s="2">
         <v>46111</v>
       </c>
       <c r="K24" t="b">
@@ -2165,7 +2191,7 @@
       <c r="H25">
         <v>-131.6</v>
       </c>
-      <c r="J25" s="1">
+      <c r="J25" s="2">
         <v>46111</v>
       </c>
       <c r="K25" t="b">
@@ -2197,7 +2223,7 @@
       <c r="H26">
         <v>-105</v>
       </c>
-      <c r="J26" s="1">
+      <c r="J26" s="2">
         <v>46161</v>
       </c>
       <c r="K26" t="b">
@@ -2229,7 +2255,7 @@
       <c r="H27">
         <v>-79.8</v>
       </c>
-      <c r="J27" s="1">
+      <c r="J27" s="2">
         <v>43340</v>
       </c>
       <c r="K27" t="b">
@@ -2261,7 +2287,7 @@
       <c r="H28">
         <v>-12.3</v>
       </c>
-      <c r="J28" s="1">
+      <c r="J28" s="2">
         <v>46048</v>
       </c>
       <c r="K28" t="b">
@@ -2293,7 +2319,7 @@
       <c r="H29">
         <v>0</v>
       </c>
-      <c r="J29" s="1">
+      <c r="J29" s="2">
         <v>46211</v>
       </c>
       <c r="K29" t="b">
@@ -2325,7 +2351,7 @@
       <c r="H30">
         <v>3.6</v>
       </c>
-      <c r="J30" s="1">
+      <c r="J30" s="2">
         <v>46234</v>
       </c>
       <c r="K30" t="b">
@@ -2357,7 +2383,7 @@
       <c r="H31">
         <v>6.2</v>
       </c>
-      <c r="J31" s="1">
+      <c r="J31" s="2">
         <v>46234</v>
       </c>
       <c r="K31" t="b">
@@ -2389,7 +2415,7 @@
       <c r="H32">
         <v>7.5</v>
       </c>
-      <c r="J32" s="1">
+      <c r="J32" s="2">
         <v>46234</v>
       </c>
       <c r="K32" t="b">
@@ -2421,7 +2447,7 @@
       <c r="H33">
         <v>10.7</v>
       </c>
-      <c r="J33" s="1">
+      <c r="J33" s="2">
         <v>46234</v>
       </c>
       <c r="K33" t="b">
@@ -2453,7 +2479,7 @@
       <c r="H34">
         <v>20</v>
       </c>
-      <c r="J34" s="1">
+      <c r="J34" s="2">
         <v>46234</v>
       </c>
       <c r="K34" t="b">
@@ -2485,7 +2511,7 @@
       <c r="H35">
         <v>30.8</v>
       </c>
-      <c r="J35" s="1">
+      <c r="J35" s="2">
         <v>46234</v>
       </c>
       <c r="K35" t="b">
@@ -2517,7 +2543,7 @@
       <c r="H36">
         <v>37.1</v>
       </c>
-      <c r="J36" s="1">
+      <c r="J36" s="2">
         <v>46256</v>
       </c>
       <c r="K36" t="b">
@@ -2549,7 +2575,7 @@
       <c r="H37">
         <v>42.8</v>
       </c>
-      <c r="J37" s="1">
+      <c r="J37" s="2">
         <v>46276</v>
       </c>
       <c r="K37" t="b">
@@ -2581,7 +2607,7 @@
       <c r="H38">
         <v>45.2</v>
       </c>
-      <c r="J38" s="1">
+      <c r="J38" s="2">
         <v>46234</v>
       </c>
       <c r="K38" t="b">
@@ -2613,7 +2639,7 @@
       <c r="H39">
         <v>46</v>
       </c>
-      <c r="J39" s="1">
+      <c r="J39" s="2">
         <v>46251</v>
       </c>
       <c r="K39" t="b">
@@ -2645,7 +2671,7 @@
       <c r="H40">
         <v>47.5</v>
       </c>
-      <c r="J40" s="1">
+      <c r="J40" s="2">
         <v>46456</v>
       </c>
       <c r="K40" t="b">
@@ -2677,7 +2703,7 @@
       <c r="H41">
         <v>57.2</v>
       </c>
-      <c r="J41" s="1">
+      <c r="J41" s="2">
         <v>46246</v>
       </c>
       <c r="K41" t="b">
@@ -2709,7 +2735,7 @@
       <c r="H42">
         <v>59.6</v>
       </c>
-      <c r="J42" s="1">
+      <c r="J42" s="2">
         <v>46487</v>
       </c>
       <c r="K42" t="b">
@@ -2741,7 +2767,7 @@
       <c r="H43">
         <v>75.40000000000001</v>
       </c>
-      <c r="J43" s="1">
+      <c r="J43" s="2">
         <v>46283</v>
       </c>
       <c r="K43" t="b">
@@ -2773,7 +2799,7 @@
       <c r="H44">
         <v>76.8</v>
       </c>
-      <c r="J44" s="1">
+      <c r="J44" s="2">
         <v>46285</v>
       </c>
       <c r="K44" t="b">
@@ -2805,7 +2831,7 @@
       <c r="H45">
         <v>83.2</v>
       </c>
-      <c r="J45" s="1">
+      <c r="J45" s="2">
         <v>46547</v>
       </c>
       <c r="K45" t="b">
@@ -2837,7 +2863,7 @@
       <c r="H46">
         <v>84.5</v>
       </c>
-      <c r="J46" s="1">
+      <c r="J46" s="2">
         <v>46240</v>
       </c>
       <c r="K46" t="b">
@@ -2869,7 +2895,7 @@
       <c r="H47">
         <v>85.8</v>
       </c>
-      <c r="J47" s="1">
+      <c r="J47" s="2">
         <v>46266</v>
       </c>
       <c r="K47" t="b">
@@ -2901,7 +2927,7 @@
       <c r="H48">
         <v>86.5</v>
       </c>
-      <c r="J48" s="1">
+      <c r="J48" s="2">
         <v>46241</v>
       </c>
       <c r="K48" t="b">
@@ -2933,7 +2959,7 @@
       <c r="H49">
         <v>91.7</v>
       </c>
-      <c r="J49" s="1">
+      <c r="J49" s="2">
         <v>46243</v>
       </c>
       <c r="K49" t="b">
@@ -2965,7 +2991,7 @@
       <c r="H50">
         <v>91.7</v>
       </c>
-      <c r="J50" s="1">
+      <c r="J50" s="2">
         <v>46243</v>
       </c>
       <c r="K50" t="b">
@@ -2997,7 +3023,7 @@
       <c r="H51">
         <v>91.7</v>
       </c>
-      <c r="J51" s="1">
+      <c r="J51" s="2">
         <v>46250</v>
       </c>
       <c r="K51" t="b">
@@ -3029,7 +3055,7 @@
       <c r="H52">
         <v>98.90000000000001</v>
       </c>
-      <c r="J52" s="1">
+      <c r="J52" s="2">
         <v>46253</v>
       </c>
       <c r="K52" t="b">
@@ -3061,7 +3087,7 @@
       <c r="H53">
         <v>105.5</v>
       </c>
-      <c r="J53" s="1">
+      <c r="J53" s="2">
         <v>46280</v>
       </c>
       <c r="K53" t="b">
@@ -3093,7 +3119,7 @@
       <c r="H54">
         <v>105.6</v>
       </c>
-      <c r="J54" s="1">
+      <c r="J54" s="2">
         <v>46361</v>
       </c>
       <c r="K54" t="b">
@@ -3125,7 +3151,7 @@
       <c r="H55">
         <v>105.7</v>
       </c>
-      <c r="J55" s="1">
+      <c r="J55" s="2">
         <v>46362</v>
       </c>
       <c r="K55" t="b">
@@ -3157,7 +3183,7 @@
       <c r="H56">
         <v>110.7</v>
       </c>
-      <c r="J56" s="1">
+      <c r="J56" s="2">
         <v>46275</v>
       </c>
       <c r="K56" t="b">
@@ -3189,7 +3215,7 @@
       <c r="H57">
         <v>113.2</v>
       </c>
-      <c r="J57" s="1">
+      <c r="J57" s="2">
         <v>46377</v>
       </c>
       <c r="K57" t="b">
@@ -3221,7 +3247,7 @@
       <c r="H58">
         <v>128.8</v>
       </c>
-      <c r="J58" s="1">
+      <c r="J58" s="2">
         <v>46434</v>
       </c>
       <c r="K58" t="b">
@@ -3253,7 +3279,7 @@
       <c r="H59">
         <v>128.8</v>
       </c>
-      <c r="J59" s="1">
+      <c r="J59" s="2">
         <v>46434</v>
       </c>
       <c r="K59" t="b">
@@ -3285,7 +3311,7 @@
       <c r="H60">
         <v>128.8</v>
       </c>
-      <c r="J60" s="1">
+      <c r="J60" s="2">
         <v>46434</v>
       </c>
       <c r="K60" t="b">
@@ -3317,7 +3343,7 @@
       <c r="H61">
         <v>128.8</v>
       </c>
-      <c r="J61" s="1">
+      <c r="J61" s="2">
         <v>46434</v>
       </c>
       <c r="K61" t="b">
@@ -3349,7 +3375,7 @@
       <c r="H62">
         <v>128.8</v>
       </c>
-      <c r="J62" s="1">
+      <c r="J62" s="2">
         <v>46434</v>
       </c>
       <c r="K62" t="b">
@@ -3381,7 +3407,7 @@
       <c r="H63">
         <v>135</v>
       </c>
-      <c r="J63" s="1">
+      <c r="J63" s="2">
         <v>46280</v>
       </c>
       <c r="K63" t="b">
@@ -3413,7 +3439,7 @@
       <c r="H64">
         <v>150.6</v>
       </c>
-      <c r="J64" s="1">
+      <c r="J64" s="2">
         <v>46271</v>
       </c>
       <c r="K64" t="b">
@@ -3445,7 +3471,7 @@
       <c r="H65">
         <v>174.2</v>
       </c>
-      <c r="J65" s="1">
+      <c r="J65" s="2">
         <v>46363</v>
       </c>
       <c r="K65" t="b">
@@ -3477,7 +3503,7 @@
       <c r="H66">
         <v>176.6</v>
       </c>
-      <c r="J66" s="1">
+      <c r="J66" s="2">
         <v>46334</v>
       </c>
       <c r="K66" t="b">
@@ -3509,7 +3535,7 @@
       <c r="H67">
         <v>177.4</v>
       </c>
-      <c r="J67" s="1">
+      <c r="J67" s="2">
         <v>46407</v>
       </c>
       <c r="K67" t="b">
@@ -3541,7 +3567,7 @@
       <c r="H68">
         <v>183.9</v>
       </c>
-      <c r="J68" s="1">
+      <c r="J68" s="2">
         <v>46341</v>
       </c>
       <c r="K68" t="b">
@@ -3573,7 +3599,7 @@
       <c r="H69">
         <v>191.7</v>
       </c>
-      <c r="J69" s="1">
+      <c r="J69" s="2">
         <v>46300</v>
       </c>
       <c r="K69" t="b">
@@ -3605,7 +3631,7 @@
       <c r="H70">
         <v>200</v>
       </c>
-      <c r="J70" s="1">
+      <c r="J70" s="2">
         <v>46336</v>
       </c>
       <c r="K70" t="b">
@@ -3637,7 +3663,7 @@
       <c r="H71">
         <v>201.1</v>
       </c>
-      <c r="J71" s="1">
+      <c r="J71" s="2">
         <v>46319</v>
       </c>
       <c r="K71" t="b">
@@ -3669,7 +3695,7 @@
       <c r="H72">
         <v>206.5</v>
       </c>
-      <c r="J72" s="1">
+      <c r="J72" s="2">
         <v>46308</v>
       </c>
       <c r="K72" t="b">
@@ -3701,7 +3727,7 @@
       <c r="H73">
         <v>207.5</v>
       </c>
-      <c r="J73" s="1">
+      <c r="J73" s="2">
         <v>46390</v>
       </c>
       <c r="K73" t="b">
@@ -3733,7 +3759,7 @@
       <c r="H74">
         <v>247</v>
       </c>
-      <c r="J74" s="1">
+      <c r="J74" s="2">
         <v>46443</v>
       </c>
       <c r="K74" t="b">
@@ -3765,7 +3791,7 @@
       <c r="H75">
         <v>285.3</v>
       </c>
-      <c r="J75" s="1">
+      <c r="J75" s="2">
         <v>46304</v>
       </c>
       <c r="K75" t="b">
@@ -3797,7 +3823,7 @@
       <c r="H76">
         <v>290.8</v>
       </c>
-      <c r="J76" s="1">
+      <c r="J76" s="2">
         <v>46362</v>
       </c>
       <c r="K76" t="b">
@@ -3829,7 +3855,7 @@
       <c r="H77">
         <v>295.2</v>
       </c>
-      <c r="J77" s="1">
+      <c r="J77" s="2">
         <v>46463</v>
       </c>
       <c r="K77" t="b">
@@ -3861,7 +3887,7 @@
       <c r="H78">
         <v>300.2</v>
       </c>
-      <c r="J78" s="1">
+      <c r="J78" s="2">
         <v>46466</v>
       </c>
       <c r="K78" t="b">
@@ -3896,7 +3922,7 @@
       <c r="I79" t="s">
         <v>313</v>
       </c>
-      <c r="J79" s="1">
+      <c r="J79" s="2">
         <v>36557</v>
       </c>
       <c r="K79" t="b">
@@ -3931,7 +3957,7 @@
       <c r="I80" t="s">
         <v>314</v>
       </c>
-      <c r="J80" s="1">
+      <c r="J80" s="2">
         <v>41275</v>
       </c>
       <c r="K80" t="b">
@@ -3966,7 +3992,7 @@
       <c r="I81" t="s">
         <v>315</v>
       </c>
-      <c r="J81" s="1">
+      <c r="J81" s="2">
         <v>45380</v>
       </c>
       <c r="K81" t="b">
@@ -4001,7 +4027,7 @@
       <c r="I82" t="s">
         <v>316</v>
       </c>
-      <c r="J82" s="1">
+      <c r="J82" s="2">
         <v>45421</v>
       </c>
       <c r="K82" t="b">
@@ -4036,7 +4062,7 @@
       <c r="I83" t="s">
         <v>316</v>
       </c>
-      <c r="J83" s="1">
+      <c r="J83" s="2">
         <v>45428</v>
       </c>
       <c r="K83" t="b">
@@ -4071,7 +4097,7 @@
       <c r="I84" t="s">
         <v>317</v>
       </c>
-      <c r="J84" s="1">
+      <c r="J84" s="2">
         <v>45490</v>
       </c>
       <c r="K84" t="b">
@@ -4106,7 +4132,7 @@
       <c r="I85" t="s">
         <v>318</v>
       </c>
-      <c r="J85" s="1">
+      <c r="J85" s="2">
         <v>45566</v>
       </c>
       <c r="K85" t="b">
@@ -4141,7 +4167,7 @@
       <c r="I86" t="s">
         <v>319</v>
       </c>
-      <c r="J86" s="1">
+      <c r="J86" s="2">
         <v>45986</v>
       </c>
       <c r="K86" t="b">
@@ -4176,7 +4202,7 @@
       <c r="I87" t="s">
         <v>320</v>
       </c>
-      <c r="J87" s="1">
+      <c r="J87" s="2">
         <v>46106</v>
       </c>
       <c r="K87" t="b">
@@ -4211,7 +4237,7 @@
       <c r="I88" t="s">
         <v>321</v>
       </c>
-      <c r="J88" s="1">
+      <c r="J88" s="2">
         <v>46142</v>
       </c>
       <c r="K88" t="b">
@@ -4246,7 +4272,7 @@
       <c r="I89" t="s">
         <v>322</v>
       </c>
-      <c r="J89" s="1">
+      <c r="J89" s="2">
         <v>46274</v>
       </c>
       <c r="K89" t="b">
@@ -4281,7 +4307,7 @@
       <c r="I90" t="s">
         <v>322</v>
       </c>
-      <c r="J90" s="1">
+      <c r="J90" s="2">
         <v>46276</v>
       </c>
       <c r="K90" t="b">
@@ -4316,7 +4342,7 @@
       <c r="I91" t="s">
         <v>322</v>
       </c>
-      <c r="J91" s="1">
+      <c r="J91" s="2">
         <v>46284</v>
       </c>
       <c r="K91" t="b">
@@ -4351,7 +4377,7 @@
       <c r="I92" t="s">
         <v>323</v>
       </c>
-      <c r="J92" s="1">
+      <c r="J92" s="2">
         <v>46317</v>
       </c>
       <c r="K92" t="b">
@@ -4386,7 +4412,7 @@
       <c r="I93" t="s">
         <v>323</v>
       </c>
-      <c r="J93" s="1">
+      <c r="J93" s="2">
         <v>46319</v>
       </c>
       <c r="K93" t="b">
@@ -4421,7 +4447,7 @@
       <c r="I94" t="s">
         <v>324</v>
       </c>
-      <c r="J94" s="1">
+      <c r="J94" s="2">
         <v>46333</v>
       </c>
       <c r="K94" t="b">
@@ -4456,7 +4482,7 @@
       <c r="I95" t="s">
         <v>324</v>
       </c>
-      <c r="J95" s="1">
+      <c r="J95" s="2">
         <v>46338</v>
       </c>
       <c r="K95" t="b">
@@ -4491,7 +4517,7 @@
       <c r="I96" t="s">
         <v>324</v>
       </c>
-      <c r="J96" s="1">
+      <c r="J96" s="2">
         <v>46338</v>
       </c>
       <c r="K96" t="b">
@@ -4526,7 +4552,7 @@
       <c r="I97" t="s">
         <v>324</v>
       </c>
-      <c r="J97" s="1">
+      <c r="J97" s="2">
         <v>46341</v>
       </c>
       <c r="K97" t="b">
@@ -4561,7 +4587,7 @@
       <c r="I98" t="s">
         <v>324</v>
       </c>
-      <c r="J98" s="1">
+      <c r="J98" s="2">
         <v>46344</v>
       </c>
       <c r="K98" t="b">
@@ -4596,7 +4622,7 @@
       <c r="I99" t="s">
         <v>324</v>
       </c>
-      <c r="J99" s="1">
+      <c r="J99" s="2">
         <v>46354</v>
       </c>
       <c r="K99" t="b">
@@ -4631,7 +4657,7 @@
       <c r="I100" t="s">
         <v>324</v>
       </c>
-      <c r="J100" s="1">
+      <c r="J100" s="2">
         <v>46360</v>
       </c>
       <c r="K100" t="b">
@@ -4666,7 +4692,7 @@
       <c r="I101" t="s">
         <v>324</v>
       </c>
-      <c r="J101" s="1">
+      <c r="J101" s="2">
         <v>46360</v>
       </c>
       <c r="K101" t="b">
@@ -4701,7 +4727,7 @@
       <c r="I102" t="s">
         <v>325</v>
       </c>
-      <c r="J102" s="1">
+      <c r="J102" s="2">
         <v>46366</v>
       </c>
       <c r="K102" t="b">
@@ -4736,7 +4762,7 @@
       <c r="I103" t="s">
         <v>325</v>
       </c>
-      <c r="J103" s="1">
+      <c r="J103" s="2">
         <v>46375</v>
       </c>
       <c r="K103" t="b">
@@ -4771,7 +4797,7 @@
       <c r="I104" t="s">
         <v>325</v>
       </c>
-      <c r="J104" s="1">
+      <c r="J104" s="2">
         <v>46388</v>
       </c>
       <c r="K104" t="b">
@@ -4806,7 +4832,7 @@
       <c r="I105" t="s">
         <v>326</v>
       </c>
-      <c r="J105" s="1">
+      <c r="J105" s="2">
         <v>46401</v>
       </c>
       <c r="K105" t="b">
@@ -4841,7 +4867,7 @@
       <c r="I106" t="s">
         <v>326</v>
       </c>
-      <c r="J106" s="1">
+      <c r="J106" s="2">
         <v>46401</v>
       </c>
       <c r="K106" t="b">
@@ -4876,7 +4902,7 @@
       <c r="I107" t="s">
         <v>326</v>
       </c>
-      <c r="J107" s="1">
+      <c r="J107" s="2">
         <v>46401</v>
       </c>
       <c r="K107" t="b">
@@ -4911,7 +4937,7 @@
       <c r="I108" t="s">
         <v>326</v>
       </c>
-      <c r="J108" s="1">
+      <c r="J108" s="2">
         <v>46413</v>
       </c>
       <c r="K108" t="b">
@@ -4946,7 +4972,7 @@
       <c r="I109" t="s">
         <v>327</v>
       </c>
-      <c r="J109" s="1">
+      <c r="J109" s="2">
         <v>46424</v>
       </c>
       <c r="K109" t="b">
@@ -4981,7 +5007,7 @@
       <c r="I110" t="s">
         <v>327</v>
       </c>
-      <c r="J110" s="1">
+      <c r="J110" s="2">
         <v>46427</v>
       </c>
       <c r="K110" t="b">
@@ -5016,7 +5042,7 @@
       <c r="I111" t="s">
         <v>327</v>
       </c>
-      <c r="J111" s="1">
+      <c r="J111" s="2">
         <v>46437</v>
       </c>
       <c r="K111" t="b">
@@ -5051,7 +5077,7 @@
       <c r="I112" t="s">
         <v>327</v>
       </c>
-      <c r="J112" s="1">
+      <c r="J112" s="2">
         <v>46451</v>
       </c>
       <c r="K112" t="b">
@@ -5086,7 +5112,7 @@
       <c r="I113" t="s">
         <v>328</v>
       </c>
-      <c r="J113" s="1">
+      <c r="J113" s="2">
         <v>46455</v>
       </c>
       <c r="K113" t="b">
@@ -5121,7 +5147,7 @@
       <c r="I114" t="s">
         <v>328</v>
       </c>
-      <c r="J114" s="1">
+      <c r="J114" s="2">
         <v>46457</v>
       </c>
       <c r="K114" t="b">
@@ -5156,7 +5182,7 @@
       <c r="I115" t="s">
         <v>328</v>
       </c>
-      <c r="J115" s="1">
+      <c r="J115" s="2">
         <v>46462</v>
       </c>
       <c r="K115" t="b">
@@ -5191,7 +5217,7 @@
       <c r="I116" t="s">
         <v>328</v>
       </c>
-      <c r="J116" s="1">
+      <c r="J116" s="2">
         <v>46464</v>
       </c>
       <c r="K116" t="b">
@@ -5226,7 +5252,7 @@
       <c r="I117" t="s">
         <v>328</v>
       </c>
-      <c r="J117" s="1">
+      <c r="J117" s="2">
         <v>46470</v>
       </c>
       <c r="K117" t="b">
@@ -5261,7 +5287,7 @@
       <c r="I118" t="s">
         <v>329</v>
       </c>
-      <c r="J118" s="1">
+      <c r="J118" s="2">
         <v>46485</v>
       </c>
       <c r="K118" t="b">
@@ -5296,7 +5322,7 @@
       <c r="I119" t="s">
         <v>329</v>
       </c>
-      <c r="J119" s="1">
+      <c r="J119" s="2">
         <v>46499</v>
       </c>
       <c r="K119" t="b">
@@ -5331,7 +5357,7 @@
       <c r="I120" t="s">
         <v>329</v>
       </c>
-      <c r="J120" s="1">
+      <c r="J120" s="2">
         <v>46504</v>
       </c>
       <c r="K120" t="b">
@@ -5366,7 +5392,7 @@
       <c r="I121" t="s">
         <v>329</v>
       </c>
-      <c r="J121" s="1">
+      <c r="J121" s="2">
         <v>46504</v>
       </c>
       <c r="K121" t="b">
@@ -5401,7 +5427,7 @@
       <c r="I122" t="s">
         <v>329</v>
       </c>
-      <c r="J122" s="1">
+      <c r="J122" s="2">
         <v>46507</v>
       </c>
       <c r="K122" t="b">
@@ -5436,7 +5462,7 @@
       <c r="I123" t="s">
         <v>329</v>
       </c>
-      <c r="J123" s="1">
+      <c r="J123" s="2">
         <v>46508</v>
       </c>
       <c r="K123" t="b">
@@ -5471,7 +5497,7 @@
       <c r="I124" t="s">
         <v>329</v>
       </c>
-      <c r="J124" s="1">
+      <c r="J124" s="2">
         <v>46512</v>
       </c>
       <c r="K124" t="b">
@@ -5506,7 +5532,7 @@
       <c r="I125" t="s">
         <v>329</v>
       </c>
-      <c r="J125" s="1">
+      <c r="J125" s="2">
         <v>46512</v>
       </c>
       <c r="K125" t="b">
@@ -5541,7 +5567,7 @@
       <c r="I126" t="s">
         <v>330</v>
       </c>
-      <c r="J126" s="1">
+      <c r="J126" s="2">
         <v>46528</v>
       </c>
       <c r="K126" t="b">
@@ -5576,7 +5602,7 @@
       <c r="I127" t="s">
         <v>330</v>
       </c>
-      <c r="J127" s="1">
+      <c r="J127" s="2">
         <v>46529</v>
       </c>
       <c r="K127" t="b">
@@ -5611,7 +5637,7 @@
       <c r="I128" t="s">
         <v>330</v>
       </c>
-      <c r="J128" s="1">
+      <c r="J128" s="2">
         <v>46537</v>
       </c>
       <c r="K128" t="b">
@@ -5646,7 +5672,7 @@
       <c r="I129" t="s">
         <v>331</v>
       </c>
-      <c r="J129" s="1">
+      <c r="J129" s="2">
         <v>46546</v>
       </c>
       <c r="K129" t="b">
@@ -5681,7 +5707,7 @@
       <c r="I130" t="s">
         <v>331</v>
       </c>
-      <c r="J130" s="1">
+      <c r="J130" s="2">
         <v>46547</v>
       </c>
       <c r="K130" t="b">
@@ -5716,7 +5742,7 @@
       <c r="I131" t="s">
         <v>331</v>
       </c>
-      <c r="J131" s="1">
+      <c r="J131" s="2">
         <v>46547</v>
       </c>
       <c r="K131" t="b">
@@ -5751,7 +5777,7 @@
       <c r="I132" t="s">
         <v>331</v>
       </c>
-      <c r="J132" s="1">
+      <c r="J132" s="2">
         <v>46547</v>
       </c>
       <c r="K132" t="b">
@@ -5786,7 +5812,7 @@
       <c r="I133" t="s">
         <v>331</v>
       </c>
-      <c r="J133" s="1">
+      <c r="J133" s="2">
         <v>46551</v>
       </c>
       <c r="K133" t="b">
@@ -5821,7 +5847,7 @@
       <c r="I134" t="s">
         <v>331</v>
       </c>
-      <c r="J134" s="1">
+      <c r="J134" s="2">
         <v>46560</v>
       </c>
       <c r="K134" t="b">
@@ -5856,7 +5882,7 @@
       <c r="I135" t="s">
         <v>331</v>
       </c>
-      <c r="J135" s="1">
+      <c r="J135" s="2">
         <v>46564</v>
       </c>
       <c r="K135" t="b">
@@ -5891,7 +5917,7 @@
       <c r="I136" t="s">
         <v>331</v>
       </c>
-      <c r="J136" s="1">
+      <c r="J136" s="2">
         <v>46567</v>
       </c>
       <c r="K136" t="b">
@@ -5926,7 +5952,7 @@
       <c r="I137" t="s">
         <v>331</v>
       </c>
-      <c r="J137" s="1">
+      <c r="J137" s="2">
         <v>46568</v>
       </c>
       <c r="K137" t="b">
@@ -5961,7 +5987,7 @@
       <c r="I138" t="s">
         <v>331</v>
       </c>
-      <c r="J138" s="1">
+      <c r="J138" s="2">
         <v>46571</v>
       </c>
       <c r="K138" t="b">
@@ -5996,7 +6022,7 @@
       <c r="I139" t="s">
         <v>332</v>
       </c>
-      <c r="J139" s="1">
+      <c r="J139" s="2">
         <v>46197</v>
       </c>
       <c r="K139" t="b">
@@ -6031,7 +6057,7 @@
       <c r="I140" t="s">
         <v>333</v>
       </c>
-      <c r="J140" s="1">
+      <c r="J140" s="2">
         <v>46212</v>
       </c>
       <c r="K140" t="b">
@@ -6066,7 +6092,7 @@
       <c r="I141" t="s">
         <v>334</v>
       </c>
-      <c r="J141" s="1">
+      <c r="J141" s="2">
         <v>46225</v>
       </c>
       <c r="K141" t="b">
@@ -6101,7 +6127,7 @@
       <c r="I142" t="s">
         <v>335</v>
       </c>
-      <c r="J142" s="1">
+      <c r="J142" s="2">
         <v>46234</v>
       </c>
       <c r="K142" t="b">
@@ -6136,7 +6162,7 @@
       <c r="I143" t="s">
         <v>336</v>
       </c>
-      <c r="J143" s="1">
+      <c r="J143" s="2">
         <v>46234</v>
       </c>
       <c r="K143" t="b">
@@ -6171,7 +6197,7 @@
       <c r="I144" t="s">
         <v>337</v>
       </c>
-      <c r="J144" s="1">
+      <c r="J144" s="2">
         <v>46263</v>
       </c>
       <c r="K144" t="b">
@@ -6206,7 +6232,7 @@
       <c r="I145" t="s">
         <v>338</v>
       </c>
-      <c r="J145" s="1">
+      <c r="J145" s="2">
         <v>46266</v>
       </c>
       <c r="K145" t="b">
@@ -6238,7 +6264,7 @@
       <c r="H146">
         <v>-1476</v>
       </c>
-      <c r="J146" s="1">
+      <c r="J146" s="2">
         <v>43773</v>
       </c>
       <c r="K146" t="b">
@@ -6270,7 +6296,7 @@
       <c r="H147">
         <v>-1469</v>
       </c>
-      <c r="J147" s="1">
+      <c r="J147" s="2">
         <v>43773</v>
       </c>
       <c r="K147" t="b">
@@ -6302,7 +6328,7 @@
       <c r="H148">
         <v>-1121</v>
       </c>
-      <c r="J148" s="1">
+      <c r="J148" s="2">
         <v>45295</v>
       </c>
       <c r="K148" t="b">
@@ -6334,7 +6360,7 @@
       <c r="H149">
         <v>-1018</v>
       </c>
-      <c r="J149" s="1">
+      <c r="J149" s="2">
         <v>45617</v>
       </c>
       <c r="K149" t="b">
@@ -6366,7 +6392,7 @@
       <c r="H150">
         <v>-950</v>
       </c>
-      <c r="J150" s="1">
+      <c r="J150" s="2">
         <v>45677</v>
       </c>
       <c r="K150" t="b">
@@ -6398,7 +6424,7 @@
       <c r="H151">
         <v>-943</v>
       </c>
-      <c r="J151" s="1">
+      <c r="J151" s="2">
         <v>44944</v>
       </c>
       <c r="K151" t="b">
@@ -6430,7 +6456,7 @@
       <c r="H152">
         <v>-252</v>
       </c>
-      <c r="J152" s="1">
+      <c r="J152" s="2">
         <v>46092</v>
       </c>
       <c r="K152" t="b">
@@ -6462,7 +6488,7 @@
       <c r="H153">
         <v>-196</v>
       </c>
-      <c r="J153" s="1">
+      <c r="J153" s="2">
         <v>45988</v>
       </c>
       <c r="K153" t="b">
@@ -6494,7 +6520,7 @@
       <c r="H154">
         <v>-196</v>
       </c>
-      <c r="J154" s="1">
+      <c r="J154" s="2">
         <v>45988</v>
       </c>
       <c r="K154" t="b">
@@ -6526,7 +6552,7 @@
       <c r="H155">
         <v>-47</v>
       </c>
-      <c r="J155" s="1">
+      <c r="J155" s="2">
         <v>46176</v>
       </c>
       <c r="K155" t="b">
@@ -6558,7 +6584,7 @@
       <c r="H156">
         <v>-47</v>
       </c>
-      <c r="J156" s="1">
+      <c r="J156" s="2">
         <v>46176</v>
       </c>
       <c r="K156" t="b">
@@ -6590,7 +6616,7 @@
       <c r="H157">
         <v>-33</v>
       </c>
-      <c r="J157" s="1">
+      <c r="J157" s="2">
         <v>46199</v>
       </c>
       <c r="K157" t="b">
@@ -6622,7 +6648,7 @@
       <c r="H158">
         <v>-33</v>
       </c>
-      <c r="J158" s="1">
+      <c r="J158" s="2">
         <v>46199</v>
       </c>
       <c r="K158" t="b">
@@ -6654,7 +6680,7 @@
       <c r="H159">
         <v>-6</v>
       </c>
-      <c r="J159" s="1">
+      <c r="J159" s="2">
         <v>45967</v>
       </c>
       <c r="K159" t="b">
@@ -6686,7 +6712,7 @@
       <c r="H160">
         <v>43</v>
       </c>
-      <c r="J160" s="1">
+      <c r="J160" s="2">
         <v>46440</v>
       </c>
       <c r="K160" t="b">
@@ -6718,7 +6744,7 @@
       <c r="H161">
         <v>43</v>
       </c>
-      <c r="J161" s="1">
+      <c r="J161" s="2">
         <v>46440</v>
       </c>
       <c r="K161" t="b">
@@ -6750,7 +6776,7 @@
       <c r="H162">
         <v>73</v>
       </c>
-      <c r="J162" s="1">
+      <c r="J162" s="2">
         <v>46264</v>
       </c>
       <c r="K162" t="b">
@@ -6782,7 +6808,7 @@
       <c r="H163">
         <v>73</v>
       </c>
-      <c r="J163" s="1">
+      <c r="J163" s="2">
         <v>46264</v>
       </c>
       <c r="K163" t="b">
@@ -6814,7 +6840,7 @@
       <c r="H164">
         <v>102</v>
       </c>
-      <c r="J164" s="1">
+      <c r="J164" s="2">
         <v>46463</v>
       </c>
       <c r="K164" t="b">
@@ -6846,7 +6872,7 @@
       <c r="H165">
         <v>118</v>
       </c>
-      <c r="J165" s="1">
+      <c r="J165" s="2">
         <v>46337</v>
       </c>
       <c r="K165" t="b">
@@ -6878,7 +6904,7 @@
       <c r="H166">
         <v>146</v>
       </c>
-      <c r="J166" s="1">
+      <c r="J166" s="2">
         <v>46451</v>
       </c>
       <c r="K166" t="b">
@@ -6910,7 +6936,7 @@
       <c r="H167">
         <v>152</v>
       </c>
-      <c r="J167" s="1">
+      <c r="J167" s="2">
         <v>46245</v>
       </c>
       <c r="K167" t="b">
@@ -6942,7 +6968,7 @@
       <c r="H168">
         <v>152</v>
       </c>
-      <c r="J168" s="1">
+      <c r="J168" s="2">
         <v>46245</v>
       </c>
       <c r="K168" t="b">
@@ -6974,7 +7000,7 @@
       <c r="H169">
         <v>163</v>
       </c>
-      <c r="J169" s="1">
+      <c r="J169" s="2">
         <v>46324</v>
       </c>
       <c r="K169" t="b">
@@ -7006,7 +7032,7 @@
       <c r="H170">
         <v>163</v>
       </c>
-      <c r="J170" s="1">
+      <c r="J170" s="2">
         <v>46324</v>
       </c>
       <c r="K170" t="b">
@@ -7038,7 +7064,7 @@
       <c r="H171">
         <v>164</v>
       </c>
-      <c r="J171" s="1">
+      <c r="J171" s="2">
         <v>46426</v>
       </c>
       <c r="K171" t="b">
@@ -7070,7 +7096,7 @@
       <c r="H172">
         <v>175</v>
       </c>
-      <c r="J172" s="1">
+      <c r="J172" s="2">
         <v>46383</v>
       </c>
       <c r="K172" t="b">
@@ -7102,7 +7128,7 @@
       <c r="H173">
         <v>186</v>
       </c>
-      <c r="J173" s="1">
+      <c r="J173" s="2">
         <v>46392</v>
       </c>
       <c r="K173" t="b">
@@ -7134,7 +7160,7 @@
       <c r="H174">
         <v>205</v>
       </c>
-      <c r="J174" s="1">
+      <c r="J174" s="2">
         <v>46390</v>
       </c>
       <c r="K174" t="b">
@@ -7166,7 +7192,7 @@
       <c r="H175">
         <v>207</v>
       </c>
-      <c r="J175" s="1">
+      <c r="J175" s="2">
         <v>46392</v>
       </c>
       <c r="K175" t="b">
@@ -7198,7 +7224,7 @@
       <c r="H176">
         <v>218</v>
       </c>
-      <c r="J176" s="1">
+      <c r="J176" s="2">
         <v>46506</v>
       </c>
       <c r="K176" t="b">
@@ -7230,7 +7256,7 @@
       <c r="H177">
         <v>246</v>
       </c>
-      <c r="J177" s="1">
+      <c r="J177" s="2">
         <v>46478</v>
       </c>
       <c r="K177" t="b">
@@ -7262,7 +7288,7 @@
       <c r="H178">
         <v>248</v>
       </c>
-      <c r="J178" s="1">
+      <c r="J178" s="2">
         <v>46500</v>
       </c>
       <c r="K178" t="b">
@@ -7294,7 +7320,7 @@
       <c r="H179">
         <v>276</v>
       </c>
-      <c r="J179" s="1">
+      <c r="J179" s="2">
         <v>46430</v>
       </c>
       <c r="K179" t="b">
@@ -7326,7 +7352,7 @@
       <c r="H180">
         <v>276</v>
       </c>
-      <c r="J180" s="1">
+      <c r="J180" s="2">
         <v>46430</v>
       </c>
       <c r="K180" t="b">
@@ -7358,7 +7384,7 @@
       <c r="H181">
         <v>290</v>
       </c>
-      <c r="J181" s="1">
+      <c r="J181" s="2">
         <v>46467</v>
       </c>
       <c r="K181" t="b">
@@ -7390,7 +7416,7 @@
       <c r="H182">
         <v>317</v>
       </c>
-      <c r="J182" s="1">
+      <c r="J182" s="2">
         <v>46529</v>
       </c>
       <c r="K182" t="b">
@@ -7422,7 +7448,7 @@
       <c r="H183">
         <v>420</v>
       </c>
-      <c r="J183" s="1">
+      <c r="J183" s="2">
         <v>46566</v>
       </c>
       <c r="K183" t="b">
@@ -7454,7 +7480,7 @@
       <c r="H184">
         <v>426</v>
       </c>
-      <c r="J184" s="1">
+      <c r="J184" s="2">
         <v>46571</v>
       </c>
       <c r="K184" t="b">
@@ -7486,7 +7512,7 @@
       <c r="H185">
         <v>721</v>
       </c>
-      <c r="J185" s="1">
+      <c r="J185" s="2">
         <v>46325</v>
       </c>
       <c r="K185" t="b">
@@ -7518,7 +7544,7 @@
       <c r="H186">
         <v>721</v>
       </c>
-      <c r="J186" s="1">
+      <c r="J186" s="2">
         <v>46325</v>
       </c>
       <c r="K186" t="b">
@@ -7550,7 +7576,7 @@
       <c r="H187">
         <v>850</v>
       </c>
-      <c r="J187" s="1">
+      <c r="J187" s="2">
         <v>46345</v>
       </c>
       <c r="K187" t="b">
@@ -7582,7 +7608,7 @@
       <c r="H188">
         <v>850</v>
       </c>
-      <c r="J188" s="1">
+      <c r="J188" s="2">
         <v>46345</v>
       </c>
       <c r="K188" t="b">
@@ -7614,7 +7640,7 @@
       <c r="H189">
         <v>1661</v>
       </c>
-      <c r="J189" s="1">
+      <c r="J189" s="2">
         <v>46498</v>
       </c>
       <c r="K189" t="b">
@@ -7646,7 +7672,7 @@
       <c r="H190">
         <v>1661</v>
       </c>
-      <c r="J190" s="1">
+      <c r="J190" s="2">
         <v>46498</v>
       </c>
       <c r="K190" t="b">
@@ -7678,7 +7704,7 @@
       <c r="H191">
         <v>488</v>
       </c>
-      <c r="J191" s="1">
+      <c r="J191" s="2">
         <v>46190</v>
       </c>
       <c r="K191" t="b">
@@ -7710,7 +7736,7 @@
       <c r="H192">
         <v>25565</v>
       </c>
-      <c r="J192" s="1">
+      <c r="J192" s="2">
         <v>46190</v>
       </c>
       <c r="K192" t="b">
@@ -7742,7 +7768,7 @@
       <c r="H193">
         <v>25567</v>
       </c>
-      <c r="J193" s="1">
+      <c r="J193" s="2">
         <v>46190</v>
       </c>
       <c r="K193" t="b">
@@ -7774,7 +7800,7 @@
       <c r="H194">
         <v>31293</v>
       </c>
-      <c r="J194" s="1">
+      <c r="J194" s="2">
         <v>46190</v>
       </c>
       <c r="K194" t="b">

</xml_diff>

<commit_message>
Atualização automática: vencimentos_tmot (23/07/2026 16:17)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
@@ -1040,16 +1040,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1065,7 +1057,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1073,30 +1065,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1396,37 +1370,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1455,7 +1429,7 @@
       <c r="H2">
         <v>-4402.8</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>41388</v>
       </c>
       <c r="K2" t="b">
@@ -1487,7 +1461,7 @@
       <c r="H3">
         <v>-4254.8</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>39285</v>
       </c>
       <c r="K3" t="b">
@@ -1519,7 +1493,7 @@
       <c r="H4">
         <v>-2354.2</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>40669</v>
       </c>
       <c r="K4" t="b">
@@ -1551,7 +1525,7 @@
       <c r="H5">
         <v>-896.8</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>40669</v>
       </c>
       <c r="K5" t="b">
@@ -1583,7 +1557,7 @@
       <c r="H6">
         <v>-854.1</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>44884</v>
       </c>
       <c r="K6" t="b">
@@ -1615,7 +1589,7 @@
       <c r="H7">
         <v>-413.2</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>43855</v>
       </c>
       <c r="K7" t="b">
@@ -1647,7 +1621,7 @@
       <c r="H8">
         <v>-391.8</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>42769</v>
       </c>
       <c r="K8" t="b">
@@ -1679,7 +1653,7 @@
       <c r="H9">
         <v>-371.5</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>46014</v>
       </c>
       <c r="K9" t="b">
@@ -1711,7 +1685,7 @@
       <c r="H10">
         <v>-368.8</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>46014</v>
       </c>
       <c r="K10" t="b">
@@ -1743,7 +1717,7 @@
       <c r="H11">
         <v>-359</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>45804</v>
       </c>
       <c r="K11" t="b">
@@ -1775,7 +1749,7 @@
       <c r="H12">
         <v>-359</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>45804</v>
       </c>
       <c r="K12" t="b">
@@ -1807,7 +1781,7 @@
       <c r="H13">
         <v>-351</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>42821</v>
       </c>
       <c r="K13" t="b">
@@ -1839,7 +1813,7 @@
       <c r="H14">
         <v>-351</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>46014</v>
       </c>
       <c r="K14" t="b">
@@ -1871,7 +1845,7 @@
       <c r="H15">
         <v>-351</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <v>46014</v>
       </c>
       <c r="K15" t="b">
@@ -1903,7 +1877,7 @@
       <c r="H16">
         <v>-351</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <v>46014</v>
       </c>
       <c r="K16" t="b">
@@ -1935,7 +1909,7 @@
       <c r="H17">
         <v>-345.8</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="1">
         <v>46017</v>
       </c>
       <c r="K17" t="b">
@@ -1967,7 +1941,7 @@
       <c r="H18">
         <v>-345.8</v>
       </c>
-      <c r="J18" s="2">
+      <c r="J18" s="1">
         <v>46017</v>
       </c>
       <c r="K18" t="b">
@@ -1999,7 +1973,7 @@
       <c r="H19">
         <v>-264.2</v>
       </c>
-      <c r="J19" s="2">
+      <c r="J19" s="1">
         <v>40979</v>
       </c>
       <c r="K19" t="b">
@@ -2031,7 +2005,7 @@
       <c r="H20">
         <v>-206.4</v>
       </c>
-      <c r="J20" s="2">
+      <c r="J20" s="1">
         <v>36669</v>
       </c>
       <c r="K20" t="b">
@@ -2063,7 +2037,7 @@
       <c r="H21">
         <v>-131.6</v>
       </c>
-      <c r="J21" s="2">
+      <c r="J21" s="1">
         <v>46111</v>
       </c>
       <c r="K21" t="b">
@@ -2095,7 +2069,7 @@
       <c r="H22">
         <v>-131.6</v>
       </c>
-      <c r="J22" s="2">
+      <c r="J22" s="1">
         <v>46111</v>
       </c>
       <c r="K22" t="b">
@@ -2127,7 +2101,7 @@
       <c r="H23">
         <v>-131.6</v>
       </c>
-      <c r="J23" s="2">
+      <c r="J23" s="1">
         <v>46111</v>
       </c>
       <c r="K23" t="b">
@@ -2159,7 +2133,7 @@
       <c r="H24">
         <v>-131.6</v>
       </c>
-      <c r="J24" s="2">
+      <c r="J24" s="1">
         <v>46111</v>
       </c>
       <c r="K24" t="b">
@@ -2191,7 +2165,7 @@
       <c r="H25">
         <v>-131.6</v>
       </c>
-      <c r="J25" s="2">
+      <c r="J25" s="1">
         <v>46111</v>
       </c>
       <c r="K25" t="b">
@@ -2223,7 +2197,7 @@
       <c r="H26">
         <v>-105</v>
       </c>
-      <c r="J26" s="2">
+      <c r="J26" s="1">
         <v>46161</v>
       </c>
       <c r="K26" t="b">
@@ -2255,7 +2229,7 @@
       <c r="H27">
         <v>-79.8</v>
       </c>
-      <c r="J27" s="2">
+      <c r="J27" s="1">
         <v>43340</v>
       </c>
       <c r="K27" t="b">
@@ -2287,7 +2261,7 @@
       <c r="H28">
         <v>-12.3</v>
       </c>
-      <c r="J28" s="2">
+      <c r="J28" s="1">
         <v>46048</v>
       </c>
       <c r="K28" t="b">
@@ -2319,7 +2293,7 @@
       <c r="H29">
         <v>0</v>
       </c>
-      <c r="J29" s="2">
+      <c r="J29" s="1">
         <v>46211</v>
       </c>
       <c r="K29" t="b">
@@ -2351,7 +2325,7 @@
       <c r="H30">
         <v>3.6</v>
       </c>
-      <c r="J30" s="2">
+      <c r="J30" s="1">
         <v>46234</v>
       </c>
       <c r="K30" t="b">
@@ -2383,7 +2357,7 @@
       <c r="H31">
         <v>6.2</v>
       </c>
-      <c r="J31" s="2">
+      <c r="J31" s="1">
         <v>46234</v>
       </c>
       <c r="K31" t="b">
@@ -2415,7 +2389,7 @@
       <c r="H32">
         <v>7.5</v>
       </c>
-      <c r="J32" s="2">
+      <c r="J32" s="1">
         <v>46234</v>
       </c>
       <c r="K32" t="b">
@@ -2447,7 +2421,7 @@
       <c r="H33">
         <v>10.7</v>
       </c>
-      <c r="J33" s="2">
+      <c r="J33" s="1">
         <v>46234</v>
       </c>
       <c r="K33" t="b">
@@ -2479,7 +2453,7 @@
       <c r="H34">
         <v>20</v>
       </c>
-      <c r="J34" s="2">
+      <c r="J34" s="1">
         <v>46234</v>
       </c>
       <c r="K34" t="b">
@@ -2511,7 +2485,7 @@
       <c r="H35">
         <v>30.8</v>
       </c>
-      <c r="J35" s="2">
+      <c r="J35" s="1">
         <v>46234</v>
       </c>
       <c r="K35" t="b">
@@ -2543,7 +2517,7 @@
       <c r="H36">
         <v>37.1</v>
       </c>
-      <c r="J36" s="2">
+      <c r="J36" s="1">
         <v>46256</v>
       </c>
       <c r="K36" t="b">
@@ -2575,7 +2549,7 @@
       <c r="H37">
         <v>42.8</v>
       </c>
-      <c r="J37" s="2">
+      <c r="J37" s="1">
         <v>46276</v>
       </c>
       <c r="K37" t="b">
@@ -2607,7 +2581,7 @@
       <c r="H38">
         <v>45.2</v>
       </c>
-      <c r="J38" s="2">
+      <c r="J38" s="1">
         <v>46234</v>
       </c>
       <c r="K38" t="b">
@@ -2639,7 +2613,7 @@
       <c r="H39">
         <v>46</v>
       </c>
-      <c r="J39" s="2">
+      <c r="J39" s="1">
         <v>46251</v>
       </c>
       <c r="K39" t="b">
@@ -2671,7 +2645,7 @@
       <c r="H40">
         <v>47.5</v>
       </c>
-      <c r="J40" s="2">
+      <c r="J40" s="1">
         <v>46456</v>
       </c>
       <c r="K40" t="b">
@@ -2703,7 +2677,7 @@
       <c r="H41">
         <v>57.2</v>
       </c>
-      <c r="J41" s="2">
+      <c r="J41" s="1">
         <v>46246</v>
       </c>
       <c r="K41" t="b">
@@ -2735,7 +2709,7 @@
       <c r="H42">
         <v>59.6</v>
       </c>
-      <c r="J42" s="2">
+      <c r="J42" s="1">
         <v>46487</v>
       </c>
       <c r="K42" t="b">
@@ -2767,7 +2741,7 @@
       <c r="H43">
         <v>75.40000000000001</v>
       </c>
-      <c r="J43" s="2">
+      <c r="J43" s="1">
         <v>46283</v>
       </c>
       <c r="K43" t="b">
@@ -2799,7 +2773,7 @@
       <c r="H44">
         <v>76.8</v>
       </c>
-      <c r="J44" s="2">
+      <c r="J44" s="1">
         <v>46285</v>
       </c>
       <c r="K44" t="b">
@@ -2831,7 +2805,7 @@
       <c r="H45">
         <v>83.2</v>
       </c>
-      <c r="J45" s="2">
+      <c r="J45" s="1">
         <v>46547</v>
       </c>
       <c r="K45" t="b">
@@ -2863,7 +2837,7 @@
       <c r="H46">
         <v>84.5</v>
       </c>
-      <c r="J46" s="2">
+      <c r="J46" s="1">
         <v>46240</v>
       </c>
       <c r="K46" t="b">
@@ -2895,7 +2869,7 @@
       <c r="H47">
         <v>85.8</v>
       </c>
-      <c r="J47" s="2">
+      <c r="J47" s="1">
         <v>46266</v>
       </c>
       <c r="K47" t="b">
@@ -2927,7 +2901,7 @@
       <c r="H48">
         <v>86.5</v>
       </c>
-      <c r="J48" s="2">
+      <c r="J48" s="1">
         <v>46241</v>
       </c>
       <c r="K48" t="b">
@@ -2959,7 +2933,7 @@
       <c r="H49">
         <v>91.7</v>
       </c>
-      <c r="J49" s="2">
+      <c r="J49" s="1">
         <v>46243</v>
       </c>
       <c r="K49" t="b">
@@ -2991,7 +2965,7 @@
       <c r="H50">
         <v>91.7</v>
       </c>
-      <c r="J50" s="2">
+      <c r="J50" s="1">
         <v>46243</v>
       </c>
       <c r="K50" t="b">
@@ -3023,7 +2997,7 @@
       <c r="H51">
         <v>91.7</v>
       </c>
-      <c r="J51" s="2">
+      <c r="J51" s="1">
         <v>46250</v>
       </c>
       <c r="K51" t="b">
@@ -3055,7 +3029,7 @@
       <c r="H52">
         <v>98.90000000000001</v>
       </c>
-      <c r="J52" s="2">
+      <c r="J52" s="1">
         <v>46253</v>
       </c>
       <c r="K52" t="b">
@@ -3087,7 +3061,7 @@
       <c r="H53">
         <v>105.5</v>
       </c>
-      <c r="J53" s="2">
+      <c r="J53" s="1">
         <v>46280</v>
       </c>
       <c r="K53" t="b">
@@ -3119,7 +3093,7 @@
       <c r="H54">
         <v>105.6</v>
       </c>
-      <c r="J54" s="2">
+      <c r="J54" s="1">
         <v>46361</v>
       </c>
       <c r="K54" t="b">
@@ -3151,7 +3125,7 @@
       <c r="H55">
         <v>105.7</v>
       </c>
-      <c r="J55" s="2">
+      <c r="J55" s="1">
         <v>46362</v>
       </c>
       <c r="K55" t="b">
@@ -3183,7 +3157,7 @@
       <c r="H56">
         <v>110.7</v>
       </c>
-      <c r="J56" s="2">
+      <c r="J56" s="1">
         <v>46275</v>
       </c>
       <c r="K56" t="b">
@@ -3215,7 +3189,7 @@
       <c r="H57">
         <v>113.2</v>
       </c>
-      <c r="J57" s="2">
+      <c r="J57" s="1">
         <v>46377</v>
       </c>
       <c r="K57" t="b">
@@ -3247,7 +3221,7 @@
       <c r="H58">
         <v>128.8</v>
       </c>
-      <c r="J58" s="2">
+      <c r="J58" s="1">
         <v>46434</v>
       </c>
       <c r="K58" t="b">
@@ -3279,7 +3253,7 @@
       <c r="H59">
         <v>128.8</v>
       </c>
-      <c r="J59" s="2">
+      <c r="J59" s="1">
         <v>46434</v>
       </c>
       <c r="K59" t="b">
@@ -3311,7 +3285,7 @@
       <c r="H60">
         <v>128.8</v>
       </c>
-      <c r="J60" s="2">
+      <c r="J60" s="1">
         <v>46434</v>
       </c>
       <c r="K60" t="b">
@@ -3343,7 +3317,7 @@
       <c r="H61">
         <v>128.8</v>
       </c>
-      <c r="J61" s="2">
+      <c r="J61" s="1">
         <v>46434</v>
       </c>
       <c r="K61" t="b">
@@ -3375,7 +3349,7 @@
       <c r="H62">
         <v>128.8</v>
       </c>
-      <c r="J62" s="2">
+      <c r="J62" s="1">
         <v>46434</v>
       </c>
       <c r="K62" t="b">
@@ -3407,7 +3381,7 @@
       <c r="H63">
         <v>135</v>
       </c>
-      <c r="J63" s="2">
+      <c r="J63" s="1">
         <v>46280</v>
       </c>
       <c r="K63" t="b">
@@ -3439,7 +3413,7 @@
       <c r="H64">
         <v>150.6</v>
       </c>
-      <c r="J64" s="2">
+      <c r="J64" s="1">
         <v>46271</v>
       </c>
       <c r="K64" t="b">
@@ -3471,7 +3445,7 @@
       <c r="H65">
         <v>174.2</v>
       </c>
-      <c r="J65" s="2">
+      <c r="J65" s="1">
         <v>46363</v>
       </c>
       <c r="K65" t="b">
@@ -3503,7 +3477,7 @@
       <c r="H66">
         <v>176.6</v>
       </c>
-      <c r="J66" s="2">
+      <c r="J66" s="1">
         <v>46334</v>
       </c>
       <c r="K66" t="b">
@@ -3535,7 +3509,7 @@
       <c r="H67">
         <v>177.4</v>
       </c>
-      <c r="J67" s="2">
+      <c r="J67" s="1">
         <v>46407</v>
       </c>
       <c r="K67" t="b">
@@ -3567,7 +3541,7 @@
       <c r="H68">
         <v>183.9</v>
       </c>
-      <c r="J68" s="2">
+      <c r="J68" s="1">
         <v>46341</v>
       </c>
       <c r="K68" t="b">
@@ -3599,7 +3573,7 @@
       <c r="H69">
         <v>191.7</v>
       </c>
-      <c r="J69" s="2">
+      <c r="J69" s="1">
         <v>46300</v>
       </c>
       <c r="K69" t="b">
@@ -3631,7 +3605,7 @@
       <c r="H70">
         <v>200</v>
       </c>
-      <c r="J70" s="2">
+      <c r="J70" s="1">
         <v>46336</v>
       </c>
       <c r="K70" t="b">
@@ -3663,7 +3637,7 @@
       <c r="H71">
         <v>201.1</v>
       </c>
-      <c r="J71" s="2">
+      <c r="J71" s="1">
         <v>46319</v>
       </c>
       <c r="K71" t="b">
@@ -3695,7 +3669,7 @@
       <c r="H72">
         <v>206.5</v>
       </c>
-      <c r="J72" s="2">
+      <c r="J72" s="1">
         <v>46308</v>
       </c>
       <c r="K72" t="b">
@@ -3727,7 +3701,7 @@
       <c r="H73">
         <v>207.5</v>
       </c>
-      <c r="J73" s="2">
+      <c r="J73" s="1">
         <v>46390</v>
       </c>
       <c r="K73" t="b">
@@ -3759,7 +3733,7 @@
       <c r="H74">
         <v>247</v>
       </c>
-      <c r="J74" s="2">
+      <c r="J74" s="1">
         <v>46443</v>
       </c>
       <c r="K74" t="b">
@@ -3791,7 +3765,7 @@
       <c r="H75">
         <v>285.3</v>
       </c>
-      <c r="J75" s="2">
+      <c r="J75" s="1">
         <v>46304</v>
       </c>
       <c r="K75" t="b">
@@ -3823,7 +3797,7 @@
       <c r="H76">
         <v>290.8</v>
       </c>
-      <c r="J76" s="2">
+      <c r="J76" s="1">
         <v>46362</v>
       </c>
       <c r="K76" t="b">
@@ -3855,7 +3829,7 @@
       <c r="H77">
         <v>295.2</v>
       </c>
-      <c r="J77" s="2">
+      <c r="J77" s="1">
         <v>46463</v>
       </c>
       <c r="K77" t="b">
@@ -3887,7 +3861,7 @@
       <c r="H78">
         <v>300.2</v>
       </c>
-      <c r="J78" s="2">
+      <c r="J78" s="1">
         <v>46466</v>
       </c>
       <c r="K78" t="b">
@@ -3922,7 +3896,7 @@
       <c r="I79" t="s">
         <v>313</v>
       </c>
-      <c r="J79" s="2">
+      <c r="J79" s="1">
         <v>36557</v>
       </c>
       <c r="K79" t="b">
@@ -3957,7 +3931,7 @@
       <c r="I80" t="s">
         <v>314</v>
       </c>
-      <c r="J80" s="2">
+      <c r="J80" s="1">
         <v>41275</v>
       </c>
       <c r="K80" t="b">
@@ -3992,7 +3966,7 @@
       <c r="I81" t="s">
         <v>315</v>
       </c>
-      <c r="J81" s="2">
+      <c r="J81" s="1">
         <v>45380</v>
       </c>
       <c r="K81" t="b">
@@ -4027,7 +4001,7 @@
       <c r="I82" t="s">
         <v>316</v>
       </c>
-      <c r="J82" s="2">
+      <c r="J82" s="1">
         <v>45421</v>
       </c>
       <c r="K82" t="b">
@@ -4062,7 +4036,7 @@
       <c r="I83" t="s">
         <v>316</v>
       </c>
-      <c r="J83" s="2">
+      <c r="J83" s="1">
         <v>45428</v>
       </c>
       <c r="K83" t="b">
@@ -4097,7 +4071,7 @@
       <c r="I84" t="s">
         <v>317</v>
       </c>
-      <c r="J84" s="2">
+      <c r="J84" s="1">
         <v>45490</v>
       </c>
       <c r="K84" t="b">
@@ -4132,7 +4106,7 @@
       <c r="I85" t="s">
         <v>318</v>
       </c>
-      <c r="J85" s="2">
+      <c r="J85" s="1">
         <v>45566</v>
       </c>
       <c r="K85" t="b">
@@ -4167,7 +4141,7 @@
       <c r="I86" t="s">
         <v>319</v>
       </c>
-      <c r="J86" s="2">
+      <c r="J86" s="1">
         <v>45986</v>
       </c>
       <c r="K86" t="b">
@@ -4202,7 +4176,7 @@
       <c r="I87" t="s">
         <v>320</v>
       </c>
-      <c r="J87" s="2">
+      <c r="J87" s="1">
         <v>46106</v>
       </c>
       <c r="K87" t="b">
@@ -4237,7 +4211,7 @@
       <c r="I88" t="s">
         <v>321</v>
       </c>
-      <c r="J88" s="2">
+      <c r="J88" s="1">
         <v>46142</v>
       </c>
       <c r="K88" t="b">
@@ -4272,7 +4246,7 @@
       <c r="I89" t="s">
         <v>322</v>
       </c>
-      <c r="J89" s="2">
+      <c r="J89" s="1">
         <v>46274</v>
       </c>
       <c r="K89" t="b">
@@ -4307,7 +4281,7 @@
       <c r="I90" t="s">
         <v>322</v>
       </c>
-      <c r="J90" s="2">
+      <c r="J90" s="1">
         <v>46276</v>
       </c>
       <c r="K90" t="b">
@@ -4342,7 +4316,7 @@
       <c r="I91" t="s">
         <v>322</v>
       </c>
-      <c r="J91" s="2">
+      <c r="J91" s="1">
         <v>46284</v>
       </c>
       <c r="K91" t="b">
@@ -4377,7 +4351,7 @@
       <c r="I92" t="s">
         <v>323</v>
       </c>
-      <c r="J92" s="2">
+      <c r="J92" s="1">
         <v>46317</v>
       </c>
       <c r="K92" t="b">
@@ -4412,7 +4386,7 @@
       <c r="I93" t="s">
         <v>323</v>
       </c>
-      <c r="J93" s="2">
+      <c r="J93" s="1">
         <v>46319</v>
       </c>
       <c r="K93" t="b">
@@ -4447,7 +4421,7 @@
       <c r="I94" t="s">
         <v>324</v>
       </c>
-      <c r="J94" s="2">
+      <c r="J94" s="1">
         <v>46333</v>
       </c>
       <c r="K94" t="b">
@@ -4482,7 +4456,7 @@
       <c r="I95" t="s">
         <v>324</v>
       </c>
-      <c r="J95" s="2">
+      <c r="J95" s="1">
         <v>46338</v>
       </c>
       <c r="K95" t="b">
@@ -4517,7 +4491,7 @@
       <c r="I96" t="s">
         <v>324</v>
       </c>
-      <c r="J96" s="2">
+      <c r="J96" s="1">
         <v>46338</v>
       </c>
       <c r="K96" t="b">
@@ -4552,7 +4526,7 @@
       <c r="I97" t="s">
         <v>324</v>
       </c>
-      <c r="J97" s="2">
+      <c r="J97" s="1">
         <v>46341</v>
       </c>
       <c r="K97" t="b">
@@ -4587,7 +4561,7 @@
       <c r="I98" t="s">
         <v>324</v>
       </c>
-      <c r="J98" s="2">
+      <c r="J98" s="1">
         <v>46344</v>
       </c>
       <c r="K98" t="b">
@@ -4622,7 +4596,7 @@
       <c r="I99" t="s">
         <v>324</v>
       </c>
-      <c r="J99" s="2">
+      <c r="J99" s="1">
         <v>46354</v>
       </c>
       <c r="K99" t="b">
@@ -4657,7 +4631,7 @@
       <c r="I100" t="s">
         <v>324</v>
       </c>
-      <c r="J100" s="2">
+      <c r="J100" s="1">
         <v>46360</v>
       </c>
       <c r="K100" t="b">
@@ -4692,7 +4666,7 @@
       <c r="I101" t="s">
         <v>324</v>
       </c>
-      <c r="J101" s="2">
+      <c r="J101" s="1">
         <v>46360</v>
       </c>
       <c r="K101" t="b">
@@ -4727,7 +4701,7 @@
       <c r="I102" t="s">
         <v>325</v>
       </c>
-      <c r="J102" s="2">
+      <c r="J102" s="1">
         <v>46366</v>
       </c>
       <c r="K102" t="b">
@@ -4762,7 +4736,7 @@
       <c r="I103" t="s">
         <v>325</v>
       </c>
-      <c r="J103" s="2">
+      <c r="J103" s="1">
         <v>46375</v>
       </c>
       <c r="K103" t="b">
@@ -4797,7 +4771,7 @@
       <c r="I104" t="s">
         <v>325</v>
       </c>
-      <c r="J104" s="2">
+      <c r="J104" s="1">
         <v>46388</v>
       </c>
       <c r="K104" t="b">
@@ -4832,7 +4806,7 @@
       <c r="I105" t="s">
         <v>326</v>
       </c>
-      <c r="J105" s="2">
+      <c r="J105" s="1">
         <v>46401</v>
       </c>
       <c r="K105" t="b">
@@ -4867,7 +4841,7 @@
       <c r="I106" t="s">
         <v>326</v>
       </c>
-      <c r="J106" s="2">
+      <c r="J106" s="1">
         <v>46401</v>
       </c>
       <c r="K106" t="b">
@@ -4902,7 +4876,7 @@
       <c r="I107" t="s">
         <v>326</v>
       </c>
-      <c r="J107" s="2">
+      <c r="J107" s="1">
         <v>46401</v>
       </c>
       <c r="K107" t="b">
@@ -4937,7 +4911,7 @@
       <c r="I108" t="s">
         <v>326</v>
       </c>
-      <c r="J108" s="2">
+      <c r="J108" s="1">
         <v>46413</v>
       </c>
       <c r="K108" t="b">
@@ -4972,7 +4946,7 @@
       <c r="I109" t="s">
         <v>327</v>
       </c>
-      <c r="J109" s="2">
+      <c r="J109" s="1">
         <v>46424</v>
       </c>
       <c r="K109" t="b">
@@ -5007,7 +4981,7 @@
       <c r="I110" t="s">
         <v>327</v>
       </c>
-      <c r="J110" s="2">
+      <c r="J110" s="1">
         <v>46427</v>
       </c>
       <c r="K110" t="b">
@@ -5042,7 +5016,7 @@
       <c r="I111" t="s">
         <v>327</v>
       </c>
-      <c r="J111" s="2">
+      <c r="J111" s="1">
         <v>46437</v>
       </c>
       <c r="K111" t="b">
@@ -5077,7 +5051,7 @@
       <c r="I112" t="s">
         <v>327</v>
       </c>
-      <c r="J112" s="2">
+      <c r="J112" s="1">
         <v>46451</v>
       </c>
       <c r="K112" t="b">
@@ -5112,7 +5086,7 @@
       <c r="I113" t="s">
         <v>328</v>
       </c>
-      <c r="J113" s="2">
+      <c r="J113" s="1">
         <v>46455</v>
       </c>
       <c r="K113" t="b">
@@ -5147,7 +5121,7 @@
       <c r="I114" t="s">
         <v>328</v>
       </c>
-      <c r="J114" s="2">
+      <c r="J114" s="1">
         <v>46457</v>
       </c>
       <c r="K114" t="b">
@@ -5182,7 +5156,7 @@
       <c r="I115" t="s">
         <v>328</v>
       </c>
-      <c r="J115" s="2">
+      <c r="J115" s="1">
         <v>46462</v>
       </c>
       <c r="K115" t="b">
@@ -5217,7 +5191,7 @@
       <c r="I116" t="s">
         <v>328</v>
       </c>
-      <c r="J116" s="2">
+      <c r="J116" s="1">
         <v>46464</v>
       </c>
       <c r="K116" t="b">
@@ -5252,7 +5226,7 @@
       <c r="I117" t="s">
         <v>328</v>
       </c>
-      <c r="J117" s="2">
+      <c r="J117" s="1">
         <v>46470</v>
       </c>
       <c r="K117" t="b">
@@ -5287,7 +5261,7 @@
       <c r="I118" t="s">
         <v>329</v>
       </c>
-      <c r="J118" s="2">
+      <c r="J118" s="1">
         <v>46485</v>
       </c>
       <c r="K118" t="b">
@@ -5322,7 +5296,7 @@
       <c r="I119" t="s">
         <v>329</v>
       </c>
-      <c r="J119" s="2">
+      <c r="J119" s="1">
         <v>46499</v>
       </c>
       <c r="K119" t="b">
@@ -5357,7 +5331,7 @@
       <c r="I120" t="s">
         <v>329</v>
       </c>
-      <c r="J120" s="2">
+      <c r="J120" s="1">
         <v>46504</v>
       </c>
       <c r="K120" t="b">
@@ -5392,7 +5366,7 @@
       <c r="I121" t="s">
         <v>329</v>
       </c>
-      <c r="J121" s="2">
+      <c r="J121" s="1">
         <v>46504</v>
       </c>
       <c r="K121" t="b">
@@ -5427,7 +5401,7 @@
       <c r="I122" t="s">
         <v>329</v>
       </c>
-      <c r="J122" s="2">
+      <c r="J122" s="1">
         <v>46507</v>
       </c>
       <c r="K122" t="b">
@@ -5462,7 +5436,7 @@
       <c r="I123" t="s">
         <v>329</v>
       </c>
-      <c r="J123" s="2">
+      <c r="J123" s="1">
         <v>46508</v>
       </c>
       <c r="K123" t="b">
@@ -5497,7 +5471,7 @@
       <c r="I124" t="s">
         <v>329</v>
       </c>
-      <c r="J124" s="2">
+      <c r="J124" s="1">
         <v>46512</v>
       </c>
       <c r="K124" t="b">
@@ -5532,7 +5506,7 @@
       <c r="I125" t="s">
         <v>329</v>
       </c>
-      <c r="J125" s="2">
+      <c r="J125" s="1">
         <v>46512</v>
       </c>
       <c r="K125" t="b">
@@ -5567,7 +5541,7 @@
       <c r="I126" t="s">
         <v>330</v>
       </c>
-      <c r="J126" s="2">
+      <c r="J126" s="1">
         <v>46528</v>
       </c>
       <c r="K126" t="b">
@@ -5602,7 +5576,7 @@
       <c r="I127" t="s">
         <v>330</v>
       </c>
-      <c r="J127" s="2">
+      <c r="J127" s="1">
         <v>46529</v>
       </c>
       <c r="K127" t="b">
@@ -5637,7 +5611,7 @@
       <c r="I128" t="s">
         <v>330</v>
       </c>
-      <c r="J128" s="2">
+      <c r="J128" s="1">
         <v>46537</v>
       </c>
       <c r="K128" t="b">
@@ -5672,7 +5646,7 @@
       <c r="I129" t="s">
         <v>331</v>
       </c>
-      <c r="J129" s="2">
+      <c r="J129" s="1">
         <v>46546</v>
       </c>
       <c r="K129" t="b">
@@ -5707,7 +5681,7 @@
       <c r="I130" t="s">
         <v>331</v>
       </c>
-      <c r="J130" s="2">
+      <c r="J130" s="1">
         <v>46547</v>
       </c>
       <c r="K130" t="b">
@@ -5742,7 +5716,7 @@
       <c r="I131" t="s">
         <v>331</v>
       </c>
-      <c r="J131" s="2">
+      <c r="J131" s="1">
         <v>46547</v>
       </c>
       <c r="K131" t="b">
@@ -5777,7 +5751,7 @@
       <c r="I132" t="s">
         <v>331</v>
       </c>
-      <c r="J132" s="2">
+      <c r="J132" s="1">
         <v>46547</v>
       </c>
       <c r="K132" t="b">
@@ -5812,7 +5786,7 @@
       <c r="I133" t="s">
         <v>331</v>
       </c>
-      <c r="J133" s="2">
+      <c r="J133" s="1">
         <v>46551</v>
       </c>
       <c r="K133" t="b">
@@ -5847,7 +5821,7 @@
       <c r="I134" t="s">
         <v>331</v>
       </c>
-      <c r="J134" s="2">
+      <c r="J134" s="1">
         <v>46560</v>
       </c>
       <c r="K134" t="b">
@@ -5882,7 +5856,7 @@
       <c r="I135" t="s">
         <v>331</v>
       </c>
-      <c r="J135" s="2">
+      <c r="J135" s="1">
         <v>46564</v>
       </c>
       <c r="K135" t="b">
@@ -5917,7 +5891,7 @@
       <c r="I136" t="s">
         <v>331</v>
       </c>
-      <c r="J136" s="2">
+      <c r="J136" s="1">
         <v>46567</v>
       </c>
       <c r="K136" t="b">
@@ -5952,7 +5926,7 @@
       <c r="I137" t="s">
         <v>331</v>
       </c>
-      <c r="J137" s="2">
+      <c r="J137" s="1">
         <v>46568</v>
       </c>
       <c r="K137" t="b">
@@ -5987,7 +5961,7 @@
       <c r="I138" t="s">
         <v>331</v>
       </c>
-      <c r="J138" s="2">
+      <c r="J138" s="1">
         <v>46571</v>
       </c>
       <c r="K138" t="b">
@@ -6022,7 +5996,7 @@
       <c r="I139" t="s">
         <v>332</v>
       </c>
-      <c r="J139" s="2">
+      <c r="J139" s="1">
         <v>46197</v>
       </c>
       <c r="K139" t="b">
@@ -6057,7 +6031,7 @@
       <c r="I140" t="s">
         <v>333</v>
       </c>
-      <c r="J140" s="2">
+      <c r="J140" s="1">
         <v>46212</v>
       </c>
       <c r="K140" t="b">
@@ -6092,7 +6066,7 @@
       <c r="I141" t="s">
         <v>334</v>
       </c>
-      <c r="J141" s="2">
+      <c r="J141" s="1">
         <v>46225</v>
       </c>
       <c r="K141" t="b">
@@ -6127,7 +6101,7 @@
       <c r="I142" t="s">
         <v>335</v>
       </c>
-      <c r="J142" s="2">
+      <c r="J142" s="1">
         <v>46234</v>
       </c>
       <c r="K142" t="b">
@@ -6162,7 +6136,7 @@
       <c r="I143" t="s">
         <v>336</v>
       </c>
-      <c r="J143" s="2">
+      <c r="J143" s="1">
         <v>46234</v>
       </c>
       <c r="K143" t="b">
@@ -6197,7 +6171,7 @@
       <c r="I144" t="s">
         <v>337</v>
       </c>
-      <c r="J144" s="2">
+      <c r="J144" s="1">
         <v>46263</v>
       </c>
       <c r="K144" t="b">
@@ -6232,7 +6206,7 @@
       <c r="I145" t="s">
         <v>338</v>
       </c>
-      <c r="J145" s="2">
+      <c r="J145" s="1">
         <v>46266</v>
       </c>
       <c r="K145" t="b">
@@ -6264,7 +6238,7 @@
       <c r="H146">
         <v>-1476</v>
       </c>
-      <c r="J146" s="2">
+      <c r="J146" s="1">
         <v>43773</v>
       </c>
       <c r="K146" t="b">
@@ -6296,7 +6270,7 @@
       <c r="H147">
         <v>-1469</v>
       </c>
-      <c r="J147" s="2">
+      <c r="J147" s="1">
         <v>43773</v>
       </c>
       <c r="K147" t="b">
@@ -6328,7 +6302,7 @@
       <c r="H148">
         <v>-1121</v>
       </c>
-      <c r="J148" s="2">
+      <c r="J148" s="1">
         <v>45295</v>
       </c>
       <c r="K148" t="b">
@@ -6360,7 +6334,7 @@
       <c r="H149">
         <v>-1018</v>
       </c>
-      <c r="J149" s="2">
+      <c r="J149" s="1">
         <v>45617</v>
       </c>
       <c r="K149" t="b">
@@ -6392,7 +6366,7 @@
       <c r="H150">
         <v>-950</v>
       </c>
-      <c r="J150" s="2">
+      <c r="J150" s="1">
         <v>45677</v>
       </c>
       <c r="K150" t="b">
@@ -6424,7 +6398,7 @@
       <c r="H151">
         <v>-943</v>
       </c>
-      <c r="J151" s="2">
+      <c r="J151" s="1">
         <v>44944</v>
       </c>
       <c r="K151" t="b">
@@ -6456,7 +6430,7 @@
       <c r="H152">
         <v>-252</v>
       </c>
-      <c r="J152" s="2">
+      <c r="J152" s="1">
         <v>46092</v>
       </c>
       <c r="K152" t="b">
@@ -6488,7 +6462,7 @@
       <c r="H153">
         <v>-196</v>
       </c>
-      <c r="J153" s="2">
+      <c r="J153" s="1">
         <v>45988</v>
       </c>
       <c r="K153" t="b">
@@ -6520,7 +6494,7 @@
       <c r="H154">
         <v>-196</v>
       </c>
-      <c r="J154" s="2">
+      <c r="J154" s="1">
         <v>45988</v>
       </c>
       <c r="K154" t="b">
@@ -6552,7 +6526,7 @@
       <c r="H155">
         <v>-47</v>
       </c>
-      <c r="J155" s="2">
+      <c r="J155" s="1">
         <v>46176</v>
       </c>
       <c r="K155" t="b">
@@ -6584,7 +6558,7 @@
       <c r="H156">
         <v>-47</v>
       </c>
-      <c r="J156" s="2">
+      <c r="J156" s="1">
         <v>46176</v>
       </c>
       <c r="K156" t="b">
@@ -6616,7 +6590,7 @@
       <c r="H157">
         <v>-33</v>
       </c>
-      <c r="J157" s="2">
+      <c r="J157" s="1">
         <v>46199</v>
       </c>
       <c r="K157" t="b">
@@ -6648,7 +6622,7 @@
       <c r="H158">
         <v>-33</v>
       </c>
-      <c r="J158" s="2">
+      <c r="J158" s="1">
         <v>46199</v>
       </c>
       <c r="K158" t="b">
@@ -6680,7 +6654,7 @@
       <c r="H159">
         <v>-6</v>
       </c>
-      <c r="J159" s="2">
+      <c r="J159" s="1">
         <v>45967</v>
       </c>
       <c r="K159" t="b">
@@ -6712,7 +6686,7 @@
       <c r="H160">
         <v>43</v>
       </c>
-      <c r="J160" s="2">
+      <c r="J160" s="1">
         <v>46440</v>
       </c>
       <c r="K160" t="b">
@@ -6744,7 +6718,7 @@
       <c r="H161">
         <v>43</v>
       </c>
-      <c r="J161" s="2">
+      <c r="J161" s="1">
         <v>46440</v>
       </c>
       <c r="K161" t="b">
@@ -6776,7 +6750,7 @@
       <c r="H162">
         <v>73</v>
       </c>
-      <c r="J162" s="2">
+      <c r="J162" s="1">
         <v>46264</v>
       </c>
       <c r="K162" t="b">
@@ -6808,7 +6782,7 @@
       <c r="H163">
         <v>73</v>
       </c>
-      <c r="J163" s="2">
+      <c r="J163" s="1">
         <v>46264</v>
       </c>
       <c r="K163" t="b">
@@ -6840,7 +6814,7 @@
       <c r="H164">
         <v>102</v>
       </c>
-      <c r="J164" s="2">
+      <c r="J164" s="1">
         <v>46463</v>
       </c>
       <c r="K164" t="b">
@@ -6872,7 +6846,7 @@
       <c r="H165">
         <v>118</v>
       </c>
-      <c r="J165" s="2">
+      <c r="J165" s="1">
         <v>46337</v>
       </c>
       <c r="K165" t="b">
@@ -6904,7 +6878,7 @@
       <c r="H166">
         <v>146</v>
       </c>
-      <c r="J166" s="2">
+      <c r="J166" s="1">
         <v>46451</v>
       </c>
       <c r="K166" t="b">
@@ -6936,7 +6910,7 @@
       <c r="H167">
         <v>152</v>
       </c>
-      <c r="J167" s="2">
+      <c r="J167" s="1">
         <v>46245</v>
       </c>
       <c r="K167" t="b">
@@ -6968,7 +6942,7 @@
       <c r="H168">
         <v>152</v>
       </c>
-      <c r="J168" s="2">
+      <c r="J168" s="1">
         <v>46245</v>
       </c>
       <c r="K168" t="b">
@@ -7000,7 +6974,7 @@
       <c r="H169">
         <v>163</v>
       </c>
-      <c r="J169" s="2">
+      <c r="J169" s="1">
         <v>46324</v>
       </c>
       <c r="K169" t="b">
@@ -7032,7 +7006,7 @@
       <c r="H170">
         <v>163</v>
       </c>
-      <c r="J170" s="2">
+      <c r="J170" s="1">
         <v>46324</v>
       </c>
       <c r="K170" t="b">
@@ -7064,7 +7038,7 @@
       <c r="H171">
         <v>164</v>
       </c>
-      <c r="J171" s="2">
+      <c r="J171" s="1">
         <v>46426</v>
       </c>
       <c r="K171" t="b">
@@ -7096,7 +7070,7 @@
       <c r="H172">
         <v>175</v>
       </c>
-      <c r="J172" s="2">
+      <c r="J172" s="1">
         <v>46383</v>
       </c>
       <c r="K172" t="b">
@@ -7128,7 +7102,7 @@
       <c r="H173">
         <v>186</v>
       </c>
-      <c r="J173" s="2">
+      <c r="J173" s="1">
         <v>46392</v>
       </c>
       <c r="K173" t="b">
@@ -7160,7 +7134,7 @@
       <c r="H174">
         <v>205</v>
       </c>
-      <c r="J174" s="2">
+      <c r="J174" s="1">
         <v>46390</v>
       </c>
       <c r="K174" t="b">
@@ -7192,7 +7166,7 @@
       <c r="H175">
         <v>207</v>
       </c>
-      <c r="J175" s="2">
+      <c r="J175" s="1">
         <v>46392</v>
       </c>
       <c r="K175" t="b">
@@ -7224,7 +7198,7 @@
       <c r="H176">
         <v>218</v>
       </c>
-      <c r="J176" s="2">
+      <c r="J176" s="1">
         <v>46506</v>
       </c>
       <c r="K176" t="b">
@@ -7256,7 +7230,7 @@
       <c r="H177">
         <v>246</v>
       </c>
-      <c r="J177" s="2">
+      <c r="J177" s="1">
         <v>46478</v>
       </c>
       <c r="K177" t="b">
@@ -7288,7 +7262,7 @@
       <c r="H178">
         <v>248</v>
       </c>
-      <c r="J178" s="2">
+      <c r="J178" s="1">
         <v>46500</v>
       </c>
       <c r="K178" t="b">
@@ -7320,7 +7294,7 @@
       <c r="H179">
         <v>276</v>
       </c>
-      <c r="J179" s="2">
+      <c r="J179" s="1">
         <v>46430</v>
       </c>
       <c r="K179" t="b">
@@ -7352,7 +7326,7 @@
       <c r="H180">
         <v>276</v>
       </c>
-      <c r="J180" s="2">
+      <c r="J180" s="1">
         <v>46430</v>
       </c>
       <c r="K180" t="b">
@@ -7384,7 +7358,7 @@
       <c r="H181">
         <v>290</v>
       </c>
-      <c r="J181" s="2">
+      <c r="J181" s="1">
         <v>46467</v>
       </c>
       <c r="K181" t="b">
@@ -7416,7 +7390,7 @@
       <c r="H182">
         <v>317</v>
       </c>
-      <c r="J182" s="2">
+      <c r="J182" s="1">
         <v>46529</v>
       </c>
       <c r="K182" t="b">
@@ -7448,7 +7422,7 @@
       <c r="H183">
         <v>420</v>
       </c>
-      <c r="J183" s="2">
+      <c r="J183" s="1">
         <v>46566</v>
       </c>
       <c r="K183" t="b">
@@ -7480,7 +7454,7 @@
       <c r="H184">
         <v>426</v>
       </c>
-      <c r="J184" s="2">
+      <c r="J184" s="1">
         <v>46571</v>
       </c>
       <c r="K184" t="b">
@@ -7512,7 +7486,7 @@
       <c r="H185">
         <v>721</v>
       </c>
-      <c r="J185" s="2">
+      <c r="J185" s="1">
         <v>46325</v>
       </c>
       <c r="K185" t="b">
@@ -7544,7 +7518,7 @@
       <c r="H186">
         <v>721</v>
       </c>
-      <c r="J186" s="2">
+      <c r="J186" s="1">
         <v>46325</v>
       </c>
       <c r="K186" t="b">
@@ -7576,7 +7550,7 @@
       <c r="H187">
         <v>850</v>
       </c>
-      <c r="J187" s="2">
+      <c r="J187" s="1">
         <v>46345</v>
       </c>
       <c r="K187" t="b">
@@ -7608,7 +7582,7 @@
       <c r="H188">
         <v>850</v>
       </c>
-      <c r="J188" s="2">
+      <c r="J188" s="1">
         <v>46345</v>
       </c>
       <c r="K188" t="b">
@@ -7640,7 +7614,7 @@
       <c r="H189">
         <v>1661</v>
       </c>
-      <c r="J189" s="2">
+      <c r="J189" s="1">
         <v>46498</v>
       </c>
       <c r="K189" t="b">
@@ -7672,7 +7646,7 @@
       <c r="H190">
         <v>1661</v>
       </c>
-      <c r="J190" s="2">
+      <c r="J190" s="1">
         <v>46498</v>
       </c>
       <c r="K190" t="b">
@@ -7704,7 +7678,7 @@
       <c r="H191">
         <v>488</v>
       </c>
-      <c r="J191" s="2">
+      <c r="J191" s="1">
         <v>46190</v>
       </c>
       <c r="K191" t="b">
@@ -7736,7 +7710,7 @@
       <c r="H192">
         <v>25565</v>
       </c>
-      <c r="J192" s="2">
+      <c r="J192" s="1">
         <v>46190</v>
       </c>
       <c r="K192" t="b">
@@ -7768,7 +7742,7 @@
       <c r="H193">
         <v>25567</v>
       </c>
-      <c r="J193" s="2">
+      <c r="J193" s="1">
         <v>46190</v>
       </c>
       <c r="K193" t="b">
@@ -7800,7 +7774,7 @@
       <c r="H194">
         <v>31293</v>
       </c>
-      <c r="J194" s="2">
+      <c r="J194" s="1">
         <v>46190</v>
       </c>
       <c r="K194" t="b">

</xml_diff>

<commit_message>
Atualiza Vencimentos — TMOT (193 itens) e Operadores (780 itens, 9 operadores)
TMOT: mesmas 7 inconsistências de formato de sempre (DISPONIBILIDADE em texto/data não padrão), sem dado novo na fonte desde 06/08.
Operadores: reprocessado com os mesmos arquivos locais de cada base (DACTA II, PAMA-LS, BAMN, BANT, BABR, BABE, BACO, BACG, CLA) — 3 inconsistências de formato conhecidas.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
@@ -1019,8 +1019,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1036,7 +1044,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1044,12 +1052,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1349,37 +1375,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1408,7 +1434,7 @@
       <c r="H2">
         <v>-4300.3</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>39285</v>
       </c>
       <c r="K2" t="b">
@@ -1440,7 +1466,7 @@
       <c r="H3">
         <v>-2354.2</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>40669</v>
       </c>
       <c r="K3" t="b">
@@ -1472,7 +1498,7 @@
       <c r="H4">
         <v>-910.7</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>40669</v>
       </c>
       <c r="K4" t="b">
@@ -1504,7 +1530,7 @@
       <c r="H5">
         <v>-868</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>44884</v>
       </c>
       <c r="K5" t="b">
@@ -1536,7 +1562,7 @@
       <c r="H6">
         <v>-483.8</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>43855</v>
       </c>
       <c r="K6" t="b">
@@ -1568,7 +1594,7 @@
       <c r="H7">
         <v>-417</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>46014</v>
       </c>
       <c r="K7" t="b">
@@ -1600,7 +1626,7 @@
       <c r="H8">
         <v>-414.2</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>46014</v>
       </c>
       <c r="K8" t="b">
@@ -1632,7 +1658,7 @@
       <c r="H9">
         <v>-391.8</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>42769</v>
       </c>
       <c r="K9" t="b">
@@ -1664,7 +1690,7 @@
       <c r="H10">
         <v>-391.6</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>45804</v>
       </c>
       <c r="K10" t="b">
@@ -1696,7 +1722,7 @@
       <c r="H11">
         <v>-391.6</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>45804</v>
       </c>
       <c r="K11" t="b">
@@ -1728,7 +1754,7 @@
       <c r="H12">
         <v>-372.9</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>42821</v>
       </c>
       <c r="K12" t="b">
@@ -1760,7 +1786,7 @@
       <c r="H13">
         <v>-372.9</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>46014</v>
       </c>
       <c r="K13" t="b">
@@ -1792,7 +1818,7 @@
       <c r="H14">
         <v>-372.9</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>46014</v>
       </c>
       <c r="K14" t="b">
@@ -1824,7 +1850,7 @@
       <c r="H15">
         <v>-372.9</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>46014</v>
       </c>
       <c r="K15" t="b">
@@ -1856,7 +1882,7 @@
       <c r="H16">
         <v>-367.8</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="2">
         <v>46017</v>
       </c>
       <c r="K16" t="b">
@@ -1888,7 +1914,7 @@
       <c r="H17">
         <v>-367.8</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="2">
         <v>46017</v>
       </c>
       <c r="K17" t="b">
@@ -1920,7 +1946,7 @@
       <c r="H18">
         <v>-347.2</v>
       </c>
-      <c r="J18" s="1">
+      <c r="J18" s="2">
         <v>40979</v>
       </c>
       <c r="K18" t="b">
@@ -1952,7 +1978,7 @@
       <c r="H19">
         <v>-293.8</v>
       </c>
-      <c r="J19" s="1">
+      <c r="J19" s="2">
         <v>45846</v>
       </c>
       <c r="K19" t="b">
@@ -1984,7 +2010,7 @@
       <c r="H20">
         <v>-206.4</v>
       </c>
-      <c r="J20" s="1">
+      <c r="J20" s="2">
         <v>36669</v>
       </c>
       <c r="K20" t="b">
@@ -2016,7 +2042,7 @@
       <c r="H21">
         <v>-131.6</v>
       </c>
-      <c r="J21" s="1">
+      <c r="J21" s="2">
         <v>46111</v>
       </c>
       <c r="K21" t="b">
@@ -2048,7 +2074,7 @@
       <c r="H22">
         <v>-131.6</v>
       </c>
-      <c r="J22" s="1">
+      <c r="J22" s="2">
         <v>46111</v>
       </c>
       <c r="K22" t="b">
@@ -2080,7 +2106,7 @@
       <c r="H23">
         <v>-131.6</v>
       </c>
-      <c r="J23" s="1">
+      <c r="J23" s="2">
         <v>46111</v>
       </c>
       <c r="K23" t="b">
@@ -2112,7 +2138,7 @@
       <c r="H24">
         <v>-131.6</v>
       </c>
-      <c r="J24" s="1">
+      <c r="J24" s="2">
         <v>46111</v>
       </c>
       <c r="K24" t="b">
@@ -2144,7 +2170,7 @@
       <c r="H25">
         <v>-131.6</v>
       </c>
-      <c r="J25" s="1">
+      <c r="J25" s="2">
         <v>46111</v>
       </c>
       <c r="K25" t="b">
@@ -2176,7 +2202,7 @@
       <c r="H26">
         <v>-98.3</v>
       </c>
-      <c r="J26" s="1">
+      <c r="J26" s="2">
         <v>41204</v>
       </c>
       <c r="K26" t="b">
@@ -2208,7 +2234,7 @@
       <c r="H27">
         <v>-47.2</v>
       </c>
-      <c r="J27" s="1">
+      <c r="J27" s="2">
         <v>44011</v>
       </c>
       <c r="K27" t="b">
@@ -2240,7 +2266,7 @@
       <c r="H28">
         <v>-22.3</v>
       </c>
-      <c r="J28" s="1">
+      <c r="J28" s="2">
         <v>46226</v>
       </c>
       <c r="K28" t="b">
@@ -2272,7 +2298,7 @@
       <c r="H29">
         <v>4.7</v>
       </c>
-      <c r="J29" s="1">
+      <c r="J29" s="2">
         <v>46265</v>
       </c>
       <c r="K29" t="b">
@@ -2304,7 +2330,7 @@
       <c r="H30">
         <v>7.5</v>
       </c>
-      <c r="J30" s="1">
+      <c r="J30" s="2">
         <v>46265</v>
       </c>
       <c r="K30" t="b">
@@ -2336,7 +2362,7 @@
       <c r="H31">
         <v>10</v>
       </c>
-      <c r="J31" s="1">
+      <c r="J31" s="2">
         <v>46265</v>
       </c>
       <c r="K31" t="b">
@@ -2368,7 +2394,7 @@
       <c r="H32">
         <v>12.8</v>
       </c>
-      <c r="J32" s="1">
+      <c r="J32" s="2">
         <v>46265</v>
       </c>
       <c r="K32" t="b">
@@ -2400,7 +2426,7 @@
       <c r="H33">
         <v>14</v>
       </c>
-      <c r="J33" s="1">
+      <c r="J33" s="2">
         <v>46265</v>
       </c>
       <c r="K33" t="b">
@@ -2432,7 +2458,7 @@
       <c r="H34">
         <v>17.8</v>
       </c>
-      <c r="J34" s="1">
+      <c r="J34" s="2">
         <v>46265</v>
       </c>
       <c r="K34" t="b">
@@ -2464,7 +2490,7 @@
       <c r="H35">
         <v>20.4</v>
       </c>
-      <c r="J35" s="1">
+      <c r="J35" s="2">
         <v>46265</v>
       </c>
       <c r="K35" t="b">
@@ -2496,7 +2522,7 @@
       <c r="H36">
         <v>21.2</v>
       </c>
-      <c r="J36" s="1">
+      <c r="J36" s="2">
         <v>46265</v>
       </c>
       <c r="K36" t="b">
@@ -2528,7 +2554,7 @@
       <c r="H37">
         <v>26.2</v>
       </c>
-      <c r="J37" s="1">
+      <c r="J37" s="2">
         <v>46265</v>
       </c>
       <c r="K37" t="b">
@@ -2560,7 +2586,7 @@
       <c r="H38">
         <v>33.6</v>
       </c>
-      <c r="J38" s="1">
+      <c r="J38" s="2">
         <v>46364</v>
       </c>
       <c r="K38" t="b">
@@ -2592,7 +2618,7 @@
       <c r="H39">
         <v>42.2</v>
       </c>
-      <c r="J39" s="1">
+      <c r="J39" s="2">
         <v>46269</v>
       </c>
       <c r="K39" t="b">
@@ -2624,7 +2650,7 @@
       <c r="H40">
         <v>42.8</v>
       </c>
-      <c r="J40" s="1">
+      <c r="J40" s="2">
         <v>46291</v>
       </c>
       <c r="K40" t="b">
@@ -2656,7 +2682,7 @@
       <c r="H41">
         <v>45.7</v>
       </c>
-      <c r="J41" s="1">
+      <c r="J41" s="2">
         <v>46395</v>
       </c>
       <c r="K41" t="b">
@@ -2688,7 +2714,7 @@
       <c r="H42">
         <v>47.2</v>
       </c>
-      <c r="J42" s="1">
+      <c r="J42" s="2">
         <v>46280</v>
       </c>
       <c r="K42" t="b">
@@ -2720,7 +2746,7 @@
       <c r="H43">
         <v>48.7</v>
       </c>
-      <c r="J43" s="1">
+      <c r="J43" s="2">
         <v>46281</v>
       </c>
       <c r="K43" t="b">
@@ -2752,7 +2778,7 @@
       <c r="H44">
         <v>60</v>
       </c>
-      <c r="J44" s="1">
+      <c r="J44" s="2">
         <v>46281</v>
       </c>
       <c r="K44" t="b">
@@ -2784,7 +2810,7 @@
       <c r="H45">
         <v>62.6</v>
       </c>
-      <c r="J45" s="1">
+      <c r="J45" s="2">
         <v>46265</v>
       </c>
       <c r="K45" t="b">
@@ -2816,7 +2842,7 @@
       <c r="H46">
         <v>64.59999999999999</v>
       </c>
-      <c r="J46" s="1">
+      <c r="J46" s="2">
         <v>46265</v>
       </c>
       <c r="K46" t="b">
@@ -2848,7 +2874,7 @@
       <c r="H47">
         <v>67.59999999999999</v>
       </c>
-      <c r="J47" s="1">
+      <c r="J47" s="2">
         <v>46267</v>
       </c>
       <c r="K47" t="b">
@@ -2880,7 +2906,7 @@
       <c r="H48">
         <v>68.3</v>
       </c>
-      <c r="J48" s="1">
+      <c r="J48" s="2">
         <v>46278</v>
       </c>
       <c r="K48" t="b">
@@ -2912,7 +2938,7 @@
       <c r="H49">
         <v>69.2</v>
       </c>
-      <c r="J49" s="1">
+      <c r="J49" s="2">
         <v>46453</v>
       </c>
       <c r="K49" t="b">
@@ -2944,7 +2970,7 @@
       <c r="H50">
         <v>69.8</v>
       </c>
-      <c r="J50" s="1">
+      <c r="J50" s="2">
         <v>46265</v>
       </c>
       <c r="K50" t="b">
@@ -2976,7 +3002,7 @@
       <c r="H51">
         <v>69.8</v>
       </c>
-      <c r="J51" s="1">
+      <c r="J51" s="2">
         <v>46265</v>
       </c>
       <c r="K51" t="b">
@@ -3008,7 +3034,7 @@
       <c r="H52">
         <v>72.2</v>
       </c>
-      <c r="J52" s="1">
+      <c r="J52" s="2">
         <v>46275</v>
       </c>
       <c r="K52" t="b">
@@ -3040,7 +3066,7 @@
       <c r="H53">
         <v>72.2</v>
       </c>
-      <c r="J53" s="1">
+      <c r="J53" s="2">
         <v>46275</v>
       </c>
       <c r="K53" t="b">
@@ -3072,7 +3098,7 @@
       <c r="H54">
         <v>78.09999999999999</v>
       </c>
-      <c r="J54" s="1">
+      <c r="J54" s="2">
         <v>46265</v>
       </c>
       <c r="K54" t="b">
@@ -3104,7 +3130,7 @@
       <c r="H55">
         <v>82.8</v>
       </c>
-      <c r="J55" s="1">
+      <c r="J55" s="2">
         <v>46487</v>
       </c>
       <c r="K55" t="b">
@@ -3136,7 +3162,7 @@
       <c r="H56">
         <v>83.09999999999999</v>
       </c>
-      <c r="J56" s="1">
+      <c r="J56" s="2">
         <v>46285</v>
       </c>
       <c r="K56" t="b">
@@ -3168,7 +3194,7 @@
       <c r="H57">
         <v>84.8</v>
       </c>
-      <c r="J57" s="1">
+      <c r="J57" s="2">
         <v>46492</v>
       </c>
       <c r="K57" t="b">
@@ -3200,7 +3226,7 @@
       <c r="H58">
         <v>104.9</v>
       </c>
-      <c r="J58" s="1">
+      <c r="J58" s="2">
         <v>46297</v>
       </c>
       <c r="K58" t="b">
@@ -3232,7 +3258,7 @@
       <c r="H59">
         <v>107.6</v>
       </c>
-      <c r="J59" s="1">
+      <c r="J59" s="2">
         <v>46283</v>
       </c>
       <c r="K59" t="b">
@@ -3264,7 +3290,7 @@
       <c r="H60">
         <v>111.9</v>
       </c>
-      <c r="J60" s="1">
+      <c r="J60" s="2">
         <v>46300</v>
       </c>
       <c r="K60" t="b">
@@ -3296,7 +3322,7 @@
       <c r="H61">
         <v>111.9</v>
       </c>
-      <c r="J61" s="1">
+      <c r="J61" s="2">
         <v>46300</v>
       </c>
       <c r="K61" t="b">
@@ -3328,7 +3354,7 @@
       <c r="H62">
         <v>111.9</v>
       </c>
-      <c r="J62" s="1">
+      <c r="J62" s="2">
         <v>46300</v>
       </c>
       <c r="K62" t="b">
@@ -3360,7 +3386,7 @@
       <c r="H63">
         <v>111.9</v>
       </c>
-      <c r="J63" s="1">
+      <c r="J63" s="2">
         <v>46300</v>
       </c>
       <c r="K63" t="b">
@@ -3392,7 +3418,7 @@
       <c r="H64">
         <v>111.9</v>
       </c>
-      <c r="J64" s="1">
+      <c r="J64" s="2">
         <v>46300</v>
       </c>
       <c r="K64" t="b">
@@ -3424,7 +3450,7 @@
       <c r="H65">
         <v>128.8</v>
       </c>
-      <c r="J65" s="1">
+      <c r="J65" s="2">
         <v>46308</v>
       </c>
       <c r="K65" t="b">
@@ -3456,7 +3482,7 @@
       <c r="H66">
         <v>131.1</v>
       </c>
-      <c r="J66" s="1">
+      <c r="J66" s="2">
         <v>46336</v>
       </c>
       <c r="K66" t="b">
@@ -3488,7 +3514,7 @@
       <c r="H67">
         <v>138.4</v>
       </c>
-      <c r="J67" s="1">
+      <c r="J67" s="2">
         <v>46343</v>
       </c>
       <c r="K67" t="b">
@@ -3520,7 +3546,7 @@
       <c r="H68">
         <v>141</v>
       </c>
-      <c r="J68" s="1">
+      <c r="J68" s="2">
         <v>46350</v>
       </c>
       <c r="K68" t="b">
@@ -3552,7 +3578,7 @@
       <c r="H69">
         <v>162</v>
       </c>
-      <c r="J69" s="1">
+      <c r="J69" s="2">
         <v>46391</v>
       </c>
       <c r="K69" t="b">
@@ -3584,7 +3610,7 @@
       <c r="H70">
         <v>167.2</v>
       </c>
-      <c r="J70" s="1">
+      <c r="J70" s="2">
         <v>46330</v>
       </c>
       <c r="K70" t="b">
@@ -3616,7 +3642,7 @@
       <c r="H71">
         <v>177.4</v>
       </c>
-      <c r="J71" s="1">
+      <c r="J71" s="2">
         <v>46418</v>
       </c>
       <c r="K71" t="b">
@@ -3648,7 +3674,7 @@
       <c r="H72">
         <v>200</v>
       </c>
-      <c r="J72" s="1">
+      <c r="J72" s="2">
         <v>46356</v>
       </c>
       <c r="K72" t="b">
@@ -3680,7 +3706,7 @@
       <c r="H73">
         <v>203.6</v>
       </c>
-      <c r="J73" s="1">
+      <c r="J73" s="2">
         <v>46436</v>
       </c>
       <c r="K73" t="b">
@@ -3712,7 +3738,7 @@
       <c r="H74">
         <v>221.2</v>
       </c>
-      <c r="J74" s="1">
+      <c r="J74" s="2">
         <v>46426</v>
       </c>
       <c r="K74" t="b">
@@ -3744,7 +3770,7 @@
       <c r="H75">
         <v>240.8</v>
       </c>
-      <c r="J75" s="1">
+      <c r="J75" s="2">
         <v>46450</v>
       </c>
       <c r="K75" t="b">
@@ -3776,7 +3802,7 @@
       <c r="H76">
         <v>245.8</v>
       </c>
-      <c r="J76" s="1">
+      <c r="J76" s="2">
         <v>46452</v>
       </c>
       <c r="K76" t="b">
@@ -3808,7 +3834,7 @@
       <c r="H77">
         <v>263.4</v>
       </c>
-      <c r="J77" s="1">
+      <c r="J77" s="2">
         <v>46322</v>
       </c>
       <c r="K77" t="b">
@@ -3840,7 +3866,7 @@
       <c r="H78">
         <v>275.2</v>
       </c>
-      <c r="J78" s="1">
+      <c r="J78" s="2">
         <v>46433</v>
       </c>
       <c r="K78" t="b">
@@ -3875,7 +3901,7 @@
       <c r="I79" t="s">
         <v>311</v>
       </c>
-      <c r="J79" s="1">
+      <c r="J79" s="2">
         <v>36557</v>
       </c>
       <c r="K79" t="b">
@@ -3910,7 +3936,7 @@
       <c r="I80" t="s">
         <v>312</v>
       </c>
-      <c r="J80" s="1">
+      <c r="J80" s="2">
         <v>41275</v>
       </c>
       <c r="K80" t="b">
@@ -3945,7 +3971,7 @@
       <c r="I81" t="s">
         <v>313</v>
       </c>
-      <c r="J81" s="1">
+      <c r="J81" s="2">
         <v>45380</v>
       </c>
       <c r="K81" t="b">
@@ -3980,7 +4006,7 @@
       <c r="I82" t="s">
         <v>314</v>
       </c>
-      <c r="J82" s="1">
+      <c r="J82" s="2">
         <v>45421</v>
       </c>
       <c r="K82" t="b">
@@ -4015,7 +4041,7 @@
       <c r="I83" t="s">
         <v>314</v>
       </c>
-      <c r="J83" s="1">
+      <c r="J83" s="2">
         <v>45428</v>
       </c>
       <c r="K83" t="b">
@@ -4050,7 +4076,7 @@
       <c r="I84" t="s">
         <v>315</v>
       </c>
-      <c r="J84" s="1">
+      <c r="J84" s="2">
         <v>45490</v>
       </c>
       <c r="K84" t="b">
@@ -4085,7 +4111,7 @@
       <c r="I85" t="s">
         <v>316</v>
       </c>
-      <c r="J85" s="1">
+      <c r="J85" s="2">
         <v>45566</v>
       </c>
       <c r="K85" t="b">
@@ -4120,7 +4146,7 @@
       <c r="I86" t="s">
         <v>317</v>
       </c>
-      <c r="J86" s="1">
+      <c r="J86" s="2">
         <v>45986</v>
       </c>
       <c r="K86" t="b">
@@ -4155,7 +4181,7 @@
       <c r="I87" t="s">
         <v>318</v>
       </c>
-      <c r="J87" s="1">
+      <c r="J87" s="2">
         <v>46284</v>
       </c>
       <c r="K87" t="b">
@@ -4190,7 +4216,7 @@
       <c r="I88" t="s">
         <v>319</v>
       </c>
-      <c r="J88" s="1">
+      <c r="J88" s="2">
         <v>46305</v>
       </c>
       <c r="K88" t="b">
@@ -4225,7 +4251,7 @@
       <c r="I89" t="s">
         <v>319</v>
       </c>
-      <c r="J89" s="1">
+      <c r="J89" s="2">
         <v>46310</v>
       </c>
       <c r="K89" t="b">
@@ -4260,7 +4286,7 @@
       <c r="I90" t="s">
         <v>319</v>
       </c>
-      <c r="J90" s="1">
+      <c r="J90" s="2">
         <v>46317</v>
       </c>
       <c r="K90" t="b">
@@ -4295,7 +4321,7 @@
       <c r="I91" t="s">
         <v>319</v>
       </c>
-      <c r="J91" s="1">
+      <c r="J91" s="2">
         <v>46319</v>
       </c>
       <c r="K91" t="b">
@@ -4330,7 +4356,7 @@
       <c r="I92" t="s">
         <v>320</v>
       </c>
-      <c r="J92" s="1">
+      <c r="J92" s="2">
         <v>46333</v>
       </c>
       <c r="K92" t="b">
@@ -4365,7 +4391,7 @@
       <c r="I93" t="s">
         <v>320</v>
       </c>
-      <c r="J93" s="1">
+      <c r="J93" s="2">
         <v>46338</v>
       </c>
       <c r="K93" t="b">
@@ -4400,7 +4426,7 @@
       <c r="I94" t="s">
         <v>320</v>
       </c>
-      <c r="J94" s="1">
+      <c r="J94" s="2">
         <v>46338</v>
       </c>
       <c r="K94" t="b">
@@ -4435,7 +4461,7 @@
       <c r="I95" t="s">
         <v>320</v>
       </c>
-      <c r="J95" s="1">
+      <c r="J95" s="2">
         <v>46341</v>
       </c>
       <c r="K95" t="b">
@@ -4470,7 +4496,7 @@
       <c r="I96" t="s">
         <v>320</v>
       </c>
-      <c r="J96" s="1">
+      <c r="J96" s="2">
         <v>46344</v>
       </c>
       <c r="K96" t="b">
@@ -4505,7 +4531,7 @@
       <c r="I97" t="s">
         <v>321</v>
       </c>
-      <c r="J97" s="1">
+      <c r="J97" s="2">
         <v>46360</v>
       </c>
       <c r="K97" t="b">
@@ -4540,7 +4566,7 @@
       <c r="I98" t="s">
         <v>321</v>
       </c>
-      <c r="J98" s="1">
+      <c r="J98" s="2">
         <v>46360</v>
       </c>
       <c r="K98" t="b">
@@ -4575,7 +4601,7 @@
       <c r="I99" t="s">
         <v>321</v>
       </c>
-      <c r="J99" s="1">
+      <c r="J99" s="2">
         <v>46367</v>
       </c>
       <c r="K99" t="b">
@@ -4610,7 +4636,7 @@
       <c r="I100" t="s">
         <v>321</v>
       </c>
-      <c r="J100" s="1">
+      <c r="J100" s="2">
         <v>46375</v>
       </c>
       <c r="K100" t="b">
@@ -4645,7 +4671,7 @@
       <c r="I101" t="s">
         <v>321</v>
       </c>
-      <c r="J101" s="1">
+      <c r="J101" s="2">
         <v>46387</v>
       </c>
       <c r="K101" t="b">
@@ -4680,7 +4706,7 @@
       <c r="I102" t="s">
         <v>321</v>
       </c>
-      <c r="J102" s="1">
+      <c r="J102" s="2">
         <v>46387</v>
       </c>
       <c r="K102" t="b">
@@ -4715,7 +4741,7 @@
       <c r="I103" t="s">
         <v>321</v>
       </c>
-      <c r="J103" s="1">
+      <c r="J103" s="2">
         <v>46387</v>
       </c>
       <c r="K103" t="b">
@@ -4750,7 +4776,7 @@
       <c r="I104" t="s">
         <v>321</v>
       </c>
-      <c r="J104" s="1">
+      <c r="J104" s="2">
         <v>46388</v>
       </c>
       <c r="K104" t="b">
@@ -4785,7 +4811,7 @@
       <c r="I105" t="s">
         <v>322</v>
       </c>
-      <c r="J105" s="1">
+      <c r="J105" s="2">
         <v>46401</v>
       </c>
       <c r="K105" t="b">
@@ -4820,7 +4846,7 @@
       <c r="I106" t="s">
         <v>322</v>
       </c>
-      <c r="J106" s="1">
+      <c r="J106" s="2">
         <v>46401</v>
       </c>
       <c r="K106" t="b">
@@ -4855,7 +4881,7 @@
       <c r="I107" t="s">
         <v>322</v>
       </c>
-      <c r="J107" s="1">
+      <c r="J107" s="2">
         <v>46401</v>
       </c>
       <c r="K107" t="b">
@@ -4890,7 +4916,7 @@
       <c r="I108" t="s">
         <v>322</v>
       </c>
-      <c r="J108" s="1">
+      <c r="J108" s="2">
         <v>46412</v>
       </c>
       <c r="K108" t="b">
@@ -4925,7 +4951,7 @@
       <c r="I109" t="s">
         <v>322</v>
       </c>
-      <c r="J109" s="1">
+      <c r="J109" s="2">
         <v>46412</v>
       </c>
       <c r="K109" t="b">
@@ -4960,7 +4986,7 @@
       <c r="I110" t="s">
         <v>322</v>
       </c>
-      <c r="J110" s="1">
+      <c r="J110" s="2">
         <v>46412</v>
       </c>
       <c r="K110" t="b">
@@ -4995,7 +5021,7 @@
       <c r="I111" t="s">
         <v>323</v>
       </c>
-      <c r="J111" s="1">
+      <c r="J111" s="2">
         <v>46424</v>
       </c>
       <c r="K111" t="b">
@@ -5030,7 +5056,7 @@
       <c r="I112" t="s">
         <v>323</v>
       </c>
-      <c r="J112" s="1">
+      <c r="J112" s="2">
         <v>46437</v>
       </c>
       <c r="K112" t="b">
@@ -5065,7 +5091,7 @@
       <c r="I113" t="s">
         <v>323</v>
       </c>
-      <c r="J113" s="1">
+      <c r="J113" s="2">
         <v>46451</v>
       </c>
       <c r="K113" t="b">
@@ -5100,7 +5126,7 @@
       <c r="I114" t="s">
         <v>323</v>
       </c>
-      <c r="J114" s="1">
+      <c r="J114" s="2">
         <v>46451</v>
       </c>
       <c r="K114" t="b">
@@ -5135,7 +5161,7 @@
       <c r="I115" t="s">
         <v>324</v>
       </c>
-      <c r="J115" s="1">
+      <c r="J115" s="2">
         <v>46455</v>
       </c>
       <c r="K115" t="b">
@@ -5170,7 +5196,7 @@
       <c r="I116" t="s">
         <v>324</v>
       </c>
-      <c r="J116" s="1">
+      <c r="J116" s="2">
         <v>46456</v>
       </c>
       <c r="K116" t="b">
@@ -5205,7 +5231,7 @@
       <c r="I117" t="s">
         <v>324</v>
       </c>
-      <c r="J117" s="1">
+      <c r="J117" s="2">
         <v>46457</v>
       </c>
       <c r="K117" t="b">
@@ -5240,7 +5266,7 @@
       <c r="I118" t="s">
         <v>324</v>
       </c>
-      <c r="J118" s="1">
+      <c r="J118" s="2">
         <v>46464</v>
       </c>
       <c r="K118" t="b">
@@ -5275,7 +5301,7 @@
       <c r="I119" t="s">
         <v>324</v>
       </c>
-      <c r="J119" s="1">
+      <c r="J119" s="2">
         <v>46470</v>
       </c>
       <c r="K119" t="b">
@@ -5310,7 +5336,7 @@
       <c r="I120" t="s">
         <v>325</v>
       </c>
-      <c r="J120" s="1">
+      <c r="J120" s="2">
         <v>46485</v>
       </c>
       <c r="K120" t="b">
@@ -5345,7 +5371,7 @@
       <c r="I121" t="s">
         <v>325</v>
       </c>
-      <c r="J121" s="1">
+      <c r="J121" s="2">
         <v>46499</v>
       </c>
       <c r="K121" t="b">
@@ -5380,7 +5406,7 @@
       <c r="I122" t="s">
         <v>325</v>
       </c>
-      <c r="J122" s="1">
+      <c r="J122" s="2">
         <v>46504</v>
       </c>
       <c r="K122" t="b">
@@ -5415,7 +5441,7 @@
       <c r="I123" t="s">
         <v>325</v>
       </c>
-      <c r="J123" s="1">
+      <c r="J123" s="2">
         <v>46504</v>
       </c>
       <c r="K123" t="b">
@@ -5450,7 +5476,7 @@
       <c r="I124" t="s">
         <v>325</v>
       </c>
-      <c r="J124" s="1">
+      <c r="J124" s="2">
         <v>46507</v>
       </c>
       <c r="K124" t="b">
@@ -5485,7 +5511,7 @@
       <c r="I125" t="s">
         <v>325</v>
       </c>
-      <c r="J125" s="1">
+      <c r="J125" s="2">
         <v>46508</v>
       </c>
       <c r="K125" t="b">
@@ -5520,7 +5546,7 @@
       <c r="I126" t="s">
         <v>325</v>
       </c>
-      <c r="J126" s="1">
+      <c r="J126" s="2">
         <v>46512</v>
       </c>
       <c r="K126" t="b">
@@ -5555,7 +5581,7 @@
       <c r="I127" t="s">
         <v>326</v>
       </c>
-      <c r="J127" s="1">
+      <c r="J127" s="2">
         <v>46512</v>
       </c>
       <c r="K127" t="b">
@@ -5590,7 +5616,7 @@
       <c r="I128" t="s">
         <v>326</v>
       </c>
-      <c r="J128" s="1">
+      <c r="J128" s="2">
         <v>46528</v>
       </c>
       <c r="K128" t="b">
@@ -5625,7 +5651,7 @@
       <c r="I129" t="s">
         <v>326</v>
       </c>
-      <c r="J129" s="1">
+      <c r="J129" s="2">
         <v>46529</v>
       </c>
       <c r="K129" t="b">
@@ -5660,7 +5686,7 @@
       <c r="I130" t="s">
         <v>326</v>
       </c>
-      <c r="J130" s="1">
+      <c r="J130" s="2">
         <v>46537</v>
       </c>
       <c r="K130" t="b">
@@ -5695,7 +5721,7 @@
       <c r="I131" t="s">
         <v>327</v>
       </c>
-      <c r="J131" s="1">
+      <c r="J131" s="2">
         <v>46546</v>
       </c>
       <c r="K131" t="b">
@@ -5730,7 +5756,7 @@
       <c r="I132" t="s">
         <v>327</v>
       </c>
-      <c r="J132" s="1">
+      <c r="J132" s="2">
         <v>46547</v>
       </c>
       <c r="K132" t="b">
@@ -5765,7 +5791,7 @@
       <c r="I133" t="s">
         <v>327</v>
       </c>
-      <c r="J133" s="1">
+      <c r="J133" s="2">
         <v>46547</v>
       </c>
       <c r="K133" t="b">
@@ -5800,7 +5826,7 @@
       <c r="I134" t="s">
         <v>327</v>
       </c>
-      <c r="J134" s="1">
+      <c r="J134" s="2">
         <v>46547</v>
       </c>
       <c r="K134" t="b">
@@ -5835,7 +5861,7 @@
       <c r="I135" t="s">
         <v>327</v>
       </c>
-      <c r="J135" s="1">
+      <c r="J135" s="2">
         <v>46551</v>
       </c>
       <c r="K135" t="b">
@@ -5870,7 +5896,7 @@
       <c r="I136" t="s">
         <v>327</v>
       </c>
-      <c r="J136" s="1">
+      <c r="J136" s="2">
         <v>46560</v>
       </c>
       <c r="K136" t="b">
@@ -5905,7 +5931,7 @@
       <c r="I137" t="s">
         <v>327</v>
       </c>
-      <c r="J137" s="1">
+      <c r="J137" s="2">
         <v>46564</v>
       </c>
       <c r="K137" t="b">
@@ -5940,7 +5966,7 @@
       <c r="I138" t="s">
         <v>327</v>
       </c>
-      <c r="J138" s="1">
+      <c r="J138" s="2">
         <v>46567</v>
       </c>
       <c r="K138" t="b">
@@ -5975,7 +6001,7 @@
       <c r="I139" t="s">
         <v>327</v>
       </c>
-      <c r="J139" s="1">
+      <c r="J139" s="2">
         <v>46568</v>
       </c>
       <c r="K139" t="b">
@@ -6010,7 +6036,7 @@
       <c r="I140" t="s">
         <v>328</v>
       </c>
-      <c r="J140" s="1">
+      <c r="J140" s="2">
         <v>46578</v>
       </c>
       <c r="K140" t="b">
@@ -6045,7 +6071,7 @@
       <c r="I141" t="s">
         <v>328</v>
       </c>
-      <c r="J141" s="1">
+      <c r="J141" s="2">
         <v>46592</v>
       </c>
       <c r="K141" t="b">
@@ -6080,7 +6106,7 @@
       <c r="I142" t="s">
         <v>328</v>
       </c>
-      <c r="J142" s="1">
+      <c r="J142" s="2">
         <v>46592</v>
       </c>
       <c r="K142" t="b">
@@ -6115,7 +6141,7 @@
       <c r="I143" t="s">
         <v>329</v>
       </c>
-      <c r="J143" s="1">
+      <c r="J143" s="2">
         <v>46212</v>
       </c>
       <c r="K143" t="b">
@@ -6150,7 +6176,7 @@
       <c r="I144" t="s">
         <v>330</v>
       </c>
-      <c r="J144" s="1">
+      <c r="J144" s="2">
         <v>46225</v>
       </c>
       <c r="K144" t="b">
@@ -6185,7 +6211,7 @@
       <c r="I145" t="s">
         <v>331</v>
       </c>
-      <c r="J145" s="1">
+      <c r="J145" s="2">
         <v>46263</v>
       </c>
       <c r="K145" t="b">
@@ -6217,7 +6243,7 @@
       <c r="H146">
         <v>-1476</v>
       </c>
-      <c r="J146" s="1">
+      <c r="J146" s="2">
         <v>43773</v>
       </c>
       <c r="K146" t="b">
@@ -6249,7 +6275,7 @@
       <c r="H147">
         <v>-1469</v>
       </c>
-      <c r="J147" s="1">
+      <c r="J147" s="2">
         <v>43773</v>
       </c>
       <c r="K147" t="b">
@@ -6281,7 +6307,7 @@
       <c r="H148">
         <v>-1186</v>
       </c>
-      <c r="J148" s="1">
+      <c r="J148" s="2">
         <v>45295</v>
       </c>
       <c r="K148" t="b">
@@ -6313,7 +6339,7 @@
       <c r="H149">
         <v>-1048</v>
       </c>
-      <c r="J149" s="1">
+      <c r="J149" s="2">
         <v>45617</v>
       </c>
       <c r="K149" t="b">
@@ -6345,7 +6371,7 @@
       <c r="H150">
         <v>-980</v>
       </c>
-      <c r="J150" s="1">
+      <c r="J150" s="2">
         <v>45677</v>
       </c>
       <c r="K150" t="b">
@@ -6377,7 +6403,7 @@
       <c r="H151">
         <v>-961</v>
       </c>
-      <c r="J151" s="1">
+      <c r="J151" s="2">
         <v>44944</v>
       </c>
       <c r="K151" t="b">
@@ -6409,7 +6435,7 @@
       <c r="H152">
         <v>-252</v>
       </c>
-      <c r="J152" s="1">
+      <c r="J152" s="2">
         <v>46092</v>
       </c>
       <c r="K152" t="b">
@@ -6441,7 +6467,7 @@
       <c r="H153">
         <v>3</v>
       </c>
-      <c r="J153" s="1">
+      <c r="J153" s="2">
         <v>46265</v>
       </c>
       <c r="K153" t="b">
@@ -6473,7 +6499,7 @@
       <c r="H154">
         <v>3</v>
       </c>
-      <c r="J154" s="1">
+      <c r="J154" s="2">
         <v>46265</v>
       </c>
       <c r="K154" t="b">
@@ -6505,7 +6531,7 @@
       <c r="H155">
         <v>43</v>
       </c>
-      <c r="J155" s="1">
+      <c r="J155" s="2">
         <v>46440</v>
       </c>
       <c r="K155" t="b">
@@ -6537,7 +6563,7 @@
       <c r="H156">
         <v>43</v>
       </c>
-      <c r="J156" s="1">
+      <c r="J156" s="2">
         <v>46440</v>
       </c>
       <c r="K156" t="b">
@@ -6569,7 +6595,7 @@
       <c r="H157">
         <v>72</v>
       </c>
-      <c r="J157" s="1">
+      <c r="J157" s="2">
         <v>46289</v>
       </c>
       <c r="K157" t="b">
@@ -6601,7 +6627,7 @@
       <c r="H158">
         <v>72</v>
       </c>
-      <c r="J158" s="1">
+      <c r="J158" s="2">
         <v>46289</v>
       </c>
       <c r="K158" t="b">
@@ -6633,7 +6659,7 @@
       <c r="H159">
         <v>81</v>
       </c>
-      <c r="J159" s="1">
+      <c r="J159" s="2">
         <v>46405</v>
       </c>
       <c r="K159" t="b">
@@ -6665,7 +6691,7 @@
       <c r="H160">
         <v>102</v>
       </c>
-      <c r="J160" s="1">
+      <c r="J160" s="2">
         <v>46463</v>
       </c>
       <c r="K160" t="b">
@@ -6697,7 +6723,7 @@
       <c r="H161">
         <v>109</v>
       </c>
-      <c r="J161" s="1">
+      <c r="J161" s="2">
         <v>46353</v>
       </c>
       <c r="K161" t="b">
@@ -6729,7 +6755,7 @@
       <c r="H162">
         <v>127</v>
       </c>
-      <c r="J162" s="1">
+      <c r="J162" s="2">
         <v>46417</v>
       </c>
       <c r="K162" t="b">
@@ -6761,7 +6787,7 @@
       <c r="H163">
         <v>152</v>
       </c>
-      <c r="J163" s="1">
+      <c r="J163" s="2">
         <v>46271</v>
       </c>
       <c r="K163" t="b">
@@ -6793,7 +6819,7 @@
       <c r="H164">
         <v>152</v>
       </c>
-      <c r="J164" s="1">
+      <c r="J164" s="2">
         <v>46271</v>
       </c>
       <c r="K164" t="b">
@@ -6825,7 +6851,7 @@
       <c r="H165">
         <v>153</v>
       </c>
-      <c r="J165" s="1">
+      <c r="J165" s="2">
         <v>46458</v>
       </c>
       <c r="K165" t="b">
@@ -6857,7 +6883,7 @@
       <c r="H166">
         <v>158</v>
       </c>
-      <c r="J166" s="1">
+      <c r="J166" s="2">
         <v>46381</v>
       </c>
       <c r="K166" t="b">
@@ -6889,7 +6915,7 @@
       <c r="H167">
         <v>163</v>
       </c>
-      <c r="J167" s="1">
+      <c r="J167" s="2">
         <v>46592</v>
       </c>
       <c r="K167" t="b">
@@ -6921,7 +6947,7 @@
       <c r="H168">
         <v>167</v>
       </c>
-      <c r="J168" s="1">
+      <c r="J168" s="2">
         <v>46441</v>
       </c>
       <c r="K168" t="b">
@@ -6953,7 +6979,7 @@
       <c r="H169">
         <v>169</v>
       </c>
-      <c r="J169" s="1">
+      <c r="J169" s="2">
         <v>46391</v>
       </c>
       <c r="K169" t="b">
@@ -6985,7 +7011,7 @@
       <c r="H170">
         <v>184</v>
       </c>
-      <c r="J170" s="1">
+      <c r="J170" s="2">
         <v>46385</v>
       </c>
       <c r="K170" t="b">
@@ -7017,7 +7043,7 @@
       <c r="H171">
         <v>186</v>
       </c>
-      <c r="J171" s="1">
+      <c r="J171" s="2">
         <v>46387</v>
       </c>
       <c r="K171" t="b">
@@ -7049,7 +7075,7 @@
       <c r="H172">
         <v>206</v>
       </c>
-      <c r="J172" s="1">
+      <c r="J172" s="2">
         <v>46399</v>
       </c>
       <c r="K172" t="b">
@@ -7081,7 +7107,7 @@
       <c r="H173">
         <v>206</v>
       </c>
-      <c r="J173" s="1">
+      <c r="J173" s="2">
         <v>46399</v>
       </c>
       <c r="K173" t="b">
@@ -7113,7 +7139,7 @@
       <c r="H174">
         <v>234</v>
       </c>
-      <c r="J174" s="1">
+      <c r="J174" s="2">
         <v>46458</v>
       </c>
       <c r="K174" t="b">
@@ -7145,7 +7171,7 @@
       <c r="H175">
         <v>248</v>
       </c>
-      <c r="J175" s="1">
+      <c r="J175" s="2">
         <v>46528</v>
       </c>
       <c r="K175" t="b">
@@ -7177,7 +7203,7 @@
       <c r="H176">
         <v>317</v>
       </c>
-      <c r="J176" s="1">
+      <c r="J176" s="2">
         <v>46540</v>
       </c>
       <c r="K176" t="b">
@@ -7209,7 +7235,7 @@
       <c r="H177">
         <v>340</v>
       </c>
-      <c r="J177" s="1">
+      <c r="J177" s="2">
         <v>46547</v>
       </c>
       <c r="K177" t="b">
@@ -7241,7 +7267,7 @@
       <c r="H178">
         <v>364</v>
       </c>
-      <c r="J178" s="1">
+      <c r="J178" s="2">
         <v>46557</v>
       </c>
       <c r="K178" t="b">
@@ -7273,7 +7299,7 @@
       <c r="H179">
         <v>368</v>
       </c>
-      <c r="J179" s="1">
+      <c r="J179" s="2">
         <v>46571</v>
       </c>
       <c r="K179" t="b">
@@ -7305,7 +7331,7 @@
       <c r="H180">
         <v>368</v>
       </c>
-      <c r="J180" s="1">
+      <c r="J180" s="2">
         <v>46571</v>
       </c>
       <c r="K180" t="b">
@@ -7337,7 +7363,7 @@
       <c r="H181">
         <v>370</v>
       </c>
-      <c r="J181" s="1">
+      <c r="J181" s="2">
         <v>46562</v>
       </c>
       <c r="K181" t="b">
@@ -7369,7 +7395,7 @@
       <c r="H182">
         <v>385</v>
       </c>
-      <c r="J182" s="1">
+      <c r="J182" s="2">
         <v>46574</v>
       </c>
       <c r="K182" t="b">
@@ -7401,7 +7427,7 @@
       <c r="H183">
         <v>385</v>
       </c>
-      <c r="J183" s="1">
+      <c r="J183" s="2">
         <v>46574</v>
       </c>
       <c r="K183" t="b">
@@ -7433,7 +7459,7 @@
       <c r="H184">
         <v>417</v>
       </c>
-      <c r="J184" s="1">
+      <c r="J184" s="2">
         <v>46578</v>
       </c>
       <c r="K184" t="b">
@@ -7465,7 +7491,7 @@
       <c r="H185">
         <v>721</v>
       </c>
-      <c r="J185" s="1">
+      <c r="J185" s="2">
         <v>46345</v>
       </c>
       <c r="K185" t="b">
@@ -7497,7 +7523,7 @@
       <c r="H186">
         <v>721</v>
       </c>
-      <c r="J186" s="1">
+      <c r="J186" s="2">
         <v>46345</v>
       </c>
       <c r="K186" t="b">
@@ -7529,7 +7555,7 @@
       <c r="H187">
         <v>850</v>
       </c>
-      <c r="J187" s="1">
+      <c r="J187" s="2">
         <v>46366</v>
       </c>
       <c r="K187" t="b">
@@ -7561,7 +7587,7 @@
       <c r="H188">
         <v>850</v>
       </c>
-      <c r="J188" s="1">
+      <c r="J188" s="2">
         <v>46366</v>
       </c>
       <c r="K188" t="b">
@@ -7593,7 +7619,7 @@
       <c r="H189">
         <v>1661</v>
       </c>
-      <c r="J189" s="1">
+      <c r="J189" s="2">
         <v>46524</v>
       </c>
       <c r="K189" t="b">
@@ -7625,7 +7651,7 @@
       <c r="H190">
         <v>1661</v>
       </c>
-      <c r="J190" s="1">
+      <c r="J190" s="2">
         <v>46524</v>
       </c>
       <c r="K190" t="b">
@@ -7657,7 +7683,7 @@
       <c r="H191">
         <v>488</v>
       </c>
-      <c r="J191" s="1">
+      <c r="J191" s="2">
         <v>46190</v>
       </c>
       <c r="K191" t="b">
@@ -7689,7 +7715,7 @@
       <c r="H192">
         <v>25565</v>
       </c>
-      <c r="J192" s="1">
+      <c r="J192" s="2">
         <v>46190</v>
       </c>
       <c r="K192" t="b">
@@ -7721,7 +7747,7 @@
       <c r="H193">
         <v>25567</v>
       </c>
-      <c r="J193" s="1">
+      <c r="J193" s="2">
         <v>46190</v>
       </c>
       <c r="K193" t="b">
@@ -7753,7 +7779,7 @@
       <c r="H194">
         <v>31293</v>
       </c>
-      <c r="J194" s="1">
+      <c r="J194" s="2">
         <v>46190</v>
       </c>
       <c r="K194" t="b">

</xml_diff>

<commit_message>
Atualização automática: vencimentos_tmot (12/08/2026 11:23)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
@@ -1019,16 +1019,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1044,7 +1036,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1052,30 +1044,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1375,37 +1349,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1434,7 +1408,7 @@
       <c r="H2">
         <v>-4300.3</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>39285</v>
       </c>
       <c r="K2" t="b">
@@ -1466,7 +1440,7 @@
       <c r="H3">
         <v>-2354.2</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>40669</v>
       </c>
       <c r="K3" t="b">
@@ -1498,7 +1472,7 @@
       <c r="H4">
         <v>-910.7</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>40669</v>
       </c>
       <c r="K4" t="b">
@@ -1530,7 +1504,7 @@
       <c r="H5">
         <v>-868</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>44884</v>
       </c>
       <c r="K5" t="b">
@@ -1562,7 +1536,7 @@
       <c r="H6">
         <v>-483.8</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>43855</v>
       </c>
       <c r="K6" t="b">
@@ -1594,7 +1568,7 @@
       <c r="H7">
         <v>-417</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>46014</v>
       </c>
       <c r="K7" t="b">
@@ -1626,7 +1600,7 @@
       <c r="H8">
         <v>-414.2</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>46014</v>
       </c>
       <c r="K8" t="b">
@@ -1658,7 +1632,7 @@
       <c r="H9">
         <v>-391.8</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>42769</v>
       </c>
       <c r="K9" t="b">
@@ -1690,7 +1664,7 @@
       <c r="H10">
         <v>-391.6</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>45804</v>
       </c>
       <c r="K10" t="b">
@@ -1722,7 +1696,7 @@
       <c r="H11">
         <v>-391.6</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>45804</v>
       </c>
       <c r="K11" t="b">
@@ -1754,7 +1728,7 @@
       <c r="H12">
         <v>-372.9</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>42821</v>
       </c>
       <c r="K12" t="b">
@@ -1786,7 +1760,7 @@
       <c r="H13">
         <v>-372.9</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>46014</v>
       </c>
       <c r="K13" t="b">
@@ -1818,7 +1792,7 @@
       <c r="H14">
         <v>-372.9</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>46014</v>
       </c>
       <c r="K14" t="b">
@@ -1850,7 +1824,7 @@
       <c r="H15">
         <v>-372.9</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <v>46014</v>
       </c>
       <c r="K15" t="b">
@@ -1882,7 +1856,7 @@
       <c r="H16">
         <v>-367.8</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <v>46017</v>
       </c>
       <c r="K16" t="b">
@@ -1914,7 +1888,7 @@
       <c r="H17">
         <v>-367.8</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="1">
         <v>46017</v>
       </c>
       <c r="K17" t="b">
@@ -1946,7 +1920,7 @@
       <c r="H18">
         <v>-347.2</v>
       </c>
-      <c r="J18" s="2">
+      <c r="J18" s="1">
         <v>40979</v>
       </c>
       <c r="K18" t="b">
@@ -1978,7 +1952,7 @@
       <c r="H19">
         <v>-293.8</v>
       </c>
-      <c r="J19" s="2">
+      <c r="J19" s="1">
         <v>45846</v>
       </c>
       <c r="K19" t="b">
@@ -2010,7 +1984,7 @@
       <c r="H20">
         <v>-206.4</v>
       </c>
-      <c r="J20" s="2">
+      <c r="J20" s="1">
         <v>36669</v>
       </c>
       <c r="K20" t="b">
@@ -2042,7 +2016,7 @@
       <c r="H21">
         <v>-131.6</v>
       </c>
-      <c r="J21" s="2">
+      <c r="J21" s="1">
         <v>46111</v>
       </c>
       <c r="K21" t="b">
@@ -2074,7 +2048,7 @@
       <c r="H22">
         <v>-131.6</v>
       </c>
-      <c r="J22" s="2">
+      <c r="J22" s="1">
         <v>46111</v>
       </c>
       <c r="K22" t="b">
@@ -2106,7 +2080,7 @@
       <c r="H23">
         <v>-131.6</v>
       </c>
-      <c r="J23" s="2">
+      <c r="J23" s="1">
         <v>46111</v>
       </c>
       <c r="K23" t="b">
@@ -2138,7 +2112,7 @@
       <c r="H24">
         <v>-131.6</v>
       </c>
-      <c r="J24" s="2">
+      <c r="J24" s="1">
         <v>46111</v>
       </c>
       <c r="K24" t="b">
@@ -2170,7 +2144,7 @@
       <c r="H25">
         <v>-131.6</v>
       </c>
-      <c r="J25" s="2">
+      <c r="J25" s="1">
         <v>46111</v>
       </c>
       <c r="K25" t="b">
@@ -2202,7 +2176,7 @@
       <c r="H26">
         <v>-98.3</v>
       </c>
-      <c r="J26" s="2">
+      <c r="J26" s="1">
         <v>41204</v>
       </c>
       <c r="K26" t="b">
@@ -2234,7 +2208,7 @@
       <c r="H27">
         <v>-47.2</v>
       </c>
-      <c r="J27" s="2">
+      <c r="J27" s="1">
         <v>44011</v>
       </c>
       <c r="K27" t="b">
@@ -2266,7 +2240,7 @@
       <c r="H28">
         <v>-22.3</v>
       </c>
-      <c r="J28" s="2">
+      <c r="J28" s="1">
         <v>46226</v>
       </c>
       <c r="K28" t="b">
@@ -2298,7 +2272,7 @@
       <c r="H29">
         <v>4.7</v>
       </c>
-      <c r="J29" s="2">
+      <c r="J29" s="1">
         <v>46265</v>
       </c>
       <c r="K29" t="b">
@@ -2330,7 +2304,7 @@
       <c r="H30">
         <v>7.5</v>
       </c>
-      <c r="J30" s="2">
+      <c r="J30" s="1">
         <v>46265</v>
       </c>
       <c r="K30" t="b">
@@ -2362,7 +2336,7 @@
       <c r="H31">
         <v>10</v>
       </c>
-      <c r="J31" s="2">
+      <c r="J31" s="1">
         <v>46265</v>
       </c>
       <c r="K31" t="b">
@@ -2394,7 +2368,7 @@
       <c r="H32">
         <v>12.8</v>
       </c>
-      <c r="J32" s="2">
+      <c r="J32" s="1">
         <v>46265</v>
       </c>
       <c r="K32" t="b">
@@ -2426,7 +2400,7 @@
       <c r="H33">
         <v>14</v>
       </c>
-      <c r="J33" s="2">
+      <c r="J33" s="1">
         <v>46265</v>
       </c>
       <c r="K33" t="b">
@@ -2458,7 +2432,7 @@
       <c r="H34">
         <v>17.8</v>
       </c>
-      <c r="J34" s="2">
+      <c r="J34" s="1">
         <v>46265</v>
       </c>
       <c r="K34" t="b">
@@ -2490,7 +2464,7 @@
       <c r="H35">
         <v>20.4</v>
       </c>
-      <c r="J35" s="2">
+      <c r="J35" s="1">
         <v>46265</v>
       </c>
       <c r="K35" t="b">
@@ -2522,7 +2496,7 @@
       <c r="H36">
         <v>21.2</v>
       </c>
-      <c r="J36" s="2">
+      <c r="J36" s="1">
         <v>46265</v>
       </c>
       <c r="K36" t="b">
@@ -2554,7 +2528,7 @@
       <c r="H37">
         <v>26.2</v>
       </c>
-      <c r="J37" s="2">
+      <c r="J37" s="1">
         <v>46265</v>
       </c>
       <c r="K37" t="b">
@@ -2586,7 +2560,7 @@
       <c r="H38">
         <v>33.6</v>
       </c>
-      <c r="J38" s="2">
+      <c r="J38" s="1">
         <v>46364</v>
       </c>
       <c r="K38" t="b">
@@ -2618,7 +2592,7 @@
       <c r="H39">
         <v>42.2</v>
       </c>
-      <c r="J39" s="2">
+      <c r="J39" s="1">
         <v>46269</v>
       </c>
       <c r="K39" t="b">
@@ -2650,7 +2624,7 @@
       <c r="H40">
         <v>42.8</v>
       </c>
-      <c r="J40" s="2">
+      <c r="J40" s="1">
         <v>46291</v>
       </c>
       <c r="K40" t="b">
@@ -2682,7 +2656,7 @@
       <c r="H41">
         <v>45.7</v>
       </c>
-      <c r="J41" s="2">
+      <c r="J41" s="1">
         <v>46395</v>
       </c>
       <c r="K41" t="b">
@@ -2714,7 +2688,7 @@
       <c r="H42">
         <v>47.2</v>
       </c>
-      <c r="J42" s="2">
+      <c r="J42" s="1">
         <v>46280</v>
       </c>
       <c r="K42" t="b">
@@ -2746,7 +2720,7 @@
       <c r="H43">
         <v>48.7</v>
       </c>
-      <c r="J43" s="2">
+      <c r="J43" s="1">
         <v>46281</v>
       </c>
       <c r="K43" t="b">
@@ -2778,7 +2752,7 @@
       <c r="H44">
         <v>60</v>
       </c>
-      <c r="J44" s="2">
+      <c r="J44" s="1">
         <v>46281</v>
       </c>
       <c r="K44" t="b">
@@ -2810,7 +2784,7 @@
       <c r="H45">
         <v>62.6</v>
       </c>
-      <c r="J45" s="2">
+      <c r="J45" s="1">
         <v>46265</v>
       </c>
       <c r="K45" t="b">
@@ -2842,7 +2816,7 @@
       <c r="H46">
         <v>64.59999999999999</v>
       </c>
-      <c r="J46" s="2">
+      <c r="J46" s="1">
         <v>46265</v>
       </c>
       <c r="K46" t="b">
@@ -2874,7 +2848,7 @@
       <c r="H47">
         <v>67.59999999999999</v>
       </c>
-      <c r="J47" s="2">
+      <c r="J47" s="1">
         <v>46267</v>
       </c>
       <c r="K47" t="b">
@@ -2906,7 +2880,7 @@
       <c r="H48">
         <v>68.3</v>
       </c>
-      <c r="J48" s="2">
+      <c r="J48" s="1">
         <v>46278</v>
       </c>
       <c r="K48" t="b">
@@ -2938,7 +2912,7 @@
       <c r="H49">
         <v>69.2</v>
       </c>
-      <c r="J49" s="2">
+      <c r="J49" s="1">
         <v>46453</v>
       </c>
       <c r="K49" t="b">
@@ -2970,7 +2944,7 @@
       <c r="H50">
         <v>69.8</v>
       </c>
-      <c r="J50" s="2">
+      <c r="J50" s="1">
         <v>46265</v>
       </c>
       <c r="K50" t="b">
@@ -3002,7 +2976,7 @@
       <c r="H51">
         <v>69.8</v>
       </c>
-      <c r="J51" s="2">
+      <c r="J51" s="1">
         <v>46265</v>
       </c>
       <c r="K51" t="b">
@@ -3034,7 +3008,7 @@
       <c r="H52">
         <v>72.2</v>
       </c>
-      <c r="J52" s="2">
+      <c r="J52" s="1">
         <v>46275</v>
       </c>
       <c r="K52" t="b">
@@ -3066,7 +3040,7 @@
       <c r="H53">
         <v>72.2</v>
       </c>
-      <c r="J53" s="2">
+      <c r="J53" s="1">
         <v>46275</v>
       </c>
       <c r="K53" t="b">
@@ -3098,7 +3072,7 @@
       <c r="H54">
         <v>78.09999999999999</v>
       </c>
-      <c r="J54" s="2">
+      <c r="J54" s="1">
         <v>46265</v>
       </c>
       <c r="K54" t="b">
@@ -3130,7 +3104,7 @@
       <c r="H55">
         <v>82.8</v>
       </c>
-      <c r="J55" s="2">
+      <c r="J55" s="1">
         <v>46487</v>
       </c>
       <c r="K55" t="b">
@@ -3162,7 +3136,7 @@
       <c r="H56">
         <v>83.09999999999999</v>
       </c>
-      <c r="J56" s="2">
+      <c r="J56" s="1">
         <v>46285</v>
       </c>
       <c r="K56" t="b">
@@ -3194,7 +3168,7 @@
       <c r="H57">
         <v>84.8</v>
       </c>
-      <c r="J57" s="2">
+      <c r="J57" s="1">
         <v>46492</v>
       </c>
       <c r="K57" t="b">
@@ -3226,7 +3200,7 @@
       <c r="H58">
         <v>104.9</v>
       </c>
-      <c r="J58" s="2">
+      <c r="J58" s="1">
         <v>46297</v>
       </c>
       <c r="K58" t="b">
@@ -3258,7 +3232,7 @@
       <c r="H59">
         <v>107.6</v>
       </c>
-      <c r="J59" s="2">
+      <c r="J59" s="1">
         <v>46283</v>
       </c>
       <c r="K59" t="b">
@@ -3290,7 +3264,7 @@
       <c r="H60">
         <v>111.9</v>
       </c>
-      <c r="J60" s="2">
+      <c r="J60" s="1">
         <v>46300</v>
       </c>
       <c r="K60" t="b">
@@ -3322,7 +3296,7 @@
       <c r="H61">
         <v>111.9</v>
       </c>
-      <c r="J61" s="2">
+      <c r="J61" s="1">
         <v>46300</v>
       </c>
       <c r="K61" t="b">
@@ -3354,7 +3328,7 @@
       <c r="H62">
         <v>111.9</v>
       </c>
-      <c r="J62" s="2">
+      <c r="J62" s="1">
         <v>46300</v>
       </c>
       <c r="K62" t="b">
@@ -3386,7 +3360,7 @@
       <c r="H63">
         <v>111.9</v>
       </c>
-      <c r="J63" s="2">
+      <c r="J63" s="1">
         <v>46300</v>
       </c>
       <c r="K63" t="b">
@@ -3418,7 +3392,7 @@
       <c r="H64">
         <v>111.9</v>
       </c>
-      <c r="J64" s="2">
+      <c r="J64" s="1">
         <v>46300</v>
       </c>
       <c r="K64" t="b">
@@ -3450,7 +3424,7 @@
       <c r="H65">
         <v>128.8</v>
       </c>
-      <c r="J65" s="2">
+      <c r="J65" s="1">
         <v>46308</v>
       </c>
       <c r="K65" t="b">
@@ -3482,7 +3456,7 @@
       <c r="H66">
         <v>131.1</v>
       </c>
-      <c r="J66" s="2">
+      <c r="J66" s="1">
         <v>46336</v>
       </c>
       <c r="K66" t="b">
@@ -3514,7 +3488,7 @@
       <c r="H67">
         <v>138.4</v>
       </c>
-      <c r="J67" s="2">
+      <c r="J67" s="1">
         <v>46343</v>
       </c>
       <c r="K67" t="b">
@@ -3546,7 +3520,7 @@
       <c r="H68">
         <v>141</v>
       </c>
-      <c r="J68" s="2">
+      <c r="J68" s="1">
         <v>46350</v>
       </c>
       <c r="K68" t="b">
@@ -3578,7 +3552,7 @@
       <c r="H69">
         <v>162</v>
       </c>
-      <c r="J69" s="2">
+      <c r="J69" s="1">
         <v>46391</v>
       </c>
       <c r="K69" t="b">
@@ -3610,7 +3584,7 @@
       <c r="H70">
         <v>167.2</v>
       </c>
-      <c r="J70" s="2">
+      <c r="J70" s="1">
         <v>46330</v>
       </c>
       <c r="K70" t="b">
@@ -3642,7 +3616,7 @@
       <c r="H71">
         <v>177.4</v>
       </c>
-      <c r="J71" s="2">
+      <c r="J71" s="1">
         <v>46418</v>
       </c>
       <c r="K71" t="b">
@@ -3674,7 +3648,7 @@
       <c r="H72">
         <v>200</v>
       </c>
-      <c r="J72" s="2">
+      <c r="J72" s="1">
         <v>46356</v>
       </c>
       <c r="K72" t="b">
@@ -3706,7 +3680,7 @@
       <c r="H73">
         <v>203.6</v>
       </c>
-      <c r="J73" s="2">
+      <c r="J73" s="1">
         <v>46436</v>
       </c>
       <c r="K73" t="b">
@@ -3738,7 +3712,7 @@
       <c r="H74">
         <v>221.2</v>
       </c>
-      <c r="J74" s="2">
+      <c r="J74" s="1">
         <v>46426</v>
       </c>
       <c r="K74" t="b">
@@ -3770,7 +3744,7 @@
       <c r="H75">
         <v>240.8</v>
       </c>
-      <c r="J75" s="2">
+      <c r="J75" s="1">
         <v>46450</v>
       </c>
       <c r="K75" t="b">
@@ -3802,7 +3776,7 @@
       <c r="H76">
         <v>245.8</v>
       </c>
-      <c r="J76" s="2">
+      <c r="J76" s="1">
         <v>46452</v>
       </c>
       <c r="K76" t="b">
@@ -3834,7 +3808,7 @@
       <c r="H77">
         <v>263.4</v>
       </c>
-      <c r="J77" s="2">
+      <c r="J77" s="1">
         <v>46322</v>
       </c>
       <c r="K77" t="b">
@@ -3866,7 +3840,7 @@
       <c r="H78">
         <v>275.2</v>
       </c>
-      <c r="J78" s="2">
+      <c r="J78" s="1">
         <v>46433</v>
       </c>
       <c r="K78" t="b">
@@ -3901,7 +3875,7 @@
       <c r="I79" t="s">
         <v>311</v>
       </c>
-      <c r="J79" s="2">
+      <c r="J79" s="1">
         <v>36557</v>
       </c>
       <c r="K79" t="b">
@@ -3936,7 +3910,7 @@
       <c r="I80" t="s">
         <v>312</v>
       </c>
-      <c r="J80" s="2">
+      <c r="J80" s="1">
         <v>41275</v>
       </c>
       <c r="K80" t="b">
@@ -3971,7 +3945,7 @@
       <c r="I81" t="s">
         <v>313</v>
       </c>
-      <c r="J81" s="2">
+      <c r="J81" s="1">
         <v>45380</v>
       </c>
       <c r="K81" t="b">
@@ -4006,7 +3980,7 @@
       <c r="I82" t="s">
         <v>314</v>
       </c>
-      <c r="J82" s="2">
+      <c r="J82" s="1">
         <v>45421</v>
       </c>
       <c r="K82" t="b">
@@ -4041,7 +4015,7 @@
       <c r="I83" t="s">
         <v>314</v>
       </c>
-      <c r="J83" s="2">
+      <c r="J83" s="1">
         <v>45428</v>
       </c>
       <c r="K83" t="b">
@@ -4076,7 +4050,7 @@
       <c r="I84" t="s">
         <v>315</v>
       </c>
-      <c r="J84" s="2">
+      <c r="J84" s="1">
         <v>45490</v>
       </c>
       <c r="K84" t="b">
@@ -4111,7 +4085,7 @@
       <c r="I85" t="s">
         <v>316</v>
       </c>
-      <c r="J85" s="2">
+      <c r="J85" s="1">
         <v>45566</v>
       </c>
       <c r="K85" t="b">
@@ -4146,7 +4120,7 @@
       <c r="I86" t="s">
         <v>317</v>
       </c>
-      <c r="J86" s="2">
+      <c r="J86" s="1">
         <v>45986</v>
       </c>
       <c r="K86" t="b">
@@ -4181,7 +4155,7 @@
       <c r="I87" t="s">
         <v>318</v>
       </c>
-      <c r="J87" s="2">
+      <c r="J87" s="1">
         <v>46284</v>
       </c>
       <c r="K87" t="b">
@@ -4216,7 +4190,7 @@
       <c r="I88" t="s">
         <v>319</v>
       </c>
-      <c r="J88" s="2">
+      <c r="J88" s="1">
         <v>46305</v>
       </c>
       <c r="K88" t="b">
@@ -4251,7 +4225,7 @@
       <c r="I89" t="s">
         <v>319</v>
       </c>
-      <c r="J89" s="2">
+      <c r="J89" s="1">
         <v>46310</v>
       </c>
       <c r="K89" t="b">
@@ -4286,7 +4260,7 @@
       <c r="I90" t="s">
         <v>319</v>
       </c>
-      <c r="J90" s="2">
+      <c r="J90" s="1">
         <v>46317</v>
       </c>
       <c r="K90" t="b">
@@ -4321,7 +4295,7 @@
       <c r="I91" t="s">
         <v>319</v>
       </c>
-      <c r="J91" s="2">
+      <c r="J91" s="1">
         <v>46319</v>
       </c>
       <c r="K91" t="b">
@@ -4356,7 +4330,7 @@
       <c r="I92" t="s">
         <v>320</v>
       </c>
-      <c r="J92" s="2">
+      <c r="J92" s="1">
         <v>46333</v>
       </c>
       <c r="K92" t="b">
@@ -4391,7 +4365,7 @@
       <c r="I93" t="s">
         <v>320</v>
       </c>
-      <c r="J93" s="2">
+      <c r="J93" s="1">
         <v>46338</v>
       </c>
       <c r="K93" t="b">
@@ -4426,7 +4400,7 @@
       <c r="I94" t="s">
         <v>320</v>
       </c>
-      <c r="J94" s="2">
+      <c r="J94" s="1">
         <v>46338</v>
       </c>
       <c r="K94" t="b">
@@ -4461,7 +4435,7 @@
       <c r="I95" t="s">
         <v>320</v>
       </c>
-      <c r="J95" s="2">
+      <c r="J95" s="1">
         <v>46341</v>
       </c>
       <c r="K95" t="b">
@@ -4496,7 +4470,7 @@
       <c r="I96" t="s">
         <v>320</v>
       </c>
-      <c r="J96" s="2">
+      <c r="J96" s="1">
         <v>46344</v>
       </c>
       <c r="K96" t="b">
@@ -4531,7 +4505,7 @@
       <c r="I97" t="s">
         <v>321</v>
       </c>
-      <c r="J97" s="2">
+      <c r="J97" s="1">
         <v>46360</v>
       </c>
       <c r="K97" t="b">
@@ -4566,7 +4540,7 @@
       <c r="I98" t="s">
         <v>321</v>
       </c>
-      <c r="J98" s="2">
+      <c r="J98" s="1">
         <v>46360</v>
       </c>
       <c r="K98" t="b">
@@ -4601,7 +4575,7 @@
       <c r="I99" t="s">
         <v>321</v>
       </c>
-      <c r="J99" s="2">
+      <c r="J99" s="1">
         <v>46367</v>
       </c>
       <c r="K99" t="b">
@@ -4636,7 +4610,7 @@
       <c r="I100" t="s">
         <v>321</v>
       </c>
-      <c r="J100" s="2">
+      <c r="J100" s="1">
         <v>46375</v>
       </c>
       <c r="K100" t="b">
@@ -4671,7 +4645,7 @@
       <c r="I101" t="s">
         <v>321</v>
       </c>
-      <c r="J101" s="2">
+      <c r="J101" s="1">
         <v>46387</v>
       </c>
       <c r="K101" t="b">
@@ -4706,7 +4680,7 @@
       <c r="I102" t="s">
         <v>321</v>
       </c>
-      <c r="J102" s="2">
+      <c r="J102" s="1">
         <v>46387</v>
       </c>
       <c r="K102" t="b">
@@ -4741,7 +4715,7 @@
       <c r="I103" t="s">
         <v>321</v>
       </c>
-      <c r="J103" s="2">
+      <c r="J103" s="1">
         <v>46387</v>
       </c>
       <c r="K103" t="b">
@@ -4776,7 +4750,7 @@
       <c r="I104" t="s">
         <v>321</v>
       </c>
-      <c r="J104" s="2">
+      <c r="J104" s="1">
         <v>46388</v>
       </c>
       <c r="K104" t="b">
@@ -4811,7 +4785,7 @@
       <c r="I105" t="s">
         <v>322</v>
       </c>
-      <c r="J105" s="2">
+      <c r="J105" s="1">
         <v>46401</v>
       </c>
       <c r="K105" t="b">
@@ -4846,7 +4820,7 @@
       <c r="I106" t="s">
         <v>322</v>
       </c>
-      <c r="J106" s="2">
+      <c r="J106" s="1">
         <v>46401</v>
       </c>
       <c r="K106" t="b">
@@ -4881,7 +4855,7 @@
       <c r="I107" t="s">
         <v>322</v>
       </c>
-      <c r="J107" s="2">
+      <c r="J107" s="1">
         <v>46401</v>
       </c>
       <c r="K107" t="b">
@@ -4916,7 +4890,7 @@
       <c r="I108" t="s">
         <v>322</v>
       </c>
-      <c r="J108" s="2">
+      <c r="J108" s="1">
         <v>46412</v>
       </c>
       <c r="K108" t="b">
@@ -4951,7 +4925,7 @@
       <c r="I109" t="s">
         <v>322</v>
       </c>
-      <c r="J109" s="2">
+      <c r="J109" s="1">
         <v>46412</v>
       </c>
       <c r="K109" t="b">
@@ -4986,7 +4960,7 @@
       <c r="I110" t="s">
         <v>322</v>
       </c>
-      <c r="J110" s="2">
+      <c r="J110" s="1">
         <v>46412</v>
       </c>
       <c r="K110" t="b">
@@ -5021,7 +4995,7 @@
       <c r="I111" t="s">
         <v>323</v>
       </c>
-      <c r="J111" s="2">
+      <c r="J111" s="1">
         <v>46424</v>
       </c>
       <c r="K111" t="b">
@@ -5056,7 +5030,7 @@
       <c r="I112" t="s">
         <v>323</v>
       </c>
-      <c r="J112" s="2">
+      <c r="J112" s="1">
         <v>46437</v>
       </c>
       <c r="K112" t="b">
@@ -5091,7 +5065,7 @@
       <c r="I113" t="s">
         <v>323</v>
       </c>
-      <c r="J113" s="2">
+      <c r="J113" s="1">
         <v>46451</v>
       </c>
       <c r="K113" t="b">
@@ -5126,7 +5100,7 @@
       <c r="I114" t="s">
         <v>323</v>
       </c>
-      <c r="J114" s="2">
+      <c r="J114" s="1">
         <v>46451</v>
       </c>
       <c r="K114" t="b">
@@ -5161,7 +5135,7 @@
       <c r="I115" t="s">
         <v>324</v>
       </c>
-      <c r="J115" s="2">
+      <c r="J115" s="1">
         <v>46455</v>
       </c>
       <c r="K115" t="b">
@@ -5196,7 +5170,7 @@
       <c r="I116" t="s">
         <v>324</v>
       </c>
-      <c r="J116" s="2">
+      <c r="J116" s="1">
         <v>46456</v>
       </c>
       <c r="K116" t="b">
@@ -5231,7 +5205,7 @@
       <c r="I117" t="s">
         <v>324</v>
       </c>
-      <c r="J117" s="2">
+      <c r="J117" s="1">
         <v>46457</v>
       </c>
       <c r="K117" t="b">
@@ -5266,7 +5240,7 @@
       <c r="I118" t="s">
         <v>324</v>
       </c>
-      <c r="J118" s="2">
+      <c r="J118" s="1">
         <v>46464</v>
       </c>
       <c r="K118" t="b">
@@ -5301,7 +5275,7 @@
       <c r="I119" t="s">
         <v>324</v>
       </c>
-      <c r="J119" s="2">
+      <c r="J119" s="1">
         <v>46470</v>
       </c>
       <c r="K119" t="b">
@@ -5336,7 +5310,7 @@
       <c r="I120" t="s">
         <v>325</v>
       </c>
-      <c r="J120" s="2">
+      <c r="J120" s="1">
         <v>46485</v>
       </c>
       <c r="K120" t="b">
@@ -5371,7 +5345,7 @@
       <c r="I121" t="s">
         <v>325</v>
       </c>
-      <c r="J121" s="2">
+      <c r="J121" s="1">
         <v>46499</v>
       </c>
       <c r="K121" t="b">
@@ -5406,7 +5380,7 @@
       <c r="I122" t="s">
         <v>325</v>
       </c>
-      <c r="J122" s="2">
+      <c r="J122" s="1">
         <v>46504</v>
       </c>
       <c r="K122" t="b">
@@ -5441,7 +5415,7 @@
       <c r="I123" t="s">
         <v>325</v>
       </c>
-      <c r="J123" s="2">
+      <c r="J123" s="1">
         <v>46504</v>
       </c>
       <c r="K123" t="b">
@@ -5476,7 +5450,7 @@
       <c r="I124" t="s">
         <v>325</v>
       </c>
-      <c r="J124" s="2">
+      <c r="J124" s="1">
         <v>46507</v>
       </c>
       <c r="K124" t="b">
@@ -5511,7 +5485,7 @@
       <c r="I125" t="s">
         <v>325</v>
       </c>
-      <c r="J125" s="2">
+      <c r="J125" s="1">
         <v>46508</v>
       </c>
       <c r="K125" t="b">
@@ -5546,7 +5520,7 @@
       <c r="I126" t="s">
         <v>325</v>
       </c>
-      <c r="J126" s="2">
+      <c r="J126" s="1">
         <v>46512</v>
       </c>
       <c r="K126" t="b">
@@ -5581,7 +5555,7 @@
       <c r="I127" t="s">
         <v>326</v>
       </c>
-      <c r="J127" s="2">
+      <c r="J127" s="1">
         <v>46512</v>
       </c>
       <c r="K127" t="b">
@@ -5616,7 +5590,7 @@
       <c r="I128" t="s">
         <v>326</v>
       </c>
-      <c r="J128" s="2">
+      <c r="J128" s="1">
         <v>46528</v>
       </c>
       <c r="K128" t="b">
@@ -5651,7 +5625,7 @@
       <c r="I129" t="s">
         <v>326</v>
       </c>
-      <c r="J129" s="2">
+      <c r="J129" s="1">
         <v>46529</v>
       </c>
       <c r="K129" t="b">
@@ -5686,7 +5660,7 @@
       <c r="I130" t="s">
         <v>326</v>
       </c>
-      <c r="J130" s="2">
+      <c r="J130" s="1">
         <v>46537</v>
       </c>
       <c r="K130" t="b">
@@ -5721,7 +5695,7 @@
       <c r="I131" t="s">
         <v>327</v>
       </c>
-      <c r="J131" s="2">
+      <c r="J131" s="1">
         <v>46546</v>
       </c>
       <c r="K131" t="b">
@@ -5756,7 +5730,7 @@
       <c r="I132" t="s">
         <v>327</v>
       </c>
-      <c r="J132" s="2">
+      <c r="J132" s="1">
         <v>46547</v>
       </c>
       <c r="K132" t="b">
@@ -5791,7 +5765,7 @@
       <c r="I133" t="s">
         <v>327</v>
       </c>
-      <c r="J133" s="2">
+      <c r="J133" s="1">
         <v>46547</v>
       </c>
       <c r="K133" t="b">
@@ -5826,7 +5800,7 @@
       <c r="I134" t="s">
         <v>327</v>
       </c>
-      <c r="J134" s="2">
+      <c r="J134" s="1">
         <v>46547</v>
       </c>
       <c r="K134" t="b">
@@ -5861,7 +5835,7 @@
       <c r="I135" t="s">
         <v>327</v>
       </c>
-      <c r="J135" s="2">
+      <c r="J135" s="1">
         <v>46551</v>
       </c>
       <c r="K135" t="b">
@@ -5896,7 +5870,7 @@
       <c r="I136" t="s">
         <v>327</v>
       </c>
-      <c r="J136" s="2">
+      <c r="J136" s="1">
         <v>46560</v>
       </c>
       <c r="K136" t="b">
@@ -5931,7 +5905,7 @@
       <c r="I137" t="s">
         <v>327</v>
       </c>
-      <c r="J137" s="2">
+      <c r="J137" s="1">
         <v>46564</v>
       </c>
       <c r="K137" t="b">
@@ -5966,7 +5940,7 @@
       <c r="I138" t="s">
         <v>327</v>
       </c>
-      <c r="J138" s="2">
+      <c r="J138" s="1">
         <v>46567</v>
       </c>
       <c r="K138" t="b">
@@ -6001,7 +5975,7 @@
       <c r="I139" t="s">
         <v>327</v>
       </c>
-      <c r="J139" s="2">
+      <c r="J139" s="1">
         <v>46568</v>
       </c>
       <c r="K139" t="b">
@@ -6036,7 +6010,7 @@
       <c r="I140" t="s">
         <v>328</v>
       </c>
-      <c r="J140" s="2">
+      <c r="J140" s="1">
         <v>46578</v>
       </c>
       <c r="K140" t="b">
@@ -6071,7 +6045,7 @@
       <c r="I141" t="s">
         <v>328</v>
       </c>
-      <c r="J141" s="2">
+      <c r="J141" s="1">
         <v>46592</v>
       </c>
       <c r="K141" t="b">
@@ -6106,7 +6080,7 @@
       <c r="I142" t="s">
         <v>328</v>
       </c>
-      <c r="J142" s="2">
+      <c r="J142" s="1">
         <v>46592</v>
       </c>
       <c r="K142" t="b">
@@ -6141,7 +6115,7 @@
       <c r="I143" t="s">
         <v>329</v>
       </c>
-      <c r="J143" s="2">
+      <c r="J143" s="1">
         <v>46212</v>
       </c>
       <c r="K143" t="b">
@@ -6176,7 +6150,7 @@
       <c r="I144" t="s">
         <v>330</v>
       </c>
-      <c r="J144" s="2">
+      <c r="J144" s="1">
         <v>46225</v>
       </c>
       <c r="K144" t="b">
@@ -6211,7 +6185,7 @@
       <c r="I145" t="s">
         <v>331</v>
       </c>
-      <c r="J145" s="2">
+      <c r="J145" s="1">
         <v>46263</v>
       </c>
       <c r="K145" t="b">
@@ -6243,7 +6217,7 @@
       <c r="H146">
         <v>-1476</v>
       </c>
-      <c r="J146" s="2">
+      <c r="J146" s="1">
         <v>43773</v>
       </c>
       <c r="K146" t="b">
@@ -6275,7 +6249,7 @@
       <c r="H147">
         <v>-1469</v>
       </c>
-      <c r="J147" s="2">
+      <c r="J147" s="1">
         <v>43773</v>
       </c>
       <c r="K147" t="b">
@@ -6307,7 +6281,7 @@
       <c r="H148">
         <v>-1186</v>
       </c>
-      <c r="J148" s="2">
+      <c r="J148" s="1">
         <v>45295</v>
       </c>
       <c r="K148" t="b">
@@ -6339,7 +6313,7 @@
       <c r="H149">
         <v>-1048</v>
       </c>
-      <c r="J149" s="2">
+      <c r="J149" s="1">
         <v>45617</v>
       </c>
       <c r="K149" t="b">
@@ -6371,7 +6345,7 @@
       <c r="H150">
         <v>-980</v>
       </c>
-      <c r="J150" s="2">
+      <c r="J150" s="1">
         <v>45677</v>
       </c>
       <c r="K150" t="b">
@@ -6403,7 +6377,7 @@
       <c r="H151">
         <v>-961</v>
       </c>
-      <c r="J151" s="2">
+      <c r="J151" s="1">
         <v>44944</v>
       </c>
       <c r="K151" t="b">
@@ -6435,7 +6409,7 @@
       <c r="H152">
         <v>-252</v>
       </c>
-      <c r="J152" s="2">
+      <c r="J152" s="1">
         <v>46092</v>
       </c>
       <c r="K152" t="b">
@@ -6467,7 +6441,7 @@
       <c r="H153">
         <v>3</v>
       </c>
-      <c r="J153" s="2">
+      <c r="J153" s="1">
         <v>46265</v>
       </c>
       <c r="K153" t="b">
@@ -6499,7 +6473,7 @@
       <c r="H154">
         <v>3</v>
       </c>
-      <c r="J154" s="2">
+      <c r="J154" s="1">
         <v>46265</v>
       </c>
       <c r="K154" t="b">
@@ -6531,7 +6505,7 @@
       <c r="H155">
         <v>43</v>
       </c>
-      <c r="J155" s="2">
+      <c r="J155" s="1">
         <v>46440</v>
       </c>
       <c r="K155" t="b">
@@ -6563,7 +6537,7 @@
       <c r="H156">
         <v>43</v>
       </c>
-      <c r="J156" s="2">
+      <c r="J156" s="1">
         <v>46440</v>
       </c>
       <c r="K156" t="b">
@@ -6595,7 +6569,7 @@
       <c r="H157">
         <v>72</v>
       </c>
-      <c r="J157" s="2">
+      <c r="J157" s="1">
         <v>46289</v>
       </c>
       <c r="K157" t="b">
@@ -6627,7 +6601,7 @@
       <c r="H158">
         <v>72</v>
       </c>
-      <c r="J158" s="2">
+      <c r="J158" s="1">
         <v>46289</v>
       </c>
       <c r="K158" t="b">
@@ -6659,7 +6633,7 @@
       <c r="H159">
         <v>81</v>
       </c>
-      <c r="J159" s="2">
+      <c r="J159" s="1">
         <v>46405</v>
       </c>
       <c r="K159" t="b">
@@ -6691,7 +6665,7 @@
       <c r="H160">
         <v>102</v>
       </c>
-      <c r="J160" s="2">
+      <c r="J160" s="1">
         <v>46463</v>
       </c>
       <c r="K160" t="b">
@@ -6723,7 +6697,7 @@
       <c r="H161">
         <v>109</v>
       </c>
-      <c r="J161" s="2">
+      <c r="J161" s="1">
         <v>46353</v>
       </c>
       <c r="K161" t="b">
@@ -6755,7 +6729,7 @@
       <c r="H162">
         <v>127</v>
       </c>
-      <c r="J162" s="2">
+      <c r="J162" s="1">
         <v>46417</v>
       </c>
       <c r="K162" t="b">
@@ -6787,7 +6761,7 @@
       <c r="H163">
         <v>152</v>
       </c>
-      <c r="J163" s="2">
+      <c r="J163" s="1">
         <v>46271</v>
       </c>
       <c r="K163" t="b">
@@ -6819,7 +6793,7 @@
       <c r="H164">
         <v>152</v>
       </c>
-      <c r="J164" s="2">
+      <c r="J164" s="1">
         <v>46271</v>
       </c>
       <c r="K164" t="b">
@@ -6851,7 +6825,7 @@
       <c r="H165">
         <v>153</v>
       </c>
-      <c r="J165" s="2">
+      <c r="J165" s="1">
         <v>46458</v>
       </c>
       <c r="K165" t="b">
@@ -6883,7 +6857,7 @@
       <c r="H166">
         <v>158</v>
       </c>
-      <c r="J166" s="2">
+      <c r="J166" s="1">
         <v>46381</v>
       </c>
       <c r="K166" t="b">
@@ -6915,7 +6889,7 @@
       <c r="H167">
         <v>163</v>
       </c>
-      <c r="J167" s="2">
+      <c r="J167" s="1">
         <v>46592</v>
       </c>
       <c r="K167" t="b">
@@ -6947,7 +6921,7 @@
       <c r="H168">
         <v>167</v>
       </c>
-      <c r="J168" s="2">
+      <c r="J168" s="1">
         <v>46441</v>
       </c>
       <c r="K168" t="b">
@@ -6979,7 +6953,7 @@
       <c r="H169">
         <v>169</v>
       </c>
-      <c r="J169" s="2">
+      <c r="J169" s="1">
         <v>46391</v>
       </c>
       <c r="K169" t="b">
@@ -7011,7 +6985,7 @@
       <c r="H170">
         <v>184</v>
       </c>
-      <c r="J170" s="2">
+      <c r="J170" s="1">
         <v>46385</v>
       </c>
       <c r="K170" t="b">
@@ -7043,7 +7017,7 @@
       <c r="H171">
         <v>186</v>
       </c>
-      <c r="J171" s="2">
+      <c r="J171" s="1">
         <v>46387</v>
       </c>
       <c r="K171" t="b">
@@ -7075,7 +7049,7 @@
       <c r="H172">
         <v>206</v>
       </c>
-      <c r="J172" s="2">
+      <c r="J172" s="1">
         <v>46399</v>
       </c>
       <c r="K172" t="b">
@@ -7107,7 +7081,7 @@
       <c r="H173">
         <v>206</v>
       </c>
-      <c r="J173" s="2">
+      <c r="J173" s="1">
         <v>46399</v>
       </c>
       <c r="K173" t="b">
@@ -7139,7 +7113,7 @@
       <c r="H174">
         <v>234</v>
       </c>
-      <c r="J174" s="2">
+      <c r="J174" s="1">
         <v>46458</v>
       </c>
       <c r="K174" t="b">
@@ -7171,7 +7145,7 @@
       <c r="H175">
         <v>248</v>
       </c>
-      <c r="J175" s="2">
+      <c r="J175" s="1">
         <v>46528</v>
       </c>
       <c r="K175" t="b">
@@ -7203,7 +7177,7 @@
       <c r="H176">
         <v>317</v>
       </c>
-      <c r="J176" s="2">
+      <c r="J176" s="1">
         <v>46540</v>
       </c>
       <c r="K176" t="b">
@@ -7235,7 +7209,7 @@
       <c r="H177">
         <v>340</v>
       </c>
-      <c r="J177" s="2">
+      <c r="J177" s="1">
         <v>46547</v>
       </c>
       <c r="K177" t="b">
@@ -7267,7 +7241,7 @@
       <c r="H178">
         <v>364</v>
       </c>
-      <c r="J178" s="2">
+      <c r="J178" s="1">
         <v>46557</v>
       </c>
       <c r="K178" t="b">
@@ -7299,7 +7273,7 @@
       <c r="H179">
         <v>368</v>
       </c>
-      <c r="J179" s="2">
+      <c r="J179" s="1">
         <v>46571</v>
       </c>
       <c r="K179" t="b">
@@ -7331,7 +7305,7 @@
       <c r="H180">
         <v>368</v>
       </c>
-      <c r="J180" s="2">
+      <c r="J180" s="1">
         <v>46571</v>
       </c>
       <c r="K180" t="b">
@@ -7363,7 +7337,7 @@
       <c r="H181">
         <v>370</v>
       </c>
-      <c r="J181" s="2">
+      <c r="J181" s="1">
         <v>46562</v>
       </c>
       <c r="K181" t="b">
@@ -7395,7 +7369,7 @@
       <c r="H182">
         <v>385</v>
       </c>
-      <c r="J182" s="2">
+      <c r="J182" s="1">
         <v>46574</v>
       </c>
       <c r="K182" t="b">
@@ -7427,7 +7401,7 @@
       <c r="H183">
         <v>385</v>
       </c>
-      <c r="J183" s="2">
+      <c r="J183" s="1">
         <v>46574</v>
       </c>
       <c r="K183" t="b">
@@ -7459,7 +7433,7 @@
       <c r="H184">
         <v>417</v>
       </c>
-      <c r="J184" s="2">
+      <c r="J184" s="1">
         <v>46578</v>
       </c>
       <c r="K184" t="b">
@@ -7491,7 +7465,7 @@
       <c r="H185">
         <v>721</v>
       </c>
-      <c r="J185" s="2">
+      <c r="J185" s="1">
         <v>46345</v>
       </c>
       <c r="K185" t="b">
@@ -7523,7 +7497,7 @@
       <c r="H186">
         <v>721</v>
       </c>
-      <c r="J186" s="2">
+      <c r="J186" s="1">
         <v>46345</v>
       </c>
       <c r="K186" t="b">
@@ -7555,7 +7529,7 @@
       <c r="H187">
         <v>850</v>
       </c>
-      <c r="J187" s="2">
+      <c r="J187" s="1">
         <v>46366</v>
       </c>
       <c r="K187" t="b">
@@ -7587,7 +7561,7 @@
       <c r="H188">
         <v>850</v>
       </c>
-      <c r="J188" s="2">
+      <c r="J188" s="1">
         <v>46366</v>
       </c>
       <c r="K188" t="b">
@@ -7619,7 +7593,7 @@
       <c r="H189">
         <v>1661</v>
       </c>
-      <c r="J189" s="2">
+      <c r="J189" s="1">
         <v>46524</v>
       </c>
       <c r="K189" t="b">
@@ -7651,7 +7625,7 @@
       <c r="H190">
         <v>1661</v>
       </c>
-      <c r="J190" s="2">
+      <c r="J190" s="1">
         <v>46524</v>
       </c>
       <c r="K190" t="b">
@@ -7683,7 +7657,7 @@
       <c r="H191">
         <v>488</v>
       </c>
-      <c r="J191" s="2">
+      <c r="J191" s="1">
         <v>46190</v>
       </c>
       <c r="K191" t="b">
@@ -7715,7 +7689,7 @@
       <c r="H192">
         <v>25565</v>
       </c>
-      <c r="J192" s="2">
+      <c r="J192" s="1">
         <v>46190</v>
       </c>
       <c r="K192" t="b">
@@ -7747,7 +7721,7 @@
       <c r="H193">
         <v>25567</v>
       </c>
-      <c r="J193" s="2">
+      <c r="J193" s="1">
         <v>46190</v>
       </c>
       <c r="K193" t="b">
@@ -7779,7 +7753,7 @@
       <c r="H194">
         <v>31293</v>
       </c>
-      <c r="J194" s="2">
+      <c r="J194" s="1">
         <v>46190</v>
       </c>
       <c r="K194" t="b">

</xml_diff>

<commit_message>
Atualização automática: vencimentos_tmot (18/08/2026 12:31)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
@@ -1019,8 +1019,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1036,7 +1044,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1044,12 +1052,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1349,37 +1375,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1408,7 +1434,7 @@
       <c r="H2">
         <v>-4300.3</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>39285</v>
       </c>
       <c r="K2" t="b">
@@ -1440,7 +1466,7 @@
       <c r="H3">
         <v>-2354.2</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>40669</v>
       </c>
       <c r="K3" t="b">
@@ -1472,7 +1498,7 @@
       <c r="H4">
         <v>-910.7</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>40669</v>
       </c>
       <c r="K4" t="b">
@@ -1504,7 +1530,7 @@
       <c r="H5">
         <v>-868</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>44884</v>
       </c>
       <c r="K5" t="b">
@@ -1536,7 +1562,7 @@
       <c r="H6">
         <v>-483.8</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>43855</v>
       </c>
       <c r="K6" t="b">
@@ -1568,7 +1594,7 @@
       <c r="H7">
         <v>-417</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>46014</v>
       </c>
       <c r="K7" t="b">
@@ -1600,7 +1626,7 @@
       <c r="H8">
         <v>-414.2</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>46014</v>
       </c>
       <c r="K8" t="b">
@@ -1632,7 +1658,7 @@
       <c r="H9">
         <v>-391.8</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>42769</v>
       </c>
       <c r="K9" t="b">
@@ -1664,7 +1690,7 @@
       <c r="H10">
         <v>-391.6</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>45804</v>
       </c>
       <c r="K10" t="b">
@@ -1696,7 +1722,7 @@
       <c r="H11">
         <v>-391.6</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>45804</v>
       </c>
       <c r="K11" t="b">
@@ -1728,7 +1754,7 @@
       <c r="H12">
         <v>-372.9</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>42821</v>
       </c>
       <c r="K12" t="b">
@@ -1760,7 +1786,7 @@
       <c r="H13">
         <v>-372.9</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>46014</v>
       </c>
       <c r="K13" t="b">
@@ -1792,7 +1818,7 @@
       <c r="H14">
         <v>-372.9</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>46014</v>
       </c>
       <c r="K14" t="b">
@@ -1824,7 +1850,7 @@
       <c r="H15">
         <v>-372.9</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>46014</v>
       </c>
       <c r="K15" t="b">
@@ -1856,7 +1882,7 @@
       <c r="H16">
         <v>-367.8</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="2">
         <v>46017</v>
       </c>
       <c r="K16" t="b">
@@ -1888,7 +1914,7 @@
       <c r="H17">
         <v>-367.8</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="2">
         <v>46017</v>
       </c>
       <c r="K17" t="b">
@@ -1920,7 +1946,7 @@
       <c r="H18">
         <v>-347.2</v>
       </c>
-      <c r="J18" s="1">
+      <c r="J18" s="2">
         <v>40979</v>
       </c>
       <c r="K18" t="b">
@@ -1952,7 +1978,7 @@
       <c r="H19">
         <v>-293.8</v>
       </c>
-      <c r="J19" s="1">
+      <c r="J19" s="2">
         <v>45846</v>
       </c>
       <c r="K19" t="b">
@@ -1984,7 +2010,7 @@
       <c r="H20">
         <v>-206.4</v>
       </c>
-      <c r="J20" s="1">
+      <c r="J20" s="2">
         <v>36669</v>
       </c>
       <c r="K20" t="b">
@@ -2016,7 +2042,7 @@
       <c r="H21">
         <v>-131.6</v>
       </c>
-      <c r="J21" s="1">
+      <c r="J21" s="2">
         <v>46111</v>
       </c>
       <c r="K21" t="b">
@@ -2048,7 +2074,7 @@
       <c r="H22">
         <v>-131.6</v>
       </c>
-      <c r="J22" s="1">
+      <c r="J22" s="2">
         <v>46111</v>
       </c>
       <c r="K22" t="b">
@@ -2080,7 +2106,7 @@
       <c r="H23">
         <v>-131.6</v>
       </c>
-      <c r="J23" s="1">
+      <c r="J23" s="2">
         <v>46111</v>
       </c>
       <c r="K23" t="b">
@@ -2112,7 +2138,7 @@
       <c r="H24">
         <v>-131.6</v>
       </c>
-      <c r="J24" s="1">
+      <c r="J24" s="2">
         <v>46111</v>
       </c>
       <c r="K24" t="b">
@@ -2144,7 +2170,7 @@
       <c r="H25">
         <v>-131.6</v>
       </c>
-      <c r="J25" s="1">
+      <c r="J25" s="2">
         <v>46111</v>
       </c>
       <c r="K25" t="b">
@@ -2176,7 +2202,7 @@
       <c r="H26">
         <v>-98.3</v>
       </c>
-      <c r="J26" s="1">
+      <c r="J26" s="2">
         <v>41204</v>
       </c>
       <c r="K26" t="b">
@@ -2208,7 +2234,7 @@
       <c r="H27">
         <v>-47.2</v>
       </c>
-      <c r="J27" s="1">
+      <c r="J27" s="2">
         <v>44011</v>
       </c>
       <c r="K27" t="b">
@@ -2240,7 +2266,7 @@
       <c r="H28">
         <v>-22.3</v>
       </c>
-      <c r="J28" s="1">
+      <c r="J28" s="2">
         <v>46226</v>
       </c>
       <c r="K28" t="b">
@@ -2272,7 +2298,7 @@
       <c r="H29">
         <v>4.7</v>
       </c>
-      <c r="J29" s="1">
+      <c r="J29" s="2">
         <v>46265</v>
       </c>
       <c r="K29" t="b">
@@ -2304,7 +2330,7 @@
       <c r="H30">
         <v>7.5</v>
       </c>
-      <c r="J30" s="1">
+      <c r="J30" s="2">
         <v>46265</v>
       </c>
       <c r="K30" t="b">
@@ -2336,7 +2362,7 @@
       <c r="H31">
         <v>10</v>
       </c>
-      <c r="J31" s="1">
+      <c r="J31" s="2">
         <v>46265</v>
       </c>
       <c r="K31" t="b">
@@ -2368,7 +2394,7 @@
       <c r="H32">
         <v>12.8</v>
       </c>
-      <c r="J32" s="1">
+      <c r="J32" s="2">
         <v>46265</v>
       </c>
       <c r="K32" t="b">
@@ -2400,7 +2426,7 @@
       <c r="H33">
         <v>14</v>
       </c>
-      <c r="J33" s="1">
+      <c r="J33" s="2">
         <v>46265</v>
       </c>
       <c r="K33" t="b">
@@ -2432,7 +2458,7 @@
       <c r="H34">
         <v>17.8</v>
       </c>
-      <c r="J34" s="1">
+      <c r="J34" s="2">
         <v>46265</v>
       </c>
       <c r="K34" t="b">
@@ -2464,7 +2490,7 @@
       <c r="H35">
         <v>20.4</v>
       </c>
-      <c r="J35" s="1">
+      <c r="J35" s="2">
         <v>46265</v>
       </c>
       <c r="K35" t="b">
@@ -2496,7 +2522,7 @@
       <c r="H36">
         <v>21.2</v>
       </c>
-      <c r="J36" s="1">
+      <c r="J36" s="2">
         <v>46265</v>
       </c>
       <c r="K36" t="b">
@@ -2528,7 +2554,7 @@
       <c r="H37">
         <v>26.2</v>
       </c>
-      <c r="J37" s="1">
+      <c r="J37" s="2">
         <v>46265</v>
       </c>
       <c r="K37" t="b">
@@ -2560,7 +2586,7 @@
       <c r="H38">
         <v>33.6</v>
       </c>
-      <c r="J38" s="1">
+      <c r="J38" s="2">
         <v>46364</v>
       </c>
       <c r="K38" t="b">
@@ -2592,7 +2618,7 @@
       <c r="H39">
         <v>42.2</v>
       </c>
-      <c r="J39" s="1">
+      <c r="J39" s="2">
         <v>46269</v>
       </c>
       <c r="K39" t="b">
@@ -2624,7 +2650,7 @@
       <c r="H40">
         <v>42.8</v>
       </c>
-      <c r="J40" s="1">
+      <c r="J40" s="2">
         <v>46291</v>
       </c>
       <c r="K40" t="b">
@@ -2656,7 +2682,7 @@
       <c r="H41">
         <v>45.7</v>
       </c>
-      <c r="J41" s="1">
+      <c r="J41" s="2">
         <v>46395</v>
       </c>
       <c r="K41" t="b">
@@ -2688,7 +2714,7 @@
       <c r="H42">
         <v>47.2</v>
       </c>
-      <c r="J42" s="1">
+      <c r="J42" s="2">
         <v>46280</v>
       </c>
       <c r="K42" t="b">
@@ -2720,7 +2746,7 @@
       <c r="H43">
         <v>48.7</v>
       </c>
-      <c r="J43" s="1">
+      <c r="J43" s="2">
         <v>46281</v>
       </c>
       <c r="K43" t="b">
@@ -2752,7 +2778,7 @@
       <c r="H44">
         <v>60</v>
       </c>
-      <c r="J44" s="1">
+      <c r="J44" s="2">
         <v>46281</v>
       </c>
       <c r="K44" t="b">
@@ -2784,7 +2810,7 @@
       <c r="H45">
         <v>62.6</v>
       </c>
-      <c r="J45" s="1">
+      <c r="J45" s="2">
         <v>46265</v>
       </c>
       <c r="K45" t="b">
@@ -2816,7 +2842,7 @@
       <c r="H46">
         <v>64.59999999999999</v>
       </c>
-      <c r="J46" s="1">
+      <c r="J46" s="2">
         <v>46265</v>
       </c>
       <c r="K46" t="b">
@@ -2848,7 +2874,7 @@
       <c r="H47">
         <v>67.59999999999999</v>
       </c>
-      <c r="J47" s="1">
+      <c r="J47" s="2">
         <v>46267</v>
       </c>
       <c r="K47" t="b">
@@ -2880,7 +2906,7 @@
       <c r="H48">
         <v>68.3</v>
       </c>
-      <c r="J48" s="1">
+      <c r="J48" s="2">
         <v>46278</v>
       </c>
       <c r="K48" t="b">
@@ -2912,7 +2938,7 @@
       <c r="H49">
         <v>69.2</v>
       </c>
-      <c r="J49" s="1">
+      <c r="J49" s="2">
         <v>46453</v>
       </c>
       <c r="K49" t="b">
@@ -2944,7 +2970,7 @@
       <c r="H50">
         <v>69.8</v>
       </c>
-      <c r="J50" s="1">
+      <c r="J50" s="2">
         <v>46265</v>
       </c>
       <c r="K50" t="b">
@@ -2976,7 +3002,7 @@
       <c r="H51">
         <v>69.8</v>
       </c>
-      <c r="J51" s="1">
+      <c r="J51" s="2">
         <v>46265</v>
       </c>
       <c r="K51" t="b">
@@ -3008,7 +3034,7 @@
       <c r="H52">
         <v>72.2</v>
       </c>
-      <c r="J52" s="1">
+      <c r="J52" s="2">
         <v>46275</v>
       </c>
       <c r="K52" t="b">
@@ -3040,7 +3066,7 @@
       <c r="H53">
         <v>72.2</v>
       </c>
-      <c r="J53" s="1">
+      <c r="J53" s="2">
         <v>46275</v>
       </c>
       <c r="K53" t="b">
@@ -3072,7 +3098,7 @@
       <c r="H54">
         <v>78.09999999999999</v>
       </c>
-      <c r="J54" s="1">
+      <c r="J54" s="2">
         <v>46265</v>
       </c>
       <c r="K54" t="b">
@@ -3104,7 +3130,7 @@
       <c r="H55">
         <v>82.8</v>
       </c>
-      <c r="J55" s="1">
+      <c r="J55" s="2">
         <v>46487</v>
       </c>
       <c r="K55" t="b">
@@ -3136,7 +3162,7 @@
       <c r="H56">
         <v>83.09999999999999</v>
       </c>
-      <c r="J56" s="1">
+      <c r="J56" s="2">
         <v>46285</v>
       </c>
       <c r="K56" t="b">
@@ -3168,7 +3194,7 @@
       <c r="H57">
         <v>84.8</v>
       </c>
-      <c r="J57" s="1">
+      <c r="J57" s="2">
         <v>46492</v>
       </c>
       <c r="K57" t="b">
@@ -3200,7 +3226,7 @@
       <c r="H58">
         <v>104.9</v>
       </c>
-      <c r="J58" s="1">
+      <c r="J58" s="2">
         <v>46297</v>
       </c>
       <c r="K58" t="b">
@@ -3232,7 +3258,7 @@
       <c r="H59">
         <v>107.6</v>
       </c>
-      <c r="J59" s="1">
+      <c r="J59" s="2">
         <v>46283</v>
       </c>
       <c r="K59" t="b">
@@ -3264,7 +3290,7 @@
       <c r="H60">
         <v>111.9</v>
       </c>
-      <c r="J60" s="1">
+      <c r="J60" s="2">
         <v>46300</v>
       </c>
       <c r="K60" t="b">
@@ -3296,7 +3322,7 @@
       <c r="H61">
         <v>111.9</v>
       </c>
-      <c r="J61" s="1">
+      <c r="J61" s="2">
         <v>46300</v>
       </c>
       <c r="K61" t="b">
@@ -3328,7 +3354,7 @@
       <c r="H62">
         <v>111.9</v>
       </c>
-      <c r="J62" s="1">
+      <c r="J62" s="2">
         <v>46300</v>
       </c>
       <c r="K62" t="b">
@@ -3360,7 +3386,7 @@
       <c r="H63">
         <v>111.9</v>
       </c>
-      <c r="J63" s="1">
+      <c r="J63" s="2">
         <v>46300</v>
       </c>
       <c r="K63" t="b">
@@ -3392,7 +3418,7 @@
       <c r="H64">
         <v>111.9</v>
       </c>
-      <c r="J64" s="1">
+      <c r="J64" s="2">
         <v>46300</v>
       </c>
       <c r="K64" t="b">
@@ -3424,7 +3450,7 @@
       <c r="H65">
         <v>128.8</v>
       </c>
-      <c r="J65" s="1">
+      <c r="J65" s="2">
         <v>46308</v>
       </c>
       <c r="K65" t="b">
@@ -3456,7 +3482,7 @@
       <c r="H66">
         <v>131.1</v>
       </c>
-      <c r="J66" s="1">
+      <c r="J66" s="2">
         <v>46336</v>
       </c>
       <c r="K66" t="b">
@@ -3488,7 +3514,7 @@
       <c r="H67">
         <v>138.4</v>
       </c>
-      <c r="J67" s="1">
+      <c r="J67" s="2">
         <v>46343</v>
       </c>
       <c r="K67" t="b">
@@ -3520,7 +3546,7 @@
       <c r="H68">
         <v>141</v>
       </c>
-      <c r="J68" s="1">
+      <c r="J68" s="2">
         <v>46350</v>
       </c>
       <c r="K68" t="b">
@@ -3552,7 +3578,7 @@
       <c r="H69">
         <v>162</v>
       </c>
-      <c r="J69" s="1">
+      <c r="J69" s="2">
         <v>46391</v>
       </c>
       <c r="K69" t="b">
@@ -3584,7 +3610,7 @@
       <c r="H70">
         <v>167.2</v>
       </c>
-      <c r="J70" s="1">
+      <c r="J70" s="2">
         <v>46330</v>
       </c>
       <c r="K70" t="b">
@@ -3616,7 +3642,7 @@
       <c r="H71">
         <v>177.4</v>
       </c>
-      <c r="J71" s="1">
+      <c r="J71" s="2">
         <v>46418</v>
       </c>
       <c r="K71" t="b">
@@ -3648,7 +3674,7 @@
       <c r="H72">
         <v>200</v>
       </c>
-      <c r="J72" s="1">
+      <c r="J72" s="2">
         <v>46356</v>
       </c>
       <c r="K72" t="b">
@@ -3680,7 +3706,7 @@
       <c r="H73">
         <v>203.6</v>
       </c>
-      <c r="J73" s="1">
+      <c r="J73" s="2">
         <v>46436</v>
       </c>
       <c r="K73" t="b">
@@ -3712,7 +3738,7 @@
       <c r="H74">
         <v>221.2</v>
       </c>
-      <c r="J74" s="1">
+      <c r="J74" s="2">
         <v>46426</v>
       </c>
       <c r="K74" t="b">
@@ -3744,7 +3770,7 @@
       <c r="H75">
         <v>240.8</v>
       </c>
-      <c r="J75" s="1">
+      <c r="J75" s="2">
         <v>46450</v>
       </c>
       <c r="K75" t="b">
@@ -3776,7 +3802,7 @@
       <c r="H76">
         <v>245.8</v>
       </c>
-      <c r="J76" s="1">
+      <c r="J76" s="2">
         <v>46452</v>
       </c>
       <c r="K76" t="b">
@@ -3808,7 +3834,7 @@
       <c r="H77">
         <v>263.4</v>
       </c>
-      <c r="J77" s="1">
+      <c r="J77" s="2">
         <v>46322</v>
       </c>
       <c r="K77" t="b">
@@ -3840,7 +3866,7 @@
       <c r="H78">
         <v>275.2</v>
       </c>
-      <c r="J78" s="1">
+      <c r="J78" s="2">
         <v>46433</v>
       </c>
       <c r="K78" t="b">
@@ -3875,7 +3901,7 @@
       <c r="I79" t="s">
         <v>311</v>
       </c>
-      <c r="J79" s="1">
+      <c r="J79" s="2">
         <v>36557</v>
       </c>
       <c r="K79" t="b">
@@ -3910,7 +3936,7 @@
       <c r="I80" t="s">
         <v>312</v>
       </c>
-      <c r="J80" s="1">
+      <c r="J80" s="2">
         <v>41275</v>
       </c>
       <c r="K80" t="b">
@@ -3945,7 +3971,7 @@
       <c r="I81" t="s">
         <v>313</v>
       </c>
-      <c r="J81" s="1">
+      <c r="J81" s="2">
         <v>45380</v>
       </c>
       <c r="K81" t="b">
@@ -3980,7 +4006,7 @@
       <c r="I82" t="s">
         <v>314</v>
       </c>
-      <c r="J82" s="1">
+      <c r="J82" s="2">
         <v>45421</v>
       </c>
       <c r="K82" t="b">
@@ -4015,7 +4041,7 @@
       <c r="I83" t="s">
         <v>314</v>
       </c>
-      <c r="J83" s="1">
+      <c r="J83" s="2">
         <v>45428</v>
       </c>
       <c r="K83" t="b">
@@ -4050,7 +4076,7 @@
       <c r="I84" t="s">
         <v>315</v>
       </c>
-      <c r="J84" s="1">
+      <c r="J84" s="2">
         <v>45490</v>
       </c>
       <c r="K84" t="b">
@@ -4085,7 +4111,7 @@
       <c r="I85" t="s">
         <v>316</v>
       </c>
-      <c r="J85" s="1">
+      <c r="J85" s="2">
         <v>45566</v>
       </c>
       <c r="K85" t="b">
@@ -4120,7 +4146,7 @@
       <c r="I86" t="s">
         <v>317</v>
       </c>
-      <c r="J86" s="1">
+      <c r="J86" s="2">
         <v>45986</v>
       </c>
       <c r="K86" t="b">
@@ -4155,7 +4181,7 @@
       <c r="I87" t="s">
         <v>318</v>
       </c>
-      <c r="J87" s="1">
+      <c r="J87" s="2">
         <v>46284</v>
       </c>
       <c r="K87" t="b">
@@ -4190,7 +4216,7 @@
       <c r="I88" t="s">
         <v>319</v>
       </c>
-      <c r="J88" s="1">
+      <c r="J88" s="2">
         <v>46305</v>
       </c>
       <c r="K88" t="b">
@@ -4225,7 +4251,7 @@
       <c r="I89" t="s">
         <v>319</v>
       </c>
-      <c r="J89" s="1">
+      <c r="J89" s="2">
         <v>46310</v>
       </c>
       <c r="K89" t="b">
@@ -4260,7 +4286,7 @@
       <c r="I90" t="s">
         <v>319</v>
       </c>
-      <c r="J90" s="1">
+      <c r="J90" s="2">
         <v>46317</v>
       </c>
       <c r="K90" t="b">
@@ -4295,7 +4321,7 @@
       <c r="I91" t="s">
         <v>319</v>
       </c>
-      <c r="J91" s="1">
+      <c r="J91" s="2">
         <v>46319</v>
       </c>
       <c r="K91" t="b">
@@ -4330,7 +4356,7 @@
       <c r="I92" t="s">
         <v>320</v>
       </c>
-      <c r="J92" s="1">
+      <c r="J92" s="2">
         <v>46333</v>
       </c>
       <c r="K92" t="b">
@@ -4365,7 +4391,7 @@
       <c r="I93" t="s">
         <v>320</v>
       </c>
-      <c r="J93" s="1">
+      <c r="J93" s="2">
         <v>46338</v>
       </c>
       <c r="K93" t="b">
@@ -4400,7 +4426,7 @@
       <c r="I94" t="s">
         <v>320</v>
       </c>
-      <c r="J94" s="1">
+      <c r="J94" s="2">
         <v>46338</v>
       </c>
       <c r="K94" t="b">
@@ -4435,7 +4461,7 @@
       <c r="I95" t="s">
         <v>320</v>
       </c>
-      <c r="J95" s="1">
+      <c r="J95" s="2">
         <v>46341</v>
       </c>
       <c r="K95" t="b">
@@ -4470,7 +4496,7 @@
       <c r="I96" t="s">
         <v>320</v>
       </c>
-      <c r="J96" s="1">
+      <c r="J96" s="2">
         <v>46344</v>
       </c>
       <c r="K96" t="b">
@@ -4505,7 +4531,7 @@
       <c r="I97" t="s">
         <v>321</v>
       </c>
-      <c r="J97" s="1">
+      <c r="J97" s="2">
         <v>46360</v>
       </c>
       <c r="K97" t="b">
@@ -4540,7 +4566,7 @@
       <c r="I98" t="s">
         <v>321</v>
       </c>
-      <c r="J98" s="1">
+      <c r="J98" s="2">
         <v>46360</v>
       </c>
       <c r="K98" t="b">
@@ -4575,7 +4601,7 @@
       <c r="I99" t="s">
         <v>321</v>
       </c>
-      <c r="J99" s="1">
+      <c r="J99" s="2">
         <v>46367</v>
       </c>
       <c r="K99" t="b">
@@ -4610,7 +4636,7 @@
       <c r="I100" t="s">
         <v>321</v>
       </c>
-      <c r="J100" s="1">
+      <c r="J100" s="2">
         <v>46375</v>
       </c>
       <c r="K100" t="b">
@@ -4645,7 +4671,7 @@
       <c r="I101" t="s">
         <v>321</v>
       </c>
-      <c r="J101" s="1">
+      <c r="J101" s="2">
         <v>46387</v>
       </c>
       <c r="K101" t="b">
@@ -4680,7 +4706,7 @@
       <c r="I102" t="s">
         <v>321</v>
       </c>
-      <c r="J102" s="1">
+      <c r="J102" s="2">
         <v>46387</v>
       </c>
       <c r="K102" t="b">
@@ -4715,7 +4741,7 @@
       <c r="I103" t="s">
         <v>321</v>
       </c>
-      <c r="J103" s="1">
+      <c r="J103" s="2">
         <v>46387</v>
       </c>
       <c r="K103" t="b">
@@ -4750,7 +4776,7 @@
       <c r="I104" t="s">
         <v>321</v>
       </c>
-      <c r="J104" s="1">
+      <c r="J104" s="2">
         <v>46388</v>
       </c>
       <c r="K104" t="b">
@@ -4785,7 +4811,7 @@
       <c r="I105" t="s">
         <v>322</v>
       </c>
-      <c r="J105" s="1">
+      <c r="J105" s="2">
         <v>46401</v>
       </c>
       <c r="K105" t="b">
@@ -4820,7 +4846,7 @@
       <c r="I106" t="s">
         <v>322</v>
       </c>
-      <c r="J106" s="1">
+      <c r="J106" s="2">
         <v>46401</v>
       </c>
       <c r="K106" t="b">
@@ -4855,7 +4881,7 @@
       <c r="I107" t="s">
         <v>322</v>
       </c>
-      <c r="J107" s="1">
+      <c r="J107" s="2">
         <v>46401</v>
       </c>
       <c r="K107" t="b">
@@ -4890,7 +4916,7 @@
       <c r="I108" t="s">
         <v>322</v>
       </c>
-      <c r="J108" s="1">
+      <c r="J108" s="2">
         <v>46412</v>
       </c>
       <c r="K108" t="b">
@@ -4925,7 +4951,7 @@
       <c r="I109" t="s">
         <v>322</v>
       </c>
-      <c r="J109" s="1">
+      <c r="J109" s="2">
         <v>46412</v>
       </c>
       <c r="K109" t="b">
@@ -4960,7 +4986,7 @@
       <c r="I110" t="s">
         <v>322</v>
       </c>
-      <c r="J110" s="1">
+      <c r="J110" s="2">
         <v>46412</v>
       </c>
       <c r="K110" t="b">
@@ -4995,7 +5021,7 @@
       <c r="I111" t="s">
         <v>323</v>
       </c>
-      <c r="J111" s="1">
+      <c r="J111" s="2">
         <v>46424</v>
       </c>
       <c r="K111" t="b">
@@ -5030,7 +5056,7 @@
       <c r="I112" t="s">
         <v>323</v>
       </c>
-      <c r="J112" s="1">
+      <c r="J112" s="2">
         <v>46437</v>
       </c>
       <c r="K112" t="b">
@@ -5065,7 +5091,7 @@
       <c r="I113" t="s">
         <v>323</v>
       </c>
-      <c r="J113" s="1">
+      <c r="J113" s="2">
         <v>46451</v>
       </c>
       <c r="K113" t="b">
@@ -5100,7 +5126,7 @@
       <c r="I114" t="s">
         <v>323</v>
       </c>
-      <c r="J114" s="1">
+      <c r="J114" s="2">
         <v>46451</v>
       </c>
       <c r="K114" t="b">
@@ -5135,7 +5161,7 @@
       <c r="I115" t="s">
         <v>324</v>
       </c>
-      <c r="J115" s="1">
+      <c r="J115" s="2">
         <v>46455</v>
       </c>
       <c r="K115" t="b">
@@ -5170,7 +5196,7 @@
       <c r="I116" t="s">
         <v>324</v>
       </c>
-      <c r="J116" s="1">
+      <c r="J116" s="2">
         <v>46456</v>
       </c>
       <c r="K116" t="b">
@@ -5205,7 +5231,7 @@
       <c r="I117" t="s">
         <v>324</v>
       </c>
-      <c r="J117" s="1">
+      <c r="J117" s="2">
         <v>46457</v>
       </c>
       <c r="K117" t="b">
@@ -5240,7 +5266,7 @@
       <c r="I118" t="s">
         <v>324</v>
       </c>
-      <c r="J118" s="1">
+      <c r="J118" s="2">
         <v>46464</v>
       </c>
       <c r="K118" t="b">
@@ -5275,7 +5301,7 @@
       <c r="I119" t="s">
         <v>324</v>
       </c>
-      <c r="J119" s="1">
+      <c r="J119" s="2">
         <v>46470</v>
       </c>
       <c r="K119" t="b">
@@ -5310,7 +5336,7 @@
       <c r="I120" t="s">
         <v>325</v>
       </c>
-      <c r="J120" s="1">
+      <c r="J120" s="2">
         <v>46485</v>
       </c>
       <c r="K120" t="b">
@@ -5345,7 +5371,7 @@
       <c r="I121" t="s">
         <v>325</v>
       </c>
-      <c r="J121" s="1">
+      <c r="J121" s="2">
         <v>46499</v>
       </c>
       <c r="K121" t="b">
@@ -5380,7 +5406,7 @@
       <c r="I122" t="s">
         <v>325</v>
       </c>
-      <c r="J122" s="1">
+      <c r="J122" s="2">
         <v>46504</v>
       </c>
       <c r="K122" t="b">
@@ -5415,7 +5441,7 @@
       <c r="I123" t="s">
         <v>325</v>
       </c>
-      <c r="J123" s="1">
+      <c r="J123" s="2">
         <v>46504</v>
       </c>
       <c r="K123" t="b">
@@ -5450,7 +5476,7 @@
       <c r="I124" t="s">
         <v>325</v>
       </c>
-      <c r="J124" s="1">
+      <c r="J124" s="2">
         <v>46507</v>
       </c>
       <c r="K124" t="b">
@@ -5485,7 +5511,7 @@
       <c r="I125" t="s">
         <v>325</v>
       </c>
-      <c r="J125" s="1">
+      <c r="J125" s="2">
         <v>46508</v>
       </c>
       <c r="K125" t="b">
@@ -5520,7 +5546,7 @@
       <c r="I126" t="s">
         <v>325</v>
       </c>
-      <c r="J126" s="1">
+      <c r="J126" s="2">
         <v>46512</v>
       </c>
       <c r="K126" t="b">
@@ -5555,7 +5581,7 @@
       <c r="I127" t="s">
         <v>326</v>
       </c>
-      <c r="J127" s="1">
+      <c r="J127" s="2">
         <v>46512</v>
       </c>
       <c r="K127" t="b">
@@ -5590,7 +5616,7 @@
       <c r="I128" t="s">
         <v>326</v>
       </c>
-      <c r="J128" s="1">
+      <c r="J128" s="2">
         <v>46528</v>
       </c>
       <c r="K128" t="b">
@@ -5625,7 +5651,7 @@
       <c r="I129" t="s">
         <v>326</v>
       </c>
-      <c r="J129" s="1">
+      <c r="J129" s="2">
         <v>46529</v>
       </c>
       <c r="K129" t="b">
@@ -5660,7 +5686,7 @@
       <c r="I130" t="s">
         <v>326</v>
       </c>
-      <c r="J130" s="1">
+      <c r="J130" s="2">
         <v>46537</v>
       </c>
       <c r="K130" t="b">
@@ -5695,7 +5721,7 @@
       <c r="I131" t="s">
         <v>327</v>
       </c>
-      <c r="J131" s="1">
+      <c r="J131" s="2">
         <v>46546</v>
       </c>
       <c r="K131" t="b">
@@ -5730,7 +5756,7 @@
       <c r="I132" t="s">
         <v>327</v>
       </c>
-      <c r="J132" s="1">
+      <c r="J132" s="2">
         <v>46547</v>
       </c>
       <c r="K132" t="b">
@@ -5765,7 +5791,7 @@
       <c r="I133" t="s">
         <v>327</v>
       </c>
-      <c r="J133" s="1">
+      <c r="J133" s="2">
         <v>46547</v>
       </c>
       <c r="K133" t="b">
@@ -5800,7 +5826,7 @@
       <c r="I134" t="s">
         <v>327</v>
       </c>
-      <c r="J134" s="1">
+      <c r="J134" s="2">
         <v>46547</v>
       </c>
       <c r="K134" t="b">
@@ -5835,7 +5861,7 @@
       <c r="I135" t="s">
         <v>327</v>
       </c>
-      <c r="J135" s="1">
+      <c r="J135" s="2">
         <v>46551</v>
       </c>
       <c r="K135" t="b">
@@ -5870,7 +5896,7 @@
       <c r="I136" t="s">
         <v>327</v>
       </c>
-      <c r="J136" s="1">
+      <c r="J136" s="2">
         <v>46560</v>
       </c>
       <c r="K136" t="b">
@@ -5905,7 +5931,7 @@
       <c r="I137" t="s">
         <v>327</v>
       </c>
-      <c r="J137" s="1">
+      <c r="J137" s="2">
         <v>46564</v>
       </c>
       <c r="K137" t="b">
@@ -5940,7 +5966,7 @@
       <c r="I138" t="s">
         <v>327</v>
       </c>
-      <c r="J138" s="1">
+      <c r="J138" s="2">
         <v>46567</v>
       </c>
       <c r="K138" t="b">
@@ -5975,7 +6001,7 @@
       <c r="I139" t="s">
         <v>327</v>
       </c>
-      <c r="J139" s="1">
+      <c r="J139" s="2">
         <v>46568</v>
       </c>
       <c r="K139" t="b">
@@ -6010,7 +6036,7 @@
       <c r="I140" t="s">
         <v>328</v>
       </c>
-      <c r="J140" s="1">
+      <c r="J140" s="2">
         <v>46578</v>
       </c>
       <c r="K140" t="b">
@@ -6045,7 +6071,7 @@
       <c r="I141" t="s">
         <v>328</v>
       </c>
-      <c r="J141" s="1">
+      <c r="J141" s="2">
         <v>46592</v>
       </c>
       <c r="K141" t="b">
@@ -6080,7 +6106,7 @@
       <c r="I142" t="s">
         <v>328</v>
       </c>
-      <c r="J142" s="1">
+      <c r="J142" s="2">
         <v>46592</v>
       </c>
       <c r="K142" t="b">
@@ -6115,7 +6141,7 @@
       <c r="I143" t="s">
         <v>329</v>
       </c>
-      <c r="J143" s="1">
+      <c r="J143" s="2">
         <v>46212</v>
       </c>
       <c r="K143" t="b">
@@ -6150,7 +6176,7 @@
       <c r="I144" t="s">
         <v>330</v>
       </c>
-      <c r="J144" s="1">
+      <c r="J144" s="2">
         <v>46225</v>
       </c>
       <c r="K144" t="b">
@@ -6185,7 +6211,7 @@
       <c r="I145" t="s">
         <v>331</v>
       </c>
-      <c r="J145" s="1">
+      <c r="J145" s="2">
         <v>46263</v>
       </c>
       <c r="K145" t="b">
@@ -6217,7 +6243,7 @@
       <c r="H146">
         <v>-1476</v>
       </c>
-      <c r="J146" s="1">
+      <c r="J146" s="2">
         <v>43773</v>
       </c>
       <c r="K146" t="b">
@@ -6249,7 +6275,7 @@
       <c r="H147">
         <v>-1469</v>
       </c>
-      <c r="J147" s="1">
+      <c r="J147" s="2">
         <v>43773</v>
       </c>
       <c r="K147" t="b">
@@ -6281,7 +6307,7 @@
       <c r="H148">
         <v>-1186</v>
       </c>
-      <c r="J148" s="1">
+      <c r="J148" s="2">
         <v>45295</v>
       </c>
       <c r="K148" t="b">
@@ -6313,7 +6339,7 @@
       <c r="H149">
         <v>-1048</v>
       </c>
-      <c r="J149" s="1">
+      <c r="J149" s="2">
         <v>45617</v>
       </c>
       <c r="K149" t="b">
@@ -6345,7 +6371,7 @@
       <c r="H150">
         <v>-980</v>
       </c>
-      <c r="J150" s="1">
+      <c r="J150" s="2">
         <v>45677</v>
       </c>
       <c r="K150" t="b">
@@ -6377,7 +6403,7 @@
       <c r="H151">
         <v>-961</v>
       </c>
-      <c r="J151" s="1">
+      <c r="J151" s="2">
         <v>44944</v>
       </c>
       <c r="K151" t="b">
@@ -6409,7 +6435,7 @@
       <c r="H152">
         <v>-252</v>
       </c>
-      <c r="J152" s="1">
+      <c r="J152" s="2">
         <v>46092</v>
       </c>
       <c r="K152" t="b">
@@ -6441,7 +6467,7 @@
       <c r="H153">
         <v>3</v>
       </c>
-      <c r="J153" s="1">
+      <c r="J153" s="2">
         <v>46265</v>
       </c>
       <c r="K153" t="b">
@@ -6473,7 +6499,7 @@
       <c r="H154">
         <v>3</v>
       </c>
-      <c r="J154" s="1">
+      <c r="J154" s="2">
         <v>46265</v>
       </c>
       <c r="K154" t="b">
@@ -6505,7 +6531,7 @@
       <c r="H155">
         <v>43</v>
       </c>
-      <c r="J155" s="1">
+      <c r="J155" s="2">
         <v>46440</v>
       </c>
       <c r="K155" t="b">
@@ -6537,7 +6563,7 @@
       <c r="H156">
         <v>43</v>
       </c>
-      <c r="J156" s="1">
+      <c r="J156" s="2">
         <v>46440</v>
       </c>
       <c r="K156" t="b">
@@ -6569,7 +6595,7 @@
       <c r="H157">
         <v>72</v>
       </c>
-      <c r="J157" s="1">
+      <c r="J157" s="2">
         <v>46289</v>
       </c>
       <c r="K157" t="b">
@@ -6601,7 +6627,7 @@
       <c r="H158">
         <v>72</v>
       </c>
-      <c r="J158" s="1">
+      <c r="J158" s="2">
         <v>46289</v>
       </c>
       <c r="K158" t="b">
@@ -6633,7 +6659,7 @@
       <c r="H159">
         <v>81</v>
       </c>
-      <c r="J159" s="1">
+      <c r="J159" s="2">
         <v>46405</v>
       </c>
       <c r="K159" t="b">
@@ -6665,7 +6691,7 @@
       <c r="H160">
         <v>102</v>
       </c>
-      <c r="J160" s="1">
+      <c r="J160" s="2">
         <v>46463</v>
       </c>
       <c r="K160" t="b">
@@ -6697,7 +6723,7 @@
       <c r="H161">
         <v>109</v>
       </c>
-      <c r="J161" s="1">
+      <c r="J161" s="2">
         <v>46353</v>
       </c>
       <c r="K161" t="b">
@@ -6729,7 +6755,7 @@
       <c r="H162">
         <v>127</v>
       </c>
-      <c r="J162" s="1">
+      <c r="J162" s="2">
         <v>46417</v>
       </c>
       <c r="K162" t="b">
@@ -6761,7 +6787,7 @@
       <c r="H163">
         <v>152</v>
       </c>
-      <c r="J163" s="1">
+      <c r="J163" s="2">
         <v>46271</v>
       </c>
       <c r="K163" t="b">
@@ -6793,7 +6819,7 @@
       <c r="H164">
         <v>152</v>
       </c>
-      <c r="J164" s="1">
+      <c r="J164" s="2">
         <v>46271</v>
       </c>
       <c r="K164" t="b">
@@ -6825,7 +6851,7 @@
       <c r="H165">
         <v>153</v>
       </c>
-      <c r="J165" s="1">
+      <c r="J165" s="2">
         <v>46458</v>
       </c>
       <c r="K165" t="b">
@@ -6857,7 +6883,7 @@
       <c r="H166">
         <v>158</v>
       </c>
-      <c r="J166" s="1">
+      <c r="J166" s="2">
         <v>46381</v>
       </c>
       <c r="K166" t="b">
@@ -6889,7 +6915,7 @@
       <c r="H167">
         <v>163</v>
       </c>
-      <c r="J167" s="1">
+      <c r="J167" s="2">
         <v>46592</v>
       </c>
       <c r="K167" t="b">
@@ -6921,7 +6947,7 @@
       <c r="H168">
         <v>167</v>
       </c>
-      <c r="J168" s="1">
+      <c r="J168" s="2">
         <v>46441</v>
       </c>
       <c r="K168" t="b">
@@ -6953,7 +6979,7 @@
       <c r="H169">
         <v>169</v>
       </c>
-      <c r="J169" s="1">
+      <c r="J169" s="2">
         <v>46391</v>
       </c>
       <c r="K169" t="b">
@@ -6985,7 +7011,7 @@
       <c r="H170">
         <v>184</v>
       </c>
-      <c r="J170" s="1">
+      <c r="J170" s="2">
         <v>46385</v>
       </c>
       <c r="K170" t="b">
@@ -7017,7 +7043,7 @@
       <c r="H171">
         <v>186</v>
       </c>
-      <c r="J171" s="1">
+      <c r="J171" s="2">
         <v>46387</v>
       </c>
       <c r="K171" t="b">
@@ -7049,7 +7075,7 @@
       <c r="H172">
         <v>206</v>
       </c>
-      <c r="J172" s="1">
+      <c r="J172" s="2">
         <v>46399</v>
       </c>
       <c r="K172" t="b">
@@ -7081,7 +7107,7 @@
       <c r="H173">
         <v>206</v>
       </c>
-      <c r="J173" s="1">
+      <c r="J173" s="2">
         <v>46399</v>
       </c>
       <c r="K173" t="b">
@@ -7113,7 +7139,7 @@
       <c r="H174">
         <v>234</v>
       </c>
-      <c r="J174" s="1">
+      <c r="J174" s="2">
         <v>46458</v>
       </c>
       <c r="K174" t="b">
@@ -7145,7 +7171,7 @@
       <c r="H175">
         <v>248</v>
       </c>
-      <c r="J175" s="1">
+      <c r="J175" s="2">
         <v>46528</v>
       </c>
       <c r="K175" t="b">
@@ -7177,7 +7203,7 @@
       <c r="H176">
         <v>317</v>
       </c>
-      <c r="J176" s="1">
+      <c r="J176" s="2">
         <v>46540</v>
       </c>
       <c r="K176" t="b">
@@ -7209,7 +7235,7 @@
       <c r="H177">
         <v>340</v>
       </c>
-      <c r="J177" s="1">
+      <c r="J177" s="2">
         <v>46547</v>
       </c>
       <c r="K177" t="b">
@@ -7241,7 +7267,7 @@
       <c r="H178">
         <v>364</v>
       </c>
-      <c r="J178" s="1">
+      <c r="J178" s="2">
         <v>46557</v>
       </c>
       <c r="K178" t="b">
@@ -7273,7 +7299,7 @@
       <c r="H179">
         <v>368</v>
       </c>
-      <c r="J179" s="1">
+      <c r="J179" s="2">
         <v>46571</v>
       </c>
       <c r="K179" t="b">
@@ -7305,7 +7331,7 @@
       <c r="H180">
         <v>368</v>
       </c>
-      <c r="J180" s="1">
+      <c r="J180" s="2">
         <v>46571</v>
       </c>
       <c r="K180" t="b">
@@ -7337,7 +7363,7 @@
       <c r="H181">
         <v>370</v>
       </c>
-      <c r="J181" s="1">
+      <c r="J181" s="2">
         <v>46562</v>
       </c>
       <c r="K181" t="b">
@@ -7369,7 +7395,7 @@
       <c r="H182">
         <v>385</v>
       </c>
-      <c r="J182" s="1">
+      <c r="J182" s="2">
         <v>46574</v>
       </c>
       <c r="K182" t="b">
@@ -7401,7 +7427,7 @@
       <c r="H183">
         <v>385</v>
       </c>
-      <c r="J183" s="1">
+      <c r="J183" s="2">
         <v>46574</v>
       </c>
       <c r="K183" t="b">
@@ -7433,7 +7459,7 @@
       <c r="H184">
         <v>417</v>
       </c>
-      <c r="J184" s="1">
+      <c r="J184" s="2">
         <v>46578</v>
       </c>
       <c r="K184" t="b">
@@ -7465,7 +7491,7 @@
       <c r="H185">
         <v>721</v>
       </c>
-      <c r="J185" s="1">
+      <c r="J185" s="2">
         <v>46345</v>
       </c>
       <c r="K185" t="b">
@@ -7497,7 +7523,7 @@
       <c r="H186">
         <v>721</v>
       </c>
-      <c r="J186" s="1">
+      <c r="J186" s="2">
         <v>46345</v>
       </c>
       <c r="K186" t="b">
@@ -7529,7 +7555,7 @@
       <c r="H187">
         <v>850</v>
       </c>
-      <c r="J187" s="1">
+      <c r="J187" s="2">
         <v>46366</v>
       </c>
       <c r="K187" t="b">
@@ -7561,7 +7587,7 @@
       <c r="H188">
         <v>850</v>
       </c>
-      <c r="J188" s="1">
+      <c r="J188" s="2">
         <v>46366</v>
       </c>
       <c r="K188" t="b">
@@ -7593,7 +7619,7 @@
       <c r="H189">
         <v>1661</v>
       </c>
-      <c r="J189" s="1">
+      <c r="J189" s="2">
         <v>46524</v>
       </c>
       <c r="K189" t="b">
@@ -7625,7 +7651,7 @@
       <c r="H190">
         <v>1661</v>
       </c>
-      <c r="J190" s="1">
+      <c r="J190" s="2">
         <v>46524</v>
       </c>
       <c r="K190" t="b">
@@ -7657,7 +7683,7 @@
       <c r="H191">
         <v>488</v>
       </c>
-      <c r="J191" s="1">
+      <c r="J191" s="2">
         <v>46190</v>
       </c>
       <c r="K191" t="b">
@@ -7689,7 +7715,7 @@
       <c r="H192">
         <v>25565</v>
       </c>
-      <c r="J192" s="1">
+      <c r="J192" s="2">
         <v>46190</v>
       </c>
       <c r="K192" t="b">
@@ -7721,7 +7747,7 @@
       <c r="H193">
         <v>25567</v>
       </c>
-      <c r="J193" s="1">
+      <c r="J193" s="2">
         <v>46190</v>
       </c>
       <c r="K193" t="b">
@@ -7753,7 +7779,7 @@
       <c r="H194">
         <v>31293</v>
       </c>
-      <c r="J194" s="1">
+      <c r="J194" s="2">
         <v>46190</v>
       </c>
       <c r="K194" t="b">

</xml_diff>

<commit_message>
Atualização automática: vencimentos_tmot (18/08/2026 12:40)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
@@ -1019,16 +1019,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1044,7 +1036,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1052,30 +1044,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1375,37 +1349,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1434,7 +1408,7 @@
       <c r="H2">
         <v>-4300.3</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>39285</v>
       </c>
       <c r="K2" t="b">
@@ -1466,7 +1440,7 @@
       <c r="H3">
         <v>-2354.2</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>40669</v>
       </c>
       <c r="K3" t="b">
@@ -1498,7 +1472,7 @@
       <c r="H4">
         <v>-910.7</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>40669</v>
       </c>
       <c r="K4" t="b">
@@ -1530,7 +1504,7 @@
       <c r="H5">
         <v>-868</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>44884</v>
       </c>
       <c r="K5" t="b">
@@ -1562,7 +1536,7 @@
       <c r="H6">
         <v>-483.8</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>43855</v>
       </c>
       <c r="K6" t="b">
@@ -1594,7 +1568,7 @@
       <c r="H7">
         <v>-417</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>46014</v>
       </c>
       <c r="K7" t="b">
@@ -1626,7 +1600,7 @@
       <c r="H8">
         <v>-414.2</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>46014</v>
       </c>
       <c r="K8" t="b">
@@ -1658,7 +1632,7 @@
       <c r="H9">
         <v>-391.8</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>42769</v>
       </c>
       <c r="K9" t="b">
@@ -1690,7 +1664,7 @@
       <c r="H10">
         <v>-391.6</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>45804</v>
       </c>
       <c r="K10" t="b">
@@ -1722,7 +1696,7 @@
       <c r="H11">
         <v>-391.6</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>45804</v>
       </c>
       <c r="K11" t="b">
@@ -1754,7 +1728,7 @@
       <c r="H12">
         <v>-372.9</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>42821</v>
       </c>
       <c r="K12" t="b">
@@ -1786,7 +1760,7 @@
       <c r="H13">
         <v>-372.9</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>46014</v>
       </c>
       <c r="K13" t="b">
@@ -1818,7 +1792,7 @@
       <c r="H14">
         <v>-372.9</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>46014</v>
       </c>
       <c r="K14" t="b">
@@ -1850,7 +1824,7 @@
       <c r="H15">
         <v>-372.9</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <v>46014</v>
       </c>
       <c r="K15" t="b">
@@ -1882,7 +1856,7 @@
       <c r="H16">
         <v>-367.8</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <v>46017</v>
       </c>
       <c r="K16" t="b">
@@ -1914,7 +1888,7 @@
       <c r="H17">
         <v>-367.8</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="1">
         <v>46017</v>
       </c>
       <c r="K17" t="b">
@@ -1946,7 +1920,7 @@
       <c r="H18">
         <v>-347.2</v>
       </c>
-      <c r="J18" s="2">
+      <c r="J18" s="1">
         <v>40979</v>
       </c>
       <c r="K18" t="b">
@@ -1978,7 +1952,7 @@
       <c r="H19">
         <v>-293.8</v>
       </c>
-      <c r="J19" s="2">
+      <c r="J19" s="1">
         <v>45846</v>
       </c>
       <c r="K19" t="b">
@@ -2010,7 +1984,7 @@
       <c r="H20">
         <v>-206.4</v>
       </c>
-      <c r="J20" s="2">
+      <c r="J20" s="1">
         <v>36669</v>
       </c>
       <c r="K20" t="b">
@@ -2042,7 +2016,7 @@
       <c r="H21">
         <v>-131.6</v>
       </c>
-      <c r="J21" s="2">
+      <c r="J21" s="1">
         <v>46111</v>
       </c>
       <c r="K21" t="b">
@@ -2074,7 +2048,7 @@
       <c r="H22">
         <v>-131.6</v>
       </c>
-      <c r="J22" s="2">
+      <c r="J22" s="1">
         <v>46111</v>
       </c>
       <c r="K22" t="b">
@@ -2106,7 +2080,7 @@
       <c r="H23">
         <v>-131.6</v>
       </c>
-      <c r="J23" s="2">
+      <c r="J23" s="1">
         <v>46111</v>
       </c>
       <c r="K23" t="b">
@@ -2138,7 +2112,7 @@
       <c r="H24">
         <v>-131.6</v>
       </c>
-      <c r="J24" s="2">
+      <c r="J24" s="1">
         <v>46111</v>
       </c>
       <c r="K24" t="b">
@@ -2170,7 +2144,7 @@
       <c r="H25">
         <v>-131.6</v>
       </c>
-      <c r="J25" s="2">
+      <c r="J25" s="1">
         <v>46111</v>
       </c>
       <c r="K25" t="b">
@@ -2202,7 +2176,7 @@
       <c r="H26">
         <v>-98.3</v>
       </c>
-      <c r="J26" s="2">
+      <c r="J26" s="1">
         <v>41204</v>
       </c>
       <c r="K26" t="b">
@@ -2234,7 +2208,7 @@
       <c r="H27">
         <v>-47.2</v>
       </c>
-      <c r="J27" s="2">
+      <c r="J27" s="1">
         <v>44011</v>
       </c>
       <c r="K27" t="b">
@@ -2266,7 +2240,7 @@
       <c r="H28">
         <v>-22.3</v>
       </c>
-      <c r="J28" s="2">
+      <c r="J28" s="1">
         <v>46226</v>
       </c>
       <c r="K28" t="b">
@@ -2298,7 +2272,7 @@
       <c r="H29">
         <v>4.7</v>
       </c>
-      <c r="J29" s="2">
+      <c r="J29" s="1">
         <v>46265</v>
       </c>
       <c r="K29" t="b">
@@ -2330,7 +2304,7 @@
       <c r="H30">
         <v>7.5</v>
       </c>
-      <c r="J30" s="2">
+      <c r="J30" s="1">
         <v>46265</v>
       </c>
       <c r="K30" t="b">
@@ -2362,7 +2336,7 @@
       <c r="H31">
         <v>10</v>
       </c>
-      <c r="J31" s="2">
+      <c r="J31" s="1">
         <v>46265</v>
       </c>
       <c r="K31" t="b">
@@ -2394,7 +2368,7 @@
       <c r="H32">
         <v>12.8</v>
       </c>
-      <c r="J32" s="2">
+      <c r="J32" s="1">
         <v>46265</v>
       </c>
       <c r="K32" t="b">
@@ -2426,7 +2400,7 @@
       <c r="H33">
         <v>14</v>
       </c>
-      <c r="J33" s="2">
+      <c r="J33" s="1">
         <v>46265</v>
       </c>
       <c r="K33" t="b">
@@ -2458,7 +2432,7 @@
       <c r="H34">
         <v>17.8</v>
       </c>
-      <c r="J34" s="2">
+      <c r="J34" s="1">
         <v>46265</v>
       </c>
       <c r="K34" t="b">
@@ -2490,7 +2464,7 @@
       <c r="H35">
         <v>20.4</v>
       </c>
-      <c r="J35" s="2">
+      <c r="J35" s="1">
         <v>46265</v>
       </c>
       <c r="K35" t="b">
@@ -2522,7 +2496,7 @@
       <c r="H36">
         <v>21.2</v>
       </c>
-      <c r="J36" s="2">
+      <c r="J36" s="1">
         <v>46265</v>
       </c>
       <c r="K36" t="b">
@@ -2554,7 +2528,7 @@
       <c r="H37">
         <v>26.2</v>
       </c>
-      <c r="J37" s="2">
+      <c r="J37" s="1">
         <v>46265</v>
       </c>
       <c r="K37" t="b">
@@ -2586,7 +2560,7 @@
       <c r="H38">
         <v>33.6</v>
       </c>
-      <c r="J38" s="2">
+      <c r="J38" s="1">
         <v>46364</v>
       </c>
       <c r="K38" t="b">
@@ -2618,7 +2592,7 @@
       <c r="H39">
         <v>42.2</v>
       </c>
-      <c r="J39" s="2">
+      <c r="J39" s="1">
         <v>46269</v>
       </c>
       <c r="K39" t="b">
@@ -2650,7 +2624,7 @@
       <c r="H40">
         <v>42.8</v>
       </c>
-      <c r="J40" s="2">
+      <c r="J40" s="1">
         <v>46291</v>
       </c>
       <c r="K40" t="b">
@@ -2682,7 +2656,7 @@
       <c r="H41">
         <v>45.7</v>
       </c>
-      <c r="J41" s="2">
+      <c r="J41" s="1">
         <v>46395</v>
       </c>
       <c r="K41" t="b">
@@ -2714,7 +2688,7 @@
       <c r="H42">
         <v>47.2</v>
       </c>
-      <c r="J42" s="2">
+      <c r="J42" s="1">
         <v>46280</v>
       </c>
       <c r="K42" t="b">
@@ -2746,7 +2720,7 @@
       <c r="H43">
         <v>48.7</v>
       </c>
-      <c r="J43" s="2">
+      <c r="J43" s="1">
         <v>46281</v>
       </c>
       <c r="K43" t="b">
@@ -2778,7 +2752,7 @@
       <c r="H44">
         <v>60</v>
       </c>
-      <c r="J44" s="2">
+      <c r="J44" s="1">
         <v>46281</v>
       </c>
       <c r="K44" t="b">
@@ -2810,7 +2784,7 @@
       <c r="H45">
         <v>62.6</v>
       </c>
-      <c r="J45" s="2">
+      <c r="J45" s="1">
         <v>46265</v>
       </c>
       <c r="K45" t="b">
@@ -2842,7 +2816,7 @@
       <c r="H46">
         <v>64.59999999999999</v>
       </c>
-      <c r="J46" s="2">
+      <c r="J46" s="1">
         <v>46265</v>
       </c>
       <c r="K46" t="b">
@@ -2874,7 +2848,7 @@
       <c r="H47">
         <v>67.59999999999999</v>
       </c>
-      <c r="J47" s="2">
+      <c r="J47" s="1">
         <v>46267</v>
       </c>
       <c r="K47" t="b">
@@ -2906,7 +2880,7 @@
       <c r="H48">
         <v>68.3</v>
       </c>
-      <c r="J48" s="2">
+      <c r="J48" s="1">
         <v>46278</v>
       </c>
       <c r="K48" t="b">
@@ -2938,7 +2912,7 @@
       <c r="H49">
         <v>69.2</v>
       </c>
-      <c r="J49" s="2">
+      <c r="J49" s="1">
         <v>46453</v>
       </c>
       <c r="K49" t="b">
@@ -2970,7 +2944,7 @@
       <c r="H50">
         <v>69.8</v>
       </c>
-      <c r="J50" s="2">
+      <c r="J50" s="1">
         <v>46265</v>
       </c>
       <c r="K50" t="b">
@@ -3002,7 +2976,7 @@
       <c r="H51">
         <v>69.8</v>
       </c>
-      <c r="J51" s="2">
+      <c r="J51" s="1">
         <v>46265</v>
       </c>
       <c r="K51" t="b">
@@ -3034,7 +3008,7 @@
       <c r="H52">
         <v>72.2</v>
       </c>
-      <c r="J52" s="2">
+      <c r="J52" s="1">
         <v>46275</v>
       </c>
       <c r="K52" t="b">
@@ -3066,7 +3040,7 @@
       <c r="H53">
         <v>72.2</v>
       </c>
-      <c r="J53" s="2">
+      <c r="J53" s="1">
         <v>46275</v>
       </c>
       <c r="K53" t="b">
@@ -3098,7 +3072,7 @@
       <c r="H54">
         <v>78.09999999999999</v>
       </c>
-      <c r="J54" s="2">
+      <c r="J54" s="1">
         <v>46265</v>
       </c>
       <c r="K54" t="b">
@@ -3130,7 +3104,7 @@
       <c r="H55">
         <v>82.8</v>
       </c>
-      <c r="J55" s="2">
+      <c r="J55" s="1">
         <v>46487</v>
       </c>
       <c r="K55" t="b">
@@ -3162,7 +3136,7 @@
       <c r="H56">
         <v>83.09999999999999</v>
       </c>
-      <c r="J56" s="2">
+      <c r="J56" s="1">
         <v>46285</v>
       </c>
       <c r="K56" t="b">
@@ -3194,7 +3168,7 @@
       <c r="H57">
         <v>84.8</v>
       </c>
-      <c r="J57" s="2">
+      <c r="J57" s="1">
         <v>46492</v>
       </c>
       <c r="K57" t="b">
@@ -3226,7 +3200,7 @@
       <c r="H58">
         <v>104.9</v>
       </c>
-      <c r="J58" s="2">
+      <c r="J58" s="1">
         <v>46297</v>
       </c>
       <c r="K58" t="b">
@@ -3258,7 +3232,7 @@
       <c r="H59">
         <v>107.6</v>
       </c>
-      <c r="J59" s="2">
+      <c r="J59" s="1">
         <v>46283</v>
       </c>
       <c r="K59" t="b">
@@ -3290,7 +3264,7 @@
       <c r="H60">
         <v>111.9</v>
       </c>
-      <c r="J60" s="2">
+      <c r="J60" s="1">
         <v>46300</v>
       </c>
       <c r="K60" t="b">
@@ -3322,7 +3296,7 @@
       <c r="H61">
         <v>111.9</v>
       </c>
-      <c r="J61" s="2">
+      <c r="J61" s="1">
         <v>46300</v>
       </c>
       <c r="K61" t="b">
@@ -3354,7 +3328,7 @@
       <c r="H62">
         <v>111.9</v>
       </c>
-      <c r="J62" s="2">
+      <c r="J62" s="1">
         <v>46300</v>
       </c>
       <c r="K62" t="b">
@@ -3386,7 +3360,7 @@
       <c r="H63">
         <v>111.9</v>
       </c>
-      <c r="J63" s="2">
+      <c r="J63" s="1">
         <v>46300</v>
       </c>
       <c r="K63" t="b">
@@ -3418,7 +3392,7 @@
       <c r="H64">
         <v>111.9</v>
       </c>
-      <c r="J64" s="2">
+      <c r="J64" s="1">
         <v>46300</v>
       </c>
       <c r="K64" t="b">
@@ -3450,7 +3424,7 @@
       <c r="H65">
         <v>128.8</v>
       </c>
-      <c r="J65" s="2">
+      <c r="J65" s="1">
         <v>46308</v>
       </c>
       <c r="K65" t="b">
@@ -3482,7 +3456,7 @@
       <c r="H66">
         <v>131.1</v>
       </c>
-      <c r="J66" s="2">
+      <c r="J66" s="1">
         <v>46336</v>
       </c>
       <c r="K66" t="b">
@@ -3514,7 +3488,7 @@
       <c r="H67">
         <v>138.4</v>
       </c>
-      <c r="J67" s="2">
+      <c r="J67" s="1">
         <v>46343</v>
       </c>
       <c r="K67" t="b">
@@ -3546,7 +3520,7 @@
       <c r="H68">
         <v>141</v>
       </c>
-      <c r="J68" s="2">
+      <c r="J68" s="1">
         <v>46350</v>
       </c>
       <c r="K68" t="b">
@@ -3578,7 +3552,7 @@
       <c r="H69">
         <v>162</v>
       </c>
-      <c r="J69" s="2">
+      <c r="J69" s="1">
         <v>46391</v>
       </c>
       <c r="K69" t="b">
@@ -3610,7 +3584,7 @@
       <c r="H70">
         <v>167.2</v>
       </c>
-      <c r="J70" s="2">
+      <c r="J70" s="1">
         <v>46330</v>
       </c>
       <c r="K70" t="b">
@@ -3642,7 +3616,7 @@
       <c r="H71">
         <v>177.4</v>
       </c>
-      <c r="J71" s="2">
+      <c r="J71" s="1">
         <v>46418</v>
       </c>
       <c r="K71" t="b">
@@ -3674,7 +3648,7 @@
       <c r="H72">
         <v>200</v>
       </c>
-      <c r="J72" s="2">
+      <c r="J72" s="1">
         <v>46356</v>
       </c>
       <c r="K72" t="b">
@@ -3706,7 +3680,7 @@
       <c r="H73">
         <v>203.6</v>
       </c>
-      <c r="J73" s="2">
+      <c r="J73" s="1">
         <v>46436</v>
       </c>
       <c r="K73" t="b">
@@ -3738,7 +3712,7 @@
       <c r="H74">
         <v>221.2</v>
       </c>
-      <c r="J74" s="2">
+      <c r="J74" s="1">
         <v>46426</v>
       </c>
       <c r="K74" t="b">
@@ -3770,7 +3744,7 @@
       <c r="H75">
         <v>240.8</v>
       </c>
-      <c r="J75" s="2">
+      <c r="J75" s="1">
         <v>46450</v>
       </c>
       <c r="K75" t="b">
@@ -3802,7 +3776,7 @@
       <c r="H76">
         <v>245.8</v>
       </c>
-      <c r="J76" s="2">
+      <c r="J76" s="1">
         <v>46452</v>
       </c>
       <c r="K76" t="b">
@@ -3834,7 +3808,7 @@
       <c r="H77">
         <v>263.4</v>
       </c>
-      <c r="J77" s="2">
+      <c r="J77" s="1">
         <v>46322</v>
       </c>
       <c r="K77" t="b">
@@ -3866,7 +3840,7 @@
       <c r="H78">
         <v>275.2</v>
       </c>
-      <c r="J78" s="2">
+      <c r="J78" s="1">
         <v>46433</v>
       </c>
       <c r="K78" t="b">
@@ -3901,7 +3875,7 @@
       <c r="I79" t="s">
         <v>311</v>
       </c>
-      <c r="J79" s="2">
+      <c r="J79" s="1">
         <v>36557</v>
       </c>
       <c r="K79" t="b">
@@ -3936,7 +3910,7 @@
       <c r="I80" t="s">
         <v>312</v>
       </c>
-      <c r="J80" s="2">
+      <c r="J80" s="1">
         <v>41275</v>
       </c>
       <c r="K80" t="b">
@@ -3971,7 +3945,7 @@
       <c r="I81" t="s">
         <v>313</v>
       </c>
-      <c r="J81" s="2">
+      <c r="J81" s="1">
         <v>45380</v>
       </c>
       <c r="K81" t="b">
@@ -4006,7 +3980,7 @@
       <c r="I82" t="s">
         <v>314</v>
       </c>
-      <c r="J82" s="2">
+      <c r="J82" s="1">
         <v>45421</v>
       </c>
       <c r="K82" t="b">
@@ -4041,7 +4015,7 @@
       <c r="I83" t="s">
         <v>314</v>
       </c>
-      <c r="J83" s="2">
+      <c r="J83" s="1">
         <v>45428</v>
       </c>
       <c r="K83" t="b">
@@ -4076,7 +4050,7 @@
       <c r="I84" t="s">
         <v>315</v>
       </c>
-      <c r="J84" s="2">
+      <c r="J84" s="1">
         <v>45490</v>
       </c>
       <c r="K84" t="b">
@@ -4111,7 +4085,7 @@
       <c r="I85" t="s">
         <v>316</v>
       </c>
-      <c r="J85" s="2">
+      <c r="J85" s="1">
         <v>45566</v>
       </c>
       <c r="K85" t="b">
@@ -4146,7 +4120,7 @@
       <c r="I86" t="s">
         <v>317</v>
       </c>
-      <c r="J86" s="2">
+      <c r="J86" s="1">
         <v>45986</v>
       </c>
       <c r="K86" t="b">
@@ -4181,7 +4155,7 @@
       <c r="I87" t="s">
         <v>318</v>
       </c>
-      <c r="J87" s="2">
+      <c r="J87" s="1">
         <v>46284</v>
       </c>
       <c r="K87" t="b">
@@ -4216,7 +4190,7 @@
       <c r="I88" t="s">
         <v>319</v>
       </c>
-      <c r="J88" s="2">
+      <c r="J88" s="1">
         <v>46305</v>
       </c>
       <c r="K88" t="b">
@@ -4251,7 +4225,7 @@
       <c r="I89" t="s">
         <v>319</v>
       </c>
-      <c r="J89" s="2">
+      <c r="J89" s="1">
         <v>46310</v>
       </c>
       <c r="K89" t="b">
@@ -4286,7 +4260,7 @@
       <c r="I90" t="s">
         <v>319</v>
       </c>
-      <c r="J90" s="2">
+      <c r="J90" s="1">
         <v>46317</v>
       </c>
       <c r="K90" t="b">
@@ -4321,7 +4295,7 @@
       <c r="I91" t="s">
         <v>319</v>
       </c>
-      <c r="J91" s="2">
+      <c r="J91" s="1">
         <v>46319</v>
       </c>
       <c r="K91" t="b">
@@ -4356,7 +4330,7 @@
       <c r="I92" t="s">
         <v>320</v>
       </c>
-      <c r="J92" s="2">
+      <c r="J92" s="1">
         <v>46333</v>
       </c>
       <c r="K92" t="b">
@@ -4391,7 +4365,7 @@
       <c r="I93" t="s">
         <v>320</v>
       </c>
-      <c r="J93" s="2">
+      <c r="J93" s="1">
         <v>46338</v>
       </c>
       <c r="K93" t="b">
@@ -4426,7 +4400,7 @@
       <c r="I94" t="s">
         <v>320</v>
       </c>
-      <c r="J94" s="2">
+      <c r="J94" s="1">
         <v>46338</v>
       </c>
       <c r="K94" t="b">
@@ -4461,7 +4435,7 @@
       <c r="I95" t="s">
         <v>320</v>
       </c>
-      <c r="J95" s="2">
+      <c r="J95" s="1">
         <v>46341</v>
       </c>
       <c r="K95" t="b">
@@ -4496,7 +4470,7 @@
       <c r="I96" t="s">
         <v>320</v>
       </c>
-      <c r="J96" s="2">
+      <c r="J96" s="1">
         <v>46344</v>
       </c>
       <c r="K96" t="b">
@@ -4531,7 +4505,7 @@
       <c r="I97" t="s">
         <v>321</v>
       </c>
-      <c r="J97" s="2">
+      <c r="J97" s="1">
         <v>46360</v>
       </c>
       <c r="K97" t="b">
@@ -4566,7 +4540,7 @@
       <c r="I98" t="s">
         <v>321</v>
       </c>
-      <c r="J98" s="2">
+      <c r="J98" s="1">
         <v>46360</v>
       </c>
       <c r="K98" t="b">
@@ -4601,7 +4575,7 @@
       <c r="I99" t="s">
         <v>321</v>
       </c>
-      <c r="J99" s="2">
+      <c r="J99" s="1">
         <v>46367</v>
       </c>
       <c r="K99" t="b">
@@ -4636,7 +4610,7 @@
       <c r="I100" t="s">
         <v>321</v>
       </c>
-      <c r="J100" s="2">
+      <c r="J100" s="1">
         <v>46375</v>
       </c>
       <c r="K100" t="b">
@@ -4671,7 +4645,7 @@
       <c r="I101" t="s">
         <v>321</v>
       </c>
-      <c r="J101" s="2">
+      <c r="J101" s="1">
         <v>46387</v>
       </c>
       <c r="K101" t="b">
@@ -4706,7 +4680,7 @@
       <c r="I102" t="s">
         <v>321</v>
       </c>
-      <c r="J102" s="2">
+      <c r="J102" s="1">
         <v>46387</v>
       </c>
       <c r="K102" t="b">
@@ -4741,7 +4715,7 @@
       <c r="I103" t="s">
         <v>321</v>
       </c>
-      <c r="J103" s="2">
+      <c r="J103" s="1">
         <v>46387</v>
       </c>
       <c r="K103" t="b">
@@ -4776,7 +4750,7 @@
       <c r="I104" t="s">
         <v>321</v>
       </c>
-      <c r="J104" s="2">
+      <c r="J104" s="1">
         <v>46388</v>
       </c>
       <c r="K104" t="b">
@@ -4811,7 +4785,7 @@
       <c r="I105" t="s">
         <v>322</v>
       </c>
-      <c r="J105" s="2">
+      <c r="J105" s="1">
         <v>46401</v>
       </c>
       <c r="K105" t="b">
@@ -4846,7 +4820,7 @@
       <c r="I106" t="s">
         <v>322</v>
       </c>
-      <c r="J106" s="2">
+      <c r="J106" s="1">
         <v>46401</v>
       </c>
       <c r="K106" t="b">
@@ -4881,7 +4855,7 @@
       <c r="I107" t="s">
         <v>322</v>
       </c>
-      <c r="J107" s="2">
+      <c r="J107" s="1">
         <v>46401</v>
       </c>
       <c r="K107" t="b">
@@ -4916,7 +4890,7 @@
       <c r="I108" t="s">
         <v>322</v>
       </c>
-      <c r="J108" s="2">
+      <c r="J108" s="1">
         <v>46412</v>
       </c>
       <c r="K108" t="b">
@@ -4951,7 +4925,7 @@
       <c r="I109" t="s">
         <v>322</v>
       </c>
-      <c r="J109" s="2">
+      <c r="J109" s="1">
         <v>46412</v>
       </c>
       <c r="K109" t="b">
@@ -4986,7 +4960,7 @@
       <c r="I110" t="s">
         <v>322</v>
       </c>
-      <c r="J110" s="2">
+      <c r="J110" s="1">
         <v>46412</v>
       </c>
       <c r="K110" t="b">
@@ -5021,7 +4995,7 @@
       <c r="I111" t="s">
         <v>323</v>
       </c>
-      <c r="J111" s="2">
+      <c r="J111" s="1">
         <v>46424</v>
       </c>
       <c r="K111" t="b">
@@ -5056,7 +5030,7 @@
       <c r="I112" t="s">
         <v>323</v>
       </c>
-      <c r="J112" s="2">
+      <c r="J112" s="1">
         <v>46437</v>
       </c>
       <c r="K112" t="b">
@@ -5091,7 +5065,7 @@
       <c r="I113" t="s">
         <v>323</v>
       </c>
-      <c r="J113" s="2">
+      <c r="J113" s="1">
         <v>46451</v>
       </c>
       <c r="K113" t="b">
@@ -5126,7 +5100,7 @@
       <c r="I114" t="s">
         <v>323</v>
       </c>
-      <c r="J114" s="2">
+      <c r="J114" s="1">
         <v>46451</v>
       </c>
       <c r="K114" t="b">
@@ -5161,7 +5135,7 @@
       <c r="I115" t="s">
         <v>324</v>
       </c>
-      <c r="J115" s="2">
+      <c r="J115" s="1">
         <v>46455</v>
       </c>
       <c r="K115" t="b">
@@ -5196,7 +5170,7 @@
       <c r="I116" t="s">
         <v>324</v>
       </c>
-      <c r="J116" s="2">
+      <c r="J116" s="1">
         <v>46456</v>
       </c>
       <c r="K116" t="b">
@@ -5231,7 +5205,7 @@
       <c r="I117" t="s">
         <v>324</v>
       </c>
-      <c r="J117" s="2">
+      <c r="J117" s="1">
         <v>46457</v>
       </c>
       <c r="K117" t="b">
@@ -5266,7 +5240,7 @@
       <c r="I118" t="s">
         <v>324</v>
       </c>
-      <c r="J118" s="2">
+      <c r="J118" s="1">
         <v>46464</v>
       </c>
       <c r="K118" t="b">
@@ -5301,7 +5275,7 @@
       <c r="I119" t="s">
         <v>324</v>
       </c>
-      <c r="J119" s="2">
+      <c r="J119" s="1">
         <v>46470</v>
       </c>
       <c r="K119" t="b">
@@ -5336,7 +5310,7 @@
       <c r="I120" t="s">
         <v>325</v>
       </c>
-      <c r="J120" s="2">
+      <c r="J120" s="1">
         <v>46485</v>
       </c>
       <c r="K120" t="b">
@@ -5371,7 +5345,7 @@
       <c r="I121" t="s">
         <v>325</v>
       </c>
-      <c r="J121" s="2">
+      <c r="J121" s="1">
         <v>46499</v>
       </c>
       <c r="K121" t="b">
@@ -5406,7 +5380,7 @@
       <c r="I122" t="s">
         <v>325</v>
       </c>
-      <c r="J122" s="2">
+      <c r="J122" s="1">
         <v>46504</v>
       </c>
       <c r="K122" t="b">
@@ -5441,7 +5415,7 @@
       <c r="I123" t="s">
         <v>325</v>
       </c>
-      <c r="J123" s="2">
+      <c r="J123" s="1">
         <v>46504</v>
       </c>
       <c r="K123" t="b">
@@ -5476,7 +5450,7 @@
       <c r="I124" t="s">
         <v>325</v>
       </c>
-      <c r="J124" s="2">
+      <c r="J124" s="1">
         <v>46507</v>
       </c>
       <c r="K124" t="b">
@@ -5511,7 +5485,7 @@
       <c r="I125" t="s">
         <v>325</v>
       </c>
-      <c r="J125" s="2">
+      <c r="J125" s="1">
         <v>46508</v>
       </c>
       <c r="K125" t="b">
@@ -5546,7 +5520,7 @@
       <c r="I126" t="s">
         <v>325</v>
       </c>
-      <c r="J126" s="2">
+      <c r="J126" s="1">
         <v>46512</v>
       </c>
       <c r="K126" t="b">
@@ -5581,7 +5555,7 @@
       <c r="I127" t="s">
         <v>326</v>
       </c>
-      <c r="J127" s="2">
+      <c r="J127" s="1">
         <v>46512</v>
       </c>
       <c r="K127" t="b">
@@ -5616,7 +5590,7 @@
       <c r="I128" t="s">
         <v>326</v>
       </c>
-      <c r="J128" s="2">
+      <c r="J128" s="1">
         <v>46528</v>
       </c>
       <c r="K128" t="b">
@@ -5651,7 +5625,7 @@
       <c r="I129" t="s">
         <v>326</v>
       </c>
-      <c r="J129" s="2">
+      <c r="J129" s="1">
         <v>46529</v>
       </c>
       <c r="K129" t="b">
@@ -5686,7 +5660,7 @@
       <c r="I130" t="s">
         <v>326</v>
       </c>
-      <c r="J130" s="2">
+      <c r="J130" s="1">
         <v>46537</v>
       </c>
       <c r="K130" t="b">
@@ -5721,7 +5695,7 @@
       <c r="I131" t="s">
         <v>327</v>
       </c>
-      <c r="J131" s="2">
+      <c r="J131" s="1">
         <v>46546</v>
       </c>
       <c r="K131" t="b">
@@ -5756,7 +5730,7 @@
       <c r="I132" t="s">
         <v>327</v>
       </c>
-      <c r="J132" s="2">
+      <c r="J132" s="1">
         <v>46547</v>
       </c>
       <c r="K132" t="b">
@@ -5791,7 +5765,7 @@
       <c r="I133" t="s">
         <v>327</v>
       </c>
-      <c r="J133" s="2">
+      <c r="J133" s="1">
         <v>46547</v>
       </c>
       <c r="K133" t="b">
@@ -5826,7 +5800,7 @@
       <c r="I134" t="s">
         <v>327</v>
       </c>
-      <c r="J134" s="2">
+      <c r="J134" s="1">
         <v>46547</v>
       </c>
       <c r="K134" t="b">
@@ -5861,7 +5835,7 @@
       <c r="I135" t="s">
         <v>327</v>
       </c>
-      <c r="J135" s="2">
+      <c r="J135" s="1">
         <v>46551</v>
       </c>
       <c r="K135" t="b">
@@ -5896,7 +5870,7 @@
       <c r="I136" t="s">
         <v>327</v>
       </c>
-      <c r="J136" s="2">
+      <c r="J136" s="1">
         <v>46560</v>
       </c>
       <c r="K136" t="b">
@@ -5931,7 +5905,7 @@
       <c r="I137" t="s">
         <v>327</v>
       </c>
-      <c r="J137" s="2">
+      <c r="J137" s="1">
         <v>46564</v>
       </c>
       <c r="K137" t="b">
@@ -5966,7 +5940,7 @@
       <c r="I138" t="s">
         <v>327</v>
       </c>
-      <c r="J138" s="2">
+      <c r="J138" s="1">
         <v>46567</v>
       </c>
       <c r="K138" t="b">
@@ -6001,7 +5975,7 @@
       <c r="I139" t="s">
         <v>327</v>
       </c>
-      <c r="J139" s="2">
+      <c r="J139" s="1">
         <v>46568</v>
       </c>
       <c r="K139" t="b">
@@ -6036,7 +6010,7 @@
       <c r="I140" t="s">
         <v>328</v>
       </c>
-      <c r="J140" s="2">
+      <c r="J140" s="1">
         <v>46578</v>
       </c>
       <c r="K140" t="b">
@@ -6071,7 +6045,7 @@
       <c r="I141" t="s">
         <v>328</v>
       </c>
-      <c r="J141" s="2">
+      <c r="J141" s="1">
         <v>46592</v>
       </c>
       <c r="K141" t="b">
@@ -6106,7 +6080,7 @@
       <c r="I142" t="s">
         <v>328</v>
       </c>
-      <c r="J142" s="2">
+      <c r="J142" s="1">
         <v>46592</v>
       </c>
       <c r="K142" t="b">
@@ -6141,7 +6115,7 @@
       <c r="I143" t="s">
         <v>329</v>
       </c>
-      <c r="J143" s="2">
+      <c r="J143" s="1">
         <v>46212</v>
       </c>
       <c r="K143" t="b">
@@ -6176,7 +6150,7 @@
       <c r="I144" t="s">
         <v>330</v>
       </c>
-      <c r="J144" s="2">
+      <c r="J144" s="1">
         <v>46225</v>
       </c>
       <c r="K144" t="b">
@@ -6211,7 +6185,7 @@
       <c r="I145" t="s">
         <v>331</v>
       </c>
-      <c r="J145" s="2">
+      <c r="J145" s="1">
         <v>46263</v>
       </c>
       <c r="K145" t="b">
@@ -6243,7 +6217,7 @@
       <c r="H146">
         <v>-1476</v>
       </c>
-      <c r="J146" s="2">
+      <c r="J146" s="1">
         <v>43773</v>
       </c>
       <c r="K146" t="b">
@@ -6275,7 +6249,7 @@
       <c r="H147">
         <v>-1469</v>
       </c>
-      <c r="J147" s="2">
+      <c r="J147" s="1">
         <v>43773</v>
       </c>
       <c r="K147" t="b">
@@ -6307,7 +6281,7 @@
       <c r="H148">
         <v>-1186</v>
       </c>
-      <c r="J148" s="2">
+      <c r="J148" s="1">
         <v>45295</v>
       </c>
       <c r="K148" t="b">
@@ -6339,7 +6313,7 @@
       <c r="H149">
         <v>-1048</v>
       </c>
-      <c r="J149" s="2">
+      <c r="J149" s="1">
         <v>45617</v>
       </c>
       <c r="K149" t="b">
@@ -6371,7 +6345,7 @@
       <c r="H150">
         <v>-980</v>
       </c>
-      <c r="J150" s="2">
+      <c r="J150" s="1">
         <v>45677</v>
       </c>
       <c r="K150" t="b">
@@ -6403,7 +6377,7 @@
       <c r="H151">
         <v>-961</v>
       </c>
-      <c r="J151" s="2">
+      <c r="J151" s="1">
         <v>44944</v>
       </c>
       <c r="K151" t="b">
@@ -6435,7 +6409,7 @@
       <c r="H152">
         <v>-252</v>
       </c>
-      <c r="J152" s="2">
+      <c r="J152" s="1">
         <v>46092</v>
       </c>
       <c r="K152" t="b">
@@ -6467,7 +6441,7 @@
       <c r="H153">
         <v>3</v>
       </c>
-      <c r="J153" s="2">
+      <c r="J153" s="1">
         <v>46265</v>
       </c>
       <c r="K153" t="b">
@@ -6499,7 +6473,7 @@
       <c r="H154">
         <v>3</v>
       </c>
-      <c r="J154" s="2">
+      <c r="J154" s="1">
         <v>46265</v>
       </c>
       <c r="K154" t="b">
@@ -6531,7 +6505,7 @@
       <c r="H155">
         <v>43</v>
       </c>
-      <c r="J155" s="2">
+      <c r="J155" s="1">
         <v>46440</v>
       </c>
       <c r="K155" t="b">
@@ -6563,7 +6537,7 @@
       <c r="H156">
         <v>43</v>
       </c>
-      <c r="J156" s="2">
+      <c r="J156" s="1">
         <v>46440</v>
       </c>
       <c r="K156" t="b">
@@ -6595,7 +6569,7 @@
       <c r="H157">
         <v>72</v>
       </c>
-      <c r="J157" s="2">
+      <c r="J157" s="1">
         <v>46289</v>
       </c>
       <c r="K157" t="b">
@@ -6627,7 +6601,7 @@
       <c r="H158">
         <v>72</v>
       </c>
-      <c r="J158" s="2">
+      <c r="J158" s="1">
         <v>46289</v>
       </c>
       <c r="K158" t="b">
@@ -6659,7 +6633,7 @@
       <c r="H159">
         <v>81</v>
       </c>
-      <c r="J159" s="2">
+      <c r="J159" s="1">
         <v>46405</v>
       </c>
       <c r="K159" t="b">
@@ -6691,7 +6665,7 @@
       <c r="H160">
         <v>102</v>
       </c>
-      <c r="J160" s="2">
+      <c r="J160" s="1">
         <v>46463</v>
       </c>
       <c r="K160" t="b">
@@ -6723,7 +6697,7 @@
       <c r="H161">
         <v>109</v>
       </c>
-      <c r="J161" s="2">
+      <c r="J161" s="1">
         <v>46353</v>
       </c>
       <c r="K161" t="b">
@@ -6755,7 +6729,7 @@
       <c r="H162">
         <v>127</v>
       </c>
-      <c r="J162" s="2">
+      <c r="J162" s="1">
         <v>46417</v>
       </c>
       <c r="K162" t="b">
@@ -6787,7 +6761,7 @@
       <c r="H163">
         <v>152</v>
       </c>
-      <c r="J163" s="2">
+      <c r="J163" s="1">
         <v>46271</v>
       </c>
       <c r="K163" t="b">
@@ -6819,7 +6793,7 @@
       <c r="H164">
         <v>152</v>
       </c>
-      <c r="J164" s="2">
+      <c r="J164" s="1">
         <v>46271</v>
       </c>
       <c r="K164" t="b">
@@ -6851,7 +6825,7 @@
       <c r="H165">
         <v>153</v>
       </c>
-      <c r="J165" s="2">
+      <c r="J165" s="1">
         <v>46458</v>
       </c>
       <c r="K165" t="b">
@@ -6883,7 +6857,7 @@
       <c r="H166">
         <v>158</v>
       </c>
-      <c r="J166" s="2">
+      <c r="J166" s="1">
         <v>46381</v>
       </c>
       <c r="K166" t="b">
@@ -6915,7 +6889,7 @@
       <c r="H167">
         <v>163</v>
       </c>
-      <c r="J167" s="2">
+      <c r="J167" s="1">
         <v>46592</v>
       </c>
       <c r="K167" t="b">
@@ -6947,7 +6921,7 @@
       <c r="H168">
         <v>167</v>
       </c>
-      <c r="J168" s="2">
+      <c r="J168" s="1">
         <v>46441</v>
       </c>
       <c r="K168" t="b">
@@ -6979,7 +6953,7 @@
       <c r="H169">
         <v>169</v>
       </c>
-      <c r="J169" s="2">
+      <c r="J169" s="1">
         <v>46391</v>
       </c>
       <c r="K169" t="b">
@@ -7011,7 +6985,7 @@
       <c r="H170">
         <v>184</v>
       </c>
-      <c r="J170" s="2">
+      <c r="J170" s="1">
         <v>46385</v>
       </c>
       <c r="K170" t="b">
@@ -7043,7 +7017,7 @@
       <c r="H171">
         <v>186</v>
       </c>
-      <c r="J171" s="2">
+      <c r="J171" s="1">
         <v>46387</v>
       </c>
       <c r="K171" t="b">
@@ -7075,7 +7049,7 @@
       <c r="H172">
         <v>206</v>
       </c>
-      <c r="J172" s="2">
+      <c r="J172" s="1">
         <v>46399</v>
       </c>
       <c r="K172" t="b">
@@ -7107,7 +7081,7 @@
       <c r="H173">
         <v>206</v>
       </c>
-      <c r="J173" s="2">
+      <c r="J173" s="1">
         <v>46399</v>
       </c>
       <c r="K173" t="b">
@@ -7139,7 +7113,7 @@
       <c r="H174">
         <v>234</v>
       </c>
-      <c r="J174" s="2">
+      <c r="J174" s="1">
         <v>46458</v>
       </c>
       <c r="K174" t="b">
@@ -7171,7 +7145,7 @@
       <c r="H175">
         <v>248</v>
       </c>
-      <c r="J175" s="2">
+      <c r="J175" s="1">
         <v>46528</v>
       </c>
       <c r="K175" t="b">
@@ -7203,7 +7177,7 @@
       <c r="H176">
         <v>317</v>
       </c>
-      <c r="J176" s="2">
+      <c r="J176" s="1">
         <v>46540</v>
       </c>
       <c r="K176" t="b">
@@ -7235,7 +7209,7 @@
       <c r="H177">
         <v>340</v>
       </c>
-      <c r="J177" s="2">
+      <c r="J177" s="1">
         <v>46547</v>
       </c>
       <c r="K177" t="b">
@@ -7267,7 +7241,7 @@
       <c r="H178">
         <v>364</v>
       </c>
-      <c r="J178" s="2">
+      <c r="J178" s="1">
         <v>46557</v>
       </c>
       <c r="K178" t="b">
@@ -7299,7 +7273,7 @@
       <c r="H179">
         <v>368</v>
       </c>
-      <c r="J179" s="2">
+      <c r="J179" s="1">
         <v>46571</v>
       </c>
       <c r="K179" t="b">
@@ -7331,7 +7305,7 @@
       <c r="H180">
         <v>368</v>
       </c>
-      <c r="J180" s="2">
+      <c r="J180" s="1">
         <v>46571</v>
       </c>
       <c r="K180" t="b">
@@ -7363,7 +7337,7 @@
       <c r="H181">
         <v>370</v>
       </c>
-      <c r="J181" s="2">
+      <c r="J181" s="1">
         <v>46562</v>
       </c>
       <c r="K181" t="b">
@@ -7395,7 +7369,7 @@
       <c r="H182">
         <v>385</v>
       </c>
-      <c r="J182" s="2">
+      <c r="J182" s="1">
         <v>46574</v>
       </c>
       <c r="K182" t="b">
@@ -7427,7 +7401,7 @@
       <c r="H183">
         <v>385</v>
       </c>
-      <c r="J183" s="2">
+      <c r="J183" s="1">
         <v>46574</v>
       </c>
       <c r="K183" t="b">
@@ -7459,7 +7433,7 @@
       <c r="H184">
         <v>417</v>
       </c>
-      <c r="J184" s="2">
+      <c r="J184" s="1">
         <v>46578</v>
       </c>
       <c r="K184" t="b">
@@ -7491,7 +7465,7 @@
       <c r="H185">
         <v>721</v>
       </c>
-      <c r="J185" s="2">
+      <c r="J185" s="1">
         <v>46345</v>
       </c>
       <c r="K185" t="b">
@@ -7523,7 +7497,7 @@
       <c r="H186">
         <v>721</v>
       </c>
-      <c r="J186" s="2">
+      <c r="J186" s="1">
         <v>46345</v>
       </c>
       <c r="K186" t="b">
@@ -7555,7 +7529,7 @@
       <c r="H187">
         <v>850</v>
       </c>
-      <c r="J187" s="2">
+      <c r="J187" s="1">
         <v>46366</v>
       </c>
       <c r="K187" t="b">
@@ -7587,7 +7561,7 @@
       <c r="H188">
         <v>850</v>
       </c>
-      <c r="J188" s="2">
+      <c r="J188" s="1">
         <v>46366</v>
       </c>
       <c r="K188" t="b">
@@ -7619,7 +7593,7 @@
       <c r="H189">
         <v>1661</v>
       </c>
-      <c r="J189" s="2">
+      <c r="J189" s="1">
         <v>46524</v>
       </c>
       <c r="K189" t="b">
@@ -7651,7 +7625,7 @@
       <c r="H190">
         <v>1661</v>
       </c>
-      <c r="J190" s="2">
+      <c r="J190" s="1">
         <v>46524</v>
       </c>
       <c r="K190" t="b">
@@ -7683,7 +7657,7 @@
       <c r="H191">
         <v>488</v>
       </c>
-      <c r="J191" s="2">
+      <c r="J191" s="1">
         <v>46190</v>
       </c>
       <c r="K191" t="b">
@@ -7715,7 +7689,7 @@
       <c r="H192">
         <v>25565</v>
       </c>
-      <c r="J192" s="2">
+      <c r="J192" s="1">
         <v>46190</v>
       </c>
       <c r="K192" t="b">
@@ -7747,7 +7721,7 @@
       <c r="H193">
         <v>25567</v>
       </c>
-      <c r="J193" s="2">
+      <c r="J193" s="1">
         <v>46190</v>
       </c>
       <c r="K193" t="b">
@@ -7779,7 +7753,7 @@
       <c r="H194">
         <v>31293</v>
       </c>
-      <c r="J194" s="2">
+      <c r="J194" s="1">
         <v>46190</v>
       </c>
       <c r="K194" t="b">

</xml_diff>

<commit_message>
Atualização automática: vencimentos_tmot (19/08/2026 13:07)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
@@ -1019,8 +1019,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1036,7 +1044,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1044,12 +1052,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1349,37 +1375,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1408,7 +1434,7 @@
       <c r="H2">
         <v>-4300.3</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>39285</v>
       </c>
       <c r="K2" t="b">
@@ -1440,7 +1466,7 @@
       <c r="H3">
         <v>-2354.2</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>40669</v>
       </c>
       <c r="K3" t="b">
@@ -1472,7 +1498,7 @@
       <c r="H4">
         <v>-910.7</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>40669</v>
       </c>
       <c r="K4" t="b">
@@ -1504,7 +1530,7 @@
       <c r="H5">
         <v>-868</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>44884</v>
       </c>
       <c r="K5" t="b">
@@ -1536,7 +1562,7 @@
       <c r="H6">
         <v>-483.8</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>43855</v>
       </c>
       <c r="K6" t="b">
@@ -1568,7 +1594,7 @@
       <c r="H7">
         <v>-417</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>46014</v>
       </c>
       <c r="K7" t="b">
@@ -1600,7 +1626,7 @@
       <c r="H8">
         <v>-414.2</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>46014</v>
       </c>
       <c r="K8" t="b">
@@ -1632,7 +1658,7 @@
       <c r="H9">
         <v>-391.8</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>42769</v>
       </c>
       <c r="K9" t="b">
@@ -1664,7 +1690,7 @@
       <c r="H10">
         <v>-391.6</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>45804</v>
       </c>
       <c r="K10" t="b">
@@ -1696,7 +1722,7 @@
       <c r="H11">
         <v>-391.6</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>45804</v>
       </c>
       <c r="K11" t="b">
@@ -1728,7 +1754,7 @@
       <c r="H12">
         <v>-372.9</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>42821</v>
       </c>
       <c r="K12" t="b">
@@ -1760,7 +1786,7 @@
       <c r="H13">
         <v>-372.9</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>46014</v>
       </c>
       <c r="K13" t="b">
@@ -1792,7 +1818,7 @@
       <c r="H14">
         <v>-372.9</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>46014</v>
       </c>
       <c r="K14" t="b">
@@ -1824,7 +1850,7 @@
       <c r="H15">
         <v>-372.9</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>46014</v>
       </c>
       <c r="K15" t="b">
@@ -1856,7 +1882,7 @@
       <c r="H16">
         <v>-367.8</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="2">
         <v>46017</v>
       </c>
       <c r="K16" t="b">
@@ -1888,7 +1914,7 @@
       <c r="H17">
         <v>-367.8</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="2">
         <v>46017</v>
       </c>
       <c r="K17" t="b">
@@ -1920,7 +1946,7 @@
       <c r="H18">
         <v>-347.2</v>
       </c>
-      <c r="J18" s="1">
+      <c r="J18" s="2">
         <v>40979</v>
       </c>
       <c r="K18" t="b">
@@ -1952,7 +1978,7 @@
       <c r="H19">
         <v>-293.8</v>
       </c>
-      <c r="J19" s="1">
+      <c r="J19" s="2">
         <v>45846</v>
       </c>
       <c r="K19" t="b">
@@ -1984,7 +2010,7 @@
       <c r="H20">
         <v>-206.4</v>
       </c>
-      <c r="J20" s="1">
+      <c r="J20" s="2">
         <v>36669</v>
       </c>
       <c r="K20" t="b">
@@ -2016,7 +2042,7 @@
       <c r="H21">
         <v>-131.6</v>
       </c>
-      <c r="J21" s="1">
+      <c r="J21" s="2">
         <v>46111</v>
       </c>
       <c r="K21" t="b">
@@ -2048,7 +2074,7 @@
       <c r="H22">
         <v>-131.6</v>
       </c>
-      <c r="J22" s="1">
+      <c r="J22" s="2">
         <v>46111</v>
       </c>
       <c r="K22" t="b">
@@ -2080,7 +2106,7 @@
       <c r="H23">
         <v>-131.6</v>
       </c>
-      <c r="J23" s="1">
+      <c r="J23" s="2">
         <v>46111</v>
       </c>
       <c r="K23" t="b">
@@ -2112,7 +2138,7 @@
       <c r="H24">
         <v>-131.6</v>
       </c>
-      <c r="J24" s="1">
+      <c r="J24" s="2">
         <v>46111</v>
       </c>
       <c r="K24" t="b">
@@ -2144,7 +2170,7 @@
       <c r="H25">
         <v>-131.6</v>
       </c>
-      <c r="J25" s="1">
+      <c r="J25" s="2">
         <v>46111</v>
       </c>
       <c r="K25" t="b">
@@ -2176,7 +2202,7 @@
       <c r="H26">
         <v>-98.3</v>
       </c>
-      <c r="J26" s="1">
+      <c r="J26" s="2">
         <v>41204</v>
       </c>
       <c r="K26" t="b">
@@ -2208,7 +2234,7 @@
       <c r="H27">
         <v>-47.2</v>
       </c>
-      <c r="J27" s="1">
+      <c r="J27" s="2">
         <v>44011</v>
       </c>
       <c r="K27" t="b">
@@ -2240,7 +2266,7 @@
       <c r="H28">
         <v>-22.3</v>
       </c>
-      <c r="J28" s="1">
+      <c r="J28" s="2">
         <v>46226</v>
       </c>
       <c r="K28" t="b">
@@ -2272,7 +2298,7 @@
       <c r="H29">
         <v>4.7</v>
       </c>
-      <c r="J29" s="1">
+      <c r="J29" s="2">
         <v>46265</v>
       </c>
       <c r="K29" t="b">
@@ -2304,7 +2330,7 @@
       <c r="H30">
         <v>7.5</v>
       </c>
-      <c r="J30" s="1">
+      <c r="J30" s="2">
         <v>46265</v>
       </c>
       <c r="K30" t="b">
@@ -2336,7 +2362,7 @@
       <c r="H31">
         <v>10</v>
       </c>
-      <c r="J31" s="1">
+      <c r="J31" s="2">
         <v>46265</v>
       </c>
       <c r="K31" t="b">
@@ -2368,7 +2394,7 @@
       <c r="H32">
         <v>12.8</v>
       </c>
-      <c r="J32" s="1">
+      <c r="J32" s="2">
         <v>46265</v>
       </c>
       <c r="K32" t="b">
@@ -2400,7 +2426,7 @@
       <c r="H33">
         <v>14</v>
       </c>
-      <c r="J33" s="1">
+      <c r="J33" s="2">
         <v>46265</v>
       </c>
       <c r="K33" t="b">
@@ -2432,7 +2458,7 @@
       <c r="H34">
         <v>17.8</v>
       </c>
-      <c r="J34" s="1">
+      <c r="J34" s="2">
         <v>46265</v>
       </c>
       <c r="K34" t="b">
@@ -2464,7 +2490,7 @@
       <c r="H35">
         <v>20.4</v>
       </c>
-      <c r="J35" s="1">
+      <c r="J35" s="2">
         <v>46265</v>
       </c>
       <c r="K35" t="b">
@@ -2496,7 +2522,7 @@
       <c r="H36">
         <v>21.2</v>
       </c>
-      <c r="J36" s="1">
+      <c r="J36" s="2">
         <v>46265</v>
       </c>
       <c r="K36" t="b">
@@ -2528,7 +2554,7 @@
       <c r="H37">
         <v>26.2</v>
       </c>
-      <c r="J37" s="1">
+      <c r="J37" s="2">
         <v>46265</v>
       </c>
       <c r="K37" t="b">
@@ -2560,7 +2586,7 @@
       <c r="H38">
         <v>33.6</v>
       </c>
-      <c r="J38" s="1">
+      <c r="J38" s="2">
         <v>46364</v>
       </c>
       <c r="K38" t="b">
@@ -2592,7 +2618,7 @@
       <c r="H39">
         <v>42.2</v>
       </c>
-      <c r="J39" s="1">
+      <c r="J39" s="2">
         <v>46269</v>
       </c>
       <c r="K39" t="b">
@@ -2624,7 +2650,7 @@
       <c r="H40">
         <v>42.8</v>
       </c>
-      <c r="J40" s="1">
+      <c r="J40" s="2">
         <v>46291</v>
       </c>
       <c r="K40" t="b">
@@ -2656,7 +2682,7 @@
       <c r="H41">
         <v>45.7</v>
       </c>
-      <c r="J41" s="1">
+      <c r="J41" s="2">
         <v>46395</v>
       </c>
       <c r="K41" t="b">
@@ -2688,7 +2714,7 @@
       <c r="H42">
         <v>47.2</v>
       </c>
-      <c r="J42" s="1">
+      <c r="J42" s="2">
         <v>46280</v>
       </c>
       <c r="K42" t="b">
@@ -2720,7 +2746,7 @@
       <c r="H43">
         <v>48.7</v>
       </c>
-      <c r="J43" s="1">
+      <c r="J43" s="2">
         <v>46281</v>
       </c>
       <c r="K43" t="b">
@@ -2752,7 +2778,7 @@
       <c r="H44">
         <v>60</v>
       </c>
-      <c r="J44" s="1">
+      <c r="J44" s="2">
         <v>46281</v>
       </c>
       <c r="K44" t="b">
@@ -2784,7 +2810,7 @@
       <c r="H45">
         <v>62.6</v>
       </c>
-      <c r="J45" s="1">
+      <c r="J45" s="2">
         <v>46265</v>
       </c>
       <c r="K45" t="b">
@@ -2816,7 +2842,7 @@
       <c r="H46">
         <v>64.59999999999999</v>
       </c>
-      <c r="J46" s="1">
+      <c r="J46" s="2">
         <v>46265</v>
       </c>
       <c r="K46" t="b">
@@ -2848,7 +2874,7 @@
       <c r="H47">
         <v>67.59999999999999</v>
       </c>
-      <c r="J47" s="1">
+      <c r="J47" s="2">
         <v>46267</v>
       </c>
       <c r="K47" t="b">
@@ -2880,7 +2906,7 @@
       <c r="H48">
         <v>68.3</v>
       </c>
-      <c r="J48" s="1">
+      <c r="J48" s="2">
         <v>46278</v>
       </c>
       <c r="K48" t="b">
@@ -2912,7 +2938,7 @@
       <c r="H49">
         <v>69.2</v>
       </c>
-      <c r="J49" s="1">
+      <c r="J49" s="2">
         <v>46453</v>
       </c>
       <c r="K49" t="b">
@@ -2944,7 +2970,7 @@
       <c r="H50">
         <v>69.8</v>
       </c>
-      <c r="J50" s="1">
+      <c r="J50" s="2">
         <v>46265</v>
       </c>
       <c r="K50" t="b">
@@ -2976,7 +3002,7 @@
       <c r="H51">
         <v>69.8</v>
       </c>
-      <c r="J51" s="1">
+      <c r="J51" s="2">
         <v>46265</v>
       </c>
       <c r="K51" t="b">
@@ -3008,7 +3034,7 @@
       <c r="H52">
         <v>72.2</v>
       </c>
-      <c r="J52" s="1">
+      <c r="J52" s="2">
         <v>46275</v>
       </c>
       <c r="K52" t="b">
@@ -3040,7 +3066,7 @@
       <c r="H53">
         <v>72.2</v>
       </c>
-      <c r="J53" s="1">
+      <c r="J53" s="2">
         <v>46275</v>
       </c>
       <c r="K53" t="b">
@@ -3072,7 +3098,7 @@
       <c r="H54">
         <v>78.09999999999999</v>
       </c>
-      <c r="J54" s="1">
+      <c r="J54" s="2">
         <v>46265</v>
       </c>
       <c r="K54" t="b">
@@ -3104,7 +3130,7 @@
       <c r="H55">
         <v>82.8</v>
       </c>
-      <c r="J55" s="1">
+      <c r="J55" s="2">
         <v>46487</v>
       </c>
       <c r="K55" t="b">
@@ -3136,7 +3162,7 @@
       <c r="H56">
         <v>83.09999999999999</v>
       </c>
-      <c r="J56" s="1">
+      <c r="J56" s="2">
         <v>46285</v>
       </c>
       <c r="K56" t="b">
@@ -3168,7 +3194,7 @@
       <c r="H57">
         <v>84.8</v>
       </c>
-      <c r="J57" s="1">
+      <c r="J57" s="2">
         <v>46492</v>
       </c>
       <c r="K57" t="b">
@@ -3200,7 +3226,7 @@
       <c r="H58">
         <v>104.9</v>
       </c>
-      <c r="J58" s="1">
+      <c r="J58" s="2">
         <v>46297</v>
       </c>
       <c r="K58" t="b">
@@ -3232,7 +3258,7 @@
       <c r="H59">
         <v>107.6</v>
       </c>
-      <c r="J59" s="1">
+      <c r="J59" s="2">
         <v>46283</v>
       </c>
       <c r="K59" t="b">
@@ -3264,7 +3290,7 @@
       <c r="H60">
         <v>111.9</v>
       </c>
-      <c r="J60" s="1">
+      <c r="J60" s="2">
         <v>46300</v>
       </c>
       <c r="K60" t="b">
@@ -3296,7 +3322,7 @@
       <c r="H61">
         <v>111.9</v>
       </c>
-      <c r="J61" s="1">
+      <c r="J61" s="2">
         <v>46300</v>
       </c>
       <c r="K61" t="b">
@@ -3328,7 +3354,7 @@
       <c r="H62">
         <v>111.9</v>
       </c>
-      <c r="J62" s="1">
+      <c r="J62" s="2">
         <v>46300</v>
       </c>
       <c r="K62" t="b">
@@ -3360,7 +3386,7 @@
       <c r="H63">
         <v>111.9</v>
       </c>
-      <c r="J63" s="1">
+      <c r="J63" s="2">
         <v>46300</v>
       </c>
       <c r="K63" t="b">
@@ -3392,7 +3418,7 @@
       <c r="H64">
         <v>111.9</v>
       </c>
-      <c r="J64" s="1">
+      <c r="J64" s="2">
         <v>46300</v>
       </c>
       <c r="K64" t="b">
@@ -3424,7 +3450,7 @@
       <c r="H65">
         <v>128.8</v>
       </c>
-      <c r="J65" s="1">
+      <c r="J65" s="2">
         <v>46308</v>
       </c>
       <c r="K65" t="b">
@@ -3456,7 +3482,7 @@
       <c r="H66">
         <v>131.1</v>
       </c>
-      <c r="J66" s="1">
+      <c r="J66" s="2">
         <v>46336</v>
       </c>
       <c r="K66" t="b">
@@ -3488,7 +3514,7 @@
       <c r="H67">
         <v>138.4</v>
       </c>
-      <c r="J67" s="1">
+      <c r="J67" s="2">
         <v>46343</v>
       </c>
       <c r="K67" t="b">
@@ -3520,7 +3546,7 @@
       <c r="H68">
         <v>141</v>
       </c>
-      <c r="J68" s="1">
+      <c r="J68" s="2">
         <v>46350</v>
       </c>
       <c r="K68" t="b">
@@ -3552,7 +3578,7 @@
       <c r="H69">
         <v>162</v>
       </c>
-      <c r="J69" s="1">
+      <c r="J69" s="2">
         <v>46391</v>
       </c>
       <c r="K69" t="b">
@@ -3584,7 +3610,7 @@
       <c r="H70">
         <v>167.2</v>
       </c>
-      <c r="J70" s="1">
+      <c r="J70" s="2">
         <v>46330</v>
       </c>
       <c r="K70" t="b">
@@ -3616,7 +3642,7 @@
       <c r="H71">
         <v>177.4</v>
       </c>
-      <c r="J71" s="1">
+      <c r="J71" s="2">
         <v>46418</v>
       </c>
       <c r="K71" t="b">
@@ -3648,7 +3674,7 @@
       <c r="H72">
         <v>200</v>
       </c>
-      <c r="J72" s="1">
+      <c r="J72" s="2">
         <v>46356</v>
       </c>
       <c r="K72" t="b">
@@ -3680,7 +3706,7 @@
       <c r="H73">
         <v>203.6</v>
       </c>
-      <c r="J73" s="1">
+      <c r="J73" s="2">
         <v>46436</v>
       </c>
       <c r="K73" t="b">
@@ -3712,7 +3738,7 @@
       <c r="H74">
         <v>221.2</v>
       </c>
-      <c r="J74" s="1">
+      <c r="J74" s="2">
         <v>46426</v>
       </c>
       <c r="K74" t="b">
@@ -3744,7 +3770,7 @@
       <c r="H75">
         <v>240.8</v>
       </c>
-      <c r="J75" s="1">
+      <c r="J75" s="2">
         <v>46450</v>
       </c>
       <c r="K75" t="b">
@@ -3776,7 +3802,7 @@
       <c r="H76">
         <v>245.8</v>
       </c>
-      <c r="J76" s="1">
+      <c r="J76" s="2">
         <v>46452</v>
       </c>
       <c r="K76" t="b">
@@ -3808,7 +3834,7 @@
       <c r="H77">
         <v>263.4</v>
       </c>
-      <c r="J77" s="1">
+      <c r="J77" s="2">
         <v>46322</v>
       </c>
       <c r="K77" t="b">
@@ -3840,7 +3866,7 @@
       <c r="H78">
         <v>275.2</v>
       </c>
-      <c r="J78" s="1">
+      <c r="J78" s="2">
         <v>46433</v>
       </c>
       <c r="K78" t="b">
@@ -3875,7 +3901,7 @@
       <c r="I79" t="s">
         <v>311</v>
       </c>
-      <c r="J79" s="1">
+      <c r="J79" s="2">
         <v>36557</v>
       </c>
       <c r="K79" t="b">
@@ -3910,7 +3936,7 @@
       <c r="I80" t="s">
         <v>312</v>
       </c>
-      <c r="J80" s="1">
+      <c r="J80" s="2">
         <v>41275</v>
       </c>
       <c r="K80" t="b">
@@ -3945,7 +3971,7 @@
       <c r="I81" t="s">
         <v>313</v>
       </c>
-      <c r="J81" s="1">
+      <c r="J81" s="2">
         <v>45380</v>
       </c>
       <c r="K81" t="b">
@@ -3980,7 +4006,7 @@
       <c r="I82" t="s">
         <v>314</v>
       </c>
-      <c r="J82" s="1">
+      <c r="J82" s="2">
         <v>45421</v>
       </c>
       <c r="K82" t="b">
@@ -4015,7 +4041,7 @@
       <c r="I83" t="s">
         <v>314</v>
       </c>
-      <c r="J83" s="1">
+      <c r="J83" s="2">
         <v>45428</v>
       </c>
       <c r="K83" t="b">
@@ -4050,7 +4076,7 @@
       <c r="I84" t="s">
         <v>315</v>
       </c>
-      <c r="J84" s="1">
+      <c r="J84" s="2">
         <v>45490</v>
       </c>
       <c r="K84" t="b">
@@ -4085,7 +4111,7 @@
       <c r="I85" t="s">
         <v>316</v>
       </c>
-      <c r="J85" s="1">
+      <c r="J85" s="2">
         <v>45566</v>
       </c>
       <c r="K85" t="b">
@@ -4120,7 +4146,7 @@
       <c r="I86" t="s">
         <v>317</v>
       </c>
-      <c r="J86" s="1">
+      <c r="J86" s="2">
         <v>45986</v>
       </c>
       <c r="K86" t="b">
@@ -4155,7 +4181,7 @@
       <c r="I87" t="s">
         <v>318</v>
       </c>
-      <c r="J87" s="1">
+      <c r="J87" s="2">
         <v>46284</v>
       </c>
       <c r="K87" t="b">
@@ -4190,7 +4216,7 @@
       <c r="I88" t="s">
         <v>319</v>
       </c>
-      <c r="J88" s="1">
+      <c r="J88" s="2">
         <v>46305</v>
       </c>
       <c r="K88" t="b">
@@ -4225,7 +4251,7 @@
       <c r="I89" t="s">
         <v>319</v>
       </c>
-      <c r="J89" s="1">
+      <c r="J89" s="2">
         <v>46310</v>
       </c>
       <c r="K89" t="b">
@@ -4260,7 +4286,7 @@
       <c r="I90" t="s">
         <v>319</v>
       </c>
-      <c r="J90" s="1">
+      <c r="J90" s="2">
         <v>46317</v>
       </c>
       <c r="K90" t="b">
@@ -4295,7 +4321,7 @@
       <c r="I91" t="s">
         <v>319</v>
       </c>
-      <c r="J91" s="1">
+      <c r="J91" s="2">
         <v>46319</v>
       </c>
       <c r="K91" t="b">
@@ -4330,7 +4356,7 @@
       <c r="I92" t="s">
         <v>320</v>
       </c>
-      <c r="J92" s="1">
+      <c r="J92" s="2">
         <v>46333</v>
       </c>
       <c r="K92" t="b">
@@ -4365,7 +4391,7 @@
       <c r="I93" t="s">
         <v>320</v>
       </c>
-      <c r="J93" s="1">
+      <c r="J93" s="2">
         <v>46338</v>
       </c>
       <c r="K93" t="b">
@@ -4400,7 +4426,7 @@
       <c r="I94" t="s">
         <v>320</v>
       </c>
-      <c r="J94" s="1">
+      <c r="J94" s="2">
         <v>46338</v>
       </c>
       <c r="K94" t="b">
@@ -4435,7 +4461,7 @@
       <c r="I95" t="s">
         <v>320</v>
       </c>
-      <c r="J95" s="1">
+      <c r="J95" s="2">
         <v>46341</v>
       </c>
       <c r="K95" t="b">
@@ -4470,7 +4496,7 @@
       <c r="I96" t="s">
         <v>320</v>
       </c>
-      <c r="J96" s="1">
+      <c r="J96" s="2">
         <v>46344</v>
       </c>
       <c r="K96" t="b">
@@ -4505,7 +4531,7 @@
       <c r="I97" t="s">
         <v>321</v>
       </c>
-      <c r="J97" s="1">
+      <c r="J97" s="2">
         <v>46360</v>
       </c>
       <c r="K97" t="b">
@@ -4540,7 +4566,7 @@
       <c r="I98" t="s">
         <v>321</v>
       </c>
-      <c r="J98" s="1">
+      <c r="J98" s="2">
         <v>46360</v>
       </c>
       <c r="K98" t="b">
@@ -4575,7 +4601,7 @@
       <c r="I99" t="s">
         <v>321</v>
       </c>
-      <c r="J99" s="1">
+      <c r="J99" s="2">
         <v>46367</v>
       </c>
       <c r="K99" t="b">
@@ -4610,7 +4636,7 @@
       <c r="I100" t="s">
         <v>321</v>
       </c>
-      <c r="J100" s="1">
+      <c r="J100" s="2">
         <v>46375</v>
       </c>
       <c r="K100" t="b">
@@ -4645,7 +4671,7 @@
       <c r="I101" t="s">
         <v>321</v>
       </c>
-      <c r="J101" s="1">
+      <c r="J101" s="2">
         <v>46387</v>
       </c>
       <c r="K101" t="b">
@@ -4680,7 +4706,7 @@
       <c r="I102" t="s">
         <v>321</v>
       </c>
-      <c r="J102" s="1">
+      <c r="J102" s="2">
         <v>46387</v>
       </c>
       <c r="K102" t="b">
@@ -4715,7 +4741,7 @@
       <c r="I103" t="s">
         <v>321</v>
       </c>
-      <c r="J103" s="1">
+      <c r="J103" s="2">
         <v>46387</v>
       </c>
       <c r="K103" t="b">
@@ -4750,7 +4776,7 @@
       <c r="I104" t="s">
         <v>321</v>
       </c>
-      <c r="J104" s="1">
+      <c r="J104" s="2">
         <v>46388</v>
       </c>
       <c r="K104" t="b">
@@ -4785,7 +4811,7 @@
       <c r="I105" t="s">
         <v>322</v>
       </c>
-      <c r="J105" s="1">
+      <c r="J105" s="2">
         <v>46401</v>
       </c>
       <c r="K105" t="b">
@@ -4820,7 +4846,7 @@
       <c r="I106" t="s">
         <v>322</v>
       </c>
-      <c r="J106" s="1">
+      <c r="J106" s="2">
         <v>46401</v>
       </c>
       <c r="K106" t="b">
@@ -4855,7 +4881,7 @@
       <c r="I107" t="s">
         <v>322</v>
       </c>
-      <c r="J107" s="1">
+      <c r="J107" s="2">
         <v>46401</v>
       </c>
       <c r="K107" t="b">
@@ -4890,7 +4916,7 @@
       <c r="I108" t="s">
         <v>322</v>
       </c>
-      <c r="J108" s="1">
+      <c r="J108" s="2">
         <v>46412</v>
       </c>
       <c r="K108" t="b">
@@ -4925,7 +4951,7 @@
       <c r="I109" t="s">
         <v>322</v>
       </c>
-      <c r="J109" s="1">
+      <c r="J109" s="2">
         <v>46412</v>
       </c>
       <c r="K109" t="b">
@@ -4960,7 +4986,7 @@
       <c r="I110" t="s">
         <v>322</v>
       </c>
-      <c r="J110" s="1">
+      <c r="J110" s="2">
         <v>46412</v>
       </c>
       <c r="K110" t="b">
@@ -4995,7 +5021,7 @@
       <c r="I111" t="s">
         <v>323</v>
       </c>
-      <c r="J111" s="1">
+      <c r="J111" s="2">
         <v>46424</v>
       </c>
       <c r="K111" t="b">
@@ -5030,7 +5056,7 @@
       <c r="I112" t="s">
         <v>323</v>
       </c>
-      <c r="J112" s="1">
+      <c r="J112" s="2">
         <v>46437</v>
       </c>
       <c r="K112" t="b">
@@ -5065,7 +5091,7 @@
       <c r="I113" t="s">
         <v>323</v>
       </c>
-      <c r="J113" s="1">
+      <c r="J113" s="2">
         <v>46451</v>
       </c>
       <c r="K113" t="b">
@@ -5100,7 +5126,7 @@
       <c r="I114" t="s">
         <v>323</v>
       </c>
-      <c r="J114" s="1">
+      <c r="J114" s="2">
         <v>46451</v>
       </c>
       <c r="K114" t="b">
@@ -5135,7 +5161,7 @@
       <c r="I115" t="s">
         <v>324</v>
       </c>
-      <c r="J115" s="1">
+      <c r="J115" s="2">
         <v>46455</v>
       </c>
       <c r="K115" t="b">
@@ -5170,7 +5196,7 @@
       <c r="I116" t="s">
         <v>324</v>
       </c>
-      <c r="J116" s="1">
+      <c r="J116" s="2">
         <v>46456</v>
       </c>
       <c r="K116" t="b">
@@ -5205,7 +5231,7 @@
       <c r="I117" t="s">
         <v>324</v>
       </c>
-      <c r="J117" s="1">
+      <c r="J117" s="2">
         <v>46457</v>
       </c>
       <c r="K117" t="b">
@@ -5240,7 +5266,7 @@
       <c r="I118" t="s">
         <v>324</v>
       </c>
-      <c r="J118" s="1">
+      <c r="J118" s="2">
         <v>46464</v>
       </c>
       <c r="K118" t="b">
@@ -5275,7 +5301,7 @@
       <c r="I119" t="s">
         <v>324</v>
       </c>
-      <c r="J119" s="1">
+      <c r="J119" s="2">
         <v>46470</v>
       </c>
       <c r="K119" t="b">
@@ -5310,7 +5336,7 @@
       <c r="I120" t="s">
         <v>325</v>
       </c>
-      <c r="J120" s="1">
+      <c r="J120" s="2">
         <v>46485</v>
       </c>
       <c r="K120" t="b">
@@ -5345,7 +5371,7 @@
       <c r="I121" t="s">
         <v>325</v>
       </c>
-      <c r="J121" s="1">
+      <c r="J121" s="2">
         <v>46499</v>
       </c>
       <c r="K121" t="b">
@@ -5380,7 +5406,7 @@
       <c r="I122" t="s">
         <v>325</v>
       </c>
-      <c r="J122" s="1">
+      <c r="J122" s="2">
         <v>46504</v>
       </c>
       <c r="K122" t="b">
@@ -5415,7 +5441,7 @@
       <c r="I123" t="s">
         <v>325</v>
       </c>
-      <c r="J123" s="1">
+      <c r="J123" s="2">
         <v>46504</v>
       </c>
       <c r="K123" t="b">
@@ -5450,7 +5476,7 @@
       <c r="I124" t="s">
         <v>325</v>
       </c>
-      <c r="J124" s="1">
+      <c r="J124" s="2">
         <v>46507</v>
       </c>
       <c r="K124" t="b">
@@ -5485,7 +5511,7 @@
       <c r="I125" t="s">
         <v>325</v>
       </c>
-      <c r="J125" s="1">
+      <c r="J125" s="2">
         <v>46508</v>
       </c>
       <c r="K125" t="b">
@@ -5520,7 +5546,7 @@
       <c r="I126" t="s">
         <v>325</v>
       </c>
-      <c r="J126" s="1">
+      <c r="J126" s="2">
         <v>46512</v>
       </c>
       <c r="K126" t="b">
@@ -5555,7 +5581,7 @@
       <c r="I127" t="s">
         <v>326</v>
       </c>
-      <c r="J127" s="1">
+      <c r="J127" s="2">
         <v>46512</v>
       </c>
       <c r="K127" t="b">
@@ -5590,7 +5616,7 @@
       <c r="I128" t="s">
         <v>326</v>
       </c>
-      <c r="J128" s="1">
+      <c r="J128" s="2">
         <v>46528</v>
       </c>
       <c r="K128" t="b">
@@ -5625,7 +5651,7 @@
       <c r="I129" t="s">
         <v>326</v>
       </c>
-      <c r="J129" s="1">
+      <c r="J129" s="2">
         <v>46529</v>
       </c>
       <c r="K129" t="b">
@@ -5660,7 +5686,7 @@
       <c r="I130" t="s">
         <v>326</v>
       </c>
-      <c r="J130" s="1">
+      <c r="J130" s="2">
         <v>46537</v>
       </c>
       <c r="K130" t="b">
@@ -5695,7 +5721,7 @@
       <c r="I131" t="s">
         <v>327</v>
       </c>
-      <c r="J131" s="1">
+      <c r="J131" s="2">
         <v>46546</v>
       </c>
       <c r="K131" t="b">
@@ -5730,7 +5756,7 @@
       <c r="I132" t="s">
         <v>327</v>
       </c>
-      <c r="J132" s="1">
+      <c r="J132" s="2">
         <v>46547</v>
       </c>
       <c r="K132" t="b">
@@ -5765,7 +5791,7 @@
       <c r="I133" t="s">
         <v>327</v>
       </c>
-      <c r="J133" s="1">
+      <c r="J133" s="2">
         <v>46547</v>
       </c>
       <c r="K133" t="b">
@@ -5800,7 +5826,7 @@
       <c r="I134" t="s">
         <v>327</v>
       </c>
-      <c r="J134" s="1">
+      <c r="J134" s="2">
         <v>46547</v>
       </c>
       <c r="K134" t="b">
@@ -5835,7 +5861,7 @@
       <c r="I135" t="s">
         <v>327</v>
       </c>
-      <c r="J135" s="1">
+      <c r="J135" s="2">
         <v>46551</v>
       </c>
       <c r="K135" t="b">
@@ -5870,7 +5896,7 @@
       <c r="I136" t="s">
         <v>327</v>
       </c>
-      <c r="J136" s="1">
+      <c r="J136" s="2">
         <v>46560</v>
       </c>
       <c r="K136" t="b">
@@ -5905,7 +5931,7 @@
       <c r="I137" t="s">
         <v>327</v>
       </c>
-      <c r="J137" s="1">
+      <c r="J137" s="2">
         <v>46564</v>
       </c>
       <c r="K137" t="b">
@@ -5940,7 +5966,7 @@
       <c r="I138" t="s">
         <v>327</v>
       </c>
-      <c r="J138" s="1">
+      <c r="J138" s="2">
         <v>46567</v>
       </c>
       <c r="K138" t="b">
@@ -5975,7 +6001,7 @@
       <c r="I139" t="s">
         <v>327</v>
       </c>
-      <c r="J139" s="1">
+      <c r="J139" s="2">
         <v>46568</v>
       </c>
       <c r="K139" t="b">
@@ -6010,7 +6036,7 @@
       <c r="I140" t="s">
         <v>328</v>
       </c>
-      <c r="J140" s="1">
+      <c r="J140" s="2">
         <v>46578</v>
       </c>
       <c r="K140" t="b">
@@ -6045,7 +6071,7 @@
       <c r="I141" t="s">
         <v>328</v>
       </c>
-      <c r="J141" s="1">
+      <c r="J141" s="2">
         <v>46592</v>
       </c>
       <c r="K141" t="b">
@@ -6080,7 +6106,7 @@
       <c r="I142" t="s">
         <v>328</v>
       </c>
-      <c r="J142" s="1">
+      <c r="J142" s="2">
         <v>46592</v>
       </c>
       <c r="K142" t="b">
@@ -6115,7 +6141,7 @@
       <c r="I143" t="s">
         <v>329</v>
       </c>
-      <c r="J143" s="1">
+      <c r="J143" s="2">
         <v>46212</v>
       </c>
       <c r="K143" t="b">
@@ -6150,7 +6176,7 @@
       <c r="I144" t="s">
         <v>330</v>
       </c>
-      <c r="J144" s="1">
+      <c r="J144" s="2">
         <v>46225</v>
       </c>
       <c r="K144" t="b">
@@ -6185,7 +6211,7 @@
       <c r="I145" t="s">
         <v>331</v>
       </c>
-      <c r="J145" s="1">
+      <c r="J145" s="2">
         <v>46263</v>
       </c>
       <c r="K145" t="b">
@@ -6217,7 +6243,7 @@
       <c r="H146">
         <v>-1476</v>
       </c>
-      <c r="J146" s="1">
+      <c r="J146" s="2">
         <v>43773</v>
       </c>
       <c r="K146" t="b">
@@ -6249,7 +6275,7 @@
       <c r="H147">
         <v>-1469</v>
       </c>
-      <c r="J147" s="1">
+      <c r="J147" s="2">
         <v>43773</v>
       </c>
       <c r="K147" t="b">
@@ -6281,7 +6307,7 @@
       <c r="H148">
         <v>-1186</v>
       </c>
-      <c r="J148" s="1">
+      <c r="J148" s="2">
         <v>45295</v>
       </c>
       <c r="K148" t="b">
@@ -6313,7 +6339,7 @@
       <c r="H149">
         <v>-1048</v>
       </c>
-      <c r="J149" s="1">
+      <c r="J149" s="2">
         <v>45617</v>
       </c>
       <c r="K149" t="b">
@@ -6345,7 +6371,7 @@
       <c r="H150">
         <v>-980</v>
       </c>
-      <c r="J150" s="1">
+      <c r="J150" s="2">
         <v>45677</v>
       </c>
       <c r="K150" t="b">
@@ -6377,7 +6403,7 @@
       <c r="H151">
         <v>-961</v>
       </c>
-      <c r="J151" s="1">
+      <c r="J151" s="2">
         <v>44944</v>
       </c>
       <c r="K151" t="b">
@@ -6409,7 +6435,7 @@
       <c r="H152">
         <v>-252</v>
       </c>
-      <c r="J152" s="1">
+      <c r="J152" s="2">
         <v>46092</v>
       </c>
       <c r="K152" t="b">
@@ -6441,7 +6467,7 @@
       <c r="H153">
         <v>3</v>
       </c>
-      <c r="J153" s="1">
+      <c r="J153" s="2">
         <v>46265</v>
       </c>
       <c r="K153" t="b">
@@ -6473,7 +6499,7 @@
       <c r="H154">
         <v>3</v>
       </c>
-      <c r="J154" s="1">
+      <c r="J154" s="2">
         <v>46265</v>
       </c>
       <c r="K154" t="b">
@@ -6505,7 +6531,7 @@
       <c r="H155">
         <v>43</v>
       </c>
-      <c r="J155" s="1">
+      <c r="J155" s="2">
         <v>46440</v>
       </c>
       <c r="K155" t="b">
@@ -6537,7 +6563,7 @@
       <c r="H156">
         <v>43</v>
       </c>
-      <c r="J156" s="1">
+      <c r="J156" s="2">
         <v>46440</v>
       </c>
       <c r="K156" t="b">
@@ -6569,7 +6595,7 @@
       <c r="H157">
         <v>72</v>
       </c>
-      <c r="J157" s="1">
+      <c r="J157" s="2">
         <v>46289</v>
       </c>
       <c r="K157" t="b">
@@ -6601,7 +6627,7 @@
       <c r="H158">
         <v>72</v>
       </c>
-      <c r="J158" s="1">
+      <c r="J158" s="2">
         <v>46289</v>
       </c>
       <c r="K158" t="b">
@@ -6633,7 +6659,7 @@
       <c r="H159">
         <v>81</v>
       </c>
-      <c r="J159" s="1">
+      <c r="J159" s="2">
         <v>46405</v>
       </c>
       <c r="K159" t="b">
@@ -6665,7 +6691,7 @@
       <c r="H160">
         <v>102</v>
       </c>
-      <c r="J160" s="1">
+      <c r="J160" s="2">
         <v>46463</v>
       </c>
       <c r="K160" t="b">
@@ -6697,7 +6723,7 @@
       <c r="H161">
         <v>109</v>
       </c>
-      <c r="J161" s="1">
+      <c r="J161" s="2">
         <v>46353</v>
       </c>
       <c r="K161" t="b">
@@ -6729,7 +6755,7 @@
       <c r="H162">
         <v>127</v>
       </c>
-      <c r="J162" s="1">
+      <c r="J162" s="2">
         <v>46417</v>
       </c>
       <c r="K162" t="b">
@@ -6761,7 +6787,7 @@
       <c r="H163">
         <v>152</v>
       </c>
-      <c r="J163" s="1">
+      <c r="J163" s="2">
         <v>46271</v>
       </c>
       <c r="K163" t="b">
@@ -6793,7 +6819,7 @@
       <c r="H164">
         <v>152</v>
       </c>
-      <c r="J164" s="1">
+      <c r="J164" s="2">
         <v>46271</v>
       </c>
       <c r="K164" t="b">
@@ -6825,7 +6851,7 @@
       <c r="H165">
         <v>153</v>
       </c>
-      <c r="J165" s="1">
+      <c r="J165" s="2">
         <v>46458</v>
       </c>
       <c r="K165" t="b">
@@ -6857,7 +6883,7 @@
       <c r="H166">
         <v>158</v>
       </c>
-      <c r="J166" s="1">
+      <c r="J166" s="2">
         <v>46381</v>
       </c>
       <c r="K166" t="b">
@@ -6889,7 +6915,7 @@
       <c r="H167">
         <v>163</v>
       </c>
-      <c r="J167" s="1">
+      <c r="J167" s="2">
         <v>46592</v>
       </c>
       <c r="K167" t="b">
@@ -6921,7 +6947,7 @@
       <c r="H168">
         <v>167</v>
       </c>
-      <c r="J168" s="1">
+      <c r="J168" s="2">
         <v>46441</v>
       </c>
       <c r="K168" t="b">
@@ -6953,7 +6979,7 @@
       <c r="H169">
         <v>169</v>
       </c>
-      <c r="J169" s="1">
+      <c r="J169" s="2">
         <v>46391</v>
       </c>
       <c r="K169" t="b">
@@ -6985,7 +7011,7 @@
       <c r="H170">
         <v>184</v>
       </c>
-      <c r="J170" s="1">
+      <c r="J170" s="2">
         <v>46385</v>
       </c>
       <c r="K170" t="b">
@@ -7017,7 +7043,7 @@
       <c r="H171">
         <v>186</v>
       </c>
-      <c r="J171" s="1">
+      <c r="J171" s="2">
         <v>46387</v>
       </c>
       <c r="K171" t="b">
@@ -7049,7 +7075,7 @@
       <c r="H172">
         <v>206</v>
       </c>
-      <c r="J172" s="1">
+      <c r="J172" s="2">
         <v>46399</v>
       </c>
       <c r="K172" t="b">
@@ -7081,7 +7107,7 @@
       <c r="H173">
         <v>206</v>
       </c>
-      <c r="J173" s="1">
+      <c r="J173" s="2">
         <v>46399</v>
       </c>
       <c r="K173" t="b">
@@ -7113,7 +7139,7 @@
       <c r="H174">
         <v>234</v>
       </c>
-      <c r="J174" s="1">
+      <c r="J174" s="2">
         <v>46458</v>
       </c>
       <c r="K174" t="b">
@@ -7145,7 +7171,7 @@
       <c r="H175">
         <v>248</v>
       </c>
-      <c r="J175" s="1">
+      <c r="J175" s="2">
         <v>46528</v>
       </c>
       <c r="K175" t="b">
@@ -7177,7 +7203,7 @@
       <c r="H176">
         <v>317</v>
       </c>
-      <c r="J176" s="1">
+      <c r="J176" s="2">
         <v>46540</v>
       </c>
       <c r="K176" t="b">
@@ -7209,7 +7235,7 @@
       <c r="H177">
         <v>340</v>
       </c>
-      <c r="J177" s="1">
+      <c r="J177" s="2">
         <v>46547</v>
       </c>
       <c r="K177" t="b">
@@ -7241,7 +7267,7 @@
       <c r="H178">
         <v>364</v>
       </c>
-      <c r="J178" s="1">
+      <c r="J178" s="2">
         <v>46557</v>
       </c>
       <c r="K178" t="b">
@@ -7273,7 +7299,7 @@
       <c r="H179">
         <v>368</v>
       </c>
-      <c r="J179" s="1">
+      <c r="J179" s="2">
         <v>46571</v>
       </c>
       <c r="K179" t="b">
@@ -7305,7 +7331,7 @@
       <c r="H180">
         <v>368</v>
       </c>
-      <c r="J180" s="1">
+      <c r="J180" s="2">
         <v>46571</v>
       </c>
       <c r="K180" t="b">
@@ -7337,7 +7363,7 @@
       <c r="H181">
         <v>370</v>
       </c>
-      <c r="J181" s="1">
+      <c r="J181" s="2">
         <v>46562</v>
       </c>
       <c r="K181" t="b">
@@ -7369,7 +7395,7 @@
       <c r="H182">
         <v>385</v>
       </c>
-      <c r="J182" s="1">
+      <c r="J182" s="2">
         <v>46574</v>
       </c>
       <c r="K182" t="b">
@@ -7401,7 +7427,7 @@
       <c r="H183">
         <v>385</v>
       </c>
-      <c r="J183" s="1">
+      <c r="J183" s="2">
         <v>46574</v>
       </c>
       <c r="K183" t="b">
@@ -7433,7 +7459,7 @@
       <c r="H184">
         <v>417</v>
       </c>
-      <c r="J184" s="1">
+      <c r="J184" s="2">
         <v>46578</v>
       </c>
       <c r="K184" t="b">
@@ -7465,7 +7491,7 @@
       <c r="H185">
         <v>721</v>
       </c>
-      <c r="J185" s="1">
+      <c r="J185" s="2">
         <v>46345</v>
       </c>
       <c r="K185" t="b">
@@ -7497,7 +7523,7 @@
       <c r="H186">
         <v>721</v>
       </c>
-      <c r="J186" s="1">
+      <c r="J186" s="2">
         <v>46345</v>
       </c>
       <c r="K186" t="b">
@@ -7529,7 +7555,7 @@
       <c r="H187">
         <v>850</v>
       </c>
-      <c r="J187" s="1">
+      <c r="J187" s="2">
         <v>46366</v>
       </c>
       <c r="K187" t="b">
@@ -7561,7 +7587,7 @@
       <c r="H188">
         <v>850</v>
       </c>
-      <c r="J188" s="1">
+      <c r="J188" s="2">
         <v>46366</v>
       </c>
       <c r="K188" t="b">
@@ -7593,7 +7619,7 @@
       <c r="H189">
         <v>1661</v>
       </c>
-      <c r="J189" s="1">
+      <c r="J189" s="2">
         <v>46524</v>
       </c>
       <c r="K189" t="b">
@@ -7625,7 +7651,7 @@
       <c r="H190">
         <v>1661</v>
       </c>
-      <c r="J190" s="1">
+      <c r="J190" s="2">
         <v>46524</v>
       </c>
       <c r="K190" t="b">
@@ -7657,7 +7683,7 @@
       <c r="H191">
         <v>488</v>
       </c>
-      <c r="J191" s="1">
+      <c r="J191" s="2">
         <v>46190</v>
       </c>
       <c r="K191" t="b">
@@ -7689,7 +7715,7 @@
       <c r="H192">
         <v>25565</v>
       </c>
-      <c r="J192" s="1">
+      <c r="J192" s="2">
         <v>46190</v>
       </c>
       <c r="K192" t="b">
@@ -7721,7 +7747,7 @@
       <c r="H193">
         <v>25567</v>
       </c>
-      <c r="J193" s="1">
+      <c r="J193" s="2">
         <v>46190</v>
       </c>
       <c r="K193" t="b">
@@ -7753,7 +7779,7 @@
       <c r="H194">
         <v>31293</v>
       </c>
-      <c r="J194" s="1">
+      <c r="J194" s="2">
         <v>46190</v>
       </c>
       <c r="K194" t="b">

</xml_diff>

<commit_message>
Atualização automática: vencimentos_tmot (19/08/2026 14:34)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
@@ -1019,16 +1019,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1044,7 +1036,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1052,30 +1044,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1375,37 +1349,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1434,7 +1408,7 @@
       <c r="H2">
         <v>-4300.3</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>39285</v>
       </c>
       <c r="K2" t="b">
@@ -1466,7 +1440,7 @@
       <c r="H3">
         <v>-2354.2</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>40669</v>
       </c>
       <c r="K3" t="b">
@@ -1498,7 +1472,7 @@
       <c r="H4">
         <v>-910.7</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>40669</v>
       </c>
       <c r="K4" t="b">
@@ -1530,7 +1504,7 @@
       <c r="H5">
         <v>-868</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>44884</v>
       </c>
       <c r="K5" t="b">
@@ -1562,7 +1536,7 @@
       <c r="H6">
         <v>-483.8</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>43855</v>
       </c>
       <c r="K6" t="b">
@@ -1594,7 +1568,7 @@
       <c r="H7">
         <v>-417</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>46014</v>
       </c>
       <c r="K7" t="b">
@@ -1626,7 +1600,7 @@
       <c r="H8">
         <v>-414.2</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>46014</v>
       </c>
       <c r="K8" t="b">
@@ -1658,7 +1632,7 @@
       <c r="H9">
         <v>-391.8</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>42769</v>
       </c>
       <c r="K9" t="b">
@@ -1690,7 +1664,7 @@
       <c r="H10">
         <v>-391.6</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>45804</v>
       </c>
       <c r="K10" t="b">
@@ -1722,7 +1696,7 @@
       <c r="H11">
         <v>-391.6</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>45804</v>
       </c>
       <c r="K11" t="b">
@@ -1754,7 +1728,7 @@
       <c r="H12">
         <v>-372.9</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>42821</v>
       </c>
       <c r="K12" t="b">
@@ -1786,7 +1760,7 @@
       <c r="H13">
         <v>-372.9</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>46014</v>
       </c>
       <c r="K13" t="b">
@@ -1818,7 +1792,7 @@
       <c r="H14">
         <v>-372.9</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>46014</v>
       </c>
       <c r="K14" t="b">
@@ -1850,7 +1824,7 @@
       <c r="H15">
         <v>-372.9</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <v>46014</v>
       </c>
       <c r="K15" t="b">
@@ -1882,7 +1856,7 @@
       <c r="H16">
         <v>-367.8</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <v>46017</v>
       </c>
       <c r="K16" t="b">
@@ -1914,7 +1888,7 @@
       <c r="H17">
         <v>-367.8</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="1">
         <v>46017</v>
       </c>
       <c r="K17" t="b">
@@ -1946,7 +1920,7 @@
       <c r="H18">
         <v>-347.2</v>
       </c>
-      <c r="J18" s="2">
+      <c r="J18" s="1">
         <v>40979</v>
       </c>
       <c r="K18" t="b">
@@ -1978,7 +1952,7 @@
       <c r="H19">
         <v>-293.8</v>
       </c>
-      <c r="J19" s="2">
+      <c r="J19" s="1">
         <v>45846</v>
       </c>
       <c r="K19" t="b">
@@ -2010,7 +1984,7 @@
       <c r="H20">
         <v>-206.4</v>
       </c>
-      <c r="J20" s="2">
+      <c r="J20" s="1">
         <v>36669</v>
       </c>
       <c r="K20" t="b">
@@ -2042,7 +2016,7 @@
       <c r="H21">
         <v>-131.6</v>
       </c>
-      <c r="J21" s="2">
+      <c r="J21" s="1">
         <v>46111</v>
       </c>
       <c r="K21" t="b">
@@ -2074,7 +2048,7 @@
       <c r="H22">
         <v>-131.6</v>
       </c>
-      <c r="J22" s="2">
+      <c r="J22" s="1">
         <v>46111</v>
       </c>
       <c r="K22" t="b">
@@ -2106,7 +2080,7 @@
       <c r="H23">
         <v>-131.6</v>
       </c>
-      <c r="J23" s="2">
+      <c r="J23" s="1">
         <v>46111</v>
       </c>
       <c r="K23" t="b">
@@ -2138,7 +2112,7 @@
       <c r="H24">
         <v>-131.6</v>
       </c>
-      <c r="J24" s="2">
+      <c r="J24" s="1">
         <v>46111</v>
       </c>
       <c r="K24" t="b">
@@ -2170,7 +2144,7 @@
       <c r="H25">
         <v>-131.6</v>
       </c>
-      <c r="J25" s="2">
+      <c r="J25" s="1">
         <v>46111</v>
       </c>
       <c r="K25" t="b">
@@ -2202,7 +2176,7 @@
       <c r="H26">
         <v>-98.3</v>
       </c>
-      <c r="J26" s="2">
+      <c r="J26" s="1">
         <v>41204</v>
       </c>
       <c r="K26" t="b">
@@ -2234,7 +2208,7 @@
       <c r="H27">
         <v>-47.2</v>
       </c>
-      <c r="J27" s="2">
+      <c r="J27" s="1">
         <v>44011</v>
       </c>
       <c r="K27" t="b">
@@ -2266,7 +2240,7 @@
       <c r="H28">
         <v>-22.3</v>
       </c>
-      <c r="J28" s="2">
+      <c r="J28" s="1">
         <v>46226</v>
       </c>
       <c r="K28" t="b">
@@ -2298,7 +2272,7 @@
       <c r="H29">
         <v>4.7</v>
       </c>
-      <c r="J29" s="2">
+      <c r="J29" s="1">
         <v>46265</v>
       </c>
       <c r="K29" t="b">
@@ -2330,7 +2304,7 @@
       <c r="H30">
         <v>7.5</v>
       </c>
-      <c r="J30" s="2">
+      <c r="J30" s="1">
         <v>46265</v>
       </c>
       <c r="K30" t="b">
@@ -2362,7 +2336,7 @@
       <c r="H31">
         <v>10</v>
       </c>
-      <c r="J31" s="2">
+      <c r="J31" s="1">
         <v>46265</v>
       </c>
       <c r="K31" t="b">
@@ -2394,7 +2368,7 @@
       <c r="H32">
         <v>12.8</v>
       </c>
-      <c r="J32" s="2">
+      <c r="J32" s="1">
         <v>46265</v>
       </c>
       <c r="K32" t="b">
@@ -2426,7 +2400,7 @@
       <c r="H33">
         <v>14</v>
       </c>
-      <c r="J33" s="2">
+      <c r="J33" s="1">
         <v>46265</v>
       </c>
       <c r="K33" t="b">
@@ -2458,7 +2432,7 @@
       <c r="H34">
         <v>17.8</v>
       </c>
-      <c r="J34" s="2">
+      <c r="J34" s="1">
         <v>46265</v>
       </c>
       <c r="K34" t="b">
@@ -2490,7 +2464,7 @@
       <c r="H35">
         <v>20.4</v>
       </c>
-      <c r="J35" s="2">
+      <c r="J35" s="1">
         <v>46265</v>
       </c>
       <c r="K35" t="b">
@@ -2522,7 +2496,7 @@
       <c r="H36">
         <v>21.2</v>
       </c>
-      <c r="J36" s="2">
+      <c r="J36" s="1">
         <v>46265</v>
       </c>
       <c r="K36" t="b">
@@ -2554,7 +2528,7 @@
       <c r="H37">
         <v>26.2</v>
       </c>
-      <c r="J37" s="2">
+      <c r="J37" s="1">
         <v>46265</v>
       </c>
       <c r="K37" t="b">
@@ -2586,7 +2560,7 @@
       <c r="H38">
         <v>33.6</v>
       </c>
-      <c r="J38" s="2">
+      <c r="J38" s="1">
         <v>46364</v>
       </c>
       <c r="K38" t="b">
@@ -2618,7 +2592,7 @@
       <c r="H39">
         <v>42.2</v>
       </c>
-      <c r="J39" s="2">
+      <c r="J39" s="1">
         <v>46269</v>
       </c>
       <c r="K39" t="b">
@@ -2650,7 +2624,7 @@
       <c r="H40">
         <v>42.8</v>
       </c>
-      <c r="J40" s="2">
+      <c r="J40" s="1">
         <v>46291</v>
       </c>
       <c r="K40" t="b">
@@ -2682,7 +2656,7 @@
       <c r="H41">
         <v>45.7</v>
       </c>
-      <c r="J41" s="2">
+      <c r="J41" s="1">
         <v>46395</v>
       </c>
       <c r="K41" t="b">
@@ -2714,7 +2688,7 @@
       <c r="H42">
         <v>47.2</v>
       </c>
-      <c r="J42" s="2">
+      <c r="J42" s="1">
         <v>46280</v>
       </c>
       <c r="K42" t="b">
@@ -2746,7 +2720,7 @@
       <c r="H43">
         <v>48.7</v>
       </c>
-      <c r="J43" s="2">
+      <c r="J43" s="1">
         <v>46281</v>
       </c>
       <c r="K43" t="b">
@@ -2778,7 +2752,7 @@
       <c r="H44">
         <v>60</v>
       </c>
-      <c r="J44" s="2">
+      <c r="J44" s="1">
         <v>46281</v>
       </c>
       <c r="K44" t="b">
@@ -2810,7 +2784,7 @@
       <c r="H45">
         <v>62.6</v>
       </c>
-      <c r="J45" s="2">
+      <c r="J45" s="1">
         <v>46265</v>
       </c>
       <c r="K45" t="b">
@@ -2842,7 +2816,7 @@
       <c r="H46">
         <v>64.59999999999999</v>
       </c>
-      <c r="J46" s="2">
+      <c r="J46" s="1">
         <v>46265</v>
       </c>
       <c r="K46" t="b">
@@ -2874,7 +2848,7 @@
       <c r="H47">
         <v>67.59999999999999</v>
       </c>
-      <c r="J47" s="2">
+      <c r="J47" s="1">
         <v>46267</v>
       </c>
       <c r="K47" t="b">
@@ -2906,7 +2880,7 @@
       <c r="H48">
         <v>68.3</v>
       </c>
-      <c r="J48" s="2">
+      <c r="J48" s="1">
         <v>46278</v>
       </c>
       <c r="K48" t="b">
@@ -2938,7 +2912,7 @@
       <c r="H49">
         <v>69.2</v>
       </c>
-      <c r="J49" s="2">
+      <c r="J49" s="1">
         <v>46453</v>
       </c>
       <c r="K49" t="b">
@@ -2970,7 +2944,7 @@
       <c r="H50">
         <v>69.8</v>
       </c>
-      <c r="J50" s="2">
+      <c r="J50" s="1">
         <v>46265</v>
       </c>
       <c r="K50" t="b">
@@ -3002,7 +2976,7 @@
       <c r="H51">
         <v>69.8</v>
       </c>
-      <c r="J51" s="2">
+      <c r="J51" s="1">
         <v>46265</v>
       </c>
       <c r="K51" t="b">
@@ -3034,7 +3008,7 @@
       <c r="H52">
         <v>72.2</v>
       </c>
-      <c r="J52" s="2">
+      <c r="J52" s="1">
         <v>46275</v>
       </c>
       <c r="K52" t="b">
@@ -3066,7 +3040,7 @@
       <c r="H53">
         <v>72.2</v>
       </c>
-      <c r="J53" s="2">
+      <c r="J53" s="1">
         <v>46275</v>
       </c>
       <c r="K53" t="b">
@@ -3098,7 +3072,7 @@
       <c r="H54">
         <v>78.09999999999999</v>
       </c>
-      <c r="J54" s="2">
+      <c r="J54" s="1">
         <v>46265</v>
       </c>
       <c r="K54" t="b">
@@ -3130,7 +3104,7 @@
       <c r="H55">
         <v>82.8</v>
       </c>
-      <c r="J55" s="2">
+      <c r="J55" s="1">
         <v>46487</v>
       </c>
       <c r="K55" t="b">
@@ -3162,7 +3136,7 @@
       <c r="H56">
         <v>83.09999999999999</v>
       </c>
-      <c r="J56" s="2">
+      <c r="J56" s="1">
         <v>46285</v>
       </c>
       <c r="K56" t="b">
@@ -3194,7 +3168,7 @@
       <c r="H57">
         <v>84.8</v>
       </c>
-      <c r="J57" s="2">
+      <c r="J57" s="1">
         <v>46492</v>
       </c>
       <c r="K57" t="b">
@@ -3226,7 +3200,7 @@
       <c r="H58">
         <v>104.9</v>
       </c>
-      <c r="J58" s="2">
+      <c r="J58" s="1">
         <v>46297</v>
       </c>
       <c r="K58" t="b">
@@ -3258,7 +3232,7 @@
       <c r="H59">
         <v>107.6</v>
       </c>
-      <c r="J59" s="2">
+      <c r="J59" s="1">
         <v>46283</v>
       </c>
       <c r="K59" t="b">
@@ -3290,7 +3264,7 @@
       <c r="H60">
         <v>111.9</v>
       </c>
-      <c r="J60" s="2">
+      <c r="J60" s="1">
         <v>46300</v>
       </c>
       <c r="K60" t="b">
@@ -3322,7 +3296,7 @@
       <c r="H61">
         <v>111.9</v>
       </c>
-      <c r="J61" s="2">
+      <c r="J61" s="1">
         <v>46300</v>
       </c>
       <c r="K61" t="b">
@@ -3354,7 +3328,7 @@
       <c r="H62">
         <v>111.9</v>
       </c>
-      <c r="J62" s="2">
+      <c r="J62" s="1">
         <v>46300</v>
       </c>
       <c r="K62" t="b">
@@ -3386,7 +3360,7 @@
       <c r="H63">
         <v>111.9</v>
       </c>
-      <c r="J63" s="2">
+      <c r="J63" s="1">
         <v>46300</v>
       </c>
       <c r="K63" t="b">
@@ -3418,7 +3392,7 @@
       <c r="H64">
         <v>111.9</v>
       </c>
-      <c r="J64" s="2">
+      <c r="J64" s="1">
         <v>46300</v>
       </c>
       <c r="K64" t="b">
@@ -3450,7 +3424,7 @@
       <c r="H65">
         <v>128.8</v>
       </c>
-      <c r="J65" s="2">
+      <c r="J65" s="1">
         <v>46308</v>
       </c>
       <c r="K65" t="b">
@@ -3482,7 +3456,7 @@
       <c r="H66">
         <v>131.1</v>
       </c>
-      <c r="J66" s="2">
+      <c r="J66" s="1">
         <v>46336</v>
       </c>
       <c r="K66" t="b">
@@ -3514,7 +3488,7 @@
       <c r="H67">
         <v>138.4</v>
       </c>
-      <c r="J67" s="2">
+      <c r="J67" s="1">
         <v>46343</v>
       </c>
       <c r="K67" t="b">
@@ -3546,7 +3520,7 @@
       <c r="H68">
         <v>141</v>
       </c>
-      <c r="J68" s="2">
+      <c r="J68" s="1">
         <v>46350</v>
       </c>
       <c r="K68" t="b">
@@ -3578,7 +3552,7 @@
       <c r="H69">
         <v>162</v>
       </c>
-      <c r="J69" s="2">
+      <c r="J69" s="1">
         <v>46391</v>
       </c>
       <c r="K69" t="b">
@@ -3610,7 +3584,7 @@
       <c r="H70">
         <v>167.2</v>
       </c>
-      <c r="J70" s="2">
+      <c r="J70" s="1">
         <v>46330</v>
       </c>
       <c r="K70" t="b">
@@ -3642,7 +3616,7 @@
       <c r="H71">
         <v>177.4</v>
       </c>
-      <c r="J71" s="2">
+      <c r="J71" s="1">
         <v>46418</v>
       </c>
       <c r="K71" t="b">
@@ -3674,7 +3648,7 @@
       <c r="H72">
         <v>200</v>
       </c>
-      <c r="J72" s="2">
+      <c r="J72" s="1">
         <v>46356</v>
       </c>
       <c r="K72" t="b">
@@ -3706,7 +3680,7 @@
       <c r="H73">
         <v>203.6</v>
       </c>
-      <c r="J73" s="2">
+      <c r="J73" s="1">
         <v>46436</v>
       </c>
       <c r="K73" t="b">
@@ -3738,7 +3712,7 @@
       <c r="H74">
         <v>221.2</v>
       </c>
-      <c r="J74" s="2">
+      <c r="J74" s="1">
         <v>46426</v>
       </c>
       <c r="K74" t="b">
@@ -3770,7 +3744,7 @@
       <c r="H75">
         <v>240.8</v>
       </c>
-      <c r="J75" s="2">
+      <c r="J75" s="1">
         <v>46450</v>
       </c>
       <c r="K75" t="b">
@@ -3802,7 +3776,7 @@
       <c r="H76">
         <v>245.8</v>
       </c>
-      <c r="J76" s="2">
+      <c r="J76" s="1">
         <v>46452</v>
       </c>
       <c r="K76" t="b">
@@ -3834,7 +3808,7 @@
       <c r="H77">
         <v>263.4</v>
       </c>
-      <c r="J77" s="2">
+      <c r="J77" s="1">
         <v>46322</v>
       </c>
       <c r="K77" t="b">
@@ -3866,7 +3840,7 @@
       <c r="H78">
         <v>275.2</v>
       </c>
-      <c r="J78" s="2">
+      <c r="J78" s="1">
         <v>46433</v>
       </c>
       <c r="K78" t="b">
@@ -3901,7 +3875,7 @@
       <c r="I79" t="s">
         <v>311</v>
       </c>
-      <c r="J79" s="2">
+      <c r="J79" s="1">
         <v>36557</v>
       </c>
       <c r="K79" t="b">
@@ -3936,7 +3910,7 @@
       <c r="I80" t="s">
         <v>312</v>
       </c>
-      <c r="J80" s="2">
+      <c r="J80" s="1">
         <v>41275</v>
       </c>
       <c r="K80" t="b">
@@ -3971,7 +3945,7 @@
       <c r="I81" t="s">
         <v>313</v>
       </c>
-      <c r="J81" s="2">
+      <c r="J81" s="1">
         <v>45380</v>
       </c>
       <c r="K81" t="b">
@@ -4006,7 +3980,7 @@
       <c r="I82" t="s">
         <v>314</v>
       </c>
-      <c r="J82" s="2">
+      <c r="J82" s="1">
         <v>45421</v>
       </c>
       <c r="K82" t="b">
@@ -4041,7 +4015,7 @@
       <c r="I83" t="s">
         <v>314</v>
       </c>
-      <c r="J83" s="2">
+      <c r="J83" s="1">
         <v>45428</v>
       </c>
       <c r="K83" t="b">
@@ -4076,7 +4050,7 @@
       <c r="I84" t="s">
         <v>315</v>
       </c>
-      <c r="J84" s="2">
+      <c r="J84" s="1">
         <v>45490</v>
       </c>
       <c r="K84" t="b">
@@ -4111,7 +4085,7 @@
       <c r="I85" t="s">
         <v>316</v>
       </c>
-      <c r="J85" s="2">
+      <c r="J85" s="1">
         <v>45566</v>
       </c>
       <c r="K85" t="b">
@@ -4146,7 +4120,7 @@
       <c r="I86" t="s">
         <v>317</v>
       </c>
-      <c r="J86" s="2">
+      <c r="J86" s="1">
         <v>45986</v>
       </c>
       <c r="K86" t="b">
@@ -4181,7 +4155,7 @@
       <c r="I87" t="s">
         <v>318</v>
       </c>
-      <c r="J87" s="2">
+      <c r="J87" s="1">
         <v>46284</v>
       </c>
       <c r="K87" t="b">
@@ -4216,7 +4190,7 @@
       <c r="I88" t="s">
         <v>319</v>
       </c>
-      <c r="J88" s="2">
+      <c r="J88" s="1">
         <v>46305</v>
       </c>
       <c r="K88" t="b">
@@ -4251,7 +4225,7 @@
       <c r="I89" t="s">
         <v>319</v>
       </c>
-      <c r="J89" s="2">
+      <c r="J89" s="1">
         <v>46310</v>
       </c>
       <c r="K89" t="b">
@@ -4286,7 +4260,7 @@
       <c r="I90" t="s">
         <v>319</v>
       </c>
-      <c r="J90" s="2">
+      <c r="J90" s="1">
         <v>46317</v>
       </c>
       <c r="K90" t="b">
@@ -4321,7 +4295,7 @@
       <c r="I91" t="s">
         <v>319</v>
       </c>
-      <c r="J91" s="2">
+      <c r="J91" s="1">
         <v>46319</v>
       </c>
       <c r="K91" t="b">
@@ -4356,7 +4330,7 @@
       <c r="I92" t="s">
         <v>320</v>
       </c>
-      <c r="J92" s="2">
+      <c r="J92" s="1">
         <v>46333</v>
       </c>
       <c r="K92" t="b">
@@ -4391,7 +4365,7 @@
       <c r="I93" t="s">
         <v>320</v>
       </c>
-      <c r="J93" s="2">
+      <c r="J93" s="1">
         <v>46338</v>
       </c>
       <c r="K93" t="b">
@@ -4426,7 +4400,7 @@
       <c r="I94" t="s">
         <v>320</v>
       </c>
-      <c r="J94" s="2">
+      <c r="J94" s="1">
         <v>46338</v>
       </c>
       <c r="K94" t="b">
@@ -4461,7 +4435,7 @@
       <c r="I95" t="s">
         <v>320</v>
       </c>
-      <c r="J95" s="2">
+      <c r="J95" s="1">
         <v>46341</v>
       </c>
       <c r="K95" t="b">
@@ -4496,7 +4470,7 @@
       <c r="I96" t="s">
         <v>320</v>
       </c>
-      <c r="J96" s="2">
+      <c r="J96" s="1">
         <v>46344</v>
       </c>
       <c r="K96" t="b">
@@ -4531,7 +4505,7 @@
       <c r="I97" t="s">
         <v>321</v>
       </c>
-      <c r="J97" s="2">
+      <c r="J97" s="1">
         <v>46360</v>
       </c>
       <c r="K97" t="b">
@@ -4566,7 +4540,7 @@
       <c r="I98" t="s">
         <v>321</v>
       </c>
-      <c r="J98" s="2">
+      <c r="J98" s="1">
         <v>46360</v>
       </c>
       <c r="K98" t="b">
@@ -4601,7 +4575,7 @@
       <c r="I99" t="s">
         <v>321</v>
       </c>
-      <c r="J99" s="2">
+      <c r="J99" s="1">
         <v>46367</v>
       </c>
       <c r="K99" t="b">
@@ -4636,7 +4610,7 @@
       <c r="I100" t="s">
         <v>321</v>
       </c>
-      <c r="J100" s="2">
+      <c r="J100" s="1">
         <v>46375</v>
       </c>
       <c r="K100" t="b">
@@ -4671,7 +4645,7 @@
       <c r="I101" t="s">
         <v>321</v>
       </c>
-      <c r="J101" s="2">
+      <c r="J101" s="1">
         <v>46387</v>
       </c>
       <c r="K101" t="b">
@@ -4706,7 +4680,7 @@
       <c r="I102" t="s">
         <v>321</v>
       </c>
-      <c r="J102" s="2">
+      <c r="J102" s="1">
         <v>46387</v>
       </c>
       <c r="K102" t="b">
@@ -4741,7 +4715,7 @@
       <c r="I103" t="s">
         <v>321</v>
       </c>
-      <c r="J103" s="2">
+      <c r="J103" s="1">
         <v>46387</v>
       </c>
       <c r="K103" t="b">
@@ -4776,7 +4750,7 @@
       <c r="I104" t="s">
         <v>321</v>
       </c>
-      <c r="J104" s="2">
+      <c r="J104" s="1">
         <v>46388</v>
       </c>
       <c r="K104" t="b">
@@ -4811,7 +4785,7 @@
       <c r="I105" t="s">
         <v>322</v>
       </c>
-      <c r="J105" s="2">
+      <c r="J105" s="1">
         <v>46401</v>
       </c>
       <c r="K105" t="b">
@@ -4846,7 +4820,7 @@
       <c r="I106" t="s">
         <v>322</v>
       </c>
-      <c r="J106" s="2">
+      <c r="J106" s="1">
         <v>46401</v>
       </c>
       <c r="K106" t="b">
@@ -4881,7 +4855,7 @@
       <c r="I107" t="s">
         <v>322</v>
       </c>
-      <c r="J107" s="2">
+      <c r="J107" s="1">
         <v>46401</v>
       </c>
       <c r="K107" t="b">
@@ -4916,7 +4890,7 @@
       <c r="I108" t="s">
         <v>322</v>
       </c>
-      <c r="J108" s="2">
+      <c r="J108" s="1">
         <v>46412</v>
       </c>
       <c r="K108" t="b">
@@ -4951,7 +4925,7 @@
       <c r="I109" t="s">
         <v>322</v>
       </c>
-      <c r="J109" s="2">
+      <c r="J109" s="1">
         <v>46412</v>
       </c>
       <c r="K109" t="b">
@@ -4986,7 +4960,7 @@
       <c r="I110" t="s">
         <v>322</v>
       </c>
-      <c r="J110" s="2">
+      <c r="J110" s="1">
         <v>46412</v>
       </c>
       <c r="K110" t="b">
@@ -5021,7 +4995,7 @@
       <c r="I111" t="s">
         <v>323</v>
       </c>
-      <c r="J111" s="2">
+      <c r="J111" s="1">
         <v>46424</v>
       </c>
       <c r="K111" t="b">
@@ -5056,7 +5030,7 @@
       <c r="I112" t="s">
         <v>323</v>
       </c>
-      <c r="J112" s="2">
+      <c r="J112" s="1">
         <v>46437</v>
       </c>
       <c r="K112" t="b">
@@ -5091,7 +5065,7 @@
       <c r="I113" t="s">
         <v>323</v>
       </c>
-      <c r="J113" s="2">
+      <c r="J113" s="1">
         <v>46451</v>
       </c>
       <c r="K113" t="b">
@@ -5126,7 +5100,7 @@
       <c r="I114" t="s">
         <v>323</v>
       </c>
-      <c r="J114" s="2">
+      <c r="J114" s="1">
         <v>46451</v>
       </c>
       <c r="K114" t="b">
@@ -5161,7 +5135,7 @@
       <c r="I115" t="s">
         <v>324</v>
       </c>
-      <c r="J115" s="2">
+      <c r="J115" s="1">
         <v>46455</v>
       </c>
       <c r="K115" t="b">
@@ -5196,7 +5170,7 @@
       <c r="I116" t="s">
         <v>324</v>
       </c>
-      <c r="J116" s="2">
+      <c r="J116" s="1">
         <v>46456</v>
       </c>
       <c r="K116" t="b">
@@ -5231,7 +5205,7 @@
       <c r="I117" t="s">
         <v>324</v>
       </c>
-      <c r="J117" s="2">
+      <c r="J117" s="1">
         <v>46457</v>
       </c>
       <c r="K117" t="b">
@@ -5266,7 +5240,7 @@
       <c r="I118" t="s">
         <v>324</v>
       </c>
-      <c r="J118" s="2">
+      <c r="J118" s="1">
         <v>46464</v>
       </c>
       <c r="K118" t="b">
@@ -5301,7 +5275,7 @@
       <c r="I119" t="s">
         <v>324</v>
       </c>
-      <c r="J119" s="2">
+      <c r="J119" s="1">
         <v>46470</v>
       </c>
       <c r="K119" t="b">
@@ -5336,7 +5310,7 @@
       <c r="I120" t="s">
         <v>325</v>
       </c>
-      <c r="J120" s="2">
+      <c r="J120" s="1">
         <v>46485</v>
       </c>
       <c r="K120" t="b">
@@ -5371,7 +5345,7 @@
       <c r="I121" t="s">
         <v>325</v>
       </c>
-      <c r="J121" s="2">
+      <c r="J121" s="1">
         <v>46499</v>
       </c>
       <c r="K121" t="b">
@@ -5406,7 +5380,7 @@
       <c r="I122" t="s">
         <v>325</v>
       </c>
-      <c r="J122" s="2">
+      <c r="J122" s="1">
         <v>46504</v>
       </c>
       <c r="K122" t="b">
@@ -5441,7 +5415,7 @@
       <c r="I123" t="s">
         <v>325</v>
       </c>
-      <c r="J123" s="2">
+      <c r="J123" s="1">
         <v>46504</v>
       </c>
       <c r="K123" t="b">
@@ -5476,7 +5450,7 @@
       <c r="I124" t="s">
         <v>325</v>
       </c>
-      <c r="J124" s="2">
+      <c r="J124" s="1">
         <v>46507</v>
       </c>
       <c r="K124" t="b">
@@ -5511,7 +5485,7 @@
       <c r="I125" t="s">
         <v>325</v>
       </c>
-      <c r="J125" s="2">
+      <c r="J125" s="1">
         <v>46508</v>
       </c>
       <c r="K125" t="b">
@@ -5546,7 +5520,7 @@
       <c r="I126" t="s">
         <v>325</v>
       </c>
-      <c r="J126" s="2">
+      <c r="J126" s="1">
         <v>46512</v>
       </c>
       <c r="K126" t="b">
@@ -5581,7 +5555,7 @@
       <c r="I127" t="s">
         <v>326</v>
       </c>
-      <c r="J127" s="2">
+      <c r="J127" s="1">
         <v>46512</v>
       </c>
       <c r="K127" t="b">
@@ -5616,7 +5590,7 @@
       <c r="I128" t="s">
         <v>326</v>
       </c>
-      <c r="J128" s="2">
+      <c r="J128" s="1">
         <v>46528</v>
       </c>
       <c r="K128" t="b">
@@ -5651,7 +5625,7 @@
       <c r="I129" t="s">
         <v>326</v>
       </c>
-      <c r="J129" s="2">
+      <c r="J129" s="1">
         <v>46529</v>
       </c>
       <c r="K129" t="b">
@@ -5686,7 +5660,7 @@
       <c r="I130" t="s">
         <v>326</v>
       </c>
-      <c r="J130" s="2">
+      <c r="J130" s="1">
         <v>46537</v>
       </c>
       <c r="K130" t="b">
@@ -5721,7 +5695,7 @@
       <c r="I131" t="s">
         <v>327</v>
       </c>
-      <c r="J131" s="2">
+      <c r="J131" s="1">
         <v>46546</v>
       </c>
       <c r="K131" t="b">
@@ -5756,7 +5730,7 @@
       <c r="I132" t="s">
         <v>327</v>
       </c>
-      <c r="J132" s="2">
+      <c r="J132" s="1">
         <v>46547</v>
       </c>
       <c r="K132" t="b">
@@ -5791,7 +5765,7 @@
       <c r="I133" t="s">
         <v>327</v>
       </c>
-      <c r="J133" s="2">
+      <c r="J133" s="1">
         <v>46547</v>
       </c>
       <c r="K133" t="b">
@@ -5826,7 +5800,7 @@
       <c r="I134" t="s">
         <v>327</v>
       </c>
-      <c r="J134" s="2">
+      <c r="J134" s="1">
         <v>46547</v>
       </c>
       <c r="K134" t="b">
@@ -5861,7 +5835,7 @@
       <c r="I135" t="s">
         <v>327</v>
       </c>
-      <c r="J135" s="2">
+      <c r="J135" s="1">
         <v>46551</v>
       </c>
       <c r="K135" t="b">
@@ -5896,7 +5870,7 @@
       <c r="I136" t="s">
         <v>327</v>
       </c>
-      <c r="J136" s="2">
+      <c r="J136" s="1">
         <v>46560</v>
       </c>
       <c r="K136" t="b">
@@ -5931,7 +5905,7 @@
       <c r="I137" t="s">
         <v>327</v>
       </c>
-      <c r="J137" s="2">
+      <c r="J137" s="1">
         <v>46564</v>
       </c>
       <c r="K137" t="b">
@@ -5966,7 +5940,7 @@
       <c r="I138" t="s">
         <v>327</v>
       </c>
-      <c r="J138" s="2">
+      <c r="J138" s="1">
         <v>46567</v>
       </c>
       <c r="K138" t="b">
@@ -6001,7 +5975,7 @@
       <c r="I139" t="s">
         <v>327</v>
       </c>
-      <c r="J139" s="2">
+      <c r="J139" s="1">
         <v>46568</v>
       </c>
       <c r="K139" t="b">
@@ -6036,7 +6010,7 @@
       <c r="I140" t="s">
         <v>328</v>
       </c>
-      <c r="J140" s="2">
+      <c r="J140" s="1">
         <v>46578</v>
       </c>
       <c r="K140" t="b">
@@ -6071,7 +6045,7 @@
       <c r="I141" t="s">
         <v>328</v>
       </c>
-      <c r="J141" s="2">
+      <c r="J141" s="1">
         <v>46592</v>
       </c>
       <c r="K141" t="b">
@@ -6106,7 +6080,7 @@
       <c r="I142" t="s">
         <v>328</v>
       </c>
-      <c r="J142" s="2">
+      <c r="J142" s="1">
         <v>46592</v>
       </c>
       <c r="K142" t="b">
@@ -6141,7 +6115,7 @@
       <c r="I143" t="s">
         <v>329</v>
       </c>
-      <c r="J143" s="2">
+      <c r="J143" s="1">
         <v>46212</v>
       </c>
       <c r="K143" t="b">
@@ -6176,7 +6150,7 @@
       <c r="I144" t="s">
         <v>330</v>
       </c>
-      <c r="J144" s="2">
+      <c r="J144" s="1">
         <v>46225</v>
       </c>
       <c r="K144" t="b">
@@ -6211,7 +6185,7 @@
       <c r="I145" t="s">
         <v>331</v>
       </c>
-      <c r="J145" s="2">
+      <c r="J145" s="1">
         <v>46263</v>
       </c>
       <c r="K145" t="b">
@@ -6243,7 +6217,7 @@
       <c r="H146">
         <v>-1476</v>
       </c>
-      <c r="J146" s="2">
+      <c r="J146" s="1">
         <v>43773</v>
       </c>
       <c r="K146" t="b">
@@ -6275,7 +6249,7 @@
       <c r="H147">
         <v>-1469</v>
       </c>
-      <c r="J147" s="2">
+      <c r="J147" s="1">
         <v>43773</v>
       </c>
       <c r="K147" t="b">
@@ -6307,7 +6281,7 @@
       <c r="H148">
         <v>-1186</v>
       </c>
-      <c r="J148" s="2">
+      <c r="J148" s="1">
         <v>45295</v>
       </c>
       <c r="K148" t="b">
@@ -6339,7 +6313,7 @@
       <c r="H149">
         <v>-1048</v>
       </c>
-      <c r="J149" s="2">
+      <c r="J149" s="1">
         <v>45617</v>
       </c>
       <c r="K149" t="b">
@@ -6371,7 +6345,7 @@
       <c r="H150">
         <v>-980</v>
       </c>
-      <c r="J150" s="2">
+      <c r="J150" s="1">
         <v>45677</v>
       </c>
       <c r="K150" t="b">
@@ -6403,7 +6377,7 @@
       <c r="H151">
         <v>-961</v>
       </c>
-      <c r="J151" s="2">
+      <c r="J151" s="1">
         <v>44944</v>
       </c>
       <c r="K151" t="b">
@@ -6435,7 +6409,7 @@
       <c r="H152">
         <v>-252</v>
       </c>
-      <c r="J152" s="2">
+      <c r="J152" s="1">
         <v>46092</v>
       </c>
       <c r="K152" t="b">
@@ -6467,7 +6441,7 @@
       <c r="H153">
         <v>3</v>
       </c>
-      <c r="J153" s="2">
+      <c r="J153" s="1">
         <v>46265</v>
       </c>
       <c r="K153" t="b">
@@ -6499,7 +6473,7 @@
       <c r="H154">
         <v>3</v>
       </c>
-      <c r="J154" s="2">
+      <c r="J154" s="1">
         <v>46265</v>
       </c>
       <c r="K154" t="b">
@@ -6531,7 +6505,7 @@
       <c r="H155">
         <v>43</v>
       </c>
-      <c r="J155" s="2">
+      <c r="J155" s="1">
         <v>46440</v>
       </c>
       <c r="K155" t="b">
@@ -6563,7 +6537,7 @@
       <c r="H156">
         <v>43</v>
       </c>
-      <c r="J156" s="2">
+      <c r="J156" s="1">
         <v>46440</v>
       </c>
       <c r="K156" t="b">
@@ -6595,7 +6569,7 @@
       <c r="H157">
         <v>72</v>
       </c>
-      <c r="J157" s="2">
+      <c r="J157" s="1">
         <v>46289</v>
       </c>
       <c r="K157" t="b">
@@ -6627,7 +6601,7 @@
       <c r="H158">
         <v>72</v>
       </c>
-      <c r="J158" s="2">
+      <c r="J158" s="1">
         <v>46289</v>
       </c>
       <c r="K158" t="b">
@@ -6659,7 +6633,7 @@
       <c r="H159">
         <v>81</v>
       </c>
-      <c r="J159" s="2">
+      <c r="J159" s="1">
         <v>46405</v>
       </c>
       <c r="K159" t="b">
@@ -6691,7 +6665,7 @@
       <c r="H160">
         <v>102</v>
       </c>
-      <c r="J160" s="2">
+      <c r="J160" s="1">
         <v>46463</v>
       </c>
       <c r="K160" t="b">
@@ -6723,7 +6697,7 @@
       <c r="H161">
         <v>109</v>
       </c>
-      <c r="J161" s="2">
+      <c r="J161" s="1">
         <v>46353</v>
       </c>
       <c r="K161" t="b">
@@ -6755,7 +6729,7 @@
       <c r="H162">
         <v>127</v>
       </c>
-      <c r="J162" s="2">
+      <c r="J162" s="1">
         <v>46417</v>
       </c>
       <c r="K162" t="b">
@@ -6787,7 +6761,7 @@
       <c r="H163">
         <v>152</v>
       </c>
-      <c r="J163" s="2">
+      <c r="J163" s="1">
         <v>46271</v>
       </c>
       <c r="K163" t="b">
@@ -6819,7 +6793,7 @@
       <c r="H164">
         <v>152</v>
       </c>
-      <c r="J164" s="2">
+      <c r="J164" s="1">
         <v>46271</v>
       </c>
       <c r="K164" t="b">
@@ -6851,7 +6825,7 @@
       <c r="H165">
         <v>153</v>
       </c>
-      <c r="J165" s="2">
+      <c r="J165" s="1">
         <v>46458</v>
       </c>
       <c r="K165" t="b">
@@ -6883,7 +6857,7 @@
       <c r="H166">
         <v>158</v>
       </c>
-      <c r="J166" s="2">
+      <c r="J166" s="1">
         <v>46381</v>
       </c>
       <c r="K166" t="b">
@@ -6915,7 +6889,7 @@
       <c r="H167">
         <v>163</v>
       </c>
-      <c r="J167" s="2">
+      <c r="J167" s="1">
         <v>46592</v>
       </c>
       <c r="K167" t="b">
@@ -6947,7 +6921,7 @@
       <c r="H168">
         <v>167</v>
       </c>
-      <c r="J168" s="2">
+      <c r="J168" s="1">
         <v>46441</v>
       </c>
       <c r="K168" t="b">
@@ -6979,7 +6953,7 @@
       <c r="H169">
         <v>169</v>
       </c>
-      <c r="J169" s="2">
+      <c r="J169" s="1">
         <v>46391</v>
       </c>
       <c r="K169" t="b">
@@ -7011,7 +6985,7 @@
       <c r="H170">
         <v>184</v>
       </c>
-      <c r="J170" s="2">
+      <c r="J170" s="1">
         <v>46385</v>
       </c>
       <c r="K170" t="b">
@@ -7043,7 +7017,7 @@
       <c r="H171">
         <v>186</v>
       </c>
-      <c r="J171" s="2">
+      <c r="J171" s="1">
         <v>46387</v>
       </c>
       <c r="K171" t="b">
@@ -7075,7 +7049,7 @@
       <c r="H172">
         <v>206</v>
       </c>
-      <c r="J172" s="2">
+      <c r="J172" s="1">
         <v>46399</v>
       </c>
       <c r="K172" t="b">
@@ -7107,7 +7081,7 @@
       <c r="H173">
         <v>206</v>
       </c>
-      <c r="J173" s="2">
+      <c r="J173" s="1">
         <v>46399</v>
       </c>
       <c r="K173" t="b">
@@ -7139,7 +7113,7 @@
       <c r="H174">
         <v>234</v>
       </c>
-      <c r="J174" s="2">
+      <c r="J174" s="1">
         <v>46458</v>
       </c>
       <c r="K174" t="b">
@@ -7171,7 +7145,7 @@
       <c r="H175">
         <v>248</v>
       </c>
-      <c r="J175" s="2">
+      <c r="J175" s="1">
         <v>46528</v>
       </c>
       <c r="K175" t="b">
@@ -7203,7 +7177,7 @@
       <c r="H176">
         <v>317</v>
       </c>
-      <c r="J176" s="2">
+      <c r="J176" s="1">
         <v>46540</v>
       </c>
       <c r="K176" t="b">
@@ -7235,7 +7209,7 @@
       <c r="H177">
         <v>340</v>
       </c>
-      <c r="J177" s="2">
+      <c r="J177" s="1">
         <v>46547</v>
       </c>
       <c r="K177" t="b">
@@ -7267,7 +7241,7 @@
       <c r="H178">
         <v>364</v>
       </c>
-      <c r="J178" s="2">
+      <c r="J178" s="1">
         <v>46557</v>
       </c>
       <c r="K178" t="b">
@@ -7299,7 +7273,7 @@
       <c r="H179">
         <v>368</v>
       </c>
-      <c r="J179" s="2">
+      <c r="J179" s="1">
         <v>46571</v>
       </c>
       <c r="K179" t="b">
@@ -7331,7 +7305,7 @@
       <c r="H180">
         <v>368</v>
       </c>
-      <c r="J180" s="2">
+      <c r="J180" s="1">
         <v>46571</v>
       </c>
       <c r="K180" t="b">
@@ -7363,7 +7337,7 @@
       <c r="H181">
         <v>370</v>
       </c>
-      <c r="J181" s="2">
+      <c r="J181" s="1">
         <v>46562</v>
       </c>
       <c r="K181" t="b">
@@ -7395,7 +7369,7 @@
       <c r="H182">
         <v>385</v>
       </c>
-      <c r="J182" s="2">
+      <c r="J182" s="1">
         <v>46574</v>
       </c>
       <c r="K182" t="b">
@@ -7427,7 +7401,7 @@
       <c r="H183">
         <v>385</v>
       </c>
-      <c r="J183" s="2">
+      <c r="J183" s="1">
         <v>46574</v>
       </c>
       <c r="K183" t="b">
@@ -7459,7 +7433,7 @@
       <c r="H184">
         <v>417</v>
       </c>
-      <c r="J184" s="2">
+      <c r="J184" s="1">
         <v>46578</v>
       </c>
       <c r="K184" t="b">
@@ -7491,7 +7465,7 @@
       <c r="H185">
         <v>721</v>
       </c>
-      <c r="J185" s="2">
+      <c r="J185" s="1">
         <v>46345</v>
       </c>
       <c r="K185" t="b">
@@ -7523,7 +7497,7 @@
       <c r="H186">
         <v>721</v>
       </c>
-      <c r="J186" s="2">
+      <c r="J186" s="1">
         <v>46345</v>
       </c>
       <c r="K186" t="b">
@@ -7555,7 +7529,7 @@
       <c r="H187">
         <v>850</v>
       </c>
-      <c r="J187" s="2">
+      <c r="J187" s="1">
         <v>46366</v>
       </c>
       <c r="K187" t="b">
@@ -7587,7 +7561,7 @@
       <c r="H188">
         <v>850</v>
       </c>
-      <c r="J188" s="2">
+      <c r="J188" s="1">
         <v>46366</v>
       </c>
       <c r="K188" t="b">
@@ -7619,7 +7593,7 @@
       <c r="H189">
         <v>1661</v>
       </c>
-      <c r="J189" s="2">
+      <c r="J189" s="1">
         <v>46524</v>
       </c>
       <c r="K189" t="b">
@@ -7651,7 +7625,7 @@
       <c r="H190">
         <v>1661</v>
       </c>
-      <c r="J190" s="2">
+      <c r="J190" s="1">
         <v>46524</v>
       </c>
       <c r="K190" t="b">
@@ -7683,7 +7657,7 @@
       <c r="H191">
         <v>488</v>
       </c>
-      <c r="J191" s="2">
+      <c r="J191" s="1">
         <v>46190</v>
       </c>
       <c r="K191" t="b">
@@ -7715,7 +7689,7 @@
       <c r="H192">
         <v>25565</v>
       </c>
-      <c r="J192" s="2">
+      <c r="J192" s="1">
         <v>46190</v>
       </c>
       <c r="K192" t="b">
@@ -7747,7 +7721,7 @@
       <c r="H193">
         <v>25567</v>
       </c>
-      <c r="J193" s="2">
+      <c r="J193" s="1">
         <v>46190</v>
       </c>
       <c r="K193" t="b">
@@ -7779,7 +7753,7 @@
       <c r="H194">
         <v>31293</v>
       </c>
-      <c r="J194" s="2">
+      <c r="J194" s="1">
         <v>46190</v>
       </c>
       <c r="K194" t="b">

</xml_diff>

<commit_message>
Atualização automática: vencimentos_tmot (21/08/2026 09:06)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
@@ -1019,8 +1019,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1036,7 +1044,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1044,12 +1052,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1349,37 +1375,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1408,7 +1434,7 @@
       <c r="H2">
         <v>-4300.3</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>39285</v>
       </c>
       <c r="K2" t="b">
@@ -1440,7 +1466,7 @@
       <c r="H3">
         <v>-2354.2</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>40669</v>
       </c>
       <c r="K3" t="b">
@@ -1472,7 +1498,7 @@
       <c r="H4">
         <v>-910.7</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>40669</v>
       </c>
       <c r="K4" t="b">
@@ -1504,7 +1530,7 @@
       <c r="H5">
         <v>-868</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>44884</v>
       </c>
       <c r="K5" t="b">
@@ -1536,7 +1562,7 @@
       <c r="H6">
         <v>-483.8</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>43855</v>
       </c>
       <c r="K6" t="b">
@@ -1568,7 +1594,7 @@
       <c r="H7">
         <v>-417</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>46014</v>
       </c>
       <c r="K7" t="b">
@@ -1600,7 +1626,7 @@
       <c r="H8">
         <v>-414.2</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>46014</v>
       </c>
       <c r="K8" t="b">
@@ -1632,7 +1658,7 @@
       <c r="H9">
         <v>-391.8</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>42769</v>
       </c>
       <c r="K9" t="b">
@@ -1664,7 +1690,7 @@
       <c r="H10">
         <v>-391.6</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>45804</v>
       </c>
       <c r="K10" t="b">
@@ -1696,7 +1722,7 @@
       <c r="H11">
         <v>-391.6</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>45804</v>
       </c>
       <c r="K11" t="b">
@@ -1728,7 +1754,7 @@
       <c r="H12">
         <v>-372.9</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>42821</v>
       </c>
       <c r="K12" t="b">
@@ -1760,7 +1786,7 @@
       <c r="H13">
         <v>-372.9</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>46014</v>
       </c>
       <c r="K13" t="b">
@@ -1792,7 +1818,7 @@
       <c r="H14">
         <v>-372.9</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>46014</v>
       </c>
       <c r="K14" t="b">
@@ -1824,7 +1850,7 @@
       <c r="H15">
         <v>-372.9</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>46014</v>
       </c>
       <c r="K15" t="b">
@@ -1856,7 +1882,7 @@
       <c r="H16">
         <v>-367.8</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="2">
         <v>46017</v>
       </c>
       <c r="K16" t="b">
@@ -1888,7 +1914,7 @@
       <c r="H17">
         <v>-367.8</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="2">
         <v>46017</v>
       </c>
       <c r="K17" t="b">
@@ -1920,7 +1946,7 @@
       <c r="H18">
         <v>-347.2</v>
       </c>
-      <c r="J18" s="1">
+      <c r="J18" s="2">
         <v>40979</v>
       </c>
       <c r="K18" t="b">
@@ -1952,7 +1978,7 @@
       <c r="H19">
         <v>-293.8</v>
       </c>
-      <c r="J19" s="1">
+      <c r="J19" s="2">
         <v>45846</v>
       </c>
       <c r="K19" t="b">
@@ -1984,7 +2010,7 @@
       <c r="H20">
         <v>-206.4</v>
       </c>
-      <c r="J20" s="1">
+      <c r="J20" s="2">
         <v>36669</v>
       </c>
       <c r="K20" t="b">
@@ -2016,7 +2042,7 @@
       <c r="H21">
         <v>-131.6</v>
       </c>
-      <c r="J21" s="1">
+      <c r="J21" s="2">
         <v>46111</v>
       </c>
       <c r="K21" t="b">
@@ -2048,7 +2074,7 @@
       <c r="H22">
         <v>-131.6</v>
       </c>
-      <c r="J22" s="1">
+      <c r="J22" s="2">
         <v>46111</v>
       </c>
       <c r="K22" t="b">
@@ -2080,7 +2106,7 @@
       <c r="H23">
         <v>-131.6</v>
       </c>
-      <c r="J23" s="1">
+      <c r="J23" s="2">
         <v>46111</v>
       </c>
       <c r="K23" t="b">
@@ -2112,7 +2138,7 @@
       <c r="H24">
         <v>-131.6</v>
       </c>
-      <c r="J24" s="1">
+      <c r="J24" s="2">
         <v>46111</v>
       </c>
       <c r="K24" t="b">
@@ -2144,7 +2170,7 @@
       <c r="H25">
         <v>-131.6</v>
       </c>
-      <c r="J25" s="1">
+      <c r="J25" s="2">
         <v>46111</v>
       </c>
       <c r="K25" t="b">
@@ -2176,7 +2202,7 @@
       <c r="H26">
         <v>-98.3</v>
       </c>
-      <c r="J26" s="1">
+      <c r="J26" s="2">
         <v>41204</v>
       </c>
       <c r="K26" t="b">
@@ -2208,7 +2234,7 @@
       <c r="H27">
         <v>-47.2</v>
       </c>
-      <c r="J27" s="1">
+      <c r="J27" s="2">
         <v>44011</v>
       </c>
       <c r="K27" t="b">
@@ -2240,7 +2266,7 @@
       <c r="H28">
         <v>-22.3</v>
       </c>
-      <c r="J28" s="1">
+      <c r="J28" s="2">
         <v>46226</v>
       </c>
       <c r="K28" t="b">
@@ -2272,7 +2298,7 @@
       <c r="H29">
         <v>4.7</v>
       </c>
-      <c r="J29" s="1">
+      <c r="J29" s="2">
         <v>46265</v>
       </c>
       <c r="K29" t="b">
@@ -2304,7 +2330,7 @@
       <c r="H30">
         <v>7.5</v>
       </c>
-      <c r="J30" s="1">
+      <c r="J30" s="2">
         <v>46265</v>
       </c>
       <c r="K30" t="b">
@@ -2336,7 +2362,7 @@
       <c r="H31">
         <v>10</v>
       </c>
-      <c r="J31" s="1">
+      <c r="J31" s="2">
         <v>46265</v>
       </c>
       <c r="K31" t="b">
@@ -2368,7 +2394,7 @@
       <c r="H32">
         <v>12.8</v>
       </c>
-      <c r="J32" s="1">
+      <c r="J32" s="2">
         <v>46265</v>
       </c>
       <c r="K32" t="b">
@@ -2400,7 +2426,7 @@
       <c r="H33">
         <v>14</v>
       </c>
-      <c r="J33" s="1">
+      <c r="J33" s="2">
         <v>46265</v>
       </c>
       <c r="K33" t="b">
@@ -2432,7 +2458,7 @@
       <c r="H34">
         <v>17.8</v>
       </c>
-      <c r="J34" s="1">
+      <c r="J34" s="2">
         <v>46265</v>
       </c>
       <c r="K34" t="b">
@@ -2464,7 +2490,7 @@
       <c r="H35">
         <v>20.4</v>
       </c>
-      <c r="J35" s="1">
+      <c r="J35" s="2">
         <v>46265</v>
       </c>
       <c r="K35" t="b">
@@ -2496,7 +2522,7 @@
       <c r="H36">
         <v>21.2</v>
       </c>
-      <c r="J36" s="1">
+      <c r="J36" s="2">
         <v>46265</v>
       </c>
       <c r="K36" t="b">
@@ -2528,7 +2554,7 @@
       <c r="H37">
         <v>26.2</v>
       </c>
-      <c r="J37" s="1">
+      <c r="J37" s="2">
         <v>46265</v>
       </c>
       <c r="K37" t="b">
@@ -2560,7 +2586,7 @@
       <c r="H38">
         <v>33.6</v>
       </c>
-      <c r="J38" s="1">
+      <c r="J38" s="2">
         <v>46364</v>
       </c>
       <c r="K38" t="b">
@@ -2592,7 +2618,7 @@
       <c r="H39">
         <v>42.2</v>
       </c>
-      <c r="J39" s="1">
+      <c r="J39" s="2">
         <v>46269</v>
       </c>
       <c r="K39" t="b">
@@ -2624,7 +2650,7 @@
       <c r="H40">
         <v>42.8</v>
       </c>
-      <c r="J40" s="1">
+      <c r="J40" s="2">
         <v>46291</v>
       </c>
       <c r="K40" t="b">
@@ -2656,7 +2682,7 @@
       <c r="H41">
         <v>45.7</v>
       </c>
-      <c r="J41" s="1">
+      <c r="J41" s="2">
         <v>46395</v>
       </c>
       <c r="K41" t="b">
@@ -2688,7 +2714,7 @@
       <c r="H42">
         <v>47.2</v>
       </c>
-      <c r="J42" s="1">
+      <c r="J42" s="2">
         <v>46280</v>
       </c>
       <c r="K42" t="b">
@@ -2720,7 +2746,7 @@
       <c r="H43">
         <v>48.7</v>
       </c>
-      <c r="J43" s="1">
+      <c r="J43" s="2">
         <v>46281</v>
       </c>
       <c r="K43" t="b">
@@ -2752,7 +2778,7 @@
       <c r="H44">
         <v>60</v>
       </c>
-      <c r="J44" s="1">
+      <c r="J44" s="2">
         <v>46281</v>
       </c>
       <c r="K44" t="b">
@@ -2784,7 +2810,7 @@
       <c r="H45">
         <v>62.6</v>
       </c>
-      <c r="J45" s="1">
+      <c r="J45" s="2">
         <v>46265</v>
       </c>
       <c r="K45" t="b">
@@ -2816,7 +2842,7 @@
       <c r="H46">
         <v>64.59999999999999</v>
       </c>
-      <c r="J46" s="1">
+      <c r="J46" s="2">
         <v>46265</v>
       </c>
       <c r="K46" t="b">
@@ -2848,7 +2874,7 @@
       <c r="H47">
         <v>67.59999999999999</v>
       </c>
-      <c r="J47" s="1">
+      <c r="J47" s="2">
         <v>46267</v>
       </c>
       <c r="K47" t="b">
@@ -2880,7 +2906,7 @@
       <c r="H48">
         <v>68.3</v>
       </c>
-      <c r="J48" s="1">
+      <c r="J48" s="2">
         <v>46278</v>
       </c>
       <c r="K48" t="b">
@@ -2912,7 +2938,7 @@
       <c r="H49">
         <v>69.2</v>
       </c>
-      <c r="J49" s="1">
+      <c r="J49" s="2">
         <v>46453</v>
       </c>
       <c r="K49" t="b">
@@ -2944,7 +2970,7 @@
       <c r="H50">
         <v>69.8</v>
       </c>
-      <c r="J50" s="1">
+      <c r="J50" s="2">
         <v>46265</v>
       </c>
       <c r="K50" t="b">
@@ -2976,7 +3002,7 @@
       <c r="H51">
         <v>69.8</v>
       </c>
-      <c r="J51" s="1">
+      <c r="J51" s="2">
         <v>46265</v>
       </c>
       <c r="K51" t="b">
@@ -3008,7 +3034,7 @@
       <c r="H52">
         <v>72.2</v>
       </c>
-      <c r="J52" s="1">
+      <c r="J52" s="2">
         <v>46275</v>
       </c>
       <c r="K52" t="b">
@@ -3040,7 +3066,7 @@
       <c r="H53">
         <v>72.2</v>
       </c>
-      <c r="J53" s="1">
+      <c r="J53" s="2">
         <v>46275</v>
       </c>
       <c r="K53" t="b">
@@ -3072,7 +3098,7 @@
       <c r="H54">
         <v>78.09999999999999</v>
       </c>
-      <c r="J54" s="1">
+      <c r="J54" s="2">
         <v>46265</v>
       </c>
       <c r="K54" t="b">
@@ -3104,7 +3130,7 @@
       <c r="H55">
         <v>82.8</v>
       </c>
-      <c r="J55" s="1">
+      <c r="J55" s="2">
         <v>46487</v>
       </c>
       <c r="K55" t="b">
@@ -3136,7 +3162,7 @@
       <c r="H56">
         <v>83.09999999999999</v>
       </c>
-      <c r="J56" s="1">
+      <c r="J56" s="2">
         <v>46285</v>
       </c>
       <c r="K56" t="b">
@@ -3168,7 +3194,7 @@
       <c r="H57">
         <v>84.8</v>
       </c>
-      <c r="J57" s="1">
+      <c r="J57" s="2">
         <v>46492</v>
       </c>
       <c r="K57" t="b">
@@ -3200,7 +3226,7 @@
       <c r="H58">
         <v>104.9</v>
       </c>
-      <c r="J58" s="1">
+      <c r="J58" s="2">
         <v>46297</v>
       </c>
       <c r="K58" t="b">
@@ -3232,7 +3258,7 @@
       <c r="H59">
         <v>107.6</v>
       </c>
-      <c r="J59" s="1">
+      <c r="J59" s="2">
         <v>46283</v>
       </c>
       <c r="K59" t="b">
@@ -3264,7 +3290,7 @@
       <c r="H60">
         <v>111.9</v>
       </c>
-      <c r="J60" s="1">
+      <c r="J60" s="2">
         <v>46300</v>
       </c>
       <c r="K60" t="b">
@@ -3296,7 +3322,7 @@
       <c r="H61">
         <v>111.9</v>
       </c>
-      <c r="J61" s="1">
+      <c r="J61" s="2">
         <v>46300</v>
       </c>
       <c r="K61" t="b">
@@ -3328,7 +3354,7 @@
       <c r="H62">
         <v>111.9</v>
       </c>
-      <c r="J62" s="1">
+      <c r="J62" s="2">
         <v>46300</v>
       </c>
       <c r="K62" t="b">
@@ -3360,7 +3386,7 @@
       <c r="H63">
         <v>111.9</v>
       </c>
-      <c r="J63" s="1">
+      <c r="J63" s="2">
         <v>46300</v>
       </c>
       <c r="K63" t="b">
@@ -3392,7 +3418,7 @@
       <c r="H64">
         <v>111.9</v>
       </c>
-      <c r="J64" s="1">
+      <c r="J64" s="2">
         <v>46300</v>
       </c>
       <c r="K64" t="b">
@@ -3424,7 +3450,7 @@
       <c r="H65">
         <v>128.8</v>
       </c>
-      <c r="J65" s="1">
+      <c r="J65" s="2">
         <v>46308</v>
       </c>
       <c r="K65" t="b">
@@ -3456,7 +3482,7 @@
       <c r="H66">
         <v>131.1</v>
       </c>
-      <c r="J66" s="1">
+      <c r="J66" s="2">
         <v>46336</v>
       </c>
       <c r="K66" t="b">
@@ -3488,7 +3514,7 @@
       <c r="H67">
         <v>138.4</v>
       </c>
-      <c r="J67" s="1">
+      <c r="J67" s="2">
         <v>46343</v>
       </c>
       <c r="K67" t="b">
@@ -3520,7 +3546,7 @@
       <c r="H68">
         <v>141</v>
       </c>
-      <c r="J68" s="1">
+      <c r="J68" s="2">
         <v>46350</v>
       </c>
       <c r="K68" t="b">
@@ -3552,7 +3578,7 @@
       <c r="H69">
         <v>162</v>
       </c>
-      <c r="J69" s="1">
+      <c r="J69" s="2">
         <v>46391</v>
       </c>
       <c r="K69" t="b">
@@ -3584,7 +3610,7 @@
       <c r="H70">
         <v>167.2</v>
       </c>
-      <c r="J70" s="1">
+      <c r="J70" s="2">
         <v>46330</v>
       </c>
       <c r="K70" t="b">
@@ -3616,7 +3642,7 @@
       <c r="H71">
         <v>177.4</v>
       </c>
-      <c r="J71" s="1">
+      <c r="J71" s="2">
         <v>46418</v>
       </c>
       <c r="K71" t="b">
@@ -3648,7 +3674,7 @@
       <c r="H72">
         <v>200</v>
       </c>
-      <c r="J72" s="1">
+      <c r="J72" s="2">
         <v>46356</v>
       </c>
       <c r="K72" t="b">
@@ -3680,7 +3706,7 @@
       <c r="H73">
         <v>203.6</v>
       </c>
-      <c r="J73" s="1">
+      <c r="J73" s="2">
         <v>46436</v>
       </c>
       <c r="K73" t="b">
@@ -3712,7 +3738,7 @@
       <c r="H74">
         <v>221.2</v>
       </c>
-      <c r="J74" s="1">
+      <c r="J74" s="2">
         <v>46426</v>
       </c>
       <c r="K74" t="b">
@@ -3744,7 +3770,7 @@
       <c r="H75">
         <v>240.8</v>
       </c>
-      <c r="J75" s="1">
+      <c r="J75" s="2">
         <v>46450</v>
       </c>
       <c r="K75" t="b">
@@ -3776,7 +3802,7 @@
       <c r="H76">
         <v>245.8</v>
       </c>
-      <c r="J76" s="1">
+      <c r="J76" s="2">
         <v>46452</v>
       </c>
       <c r="K76" t="b">
@@ -3808,7 +3834,7 @@
       <c r="H77">
         <v>263.4</v>
       </c>
-      <c r="J77" s="1">
+      <c r="J77" s="2">
         <v>46322</v>
       </c>
       <c r="K77" t="b">
@@ -3840,7 +3866,7 @@
       <c r="H78">
         <v>275.2</v>
       </c>
-      <c r="J78" s="1">
+      <c r="J78" s="2">
         <v>46433</v>
       </c>
       <c r="K78" t="b">
@@ -3875,7 +3901,7 @@
       <c r="I79" t="s">
         <v>311</v>
       </c>
-      <c r="J79" s="1">
+      <c r="J79" s="2">
         <v>36557</v>
       </c>
       <c r="K79" t="b">
@@ -3910,7 +3936,7 @@
       <c r="I80" t="s">
         <v>312</v>
       </c>
-      <c r="J80" s="1">
+      <c r="J80" s="2">
         <v>41275</v>
       </c>
       <c r="K80" t="b">
@@ -3945,7 +3971,7 @@
       <c r="I81" t="s">
         <v>313</v>
       </c>
-      <c r="J81" s="1">
+      <c r="J81" s="2">
         <v>45380</v>
       </c>
       <c r="K81" t="b">
@@ -3980,7 +4006,7 @@
       <c r="I82" t="s">
         <v>314</v>
       </c>
-      <c r="J82" s="1">
+      <c r="J82" s="2">
         <v>45421</v>
       </c>
       <c r="K82" t="b">
@@ -4015,7 +4041,7 @@
       <c r="I83" t="s">
         <v>314</v>
       </c>
-      <c r="J83" s="1">
+      <c r="J83" s="2">
         <v>45428</v>
       </c>
       <c r="K83" t="b">
@@ -4050,7 +4076,7 @@
       <c r="I84" t="s">
         <v>315</v>
       </c>
-      <c r="J84" s="1">
+      <c r="J84" s="2">
         <v>45490</v>
       </c>
       <c r="K84" t="b">
@@ -4085,7 +4111,7 @@
       <c r="I85" t="s">
         <v>316</v>
       </c>
-      <c r="J85" s="1">
+      <c r="J85" s="2">
         <v>45566</v>
       </c>
       <c r="K85" t="b">
@@ -4120,7 +4146,7 @@
       <c r="I86" t="s">
         <v>317</v>
       </c>
-      <c r="J86" s="1">
+      <c r="J86" s="2">
         <v>45986</v>
       </c>
       <c r="K86" t="b">
@@ -4155,7 +4181,7 @@
       <c r="I87" t="s">
         <v>318</v>
       </c>
-      <c r="J87" s="1">
+      <c r="J87" s="2">
         <v>46284</v>
       </c>
       <c r="K87" t="b">
@@ -4190,7 +4216,7 @@
       <c r="I88" t="s">
         <v>319</v>
       </c>
-      <c r="J88" s="1">
+      <c r="J88" s="2">
         <v>46305</v>
       </c>
       <c r="K88" t="b">
@@ -4225,7 +4251,7 @@
       <c r="I89" t="s">
         <v>319</v>
       </c>
-      <c r="J89" s="1">
+      <c r="J89" s="2">
         <v>46310</v>
       </c>
       <c r="K89" t="b">
@@ -4260,7 +4286,7 @@
       <c r="I90" t="s">
         <v>319</v>
       </c>
-      <c r="J90" s="1">
+      <c r="J90" s="2">
         <v>46317</v>
       </c>
       <c r="K90" t="b">
@@ -4295,7 +4321,7 @@
       <c r="I91" t="s">
         <v>319</v>
       </c>
-      <c r="J91" s="1">
+      <c r="J91" s="2">
         <v>46319</v>
       </c>
       <c r="K91" t="b">
@@ -4330,7 +4356,7 @@
       <c r="I92" t="s">
         <v>320</v>
       </c>
-      <c r="J92" s="1">
+      <c r="J92" s="2">
         <v>46333</v>
       </c>
       <c r="K92" t="b">
@@ -4365,7 +4391,7 @@
       <c r="I93" t="s">
         <v>320</v>
       </c>
-      <c r="J93" s="1">
+      <c r="J93" s="2">
         <v>46338</v>
       </c>
       <c r="K93" t="b">
@@ -4400,7 +4426,7 @@
       <c r="I94" t="s">
         <v>320</v>
       </c>
-      <c r="J94" s="1">
+      <c r="J94" s="2">
         <v>46338</v>
       </c>
       <c r="K94" t="b">
@@ -4435,7 +4461,7 @@
       <c r="I95" t="s">
         <v>320</v>
       </c>
-      <c r="J95" s="1">
+      <c r="J95" s="2">
         <v>46341</v>
       </c>
       <c r="K95" t="b">
@@ -4470,7 +4496,7 @@
       <c r="I96" t="s">
         <v>320</v>
       </c>
-      <c r="J96" s="1">
+      <c r="J96" s="2">
         <v>46344</v>
       </c>
       <c r="K96" t="b">
@@ -4505,7 +4531,7 @@
       <c r="I97" t="s">
         <v>321</v>
       </c>
-      <c r="J97" s="1">
+      <c r="J97" s="2">
         <v>46360</v>
       </c>
       <c r="K97" t="b">
@@ -4540,7 +4566,7 @@
       <c r="I98" t="s">
         <v>321</v>
       </c>
-      <c r="J98" s="1">
+      <c r="J98" s="2">
         <v>46360</v>
       </c>
       <c r="K98" t="b">
@@ -4575,7 +4601,7 @@
       <c r="I99" t="s">
         <v>321</v>
       </c>
-      <c r="J99" s="1">
+      <c r="J99" s="2">
         <v>46367</v>
       </c>
       <c r="K99" t="b">
@@ -4610,7 +4636,7 @@
       <c r="I100" t="s">
         <v>321</v>
       </c>
-      <c r="J100" s="1">
+      <c r="J100" s="2">
         <v>46375</v>
       </c>
       <c r="K100" t="b">
@@ -4645,7 +4671,7 @@
       <c r="I101" t="s">
         <v>321</v>
       </c>
-      <c r="J101" s="1">
+      <c r="J101" s="2">
         <v>46387</v>
       </c>
       <c r="K101" t="b">
@@ -4680,7 +4706,7 @@
       <c r="I102" t="s">
         <v>321</v>
       </c>
-      <c r="J102" s="1">
+      <c r="J102" s="2">
         <v>46387</v>
       </c>
       <c r="K102" t="b">
@@ -4715,7 +4741,7 @@
       <c r="I103" t="s">
         <v>321</v>
       </c>
-      <c r="J103" s="1">
+      <c r="J103" s="2">
         <v>46387</v>
       </c>
       <c r="K103" t="b">
@@ -4750,7 +4776,7 @@
       <c r="I104" t="s">
         <v>321</v>
       </c>
-      <c r="J104" s="1">
+      <c r="J104" s="2">
         <v>46388</v>
       </c>
       <c r="K104" t="b">
@@ -4785,7 +4811,7 @@
       <c r="I105" t="s">
         <v>322</v>
       </c>
-      <c r="J105" s="1">
+      <c r="J105" s="2">
         <v>46401</v>
       </c>
       <c r="K105" t="b">
@@ -4820,7 +4846,7 @@
       <c r="I106" t="s">
         <v>322</v>
       </c>
-      <c r="J106" s="1">
+      <c r="J106" s="2">
         <v>46401</v>
       </c>
       <c r="K106" t="b">
@@ -4855,7 +4881,7 @@
       <c r="I107" t="s">
         <v>322</v>
       </c>
-      <c r="J107" s="1">
+      <c r="J107" s="2">
         <v>46401</v>
       </c>
       <c r="K107" t="b">
@@ -4890,7 +4916,7 @@
       <c r="I108" t="s">
         <v>322</v>
       </c>
-      <c r="J108" s="1">
+      <c r="J108" s="2">
         <v>46412</v>
       </c>
       <c r="K108" t="b">
@@ -4925,7 +4951,7 @@
       <c r="I109" t="s">
         <v>322</v>
       </c>
-      <c r="J109" s="1">
+      <c r="J109" s="2">
         <v>46412</v>
       </c>
       <c r="K109" t="b">
@@ -4960,7 +4986,7 @@
       <c r="I110" t="s">
         <v>322</v>
       </c>
-      <c r="J110" s="1">
+      <c r="J110" s="2">
         <v>46412</v>
       </c>
       <c r="K110" t="b">
@@ -4995,7 +5021,7 @@
       <c r="I111" t="s">
         <v>323</v>
       </c>
-      <c r="J111" s="1">
+      <c r="J111" s="2">
         <v>46424</v>
       </c>
       <c r="K111" t="b">
@@ -5030,7 +5056,7 @@
       <c r="I112" t="s">
         <v>323</v>
       </c>
-      <c r="J112" s="1">
+      <c r="J112" s="2">
         <v>46437</v>
       </c>
       <c r="K112" t="b">
@@ -5065,7 +5091,7 @@
       <c r="I113" t="s">
         <v>323</v>
       </c>
-      <c r="J113" s="1">
+      <c r="J113" s="2">
         <v>46451</v>
       </c>
       <c r="K113" t="b">
@@ -5100,7 +5126,7 @@
       <c r="I114" t="s">
         <v>323</v>
       </c>
-      <c r="J114" s="1">
+      <c r="J114" s="2">
         <v>46451</v>
       </c>
       <c r="K114" t="b">
@@ -5135,7 +5161,7 @@
       <c r="I115" t="s">
         <v>324</v>
       </c>
-      <c r="J115" s="1">
+      <c r="J115" s="2">
         <v>46455</v>
       </c>
       <c r="K115" t="b">
@@ -5170,7 +5196,7 @@
       <c r="I116" t="s">
         <v>324</v>
       </c>
-      <c r="J116" s="1">
+      <c r="J116" s="2">
         <v>46456</v>
       </c>
       <c r="K116" t="b">
@@ -5205,7 +5231,7 @@
       <c r="I117" t="s">
         <v>324</v>
       </c>
-      <c r="J117" s="1">
+      <c r="J117" s="2">
         <v>46457</v>
       </c>
       <c r="K117" t="b">
@@ -5240,7 +5266,7 @@
       <c r="I118" t="s">
         <v>324</v>
       </c>
-      <c r="J118" s="1">
+      <c r="J118" s="2">
         <v>46464</v>
       </c>
       <c r="K118" t="b">
@@ -5275,7 +5301,7 @@
       <c r="I119" t="s">
         <v>324</v>
       </c>
-      <c r="J119" s="1">
+      <c r="J119" s="2">
         <v>46470</v>
       </c>
       <c r="K119" t="b">
@@ -5310,7 +5336,7 @@
       <c r="I120" t="s">
         <v>325</v>
       </c>
-      <c r="J120" s="1">
+      <c r="J120" s="2">
         <v>46485</v>
       </c>
       <c r="K120" t="b">
@@ -5345,7 +5371,7 @@
       <c r="I121" t="s">
         <v>325</v>
       </c>
-      <c r="J121" s="1">
+      <c r="J121" s="2">
         <v>46499</v>
       </c>
       <c r="K121" t="b">
@@ -5380,7 +5406,7 @@
       <c r="I122" t="s">
         <v>325</v>
       </c>
-      <c r="J122" s="1">
+      <c r="J122" s="2">
         <v>46504</v>
       </c>
       <c r="K122" t="b">
@@ -5415,7 +5441,7 @@
       <c r="I123" t="s">
         <v>325</v>
       </c>
-      <c r="J123" s="1">
+      <c r="J123" s="2">
         <v>46504</v>
       </c>
       <c r="K123" t="b">
@@ -5450,7 +5476,7 @@
       <c r="I124" t="s">
         <v>325</v>
       </c>
-      <c r="J124" s="1">
+      <c r="J124" s="2">
         <v>46507</v>
       </c>
       <c r="K124" t="b">
@@ -5485,7 +5511,7 @@
       <c r="I125" t="s">
         <v>325</v>
       </c>
-      <c r="J125" s="1">
+      <c r="J125" s="2">
         <v>46508</v>
       </c>
       <c r="K125" t="b">
@@ -5520,7 +5546,7 @@
       <c r="I126" t="s">
         <v>325</v>
       </c>
-      <c r="J126" s="1">
+      <c r="J126" s="2">
         <v>46512</v>
       </c>
       <c r="K126" t="b">
@@ -5555,7 +5581,7 @@
       <c r="I127" t="s">
         <v>326</v>
       </c>
-      <c r="J127" s="1">
+      <c r="J127" s="2">
         <v>46512</v>
       </c>
       <c r="K127" t="b">
@@ -5590,7 +5616,7 @@
       <c r="I128" t="s">
         <v>326</v>
       </c>
-      <c r="J128" s="1">
+      <c r="J128" s="2">
         <v>46528</v>
       </c>
       <c r="K128" t="b">
@@ -5625,7 +5651,7 @@
       <c r="I129" t="s">
         <v>326</v>
       </c>
-      <c r="J129" s="1">
+      <c r="J129" s="2">
         <v>46529</v>
       </c>
       <c r="K129" t="b">
@@ -5660,7 +5686,7 @@
       <c r="I130" t="s">
         <v>326</v>
       </c>
-      <c r="J130" s="1">
+      <c r="J130" s="2">
         <v>46537</v>
       </c>
       <c r="K130" t="b">
@@ -5695,7 +5721,7 @@
       <c r="I131" t="s">
         <v>327</v>
       </c>
-      <c r="J131" s="1">
+      <c r="J131" s="2">
         <v>46546</v>
       </c>
       <c r="K131" t="b">
@@ -5730,7 +5756,7 @@
       <c r="I132" t="s">
         <v>327</v>
       </c>
-      <c r="J132" s="1">
+      <c r="J132" s="2">
         <v>46547</v>
       </c>
       <c r="K132" t="b">
@@ -5765,7 +5791,7 @@
       <c r="I133" t="s">
         <v>327</v>
       </c>
-      <c r="J133" s="1">
+      <c r="J133" s="2">
         <v>46547</v>
       </c>
       <c r="K133" t="b">
@@ -5800,7 +5826,7 @@
       <c r="I134" t="s">
         <v>327</v>
       </c>
-      <c r="J134" s="1">
+      <c r="J134" s="2">
         <v>46547</v>
       </c>
       <c r="K134" t="b">
@@ -5835,7 +5861,7 @@
       <c r="I135" t="s">
         <v>327</v>
       </c>
-      <c r="J135" s="1">
+      <c r="J135" s="2">
         <v>46551</v>
       </c>
       <c r="K135" t="b">
@@ -5870,7 +5896,7 @@
       <c r="I136" t="s">
         <v>327</v>
       </c>
-      <c r="J136" s="1">
+      <c r="J136" s="2">
         <v>46560</v>
       </c>
       <c r="K136" t="b">
@@ -5905,7 +5931,7 @@
       <c r="I137" t="s">
         <v>327</v>
       </c>
-      <c r="J137" s="1">
+      <c r="J137" s="2">
         <v>46564</v>
       </c>
       <c r="K137" t="b">
@@ -5940,7 +5966,7 @@
       <c r="I138" t="s">
         <v>327</v>
       </c>
-      <c r="J138" s="1">
+      <c r="J138" s="2">
         <v>46567</v>
       </c>
       <c r="K138" t="b">
@@ -5975,7 +6001,7 @@
       <c r="I139" t="s">
         <v>327</v>
       </c>
-      <c r="J139" s="1">
+      <c r="J139" s="2">
         <v>46568</v>
       </c>
       <c r="K139" t="b">
@@ -6010,7 +6036,7 @@
       <c r="I140" t="s">
         <v>328</v>
       </c>
-      <c r="J140" s="1">
+      <c r="J140" s="2">
         <v>46578</v>
       </c>
       <c r="K140" t="b">
@@ -6045,7 +6071,7 @@
       <c r="I141" t="s">
         <v>328</v>
       </c>
-      <c r="J141" s="1">
+      <c r="J141" s="2">
         <v>46592</v>
       </c>
       <c r="K141" t="b">
@@ -6080,7 +6106,7 @@
       <c r="I142" t="s">
         <v>328</v>
       </c>
-      <c r="J142" s="1">
+      <c r="J142" s="2">
         <v>46592</v>
       </c>
       <c r="K142" t="b">
@@ -6115,7 +6141,7 @@
       <c r="I143" t="s">
         <v>329</v>
       </c>
-      <c r="J143" s="1">
+      <c r="J143" s="2">
         <v>46212</v>
       </c>
       <c r="K143" t="b">
@@ -6150,7 +6176,7 @@
       <c r="I144" t="s">
         <v>330</v>
       </c>
-      <c r="J144" s="1">
+      <c r="J144" s="2">
         <v>46225</v>
       </c>
       <c r="K144" t="b">
@@ -6185,7 +6211,7 @@
       <c r="I145" t="s">
         <v>331</v>
       </c>
-      <c r="J145" s="1">
+      <c r="J145" s="2">
         <v>46263</v>
       </c>
       <c r="K145" t="b">
@@ -6217,7 +6243,7 @@
       <c r="H146">
         <v>-1476</v>
       </c>
-      <c r="J146" s="1">
+      <c r="J146" s="2">
         <v>43773</v>
       </c>
       <c r="K146" t="b">
@@ -6249,7 +6275,7 @@
       <c r="H147">
         <v>-1469</v>
       </c>
-      <c r="J147" s="1">
+      <c r="J147" s="2">
         <v>43773</v>
       </c>
       <c r="K147" t="b">
@@ -6281,7 +6307,7 @@
       <c r="H148">
         <v>-1186</v>
       </c>
-      <c r="J148" s="1">
+      <c r="J148" s="2">
         <v>45295</v>
       </c>
       <c r="K148" t="b">
@@ -6313,7 +6339,7 @@
       <c r="H149">
         <v>-1048</v>
       </c>
-      <c r="J149" s="1">
+      <c r="J149" s="2">
         <v>45617</v>
       </c>
       <c r="K149" t="b">
@@ -6345,7 +6371,7 @@
       <c r="H150">
         <v>-980</v>
       </c>
-      <c r="J150" s="1">
+      <c r="J150" s="2">
         <v>45677</v>
       </c>
       <c r="K150" t="b">
@@ -6377,7 +6403,7 @@
       <c r="H151">
         <v>-961</v>
       </c>
-      <c r="J151" s="1">
+      <c r="J151" s="2">
         <v>44944</v>
       </c>
       <c r="K151" t="b">
@@ -6409,7 +6435,7 @@
       <c r="H152">
         <v>-252</v>
       </c>
-      <c r="J152" s="1">
+      <c r="J152" s="2">
         <v>46092</v>
       </c>
       <c r="K152" t="b">
@@ -6441,7 +6467,7 @@
       <c r="H153">
         <v>3</v>
       </c>
-      <c r="J153" s="1">
+      <c r="J153" s="2">
         <v>46265</v>
       </c>
       <c r="K153" t="b">
@@ -6473,7 +6499,7 @@
       <c r="H154">
         <v>3</v>
       </c>
-      <c r="J154" s="1">
+      <c r="J154" s="2">
         <v>46265</v>
       </c>
       <c r="K154" t="b">
@@ -6505,7 +6531,7 @@
       <c r="H155">
         <v>43</v>
       </c>
-      <c r="J155" s="1">
+      <c r="J155" s="2">
         <v>46440</v>
       </c>
       <c r="K155" t="b">
@@ -6537,7 +6563,7 @@
       <c r="H156">
         <v>43</v>
       </c>
-      <c r="J156" s="1">
+      <c r="J156" s="2">
         <v>46440</v>
       </c>
       <c r="K156" t="b">
@@ -6569,7 +6595,7 @@
       <c r="H157">
         <v>72</v>
       </c>
-      <c r="J157" s="1">
+      <c r="J157" s="2">
         <v>46289</v>
       </c>
       <c r="K157" t="b">
@@ -6601,7 +6627,7 @@
       <c r="H158">
         <v>72</v>
       </c>
-      <c r="J158" s="1">
+      <c r="J158" s="2">
         <v>46289</v>
       </c>
       <c r="K158" t="b">
@@ -6633,7 +6659,7 @@
       <c r="H159">
         <v>81</v>
       </c>
-      <c r="J159" s="1">
+      <c r="J159" s="2">
         <v>46405</v>
       </c>
       <c r="K159" t="b">
@@ -6665,7 +6691,7 @@
       <c r="H160">
         <v>102</v>
       </c>
-      <c r="J160" s="1">
+      <c r="J160" s="2">
         <v>46463</v>
       </c>
       <c r="K160" t="b">
@@ -6697,7 +6723,7 @@
       <c r="H161">
         <v>109</v>
       </c>
-      <c r="J161" s="1">
+      <c r="J161" s="2">
         <v>46353</v>
       </c>
       <c r="K161" t="b">
@@ -6729,7 +6755,7 @@
       <c r="H162">
         <v>127</v>
       </c>
-      <c r="J162" s="1">
+      <c r="J162" s="2">
         <v>46417</v>
       </c>
       <c r="K162" t="b">
@@ -6761,7 +6787,7 @@
       <c r="H163">
         <v>152</v>
       </c>
-      <c r="J163" s="1">
+      <c r="J163" s="2">
         <v>46271</v>
       </c>
       <c r="K163" t="b">
@@ -6793,7 +6819,7 @@
       <c r="H164">
         <v>152</v>
       </c>
-      <c r="J164" s="1">
+      <c r="J164" s="2">
         <v>46271</v>
       </c>
       <c r="K164" t="b">
@@ -6825,7 +6851,7 @@
       <c r="H165">
         <v>153</v>
       </c>
-      <c r="J165" s="1">
+      <c r="J165" s="2">
         <v>46458</v>
       </c>
       <c r="K165" t="b">
@@ -6857,7 +6883,7 @@
       <c r="H166">
         <v>158</v>
       </c>
-      <c r="J166" s="1">
+      <c r="J166" s="2">
         <v>46381</v>
       </c>
       <c r="K166" t="b">
@@ -6889,7 +6915,7 @@
       <c r="H167">
         <v>163</v>
       </c>
-      <c r="J167" s="1">
+      <c r="J167" s="2">
         <v>46592</v>
       </c>
       <c r="K167" t="b">
@@ -6921,7 +6947,7 @@
       <c r="H168">
         <v>167</v>
       </c>
-      <c r="J168" s="1">
+      <c r="J168" s="2">
         <v>46441</v>
       </c>
       <c r="K168" t="b">
@@ -6953,7 +6979,7 @@
       <c r="H169">
         <v>169</v>
       </c>
-      <c r="J169" s="1">
+      <c r="J169" s="2">
         <v>46391</v>
       </c>
       <c r="K169" t="b">
@@ -6985,7 +7011,7 @@
       <c r="H170">
         <v>184</v>
       </c>
-      <c r="J170" s="1">
+      <c r="J170" s="2">
         <v>46385</v>
       </c>
       <c r="K170" t="b">
@@ -7017,7 +7043,7 @@
       <c r="H171">
         <v>186</v>
       </c>
-      <c r="J171" s="1">
+      <c r="J171" s="2">
         <v>46387</v>
       </c>
       <c r="K171" t="b">
@@ -7049,7 +7075,7 @@
       <c r="H172">
         <v>206</v>
       </c>
-      <c r="J172" s="1">
+      <c r="J172" s="2">
         <v>46399</v>
       </c>
       <c r="K172" t="b">
@@ -7081,7 +7107,7 @@
       <c r="H173">
         <v>206</v>
       </c>
-      <c r="J173" s="1">
+      <c r="J173" s="2">
         <v>46399</v>
       </c>
       <c r="K173" t="b">
@@ -7113,7 +7139,7 @@
       <c r="H174">
         <v>234</v>
       </c>
-      <c r="J174" s="1">
+      <c r="J174" s="2">
         <v>46458</v>
       </c>
       <c r="K174" t="b">
@@ -7145,7 +7171,7 @@
       <c r="H175">
         <v>248</v>
       </c>
-      <c r="J175" s="1">
+      <c r="J175" s="2">
         <v>46528</v>
       </c>
       <c r="K175" t="b">
@@ -7177,7 +7203,7 @@
       <c r="H176">
         <v>317</v>
       </c>
-      <c r="J176" s="1">
+      <c r="J176" s="2">
         <v>46540</v>
       </c>
       <c r="K176" t="b">
@@ -7209,7 +7235,7 @@
       <c r="H177">
         <v>340</v>
       </c>
-      <c r="J177" s="1">
+      <c r="J177" s="2">
         <v>46547</v>
       </c>
       <c r="K177" t="b">
@@ -7241,7 +7267,7 @@
       <c r="H178">
         <v>364</v>
       </c>
-      <c r="J178" s="1">
+      <c r="J178" s="2">
         <v>46557</v>
       </c>
       <c r="K178" t="b">
@@ -7273,7 +7299,7 @@
       <c r="H179">
         <v>368</v>
       </c>
-      <c r="J179" s="1">
+      <c r="J179" s="2">
         <v>46571</v>
       </c>
       <c r="K179" t="b">
@@ -7305,7 +7331,7 @@
       <c r="H180">
         <v>368</v>
       </c>
-      <c r="J180" s="1">
+      <c r="J180" s="2">
         <v>46571</v>
       </c>
       <c r="K180" t="b">
@@ -7337,7 +7363,7 @@
       <c r="H181">
         <v>370</v>
       </c>
-      <c r="J181" s="1">
+      <c r="J181" s="2">
         <v>46562</v>
       </c>
       <c r="K181" t="b">
@@ -7369,7 +7395,7 @@
       <c r="H182">
         <v>385</v>
       </c>
-      <c r="J182" s="1">
+      <c r="J182" s="2">
         <v>46574</v>
       </c>
       <c r="K182" t="b">
@@ -7401,7 +7427,7 @@
       <c r="H183">
         <v>385</v>
       </c>
-      <c r="J183" s="1">
+      <c r="J183" s="2">
         <v>46574</v>
       </c>
       <c r="K183" t="b">
@@ -7433,7 +7459,7 @@
       <c r="H184">
         <v>417</v>
       </c>
-      <c r="J184" s="1">
+      <c r="J184" s="2">
         <v>46578</v>
       </c>
       <c r="K184" t="b">
@@ -7465,7 +7491,7 @@
       <c r="H185">
         <v>721</v>
       </c>
-      <c r="J185" s="1">
+      <c r="J185" s="2">
         <v>46345</v>
       </c>
       <c r="K185" t="b">
@@ -7497,7 +7523,7 @@
       <c r="H186">
         <v>721</v>
       </c>
-      <c r="J186" s="1">
+      <c r="J186" s="2">
         <v>46345</v>
       </c>
       <c r="K186" t="b">
@@ -7529,7 +7555,7 @@
       <c r="H187">
         <v>850</v>
       </c>
-      <c r="J187" s="1">
+      <c r="J187" s="2">
         <v>46366</v>
       </c>
       <c r="K187" t="b">
@@ -7561,7 +7587,7 @@
       <c r="H188">
         <v>850</v>
       </c>
-      <c r="J188" s="1">
+      <c r="J188" s="2">
         <v>46366</v>
       </c>
       <c r="K188" t="b">
@@ -7593,7 +7619,7 @@
       <c r="H189">
         <v>1661</v>
       </c>
-      <c r="J189" s="1">
+      <c r="J189" s="2">
         <v>46524</v>
       </c>
       <c r="K189" t="b">
@@ -7625,7 +7651,7 @@
       <c r="H190">
         <v>1661</v>
       </c>
-      <c r="J190" s="1">
+      <c r="J190" s="2">
         <v>46524</v>
       </c>
       <c r="K190" t="b">
@@ -7657,7 +7683,7 @@
       <c r="H191">
         <v>488</v>
       </c>
-      <c r="J191" s="1">
+      <c r="J191" s="2">
         <v>46190</v>
       </c>
       <c r="K191" t="b">
@@ -7689,7 +7715,7 @@
       <c r="H192">
         <v>25565</v>
       </c>
-      <c r="J192" s="1">
+      <c r="J192" s="2">
         <v>46190</v>
       </c>
       <c r="K192" t="b">
@@ -7721,7 +7747,7 @@
       <c r="H193">
         <v>25567</v>
       </c>
-      <c r="J193" s="1">
+      <c r="J193" s="2">
         <v>46190</v>
       </c>
       <c r="K193" t="b">
@@ -7753,7 +7779,7 @@
       <c r="H194">
         <v>31293</v>
       </c>
-      <c r="J194" s="1">
+      <c r="J194" s="2">
         <v>46190</v>
       </c>
       <c r="K194" t="b">

</xml_diff>

<commit_message>
Atualização automática: vencimentos_tmot (21/08/2026 10:51)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
@@ -1019,16 +1019,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1044,7 +1036,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1052,30 +1044,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1375,37 +1349,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1434,7 +1408,7 @@
       <c r="H2">
         <v>-4300.3</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>39285</v>
       </c>
       <c r="K2" t="b">
@@ -1466,7 +1440,7 @@
       <c r="H3">
         <v>-2354.2</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>40669</v>
       </c>
       <c r="K3" t="b">
@@ -1498,7 +1472,7 @@
       <c r="H4">
         <v>-910.7</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>40669</v>
       </c>
       <c r="K4" t="b">
@@ -1530,7 +1504,7 @@
       <c r="H5">
         <v>-868</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>44884</v>
       </c>
       <c r="K5" t="b">
@@ -1562,7 +1536,7 @@
       <c r="H6">
         <v>-483.8</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>43855</v>
       </c>
       <c r="K6" t="b">
@@ -1594,7 +1568,7 @@
       <c r="H7">
         <v>-417</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>46014</v>
       </c>
       <c r="K7" t="b">
@@ -1626,7 +1600,7 @@
       <c r="H8">
         <v>-414.2</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>46014</v>
       </c>
       <c r="K8" t="b">
@@ -1658,7 +1632,7 @@
       <c r="H9">
         <v>-391.8</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>42769</v>
       </c>
       <c r="K9" t="b">
@@ -1690,7 +1664,7 @@
       <c r="H10">
         <v>-391.6</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>45804</v>
       </c>
       <c r="K10" t="b">
@@ -1722,7 +1696,7 @@
       <c r="H11">
         <v>-391.6</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>45804</v>
       </c>
       <c r="K11" t="b">
@@ -1754,7 +1728,7 @@
       <c r="H12">
         <v>-372.9</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>42821</v>
       </c>
       <c r="K12" t="b">
@@ -1786,7 +1760,7 @@
       <c r="H13">
         <v>-372.9</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>46014</v>
       </c>
       <c r="K13" t="b">
@@ -1818,7 +1792,7 @@
       <c r="H14">
         <v>-372.9</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>46014</v>
       </c>
       <c r="K14" t="b">
@@ -1850,7 +1824,7 @@
       <c r="H15">
         <v>-372.9</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <v>46014</v>
       </c>
       <c r="K15" t="b">
@@ -1882,7 +1856,7 @@
       <c r="H16">
         <v>-367.8</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <v>46017</v>
       </c>
       <c r="K16" t="b">
@@ -1914,7 +1888,7 @@
       <c r="H17">
         <v>-367.8</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="1">
         <v>46017</v>
       </c>
       <c r="K17" t="b">
@@ -1946,7 +1920,7 @@
       <c r="H18">
         <v>-347.2</v>
       </c>
-      <c r="J18" s="2">
+      <c r="J18" s="1">
         <v>40979</v>
       </c>
       <c r="K18" t="b">
@@ -1978,7 +1952,7 @@
       <c r="H19">
         <v>-293.8</v>
       </c>
-      <c r="J19" s="2">
+      <c r="J19" s="1">
         <v>45846</v>
       </c>
       <c r="K19" t="b">
@@ -2010,7 +1984,7 @@
       <c r="H20">
         <v>-206.4</v>
       </c>
-      <c r="J20" s="2">
+      <c r="J20" s="1">
         <v>36669</v>
       </c>
       <c r="K20" t="b">
@@ -2042,7 +2016,7 @@
       <c r="H21">
         <v>-131.6</v>
       </c>
-      <c r="J21" s="2">
+      <c r="J21" s="1">
         <v>46111</v>
       </c>
       <c r="K21" t="b">
@@ -2074,7 +2048,7 @@
       <c r="H22">
         <v>-131.6</v>
       </c>
-      <c r="J22" s="2">
+      <c r="J22" s="1">
         <v>46111</v>
       </c>
       <c r="K22" t="b">
@@ -2106,7 +2080,7 @@
       <c r="H23">
         <v>-131.6</v>
       </c>
-      <c r="J23" s="2">
+      <c r="J23" s="1">
         <v>46111</v>
       </c>
       <c r="K23" t="b">
@@ -2138,7 +2112,7 @@
       <c r="H24">
         <v>-131.6</v>
       </c>
-      <c r="J24" s="2">
+      <c r="J24" s="1">
         <v>46111</v>
       </c>
       <c r="K24" t="b">
@@ -2170,7 +2144,7 @@
       <c r="H25">
         <v>-131.6</v>
       </c>
-      <c r="J25" s="2">
+      <c r="J25" s="1">
         <v>46111</v>
       </c>
       <c r="K25" t="b">
@@ -2202,7 +2176,7 @@
       <c r="H26">
         <v>-98.3</v>
       </c>
-      <c r="J26" s="2">
+      <c r="J26" s="1">
         <v>41204</v>
       </c>
       <c r="K26" t="b">
@@ -2234,7 +2208,7 @@
       <c r="H27">
         <v>-47.2</v>
       </c>
-      <c r="J27" s="2">
+      <c r="J27" s="1">
         <v>44011</v>
       </c>
       <c r="K27" t="b">
@@ -2266,7 +2240,7 @@
       <c r="H28">
         <v>-22.3</v>
       </c>
-      <c r="J28" s="2">
+      <c r="J28" s="1">
         <v>46226</v>
       </c>
       <c r="K28" t="b">
@@ -2298,7 +2272,7 @@
       <c r="H29">
         <v>4.7</v>
       </c>
-      <c r="J29" s="2">
+      <c r="J29" s="1">
         <v>46265</v>
       </c>
       <c r="K29" t="b">
@@ -2330,7 +2304,7 @@
       <c r="H30">
         <v>7.5</v>
       </c>
-      <c r="J30" s="2">
+      <c r="J30" s="1">
         <v>46265</v>
       </c>
       <c r="K30" t="b">
@@ -2362,7 +2336,7 @@
       <c r="H31">
         <v>10</v>
       </c>
-      <c r="J31" s="2">
+      <c r="J31" s="1">
         <v>46265</v>
       </c>
       <c r="K31" t="b">
@@ -2394,7 +2368,7 @@
       <c r="H32">
         <v>12.8</v>
       </c>
-      <c r="J32" s="2">
+      <c r="J32" s="1">
         <v>46265</v>
       </c>
       <c r="K32" t="b">
@@ -2426,7 +2400,7 @@
       <c r="H33">
         <v>14</v>
       </c>
-      <c r="J33" s="2">
+      <c r="J33" s="1">
         <v>46265</v>
       </c>
       <c r="K33" t="b">
@@ -2458,7 +2432,7 @@
       <c r="H34">
         <v>17.8</v>
       </c>
-      <c r="J34" s="2">
+      <c r="J34" s="1">
         <v>46265</v>
       </c>
       <c r="K34" t="b">
@@ -2490,7 +2464,7 @@
       <c r="H35">
         <v>20.4</v>
       </c>
-      <c r="J35" s="2">
+      <c r="J35" s="1">
         <v>46265</v>
       </c>
       <c r="K35" t="b">
@@ -2522,7 +2496,7 @@
       <c r="H36">
         <v>21.2</v>
       </c>
-      <c r="J36" s="2">
+      <c r="J36" s="1">
         <v>46265</v>
       </c>
       <c r="K36" t="b">
@@ -2554,7 +2528,7 @@
       <c r="H37">
         <v>26.2</v>
       </c>
-      <c r="J37" s="2">
+      <c r="J37" s="1">
         <v>46265</v>
       </c>
       <c r="K37" t="b">
@@ -2586,7 +2560,7 @@
       <c r="H38">
         <v>33.6</v>
       </c>
-      <c r="J38" s="2">
+      <c r="J38" s="1">
         <v>46364</v>
       </c>
       <c r="K38" t="b">
@@ -2618,7 +2592,7 @@
       <c r="H39">
         <v>42.2</v>
       </c>
-      <c r="J39" s="2">
+      <c r="J39" s="1">
         <v>46269</v>
       </c>
       <c r="K39" t="b">
@@ -2650,7 +2624,7 @@
       <c r="H40">
         <v>42.8</v>
       </c>
-      <c r="J40" s="2">
+      <c r="J40" s="1">
         <v>46291</v>
       </c>
       <c r="K40" t="b">
@@ -2682,7 +2656,7 @@
       <c r="H41">
         <v>45.7</v>
       </c>
-      <c r="J41" s="2">
+      <c r="J41" s="1">
         <v>46395</v>
       </c>
       <c r="K41" t="b">
@@ -2714,7 +2688,7 @@
       <c r="H42">
         <v>47.2</v>
       </c>
-      <c r="J42" s="2">
+      <c r="J42" s="1">
         <v>46280</v>
       </c>
       <c r="K42" t="b">
@@ -2746,7 +2720,7 @@
       <c r="H43">
         <v>48.7</v>
       </c>
-      <c r="J43" s="2">
+      <c r="J43" s="1">
         <v>46281</v>
       </c>
       <c r="K43" t="b">
@@ -2778,7 +2752,7 @@
       <c r="H44">
         <v>60</v>
       </c>
-      <c r="J44" s="2">
+      <c r="J44" s="1">
         <v>46281</v>
       </c>
       <c r="K44" t="b">
@@ -2810,7 +2784,7 @@
       <c r="H45">
         <v>62.6</v>
       </c>
-      <c r="J45" s="2">
+      <c r="J45" s="1">
         <v>46265</v>
       </c>
       <c r="K45" t="b">
@@ -2842,7 +2816,7 @@
       <c r="H46">
         <v>64.59999999999999</v>
       </c>
-      <c r="J46" s="2">
+      <c r="J46" s="1">
         <v>46265</v>
       </c>
       <c r="K46" t="b">
@@ -2874,7 +2848,7 @@
       <c r="H47">
         <v>67.59999999999999</v>
       </c>
-      <c r="J47" s="2">
+      <c r="J47" s="1">
         <v>46267</v>
       </c>
       <c r="K47" t="b">
@@ -2906,7 +2880,7 @@
       <c r="H48">
         <v>68.3</v>
       </c>
-      <c r="J48" s="2">
+      <c r="J48" s="1">
         <v>46278</v>
       </c>
       <c r="K48" t="b">
@@ -2938,7 +2912,7 @@
       <c r="H49">
         <v>69.2</v>
       </c>
-      <c r="J49" s="2">
+      <c r="J49" s="1">
         <v>46453</v>
       </c>
       <c r="K49" t="b">
@@ -2970,7 +2944,7 @@
       <c r="H50">
         <v>69.8</v>
       </c>
-      <c r="J50" s="2">
+      <c r="J50" s="1">
         <v>46265</v>
       </c>
       <c r="K50" t="b">
@@ -3002,7 +2976,7 @@
       <c r="H51">
         <v>69.8</v>
       </c>
-      <c r="J51" s="2">
+      <c r="J51" s="1">
         <v>46265</v>
       </c>
       <c r="K51" t="b">
@@ -3034,7 +3008,7 @@
       <c r="H52">
         <v>72.2</v>
       </c>
-      <c r="J52" s="2">
+      <c r="J52" s="1">
         <v>46275</v>
       </c>
       <c r="K52" t="b">
@@ -3066,7 +3040,7 @@
       <c r="H53">
         <v>72.2</v>
       </c>
-      <c r="J53" s="2">
+      <c r="J53" s="1">
         <v>46275</v>
       </c>
       <c r="K53" t="b">
@@ -3098,7 +3072,7 @@
       <c r="H54">
         <v>78.09999999999999</v>
       </c>
-      <c r="J54" s="2">
+      <c r="J54" s="1">
         <v>46265</v>
       </c>
       <c r="K54" t="b">
@@ -3130,7 +3104,7 @@
       <c r="H55">
         <v>82.8</v>
       </c>
-      <c r="J55" s="2">
+      <c r="J55" s="1">
         <v>46487</v>
       </c>
       <c r="K55" t="b">
@@ -3162,7 +3136,7 @@
       <c r="H56">
         <v>83.09999999999999</v>
       </c>
-      <c r="J56" s="2">
+      <c r="J56" s="1">
         <v>46285</v>
       </c>
       <c r="K56" t="b">
@@ -3194,7 +3168,7 @@
       <c r="H57">
         <v>84.8</v>
       </c>
-      <c r="J57" s="2">
+      <c r="J57" s="1">
         <v>46492</v>
       </c>
       <c r="K57" t="b">
@@ -3226,7 +3200,7 @@
       <c r="H58">
         <v>104.9</v>
       </c>
-      <c r="J58" s="2">
+      <c r="J58" s="1">
         <v>46297</v>
       </c>
       <c r="K58" t="b">
@@ -3258,7 +3232,7 @@
       <c r="H59">
         <v>107.6</v>
       </c>
-      <c r="J59" s="2">
+      <c r="J59" s="1">
         <v>46283</v>
       </c>
       <c r="K59" t="b">
@@ -3290,7 +3264,7 @@
       <c r="H60">
         <v>111.9</v>
       </c>
-      <c r="J60" s="2">
+      <c r="J60" s="1">
         <v>46300</v>
       </c>
       <c r="K60" t="b">
@@ -3322,7 +3296,7 @@
       <c r="H61">
         <v>111.9</v>
       </c>
-      <c r="J61" s="2">
+      <c r="J61" s="1">
         <v>46300</v>
       </c>
       <c r="K61" t="b">
@@ -3354,7 +3328,7 @@
       <c r="H62">
         <v>111.9</v>
       </c>
-      <c r="J62" s="2">
+      <c r="J62" s="1">
         <v>46300</v>
       </c>
       <c r="K62" t="b">
@@ -3386,7 +3360,7 @@
       <c r="H63">
         <v>111.9</v>
       </c>
-      <c r="J63" s="2">
+      <c r="J63" s="1">
         <v>46300</v>
       </c>
       <c r="K63" t="b">
@@ -3418,7 +3392,7 @@
       <c r="H64">
         <v>111.9</v>
       </c>
-      <c r="J64" s="2">
+      <c r="J64" s="1">
         <v>46300</v>
       </c>
       <c r="K64" t="b">
@@ -3450,7 +3424,7 @@
       <c r="H65">
         <v>128.8</v>
       </c>
-      <c r="J65" s="2">
+      <c r="J65" s="1">
         <v>46308</v>
       </c>
       <c r="K65" t="b">
@@ -3482,7 +3456,7 @@
       <c r="H66">
         <v>131.1</v>
       </c>
-      <c r="J66" s="2">
+      <c r="J66" s="1">
         <v>46336</v>
       </c>
       <c r="K66" t="b">
@@ -3514,7 +3488,7 @@
       <c r="H67">
         <v>138.4</v>
       </c>
-      <c r="J67" s="2">
+      <c r="J67" s="1">
         <v>46343</v>
       </c>
       <c r="K67" t="b">
@@ -3546,7 +3520,7 @@
       <c r="H68">
         <v>141</v>
       </c>
-      <c r="J68" s="2">
+      <c r="J68" s="1">
         <v>46350</v>
       </c>
       <c r="K68" t="b">
@@ -3578,7 +3552,7 @@
       <c r="H69">
         <v>162</v>
       </c>
-      <c r="J69" s="2">
+      <c r="J69" s="1">
         <v>46391</v>
       </c>
       <c r="K69" t="b">
@@ -3610,7 +3584,7 @@
       <c r="H70">
         <v>167.2</v>
       </c>
-      <c r="J70" s="2">
+      <c r="J70" s="1">
         <v>46330</v>
       </c>
       <c r="K70" t="b">
@@ -3642,7 +3616,7 @@
       <c r="H71">
         <v>177.4</v>
       </c>
-      <c r="J71" s="2">
+      <c r="J71" s="1">
         <v>46418</v>
       </c>
       <c r="K71" t="b">
@@ -3674,7 +3648,7 @@
       <c r="H72">
         <v>200</v>
       </c>
-      <c r="J72" s="2">
+      <c r="J72" s="1">
         <v>46356</v>
       </c>
       <c r="K72" t="b">
@@ -3706,7 +3680,7 @@
       <c r="H73">
         <v>203.6</v>
       </c>
-      <c r="J73" s="2">
+      <c r="J73" s="1">
         <v>46436</v>
       </c>
       <c r="K73" t="b">
@@ -3738,7 +3712,7 @@
       <c r="H74">
         <v>221.2</v>
       </c>
-      <c r="J74" s="2">
+      <c r="J74" s="1">
         <v>46426</v>
       </c>
       <c r="K74" t="b">
@@ -3770,7 +3744,7 @@
       <c r="H75">
         <v>240.8</v>
       </c>
-      <c r="J75" s="2">
+      <c r="J75" s="1">
         <v>46450</v>
       </c>
       <c r="K75" t="b">
@@ -3802,7 +3776,7 @@
       <c r="H76">
         <v>245.8</v>
       </c>
-      <c r="J76" s="2">
+      <c r="J76" s="1">
         <v>46452</v>
       </c>
       <c r="K76" t="b">
@@ -3834,7 +3808,7 @@
       <c r="H77">
         <v>263.4</v>
       </c>
-      <c r="J77" s="2">
+      <c r="J77" s="1">
         <v>46322</v>
       </c>
       <c r="K77" t="b">
@@ -3866,7 +3840,7 @@
       <c r="H78">
         <v>275.2</v>
       </c>
-      <c r="J78" s="2">
+      <c r="J78" s="1">
         <v>46433</v>
       </c>
       <c r="K78" t="b">
@@ -3901,7 +3875,7 @@
       <c r="I79" t="s">
         <v>311</v>
       </c>
-      <c r="J79" s="2">
+      <c r="J79" s="1">
         <v>36557</v>
       </c>
       <c r="K79" t="b">
@@ -3936,7 +3910,7 @@
       <c r="I80" t="s">
         <v>312</v>
       </c>
-      <c r="J80" s="2">
+      <c r="J80" s="1">
         <v>41275</v>
       </c>
       <c r="K80" t="b">
@@ -3971,7 +3945,7 @@
       <c r="I81" t="s">
         <v>313</v>
       </c>
-      <c r="J81" s="2">
+      <c r="J81" s="1">
         <v>45380</v>
       </c>
       <c r="K81" t="b">
@@ -4006,7 +3980,7 @@
       <c r="I82" t="s">
         <v>314</v>
       </c>
-      <c r="J82" s="2">
+      <c r="J82" s="1">
         <v>45421</v>
       </c>
       <c r="K82" t="b">
@@ -4041,7 +4015,7 @@
       <c r="I83" t="s">
         <v>314</v>
       </c>
-      <c r="J83" s="2">
+      <c r="J83" s="1">
         <v>45428</v>
       </c>
       <c r="K83" t="b">
@@ -4076,7 +4050,7 @@
       <c r="I84" t="s">
         <v>315</v>
       </c>
-      <c r="J84" s="2">
+      <c r="J84" s="1">
         <v>45490</v>
       </c>
       <c r="K84" t="b">
@@ -4111,7 +4085,7 @@
       <c r="I85" t="s">
         <v>316</v>
       </c>
-      <c r="J85" s="2">
+      <c r="J85" s="1">
         <v>45566</v>
       </c>
       <c r="K85" t="b">
@@ -4146,7 +4120,7 @@
       <c r="I86" t="s">
         <v>317</v>
       </c>
-      <c r="J86" s="2">
+      <c r="J86" s="1">
         <v>45986</v>
       </c>
       <c r="K86" t="b">
@@ -4181,7 +4155,7 @@
       <c r="I87" t="s">
         <v>318</v>
       </c>
-      <c r="J87" s="2">
+      <c r="J87" s="1">
         <v>46284</v>
       </c>
       <c r="K87" t="b">
@@ -4216,7 +4190,7 @@
       <c r="I88" t="s">
         <v>319</v>
       </c>
-      <c r="J88" s="2">
+      <c r="J88" s="1">
         <v>46305</v>
       </c>
       <c r="K88" t="b">
@@ -4251,7 +4225,7 @@
       <c r="I89" t="s">
         <v>319</v>
       </c>
-      <c r="J89" s="2">
+      <c r="J89" s="1">
         <v>46310</v>
       </c>
       <c r="K89" t="b">
@@ -4286,7 +4260,7 @@
       <c r="I90" t="s">
         <v>319</v>
       </c>
-      <c r="J90" s="2">
+      <c r="J90" s="1">
         <v>46317</v>
       </c>
       <c r="K90" t="b">
@@ -4321,7 +4295,7 @@
       <c r="I91" t="s">
         <v>319</v>
       </c>
-      <c r="J91" s="2">
+      <c r="J91" s="1">
         <v>46319</v>
       </c>
       <c r="K91" t="b">
@@ -4356,7 +4330,7 @@
       <c r="I92" t="s">
         <v>320</v>
       </c>
-      <c r="J92" s="2">
+      <c r="J92" s="1">
         <v>46333</v>
       </c>
       <c r="K92" t="b">
@@ -4391,7 +4365,7 @@
       <c r="I93" t="s">
         <v>320</v>
       </c>
-      <c r="J93" s="2">
+      <c r="J93" s="1">
         <v>46338</v>
       </c>
       <c r="K93" t="b">
@@ -4426,7 +4400,7 @@
       <c r="I94" t="s">
         <v>320</v>
       </c>
-      <c r="J94" s="2">
+      <c r="J94" s="1">
         <v>46338</v>
       </c>
       <c r="K94" t="b">
@@ -4461,7 +4435,7 @@
       <c r="I95" t="s">
         <v>320</v>
       </c>
-      <c r="J95" s="2">
+      <c r="J95" s="1">
         <v>46341</v>
       </c>
       <c r="K95" t="b">
@@ -4496,7 +4470,7 @@
       <c r="I96" t="s">
         <v>320</v>
       </c>
-      <c r="J96" s="2">
+      <c r="J96" s="1">
         <v>46344</v>
       </c>
       <c r="K96" t="b">
@@ -4531,7 +4505,7 @@
       <c r="I97" t="s">
         <v>321</v>
       </c>
-      <c r="J97" s="2">
+      <c r="J97" s="1">
         <v>46360</v>
       </c>
       <c r="K97" t="b">
@@ -4566,7 +4540,7 @@
       <c r="I98" t="s">
         <v>321</v>
       </c>
-      <c r="J98" s="2">
+      <c r="J98" s="1">
         <v>46360</v>
       </c>
       <c r="K98" t="b">
@@ -4601,7 +4575,7 @@
       <c r="I99" t="s">
         <v>321</v>
       </c>
-      <c r="J99" s="2">
+      <c r="J99" s="1">
         <v>46367</v>
       </c>
       <c r="K99" t="b">
@@ -4636,7 +4610,7 @@
       <c r="I100" t="s">
         <v>321</v>
       </c>
-      <c r="J100" s="2">
+      <c r="J100" s="1">
         <v>46375</v>
       </c>
       <c r="K100" t="b">
@@ -4671,7 +4645,7 @@
       <c r="I101" t="s">
         <v>321</v>
       </c>
-      <c r="J101" s="2">
+      <c r="J101" s="1">
         <v>46387</v>
       </c>
       <c r="K101" t="b">
@@ -4706,7 +4680,7 @@
       <c r="I102" t="s">
         <v>321</v>
       </c>
-      <c r="J102" s="2">
+      <c r="J102" s="1">
         <v>46387</v>
       </c>
       <c r="K102" t="b">
@@ -4741,7 +4715,7 @@
       <c r="I103" t="s">
         <v>321</v>
       </c>
-      <c r="J103" s="2">
+      <c r="J103" s="1">
         <v>46387</v>
       </c>
       <c r="K103" t="b">
@@ -4776,7 +4750,7 @@
       <c r="I104" t="s">
         <v>321</v>
       </c>
-      <c r="J104" s="2">
+      <c r="J104" s="1">
         <v>46388</v>
       </c>
       <c r="K104" t="b">
@@ -4811,7 +4785,7 @@
       <c r="I105" t="s">
         <v>322</v>
       </c>
-      <c r="J105" s="2">
+      <c r="J105" s="1">
         <v>46401</v>
       </c>
       <c r="K105" t="b">
@@ -4846,7 +4820,7 @@
       <c r="I106" t="s">
         <v>322</v>
       </c>
-      <c r="J106" s="2">
+      <c r="J106" s="1">
         <v>46401</v>
       </c>
       <c r="K106" t="b">
@@ -4881,7 +4855,7 @@
       <c r="I107" t="s">
         <v>322</v>
       </c>
-      <c r="J107" s="2">
+      <c r="J107" s="1">
         <v>46401</v>
       </c>
       <c r="K107" t="b">
@@ -4916,7 +4890,7 @@
       <c r="I108" t="s">
         <v>322</v>
       </c>
-      <c r="J108" s="2">
+      <c r="J108" s="1">
         <v>46412</v>
       </c>
       <c r="K108" t="b">
@@ -4951,7 +4925,7 @@
       <c r="I109" t="s">
         <v>322</v>
       </c>
-      <c r="J109" s="2">
+      <c r="J109" s="1">
         <v>46412</v>
       </c>
       <c r="K109" t="b">
@@ -4986,7 +4960,7 @@
       <c r="I110" t="s">
         <v>322</v>
       </c>
-      <c r="J110" s="2">
+      <c r="J110" s="1">
         <v>46412</v>
       </c>
       <c r="K110" t="b">
@@ -5021,7 +4995,7 @@
       <c r="I111" t="s">
         <v>323</v>
       </c>
-      <c r="J111" s="2">
+      <c r="J111" s="1">
         <v>46424</v>
       </c>
       <c r="K111" t="b">
@@ -5056,7 +5030,7 @@
       <c r="I112" t="s">
         <v>323</v>
       </c>
-      <c r="J112" s="2">
+      <c r="J112" s="1">
         <v>46437</v>
       </c>
       <c r="K112" t="b">
@@ -5091,7 +5065,7 @@
       <c r="I113" t="s">
         <v>323</v>
       </c>
-      <c r="J113" s="2">
+      <c r="J113" s="1">
         <v>46451</v>
       </c>
       <c r="K113" t="b">
@@ -5126,7 +5100,7 @@
       <c r="I114" t="s">
         <v>323</v>
       </c>
-      <c r="J114" s="2">
+      <c r="J114" s="1">
         <v>46451</v>
       </c>
       <c r="K114" t="b">
@@ -5161,7 +5135,7 @@
       <c r="I115" t="s">
         <v>324</v>
       </c>
-      <c r="J115" s="2">
+      <c r="J115" s="1">
         <v>46455</v>
       </c>
       <c r="K115" t="b">
@@ -5196,7 +5170,7 @@
       <c r="I116" t="s">
         <v>324</v>
       </c>
-      <c r="J116" s="2">
+      <c r="J116" s="1">
         <v>46456</v>
       </c>
       <c r="K116" t="b">
@@ -5231,7 +5205,7 @@
       <c r="I117" t="s">
         <v>324</v>
       </c>
-      <c r="J117" s="2">
+      <c r="J117" s="1">
         <v>46457</v>
       </c>
       <c r="K117" t="b">
@@ -5266,7 +5240,7 @@
       <c r="I118" t="s">
         <v>324</v>
       </c>
-      <c r="J118" s="2">
+      <c r="J118" s="1">
         <v>46464</v>
       </c>
       <c r="K118" t="b">
@@ -5301,7 +5275,7 @@
       <c r="I119" t="s">
         <v>324</v>
       </c>
-      <c r="J119" s="2">
+      <c r="J119" s="1">
         <v>46470</v>
       </c>
       <c r="K119" t="b">
@@ -5336,7 +5310,7 @@
       <c r="I120" t="s">
         <v>325</v>
       </c>
-      <c r="J120" s="2">
+      <c r="J120" s="1">
         <v>46485</v>
       </c>
       <c r="K120" t="b">
@@ -5371,7 +5345,7 @@
       <c r="I121" t="s">
         <v>325</v>
       </c>
-      <c r="J121" s="2">
+      <c r="J121" s="1">
         <v>46499</v>
       </c>
       <c r="K121" t="b">
@@ -5406,7 +5380,7 @@
       <c r="I122" t="s">
         <v>325</v>
       </c>
-      <c r="J122" s="2">
+      <c r="J122" s="1">
         <v>46504</v>
       </c>
       <c r="K122" t="b">
@@ -5441,7 +5415,7 @@
       <c r="I123" t="s">
         <v>325</v>
       </c>
-      <c r="J123" s="2">
+      <c r="J123" s="1">
         <v>46504</v>
       </c>
       <c r="K123" t="b">
@@ -5476,7 +5450,7 @@
       <c r="I124" t="s">
         <v>325</v>
       </c>
-      <c r="J124" s="2">
+      <c r="J124" s="1">
         <v>46507</v>
       </c>
       <c r="K124" t="b">
@@ -5511,7 +5485,7 @@
       <c r="I125" t="s">
         <v>325</v>
       </c>
-      <c r="J125" s="2">
+      <c r="J125" s="1">
         <v>46508</v>
       </c>
       <c r="K125" t="b">
@@ -5546,7 +5520,7 @@
       <c r="I126" t="s">
         <v>325</v>
       </c>
-      <c r="J126" s="2">
+      <c r="J126" s="1">
         <v>46512</v>
       </c>
       <c r="K126" t="b">
@@ -5581,7 +5555,7 @@
       <c r="I127" t="s">
         <v>326</v>
       </c>
-      <c r="J127" s="2">
+      <c r="J127" s="1">
         <v>46512</v>
       </c>
       <c r="K127" t="b">
@@ -5616,7 +5590,7 @@
       <c r="I128" t="s">
         <v>326</v>
       </c>
-      <c r="J128" s="2">
+      <c r="J128" s="1">
         <v>46528</v>
       </c>
       <c r="K128" t="b">
@@ -5651,7 +5625,7 @@
       <c r="I129" t="s">
         <v>326</v>
       </c>
-      <c r="J129" s="2">
+      <c r="J129" s="1">
         <v>46529</v>
       </c>
       <c r="K129" t="b">
@@ -5686,7 +5660,7 @@
       <c r="I130" t="s">
         <v>326</v>
       </c>
-      <c r="J130" s="2">
+      <c r="J130" s="1">
         <v>46537</v>
       </c>
       <c r="K130" t="b">
@@ -5721,7 +5695,7 @@
       <c r="I131" t="s">
         <v>327</v>
       </c>
-      <c r="J131" s="2">
+      <c r="J131" s="1">
         <v>46546</v>
       </c>
       <c r="K131" t="b">
@@ -5756,7 +5730,7 @@
       <c r="I132" t="s">
         <v>327</v>
       </c>
-      <c r="J132" s="2">
+      <c r="J132" s="1">
         <v>46547</v>
       </c>
       <c r="K132" t="b">
@@ -5791,7 +5765,7 @@
       <c r="I133" t="s">
         <v>327</v>
       </c>
-      <c r="J133" s="2">
+      <c r="J133" s="1">
         <v>46547</v>
       </c>
       <c r="K133" t="b">
@@ -5826,7 +5800,7 @@
       <c r="I134" t="s">
         <v>327</v>
       </c>
-      <c r="J134" s="2">
+      <c r="J134" s="1">
         <v>46547</v>
       </c>
       <c r="K134" t="b">
@@ -5861,7 +5835,7 @@
       <c r="I135" t="s">
         <v>327</v>
       </c>
-      <c r="J135" s="2">
+      <c r="J135" s="1">
         <v>46551</v>
       </c>
       <c r="K135" t="b">
@@ -5896,7 +5870,7 @@
       <c r="I136" t="s">
         <v>327</v>
       </c>
-      <c r="J136" s="2">
+      <c r="J136" s="1">
         <v>46560</v>
       </c>
       <c r="K136" t="b">
@@ -5931,7 +5905,7 @@
       <c r="I137" t="s">
         <v>327</v>
       </c>
-      <c r="J137" s="2">
+      <c r="J137" s="1">
         <v>46564</v>
       </c>
       <c r="K137" t="b">
@@ -5966,7 +5940,7 @@
       <c r="I138" t="s">
         <v>327</v>
       </c>
-      <c r="J138" s="2">
+      <c r="J138" s="1">
         <v>46567</v>
       </c>
       <c r="K138" t="b">
@@ -6001,7 +5975,7 @@
       <c r="I139" t="s">
         <v>327</v>
       </c>
-      <c r="J139" s="2">
+      <c r="J139" s="1">
         <v>46568</v>
       </c>
       <c r="K139" t="b">
@@ -6036,7 +6010,7 @@
       <c r="I140" t="s">
         <v>328</v>
       </c>
-      <c r="J140" s="2">
+      <c r="J140" s="1">
         <v>46578</v>
       </c>
       <c r="K140" t="b">
@@ -6071,7 +6045,7 @@
       <c r="I141" t="s">
         <v>328</v>
       </c>
-      <c r="J141" s="2">
+      <c r="J141" s="1">
         <v>46592</v>
       </c>
       <c r="K141" t="b">
@@ -6106,7 +6080,7 @@
       <c r="I142" t="s">
         <v>328</v>
       </c>
-      <c r="J142" s="2">
+      <c r="J142" s="1">
         <v>46592</v>
       </c>
       <c r="K142" t="b">
@@ -6141,7 +6115,7 @@
       <c r="I143" t="s">
         <v>329</v>
       </c>
-      <c r="J143" s="2">
+      <c r="J143" s="1">
         <v>46212</v>
       </c>
       <c r="K143" t="b">
@@ -6176,7 +6150,7 @@
       <c r="I144" t="s">
         <v>330</v>
       </c>
-      <c r="J144" s="2">
+      <c r="J144" s="1">
         <v>46225</v>
       </c>
       <c r="K144" t="b">
@@ -6211,7 +6185,7 @@
       <c r="I145" t="s">
         <v>331</v>
       </c>
-      <c r="J145" s="2">
+      <c r="J145" s="1">
         <v>46263</v>
       </c>
       <c r="K145" t="b">
@@ -6243,7 +6217,7 @@
       <c r="H146">
         <v>-1476</v>
       </c>
-      <c r="J146" s="2">
+      <c r="J146" s="1">
         <v>43773</v>
       </c>
       <c r="K146" t="b">
@@ -6275,7 +6249,7 @@
       <c r="H147">
         <v>-1469</v>
       </c>
-      <c r="J147" s="2">
+      <c r="J147" s="1">
         <v>43773</v>
       </c>
       <c r="K147" t="b">
@@ -6307,7 +6281,7 @@
       <c r="H148">
         <v>-1186</v>
       </c>
-      <c r="J148" s="2">
+      <c r="J148" s="1">
         <v>45295</v>
       </c>
       <c r="K148" t="b">
@@ -6339,7 +6313,7 @@
       <c r="H149">
         <v>-1048</v>
       </c>
-      <c r="J149" s="2">
+      <c r="J149" s="1">
         <v>45617</v>
       </c>
       <c r="K149" t="b">
@@ -6371,7 +6345,7 @@
       <c r="H150">
         <v>-980</v>
       </c>
-      <c r="J150" s="2">
+      <c r="J150" s="1">
         <v>45677</v>
       </c>
       <c r="K150" t="b">
@@ -6403,7 +6377,7 @@
       <c r="H151">
         <v>-961</v>
       </c>
-      <c r="J151" s="2">
+      <c r="J151" s="1">
         <v>44944</v>
       </c>
       <c r="K151" t="b">
@@ -6435,7 +6409,7 @@
       <c r="H152">
         <v>-252</v>
       </c>
-      <c r="J152" s="2">
+      <c r="J152" s="1">
         <v>46092</v>
       </c>
       <c r="K152" t="b">
@@ -6467,7 +6441,7 @@
       <c r="H153">
         <v>3</v>
       </c>
-      <c r="J153" s="2">
+      <c r="J153" s="1">
         <v>46265</v>
       </c>
       <c r="K153" t="b">
@@ -6499,7 +6473,7 @@
       <c r="H154">
         <v>3</v>
       </c>
-      <c r="J154" s="2">
+      <c r="J154" s="1">
         <v>46265</v>
       </c>
       <c r="K154" t="b">
@@ -6531,7 +6505,7 @@
       <c r="H155">
         <v>43</v>
       </c>
-      <c r="J155" s="2">
+      <c r="J155" s="1">
         <v>46440</v>
       </c>
       <c r="K155" t="b">
@@ -6563,7 +6537,7 @@
       <c r="H156">
         <v>43</v>
       </c>
-      <c r="J156" s="2">
+      <c r="J156" s="1">
         <v>46440</v>
       </c>
       <c r="K156" t="b">
@@ -6595,7 +6569,7 @@
       <c r="H157">
         <v>72</v>
       </c>
-      <c r="J157" s="2">
+      <c r="J157" s="1">
         <v>46289</v>
       </c>
       <c r="K157" t="b">
@@ -6627,7 +6601,7 @@
       <c r="H158">
         <v>72</v>
       </c>
-      <c r="J158" s="2">
+      <c r="J158" s="1">
         <v>46289</v>
       </c>
       <c r="K158" t="b">
@@ -6659,7 +6633,7 @@
       <c r="H159">
         <v>81</v>
       </c>
-      <c r="J159" s="2">
+      <c r="J159" s="1">
         <v>46405</v>
       </c>
       <c r="K159" t="b">
@@ -6691,7 +6665,7 @@
       <c r="H160">
         <v>102</v>
       </c>
-      <c r="J160" s="2">
+      <c r="J160" s="1">
         <v>46463</v>
       </c>
       <c r="K160" t="b">
@@ -6723,7 +6697,7 @@
       <c r="H161">
         <v>109</v>
       </c>
-      <c r="J161" s="2">
+      <c r="J161" s="1">
         <v>46353</v>
       </c>
       <c r="K161" t="b">
@@ -6755,7 +6729,7 @@
       <c r="H162">
         <v>127</v>
       </c>
-      <c r="J162" s="2">
+      <c r="J162" s="1">
         <v>46417</v>
       </c>
       <c r="K162" t="b">
@@ -6787,7 +6761,7 @@
       <c r="H163">
         <v>152</v>
       </c>
-      <c r="J163" s="2">
+      <c r="J163" s="1">
         <v>46271</v>
       </c>
       <c r="K163" t="b">
@@ -6819,7 +6793,7 @@
       <c r="H164">
         <v>152</v>
       </c>
-      <c r="J164" s="2">
+      <c r="J164" s="1">
         <v>46271</v>
       </c>
       <c r="K164" t="b">
@@ -6851,7 +6825,7 @@
       <c r="H165">
         <v>153</v>
       </c>
-      <c r="J165" s="2">
+      <c r="J165" s="1">
         <v>46458</v>
       </c>
       <c r="K165" t="b">
@@ -6883,7 +6857,7 @@
       <c r="H166">
         <v>158</v>
       </c>
-      <c r="J166" s="2">
+      <c r="J166" s="1">
         <v>46381</v>
       </c>
       <c r="K166" t="b">
@@ -6915,7 +6889,7 @@
       <c r="H167">
         <v>163</v>
       </c>
-      <c r="J167" s="2">
+      <c r="J167" s="1">
         <v>46592</v>
       </c>
       <c r="K167" t="b">
@@ -6947,7 +6921,7 @@
       <c r="H168">
         <v>167</v>
       </c>
-      <c r="J168" s="2">
+      <c r="J168" s="1">
         <v>46441</v>
       </c>
       <c r="K168" t="b">
@@ -6979,7 +6953,7 @@
       <c r="H169">
         <v>169</v>
       </c>
-      <c r="J169" s="2">
+      <c r="J169" s="1">
         <v>46391</v>
       </c>
       <c r="K169" t="b">
@@ -7011,7 +6985,7 @@
       <c r="H170">
         <v>184</v>
       </c>
-      <c r="J170" s="2">
+      <c r="J170" s="1">
         <v>46385</v>
       </c>
       <c r="K170" t="b">
@@ -7043,7 +7017,7 @@
       <c r="H171">
         <v>186</v>
       </c>
-      <c r="J171" s="2">
+      <c r="J171" s="1">
         <v>46387</v>
       </c>
       <c r="K171" t="b">
@@ -7075,7 +7049,7 @@
       <c r="H172">
         <v>206</v>
       </c>
-      <c r="J172" s="2">
+      <c r="J172" s="1">
         <v>46399</v>
       </c>
       <c r="K172" t="b">
@@ -7107,7 +7081,7 @@
       <c r="H173">
         <v>206</v>
       </c>
-      <c r="J173" s="2">
+      <c r="J173" s="1">
         <v>46399</v>
       </c>
       <c r="K173" t="b">
@@ -7139,7 +7113,7 @@
       <c r="H174">
         <v>234</v>
       </c>
-      <c r="J174" s="2">
+      <c r="J174" s="1">
         <v>46458</v>
       </c>
       <c r="K174" t="b">
@@ -7171,7 +7145,7 @@
       <c r="H175">
         <v>248</v>
       </c>
-      <c r="J175" s="2">
+      <c r="J175" s="1">
         <v>46528</v>
       </c>
       <c r="K175" t="b">
@@ -7203,7 +7177,7 @@
       <c r="H176">
         <v>317</v>
       </c>
-      <c r="J176" s="2">
+      <c r="J176" s="1">
         <v>46540</v>
       </c>
       <c r="K176" t="b">
@@ -7235,7 +7209,7 @@
       <c r="H177">
         <v>340</v>
       </c>
-      <c r="J177" s="2">
+      <c r="J177" s="1">
         <v>46547</v>
       </c>
       <c r="K177" t="b">
@@ -7267,7 +7241,7 @@
       <c r="H178">
         <v>364</v>
       </c>
-      <c r="J178" s="2">
+      <c r="J178" s="1">
         <v>46557</v>
       </c>
       <c r="K178" t="b">
@@ -7299,7 +7273,7 @@
       <c r="H179">
         <v>368</v>
       </c>
-      <c r="J179" s="2">
+      <c r="J179" s="1">
         <v>46571</v>
       </c>
       <c r="K179" t="b">
@@ -7331,7 +7305,7 @@
       <c r="H180">
         <v>368</v>
       </c>
-      <c r="J180" s="2">
+      <c r="J180" s="1">
         <v>46571</v>
       </c>
       <c r="K180" t="b">
@@ -7363,7 +7337,7 @@
       <c r="H181">
         <v>370</v>
       </c>
-      <c r="J181" s="2">
+      <c r="J181" s="1">
         <v>46562</v>
       </c>
       <c r="K181" t="b">
@@ -7395,7 +7369,7 @@
       <c r="H182">
         <v>385</v>
       </c>
-      <c r="J182" s="2">
+      <c r="J182" s="1">
         <v>46574</v>
       </c>
       <c r="K182" t="b">
@@ -7427,7 +7401,7 @@
       <c r="H183">
         <v>385</v>
       </c>
-      <c r="J183" s="2">
+      <c r="J183" s="1">
         <v>46574</v>
       </c>
       <c r="K183" t="b">
@@ -7459,7 +7433,7 @@
       <c r="H184">
         <v>417</v>
       </c>
-      <c r="J184" s="2">
+      <c r="J184" s="1">
         <v>46578</v>
       </c>
       <c r="K184" t="b">
@@ -7491,7 +7465,7 @@
       <c r="H185">
         <v>721</v>
       </c>
-      <c r="J185" s="2">
+      <c r="J185" s="1">
         <v>46345</v>
       </c>
       <c r="K185" t="b">
@@ -7523,7 +7497,7 @@
       <c r="H186">
         <v>721</v>
       </c>
-      <c r="J186" s="2">
+      <c r="J186" s="1">
         <v>46345</v>
       </c>
       <c r="K186" t="b">
@@ -7555,7 +7529,7 @@
       <c r="H187">
         <v>850</v>
       </c>
-      <c r="J187" s="2">
+      <c r="J187" s="1">
         <v>46366</v>
       </c>
       <c r="K187" t="b">
@@ -7587,7 +7561,7 @@
       <c r="H188">
         <v>850</v>
       </c>
-      <c r="J188" s="2">
+      <c r="J188" s="1">
         <v>46366</v>
       </c>
       <c r="K188" t="b">
@@ -7619,7 +7593,7 @@
       <c r="H189">
         <v>1661</v>
       </c>
-      <c r="J189" s="2">
+      <c r="J189" s="1">
         <v>46524</v>
       </c>
       <c r="K189" t="b">
@@ -7651,7 +7625,7 @@
       <c r="H190">
         <v>1661</v>
       </c>
-      <c r="J190" s="2">
+      <c r="J190" s="1">
         <v>46524</v>
       </c>
       <c r="K190" t="b">
@@ -7683,7 +7657,7 @@
       <c r="H191">
         <v>488</v>
       </c>
-      <c r="J191" s="2">
+      <c r="J191" s="1">
         <v>46190</v>
       </c>
       <c r="K191" t="b">
@@ -7715,7 +7689,7 @@
       <c r="H192">
         <v>25565</v>
       </c>
-      <c r="J192" s="2">
+      <c r="J192" s="1">
         <v>46190</v>
       </c>
       <c r="K192" t="b">
@@ -7747,7 +7721,7 @@
       <c r="H193">
         <v>25567</v>
       </c>
-      <c r="J193" s="2">
+      <c r="J193" s="1">
         <v>46190</v>
       </c>
       <c r="K193" t="b">
@@ -7779,7 +7753,7 @@
       <c r="H194">
         <v>31293</v>
       </c>
-      <c r="J194" s="2">
+      <c r="J194" s="1">
         <v>46190</v>
       </c>
       <c r="K194" t="b">

</xml_diff>

<commit_message>
Atualização automática: vencimentos_tmot (25/08/2026 08:31)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
@@ -1019,8 +1019,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1036,7 +1044,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1044,12 +1052,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1349,37 +1375,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1408,7 +1434,7 @@
       <c r="H2">
         <v>-4300.3</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>39285</v>
       </c>
       <c r="K2" t="b">
@@ -1440,7 +1466,7 @@
       <c r="H3">
         <v>-2354.2</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>40669</v>
       </c>
       <c r="K3" t="b">
@@ -1472,7 +1498,7 @@
       <c r="H4">
         <v>-910.7</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>40669</v>
       </c>
       <c r="K4" t="b">
@@ -1504,7 +1530,7 @@
       <c r="H5">
         <v>-868</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>44884</v>
       </c>
       <c r="K5" t="b">
@@ -1536,7 +1562,7 @@
       <c r="H6">
         <v>-483.8</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>43855</v>
       </c>
       <c r="K6" t="b">
@@ -1568,7 +1594,7 @@
       <c r="H7">
         <v>-417</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>46014</v>
       </c>
       <c r="K7" t="b">
@@ -1600,7 +1626,7 @@
       <c r="H8">
         <v>-414.2</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>46014</v>
       </c>
       <c r="K8" t="b">
@@ -1632,7 +1658,7 @@
       <c r="H9">
         <v>-391.8</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>42769</v>
       </c>
       <c r="K9" t="b">
@@ -1664,7 +1690,7 @@
       <c r="H10">
         <v>-391.6</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>45804</v>
       </c>
       <c r="K10" t="b">
@@ -1696,7 +1722,7 @@
       <c r="H11">
         <v>-391.6</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>45804</v>
       </c>
       <c r="K11" t="b">
@@ -1728,7 +1754,7 @@
       <c r="H12">
         <v>-372.9</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>42821</v>
       </c>
       <c r="K12" t="b">
@@ -1760,7 +1786,7 @@
       <c r="H13">
         <v>-372.9</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>46014</v>
       </c>
       <c r="K13" t="b">
@@ -1792,7 +1818,7 @@
       <c r="H14">
         <v>-372.9</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>46014</v>
       </c>
       <c r="K14" t="b">
@@ -1824,7 +1850,7 @@
       <c r="H15">
         <v>-372.9</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>46014</v>
       </c>
       <c r="K15" t="b">
@@ -1856,7 +1882,7 @@
       <c r="H16">
         <v>-367.8</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="2">
         <v>46017</v>
       </c>
       <c r="K16" t="b">
@@ -1888,7 +1914,7 @@
       <c r="H17">
         <v>-367.8</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="2">
         <v>46017</v>
       </c>
       <c r="K17" t="b">
@@ -1920,7 +1946,7 @@
       <c r="H18">
         <v>-347.2</v>
       </c>
-      <c r="J18" s="1">
+      <c r="J18" s="2">
         <v>40979</v>
       </c>
       <c r="K18" t="b">
@@ -1952,7 +1978,7 @@
       <c r="H19">
         <v>-293.8</v>
       </c>
-      <c r="J19" s="1">
+      <c r="J19" s="2">
         <v>45846</v>
       </c>
       <c r="K19" t="b">
@@ -1984,7 +2010,7 @@
       <c r="H20">
         <v>-206.4</v>
       </c>
-      <c r="J20" s="1">
+      <c r="J20" s="2">
         <v>36669</v>
       </c>
       <c r="K20" t="b">
@@ -2016,7 +2042,7 @@
       <c r="H21">
         <v>-131.6</v>
       </c>
-      <c r="J21" s="1">
+      <c r="J21" s="2">
         <v>46111</v>
       </c>
       <c r="K21" t="b">
@@ -2048,7 +2074,7 @@
       <c r="H22">
         <v>-131.6</v>
       </c>
-      <c r="J22" s="1">
+      <c r="J22" s="2">
         <v>46111</v>
       </c>
       <c r="K22" t="b">
@@ -2080,7 +2106,7 @@
       <c r="H23">
         <v>-131.6</v>
       </c>
-      <c r="J23" s="1">
+      <c r="J23" s="2">
         <v>46111</v>
       </c>
       <c r="K23" t="b">
@@ -2112,7 +2138,7 @@
       <c r="H24">
         <v>-131.6</v>
       </c>
-      <c r="J24" s="1">
+      <c r="J24" s="2">
         <v>46111</v>
       </c>
       <c r="K24" t="b">
@@ -2144,7 +2170,7 @@
       <c r="H25">
         <v>-131.6</v>
       </c>
-      <c r="J25" s="1">
+      <c r="J25" s="2">
         <v>46111</v>
       </c>
       <c r="K25" t="b">
@@ -2176,7 +2202,7 @@
       <c r="H26">
         <v>-98.3</v>
       </c>
-      <c r="J26" s="1">
+      <c r="J26" s="2">
         <v>41204</v>
       </c>
       <c r="K26" t="b">
@@ -2208,7 +2234,7 @@
       <c r="H27">
         <v>-47.2</v>
       </c>
-      <c r="J27" s="1">
+      <c r="J27" s="2">
         <v>44011</v>
       </c>
       <c r="K27" t="b">
@@ -2240,7 +2266,7 @@
       <c r="H28">
         <v>-22.3</v>
       </c>
-      <c r="J28" s="1">
+      <c r="J28" s="2">
         <v>46226</v>
       </c>
       <c r="K28" t="b">
@@ -2272,7 +2298,7 @@
       <c r="H29">
         <v>4.7</v>
       </c>
-      <c r="J29" s="1">
+      <c r="J29" s="2">
         <v>46265</v>
       </c>
       <c r="K29" t="b">
@@ -2304,7 +2330,7 @@
       <c r="H30">
         <v>7.5</v>
       </c>
-      <c r="J30" s="1">
+      <c r="J30" s="2">
         <v>46265</v>
       </c>
       <c r="K30" t="b">
@@ -2336,7 +2362,7 @@
       <c r="H31">
         <v>10</v>
       </c>
-      <c r="J31" s="1">
+      <c r="J31" s="2">
         <v>46265</v>
       </c>
       <c r="K31" t="b">
@@ -2368,7 +2394,7 @@
       <c r="H32">
         <v>12.8</v>
       </c>
-      <c r="J32" s="1">
+      <c r="J32" s="2">
         <v>46265</v>
       </c>
       <c r="K32" t="b">
@@ -2400,7 +2426,7 @@
       <c r="H33">
         <v>14</v>
       </c>
-      <c r="J33" s="1">
+      <c r="J33" s="2">
         <v>46265</v>
       </c>
       <c r="K33" t="b">
@@ -2432,7 +2458,7 @@
       <c r="H34">
         <v>17.8</v>
       </c>
-      <c r="J34" s="1">
+      <c r="J34" s="2">
         <v>46265</v>
       </c>
       <c r="K34" t="b">
@@ -2464,7 +2490,7 @@
       <c r="H35">
         <v>20.4</v>
       </c>
-      <c r="J35" s="1">
+      <c r="J35" s="2">
         <v>46265</v>
       </c>
       <c r="K35" t="b">
@@ -2496,7 +2522,7 @@
       <c r="H36">
         <v>21.2</v>
       </c>
-      <c r="J36" s="1">
+      <c r="J36" s="2">
         <v>46265</v>
       </c>
       <c r="K36" t="b">
@@ -2528,7 +2554,7 @@
       <c r="H37">
         <v>26.2</v>
       </c>
-      <c r="J37" s="1">
+      <c r="J37" s="2">
         <v>46265</v>
       </c>
       <c r="K37" t="b">
@@ -2560,7 +2586,7 @@
       <c r="H38">
         <v>33.6</v>
       </c>
-      <c r="J38" s="1">
+      <c r="J38" s="2">
         <v>46364</v>
       </c>
       <c r="K38" t="b">
@@ -2592,7 +2618,7 @@
       <c r="H39">
         <v>42.2</v>
       </c>
-      <c r="J39" s="1">
+      <c r="J39" s="2">
         <v>46269</v>
       </c>
       <c r="K39" t="b">
@@ -2624,7 +2650,7 @@
       <c r="H40">
         <v>42.8</v>
       </c>
-      <c r="J40" s="1">
+      <c r="J40" s="2">
         <v>46291</v>
       </c>
       <c r="K40" t="b">
@@ -2656,7 +2682,7 @@
       <c r="H41">
         <v>45.7</v>
       </c>
-      <c r="J41" s="1">
+      <c r="J41" s="2">
         <v>46395</v>
       </c>
       <c r="K41" t="b">
@@ -2688,7 +2714,7 @@
       <c r="H42">
         <v>47.2</v>
       </c>
-      <c r="J42" s="1">
+      <c r="J42" s="2">
         <v>46280</v>
       </c>
       <c r="K42" t="b">
@@ -2720,7 +2746,7 @@
       <c r="H43">
         <v>48.7</v>
       </c>
-      <c r="J43" s="1">
+      <c r="J43" s="2">
         <v>46281</v>
       </c>
       <c r="K43" t="b">
@@ -2752,7 +2778,7 @@
       <c r="H44">
         <v>60</v>
       </c>
-      <c r="J44" s="1">
+      <c r="J44" s="2">
         <v>46281</v>
       </c>
       <c r="K44" t="b">
@@ -2784,7 +2810,7 @@
       <c r="H45">
         <v>62.6</v>
       </c>
-      <c r="J45" s="1">
+      <c r="J45" s="2">
         <v>46265</v>
       </c>
       <c r="K45" t="b">
@@ -2816,7 +2842,7 @@
       <c r="H46">
         <v>64.59999999999999</v>
       </c>
-      <c r="J46" s="1">
+      <c r="J46" s="2">
         <v>46265</v>
       </c>
       <c r="K46" t="b">
@@ -2848,7 +2874,7 @@
       <c r="H47">
         <v>67.59999999999999</v>
       </c>
-      <c r="J47" s="1">
+      <c r="J47" s="2">
         <v>46267</v>
       </c>
       <c r="K47" t="b">
@@ -2880,7 +2906,7 @@
       <c r="H48">
         <v>68.3</v>
       </c>
-      <c r="J48" s="1">
+      <c r="J48" s="2">
         <v>46278</v>
       </c>
       <c r="K48" t="b">
@@ -2912,7 +2938,7 @@
       <c r="H49">
         <v>69.2</v>
       </c>
-      <c r="J49" s="1">
+      <c r="J49" s="2">
         <v>46453</v>
       </c>
       <c r="K49" t="b">
@@ -2944,7 +2970,7 @@
       <c r="H50">
         <v>69.8</v>
       </c>
-      <c r="J50" s="1">
+      <c r="J50" s="2">
         <v>46265</v>
       </c>
       <c r="K50" t="b">
@@ -2976,7 +3002,7 @@
       <c r="H51">
         <v>69.8</v>
       </c>
-      <c r="J51" s="1">
+      <c r="J51" s="2">
         <v>46265</v>
       </c>
       <c r="K51" t="b">
@@ -3008,7 +3034,7 @@
       <c r="H52">
         <v>72.2</v>
       </c>
-      <c r="J52" s="1">
+      <c r="J52" s="2">
         <v>46275</v>
       </c>
       <c r="K52" t="b">
@@ -3040,7 +3066,7 @@
       <c r="H53">
         <v>72.2</v>
       </c>
-      <c r="J53" s="1">
+      <c r="J53" s="2">
         <v>46275</v>
       </c>
       <c r="K53" t="b">
@@ -3072,7 +3098,7 @@
       <c r="H54">
         <v>78.09999999999999</v>
       </c>
-      <c r="J54" s="1">
+      <c r="J54" s="2">
         <v>46265</v>
       </c>
       <c r="K54" t="b">
@@ -3104,7 +3130,7 @@
       <c r="H55">
         <v>82.8</v>
       </c>
-      <c r="J55" s="1">
+      <c r="J55" s="2">
         <v>46487</v>
       </c>
       <c r="K55" t="b">
@@ -3136,7 +3162,7 @@
       <c r="H56">
         <v>83.09999999999999</v>
       </c>
-      <c r="J56" s="1">
+      <c r="J56" s="2">
         <v>46285</v>
       </c>
       <c r="K56" t="b">
@@ -3168,7 +3194,7 @@
       <c r="H57">
         <v>84.8</v>
       </c>
-      <c r="J57" s="1">
+      <c r="J57" s="2">
         <v>46492</v>
       </c>
       <c r="K57" t="b">
@@ -3200,7 +3226,7 @@
       <c r="H58">
         <v>104.9</v>
       </c>
-      <c r="J58" s="1">
+      <c r="J58" s="2">
         <v>46297</v>
       </c>
       <c r="K58" t="b">
@@ -3232,7 +3258,7 @@
       <c r="H59">
         <v>107.6</v>
       </c>
-      <c r="J59" s="1">
+      <c r="J59" s="2">
         <v>46283</v>
       </c>
       <c r="K59" t="b">
@@ -3264,7 +3290,7 @@
       <c r="H60">
         <v>111.9</v>
       </c>
-      <c r="J60" s="1">
+      <c r="J60" s="2">
         <v>46300</v>
       </c>
       <c r="K60" t="b">
@@ -3296,7 +3322,7 @@
       <c r="H61">
         <v>111.9</v>
       </c>
-      <c r="J61" s="1">
+      <c r="J61" s="2">
         <v>46300</v>
       </c>
       <c r="K61" t="b">
@@ -3328,7 +3354,7 @@
       <c r="H62">
         <v>111.9</v>
       </c>
-      <c r="J62" s="1">
+      <c r="J62" s="2">
         <v>46300</v>
       </c>
       <c r="K62" t="b">
@@ -3360,7 +3386,7 @@
       <c r="H63">
         <v>111.9</v>
       </c>
-      <c r="J63" s="1">
+      <c r="J63" s="2">
         <v>46300</v>
       </c>
       <c r="K63" t="b">
@@ -3392,7 +3418,7 @@
       <c r="H64">
         <v>111.9</v>
       </c>
-      <c r="J64" s="1">
+      <c r="J64" s="2">
         <v>46300</v>
       </c>
       <c r="K64" t="b">
@@ -3424,7 +3450,7 @@
       <c r="H65">
         <v>128.8</v>
       </c>
-      <c r="J65" s="1">
+      <c r="J65" s="2">
         <v>46308</v>
       </c>
       <c r="K65" t="b">
@@ -3456,7 +3482,7 @@
       <c r="H66">
         <v>131.1</v>
       </c>
-      <c r="J66" s="1">
+      <c r="J66" s="2">
         <v>46336</v>
       </c>
       <c r="K66" t="b">
@@ -3488,7 +3514,7 @@
       <c r="H67">
         <v>138.4</v>
       </c>
-      <c r="J67" s="1">
+      <c r="J67" s="2">
         <v>46343</v>
       </c>
       <c r="K67" t="b">
@@ -3520,7 +3546,7 @@
       <c r="H68">
         <v>141</v>
       </c>
-      <c r="J68" s="1">
+      <c r="J68" s="2">
         <v>46350</v>
       </c>
       <c r="K68" t="b">
@@ -3552,7 +3578,7 @@
       <c r="H69">
         <v>162</v>
       </c>
-      <c r="J69" s="1">
+      <c r="J69" s="2">
         <v>46391</v>
       </c>
       <c r="K69" t="b">
@@ -3584,7 +3610,7 @@
       <c r="H70">
         <v>167.2</v>
       </c>
-      <c r="J70" s="1">
+      <c r="J70" s="2">
         <v>46330</v>
       </c>
       <c r="K70" t="b">
@@ -3616,7 +3642,7 @@
       <c r="H71">
         <v>177.4</v>
       </c>
-      <c r="J71" s="1">
+      <c r="J71" s="2">
         <v>46418</v>
       </c>
       <c r="K71" t="b">
@@ -3648,7 +3674,7 @@
       <c r="H72">
         <v>200</v>
       </c>
-      <c r="J72" s="1">
+      <c r="J72" s="2">
         <v>46356</v>
       </c>
       <c r="K72" t="b">
@@ -3680,7 +3706,7 @@
       <c r="H73">
         <v>203.6</v>
       </c>
-      <c r="J73" s="1">
+      <c r="J73" s="2">
         <v>46436</v>
       </c>
       <c r="K73" t="b">
@@ -3712,7 +3738,7 @@
       <c r="H74">
         <v>221.2</v>
       </c>
-      <c r="J74" s="1">
+      <c r="J74" s="2">
         <v>46426</v>
       </c>
       <c r="K74" t="b">
@@ -3744,7 +3770,7 @@
       <c r="H75">
         <v>240.8</v>
       </c>
-      <c r="J75" s="1">
+      <c r="J75" s="2">
         <v>46450</v>
       </c>
       <c r="K75" t="b">
@@ -3776,7 +3802,7 @@
       <c r="H76">
         <v>245.8</v>
       </c>
-      <c r="J76" s="1">
+      <c r="J76" s="2">
         <v>46452</v>
       </c>
       <c r="K76" t="b">
@@ -3808,7 +3834,7 @@
       <c r="H77">
         <v>263.4</v>
       </c>
-      <c r="J77" s="1">
+      <c r="J77" s="2">
         <v>46322</v>
       </c>
       <c r="K77" t="b">
@@ -3840,7 +3866,7 @@
       <c r="H78">
         <v>275.2</v>
       </c>
-      <c r="J78" s="1">
+      <c r="J78" s="2">
         <v>46433</v>
       </c>
       <c r="K78" t="b">
@@ -3875,7 +3901,7 @@
       <c r="I79" t="s">
         <v>311</v>
       </c>
-      <c r="J79" s="1">
+      <c r="J79" s="2">
         <v>36557</v>
       </c>
       <c r="K79" t="b">
@@ -3910,7 +3936,7 @@
       <c r="I80" t="s">
         <v>312</v>
       </c>
-      <c r="J80" s="1">
+      <c r="J80" s="2">
         <v>41275</v>
       </c>
       <c r="K80" t="b">
@@ -3945,7 +3971,7 @@
       <c r="I81" t="s">
         <v>313</v>
       </c>
-      <c r="J81" s="1">
+      <c r="J81" s="2">
         <v>45380</v>
       </c>
       <c r="K81" t="b">
@@ -3980,7 +4006,7 @@
       <c r="I82" t="s">
         <v>314</v>
       </c>
-      <c r="J82" s="1">
+      <c r="J82" s="2">
         <v>45421</v>
       </c>
       <c r="K82" t="b">
@@ -4015,7 +4041,7 @@
       <c r="I83" t="s">
         <v>314</v>
       </c>
-      <c r="J83" s="1">
+      <c r="J83" s="2">
         <v>45428</v>
       </c>
       <c r="K83" t="b">
@@ -4050,7 +4076,7 @@
       <c r="I84" t="s">
         <v>315</v>
       </c>
-      <c r="J84" s="1">
+      <c r="J84" s="2">
         <v>45490</v>
       </c>
       <c r="K84" t="b">
@@ -4085,7 +4111,7 @@
       <c r="I85" t="s">
         <v>316</v>
       </c>
-      <c r="J85" s="1">
+      <c r="J85" s="2">
         <v>45566</v>
       </c>
       <c r="K85" t="b">
@@ -4120,7 +4146,7 @@
       <c r="I86" t="s">
         <v>317</v>
       </c>
-      <c r="J86" s="1">
+      <c r="J86" s="2">
         <v>45986</v>
       </c>
       <c r="K86" t="b">
@@ -4155,7 +4181,7 @@
       <c r="I87" t="s">
         <v>318</v>
       </c>
-      <c r="J87" s="1">
+      <c r="J87" s="2">
         <v>46284</v>
       </c>
       <c r="K87" t="b">
@@ -4190,7 +4216,7 @@
       <c r="I88" t="s">
         <v>319</v>
       </c>
-      <c r="J88" s="1">
+      <c r="J88" s="2">
         <v>46305</v>
       </c>
       <c r="K88" t="b">
@@ -4225,7 +4251,7 @@
       <c r="I89" t="s">
         <v>319</v>
       </c>
-      <c r="J89" s="1">
+      <c r="J89" s="2">
         <v>46310</v>
       </c>
       <c r="K89" t="b">
@@ -4260,7 +4286,7 @@
       <c r="I90" t="s">
         <v>319</v>
       </c>
-      <c r="J90" s="1">
+      <c r="J90" s="2">
         <v>46317</v>
       </c>
       <c r="K90" t="b">
@@ -4295,7 +4321,7 @@
       <c r="I91" t="s">
         <v>319</v>
       </c>
-      <c r="J91" s="1">
+      <c r="J91" s="2">
         <v>46319</v>
       </c>
       <c r="K91" t="b">
@@ -4330,7 +4356,7 @@
       <c r="I92" t="s">
         <v>320</v>
       </c>
-      <c r="J92" s="1">
+      <c r="J92" s="2">
         <v>46333</v>
       </c>
       <c r="K92" t="b">
@@ -4365,7 +4391,7 @@
       <c r="I93" t="s">
         <v>320</v>
       </c>
-      <c r="J93" s="1">
+      <c r="J93" s="2">
         <v>46338</v>
       </c>
       <c r="K93" t="b">
@@ -4400,7 +4426,7 @@
       <c r="I94" t="s">
         <v>320</v>
       </c>
-      <c r="J94" s="1">
+      <c r="J94" s="2">
         <v>46338</v>
       </c>
       <c r="K94" t="b">
@@ -4435,7 +4461,7 @@
       <c r="I95" t="s">
         <v>320</v>
       </c>
-      <c r="J95" s="1">
+      <c r="J95" s="2">
         <v>46341</v>
       </c>
       <c r="K95" t="b">
@@ -4470,7 +4496,7 @@
       <c r="I96" t="s">
         <v>320</v>
       </c>
-      <c r="J96" s="1">
+      <c r="J96" s="2">
         <v>46344</v>
       </c>
       <c r="K96" t="b">
@@ -4505,7 +4531,7 @@
       <c r="I97" t="s">
         <v>321</v>
       </c>
-      <c r="J97" s="1">
+      <c r="J97" s="2">
         <v>46360</v>
       </c>
       <c r="K97" t="b">
@@ -4540,7 +4566,7 @@
       <c r="I98" t="s">
         <v>321</v>
       </c>
-      <c r="J98" s="1">
+      <c r="J98" s="2">
         <v>46360</v>
       </c>
       <c r="K98" t="b">
@@ -4575,7 +4601,7 @@
       <c r="I99" t="s">
         <v>321</v>
       </c>
-      <c r="J99" s="1">
+      <c r="J99" s="2">
         <v>46367</v>
       </c>
       <c r="K99" t="b">
@@ -4610,7 +4636,7 @@
       <c r="I100" t="s">
         <v>321</v>
       </c>
-      <c r="J100" s="1">
+      <c r="J100" s="2">
         <v>46375</v>
       </c>
       <c r="K100" t="b">
@@ -4645,7 +4671,7 @@
       <c r="I101" t="s">
         <v>321</v>
       </c>
-      <c r="J101" s="1">
+      <c r="J101" s="2">
         <v>46387</v>
       </c>
       <c r="K101" t="b">
@@ -4680,7 +4706,7 @@
       <c r="I102" t="s">
         <v>321</v>
       </c>
-      <c r="J102" s="1">
+      <c r="J102" s="2">
         <v>46387</v>
       </c>
       <c r="K102" t="b">
@@ -4715,7 +4741,7 @@
       <c r="I103" t="s">
         <v>321</v>
       </c>
-      <c r="J103" s="1">
+      <c r="J103" s="2">
         <v>46387</v>
       </c>
       <c r="K103" t="b">
@@ -4750,7 +4776,7 @@
       <c r="I104" t="s">
         <v>321</v>
       </c>
-      <c r="J104" s="1">
+      <c r="J104" s="2">
         <v>46388</v>
       </c>
       <c r="K104" t="b">
@@ -4785,7 +4811,7 @@
       <c r="I105" t="s">
         <v>322</v>
       </c>
-      <c r="J105" s="1">
+      <c r="J105" s="2">
         <v>46401</v>
       </c>
       <c r="K105" t="b">
@@ -4820,7 +4846,7 @@
       <c r="I106" t="s">
         <v>322</v>
       </c>
-      <c r="J106" s="1">
+      <c r="J106" s="2">
         <v>46401</v>
       </c>
       <c r="K106" t="b">
@@ -4855,7 +4881,7 @@
       <c r="I107" t="s">
         <v>322</v>
       </c>
-      <c r="J107" s="1">
+      <c r="J107" s="2">
         <v>46401</v>
       </c>
       <c r="K107" t="b">
@@ -4890,7 +4916,7 @@
       <c r="I108" t="s">
         <v>322</v>
       </c>
-      <c r="J108" s="1">
+      <c r="J108" s="2">
         <v>46412</v>
       </c>
       <c r="K108" t="b">
@@ -4925,7 +4951,7 @@
       <c r="I109" t="s">
         <v>322</v>
       </c>
-      <c r="J109" s="1">
+      <c r="J109" s="2">
         <v>46412</v>
       </c>
       <c r="K109" t="b">
@@ -4960,7 +4986,7 @@
       <c r="I110" t="s">
         <v>322</v>
       </c>
-      <c r="J110" s="1">
+      <c r="J110" s="2">
         <v>46412</v>
       </c>
       <c r="K110" t="b">
@@ -4995,7 +5021,7 @@
       <c r="I111" t="s">
         <v>323</v>
       </c>
-      <c r="J111" s="1">
+      <c r="J111" s="2">
         <v>46424</v>
       </c>
       <c r="K111" t="b">
@@ -5030,7 +5056,7 @@
       <c r="I112" t="s">
         <v>323</v>
       </c>
-      <c r="J112" s="1">
+      <c r="J112" s="2">
         <v>46437</v>
       </c>
       <c r="K112" t="b">
@@ -5065,7 +5091,7 @@
       <c r="I113" t="s">
         <v>323</v>
       </c>
-      <c r="J113" s="1">
+      <c r="J113" s="2">
         <v>46451</v>
       </c>
       <c r="K113" t="b">
@@ -5100,7 +5126,7 @@
       <c r="I114" t="s">
         <v>323</v>
       </c>
-      <c r="J114" s="1">
+      <c r="J114" s="2">
         <v>46451</v>
       </c>
       <c r="K114" t="b">
@@ -5135,7 +5161,7 @@
       <c r="I115" t="s">
         <v>324</v>
       </c>
-      <c r="J115" s="1">
+      <c r="J115" s="2">
         <v>46455</v>
       </c>
       <c r="K115" t="b">
@@ -5170,7 +5196,7 @@
       <c r="I116" t="s">
         <v>324</v>
       </c>
-      <c r="J116" s="1">
+      <c r="J116" s="2">
         <v>46456</v>
       </c>
       <c r="K116" t="b">
@@ -5205,7 +5231,7 @@
       <c r="I117" t="s">
         <v>324</v>
       </c>
-      <c r="J117" s="1">
+      <c r="J117" s="2">
         <v>46457</v>
       </c>
       <c r="K117" t="b">
@@ -5240,7 +5266,7 @@
       <c r="I118" t="s">
         <v>324</v>
       </c>
-      <c r="J118" s="1">
+      <c r="J118" s="2">
         <v>46464</v>
       </c>
       <c r="K118" t="b">
@@ -5275,7 +5301,7 @@
       <c r="I119" t="s">
         <v>324</v>
       </c>
-      <c r="J119" s="1">
+      <c r="J119" s="2">
         <v>46470</v>
       </c>
       <c r="K119" t="b">
@@ -5310,7 +5336,7 @@
       <c r="I120" t="s">
         <v>325</v>
       </c>
-      <c r="J120" s="1">
+      <c r="J120" s="2">
         <v>46485</v>
       </c>
       <c r="K120" t="b">
@@ -5345,7 +5371,7 @@
       <c r="I121" t="s">
         <v>325</v>
       </c>
-      <c r="J121" s="1">
+      <c r="J121" s="2">
         <v>46499</v>
       </c>
       <c r="K121" t="b">
@@ -5380,7 +5406,7 @@
       <c r="I122" t="s">
         <v>325</v>
       </c>
-      <c r="J122" s="1">
+      <c r="J122" s="2">
         <v>46504</v>
       </c>
       <c r="K122" t="b">
@@ -5415,7 +5441,7 @@
       <c r="I123" t="s">
         <v>325</v>
       </c>
-      <c r="J123" s="1">
+      <c r="J123" s="2">
         <v>46504</v>
       </c>
       <c r="K123" t="b">
@@ -5450,7 +5476,7 @@
       <c r="I124" t="s">
         <v>325</v>
       </c>
-      <c r="J124" s="1">
+      <c r="J124" s="2">
         <v>46507</v>
       </c>
       <c r="K124" t="b">
@@ -5485,7 +5511,7 @@
       <c r="I125" t="s">
         <v>325</v>
       </c>
-      <c r="J125" s="1">
+      <c r="J125" s="2">
         <v>46508</v>
       </c>
       <c r="K125" t="b">
@@ -5520,7 +5546,7 @@
       <c r="I126" t="s">
         <v>325</v>
       </c>
-      <c r="J126" s="1">
+      <c r="J126" s="2">
         <v>46512</v>
       </c>
       <c r="K126" t="b">
@@ -5555,7 +5581,7 @@
       <c r="I127" t="s">
         <v>326</v>
       </c>
-      <c r="J127" s="1">
+      <c r="J127" s="2">
         <v>46512</v>
       </c>
       <c r="K127" t="b">
@@ -5590,7 +5616,7 @@
       <c r="I128" t="s">
         <v>326</v>
       </c>
-      <c r="J128" s="1">
+      <c r="J128" s="2">
         <v>46528</v>
       </c>
       <c r="K128" t="b">
@@ -5625,7 +5651,7 @@
       <c r="I129" t="s">
         <v>326</v>
       </c>
-      <c r="J129" s="1">
+      <c r="J129" s="2">
         <v>46529</v>
       </c>
       <c r="K129" t="b">
@@ -5660,7 +5686,7 @@
       <c r="I130" t="s">
         <v>326</v>
       </c>
-      <c r="J130" s="1">
+      <c r="J130" s="2">
         <v>46537</v>
       </c>
       <c r="K130" t="b">
@@ -5695,7 +5721,7 @@
       <c r="I131" t="s">
         <v>327</v>
       </c>
-      <c r="J131" s="1">
+      <c r="J131" s="2">
         <v>46546</v>
       </c>
       <c r="K131" t="b">
@@ -5730,7 +5756,7 @@
       <c r="I132" t="s">
         <v>327</v>
       </c>
-      <c r="J132" s="1">
+      <c r="J132" s="2">
         <v>46547</v>
       </c>
       <c r="K132" t="b">
@@ -5765,7 +5791,7 @@
       <c r="I133" t="s">
         <v>327</v>
       </c>
-      <c r="J133" s="1">
+      <c r="J133" s="2">
         <v>46547</v>
       </c>
       <c r="K133" t="b">
@@ -5800,7 +5826,7 @@
       <c r="I134" t="s">
         <v>327</v>
       </c>
-      <c r="J134" s="1">
+      <c r="J134" s="2">
         <v>46547</v>
       </c>
       <c r="K134" t="b">
@@ -5835,7 +5861,7 @@
       <c r="I135" t="s">
         <v>327</v>
       </c>
-      <c r="J135" s="1">
+      <c r="J135" s="2">
         <v>46551</v>
       </c>
       <c r="K135" t="b">
@@ -5870,7 +5896,7 @@
       <c r="I136" t="s">
         <v>327</v>
       </c>
-      <c r="J136" s="1">
+      <c r="J136" s="2">
         <v>46560</v>
       </c>
       <c r="K136" t="b">
@@ -5905,7 +5931,7 @@
       <c r="I137" t="s">
         <v>327</v>
       </c>
-      <c r="J137" s="1">
+      <c r="J137" s="2">
         <v>46564</v>
       </c>
       <c r="K137" t="b">
@@ -5940,7 +5966,7 @@
       <c r="I138" t="s">
         <v>327</v>
       </c>
-      <c r="J138" s="1">
+      <c r="J138" s="2">
         <v>46567</v>
       </c>
       <c r="K138" t="b">
@@ -5975,7 +6001,7 @@
       <c r="I139" t="s">
         <v>327</v>
       </c>
-      <c r="J139" s="1">
+      <c r="J139" s="2">
         <v>46568</v>
       </c>
       <c r="K139" t="b">
@@ -6010,7 +6036,7 @@
       <c r="I140" t="s">
         <v>328</v>
       </c>
-      <c r="J140" s="1">
+      <c r="J140" s="2">
         <v>46578</v>
       </c>
       <c r="K140" t="b">
@@ -6045,7 +6071,7 @@
       <c r="I141" t="s">
         <v>328</v>
       </c>
-      <c r="J141" s="1">
+      <c r="J141" s="2">
         <v>46592</v>
       </c>
       <c r="K141" t="b">
@@ -6080,7 +6106,7 @@
       <c r="I142" t="s">
         <v>328</v>
       </c>
-      <c r="J142" s="1">
+      <c r="J142" s="2">
         <v>46592</v>
       </c>
       <c r="K142" t="b">
@@ -6115,7 +6141,7 @@
       <c r="I143" t="s">
         <v>329</v>
       </c>
-      <c r="J143" s="1">
+      <c r="J143" s="2">
         <v>46212</v>
       </c>
       <c r="K143" t="b">
@@ -6150,7 +6176,7 @@
       <c r="I144" t="s">
         <v>330</v>
       </c>
-      <c r="J144" s="1">
+      <c r="J144" s="2">
         <v>46225</v>
       </c>
       <c r="K144" t="b">
@@ -6185,7 +6211,7 @@
       <c r="I145" t="s">
         <v>331</v>
       </c>
-      <c r="J145" s="1">
+      <c r="J145" s="2">
         <v>46263</v>
       </c>
       <c r="K145" t="b">
@@ -6217,7 +6243,7 @@
       <c r="H146">
         <v>-1476</v>
       </c>
-      <c r="J146" s="1">
+      <c r="J146" s="2">
         <v>43773</v>
       </c>
       <c r="K146" t="b">
@@ -6249,7 +6275,7 @@
       <c r="H147">
         <v>-1469</v>
       </c>
-      <c r="J147" s="1">
+      <c r="J147" s="2">
         <v>43773</v>
       </c>
       <c r="K147" t="b">
@@ -6281,7 +6307,7 @@
       <c r="H148">
         <v>-1186</v>
       </c>
-      <c r="J148" s="1">
+      <c r="J148" s="2">
         <v>45295</v>
       </c>
       <c r="K148" t="b">
@@ -6313,7 +6339,7 @@
       <c r="H149">
         <v>-1048</v>
       </c>
-      <c r="J149" s="1">
+      <c r="J149" s="2">
         <v>45617</v>
       </c>
       <c r="K149" t="b">
@@ -6345,7 +6371,7 @@
       <c r="H150">
         <v>-980</v>
       </c>
-      <c r="J150" s="1">
+      <c r="J150" s="2">
         <v>45677</v>
       </c>
       <c r="K150" t="b">
@@ -6377,7 +6403,7 @@
       <c r="H151">
         <v>-961</v>
       </c>
-      <c r="J151" s="1">
+      <c r="J151" s="2">
         <v>44944</v>
       </c>
       <c r="K151" t="b">
@@ -6409,7 +6435,7 @@
       <c r="H152">
         <v>-252</v>
       </c>
-      <c r="J152" s="1">
+      <c r="J152" s="2">
         <v>46092</v>
       </c>
       <c r="K152" t="b">
@@ -6441,7 +6467,7 @@
       <c r="H153">
         <v>3</v>
       </c>
-      <c r="J153" s="1">
+      <c r="J153" s="2">
         <v>46265</v>
       </c>
       <c r="K153" t="b">
@@ -6473,7 +6499,7 @@
       <c r="H154">
         <v>3</v>
       </c>
-      <c r="J154" s="1">
+      <c r="J154" s="2">
         <v>46265</v>
       </c>
       <c r="K154" t="b">
@@ -6505,7 +6531,7 @@
       <c r="H155">
         <v>43</v>
       </c>
-      <c r="J155" s="1">
+      <c r="J155" s="2">
         <v>46440</v>
       </c>
       <c r="K155" t="b">
@@ -6537,7 +6563,7 @@
       <c r="H156">
         <v>43</v>
       </c>
-      <c r="J156" s="1">
+      <c r="J156" s="2">
         <v>46440</v>
       </c>
       <c r="K156" t="b">
@@ -6569,7 +6595,7 @@
       <c r="H157">
         <v>72</v>
       </c>
-      <c r="J157" s="1">
+      <c r="J157" s="2">
         <v>46289</v>
       </c>
       <c r="K157" t="b">
@@ -6601,7 +6627,7 @@
       <c r="H158">
         <v>72</v>
       </c>
-      <c r="J158" s="1">
+      <c r="J158" s="2">
         <v>46289</v>
       </c>
       <c r="K158" t="b">
@@ -6633,7 +6659,7 @@
       <c r="H159">
         <v>81</v>
       </c>
-      <c r="J159" s="1">
+      <c r="J159" s="2">
         <v>46405</v>
       </c>
       <c r="K159" t="b">
@@ -6665,7 +6691,7 @@
       <c r="H160">
         <v>102</v>
       </c>
-      <c r="J160" s="1">
+      <c r="J160" s="2">
         <v>46463</v>
       </c>
       <c r="K160" t="b">
@@ -6697,7 +6723,7 @@
       <c r="H161">
         <v>109</v>
       </c>
-      <c r="J161" s="1">
+      <c r="J161" s="2">
         <v>46353</v>
       </c>
       <c r="K161" t="b">
@@ -6729,7 +6755,7 @@
       <c r="H162">
         <v>127</v>
       </c>
-      <c r="J162" s="1">
+      <c r="J162" s="2">
         <v>46417</v>
       </c>
       <c r="K162" t="b">
@@ -6761,7 +6787,7 @@
       <c r="H163">
         <v>152</v>
       </c>
-      <c r="J163" s="1">
+      <c r="J163" s="2">
         <v>46271</v>
       </c>
       <c r="K163" t="b">
@@ -6793,7 +6819,7 @@
       <c r="H164">
         <v>152</v>
       </c>
-      <c r="J164" s="1">
+      <c r="J164" s="2">
         <v>46271</v>
       </c>
       <c r="K164" t="b">
@@ -6825,7 +6851,7 @@
       <c r="H165">
         <v>153</v>
       </c>
-      <c r="J165" s="1">
+      <c r="J165" s="2">
         <v>46458</v>
       </c>
       <c r="K165" t="b">
@@ -6857,7 +6883,7 @@
       <c r="H166">
         <v>158</v>
       </c>
-      <c r="J166" s="1">
+      <c r="J166" s="2">
         <v>46381</v>
       </c>
       <c r="K166" t="b">
@@ -6889,7 +6915,7 @@
       <c r="H167">
         <v>163</v>
       </c>
-      <c r="J167" s="1">
+      <c r="J167" s="2">
         <v>46592</v>
       </c>
       <c r="K167" t="b">
@@ -6921,7 +6947,7 @@
       <c r="H168">
         <v>167</v>
       </c>
-      <c r="J168" s="1">
+      <c r="J168" s="2">
         <v>46441</v>
       </c>
       <c r="K168" t="b">
@@ -6953,7 +6979,7 @@
       <c r="H169">
         <v>169</v>
       </c>
-      <c r="J169" s="1">
+      <c r="J169" s="2">
         <v>46391</v>
       </c>
       <c r="K169" t="b">
@@ -6985,7 +7011,7 @@
       <c r="H170">
         <v>184</v>
       </c>
-      <c r="J170" s="1">
+      <c r="J170" s="2">
         <v>46385</v>
       </c>
       <c r="K170" t="b">
@@ -7017,7 +7043,7 @@
       <c r="H171">
         <v>186</v>
       </c>
-      <c r="J171" s="1">
+      <c r="J171" s="2">
         <v>46387</v>
       </c>
       <c r="K171" t="b">
@@ -7049,7 +7075,7 @@
       <c r="H172">
         <v>206</v>
       </c>
-      <c r="J172" s="1">
+      <c r="J172" s="2">
         <v>46399</v>
       </c>
       <c r="K172" t="b">
@@ -7081,7 +7107,7 @@
       <c r="H173">
         <v>206</v>
       </c>
-      <c r="J173" s="1">
+      <c r="J173" s="2">
         <v>46399</v>
       </c>
       <c r="K173" t="b">
@@ -7113,7 +7139,7 @@
       <c r="H174">
         <v>234</v>
       </c>
-      <c r="J174" s="1">
+      <c r="J174" s="2">
         <v>46458</v>
       </c>
       <c r="K174" t="b">
@@ -7145,7 +7171,7 @@
       <c r="H175">
         <v>248</v>
       </c>
-      <c r="J175" s="1">
+      <c r="J175" s="2">
         <v>46528</v>
       </c>
       <c r="K175" t="b">
@@ -7177,7 +7203,7 @@
       <c r="H176">
         <v>317</v>
       </c>
-      <c r="J176" s="1">
+      <c r="J176" s="2">
         <v>46540</v>
       </c>
       <c r="K176" t="b">
@@ -7209,7 +7235,7 @@
       <c r="H177">
         <v>340</v>
       </c>
-      <c r="J177" s="1">
+      <c r="J177" s="2">
         <v>46547</v>
       </c>
       <c r="K177" t="b">
@@ -7241,7 +7267,7 @@
       <c r="H178">
         <v>364</v>
       </c>
-      <c r="J178" s="1">
+      <c r="J178" s="2">
         <v>46557</v>
       </c>
       <c r="K178" t="b">
@@ -7273,7 +7299,7 @@
       <c r="H179">
         <v>368</v>
       </c>
-      <c r="J179" s="1">
+      <c r="J179" s="2">
         <v>46571</v>
       </c>
       <c r="K179" t="b">
@@ -7305,7 +7331,7 @@
       <c r="H180">
         <v>368</v>
       </c>
-      <c r="J180" s="1">
+      <c r="J180" s="2">
         <v>46571</v>
       </c>
       <c r="K180" t="b">
@@ -7337,7 +7363,7 @@
       <c r="H181">
         <v>370</v>
       </c>
-      <c r="J181" s="1">
+      <c r="J181" s="2">
         <v>46562</v>
       </c>
       <c r="K181" t="b">
@@ -7369,7 +7395,7 @@
       <c r="H182">
         <v>385</v>
       </c>
-      <c r="J182" s="1">
+      <c r="J182" s="2">
         <v>46574</v>
       </c>
       <c r="K182" t="b">
@@ -7401,7 +7427,7 @@
       <c r="H183">
         <v>385</v>
       </c>
-      <c r="J183" s="1">
+      <c r="J183" s="2">
         <v>46574</v>
       </c>
       <c r="K183" t="b">
@@ -7433,7 +7459,7 @@
       <c r="H184">
         <v>417</v>
       </c>
-      <c r="J184" s="1">
+      <c r="J184" s="2">
         <v>46578</v>
       </c>
       <c r="K184" t="b">
@@ -7465,7 +7491,7 @@
       <c r="H185">
         <v>721</v>
       </c>
-      <c r="J185" s="1">
+      <c r="J185" s="2">
         <v>46345</v>
       </c>
       <c r="K185" t="b">
@@ -7497,7 +7523,7 @@
       <c r="H186">
         <v>721</v>
       </c>
-      <c r="J186" s="1">
+      <c r="J186" s="2">
         <v>46345</v>
       </c>
       <c r="K186" t="b">
@@ -7529,7 +7555,7 @@
       <c r="H187">
         <v>850</v>
       </c>
-      <c r="J187" s="1">
+      <c r="J187" s="2">
         <v>46366</v>
       </c>
       <c r="K187" t="b">
@@ -7561,7 +7587,7 @@
       <c r="H188">
         <v>850</v>
       </c>
-      <c r="J188" s="1">
+      <c r="J188" s="2">
         <v>46366</v>
       </c>
       <c r="K188" t="b">
@@ -7593,7 +7619,7 @@
       <c r="H189">
         <v>1661</v>
       </c>
-      <c r="J189" s="1">
+      <c r="J189" s="2">
         <v>46524</v>
       </c>
       <c r="K189" t="b">
@@ -7625,7 +7651,7 @@
       <c r="H190">
         <v>1661</v>
       </c>
-      <c r="J190" s="1">
+      <c r="J190" s="2">
         <v>46524</v>
       </c>
       <c r="K190" t="b">
@@ -7657,7 +7683,7 @@
       <c r="H191">
         <v>488</v>
       </c>
-      <c r="J191" s="1">
+      <c r="J191" s="2">
         <v>46190</v>
       </c>
       <c r="K191" t="b">
@@ -7689,7 +7715,7 @@
       <c r="H192">
         <v>25565</v>
       </c>
-      <c r="J192" s="1">
+      <c r="J192" s="2">
         <v>46190</v>
       </c>
       <c r="K192" t="b">
@@ -7721,7 +7747,7 @@
       <c r="H193">
         <v>25567</v>
       </c>
-      <c r="J193" s="1">
+      <c r="J193" s="2">
         <v>46190</v>
       </c>
       <c r="K193" t="b">
@@ -7753,7 +7779,7 @@
       <c r="H194">
         <v>31293</v>
       </c>
-      <c r="J194" s="1">
+      <c r="J194" s="2">
         <v>46190</v>
       </c>
       <c r="K194" t="b">

</xml_diff>

<commit_message>
Atualização automática: vencimentos_tmot (25/08/2026 08:36)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
@@ -1019,16 +1019,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1044,7 +1036,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1052,30 +1044,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1375,37 +1349,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1434,7 +1408,7 @@
       <c r="H2">
         <v>-4300.3</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>39285</v>
       </c>
       <c r="K2" t="b">
@@ -1466,7 +1440,7 @@
       <c r="H3">
         <v>-2354.2</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>40669</v>
       </c>
       <c r="K3" t="b">
@@ -1498,7 +1472,7 @@
       <c r="H4">
         <v>-910.7</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>40669</v>
       </c>
       <c r="K4" t="b">
@@ -1530,7 +1504,7 @@
       <c r="H5">
         <v>-868</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>44884</v>
       </c>
       <c r="K5" t="b">
@@ -1562,7 +1536,7 @@
       <c r="H6">
         <v>-483.8</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>43855</v>
       </c>
       <c r="K6" t="b">
@@ -1594,7 +1568,7 @@
       <c r="H7">
         <v>-417</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>46014</v>
       </c>
       <c r="K7" t="b">
@@ -1626,7 +1600,7 @@
       <c r="H8">
         <v>-414.2</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>46014</v>
       </c>
       <c r="K8" t="b">
@@ -1658,7 +1632,7 @@
       <c r="H9">
         <v>-391.8</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>42769</v>
       </c>
       <c r="K9" t="b">
@@ -1690,7 +1664,7 @@
       <c r="H10">
         <v>-391.6</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>45804</v>
       </c>
       <c r="K10" t="b">
@@ -1722,7 +1696,7 @@
       <c r="H11">
         <v>-391.6</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>45804</v>
       </c>
       <c r="K11" t="b">
@@ -1754,7 +1728,7 @@
       <c r="H12">
         <v>-372.9</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>42821</v>
       </c>
       <c r="K12" t="b">
@@ -1786,7 +1760,7 @@
       <c r="H13">
         <v>-372.9</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>46014</v>
       </c>
       <c r="K13" t="b">
@@ -1818,7 +1792,7 @@
       <c r="H14">
         <v>-372.9</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>46014</v>
       </c>
       <c r="K14" t="b">
@@ -1850,7 +1824,7 @@
       <c r="H15">
         <v>-372.9</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <v>46014</v>
       </c>
       <c r="K15" t="b">
@@ -1882,7 +1856,7 @@
       <c r="H16">
         <v>-367.8</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <v>46017</v>
       </c>
       <c r="K16" t="b">
@@ -1914,7 +1888,7 @@
       <c r="H17">
         <v>-367.8</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="1">
         <v>46017</v>
       </c>
       <c r="K17" t="b">
@@ -1946,7 +1920,7 @@
       <c r="H18">
         <v>-347.2</v>
       </c>
-      <c r="J18" s="2">
+      <c r="J18" s="1">
         <v>40979</v>
       </c>
       <c r="K18" t="b">
@@ -1978,7 +1952,7 @@
       <c r="H19">
         <v>-293.8</v>
       </c>
-      <c r="J19" s="2">
+      <c r="J19" s="1">
         <v>45846</v>
       </c>
       <c r="K19" t="b">
@@ -2010,7 +1984,7 @@
       <c r="H20">
         <v>-206.4</v>
       </c>
-      <c r="J20" s="2">
+      <c r="J20" s="1">
         <v>36669</v>
       </c>
       <c r="K20" t="b">
@@ -2042,7 +2016,7 @@
       <c r="H21">
         <v>-131.6</v>
       </c>
-      <c r="J21" s="2">
+      <c r="J21" s="1">
         <v>46111</v>
       </c>
       <c r="K21" t="b">
@@ -2074,7 +2048,7 @@
       <c r="H22">
         <v>-131.6</v>
       </c>
-      <c r="J22" s="2">
+      <c r="J22" s="1">
         <v>46111</v>
       </c>
       <c r="K22" t="b">
@@ -2106,7 +2080,7 @@
       <c r="H23">
         <v>-131.6</v>
       </c>
-      <c r="J23" s="2">
+      <c r="J23" s="1">
         <v>46111</v>
       </c>
       <c r="K23" t="b">
@@ -2138,7 +2112,7 @@
       <c r="H24">
         <v>-131.6</v>
       </c>
-      <c r="J24" s="2">
+      <c r="J24" s="1">
         <v>46111</v>
       </c>
       <c r="K24" t="b">
@@ -2170,7 +2144,7 @@
       <c r="H25">
         <v>-131.6</v>
       </c>
-      <c r="J25" s="2">
+      <c r="J25" s="1">
         <v>46111</v>
       </c>
       <c r="K25" t="b">
@@ -2202,7 +2176,7 @@
       <c r="H26">
         <v>-98.3</v>
       </c>
-      <c r="J26" s="2">
+      <c r="J26" s="1">
         <v>41204</v>
       </c>
       <c r="K26" t="b">
@@ -2234,7 +2208,7 @@
       <c r="H27">
         <v>-47.2</v>
       </c>
-      <c r="J27" s="2">
+      <c r="J27" s="1">
         <v>44011</v>
       </c>
       <c r="K27" t="b">
@@ -2266,7 +2240,7 @@
       <c r="H28">
         <v>-22.3</v>
       </c>
-      <c r="J28" s="2">
+      <c r="J28" s="1">
         <v>46226</v>
       </c>
       <c r="K28" t="b">
@@ -2298,7 +2272,7 @@
       <c r="H29">
         <v>4.7</v>
       </c>
-      <c r="J29" s="2">
+      <c r="J29" s="1">
         <v>46265</v>
       </c>
       <c r="K29" t="b">
@@ -2330,7 +2304,7 @@
       <c r="H30">
         <v>7.5</v>
       </c>
-      <c r="J30" s="2">
+      <c r="J30" s="1">
         <v>46265</v>
       </c>
       <c r="K30" t="b">
@@ -2362,7 +2336,7 @@
       <c r="H31">
         <v>10</v>
       </c>
-      <c r="J31" s="2">
+      <c r="J31" s="1">
         <v>46265</v>
       </c>
       <c r="K31" t="b">
@@ -2394,7 +2368,7 @@
       <c r="H32">
         <v>12.8</v>
       </c>
-      <c r="J32" s="2">
+      <c r="J32" s="1">
         <v>46265</v>
       </c>
       <c r="K32" t="b">
@@ -2426,7 +2400,7 @@
       <c r="H33">
         <v>14</v>
       </c>
-      <c r="J33" s="2">
+      <c r="J33" s="1">
         <v>46265</v>
       </c>
       <c r="K33" t="b">
@@ -2458,7 +2432,7 @@
       <c r="H34">
         <v>17.8</v>
       </c>
-      <c r="J34" s="2">
+      <c r="J34" s="1">
         <v>46265</v>
       </c>
       <c r="K34" t="b">
@@ -2490,7 +2464,7 @@
       <c r="H35">
         <v>20.4</v>
       </c>
-      <c r="J35" s="2">
+      <c r="J35" s="1">
         <v>46265</v>
       </c>
       <c r="K35" t="b">
@@ -2522,7 +2496,7 @@
       <c r="H36">
         <v>21.2</v>
       </c>
-      <c r="J36" s="2">
+      <c r="J36" s="1">
         <v>46265</v>
       </c>
       <c r="K36" t="b">
@@ -2554,7 +2528,7 @@
       <c r="H37">
         <v>26.2</v>
       </c>
-      <c r="J37" s="2">
+      <c r="J37" s="1">
         <v>46265</v>
       </c>
       <c r="K37" t="b">
@@ -2586,7 +2560,7 @@
       <c r="H38">
         <v>33.6</v>
       </c>
-      <c r="J38" s="2">
+      <c r="J38" s="1">
         <v>46364</v>
       </c>
       <c r="K38" t="b">
@@ -2618,7 +2592,7 @@
       <c r="H39">
         <v>42.2</v>
       </c>
-      <c r="J39" s="2">
+      <c r="J39" s="1">
         <v>46269</v>
       </c>
       <c r="K39" t="b">
@@ -2650,7 +2624,7 @@
       <c r="H40">
         <v>42.8</v>
       </c>
-      <c r="J40" s="2">
+      <c r="J40" s="1">
         <v>46291</v>
       </c>
       <c r="K40" t="b">
@@ -2682,7 +2656,7 @@
       <c r="H41">
         <v>45.7</v>
       </c>
-      <c r="J41" s="2">
+      <c r="J41" s="1">
         <v>46395</v>
       </c>
       <c r="K41" t="b">
@@ -2714,7 +2688,7 @@
       <c r="H42">
         <v>47.2</v>
       </c>
-      <c r="J42" s="2">
+      <c r="J42" s="1">
         <v>46280</v>
       </c>
       <c r="K42" t="b">
@@ -2746,7 +2720,7 @@
       <c r="H43">
         <v>48.7</v>
       </c>
-      <c r="J43" s="2">
+      <c r="J43" s="1">
         <v>46281</v>
       </c>
       <c r="K43" t="b">
@@ -2778,7 +2752,7 @@
       <c r="H44">
         <v>60</v>
       </c>
-      <c r="J44" s="2">
+      <c r="J44" s="1">
         <v>46281</v>
       </c>
       <c r="K44" t="b">
@@ -2810,7 +2784,7 @@
       <c r="H45">
         <v>62.6</v>
       </c>
-      <c r="J45" s="2">
+      <c r="J45" s="1">
         <v>46265</v>
       </c>
       <c r="K45" t="b">
@@ -2842,7 +2816,7 @@
       <c r="H46">
         <v>64.59999999999999</v>
       </c>
-      <c r="J46" s="2">
+      <c r="J46" s="1">
         <v>46265</v>
       </c>
       <c r="K46" t="b">
@@ -2874,7 +2848,7 @@
       <c r="H47">
         <v>67.59999999999999</v>
       </c>
-      <c r="J47" s="2">
+      <c r="J47" s="1">
         <v>46267</v>
       </c>
       <c r="K47" t="b">
@@ -2906,7 +2880,7 @@
       <c r="H48">
         <v>68.3</v>
       </c>
-      <c r="J48" s="2">
+      <c r="J48" s="1">
         <v>46278</v>
       </c>
       <c r="K48" t="b">
@@ -2938,7 +2912,7 @@
       <c r="H49">
         <v>69.2</v>
       </c>
-      <c r="J49" s="2">
+      <c r="J49" s="1">
         <v>46453</v>
       </c>
       <c r="K49" t="b">
@@ -2970,7 +2944,7 @@
       <c r="H50">
         <v>69.8</v>
       </c>
-      <c r="J50" s="2">
+      <c r="J50" s="1">
         <v>46265</v>
       </c>
       <c r="K50" t="b">
@@ -3002,7 +2976,7 @@
       <c r="H51">
         <v>69.8</v>
       </c>
-      <c r="J51" s="2">
+      <c r="J51" s="1">
         <v>46265</v>
       </c>
       <c r="K51" t="b">
@@ -3034,7 +3008,7 @@
       <c r="H52">
         <v>72.2</v>
       </c>
-      <c r="J52" s="2">
+      <c r="J52" s="1">
         <v>46275</v>
       </c>
       <c r="K52" t="b">
@@ -3066,7 +3040,7 @@
       <c r="H53">
         <v>72.2</v>
       </c>
-      <c r="J53" s="2">
+      <c r="J53" s="1">
         <v>46275</v>
       </c>
       <c r="K53" t="b">
@@ -3098,7 +3072,7 @@
       <c r="H54">
         <v>78.09999999999999</v>
       </c>
-      <c r="J54" s="2">
+      <c r="J54" s="1">
         <v>46265</v>
       </c>
       <c r="K54" t="b">
@@ -3130,7 +3104,7 @@
       <c r="H55">
         <v>82.8</v>
       </c>
-      <c r="J55" s="2">
+      <c r="J55" s="1">
         <v>46487</v>
       </c>
       <c r="K55" t="b">
@@ -3162,7 +3136,7 @@
       <c r="H56">
         <v>83.09999999999999</v>
       </c>
-      <c r="J56" s="2">
+      <c r="J56" s="1">
         <v>46285</v>
       </c>
       <c r="K56" t="b">
@@ -3194,7 +3168,7 @@
       <c r="H57">
         <v>84.8</v>
       </c>
-      <c r="J57" s="2">
+      <c r="J57" s="1">
         <v>46492</v>
       </c>
       <c r="K57" t="b">
@@ -3226,7 +3200,7 @@
       <c r="H58">
         <v>104.9</v>
       </c>
-      <c r="J58" s="2">
+      <c r="J58" s="1">
         <v>46297</v>
       </c>
       <c r="K58" t="b">
@@ -3258,7 +3232,7 @@
       <c r="H59">
         <v>107.6</v>
       </c>
-      <c r="J59" s="2">
+      <c r="J59" s="1">
         <v>46283</v>
       </c>
       <c r="K59" t="b">
@@ -3290,7 +3264,7 @@
       <c r="H60">
         <v>111.9</v>
       </c>
-      <c r="J60" s="2">
+      <c r="J60" s="1">
         <v>46300</v>
       </c>
       <c r="K60" t="b">
@@ -3322,7 +3296,7 @@
       <c r="H61">
         <v>111.9</v>
       </c>
-      <c r="J61" s="2">
+      <c r="J61" s="1">
         <v>46300</v>
       </c>
       <c r="K61" t="b">
@@ -3354,7 +3328,7 @@
       <c r="H62">
         <v>111.9</v>
       </c>
-      <c r="J62" s="2">
+      <c r="J62" s="1">
         <v>46300</v>
       </c>
       <c r="K62" t="b">
@@ -3386,7 +3360,7 @@
       <c r="H63">
         <v>111.9</v>
       </c>
-      <c r="J63" s="2">
+      <c r="J63" s="1">
         <v>46300</v>
       </c>
       <c r="K63" t="b">
@@ -3418,7 +3392,7 @@
       <c r="H64">
         <v>111.9</v>
       </c>
-      <c r="J64" s="2">
+      <c r="J64" s="1">
         <v>46300</v>
       </c>
       <c r="K64" t="b">
@@ -3450,7 +3424,7 @@
       <c r="H65">
         <v>128.8</v>
       </c>
-      <c r="J65" s="2">
+      <c r="J65" s="1">
         <v>46308</v>
       </c>
       <c r="K65" t="b">
@@ -3482,7 +3456,7 @@
       <c r="H66">
         <v>131.1</v>
       </c>
-      <c r="J66" s="2">
+      <c r="J66" s="1">
         <v>46336</v>
       </c>
       <c r="K66" t="b">
@@ -3514,7 +3488,7 @@
       <c r="H67">
         <v>138.4</v>
       </c>
-      <c r="J67" s="2">
+      <c r="J67" s="1">
         <v>46343</v>
       </c>
       <c r="K67" t="b">
@@ -3546,7 +3520,7 @@
       <c r="H68">
         <v>141</v>
       </c>
-      <c r="J68" s="2">
+      <c r="J68" s="1">
         <v>46350</v>
       </c>
       <c r="K68" t="b">
@@ -3578,7 +3552,7 @@
       <c r="H69">
         <v>162</v>
       </c>
-      <c r="J69" s="2">
+      <c r="J69" s="1">
         <v>46391</v>
       </c>
       <c r="K69" t="b">
@@ -3610,7 +3584,7 @@
       <c r="H70">
         <v>167.2</v>
       </c>
-      <c r="J70" s="2">
+      <c r="J70" s="1">
         <v>46330</v>
       </c>
       <c r="K70" t="b">
@@ -3642,7 +3616,7 @@
       <c r="H71">
         <v>177.4</v>
       </c>
-      <c r="J71" s="2">
+      <c r="J71" s="1">
         <v>46418</v>
       </c>
       <c r="K71" t="b">
@@ -3674,7 +3648,7 @@
       <c r="H72">
         <v>200</v>
       </c>
-      <c r="J72" s="2">
+      <c r="J72" s="1">
         <v>46356</v>
       </c>
       <c r="K72" t="b">
@@ -3706,7 +3680,7 @@
       <c r="H73">
         <v>203.6</v>
       </c>
-      <c r="J73" s="2">
+      <c r="J73" s="1">
         <v>46436</v>
       </c>
       <c r="K73" t="b">
@@ -3738,7 +3712,7 @@
       <c r="H74">
         <v>221.2</v>
       </c>
-      <c r="J74" s="2">
+      <c r="J74" s="1">
         <v>46426</v>
       </c>
       <c r="K74" t="b">
@@ -3770,7 +3744,7 @@
       <c r="H75">
         <v>240.8</v>
       </c>
-      <c r="J75" s="2">
+      <c r="J75" s="1">
         <v>46450</v>
       </c>
       <c r="K75" t="b">
@@ -3802,7 +3776,7 @@
       <c r="H76">
         <v>245.8</v>
       </c>
-      <c r="J76" s="2">
+      <c r="J76" s="1">
         <v>46452</v>
       </c>
       <c r="K76" t="b">
@@ -3834,7 +3808,7 @@
       <c r="H77">
         <v>263.4</v>
       </c>
-      <c r="J77" s="2">
+      <c r="J77" s="1">
         <v>46322</v>
       </c>
       <c r="K77" t="b">
@@ -3866,7 +3840,7 @@
       <c r="H78">
         <v>275.2</v>
       </c>
-      <c r="J78" s="2">
+      <c r="J78" s="1">
         <v>46433</v>
       </c>
       <c r="K78" t="b">
@@ -3901,7 +3875,7 @@
       <c r="I79" t="s">
         <v>311</v>
       </c>
-      <c r="J79" s="2">
+      <c r="J79" s="1">
         <v>36557</v>
       </c>
       <c r="K79" t="b">
@@ -3936,7 +3910,7 @@
       <c r="I80" t="s">
         <v>312</v>
       </c>
-      <c r="J80" s="2">
+      <c r="J80" s="1">
         <v>41275</v>
       </c>
       <c r="K80" t="b">
@@ -3971,7 +3945,7 @@
       <c r="I81" t="s">
         <v>313</v>
       </c>
-      <c r="J81" s="2">
+      <c r="J81" s="1">
         <v>45380</v>
       </c>
       <c r="K81" t="b">
@@ -4006,7 +3980,7 @@
       <c r="I82" t="s">
         <v>314</v>
       </c>
-      <c r="J82" s="2">
+      <c r="J82" s="1">
         <v>45421</v>
       </c>
       <c r="K82" t="b">
@@ -4041,7 +4015,7 @@
       <c r="I83" t="s">
         <v>314</v>
       </c>
-      <c r="J83" s="2">
+      <c r="J83" s="1">
         <v>45428</v>
       </c>
       <c r="K83" t="b">
@@ -4076,7 +4050,7 @@
       <c r="I84" t="s">
         <v>315</v>
       </c>
-      <c r="J84" s="2">
+      <c r="J84" s="1">
         <v>45490</v>
       </c>
       <c r="K84" t="b">
@@ -4111,7 +4085,7 @@
       <c r="I85" t="s">
         <v>316</v>
       </c>
-      <c r="J85" s="2">
+      <c r="J85" s="1">
         <v>45566</v>
       </c>
       <c r="K85" t="b">
@@ -4146,7 +4120,7 @@
       <c r="I86" t="s">
         <v>317</v>
       </c>
-      <c r="J86" s="2">
+      <c r="J86" s="1">
         <v>45986</v>
       </c>
       <c r="K86" t="b">
@@ -4181,7 +4155,7 @@
       <c r="I87" t="s">
         <v>318</v>
       </c>
-      <c r="J87" s="2">
+      <c r="J87" s="1">
         <v>46284</v>
       </c>
       <c r="K87" t="b">
@@ -4216,7 +4190,7 @@
       <c r="I88" t="s">
         <v>319</v>
       </c>
-      <c r="J88" s="2">
+      <c r="J88" s="1">
         <v>46305</v>
       </c>
       <c r="K88" t="b">
@@ -4251,7 +4225,7 @@
       <c r="I89" t="s">
         <v>319</v>
       </c>
-      <c r="J89" s="2">
+      <c r="J89" s="1">
         <v>46310</v>
       </c>
       <c r="K89" t="b">
@@ -4286,7 +4260,7 @@
       <c r="I90" t="s">
         <v>319</v>
       </c>
-      <c r="J90" s="2">
+      <c r="J90" s="1">
         <v>46317</v>
       </c>
       <c r="K90" t="b">
@@ -4321,7 +4295,7 @@
       <c r="I91" t="s">
         <v>319</v>
       </c>
-      <c r="J91" s="2">
+      <c r="J91" s="1">
         <v>46319</v>
       </c>
       <c r="K91" t="b">
@@ -4356,7 +4330,7 @@
       <c r="I92" t="s">
         <v>320</v>
       </c>
-      <c r="J92" s="2">
+      <c r="J92" s="1">
         <v>46333</v>
       </c>
       <c r="K92" t="b">
@@ -4391,7 +4365,7 @@
       <c r="I93" t="s">
         <v>320</v>
       </c>
-      <c r="J93" s="2">
+      <c r="J93" s="1">
         <v>46338</v>
       </c>
       <c r="K93" t="b">
@@ -4426,7 +4400,7 @@
       <c r="I94" t="s">
         <v>320</v>
       </c>
-      <c r="J94" s="2">
+      <c r="J94" s="1">
         <v>46338</v>
       </c>
       <c r="K94" t="b">
@@ -4461,7 +4435,7 @@
       <c r="I95" t="s">
         <v>320</v>
       </c>
-      <c r="J95" s="2">
+      <c r="J95" s="1">
         <v>46341</v>
       </c>
       <c r="K95" t="b">
@@ -4496,7 +4470,7 @@
       <c r="I96" t="s">
         <v>320</v>
       </c>
-      <c r="J96" s="2">
+      <c r="J96" s="1">
         <v>46344</v>
       </c>
       <c r="K96" t="b">
@@ -4531,7 +4505,7 @@
       <c r="I97" t="s">
         <v>321</v>
       </c>
-      <c r="J97" s="2">
+      <c r="J97" s="1">
         <v>46360</v>
       </c>
       <c r="K97" t="b">
@@ -4566,7 +4540,7 @@
       <c r="I98" t="s">
         <v>321</v>
       </c>
-      <c r="J98" s="2">
+      <c r="J98" s="1">
         <v>46360</v>
       </c>
       <c r="K98" t="b">
@@ -4601,7 +4575,7 @@
       <c r="I99" t="s">
         <v>321</v>
       </c>
-      <c r="J99" s="2">
+      <c r="J99" s="1">
         <v>46367</v>
       </c>
       <c r="K99" t="b">
@@ -4636,7 +4610,7 @@
       <c r="I100" t="s">
         <v>321</v>
       </c>
-      <c r="J100" s="2">
+      <c r="J100" s="1">
         <v>46375</v>
       </c>
       <c r="K100" t="b">
@@ -4671,7 +4645,7 @@
       <c r="I101" t="s">
         <v>321</v>
       </c>
-      <c r="J101" s="2">
+      <c r="J101" s="1">
         <v>46387</v>
       </c>
       <c r="K101" t="b">
@@ -4706,7 +4680,7 @@
       <c r="I102" t="s">
         <v>321</v>
       </c>
-      <c r="J102" s="2">
+      <c r="J102" s="1">
         <v>46387</v>
       </c>
       <c r="K102" t="b">
@@ -4741,7 +4715,7 @@
       <c r="I103" t="s">
         <v>321</v>
       </c>
-      <c r="J103" s="2">
+      <c r="J103" s="1">
         <v>46387</v>
       </c>
       <c r="K103" t="b">
@@ -4776,7 +4750,7 @@
       <c r="I104" t="s">
         <v>321</v>
       </c>
-      <c r="J104" s="2">
+      <c r="J104" s="1">
         <v>46388</v>
       </c>
       <c r="K104" t="b">
@@ -4811,7 +4785,7 @@
       <c r="I105" t="s">
         <v>322</v>
       </c>
-      <c r="J105" s="2">
+      <c r="J105" s="1">
         <v>46401</v>
       </c>
       <c r="K105" t="b">
@@ -4846,7 +4820,7 @@
       <c r="I106" t="s">
         <v>322</v>
       </c>
-      <c r="J106" s="2">
+      <c r="J106" s="1">
         <v>46401</v>
       </c>
       <c r="K106" t="b">
@@ -4881,7 +4855,7 @@
       <c r="I107" t="s">
         <v>322</v>
       </c>
-      <c r="J107" s="2">
+      <c r="J107" s="1">
         <v>46401</v>
       </c>
       <c r="K107" t="b">
@@ -4916,7 +4890,7 @@
       <c r="I108" t="s">
         <v>322</v>
       </c>
-      <c r="J108" s="2">
+      <c r="J108" s="1">
         <v>46412</v>
       </c>
       <c r="K108" t="b">
@@ -4951,7 +4925,7 @@
       <c r="I109" t="s">
         <v>322</v>
       </c>
-      <c r="J109" s="2">
+      <c r="J109" s="1">
         <v>46412</v>
       </c>
       <c r="K109" t="b">
@@ -4986,7 +4960,7 @@
       <c r="I110" t="s">
         <v>322</v>
       </c>
-      <c r="J110" s="2">
+      <c r="J110" s="1">
         <v>46412</v>
       </c>
       <c r="K110" t="b">
@@ -5021,7 +4995,7 @@
       <c r="I111" t="s">
         <v>323</v>
       </c>
-      <c r="J111" s="2">
+      <c r="J111" s="1">
         <v>46424</v>
       </c>
       <c r="K111" t="b">
@@ -5056,7 +5030,7 @@
       <c r="I112" t="s">
         <v>323</v>
       </c>
-      <c r="J112" s="2">
+      <c r="J112" s="1">
         <v>46437</v>
       </c>
       <c r="K112" t="b">
@@ -5091,7 +5065,7 @@
       <c r="I113" t="s">
         <v>323</v>
       </c>
-      <c r="J113" s="2">
+      <c r="J113" s="1">
         <v>46451</v>
       </c>
       <c r="K113" t="b">
@@ -5126,7 +5100,7 @@
       <c r="I114" t="s">
         <v>323</v>
       </c>
-      <c r="J114" s="2">
+      <c r="J114" s="1">
         <v>46451</v>
       </c>
       <c r="K114" t="b">
@@ -5161,7 +5135,7 @@
       <c r="I115" t="s">
         <v>324</v>
       </c>
-      <c r="J115" s="2">
+      <c r="J115" s="1">
         <v>46455</v>
       </c>
       <c r="K115" t="b">
@@ -5196,7 +5170,7 @@
       <c r="I116" t="s">
         <v>324</v>
       </c>
-      <c r="J116" s="2">
+      <c r="J116" s="1">
         <v>46456</v>
       </c>
       <c r="K116" t="b">
@@ -5231,7 +5205,7 @@
       <c r="I117" t="s">
         <v>324</v>
       </c>
-      <c r="J117" s="2">
+      <c r="J117" s="1">
         <v>46457</v>
       </c>
       <c r="K117" t="b">
@@ -5266,7 +5240,7 @@
       <c r="I118" t="s">
         <v>324</v>
       </c>
-      <c r="J118" s="2">
+      <c r="J118" s="1">
         <v>46464</v>
       </c>
       <c r="K118" t="b">
@@ -5301,7 +5275,7 @@
       <c r="I119" t="s">
         <v>324</v>
       </c>
-      <c r="J119" s="2">
+      <c r="J119" s="1">
         <v>46470</v>
       </c>
       <c r="K119" t="b">
@@ -5336,7 +5310,7 @@
       <c r="I120" t="s">
         <v>325</v>
       </c>
-      <c r="J120" s="2">
+      <c r="J120" s="1">
         <v>46485</v>
       </c>
       <c r="K120" t="b">
@@ -5371,7 +5345,7 @@
       <c r="I121" t="s">
         <v>325</v>
       </c>
-      <c r="J121" s="2">
+      <c r="J121" s="1">
         <v>46499</v>
       </c>
       <c r="K121" t="b">
@@ -5406,7 +5380,7 @@
       <c r="I122" t="s">
         <v>325</v>
       </c>
-      <c r="J122" s="2">
+      <c r="J122" s="1">
         <v>46504</v>
       </c>
       <c r="K122" t="b">
@@ -5441,7 +5415,7 @@
       <c r="I123" t="s">
         <v>325</v>
       </c>
-      <c r="J123" s="2">
+      <c r="J123" s="1">
         <v>46504</v>
       </c>
       <c r="K123" t="b">
@@ -5476,7 +5450,7 @@
       <c r="I124" t="s">
         <v>325</v>
       </c>
-      <c r="J124" s="2">
+      <c r="J124" s="1">
         <v>46507</v>
       </c>
       <c r="K124" t="b">
@@ -5511,7 +5485,7 @@
       <c r="I125" t="s">
         <v>325</v>
       </c>
-      <c r="J125" s="2">
+      <c r="J125" s="1">
         <v>46508</v>
       </c>
       <c r="K125" t="b">
@@ -5546,7 +5520,7 @@
       <c r="I126" t="s">
         <v>325</v>
       </c>
-      <c r="J126" s="2">
+      <c r="J126" s="1">
         <v>46512</v>
       </c>
       <c r="K126" t="b">
@@ -5581,7 +5555,7 @@
       <c r="I127" t="s">
         <v>326</v>
       </c>
-      <c r="J127" s="2">
+      <c r="J127" s="1">
         <v>46512</v>
       </c>
       <c r="K127" t="b">
@@ -5616,7 +5590,7 @@
       <c r="I128" t="s">
         <v>326</v>
       </c>
-      <c r="J128" s="2">
+      <c r="J128" s="1">
         <v>46528</v>
       </c>
       <c r="K128" t="b">
@@ -5651,7 +5625,7 @@
       <c r="I129" t="s">
         <v>326</v>
       </c>
-      <c r="J129" s="2">
+      <c r="J129" s="1">
         <v>46529</v>
       </c>
       <c r="K129" t="b">
@@ -5686,7 +5660,7 @@
       <c r="I130" t="s">
         <v>326</v>
       </c>
-      <c r="J130" s="2">
+      <c r="J130" s="1">
         <v>46537</v>
       </c>
       <c r="K130" t="b">
@@ -5721,7 +5695,7 @@
       <c r="I131" t="s">
         <v>327</v>
       </c>
-      <c r="J131" s="2">
+      <c r="J131" s="1">
         <v>46546</v>
       </c>
       <c r="K131" t="b">
@@ -5756,7 +5730,7 @@
       <c r="I132" t="s">
         <v>327</v>
       </c>
-      <c r="J132" s="2">
+      <c r="J132" s="1">
         <v>46547</v>
       </c>
       <c r="K132" t="b">
@@ -5791,7 +5765,7 @@
       <c r="I133" t="s">
         <v>327</v>
       </c>
-      <c r="J133" s="2">
+      <c r="J133" s="1">
         <v>46547</v>
       </c>
       <c r="K133" t="b">
@@ -5826,7 +5800,7 @@
       <c r="I134" t="s">
         <v>327</v>
       </c>
-      <c r="J134" s="2">
+      <c r="J134" s="1">
         <v>46547</v>
       </c>
       <c r="K134" t="b">
@@ -5861,7 +5835,7 @@
       <c r="I135" t="s">
         <v>327</v>
       </c>
-      <c r="J135" s="2">
+      <c r="J135" s="1">
         <v>46551</v>
       </c>
       <c r="K135" t="b">
@@ -5896,7 +5870,7 @@
       <c r="I136" t="s">
         <v>327</v>
       </c>
-      <c r="J136" s="2">
+      <c r="J136" s="1">
         <v>46560</v>
       </c>
       <c r="K136" t="b">
@@ -5931,7 +5905,7 @@
       <c r="I137" t="s">
         <v>327</v>
       </c>
-      <c r="J137" s="2">
+      <c r="J137" s="1">
         <v>46564</v>
       </c>
       <c r="K137" t="b">
@@ -5966,7 +5940,7 @@
       <c r="I138" t="s">
         <v>327</v>
       </c>
-      <c r="J138" s="2">
+      <c r="J138" s="1">
         <v>46567</v>
       </c>
       <c r="K138" t="b">
@@ -6001,7 +5975,7 @@
       <c r="I139" t="s">
         <v>327</v>
       </c>
-      <c r="J139" s="2">
+      <c r="J139" s="1">
         <v>46568</v>
       </c>
       <c r="K139" t="b">
@@ -6036,7 +6010,7 @@
       <c r="I140" t="s">
         <v>328</v>
       </c>
-      <c r="J140" s="2">
+      <c r="J140" s="1">
         <v>46578</v>
       </c>
       <c r="K140" t="b">
@@ -6071,7 +6045,7 @@
       <c r="I141" t="s">
         <v>328</v>
       </c>
-      <c r="J141" s="2">
+      <c r="J141" s="1">
         <v>46592</v>
       </c>
       <c r="K141" t="b">
@@ -6106,7 +6080,7 @@
       <c r="I142" t="s">
         <v>328</v>
       </c>
-      <c r="J142" s="2">
+      <c r="J142" s="1">
         <v>46592</v>
       </c>
       <c r="K142" t="b">
@@ -6141,7 +6115,7 @@
       <c r="I143" t="s">
         <v>329</v>
       </c>
-      <c r="J143" s="2">
+      <c r="J143" s="1">
         <v>46212</v>
       </c>
       <c r="K143" t="b">
@@ -6176,7 +6150,7 @@
       <c r="I144" t="s">
         <v>330</v>
       </c>
-      <c r="J144" s="2">
+      <c r="J144" s="1">
         <v>46225</v>
       </c>
       <c r="K144" t="b">
@@ -6211,7 +6185,7 @@
       <c r="I145" t="s">
         <v>331</v>
       </c>
-      <c r="J145" s="2">
+      <c r="J145" s="1">
         <v>46263</v>
       </c>
       <c r="K145" t="b">
@@ -6243,7 +6217,7 @@
       <c r="H146">
         <v>-1476</v>
       </c>
-      <c r="J146" s="2">
+      <c r="J146" s="1">
         <v>43773</v>
       </c>
       <c r="K146" t="b">
@@ -6275,7 +6249,7 @@
       <c r="H147">
         <v>-1469</v>
       </c>
-      <c r="J147" s="2">
+      <c r="J147" s="1">
         <v>43773</v>
       </c>
       <c r="K147" t="b">
@@ -6307,7 +6281,7 @@
       <c r="H148">
         <v>-1186</v>
       </c>
-      <c r="J148" s="2">
+      <c r="J148" s="1">
         <v>45295</v>
       </c>
       <c r="K148" t="b">
@@ -6339,7 +6313,7 @@
       <c r="H149">
         <v>-1048</v>
       </c>
-      <c r="J149" s="2">
+      <c r="J149" s="1">
         <v>45617</v>
       </c>
       <c r="K149" t="b">
@@ -6371,7 +6345,7 @@
       <c r="H150">
         <v>-980</v>
       </c>
-      <c r="J150" s="2">
+      <c r="J150" s="1">
         <v>45677</v>
       </c>
       <c r="K150" t="b">
@@ -6403,7 +6377,7 @@
       <c r="H151">
         <v>-961</v>
       </c>
-      <c r="J151" s="2">
+      <c r="J151" s="1">
         <v>44944</v>
       </c>
       <c r="K151" t="b">
@@ -6435,7 +6409,7 @@
       <c r="H152">
         <v>-252</v>
       </c>
-      <c r="J152" s="2">
+      <c r="J152" s="1">
         <v>46092</v>
       </c>
       <c r="K152" t="b">
@@ -6467,7 +6441,7 @@
       <c r="H153">
         <v>3</v>
       </c>
-      <c r="J153" s="2">
+      <c r="J153" s="1">
         <v>46265</v>
       </c>
       <c r="K153" t="b">
@@ -6499,7 +6473,7 @@
       <c r="H154">
         <v>3</v>
       </c>
-      <c r="J154" s="2">
+      <c r="J154" s="1">
         <v>46265</v>
       </c>
       <c r="K154" t="b">
@@ -6531,7 +6505,7 @@
       <c r="H155">
         <v>43</v>
       </c>
-      <c r="J155" s="2">
+      <c r="J155" s="1">
         <v>46440</v>
       </c>
       <c r="K155" t="b">
@@ -6563,7 +6537,7 @@
       <c r="H156">
         <v>43</v>
       </c>
-      <c r="J156" s="2">
+      <c r="J156" s="1">
         <v>46440</v>
       </c>
       <c r="K156" t="b">
@@ -6595,7 +6569,7 @@
       <c r="H157">
         <v>72</v>
       </c>
-      <c r="J157" s="2">
+      <c r="J157" s="1">
         <v>46289</v>
       </c>
       <c r="K157" t="b">
@@ -6627,7 +6601,7 @@
       <c r="H158">
         <v>72</v>
       </c>
-      <c r="J158" s="2">
+      <c r="J158" s="1">
         <v>46289</v>
       </c>
       <c r="K158" t="b">
@@ -6659,7 +6633,7 @@
       <c r="H159">
         <v>81</v>
       </c>
-      <c r="J159" s="2">
+      <c r="J159" s="1">
         <v>46405</v>
       </c>
       <c r="K159" t="b">
@@ -6691,7 +6665,7 @@
       <c r="H160">
         <v>102</v>
       </c>
-      <c r="J160" s="2">
+      <c r="J160" s="1">
         <v>46463</v>
       </c>
       <c r="K160" t="b">
@@ -6723,7 +6697,7 @@
       <c r="H161">
         <v>109</v>
       </c>
-      <c r="J161" s="2">
+      <c r="J161" s="1">
         <v>46353</v>
       </c>
       <c r="K161" t="b">
@@ -6755,7 +6729,7 @@
       <c r="H162">
         <v>127</v>
       </c>
-      <c r="J162" s="2">
+      <c r="J162" s="1">
         <v>46417</v>
       </c>
       <c r="K162" t="b">
@@ -6787,7 +6761,7 @@
       <c r="H163">
         <v>152</v>
       </c>
-      <c r="J163" s="2">
+      <c r="J163" s="1">
         <v>46271</v>
       </c>
       <c r="K163" t="b">
@@ -6819,7 +6793,7 @@
       <c r="H164">
         <v>152</v>
       </c>
-      <c r="J164" s="2">
+      <c r="J164" s="1">
         <v>46271</v>
       </c>
       <c r="K164" t="b">
@@ -6851,7 +6825,7 @@
       <c r="H165">
         <v>153</v>
       </c>
-      <c r="J165" s="2">
+      <c r="J165" s="1">
         <v>46458</v>
       </c>
       <c r="K165" t="b">
@@ -6883,7 +6857,7 @@
       <c r="H166">
         <v>158</v>
       </c>
-      <c r="J166" s="2">
+      <c r="J166" s="1">
         <v>46381</v>
       </c>
       <c r="K166" t="b">
@@ -6915,7 +6889,7 @@
       <c r="H167">
         <v>163</v>
       </c>
-      <c r="J167" s="2">
+      <c r="J167" s="1">
         <v>46592</v>
       </c>
       <c r="K167" t="b">
@@ -6947,7 +6921,7 @@
       <c r="H168">
         <v>167</v>
       </c>
-      <c r="J168" s="2">
+      <c r="J168" s="1">
         <v>46441</v>
       </c>
       <c r="K168" t="b">
@@ -6979,7 +6953,7 @@
       <c r="H169">
         <v>169</v>
       </c>
-      <c r="J169" s="2">
+      <c r="J169" s="1">
         <v>46391</v>
       </c>
       <c r="K169" t="b">
@@ -7011,7 +6985,7 @@
       <c r="H170">
         <v>184</v>
       </c>
-      <c r="J170" s="2">
+      <c r="J170" s="1">
         <v>46385</v>
       </c>
       <c r="K170" t="b">
@@ -7043,7 +7017,7 @@
       <c r="H171">
         <v>186</v>
       </c>
-      <c r="J171" s="2">
+      <c r="J171" s="1">
         <v>46387</v>
       </c>
       <c r="K171" t="b">
@@ -7075,7 +7049,7 @@
       <c r="H172">
         <v>206</v>
       </c>
-      <c r="J172" s="2">
+      <c r="J172" s="1">
         <v>46399</v>
       </c>
       <c r="K172" t="b">
@@ -7107,7 +7081,7 @@
       <c r="H173">
         <v>206</v>
       </c>
-      <c r="J173" s="2">
+      <c r="J173" s="1">
         <v>46399</v>
       </c>
       <c r="K173" t="b">
@@ -7139,7 +7113,7 @@
       <c r="H174">
         <v>234</v>
       </c>
-      <c r="J174" s="2">
+      <c r="J174" s="1">
         <v>46458</v>
       </c>
       <c r="K174" t="b">
@@ -7171,7 +7145,7 @@
       <c r="H175">
         <v>248</v>
       </c>
-      <c r="J175" s="2">
+      <c r="J175" s="1">
         <v>46528</v>
       </c>
       <c r="K175" t="b">
@@ -7203,7 +7177,7 @@
       <c r="H176">
         <v>317</v>
       </c>
-      <c r="J176" s="2">
+      <c r="J176" s="1">
         <v>46540</v>
       </c>
       <c r="K176" t="b">
@@ -7235,7 +7209,7 @@
       <c r="H177">
         <v>340</v>
       </c>
-      <c r="J177" s="2">
+      <c r="J177" s="1">
         <v>46547</v>
       </c>
       <c r="K177" t="b">
@@ -7267,7 +7241,7 @@
       <c r="H178">
         <v>364</v>
       </c>
-      <c r="J178" s="2">
+      <c r="J178" s="1">
         <v>46557</v>
       </c>
       <c r="K178" t="b">
@@ -7299,7 +7273,7 @@
       <c r="H179">
         <v>368</v>
       </c>
-      <c r="J179" s="2">
+      <c r="J179" s="1">
         <v>46571</v>
       </c>
       <c r="K179" t="b">
@@ -7331,7 +7305,7 @@
       <c r="H180">
         <v>368</v>
       </c>
-      <c r="J180" s="2">
+      <c r="J180" s="1">
         <v>46571</v>
       </c>
       <c r="K180" t="b">
@@ -7363,7 +7337,7 @@
       <c r="H181">
         <v>370</v>
       </c>
-      <c r="J181" s="2">
+      <c r="J181" s="1">
         <v>46562</v>
       </c>
       <c r="K181" t="b">
@@ -7395,7 +7369,7 @@
       <c r="H182">
         <v>385</v>
       </c>
-      <c r="J182" s="2">
+      <c r="J182" s="1">
         <v>46574</v>
       </c>
       <c r="K182" t="b">
@@ -7427,7 +7401,7 @@
       <c r="H183">
         <v>385</v>
       </c>
-      <c r="J183" s="2">
+      <c r="J183" s="1">
         <v>46574</v>
       </c>
       <c r="K183" t="b">
@@ -7459,7 +7433,7 @@
       <c r="H184">
         <v>417</v>
       </c>
-      <c r="J184" s="2">
+      <c r="J184" s="1">
         <v>46578</v>
       </c>
       <c r="K184" t="b">
@@ -7491,7 +7465,7 @@
       <c r="H185">
         <v>721</v>
       </c>
-      <c r="J185" s="2">
+      <c r="J185" s="1">
         <v>46345</v>
       </c>
       <c r="K185" t="b">
@@ -7523,7 +7497,7 @@
       <c r="H186">
         <v>721</v>
       </c>
-      <c r="J186" s="2">
+      <c r="J186" s="1">
         <v>46345</v>
       </c>
       <c r="K186" t="b">
@@ -7555,7 +7529,7 @@
       <c r="H187">
         <v>850</v>
       </c>
-      <c r="J187" s="2">
+      <c r="J187" s="1">
         <v>46366</v>
       </c>
       <c r="K187" t="b">
@@ -7587,7 +7561,7 @@
       <c r="H188">
         <v>850</v>
       </c>
-      <c r="J188" s="2">
+      <c r="J188" s="1">
         <v>46366</v>
       </c>
       <c r="K188" t="b">
@@ -7619,7 +7593,7 @@
       <c r="H189">
         <v>1661</v>
       </c>
-      <c r="J189" s="2">
+      <c r="J189" s="1">
         <v>46524</v>
       </c>
       <c r="K189" t="b">
@@ -7651,7 +7625,7 @@
       <c r="H190">
         <v>1661</v>
       </c>
-      <c r="J190" s="2">
+      <c r="J190" s="1">
         <v>46524</v>
       </c>
       <c r="K190" t="b">
@@ -7683,7 +7657,7 @@
       <c r="H191">
         <v>488</v>
       </c>
-      <c r="J191" s="2">
+      <c r="J191" s="1">
         <v>46190</v>
       </c>
       <c r="K191" t="b">
@@ -7715,7 +7689,7 @@
       <c r="H192">
         <v>25565</v>
       </c>
-      <c r="J192" s="2">
+      <c r="J192" s="1">
         <v>46190</v>
       </c>
       <c r="K192" t="b">
@@ -7747,7 +7721,7 @@
       <c r="H193">
         <v>25567</v>
       </c>
-      <c r="J193" s="2">
+      <c r="J193" s="1">
         <v>46190</v>
       </c>
       <c r="K193" t="b">
@@ -7779,7 +7753,7 @@
       <c r="H194">
         <v>31293</v>
       </c>
-      <c r="J194" s="2">
+      <c r="J194" s="1">
         <v>46190</v>
       </c>
       <c r="K194" t="b">

</xml_diff>

<commit_message>
Atualização automática: vencimentos_tmot (01/09/2026 11:15)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
@@ -1019,8 +1019,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1036,7 +1044,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1044,12 +1052,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1349,37 +1375,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1408,7 +1434,7 @@
       <c r="H2">
         <v>-4300.3</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>39285</v>
       </c>
       <c r="K2" t="b">
@@ -1440,7 +1466,7 @@
       <c r="H3">
         <v>-2354.2</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>40669</v>
       </c>
       <c r="K3" t="b">
@@ -1472,7 +1498,7 @@
       <c r="H4">
         <v>-910.7</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>40669</v>
       </c>
       <c r="K4" t="b">
@@ -1504,7 +1530,7 @@
       <c r="H5">
         <v>-868</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>44884</v>
       </c>
       <c r="K5" t="b">
@@ -1536,7 +1562,7 @@
       <c r="H6">
         <v>-483.8</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>43855</v>
       </c>
       <c r="K6" t="b">
@@ -1568,7 +1594,7 @@
       <c r="H7">
         <v>-417</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>46014</v>
       </c>
       <c r="K7" t="b">
@@ -1600,7 +1626,7 @@
       <c r="H8">
         <v>-414.2</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>46014</v>
       </c>
       <c r="K8" t="b">
@@ -1632,7 +1658,7 @@
       <c r="H9">
         <v>-391.8</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>42769</v>
       </c>
       <c r="K9" t="b">
@@ -1664,7 +1690,7 @@
       <c r="H10">
         <v>-391.6</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>45804</v>
       </c>
       <c r="K10" t="b">
@@ -1696,7 +1722,7 @@
       <c r="H11">
         <v>-391.6</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>45804</v>
       </c>
       <c r="K11" t="b">
@@ -1728,7 +1754,7 @@
       <c r="H12">
         <v>-372.9</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>42821</v>
       </c>
       <c r="K12" t="b">
@@ -1760,7 +1786,7 @@
       <c r="H13">
         <v>-372.9</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>46014</v>
       </c>
       <c r="K13" t="b">
@@ -1792,7 +1818,7 @@
       <c r="H14">
         <v>-372.9</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>46014</v>
       </c>
       <c r="K14" t="b">
@@ -1824,7 +1850,7 @@
       <c r="H15">
         <v>-372.9</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>46014</v>
       </c>
       <c r="K15" t="b">
@@ -1856,7 +1882,7 @@
       <c r="H16">
         <v>-367.8</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="2">
         <v>46017</v>
       </c>
       <c r="K16" t="b">
@@ -1888,7 +1914,7 @@
       <c r="H17">
         <v>-367.8</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="2">
         <v>46017</v>
       </c>
       <c r="K17" t="b">
@@ -1920,7 +1946,7 @@
       <c r="H18">
         <v>-347.2</v>
       </c>
-      <c r="J18" s="1">
+      <c r="J18" s="2">
         <v>40979</v>
       </c>
       <c r="K18" t="b">
@@ -1952,7 +1978,7 @@
       <c r="H19">
         <v>-293.8</v>
       </c>
-      <c r="J19" s="1">
+      <c r="J19" s="2">
         <v>45846</v>
       </c>
       <c r="K19" t="b">
@@ -1984,7 +2010,7 @@
       <c r="H20">
         <v>-206.4</v>
       </c>
-      <c r="J20" s="1">
+      <c r="J20" s="2">
         <v>36669</v>
       </c>
       <c r="K20" t="b">
@@ -2016,7 +2042,7 @@
       <c r="H21">
         <v>-131.6</v>
       </c>
-      <c r="J21" s="1">
+      <c r="J21" s="2">
         <v>46111</v>
       </c>
       <c r="K21" t="b">
@@ -2048,7 +2074,7 @@
       <c r="H22">
         <v>-131.6</v>
       </c>
-      <c r="J22" s="1">
+      <c r="J22" s="2">
         <v>46111</v>
       </c>
       <c r="K22" t="b">
@@ -2080,7 +2106,7 @@
       <c r="H23">
         <v>-131.6</v>
       </c>
-      <c r="J23" s="1">
+      <c r="J23" s="2">
         <v>46111</v>
       </c>
       <c r="K23" t="b">
@@ -2112,7 +2138,7 @@
       <c r="H24">
         <v>-131.6</v>
       </c>
-      <c r="J24" s="1">
+      <c r="J24" s="2">
         <v>46111</v>
       </c>
       <c r="K24" t="b">
@@ -2144,7 +2170,7 @@
       <c r="H25">
         <v>-131.6</v>
       </c>
-      <c r="J25" s="1">
+      <c r="J25" s="2">
         <v>46111</v>
       </c>
       <c r="K25" t="b">
@@ -2176,7 +2202,7 @@
       <c r="H26">
         <v>-98.3</v>
       </c>
-      <c r="J26" s="1">
+      <c r="J26" s="2">
         <v>41204</v>
       </c>
       <c r="K26" t="b">
@@ -2208,7 +2234,7 @@
       <c r="H27">
         <v>-47.2</v>
       </c>
-      <c r="J27" s="1">
+      <c r="J27" s="2">
         <v>44011</v>
       </c>
       <c r="K27" t="b">
@@ -2240,7 +2266,7 @@
       <c r="H28">
         <v>-22.3</v>
       </c>
-      <c r="J28" s="1">
+      <c r="J28" s="2">
         <v>46226</v>
       </c>
       <c r="K28" t="b">
@@ -2272,7 +2298,7 @@
       <c r="H29">
         <v>4.7</v>
       </c>
-      <c r="J29" s="1">
+      <c r="J29" s="2">
         <v>46265</v>
       </c>
       <c r="K29" t="b">
@@ -2304,7 +2330,7 @@
       <c r="H30">
         <v>7.5</v>
       </c>
-      <c r="J30" s="1">
+      <c r="J30" s="2">
         <v>46265</v>
       </c>
       <c r="K30" t="b">
@@ -2336,7 +2362,7 @@
       <c r="H31">
         <v>10</v>
       </c>
-      <c r="J31" s="1">
+      <c r="J31" s="2">
         <v>46265</v>
       </c>
       <c r="K31" t="b">
@@ -2368,7 +2394,7 @@
       <c r="H32">
         <v>12.8</v>
       </c>
-      <c r="J32" s="1">
+      <c r="J32" s="2">
         <v>46265</v>
       </c>
       <c r="K32" t="b">
@@ -2400,7 +2426,7 @@
       <c r="H33">
         <v>14</v>
       </c>
-      <c r="J33" s="1">
+      <c r="J33" s="2">
         <v>46265</v>
       </c>
       <c r="K33" t="b">
@@ -2432,7 +2458,7 @@
       <c r="H34">
         <v>17.8</v>
       </c>
-      <c r="J34" s="1">
+      <c r="J34" s="2">
         <v>46265</v>
       </c>
       <c r="K34" t="b">
@@ -2464,7 +2490,7 @@
       <c r="H35">
         <v>20.4</v>
       </c>
-      <c r="J35" s="1">
+      <c r="J35" s="2">
         <v>46265</v>
       </c>
       <c r="K35" t="b">
@@ -2496,7 +2522,7 @@
       <c r="H36">
         <v>21.2</v>
       </c>
-      <c r="J36" s="1">
+      <c r="J36" s="2">
         <v>46265</v>
       </c>
       <c r="K36" t="b">
@@ -2528,7 +2554,7 @@
       <c r="H37">
         <v>26.2</v>
       </c>
-      <c r="J37" s="1">
+      <c r="J37" s="2">
         <v>46265</v>
       </c>
       <c r="K37" t="b">
@@ -2560,7 +2586,7 @@
       <c r="H38">
         <v>33.6</v>
       </c>
-      <c r="J38" s="1">
+      <c r="J38" s="2">
         <v>46364</v>
       </c>
       <c r="K38" t="b">
@@ -2592,7 +2618,7 @@
       <c r="H39">
         <v>42.2</v>
       </c>
-      <c r="J39" s="1">
+      <c r="J39" s="2">
         <v>46269</v>
       </c>
       <c r="K39" t="b">
@@ -2624,7 +2650,7 @@
       <c r="H40">
         <v>42.8</v>
       </c>
-      <c r="J40" s="1">
+      <c r="J40" s="2">
         <v>46291</v>
       </c>
       <c r="K40" t="b">
@@ -2656,7 +2682,7 @@
       <c r="H41">
         <v>45.7</v>
       </c>
-      <c r="J41" s="1">
+      <c r="J41" s="2">
         <v>46395</v>
       </c>
       <c r="K41" t="b">
@@ -2688,7 +2714,7 @@
       <c r="H42">
         <v>47.2</v>
       </c>
-      <c r="J42" s="1">
+      <c r="J42" s="2">
         <v>46280</v>
       </c>
       <c r="K42" t="b">
@@ -2720,7 +2746,7 @@
       <c r="H43">
         <v>48.7</v>
       </c>
-      <c r="J43" s="1">
+      <c r="J43" s="2">
         <v>46281</v>
       </c>
       <c r="K43" t="b">
@@ -2752,7 +2778,7 @@
       <c r="H44">
         <v>60</v>
       </c>
-      <c r="J44" s="1">
+      <c r="J44" s="2">
         <v>46281</v>
       </c>
       <c r="K44" t="b">
@@ -2784,7 +2810,7 @@
       <c r="H45">
         <v>62.6</v>
       </c>
-      <c r="J45" s="1">
+      <c r="J45" s="2">
         <v>46265</v>
       </c>
       <c r="K45" t="b">
@@ -2816,7 +2842,7 @@
       <c r="H46">
         <v>64.59999999999999</v>
       </c>
-      <c r="J46" s="1">
+      <c r="J46" s="2">
         <v>46265</v>
       </c>
       <c r="K46" t="b">
@@ -2848,7 +2874,7 @@
       <c r="H47">
         <v>67.59999999999999</v>
       </c>
-      <c r="J47" s="1">
+      <c r="J47" s="2">
         <v>46267</v>
       </c>
       <c r="K47" t="b">
@@ -2880,7 +2906,7 @@
       <c r="H48">
         <v>68.3</v>
       </c>
-      <c r="J48" s="1">
+      <c r="J48" s="2">
         <v>46278</v>
       </c>
       <c r="K48" t="b">
@@ -2912,7 +2938,7 @@
       <c r="H49">
         <v>69.2</v>
       </c>
-      <c r="J49" s="1">
+      <c r="J49" s="2">
         <v>46453</v>
       </c>
       <c r="K49" t="b">
@@ -2944,7 +2970,7 @@
       <c r="H50">
         <v>69.8</v>
       </c>
-      <c r="J50" s="1">
+      <c r="J50" s="2">
         <v>46265</v>
       </c>
       <c r="K50" t="b">
@@ -2976,7 +3002,7 @@
       <c r="H51">
         <v>69.8</v>
       </c>
-      <c r="J51" s="1">
+      <c r="J51" s="2">
         <v>46265</v>
       </c>
       <c r="K51" t="b">
@@ -3008,7 +3034,7 @@
       <c r="H52">
         <v>72.2</v>
       </c>
-      <c r="J52" s="1">
+      <c r="J52" s="2">
         <v>46275</v>
       </c>
       <c r="K52" t="b">
@@ -3040,7 +3066,7 @@
       <c r="H53">
         <v>72.2</v>
       </c>
-      <c r="J53" s="1">
+      <c r="J53" s="2">
         <v>46275</v>
       </c>
       <c r="K53" t="b">
@@ -3072,7 +3098,7 @@
       <c r="H54">
         <v>78.09999999999999</v>
       </c>
-      <c r="J54" s="1">
+      <c r="J54" s="2">
         <v>46265</v>
       </c>
       <c r="K54" t="b">
@@ -3104,7 +3130,7 @@
       <c r="H55">
         <v>82.8</v>
       </c>
-      <c r="J55" s="1">
+      <c r="J55" s="2">
         <v>46487</v>
       </c>
       <c r="K55" t="b">
@@ -3136,7 +3162,7 @@
       <c r="H56">
         <v>83.09999999999999</v>
       </c>
-      <c r="J56" s="1">
+      <c r="J56" s="2">
         <v>46285</v>
       </c>
       <c r="K56" t="b">
@@ -3168,7 +3194,7 @@
       <c r="H57">
         <v>84.8</v>
       </c>
-      <c r="J57" s="1">
+      <c r="J57" s="2">
         <v>46492</v>
       </c>
       <c r="K57" t="b">
@@ -3200,7 +3226,7 @@
       <c r="H58">
         <v>104.9</v>
       </c>
-      <c r="J58" s="1">
+      <c r="J58" s="2">
         <v>46297</v>
       </c>
       <c r="K58" t="b">
@@ -3232,7 +3258,7 @@
       <c r="H59">
         <v>107.6</v>
       </c>
-      <c r="J59" s="1">
+      <c r="J59" s="2">
         <v>46283</v>
       </c>
       <c r="K59" t="b">
@@ -3264,7 +3290,7 @@
       <c r="H60">
         <v>111.9</v>
       </c>
-      <c r="J60" s="1">
+      <c r="J60" s="2">
         <v>46300</v>
       </c>
       <c r="K60" t="b">
@@ -3296,7 +3322,7 @@
       <c r="H61">
         <v>111.9</v>
       </c>
-      <c r="J61" s="1">
+      <c r="J61" s="2">
         <v>46300</v>
       </c>
       <c r="K61" t="b">
@@ -3328,7 +3354,7 @@
       <c r="H62">
         <v>111.9</v>
       </c>
-      <c r="J62" s="1">
+      <c r="J62" s="2">
         <v>46300</v>
       </c>
       <c r="K62" t="b">
@@ -3360,7 +3386,7 @@
       <c r="H63">
         <v>111.9</v>
       </c>
-      <c r="J63" s="1">
+      <c r="J63" s="2">
         <v>46300</v>
       </c>
       <c r="K63" t="b">
@@ -3392,7 +3418,7 @@
       <c r="H64">
         <v>111.9</v>
       </c>
-      <c r="J64" s="1">
+      <c r="J64" s="2">
         <v>46300</v>
       </c>
       <c r="K64" t="b">
@@ -3424,7 +3450,7 @@
       <c r="H65">
         <v>128.8</v>
       </c>
-      <c r="J65" s="1">
+      <c r="J65" s="2">
         <v>46308</v>
       </c>
       <c r="K65" t="b">
@@ -3456,7 +3482,7 @@
       <c r="H66">
         <v>131.1</v>
       </c>
-      <c r="J66" s="1">
+      <c r="J66" s="2">
         <v>46336</v>
       </c>
       <c r="K66" t="b">
@@ -3488,7 +3514,7 @@
       <c r="H67">
         <v>138.4</v>
       </c>
-      <c r="J67" s="1">
+      <c r="J67" s="2">
         <v>46343</v>
       </c>
       <c r="K67" t="b">
@@ -3520,7 +3546,7 @@
       <c r="H68">
         <v>141</v>
       </c>
-      <c r="J68" s="1">
+      <c r="J68" s="2">
         <v>46350</v>
       </c>
       <c r="K68" t="b">
@@ -3552,7 +3578,7 @@
       <c r="H69">
         <v>162</v>
       </c>
-      <c r="J69" s="1">
+      <c r="J69" s="2">
         <v>46391</v>
       </c>
       <c r="K69" t="b">
@@ -3584,7 +3610,7 @@
       <c r="H70">
         <v>167.2</v>
       </c>
-      <c r="J70" s="1">
+      <c r="J70" s="2">
         <v>46330</v>
       </c>
       <c r="K70" t="b">
@@ -3616,7 +3642,7 @@
       <c r="H71">
         <v>177.4</v>
       </c>
-      <c r="J71" s="1">
+      <c r="J71" s="2">
         <v>46418</v>
       </c>
       <c r="K71" t="b">
@@ -3648,7 +3674,7 @@
       <c r="H72">
         <v>200</v>
       </c>
-      <c r="J72" s="1">
+      <c r="J72" s="2">
         <v>46356</v>
       </c>
       <c r="K72" t="b">
@@ -3680,7 +3706,7 @@
       <c r="H73">
         <v>203.6</v>
       </c>
-      <c r="J73" s="1">
+      <c r="J73" s="2">
         <v>46436</v>
       </c>
       <c r="K73" t="b">
@@ -3712,7 +3738,7 @@
       <c r="H74">
         <v>221.2</v>
       </c>
-      <c r="J74" s="1">
+      <c r="J74" s="2">
         <v>46426</v>
       </c>
       <c r="K74" t="b">
@@ -3744,7 +3770,7 @@
       <c r="H75">
         <v>240.8</v>
       </c>
-      <c r="J75" s="1">
+      <c r="J75" s="2">
         <v>46450</v>
       </c>
       <c r="K75" t="b">
@@ -3776,7 +3802,7 @@
       <c r="H76">
         <v>245.8</v>
       </c>
-      <c r="J76" s="1">
+      <c r="J76" s="2">
         <v>46452</v>
       </c>
       <c r="K76" t="b">
@@ -3808,7 +3834,7 @@
       <c r="H77">
         <v>263.4</v>
       </c>
-      <c r="J77" s="1">
+      <c r="J77" s="2">
         <v>46322</v>
       </c>
       <c r="K77" t="b">
@@ -3840,7 +3866,7 @@
       <c r="H78">
         <v>275.2</v>
       </c>
-      <c r="J78" s="1">
+      <c r="J78" s="2">
         <v>46433</v>
       </c>
       <c r="K78" t="b">
@@ -3875,7 +3901,7 @@
       <c r="I79" t="s">
         <v>311</v>
       </c>
-      <c r="J79" s="1">
+      <c r="J79" s="2">
         <v>36557</v>
       </c>
       <c r="K79" t="b">
@@ -3910,7 +3936,7 @@
       <c r="I80" t="s">
         <v>312</v>
       </c>
-      <c r="J80" s="1">
+      <c r="J80" s="2">
         <v>41275</v>
       </c>
       <c r="K80" t="b">
@@ -3945,7 +3971,7 @@
       <c r="I81" t="s">
         <v>313</v>
       </c>
-      <c r="J81" s="1">
+      <c r="J81" s="2">
         <v>45380</v>
       </c>
       <c r="K81" t="b">
@@ -3980,7 +4006,7 @@
       <c r="I82" t="s">
         <v>314</v>
       </c>
-      <c r="J82" s="1">
+      <c r="J82" s="2">
         <v>45421</v>
       </c>
       <c r="K82" t="b">
@@ -4015,7 +4041,7 @@
       <c r="I83" t="s">
         <v>314</v>
       </c>
-      <c r="J83" s="1">
+      <c r="J83" s="2">
         <v>45428</v>
       </c>
       <c r="K83" t="b">
@@ -4050,7 +4076,7 @@
       <c r="I84" t="s">
         <v>315</v>
       </c>
-      <c r="J84" s="1">
+      <c r="J84" s="2">
         <v>45490</v>
       </c>
       <c r="K84" t="b">
@@ -4085,7 +4111,7 @@
       <c r="I85" t="s">
         <v>316</v>
       </c>
-      <c r="J85" s="1">
+      <c r="J85" s="2">
         <v>45566</v>
       </c>
       <c r="K85" t="b">
@@ -4120,7 +4146,7 @@
       <c r="I86" t="s">
         <v>317</v>
       </c>
-      <c r="J86" s="1">
+      <c r="J86" s="2">
         <v>45986</v>
       </c>
       <c r="K86" t="b">
@@ -4155,7 +4181,7 @@
       <c r="I87" t="s">
         <v>318</v>
       </c>
-      <c r="J87" s="1">
+      <c r="J87" s="2">
         <v>46284</v>
       </c>
       <c r="K87" t="b">
@@ -4190,7 +4216,7 @@
       <c r="I88" t="s">
         <v>319</v>
       </c>
-      <c r="J88" s="1">
+      <c r="J88" s="2">
         <v>46305</v>
       </c>
       <c r="K88" t="b">
@@ -4225,7 +4251,7 @@
       <c r="I89" t="s">
         <v>319</v>
       </c>
-      <c r="J89" s="1">
+      <c r="J89" s="2">
         <v>46310</v>
       </c>
       <c r="K89" t="b">
@@ -4260,7 +4286,7 @@
       <c r="I90" t="s">
         <v>319</v>
       </c>
-      <c r="J90" s="1">
+      <c r="J90" s="2">
         <v>46317</v>
       </c>
       <c r="K90" t="b">
@@ -4295,7 +4321,7 @@
       <c r="I91" t="s">
         <v>319</v>
       </c>
-      <c r="J91" s="1">
+      <c r="J91" s="2">
         <v>46319</v>
       </c>
       <c r="K91" t="b">
@@ -4330,7 +4356,7 @@
       <c r="I92" t="s">
         <v>320</v>
       </c>
-      <c r="J92" s="1">
+      <c r="J92" s="2">
         <v>46333</v>
       </c>
       <c r="K92" t="b">
@@ -4365,7 +4391,7 @@
       <c r="I93" t="s">
         <v>320</v>
       </c>
-      <c r="J93" s="1">
+      <c r="J93" s="2">
         <v>46338</v>
       </c>
       <c r="K93" t="b">
@@ -4400,7 +4426,7 @@
       <c r="I94" t="s">
         <v>320</v>
       </c>
-      <c r="J94" s="1">
+      <c r="J94" s="2">
         <v>46338</v>
       </c>
       <c r="K94" t="b">
@@ -4435,7 +4461,7 @@
       <c r="I95" t="s">
         <v>320</v>
       </c>
-      <c r="J95" s="1">
+      <c r="J95" s="2">
         <v>46341</v>
       </c>
       <c r="K95" t="b">
@@ -4470,7 +4496,7 @@
       <c r="I96" t="s">
         <v>320</v>
       </c>
-      <c r="J96" s="1">
+      <c r="J96" s="2">
         <v>46344</v>
       </c>
       <c r="K96" t="b">
@@ -4505,7 +4531,7 @@
       <c r="I97" t="s">
         <v>321</v>
       </c>
-      <c r="J97" s="1">
+      <c r="J97" s="2">
         <v>46360</v>
       </c>
       <c r="K97" t="b">
@@ -4540,7 +4566,7 @@
       <c r="I98" t="s">
         <v>321</v>
       </c>
-      <c r="J98" s="1">
+      <c r="J98" s="2">
         <v>46360</v>
       </c>
       <c r="K98" t="b">
@@ -4575,7 +4601,7 @@
       <c r="I99" t="s">
         <v>321</v>
       </c>
-      <c r="J99" s="1">
+      <c r="J99" s="2">
         <v>46367</v>
       </c>
       <c r="K99" t="b">
@@ -4610,7 +4636,7 @@
       <c r="I100" t="s">
         <v>321</v>
       </c>
-      <c r="J100" s="1">
+      <c r="J100" s="2">
         <v>46375</v>
       </c>
       <c r="K100" t="b">
@@ -4645,7 +4671,7 @@
       <c r="I101" t="s">
         <v>321</v>
       </c>
-      <c r="J101" s="1">
+      <c r="J101" s="2">
         <v>46387</v>
       </c>
       <c r="K101" t="b">
@@ -4680,7 +4706,7 @@
       <c r="I102" t="s">
         <v>321</v>
       </c>
-      <c r="J102" s="1">
+      <c r="J102" s="2">
         <v>46387</v>
       </c>
       <c r="K102" t="b">
@@ -4715,7 +4741,7 @@
       <c r="I103" t="s">
         <v>321</v>
       </c>
-      <c r="J103" s="1">
+      <c r="J103" s="2">
         <v>46387</v>
       </c>
       <c r="K103" t="b">
@@ -4750,7 +4776,7 @@
       <c r="I104" t="s">
         <v>321</v>
       </c>
-      <c r="J104" s="1">
+      <c r="J104" s="2">
         <v>46388</v>
       </c>
       <c r="K104" t="b">
@@ -4785,7 +4811,7 @@
       <c r="I105" t="s">
         <v>322</v>
       </c>
-      <c r="J105" s="1">
+      <c r="J105" s="2">
         <v>46401</v>
       </c>
       <c r="K105" t="b">
@@ -4820,7 +4846,7 @@
       <c r="I106" t="s">
         <v>322</v>
       </c>
-      <c r="J106" s="1">
+      <c r="J106" s="2">
         <v>46401</v>
       </c>
       <c r="K106" t="b">
@@ -4855,7 +4881,7 @@
       <c r="I107" t="s">
         <v>322</v>
       </c>
-      <c r="J107" s="1">
+      <c r="J107" s="2">
         <v>46401</v>
       </c>
       <c r="K107" t="b">
@@ -4890,7 +4916,7 @@
       <c r="I108" t="s">
         <v>322</v>
       </c>
-      <c r="J108" s="1">
+      <c r="J108" s="2">
         <v>46412</v>
       </c>
       <c r="K108" t="b">
@@ -4925,7 +4951,7 @@
       <c r="I109" t="s">
         <v>322</v>
       </c>
-      <c r="J109" s="1">
+      <c r="J109" s="2">
         <v>46412</v>
       </c>
       <c r="K109" t="b">
@@ -4960,7 +4986,7 @@
       <c r="I110" t="s">
         <v>322</v>
       </c>
-      <c r="J110" s="1">
+      <c r="J110" s="2">
         <v>46412</v>
       </c>
       <c r="K110" t="b">
@@ -4995,7 +5021,7 @@
       <c r="I111" t="s">
         <v>323</v>
       </c>
-      <c r="J111" s="1">
+      <c r="J111" s="2">
         <v>46424</v>
       </c>
       <c r="K111" t="b">
@@ -5030,7 +5056,7 @@
       <c r="I112" t="s">
         <v>323</v>
       </c>
-      <c r="J112" s="1">
+      <c r="J112" s="2">
         <v>46437</v>
       </c>
       <c r="K112" t="b">
@@ -5065,7 +5091,7 @@
       <c r="I113" t="s">
         <v>323</v>
       </c>
-      <c r="J113" s="1">
+      <c r="J113" s="2">
         <v>46451</v>
       </c>
       <c r="K113" t="b">
@@ -5100,7 +5126,7 @@
       <c r="I114" t="s">
         <v>323</v>
       </c>
-      <c r="J114" s="1">
+      <c r="J114" s="2">
         <v>46451</v>
       </c>
       <c r="K114" t="b">
@@ -5135,7 +5161,7 @@
       <c r="I115" t="s">
         <v>324</v>
       </c>
-      <c r="J115" s="1">
+      <c r="J115" s="2">
         <v>46455</v>
       </c>
       <c r="K115" t="b">
@@ -5170,7 +5196,7 @@
       <c r="I116" t="s">
         <v>324</v>
       </c>
-      <c r="J116" s="1">
+      <c r="J116" s="2">
         <v>46456</v>
       </c>
       <c r="K116" t="b">
@@ -5205,7 +5231,7 @@
       <c r="I117" t="s">
         <v>324</v>
       </c>
-      <c r="J117" s="1">
+      <c r="J117" s="2">
         <v>46457</v>
       </c>
       <c r="K117" t="b">
@@ -5240,7 +5266,7 @@
       <c r="I118" t="s">
         <v>324</v>
       </c>
-      <c r="J118" s="1">
+      <c r="J118" s="2">
         <v>46464</v>
       </c>
       <c r="K118" t="b">
@@ -5275,7 +5301,7 @@
       <c r="I119" t="s">
         <v>324</v>
       </c>
-      <c r="J119" s="1">
+      <c r="J119" s="2">
         <v>46470</v>
       </c>
       <c r="K119" t="b">
@@ -5310,7 +5336,7 @@
       <c r="I120" t="s">
         <v>325</v>
       </c>
-      <c r="J120" s="1">
+      <c r="J120" s="2">
         <v>46485</v>
       </c>
       <c r="K120" t="b">
@@ -5345,7 +5371,7 @@
       <c r="I121" t="s">
         <v>325</v>
       </c>
-      <c r="J121" s="1">
+      <c r="J121" s="2">
         <v>46499</v>
       </c>
       <c r="K121" t="b">
@@ -5380,7 +5406,7 @@
       <c r="I122" t="s">
         <v>325</v>
       </c>
-      <c r="J122" s="1">
+      <c r="J122" s="2">
         <v>46504</v>
       </c>
       <c r="K122" t="b">
@@ -5415,7 +5441,7 @@
       <c r="I123" t="s">
         <v>325</v>
       </c>
-      <c r="J123" s="1">
+      <c r="J123" s="2">
         <v>46504</v>
       </c>
       <c r="K123" t="b">
@@ -5450,7 +5476,7 @@
       <c r="I124" t="s">
         <v>325</v>
       </c>
-      <c r="J124" s="1">
+      <c r="J124" s="2">
         <v>46507</v>
       </c>
       <c r="K124" t="b">
@@ -5485,7 +5511,7 @@
       <c r="I125" t="s">
         <v>325</v>
       </c>
-      <c r="J125" s="1">
+      <c r="J125" s="2">
         <v>46508</v>
       </c>
       <c r="K125" t="b">
@@ -5520,7 +5546,7 @@
       <c r="I126" t="s">
         <v>325</v>
       </c>
-      <c r="J126" s="1">
+      <c r="J126" s="2">
         <v>46512</v>
       </c>
       <c r="K126" t="b">
@@ -5555,7 +5581,7 @@
       <c r="I127" t="s">
         <v>326</v>
       </c>
-      <c r="J127" s="1">
+      <c r="J127" s="2">
         <v>46512</v>
       </c>
       <c r="K127" t="b">
@@ -5590,7 +5616,7 @@
       <c r="I128" t="s">
         <v>326</v>
       </c>
-      <c r="J128" s="1">
+      <c r="J128" s="2">
         <v>46528</v>
       </c>
       <c r="K128" t="b">
@@ -5625,7 +5651,7 @@
       <c r="I129" t="s">
         <v>326</v>
       </c>
-      <c r="J129" s="1">
+      <c r="J129" s="2">
         <v>46529</v>
       </c>
       <c r="K129" t="b">
@@ -5660,7 +5686,7 @@
       <c r="I130" t="s">
         <v>326</v>
       </c>
-      <c r="J130" s="1">
+      <c r="J130" s="2">
         <v>46537</v>
       </c>
       <c r="K130" t="b">
@@ -5695,7 +5721,7 @@
       <c r="I131" t="s">
         <v>327</v>
       </c>
-      <c r="J131" s="1">
+      <c r="J131" s="2">
         <v>46546</v>
       </c>
       <c r="K131" t="b">
@@ -5730,7 +5756,7 @@
       <c r="I132" t="s">
         <v>327</v>
       </c>
-      <c r="J132" s="1">
+      <c r="J132" s="2">
         <v>46547</v>
       </c>
       <c r="K132" t="b">
@@ -5765,7 +5791,7 @@
       <c r="I133" t="s">
         <v>327</v>
       </c>
-      <c r="J133" s="1">
+      <c r="J133" s="2">
         <v>46547</v>
       </c>
       <c r="K133" t="b">
@@ -5800,7 +5826,7 @@
       <c r="I134" t="s">
         <v>327</v>
       </c>
-      <c r="J134" s="1">
+      <c r="J134" s="2">
         <v>46547</v>
       </c>
       <c r="K134" t="b">
@@ -5835,7 +5861,7 @@
       <c r="I135" t="s">
         <v>327</v>
       </c>
-      <c r="J135" s="1">
+      <c r="J135" s="2">
         <v>46551</v>
       </c>
       <c r="K135" t="b">
@@ -5870,7 +5896,7 @@
       <c r="I136" t="s">
         <v>327</v>
       </c>
-      <c r="J136" s="1">
+      <c r="J136" s="2">
         <v>46560</v>
       </c>
       <c r="K136" t="b">
@@ -5905,7 +5931,7 @@
       <c r="I137" t="s">
         <v>327</v>
       </c>
-      <c r="J137" s="1">
+      <c r="J137" s="2">
         <v>46564</v>
       </c>
       <c r="K137" t="b">
@@ -5940,7 +5966,7 @@
       <c r="I138" t="s">
         <v>327</v>
       </c>
-      <c r="J138" s="1">
+      <c r="J138" s="2">
         <v>46567</v>
       </c>
       <c r="K138" t="b">
@@ -5975,7 +6001,7 @@
       <c r="I139" t="s">
         <v>327</v>
       </c>
-      <c r="J139" s="1">
+      <c r="J139" s="2">
         <v>46568</v>
       </c>
       <c r="K139" t="b">
@@ -6010,7 +6036,7 @@
       <c r="I140" t="s">
         <v>328</v>
       </c>
-      <c r="J140" s="1">
+      <c r="J140" s="2">
         <v>46578</v>
       </c>
       <c r="K140" t="b">
@@ -6045,7 +6071,7 @@
       <c r="I141" t="s">
         <v>328</v>
       </c>
-      <c r="J141" s="1">
+      <c r="J141" s="2">
         <v>46592</v>
       </c>
       <c r="K141" t="b">
@@ -6080,7 +6106,7 @@
       <c r="I142" t="s">
         <v>328</v>
       </c>
-      <c r="J142" s="1">
+      <c r="J142" s="2">
         <v>46592</v>
       </c>
       <c r="K142" t="b">
@@ -6115,7 +6141,7 @@
       <c r="I143" t="s">
         <v>329</v>
       </c>
-      <c r="J143" s="1">
+      <c r="J143" s="2">
         <v>46212</v>
       </c>
       <c r="K143" t="b">
@@ -6150,7 +6176,7 @@
       <c r="I144" t="s">
         <v>330</v>
       </c>
-      <c r="J144" s="1">
+      <c r="J144" s="2">
         <v>46225</v>
       </c>
       <c r="K144" t="b">
@@ -6185,7 +6211,7 @@
       <c r="I145" t="s">
         <v>331</v>
       </c>
-      <c r="J145" s="1">
+      <c r="J145" s="2">
         <v>46263</v>
       </c>
       <c r="K145" t="b">
@@ -6217,7 +6243,7 @@
       <c r="H146">
         <v>-1476</v>
       </c>
-      <c r="J146" s="1">
+      <c r="J146" s="2">
         <v>43773</v>
       </c>
       <c r="K146" t="b">
@@ -6249,7 +6275,7 @@
       <c r="H147">
         <v>-1469</v>
       </c>
-      <c r="J147" s="1">
+      <c r="J147" s="2">
         <v>43773</v>
       </c>
       <c r="K147" t="b">
@@ -6281,7 +6307,7 @@
       <c r="H148">
         <v>-1186</v>
       </c>
-      <c r="J148" s="1">
+      <c r="J148" s="2">
         <v>45295</v>
       </c>
       <c r="K148" t="b">
@@ -6313,7 +6339,7 @@
       <c r="H149">
         <v>-1048</v>
       </c>
-      <c r="J149" s="1">
+      <c r="J149" s="2">
         <v>45617</v>
       </c>
       <c r="K149" t="b">
@@ -6345,7 +6371,7 @@
       <c r="H150">
         <v>-980</v>
       </c>
-      <c r="J150" s="1">
+      <c r="J150" s="2">
         <v>45677</v>
       </c>
       <c r="K150" t="b">
@@ -6377,7 +6403,7 @@
       <c r="H151">
         <v>-961</v>
       </c>
-      <c r="J151" s="1">
+      <c r="J151" s="2">
         <v>44944</v>
       </c>
       <c r="K151" t="b">
@@ -6409,7 +6435,7 @@
       <c r="H152">
         <v>-252</v>
       </c>
-      <c r="J152" s="1">
+      <c r="J152" s="2">
         <v>46092</v>
       </c>
       <c r="K152" t="b">
@@ -6441,7 +6467,7 @@
       <c r="H153">
         <v>3</v>
       </c>
-      <c r="J153" s="1">
+      <c r="J153" s="2">
         <v>46265</v>
       </c>
       <c r="K153" t="b">
@@ -6473,7 +6499,7 @@
       <c r="H154">
         <v>3</v>
       </c>
-      <c r="J154" s="1">
+      <c r="J154" s="2">
         <v>46265</v>
       </c>
       <c r="K154" t="b">
@@ -6505,7 +6531,7 @@
       <c r="H155">
         <v>43</v>
       </c>
-      <c r="J155" s="1">
+      <c r="J155" s="2">
         <v>46440</v>
       </c>
       <c r="K155" t="b">
@@ -6537,7 +6563,7 @@
       <c r="H156">
         <v>43</v>
       </c>
-      <c r="J156" s="1">
+      <c r="J156" s="2">
         <v>46440</v>
       </c>
       <c r="K156" t="b">
@@ -6569,7 +6595,7 @@
       <c r="H157">
         <v>72</v>
       </c>
-      <c r="J157" s="1">
+      <c r="J157" s="2">
         <v>46289</v>
       </c>
       <c r="K157" t="b">
@@ -6601,7 +6627,7 @@
       <c r="H158">
         <v>72</v>
       </c>
-      <c r="J158" s="1">
+      <c r="J158" s="2">
         <v>46289</v>
       </c>
       <c r="K158" t="b">
@@ -6633,7 +6659,7 @@
       <c r="H159">
         <v>81</v>
       </c>
-      <c r="J159" s="1">
+      <c r="J159" s="2">
         <v>46405</v>
       </c>
       <c r="K159" t="b">
@@ -6665,7 +6691,7 @@
       <c r="H160">
         <v>102</v>
       </c>
-      <c r="J160" s="1">
+      <c r="J160" s="2">
         <v>46463</v>
       </c>
       <c r="K160" t="b">
@@ -6697,7 +6723,7 @@
       <c r="H161">
         <v>109</v>
       </c>
-      <c r="J161" s="1">
+      <c r="J161" s="2">
         <v>46353</v>
       </c>
       <c r="K161" t="b">
@@ -6729,7 +6755,7 @@
       <c r="H162">
         <v>127</v>
       </c>
-      <c r="J162" s="1">
+      <c r="J162" s="2">
         <v>46417</v>
       </c>
       <c r="K162" t="b">
@@ -6761,7 +6787,7 @@
       <c r="H163">
         <v>152</v>
       </c>
-      <c r="J163" s="1">
+      <c r="J163" s="2">
         <v>46271</v>
       </c>
       <c r="K163" t="b">
@@ -6793,7 +6819,7 @@
       <c r="H164">
         <v>152</v>
       </c>
-      <c r="J164" s="1">
+      <c r="J164" s="2">
         <v>46271</v>
       </c>
       <c r="K164" t="b">
@@ -6825,7 +6851,7 @@
       <c r="H165">
         <v>153</v>
       </c>
-      <c r="J165" s="1">
+      <c r="J165" s="2">
         <v>46458</v>
       </c>
       <c r="K165" t="b">
@@ -6857,7 +6883,7 @@
       <c r="H166">
         <v>158</v>
       </c>
-      <c r="J166" s="1">
+      <c r="J166" s="2">
         <v>46381</v>
       </c>
       <c r="K166" t="b">
@@ -6889,7 +6915,7 @@
       <c r="H167">
         <v>163</v>
       </c>
-      <c r="J167" s="1">
+      <c r="J167" s="2">
         <v>46592</v>
       </c>
       <c r="K167" t="b">
@@ -6921,7 +6947,7 @@
       <c r="H168">
         <v>167</v>
       </c>
-      <c r="J168" s="1">
+      <c r="J168" s="2">
         <v>46441</v>
       </c>
       <c r="K168" t="b">
@@ -6953,7 +6979,7 @@
       <c r="H169">
         <v>169</v>
       </c>
-      <c r="J169" s="1">
+      <c r="J169" s="2">
         <v>46391</v>
       </c>
       <c r="K169" t="b">
@@ -6985,7 +7011,7 @@
       <c r="H170">
         <v>184</v>
       </c>
-      <c r="J170" s="1">
+      <c r="J170" s="2">
         <v>46385</v>
       </c>
       <c r="K170" t="b">
@@ -7017,7 +7043,7 @@
       <c r="H171">
         <v>186</v>
       </c>
-      <c r="J171" s="1">
+      <c r="J171" s="2">
         <v>46387</v>
       </c>
       <c r="K171" t="b">
@@ -7049,7 +7075,7 @@
       <c r="H172">
         <v>206</v>
       </c>
-      <c r="J172" s="1">
+      <c r="J172" s="2">
         <v>46399</v>
       </c>
       <c r="K172" t="b">
@@ -7081,7 +7107,7 @@
       <c r="H173">
         <v>206</v>
       </c>
-      <c r="J173" s="1">
+      <c r="J173" s="2">
         <v>46399</v>
       </c>
       <c r="K173" t="b">
@@ -7113,7 +7139,7 @@
       <c r="H174">
         <v>234</v>
       </c>
-      <c r="J174" s="1">
+      <c r="J174" s="2">
         <v>46458</v>
       </c>
       <c r="K174" t="b">
@@ -7145,7 +7171,7 @@
       <c r="H175">
         <v>248</v>
       </c>
-      <c r="J175" s="1">
+      <c r="J175" s="2">
         <v>46528</v>
       </c>
       <c r="K175" t="b">
@@ -7177,7 +7203,7 @@
       <c r="H176">
         <v>317</v>
       </c>
-      <c r="J176" s="1">
+      <c r="J176" s="2">
         <v>46540</v>
       </c>
       <c r="K176" t="b">
@@ -7209,7 +7235,7 @@
       <c r="H177">
         <v>340</v>
       </c>
-      <c r="J177" s="1">
+      <c r="J177" s="2">
         <v>46547</v>
       </c>
       <c r="K177" t="b">
@@ -7241,7 +7267,7 @@
       <c r="H178">
         <v>364</v>
       </c>
-      <c r="J178" s="1">
+      <c r="J178" s="2">
         <v>46557</v>
       </c>
       <c r="K178" t="b">
@@ -7273,7 +7299,7 @@
       <c r="H179">
         <v>368</v>
       </c>
-      <c r="J179" s="1">
+      <c r="J179" s="2">
         <v>46571</v>
       </c>
       <c r="K179" t="b">
@@ -7305,7 +7331,7 @@
       <c r="H180">
         <v>368</v>
       </c>
-      <c r="J180" s="1">
+      <c r="J180" s="2">
         <v>46571</v>
       </c>
       <c r="K180" t="b">
@@ -7337,7 +7363,7 @@
       <c r="H181">
         <v>370</v>
       </c>
-      <c r="J181" s="1">
+      <c r="J181" s="2">
         <v>46562</v>
       </c>
       <c r="K181" t="b">
@@ -7369,7 +7395,7 @@
       <c r="H182">
         <v>385</v>
       </c>
-      <c r="J182" s="1">
+      <c r="J182" s="2">
         <v>46574</v>
       </c>
       <c r="K182" t="b">
@@ -7401,7 +7427,7 @@
       <c r="H183">
         <v>385</v>
       </c>
-      <c r="J183" s="1">
+      <c r="J183" s="2">
         <v>46574</v>
       </c>
       <c r="K183" t="b">
@@ -7433,7 +7459,7 @@
       <c r="H184">
         <v>417</v>
       </c>
-      <c r="J184" s="1">
+      <c r="J184" s="2">
         <v>46578</v>
       </c>
       <c r="K184" t="b">
@@ -7465,7 +7491,7 @@
       <c r="H185">
         <v>721</v>
       </c>
-      <c r="J185" s="1">
+      <c r="J185" s="2">
         <v>46345</v>
       </c>
       <c r="K185" t="b">
@@ -7497,7 +7523,7 @@
       <c r="H186">
         <v>721</v>
       </c>
-      <c r="J186" s="1">
+      <c r="J186" s="2">
         <v>46345</v>
       </c>
       <c r="K186" t="b">
@@ -7529,7 +7555,7 @@
       <c r="H187">
         <v>850</v>
       </c>
-      <c r="J187" s="1">
+      <c r="J187" s="2">
         <v>46366</v>
       </c>
       <c r="K187" t="b">
@@ -7561,7 +7587,7 @@
       <c r="H188">
         <v>850</v>
       </c>
-      <c r="J188" s="1">
+      <c r="J188" s="2">
         <v>46366</v>
       </c>
       <c r="K188" t="b">
@@ -7593,7 +7619,7 @@
       <c r="H189">
         <v>1661</v>
       </c>
-      <c r="J189" s="1">
+      <c r="J189" s="2">
         <v>46524</v>
       </c>
       <c r="K189" t="b">
@@ -7625,7 +7651,7 @@
       <c r="H190">
         <v>1661</v>
       </c>
-      <c r="J190" s="1">
+      <c r="J190" s="2">
         <v>46524</v>
       </c>
       <c r="K190" t="b">
@@ -7657,7 +7683,7 @@
       <c r="H191">
         <v>488</v>
       </c>
-      <c r="J191" s="1">
+      <c r="J191" s="2">
         <v>46190</v>
       </c>
       <c r="K191" t="b">
@@ -7689,7 +7715,7 @@
       <c r="H192">
         <v>25565</v>
       </c>
-      <c r="J192" s="1">
+      <c r="J192" s="2">
         <v>46190</v>
       </c>
       <c r="K192" t="b">
@@ -7721,7 +7747,7 @@
       <c r="H193">
         <v>25567</v>
       </c>
-      <c r="J193" s="1">
+      <c r="J193" s="2">
         <v>46190</v>
       </c>
       <c r="K193" t="b">
@@ -7753,7 +7779,7 @@
       <c r="H194">
         <v>31293</v>
       </c>
-      <c r="J194" s="1">
+      <c r="J194" s="2">
         <v>46190</v>
       </c>
       <c r="K194" t="b">

</xml_diff>

<commit_message>
Atualização automática: vencimentos_tmot (01/09/2026 12:27)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
@@ -1019,16 +1019,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1044,7 +1036,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1052,30 +1044,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1375,37 +1349,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1434,7 +1408,7 @@
       <c r="H2">
         <v>-4300.3</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>39285</v>
       </c>
       <c r="K2" t="b">
@@ -1466,7 +1440,7 @@
       <c r="H3">
         <v>-2354.2</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>40669</v>
       </c>
       <c r="K3" t="b">
@@ -1498,7 +1472,7 @@
       <c r="H4">
         <v>-910.7</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>40669</v>
       </c>
       <c r="K4" t="b">
@@ -1530,7 +1504,7 @@
       <c r="H5">
         <v>-868</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>44884</v>
       </c>
       <c r="K5" t="b">
@@ -1562,7 +1536,7 @@
       <c r="H6">
         <v>-483.8</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>43855</v>
       </c>
       <c r="K6" t="b">
@@ -1594,7 +1568,7 @@
       <c r="H7">
         <v>-417</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>46014</v>
       </c>
       <c r="K7" t="b">
@@ -1626,7 +1600,7 @@
       <c r="H8">
         <v>-414.2</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>46014</v>
       </c>
       <c r="K8" t="b">
@@ -1658,7 +1632,7 @@
       <c r="H9">
         <v>-391.8</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>42769</v>
       </c>
       <c r="K9" t="b">
@@ -1690,7 +1664,7 @@
       <c r="H10">
         <v>-391.6</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>45804</v>
       </c>
       <c r="K10" t="b">
@@ -1722,7 +1696,7 @@
       <c r="H11">
         <v>-391.6</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>45804</v>
       </c>
       <c r="K11" t="b">
@@ -1754,7 +1728,7 @@
       <c r="H12">
         <v>-372.9</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>42821</v>
       </c>
       <c r="K12" t="b">
@@ -1786,7 +1760,7 @@
       <c r="H13">
         <v>-372.9</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>46014</v>
       </c>
       <c r="K13" t="b">
@@ -1818,7 +1792,7 @@
       <c r="H14">
         <v>-372.9</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>46014</v>
       </c>
       <c r="K14" t="b">
@@ -1850,7 +1824,7 @@
       <c r="H15">
         <v>-372.9</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <v>46014</v>
       </c>
       <c r="K15" t="b">
@@ -1882,7 +1856,7 @@
       <c r="H16">
         <v>-367.8</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <v>46017</v>
       </c>
       <c r="K16" t="b">
@@ -1914,7 +1888,7 @@
       <c r="H17">
         <v>-367.8</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="1">
         <v>46017</v>
       </c>
       <c r="K17" t="b">
@@ -1946,7 +1920,7 @@
       <c r="H18">
         <v>-347.2</v>
       </c>
-      <c r="J18" s="2">
+      <c r="J18" s="1">
         <v>40979</v>
       </c>
       <c r="K18" t="b">
@@ -1978,7 +1952,7 @@
       <c r="H19">
         <v>-293.8</v>
       </c>
-      <c r="J19" s="2">
+      <c r="J19" s="1">
         <v>45846</v>
       </c>
       <c r="K19" t="b">
@@ -2010,7 +1984,7 @@
       <c r="H20">
         <v>-206.4</v>
       </c>
-      <c r="J20" s="2">
+      <c r="J20" s="1">
         <v>36669</v>
       </c>
       <c r="K20" t="b">
@@ -2042,7 +2016,7 @@
       <c r="H21">
         <v>-131.6</v>
       </c>
-      <c r="J21" s="2">
+      <c r="J21" s="1">
         <v>46111</v>
       </c>
       <c r="K21" t="b">
@@ -2074,7 +2048,7 @@
       <c r="H22">
         <v>-131.6</v>
       </c>
-      <c r="J22" s="2">
+      <c r="J22" s="1">
         <v>46111</v>
       </c>
       <c r="K22" t="b">
@@ -2106,7 +2080,7 @@
       <c r="H23">
         <v>-131.6</v>
       </c>
-      <c r="J23" s="2">
+      <c r="J23" s="1">
         <v>46111</v>
       </c>
       <c r="K23" t="b">
@@ -2138,7 +2112,7 @@
       <c r="H24">
         <v>-131.6</v>
       </c>
-      <c r="J24" s="2">
+      <c r="J24" s="1">
         <v>46111</v>
       </c>
       <c r="K24" t="b">
@@ -2170,7 +2144,7 @@
       <c r="H25">
         <v>-131.6</v>
       </c>
-      <c r="J25" s="2">
+      <c r="J25" s="1">
         <v>46111</v>
       </c>
       <c r="K25" t="b">
@@ -2202,7 +2176,7 @@
       <c r="H26">
         <v>-98.3</v>
       </c>
-      <c r="J26" s="2">
+      <c r="J26" s="1">
         <v>41204</v>
       </c>
       <c r="K26" t="b">
@@ -2234,7 +2208,7 @@
       <c r="H27">
         <v>-47.2</v>
       </c>
-      <c r="J27" s="2">
+      <c r="J27" s="1">
         <v>44011</v>
       </c>
       <c r="K27" t="b">
@@ -2266,7 +2240,7 @@
       <c r="H28">
         <v>-22.3</v>
       </c>
-      <c r="J28" s="2">
+      <c r="J28" s="1">
         <v>46226</v>
       </c>
       <c r="K28" t="b">
@@ -2298,7 +2272,7 @@
       <c r="H29">
         <v>4.7</v>
       </c>
-      <c r="J29" s="2">
+      <c r="J29" s="1">
         <v>46265</v>
       </c>
       <c r="K29" t="b">
@@ -2330,7 +2304,7 @@
       <c r="H30">
         <v>7.5</v>
       </c>
-      <c r="J30" s="2">
+      <c r="J30" s="1">
         <v>46265</v>
       </c>
       <c r="K30" t="b">
@@ -2362,7 +2336,7 @@
       <c r="H31">
         <v>10</v>
       </c>
-      <c r="J31" s="2">
+      <c r="J31" s="1">
         <v>46265</v>
       </c>
       <c r="K31" t="b">
@@ -2394,7 +2368,7 @@
       <c r="H32">
         <v>12.8</v>
       </c>
-      <c r="J32" s="2">
+      <c r="J32" s="1">
         <v>46265</v>
       </c>
       <c r="K32" t="b">
@@ -2426,7 +2400,7 @@
       <c r="H33">
         <v>14</v>
       </c>
-      <c r="J33" s="2">
+      <c r="J33" s="1">
         <v>46265</v>
       </c>
       <c r="K33" t="b">
@@ -2458,7 +2432,7 @@
       <c r="H34">
         <v>17.8</v>
       </c>
-      <c r="J34" s="2">
+      <c r="J34" s="1">
         <v>46265</v>
       </c>
       <c r="K34" t="b">
@@ -2490,7 +2464,7 @@
       <c r="H35">
         <v>20.4</v>
       </c>
-      <c r="J35" s="2">
+      <c r="J35" s="1">
         <v>46265</v>
       </c>
       <c r="K35" t="b">
@@ -2522,7 +2496,7 @@
       <c r="H36">
         <v>21.2</v>
       </c>
-      <c r="J36" s="2">
+      <c r="J36" s="1">
         <v>46265</v>
       </c>
       <c r="K36" t="b">
@@ -2554,7 +2528,7 @@
       <c r="H37">
         <v>26.2</v>
       </c>
-      <c r="J37" s="2">
+      <c r="J37" s="1">
         <v>46265</v>
       </c>
       <c r="K37" t="b">
@@ -2586,7 +2560,7 @@
       <c r="H38">
         <v>33.6</v>
       </c>
-      <c r="J38" s="2">
+      <c r="J38" s="1">
         <v>46364</v>
       </c>
       <c r="K38" t="b">
@@ -2618,7 +2592,7 @@
       <c r="H39">
         <v>42.2</v>
       </c>
-      <c r="J39" s="2">
+      <c r="J39" s="1">
         <v>46269</v>
       </c>
       <c r="K39" t="b">
@@ -2650,7 +2624,7 @@
       <c r="H40">
         <v>42.8</v>
       </c>
-      <c r="J40" s="2">
+      <c r="J40" s="1">
         <v>46291</v>
       </c>
       <c r="K40" t="b">
@@ -2682,7 +2656,7 @@
       <c r="H41">
         <v>45.7</v>
       </c>
-      <c r="J41" s="2">
+      <c r="J41" s="1">
         <v>46395</v>
       </c>
       <c r="K41" t="b">
@@ -2714,7 +2688,7 @@
       <c r="H42">
         <v>47.2</v>
       </c>
-      <c r="J42" s="2">
+      <c r="J42" s="1">
         <v>46280</v>
       </c>
       <c r="K42" t="b">
@@ -2746,7 +2720,7 @@
       <c r="H43">
         <v>48.7</v>
       </c>
-      <c r="J43" s="2">
+      <c r="J43" s="1">
         <v>46281</v>
       </c>
       <c r="K43" t="b">
@@ -2778,7 +2752,7 @@
       <c r="H44">
         <v>60</v>
       </c>
-      <c r="J44" s="2">
+      <c r="J44" s="1">
         <v>46281</v>
       </c>
       <c r="K44" t="b">
@@ -2810,7 +2784,7 @@
       <c r="H45">
         <v>62.6</v>
       </c>
-      <c r="J45" s="2">
+      <c r="J45" s="1">
         <v>46265</v>
       </c>
       <c r="K45" t="b">
@@ -2842,7 +2816,7 @@
       <c r="H46">
         <v>64.59999999999999</v>
       </c>
-      <c r="J46" s="2">
+      <c r="J46" s="1">
         <v>46265</v>
       </c>
       <c r="K46" t="b">
@@ -2874,7 +2848,7 @@
       <c r="H47">
         <v>67.59999999999999</v>
       </c>
-      <c r="J47" s="2">
+      <c r="J47" s="1">
         <v>46267</v>
       </c>
       <c r="K47" t="b">
@@ -2906,7 +2880,7 @@
       <c r="H48">
         <v>68.3</v>
       </c>
-      <c r="J48" s="2">
+      <c r="J48" s="1">
         <v>46278</v>
       </c>
       <c r="K48" t="b">
@@ -2938,7 +2912,7 @@
       <c r="H49">
         <v>69.2</v>
       </c>
-      <c r="J49" s="2">
+      <c r="J49" s="1">
         <v>46453</v>
       </c>
       <c r="K49" t="b">
@@ -2970,7 +2944,7 @@
       <c r="H50">
         <v>69.8</v>
       </c>
-      <c r="J50" s="2">
+      <c r="J50" s="1">
         <v>46265</v>
       </c>
       <c r="K50" t="b">
@@ -3002,7 +2976,7 @@
       <c r="H51">
         <v>69.8</v>
       </c>
-      <c r="J51" s="2">
+      <c r="J51" s="1">
         <v>46265</v>
       </c>
       <c r="K51" t="b">
@@ -3034,7 +3008,7 @@
       <c r="H52">
         <v>72.2</v>
       </c>
-      <c r="J52" s="2">
+      <c r="J52" s="1">
         <v>46275</v>
       </c>
       <c r="K52" t="b">
@@ -3066,7 +3040,7 @@
       <c r="H53">
         <v>72.2</v>
       </c>
-      <c r="J53" s="2">
+      <c r="J53" s="1">
         <v>46275</v>
       </c>
       <c r="K53" t="b">
@@ -3098,7 +3072,7 @@
       <c r="H54">
         <v>78.09999999999999</v>
       </c>
-      <c r="J54" s="2">
+      <c r="J54" s="1">
         <v>46265</v>
       </c>
       <c r="K54" t="b">
@@ -3130,7 +3104,7 @@
       <c r="H55">
         <v>82.8</v>
       </c>
-      <c r="J55" s="2">
+      <c r="J55" s="1">
         <v>46487</v>
       </c>
       <c r="K55" t="b">
@@ -3162,7 +3136,7 @@
       <c r="H56">
         <v>83.09999999999999</v>
       </c>
-      <c r="J56" s="2">
+      <c r="J56" s="1">
         <v>46285</v>
       </c>
       <c r="K56" t="b">
@@ -3194,7 +3168,7 @@
       <c r="H57">
         <v>84.8</v>
       </c>
-      <c r="J57" s="2">
+      <c r="J57" s="1">
         <v>46492</v>
       </c>
       <c r="K57" t="b">
@@ -3226,7 +3200,7 @@
       <c r="H58">
         <v>104.9</v>
       </c>
-      <c r="J58" s="2">
+      <c r="J58" s="1">
         <v>46297</v>
       </c>
       <c r="K58" t="b">
@@ -3258,7 +3232,7 @@
       <c r="H59">
         <v>107.6</v>
       </c>
-      <c r="J59" s="2">
+      <c r="J59" s="1">
         <v>46283</v>
       </c>
       <c r="K59" t="b">
@@ -3290,7 +3264,7 @@
       <c r="H60">
         <v>111.9</v>
       </c>
-      <c r="J60" s="2">
+      <c r="J60" s="1">
         <v>46300</v>
       </c>
       <c r="K60" t="b">
@@ -3322,7 +3296,7 @@
       <c r="H61">
         <v>111.9</v>
       </c>
-      <c r="J61" s="2">
+      <c r="J61" s="1">
         <v>46300</v>
       </c>
       <c r="K61" t="b">
@@ -3354,7 +3328,7 @@
       <c r="H62">
         <v>111.9</v>
       </c>
-      <c r="J62" s="2">
+      <c r="J62" s="1">
         <v>46300</v>
       </c>
       <c r="K62" t="b">
@@ -3386,7 +3360,7 @@
       <c r="H63">
         <v>111.9</v>
       </c>
-      <c r="J63" s="2">
+      <c r="J63" s="1">
         <v>46300</v>
       </c>
       <c r="K63" t="b">
@@ -3418,7 +3392,7 @@
       <c r="H64">
         <v>111.9</v>
       </c>
-      <c r="J64" s="2">
+      <c r="J64" s="1">
         <v>46300</v>
       </c>
       <c r="K64" t="b">
@@ -3450,7 +3424,7 @@
       <c r="H65">
         <v>128.8</v>
       </c>
-      <c r="J65" s="2">
+      <c r="J65" s="1">
         <v>46308</v>
       </c>
       <c r="K65" t="b">
@@ -3482,7 +3456,7 @@
       <c r="H66">
         <v>131.1</v>
       </c>
-      <c r="J66" s="2">
+      <c r="J66" s="1">
         <v>46336</v>
       </c>
       <c r="K66" t="b">
@@ -3514,7 +3488,7 @@
       <c r="H67">
         <v>138.4</v>
       </c>
-      <c r="J67" s="2">
+      <c r="J67" s="1">
         <v>46343</v>
       </c>
       <c r="K67" t="b">
@@ -3546,7 +3520,7 @@
       <c r="H68">
         <v>141</v>
       </c>
-      <c r="J68" s="2">
+      <c r="J68" s="1">
         <v>46350</v>
       </c>
       <c r="K68" t="b">
@@ -3578,7 +3552,7 @@
       <c r="H69">
         <v>162</v>
       </c>
-      <c r="J69" s="2">
+      <c r="J69" s="1">
         <v>46391</v>
       </c>
       <c r="K69" t="b">
@@ -3610,7 +3584,7 @@
       <c r="H70">
         <v>167.2</v>
       </c>
-      <c r="J70" s="2">
+      <c r="J70" s="1">
         <v>46330</v>
       </c>
       <c r="K70" t="b">
@@ -3642,7 +3616,7 @@
       <c r="H71">
         <v>177.4</v>
       </c>
-      <c r="J71" s="2">
+      <c r="J71" s="1">
         <v>46418</v>
       </c>
       <c r="K71" t="b">
@@ -3674,7 +3648,7 @@
       <c r="H72">
         <v>200</v>
       </c>
-      <c r="J72" s="2">
+      <c r="J72" s="1">
         <v>46356</v>
       </c>
       <c r="K72" t="b">
@@ -3706,7 +3680,7 @@
       <c r="H73">
         <v>203.6</v>
       </c>
-      <c r="J73" s="2">
+      <c r="J73" s="1">
         <v>46436</v>
       </c>
       <c r="K73" t="b">
@@ -3738,7 +3712,7 @@
       <c r="H74">
         <v>221.2</v>
       </c>
-      <c r="J74" s="2">
+      <c r="J74" s="1">
         <v>46426</v>
       </c>
       <c r="K74" t="b">
@@ -3770,7 +3744,7 @@
       <c r="H75">
         <v>240.8</v>
       </c>
-      <c r="J75" s="2">
+      <c r="J75" s="1">
         <v>46450</v>
       </c>
       <c r="K75" t="b">
@@ -3802,7 +3776,7 @@
       <c r="H76">
         <v>245.8</v>
       </c>
-      <c r="J76" s="2">
+      <c r="J76" s="1">
         <v>46452</v>
       </c>
       <c r="K76" t="b">
@@ -3834,7 +3808,7 @@
       <c r="H77">
         <v>263.4</v>
       </c>
-      <c r="J77" s="2">
+      <c r="J77" s="1">
         <v>46322</v>
       </c>
       <c r="K77" t="b">
@@ -3866,7 +3840,7 @@
       <c r="H78">
         <v>275.2</v>
       </c>
-      <c r="J78" s="2">
+      <c r="J78" s="1">
         <v>46433</v>
       </c>
       <c r="K78" t="b">
@@ -3901,7 +3875,7 @@
       <c r="I79" t="s">
         <v>311</v>
       </c>
-      <c r="J79" s="2">
+      <c r="J79" s="1">
         <v>36557</v>
       </c>
       <c r="K79" t="b">
@@ -3936,7 +3910,7 @@
       <c r="I80" t="s">
         <v>312</v>
       </c>
-      <c r="J80" s="2">
+      <c r="J80" s="1">
         <v>41275</v>
       </c>
       <c r="K80" t="b">
@@ -3971,7 +3945,7 @@
       <c r="I81" t="s">
         <v>313</v>
       </c>
-      <c r="J81" s="2">
+      <c r="J81" s="1">
         <v>45380</v>
       </c>
       <c r="K81" t="b">
@@ -4006,7 +3980,7 @@
       <c r="I82" t="s">
         <v>314</v>
       </c>
-      <c r="J82" s="2">
+      <c r="J82" s="1">
         <v>45421</v>
       </c>
       <c r="K82" t="b">
@@ -4041,7 +4015,7 @@
       <c r="I83" t="s">
         <v>314</v>
       </c>
-      <c r="J83" s="2">
+      <c r="J83" s="1">
         <v>45428</v>
       </c>
       <c r="K83" t="b">
@@ -4076,7 +4050,7 @@
       <c r="I84" t="s">
         <v>315</v>
       </c>
-      <c r="J84" s="2">
+      <c r="J84" s="1">
         <v>45490</v>
       </c>
       <c r="K84" t="b">
@@ -4111,7 +4085,7 @@
       <c r="I85" t="s">
         <v>316</v>
       </c>
-      <c r="J85" s="2">
+      <c r="J85" s="1">
         <v>45566</v>
       </c>
       <c r="K85" t="b">
@@ -4146,7 +4120,7 @@
       <c r="I86" t="s">
         <v>317</v>
       </c>
-      <c r="J86" s="2">
+      <c r="J86" s="1">
         <v>45986</v>
       </c>
       <c r="K86" t="b">
@@ -4181,7 +4155,7 @@
       <c r="I87" t="s">
         <v>318</v>
       </c>
-      <c r="J87" s="2">
+      <c r="J87" s="1">
         <v>46284</v>
       </c>
       <c r="K87" t="b">
@@ -4216,7 +4190,7 @@
       <c r="I88" t="s">
         <v>319</v>
       </c>
-      <c r="J88" s="2">
+      <c r="J88" s="1">
         <v>46305</v>
       </c>
       <c r="K88" t="b">
@@ -4251,7 +4225,7 @@
       <c r="I89" t="s">
         <v>319</v>
       </c>
-      <c r="J89" s="2">
+      <c r="J89" s="1">
         <v>46310</v>
       </c>
       <c r="K89" t="b">
@@ -4286,7 +4260,7 @@
       <c r="I90" t="s">
         <v>319</v>
       </c>
-      <c r="J90" s="2">
+      <c r="J90" s="1">
         <v>46317</v>
       </c>
       <c r="K90" t="b">
@@ -4321,7 +4295,7 @@
       <c r="I91" t="s">
         <v>319</v>
       </c>
-      <c r="J91" s="2">
+      <c r="J91" s="1">
         <v>46319</v>
       </c>
       <c r="K91" t="b">
@@ -4356,7 +4330,7 @@
       <c r="I92" t="s">
         <v>320</v>
       </c>
-      <c r="J92" s="2">
+      <c r="J92" s="1">
         <v>46333</v>
       </c>
       <c r="K92" t="b">
@@ -4391,7 +4365,7 @@
       <c r="I93" t="s">
         <v>320</v>
       </c>
-      <c r="J93" s="2">
+      <c r="J93" s="1">
         <v>46338</v>
       </c>
       <c r="K93" t="b">
@@ -4426,7 +4400,7 @@
       <c r="I94" t="s">
         <v>320</v>
       </c>
-      <c r="J94" s="2">
+      <c r="J94" s="1">
         <v>46338</v>
       </c>
       <c r="K94" t="b">
@@ -4461,7 +4435,7 @@
       <c r="I95" t="s">
         <v>320</v>
       </c>
-      <c r="J95" s="2">
+      <c r="J95" s="1">
         <v>46341</v>
       </c>
       <c r="K95" t="b">
@@ -4496,7 +4470,7 @@
       <c r="I96" t="s">
         <v>320</v>
       </c>
-      <c r="J96" s="2">
+      <c r="J96" s="1">
         <v>46344</v>
       </c>
       <c r="K96" t="b">
@@ -4531,7 +4505,7 @@
       <c r="I97" t="s">
         <v>321</v>
       </c>
-      <c r="J97" s="2">
+      <c r="J97" s="1">
         <v>46360</v>
       </c>
       <c r="K97" t="b">
@@ -4566,7 +4540,7 @@
       <c r="I98" t="s">
         <v>321</v>
       </c>
-      <c r="J98" s="2">
+      <c r="J98" s="1">
         <v>46360</v>
       </c>
       <c r="K98" t="b">
@@ -4601,7 +4575,7 @@
       <c r="I99" t="s">
         <v>321</v>
       </c>
-      <c r="J99" s="2">
+      <c r="J99" s="1">
         <v>46367</v>
       </c>
       <c r="K99" t="b">
@@ -4636,7 +4610,7 @@
       <c r="I100" t="s">
         <v>321</v>
       </c>
-      <c r="J100" s="2">
+      <c r="J100" s="1">
         <v>46375</v>
       </c>
       <c r="K100" t="b">
@@ -4671,7 +4645,7 @@
       <c r="I101" t="s">
         <v>321</v>
       </c>
-      <c r="J101" s="2">
+      <c r="J101" s="1">
         <v>46387</v>
       </c>
       <c r="K101" t="b">
@@ -4706,7 +4680,7 @@
       <c r="I102" t="s">
         <v>321</v>
       </c>
-      <c r="J102" s="2">
+      <c r="J102" s="1">
         <v>46387</v>
       </c>
       <c r="K102" t="b">
@@ -4741,7 +4715,7 @@
       <c r="I103" t="s">
         <v>321</v>
       </c>
-      <c r="J103" s="2">
+      <c r="J103" s="1">
         <v>46387</v>
       </c>
       <c r="K103" t="b">
@@ -4776,7 +4750,7 @@
       <c r="I104" t="s">
         <v>321</v>
       </c>
-      <c r="J104" s="2">
+      <c r="J104" s="1">
         <v>46388</v>
       </c>
       <c r="K104" t="b">
@@ -4811,7 +4785,7 @@
       <c r="I105" t="s">
         <v>322</v>
       </c>
-      <c r="J105" s="2">
+      <c r="J105" s="1">
         <v>46401</v>
       </c>
       <c r="K105" t="b">
@@ -4846,7 +4820,7 @@
       <c r="I106" t="s">
         <v>322</v>
       </c>
-      <c r="J106" s="2">
+      <c r="J106" s="1">
         <v>46401</v>
       </c>
       <c r="K106" t="b">
@@ -4881,7 +4855,7 @@
       <c r="I107" t="s">
         <v>322</v>
       </c>
-      <c r="J107" s="2">
+      <c r="J107" s="1">
         <v>46401</v>
       </c>
       <c r="K107" t="b">
@@ -4916,7 +4890,7 @@
       <c r="I108" t="s">
         <v>322</v>
       </c>
-      <c r="J108" s="2">
+      <c r="J108" s="1">
         <v>46412</v>
       </c>
       <c r="K108" t="b">
@@ -4951,7 +4925,7 @@
       <c r="I109" t="s">
         <v>322</v>
       </c>
-      <c r="J109" s="2">
+      <c r="J109" s="1">
         <v>46412</v>
       </c>
       <c r="K109" t="b">
@@ -4986,7 +4960,7 @@
       <c r="I110" t="s">
         <v>322</v>
       </c>
-      <c r="J110" s="2">
+      <c r="J110" s="1">
         <v>46412</v>
       </c>
       <c r="K110" t="b">
@@ -5021,7 +4995,7 @@
       <c r="I111" t="s">
         <v>323</v>
       </c>
-      <c r="J111" s="2">
+      <c r="J111" s="1">
         <v>46424</v>
       </c>
       <c r="K111" t="b">
@@ -5056,7 +5030,7 @@
       <c r="I112" t="s">
         <v>323</v>
       </c>
-      <c r="J112" s="2">
+      <c r="J112" s="1">
         <v>46437</v>
       </c>
       <c r="K112" t="b">
@@ -5091,7 +5065,7 @@
       <c r="I113" t="s">
         <v>323</v>
       </c>
-      <c r="J113" s="2">
+      <c r="J113" s="1">
         <v>46451</v>
       </c>
       <c r="K113" t="b">
@@ -5126,7 +5100,7 @@
       <c r="I114" t="s">
         <v>323</v>
       </c>
-      <c r="J114" s="2">
+      <c r="J114" s="1">
         <v>46451</v>
       </c>
       <c r="K114" t="b">
@@ -5161,7 +5135,7 @@
       <c r="I115" t="s">
         <v>324</v>
       </c>
-      <c r="J115" s="2">
+      <c r="J115" s="1">
         <v>46455</v>
       </c>
       <c r="K115" t="b">
@@ -5196,7 +5170,7 @@
       <c r="I116" t="s">
         <v>324</v>
       </c>
-      <c r="J116" s="2">
+      <c r="J116" s="1">
         <v>46456</v>
       </c>
       <c r="K116" t="b">
@@ -5231,7 +5205,7 @@
       <c r="I117" t="s">
         <v>324</v>
       </c>
-      <c r="J117" s="2">
+      <c r="J117" s="1">
         <v>46457</v>
       </c>
       <c r="K117" t="b">
@@ -5266,7 +5240,7 @@
       <c r="I118" t="s">
         <v>324</v>
       </c>
-      <c r="J118" s="2">
+      <c r="J118" s="1">
         <v>46464</v>
       </c>
       <c r="K118" t="b">
@@ -5301,7 +5275,7 @@
       <c r="I119" t="s">
         <v>324</v>
       </c>
-      <c r="J119" s="2">
+      <c r="J119" s="1">
         <v>46470</v>
       </c>
       <c r="K119" t="b">
@@ -5336,7 +5310,7 @@
       <c r="I120" t="s">
         <v>325</v>
       </c>
-      <c r="J120" s="2">
+      <c r="J120" s="1">
         <v>46485</v>
       </c>
       <c r="K120" t="b">
@@ -5371,7 +5345,7 @@
       <c r="I121" t="s">
         <v>325</v>
       </c>
-      <c r="J121" s="2">
+      <c r="J121" s="1">
         <v>46499</v>
       </c>
       <c r="K121" t="b">
@@ -5406,7 +5380,7 @@
       <c r="I122" t="s">
         <v>325</v>
       </c>
-      <c r="J122" s="2">
+      <c r="J122" s="1">
         <v>46504</v>
       </c>
       <c r="K122" t="b">
@@ -5441,7 +5415,7 @@
       <c r="I123" t="s">
         <v>325</v>
       </c>
-      <c r="J123" s="2">
+      <c r="J123" s="1">
         <v>46504</v>
       </c>
       <c r="K123" t="b">
@@ -5476,7 +5450,7 @@
       <c r="I124" t="s">
         <v>325</v>
       </c>
-      <c r="J124" s="2">
+      <c r="J124" s="1">
         <v>46507</v>
       </c>
       <c r="K124" t="b">
@@ -5511,7 +5485,7 @@
       <c r="I125" t="s">
         <v>325</v>
       </c>
-      <c r="J125" s="2">
+      <c r="J125" s="1">
         <v>46508</v>
       </c>
       <c r="K125" t="b">
@@ -5546,7 +5520,7 @@
       <c r="I126" t="s">
         <v>325</v>
       </c>
-      <c r="J126" s="2">
+      <c r="J126" s="1">
         <v>46512</v>
       </c>
       <c r="K126" t="b">
@@ -5581,7 +5555,7 @@
       <c r="I127" t="s">
         <v>326</v>
       </c>
-      <c r="J127" s="2">
+      <c r="J127" s="1">
         <v>46512</v>
       </c>
       <c r="K127" t="b">
@@ -5616,7 +5590,7 @@
       <c r="I128" t="s">
         <v>326</v>
       </c>
-      <c r="J128" s="2">
+      <c r="J128" s="1">
         <v>46528</v>
       </c>
       <c r="K128" t="b">
@@ -5651,7 +5625,7 @@
       <c r="I129" t="s">
         <v>326</v>
       </c>
-      <c r="J129" s="2">
+      <c r="J129" s="1">
         <v>46529</v>
       </c>
       <c r="K129" t="b">
@@ -5686,7 +5660,7 @@
       <c r="I130" t="s">
         <v>326</v>
       </c>
-      <c r="J130" s="2">
+      <c r="J130" s="1">
         <v>46537</v>
       </c>
       <c r="K130" t="b">
@@ -5721,7 +5695,7 @@
       <c r="I131" t="s">
         <v>327</v>
       </c>
-      <c r="J131" s="2">
+      <c r="J131" s="1">
         <v>46546</v>
       </c>
       <c r="K131" t="b">
@@ -5756,7 +5730,7 @@
       <c r="I132" t="s">
         <v>327</v>
       </c>
-      <c r="J132" s="2">
+      <c r="J132" s="1">
         <v>46547</v>
       </c>
       <c r="K132" t="b">
@@ -5791,7 +5765,7 @@
       <c r="I133" t="s">
         <v>327</v>
       </c>
-      <c r="J133" s="2">
+      <c r="J133" s="1">
         <v>46547</v>
       </c>
       <c r="K133" t="b">
@@ -5826,7 +5800,7 @@
       <c r="I134" t="s">
         <v>327</v>
       </c>
-      <c r="J134" s="2">
+      <c r="J134" s="1">
         <v>46547</v>
       </c>
       <c r="K134" t="b">
@@ -5861,7 +5835,7 @@
       <c r="I135" t="s">
         <v>327</v>
       </c>
-      <c r="J135" s="2">
+      <c r="J135" s="1">
         <v>46551</v>
       </c>
       <c r="K135" t="b">
@@ -5896,7 +5870,7 @@
       <c r="I136" t="s">
         <v>327</v>
       </c>
-      <c r="J136" s="2">
+      <c r="J136" s="1">
         <v>46560</v>
       </c>
       <c r="K136" t="b">
@@ -5931,7 +5905,7 @@
       <c r="I137" t="s">
         <v>327</v>
       </c>
-      <c r="J137" s="2">
+      <c r="J137" s="1">
         <v>46564</v>
       </c>
       <c r="K137" t="b">
@@ -5966,7 +5940,7 @@
       <c r="I138" t="s">
         <v>327</v>
       </c>
-      <c r="J138" s="2">
+      <c r="J138" s="1">
         <v>46567</v>
       </c>
       <c r="K138" t="b">
@@ -6001,7 +5975,7 @@
       <c r="I139" t="s">
         <v>327</v>
       </c>
-      <c r="J139" s="2">
+      <c r="J139" s="1">
         <v>46568</v>
       </c>
       <c r="K139" t="b">
@@ -6036,7 +6010,7 @@
       <c r="I140" t="s">
         <v>328</v>
       </c>
-      <c r="J140" s="2">
+      <c r="J140" s="1">
         <v>46578</v>
       </c>
       <c r="K140" t="b">
@@ -6071,7 +6045,7 @@
       <c r="I141" t="s">
         <v>328</v>
       </c>
-      <c r="J141" s="2">
+      <c r="J141" s="1">
         <v>46592</v>
       </c>
       <c r="K141" t="b">
@@ -6106,7 +6080,7 @@
       <c r="I142" t="s">
         <v>328</v>
       </c>
-      <c r="J142" s="2">
+      <c r="J142" s="1">
         <v>46592</v>
       </c>
       <c r="K142" t="b">
@@ -6141,7 +6115,7 @@
       <c r="I143" t="s">
         <v>329</v>
       </c>
-      <c r="J143" s="2">
+      <c r="J143" s="1">
         <v>46212</v>
       </c>
       <c r="K143" t="b">
@@ -6176,7 +6150,7 @@
       <c r="I144" t="s">
         <v>330</v>
       </c>
-      <c r="J144" s="2">
+      <c r="J144" s="1">
         <v>46225</v>
       </c>
       <c r="K144" t="b">
@@ -6211,7 +6185,7 @@
       <c r="I145" t="s">
         <v>331</v>
       </c>
-      <c r="J145" s="2">
+      <c r="J145" s="1">
         <v>46263</v>
       </c>
       <c r="K145" t="b">
@@ -6243,7 +6217,7 @@
       <c r="H146">
         <v>-1476</v>
       </c>
-      <c r="J146" s="2">
+      <c r="J146" s="1">
         <v>43773</v>
       </c>
       <c r="K146" t="b">
@@ -6275,7 +6249,7 @@
       <c r="H147">
         <v>-1469</v>
       </c>
-      <c r="J147" s="2">
+      <c r="J147" s="1">
         <v>43773</v>
       </c>
       <c r="K147" t="b">
@@ -6307,7 +6281,7 @@
       <c r="H148">
         <v>-1186</v>
       </c>
-      <c r="J148" s="2">
+      <c r="J148" s="1">
         <v>45295</v>
       </c>
       <c r="K148" t="b">
@@ -6339,7 +6313,7 @@
       <c r="H149">
         <v>-1048</v>
       </c>
-      <c r="J149" s="2">
+      <c r="J149" s="1">
         <v>45617</v>
       </c>
       <c r="K149" t="b">
@@ -6371,7 +6345,7 @@
       <c r="H150">
         <v>-980</v>
       </c>
-      <c r="J150" s="2">
+      <c r="J150" s="1">
         <v>45677</v>
       </c>
       <c r="K150" t="b">
@@ -6403,7 +6377,7 @@
       <c r="H151">
         <v>-961</v>
       </c>
-      <c r="J151" s="2">
+      <c r="J151" s="1">
         <v>44944</v>
       </c>
       <c r="K151" t="b">
@@ -6435,7 +6409,7 @@
       <c r="H152">
         <v>-252</v>
       </c>
-      <c r="J152" s="2">
+      <c r="J152" s="1">
         <v>46092</v>
       </c>
       <c r="K152" t="b">
@@ -6467,7 +6441,7 @@
       <c r="H153">
         <v>3</v>
       </c>
-      <c r="J153" s="2">
+      <c r="J153" s="1">
         <v>46265</v>
       </c>
       <c r="K153" t="b">
@@ -6499,7 +6473,7 @@
       <c r="H154">
         <v>3</v>
       </c>
-      <c r="J154" s="2">
+      <c r="J154" s="1">
         <v>46265</v>
       </c>
       <c r="K154" t="b">
@@ -6531,7 +6505,7 @@
       <c r="H155">
         <v>43</v>
       </c>
-      <c r="J155" s="2">
+      <c r="J155" s="1">
         <v>46440</v>
       </c>
       <c r="K155" t="b">
@@ -6563,7 +6537,7 @@
       <c r="H156">
         <v>43</v>
       </c>
-      <c r="J156" s="2">
+      <c r="J156" s="1">
         <v>46440</v>
       </c>
       <c r="K156" t="b">
@@ -6595,7 +6569,7 @@
       <c r="H157">
         <v>72</v>
       </c>
-      <c r="J157" s="2">
+      <c r="J157" s="1">
         <v>46289</v>
       </c>
       <c r="K157" t="b">
@@ -6627,7 +6601,7 @@
       <c r="H158">
         <v>72</v>
       </c>
-      <c r="J158" s="2">
+      <c r="J158" s="1">
         <v>46289</v>
       </c>
       <c r="K158" t="b">
@@ -6659,7 +6633,7 @@
       <c r="H159">
         <v>81</v>
       </c>
-      <c r="J159" s="2">
+      <c r="J159" s="1">
         <v>46405</v>
       </c>
       <c r="K159" t="b">
@@ -6691,7 +6665,7 @@
       <c r="H160">
         <v>102</v>
       </c>
-      <c r="J160" s="2">
+      <c r="J160" s="1">
         <v>46463</v>
       </c>
       <c r="K160" t="b">
@@ -6723,7 +6697,7 @@
       <c r="H161">
         <v>109</v>
       </c>
-      <c r="J161" s="2">
+      <c r="J161" s="1">
         <v>46353</v>
       </c>
       <c r="K161" t="b">
@@ -6755,7 +6729,7 @@
       <c r="H162">
         <v>127</v>
       </c>
-      <c r="J162" s="2">
+      <c r="J162" s="1">
         <v>46417</v>
       </c>
       <c r="K162" t="b">
@@ -6787,7 +6761,7 @@
       <c r="H163">
         <v>152</v>
       </c>
-      <c r="J163" s="2">
+      <c r="J163" s="1">
         <v>46271</v>
       </c>
       <c r="K163" t="b">
@@ -6819,7 +6793,7 @@
       <c r="H164">
         <v>152</v>
       </c>
-      <c r="J164" s="2">
+      <c r="J164" s="1">
         <v>46271</v>
       </c>
       <c r="K164" t="b">
@@ -6851,7 +6825,7 @@
       <c r="H165">
         <v>153</v>
       </c>
-      <c r="J165" s="2">
+      <c r="J165" s="1">
         <v>46458</v>
       </c>
       <c r="K165" t="b">
@@ -6883,7 +6857,7 @@
       <c r="H166">
         <v>158</v>
       </c>
-      <c r="J166" s="2">
+      <c r="J166" s="1">
         <v>46381</v>
       </c>
       <c r="K166" t="b">
@@ -6915,7 +6889,7 @@
       <c r="H167">
         <v>163</v>
       </c>
-      <c r="J167" s="2">
+      <c r="J167" s="1">
         <v>46592</v>
       </c>
       <c r="K167" t="b">
@@ -6947,7 +6921,7 @@
       <c r="H168">
         <v>167</v>
       </c>
-      <c r="J168" s="2">
+      <c r="J168" s="1">
         <v>46441</v>
       </c>
       <c r="K168" t="b">
@@ -6979,7 +6953,7 @@
       <c r="H169">
         <v>169</v>
       </c>
-      <c r="J169" s="2">
+      <c r="J169" s="1">
         <v>46391</v>
       </c>
       <c r="K169" t="b">
@@ -7011,7 +6985,7 @@
       <c r="H170">
         <v>184</v>
       </c>
-      <c r="J170" s="2">
+      <c r="J170" s="1">
         <v>46385</v>
       </c>
       <c r="K170" t="b">
@@ -7043,7 +7017,7 @@
       <c r="H171">
         <v>186</v>
       </c>
-      <c r="J171" s="2">
+      <c r="J171" s="1">
         <v>46387</v>
       </c>
       <c r="K171" t="b">
@@ -7075,7 +7049,7 @@
       <c r="H172">
         <v>206</v>
       </c>
-      <c r="J172" s="2">
+      <c r="J172" s="1">
         <v>46399</v>
       </c>
       <c r="K172" t="b">
@@ -7107,7 +7081,7 @@
       <c r="H173">
         <v>206</v>
       </c>
-      <c r="J173" s="2">
+      <c r="J173" s="1">
         <v>46399</v>
       </c>
       <c r="K173" t="b">
@@ -7139,7 +7113,7 @@
       <c r="H174">
         <v>234</v>
       </c>
-      <c r="J174" s="2">
+      <c r="J174" s="1">
         <v>46458</v>
       </c>
       <c r="K174" t="b">
@@ -7171,7 +7145,7 @@
       <c r="H175">
         <v>248</v>
       </c>
-      <c r="J175" s="2">
+      <c r="J175" s="1">
         <v>46528</v>
       </c>
       <c r="K175" t="b">
@@ -7203,7 +7177,7 @@
       <c r="H176">
         <v>317</v>
       </c>
-      <c r="J176" s="2">
+      <c r="J176" s="1">
         <v>46540</v>
       </c>
       <c r="K176" t="b">
@@ -7235,7 +7209,7 @@
       <c r="H177">
         <v>340</v>
       </c>
-      <c r="J177" s="2">
+      <c r="J177" s="1">
         <v>46547</v>
       </c>
       <c r="K177" t="b">
@@ -7267,7 +7241,7 @@
       <c r="H178">
         <v>364</v>
       </c>
-      <c r="J178" s="2">
+      <c r="J178" s="1">
         <v>46557</v>
       </c>
       <c r="K178" t="b">
@@ -7299,7 +7273,7 @@
       <c r="H179">
         <v>368</v>
       </c>
-      <c r="J179" s="2">
+      <c r="J179" s="1">
         <v>46571</v>
       </c>
       <c r="K179" t="b">
@@ -7331,7 +7305,7 @@
       <c r="H180">
         <v>368</v>
       </c>
-      <c r="J180" s="2">
+      <c r="J180" s="1">
         <v>46571</v>
       </c>
       <c r="K180" t="b">
@@ -7363,7 +7337,7 @@
       <c r="H181">
         <v>370</v>
       </c>
-      <c r="J181" s="2">
+      <c r="J181" s="1">
         <v>46562</v>
       </c>
       <c r="K181" t="b">
@@ -7395,7 +7369,7 @@
       <c r="H182">
         <v>385</v>
       </c>
-      <c r="J182" s="2">
+      <c r="J182" s="1">
         <v>46574</v>
       </c>
       <c r="K182" t="b">
@@ -7427,7 +7401,7 @@
       <c r="H183">
         <v>385</v>
       </c>
-      <c r="J183" s="2">
+      <c r="J183" s="1">
         <v>46574</v>
       </c>
       <c r="K183" t="b">
@@ -7459,7 +7433,7 @@
       <c r="H184">
         <v>417</v>
       </c>
-      <c r="J184" s="2">
+      <c r="J184" s="1">
         <v>46578</v>
       </c>
       <c r="K184" t="b">
@@ -7491,7 +7465,7 @@
       <c r="H185">
         <v>721</v>
       </c>
-      <c r="J185" s="2">
+      <c r="J185" s="1">
         <v>46345</v>
       </c>
       <c r="K185" t="b">
@@ -7523,7 +7497,7 @@
       <c r="H186">
         <v>721</v>
       </c>
-      <c r="J186" s="2">
+      <c r="J186" s="1">
         <v>46345</v>
       </c>
       <c r="K186" t="b">
@@ -7555,7 +7529,7 @@
       <c r="H187">
         <v>850</v>
       </c>
-      <c r="J187" s="2">
+      <c r="J187" s="1">
         <v>46366</v>
       </c>
       <c r="K187" t="b">
@@ -7587,7 +7561,7 @@
       <c r="H188">
         <v>850</v>
       </c>
-      <c r="J188" s="2">
+      <c r="J188" s="1">
         <v>46366</v>
       </c>
       <c r="K188" t="b">
@@ -7619,7 +7593,7 @@
       <c r="H189">
         <v>1661</v>
       </c>
-      <c r="J189" s="2">
+      <c r="J189" s="1">
         <v>46524</v>
       </c>
       <c r="K189" t="b">
@@ -7651,7 +7625,7 @@
       <c r="H190">
         <v>1661</v>
       </c>
-      <c r="J190" s="2">
+      <c r="J190" s="1">
         <v>46524</v>
       </c>
       <c r="K190" t="b">
@@ -7683,7 +7657,7 @@
       <c r="H191">
         <v>488</v>
       </c>
-      <c r="J191" s="2">
+      <c r="J191" s="1">
         <v>46190</v>
       </c>
       <c r="K191" t="b">
@@ -7715,7 +7689,7 @@
       <c r="H192">
         <v>25565</v>
       </c>
-      <c r="J192" s="2">
+      <c r="J192" s="1">
         <v>46190</v>
       </c>
       <c r="K192" t="b">
@@ -7747,7 +7721,7 @@
       <c r="H193">
         <v>25567</v>
       </c>
-      <c r="J193" s="2">
+      <c r="J193" s="1">
         <v>46190</v>
       </c>
       <c r="K193" t="b">
@@ -7779,7 +7753,7 @@
       <c r="H194">
         <v>31293</v>
       </c>
-      <c r="J194" s="2">
+      <c r="J194" s="1">
         <v>46190</v>
       </c>
       <c r="K194" t="b">

</xml_diff>

<commit_message>
Atualização automática: vencimentos_tmot (02/09/2026 09:38)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
@@ -1019,8 +1019,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1036,7 +1044,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1044,12 +1052,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1349,37 +1375,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1408,7 +1434,7 @@
       <c r="H2">
         <v>-4300.3</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>39285</v>
       </c>
       <c r="K2" t="b">
@@ -1440,7 +1466,7 @@
       <c r="H3">
         <v>-2354.2</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>40669</v>
       </c>
       <c r="K3" t="b">
@@ -1472,7 +1498,7 @@
       <c r="H4">
         <v>-910.7</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>40669</v>
       </c>
       <c r="K4" t="b">
@@ -1504,7 +1530,7 @@
       <c r="H5">
         <v>-868</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>44884</v>
       </c>
       <c r="K5" t="b">
@@ -1536,7 +1562,7 @@
       <c r="H6">
         <v>-483.8</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>43855</v>
       </c>
       <c r="K6" t="b">
@@ -1568,7 +1594,7 @@
       <c r="H7">
         <v>-417</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>46014</v>
       </c>
       <c r="K7" t="b">
@@ -1600,7 +1626,7 @@
       <c r="H8">
         <v>-414.2</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>46014</v>
       </c>
       <c r="K8" t="b">
@@ -1632,7 +1658,7 @@
       <c r="H9">
         <v>-391.8</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>42769</v>
       </c>
       <c r="K9" t="b">
@@ -1664,7 +1690,7 @@
       <c r="H10">
         <v>-391.6</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>45804</v>
       </c>
       <c r="K10" t="b">
@@ -1696,7 +1722,7 @@
       <c r="H11">
         <v>-391.6</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>45804</v>
       </c>
       <c r="K11" t="b">
@@ -1728,7 +1754,7 @@
       <c r="H12">
         <v>-372.9</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>42821</v>
       </c>
       <c r="K12" t="b">
@@ -1760,7 +1786,7 @@
       <c r="H13">
         <v>-372.9</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>46014</v>
       </c>
       <c r="K13" t="b">
@@ -1792,7 +1818,7 @@
       <c r="H14">
         <v>-372.9</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>46014</v>
       </c>
       <c r="K14" t="b">
@@ -1824,7 +1850,7 @@
       <c r="H15">
         <v>-372.9</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>46014</v>
       </c>
       <c r="K15" t="b">
@@ -1856,7 +1882,7 @@
       <c r="H16">
         <v>-367.8</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="2">
         <v>46017</v>
       </c>
       <c r="K16" t="b">
@@ -1888,7 +1914,7 @@
       <c r="H17">
         <v>-367.8</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="2">
         <v>46017</v>
       </c>
       <c r="K17" t="b">
@@ -1920,7 +1946,7 @@
       <c r="H18">
         <v>-347.2</v>
       </c>
-      <c r="J18" s="1">
+      <c r="J18" s="2">
         <v>40979</v>
       </c>
       <c r="K18" t="b">
@@ -1952,7 +1978,7 @@
       <c r="H19">
         <v>-293.8</v>
       </c>
-      <c r="J19" s="1">
+      <c r="J19" s="2">
         <v>45846</v>
       </c>
       <c r="K19" t="b">
@@ -1984,7 +2010,7 @@
       <c r="H20">
         <v>-206.4</v>
       </c>
-      <c r="J20" s="1">
+      <c r="J20" s="2">
         <v>36669</v>
       </c>
       <c r="K20" t="b">
@@ -2016,7 +2042,7 @@
       <c r="H21">
         <v>-131.6</v>
       </c>
-      <c r="J21" s="1">
+      <c r="J21" s="2">
         <v>46111</v>
       </c>
       <c r="K21" t="b">
@@ -2048,7 +2074,7 @@
       <c r="H22">
         <v>-131.6</v>
       </c>
-      <c r="J22" s="1">
+      <c r="J22" s="2">
         <v>46111</v>
       </c>
       <c r="K22" t="b">
@@ -2080,7 +2106,7 @@
       <c r="H23">
         <v>-131.6</v>
       </c>
-      <c r="J23" s="1">
+      <c r="J23" s="2">
         <v>46111</v>
       </c>
       <c r="K23" t="b">
@@ -2112,7 +2138,7 @@
       <c r="H24">
         <v>-131.6</v>
       </c>
-      <c r="J24" s="1">
+      <c r="J24" s="2">
         <v>46111</v>
       </c>
       <c r="K24" t="b">
@@ -2144,7 +2170,7 @@
       <c r="H25">
         <v>-131.6</v>
       </c>
-      <c r="J25" s="1">
+      <c r="J25" s="2">
         <v>46111</v>
       </c>
       <c r="K25" t="b">
@@ -2176,7 +2202,7 @@
       <c r="H26">
         <v>-98.3</v>
       </c>
-      <c r="J26" s="1">
+      <c r="J26" s="2">
         <v>41204</v>
       </c>
       <c r="K26" t="b">
@@ -2208,7 +2234,7 @@
       <c r="H27">
         <v>-47.2</v>
       </c>
-      <c r="J27" s="1">
+      <c r="J27" s="2">
         <v>44011</v>
       </c>
       <c r="K27" t="b">
@@ -2240,7 +2266,7 @@
       <c r="H28">
         <v>-22.3</v>
       </c>
-      <c r="J28" s="1">
+      <c r="J28" s="2">
         <v>46226</v>
       </c>
       <c r="K28" t="b">
@@ -2272,7 +2298,7 @@
       <c r="H29">
         <v>4.7</v>
       </c>
-      <c r="J29" s="1">
+      <c r="J29" s="2">
         <v>46265</v>
       </c>
       <c r="K29" t="b">
@@ -2304,7 +2330,7 @@
       <c r="H30">
         <v>7.5</v>
       </c>
-      <c r="J30" s="1">
+      <c r="J30" s="2">
         <v>46265</v>
       </c>
       <c r="K30" t="b">
@@ -2336,7 +2362,7 @@
       <c r="H31">
         <v>10</v>
       </c>
-      <c r="J31" s="1">
+      <c r="J31" s="2">
         <v>46265</v>
       </c>
       <c r="K31" t="b">
@@ -2368,7 +2394,7 @@
       <c r="H32">
         <v>12.8</v>
       </c>
-      <c r="J32" s="1">
+      <c r="J32" s="2">
         <v>46265</v>
       </c>
       <c r="K32" t="b">
@@ -2400,7 +2426,7 @@
       <c r="H33">
         <v>14</v>
       </c>
-      <c r="J33" s="1">
+      <c r="J33" s="2">
         <v>46265</v>
       </c>
       <c r="K33" t="b">
@@ -2432,7 +2458,7 @@
       <c r="H34">
         <v>17.8</v>
       </c>
-      <c r="J34" s="1">
+      <c r="J34" s="2">
         <v>46265</v>
       </c>
       <c r="K34" t="b">
@@ -2464,7 +2490,7 @@
       <c r="H35">
         <v>20.4</v>
       </c>
-      <c r="J35" s="1">
+      <c r="J35" s="2">
         <v>46265</v>
       </c>
       <c r="K35" t="b">
@@ -2496,7 +2522,7 @@
       <c r="H36">
         <v>21.2</v>
       </c>
-      <c r="J36" s="1">
+      <c r="J36" s="2">
         <v>46265</v>
       </c>
       <c r="K36" t="b">
@@ -2528,7 +2554,7 @@
       <c r="H37">
         <v>26.2</v>
       </c>
-      <c r="J37" s="1">
+      <c r="J37" s="2">
         <v>46265</v>
       </c>
       <c r="K37" t="b">
@@ -2560,7 +2586,7 @@
       <c r="H38">
         <v>33.6</v>
       </c>
-      <c r="J38" s="1">
+      <c r="J38" s="2">
         <v>46364</v>
       </c>
       <c r="K38" t="b">
@@ -2592,7 +2618,7 @@
       <c r="H39">
         <v>42.2</v>
       </c>
-      <c r="J39" s="1">
+      <c r="J39" s="2">
         <v>46269</v>
       </c>
       <c r="K39" t="b">
@@ -2624,7 +2650,7 @@
       <c r="H40">
         <v>42.8</v>
       </c>
-      <c r="J40" s="1">
+      <c r="J40" s="2">
         <v>46291</v>
       </c>
       <c r="K40" t="b">
@@ -2656,7 +2682,7 @@
       <c r="H41">
         <v>45.7</v>
       </c>
-      <c r="J41" s="1">
+      <c r="J41" s="2">
         <v>46395</v>
       </c>
       <c r="K41" t="b">
@@ -2688,7 +2714,7 @@
       <c r="H42">
         <v>47.2</v>
       </c>
-      <c r="J42" s="1">
+      <c r="J42" s="2">
         <v>46280</v>
       </c>
       <c r="K42" t="b">
@@ -2720,7 +2746,7 @@
       <c r="H43">
         <v>48.7</v>
       </c>
-      <c r="J43" s="1">
+      <c r="J43" s="2">
         <v>46281</v>
       </c>
       <c r="K43" t="b">
@@ -2752,7 +2778,7 @@
       <c r="H44">
         <v>60</v>
       </c>
-      <c r="J44" s="1">
+      <c r="J44" s="2">
         <v>46281</v>
       </c>
       <c r="K44" t="b">
@@ -2784,7 +2810,7 @@
       <c r="H45">
         <v>62.6</v>
       </c>
-      <c r="J45" s="1">
+      <c r="J45" s="2">
         <v>46265</v>
       </c>
       <c r="K45" t="b">
@@ -2816,7 +2842,7 @@
       <c r="H46">
         <v>64.59999999999999</v>
       </c>
-      <c r="J46" s="1">
+      <c r="J46" s="2">
         <v>46265</v>
       </c>
       <c r="K46" t="b">
@@ -2848,7 +2874,7 @@
       <c r="H47">
         <v>67.59999999999999</v>
       </c>
-      <c r="J47" s="1">
+      <c r="J47" s="2">
         <v>46267</v>
       </c>
       <c r="K47" t="b">
@@ -2880,7 +2906,7 @@
       <c r="H48">
         <v>68.3</v>
       </c>
-      <c r="J48" s="1">
+      <c r="J48" s="2">
         <v>46278</v>
       </c>
       <c r="K48" t="b">
@@ -2912,7 +2938,7 @@
       <c r="H49">
         <v>69.2</v>
       </c>
-      <c r="J49" s="1">
+      <c r="J49" s="2">
         <v>46453</v>
       </c>
       <c r="K49" t="b">
@@ -2944,7 +2970,7 @@
       <c r="H50">
         <v>69.8</v>
       </c>
-      <c r="J50" s="1">
+      <c r="J50" s="2">
         <v>46265</v>
       </c>
       <c r="K50" t="b">
@@ -2976,7 +3002,7 @@
       <c r="H51">
         <v>69.8</v>
       </c>
-      <c r="J51" s="1">
+      <c r="J51" s="2">
         <v>46265</v>
       </c>
       <c r="K51" t="b">
@@ -3008,7 +3034,7 @@
       <c r="H52">
         <v>72.2</v>
       </c>
-      <c r="J52" s="1">
+      <c r="J52" s="2">
         <v>46275</v>
       </c>
       <c r="K52" t="b">
@@ -3040,7 +3066,7 @@
       <c r="H53">
         <v>72.2</v>
       </c>
-      <c r="J53" s="1">
+      <c r="J53" s="2">
         <v>46275</v>
       </c>
       <c r="K53" t="b">
@@ -3072,7 +3098,7 @@
       <c r="H54">
         <v>78.09999999999999</v>
       </c>
-      <c r="J54" s="1">
+      <c r="J54" s="2">
         <v>46265</v>
       </c>
       <c r="K54" t="b">
@@ -3104,7 +3130,7 @@
       <c r="H55">
         <v>82.8</v>
       </c>
-      <c r="J55" s="1">
+      <c r="J55" s="2">
         <v>46487</v>
       </c>
       <c r="K55" t="b">
@@ -3136,7 +3162,7 @@
       <c r="H56">
         <v>83.09999999999999</v>
       </c>
-      <c r="J56" s="1">
+      <c r="J56" s="2">
         <v>46285</v>
       </c>
       <c r="K56" t="b">
@@ -3168,7 +3194,7 @@
       <c r="H57">
         <v>84.8</v>
       </c>
-      <c r="J57" s="1">
+      <c r="J57" s="2">
         <v>46492</v>
       </c>
       <c r="K57" t="b">
@@ -3200,7 +3226,7 @@
       <c r="H58">
         <v>104.9</v>
       </c>
-      <c r="J58" s="1">
+      <c r="J58" s="2">
         <v>46297</v>
       </c>
       <c r="K58" t="b">
@@ -3232,7 +3258,7 @@
       <c r="H59">
         <v>107.6</v>
       </c>
-      <c r="J59" s="1">
+      <c r="J59" s="2">
         <v>46283</v>
       </c>
       <c r="K59" t="b">
@@ -3264,7 +3290,7 @@
       <c r="H60">
         <v>111.9</v>
       </c>
-      <c r="J60" s="1">
+      <c r="J60" s="2">
         <v>46300</v>
       </c>
       <c r="K60" t="b">
@@ -3296,7 +3322,7 @@
       <c r="H61">
         <v>111.9</v>
       </c>
-      <c r="J61" s="1">
+      <c r="J61" s="2">
         <v>46300</v>
       </c>
       <c r="K61" t="b">
@@ -3328,7 +3354,7 @@
       <c r="H62">
         <v>111.9</v>
       </c>
-      <c r="J62" s="1">
+      <c r="J62" s="2">
         <v>46300</v>
       </c>
       <c r="K62" t="b">
@@ -3360,7 +3386,7 @@
       <c r="H63">
         <v>111.9</v>
       </c>
-      <c r="J63" s="1">
+      <c r="J63" s="2">
         <v>46300</v>
       </c>
       <c r="K63" t="b">
@@ -3392,7 +3418,7 @@
       <c r="H64">
         <v>111.9</v>
       </c>
-      <c r="J64" s="1">
+      <c r="J64" s="2">
         <v>46300</v>
       </c>
       <c r="K64" t="b">
@@ -3424,7 +3450,7 @@
       <c r="H65">
         <v>128.8</v>
       </c>
-      <c r="J65" s="1">
+      <c r="J65" s="2">
         <v>46308</v>
       </c>
       <c r="K65" t="b">
@@ -3456,7 +3482,7 @@
       <c r="H66">
         <v>131.1</v>
       </c>
-      <c r="J66" s="1">
+      <c r="J66" s="2">
         <v>46336</v>
       </c>
       <c r="K66" t="b">
@@ -3488,7 +3514,7 @@
       <c r="H67">
         <v>138.4</v>
       </c>
-      <c r="J67" s="1">
+      <c r="J67" s="2">
         <v>46343</v>
       </c>
       <c r="K67" t="b">
@@ -3520,7 +3546,7 @@
       <c r="H68">
         <v>141</v>
       </c>
-      <c r="J68" s="1">
+      <c r="J68" s="2">
         <v>46350</v>
       </c>
       <c r="K68" t="b">
@@ -3552,7 +3578,7 @@
       <c r="H69">
         <v>162</v>
       </c>
-      <c r="J69" s="1">
+      <c r="J69" s="2">
         <v>46391</v>
       </c>
       <c r="K69" t="b">
@@ -3584,7 +3610,7 @@
       <c r="H70">
         <v>167.2</v>
       </c>
-      <c r="J70" s="1">
+      <c r="J70" s="2">
         <v>46330</v>
       </c>
       <c r="K70" t="b">
@@ -3616,7 +3642,7 @@
       <c r="H71">
         <v>177.4</v>
       </c>
-      <c r="J71" s="1">
+      <c r="J71" s="2">
         <v>46418</v>
       </c>
       <c r="K71" t="b">
@@ -3648,7 +3674,7 @@
       <c r="H72">
         <v>200</v>
       </c>
-      <c r="J72" s="1">
+      <c r="J72" s="2">
         <v>46356</v>
       </c>
       <c r="K72" t="b">
@@ -3680,7 +3706,7 @@
       <c r="H73">
         <v>203.6</v>
       </c>
-      <c r="J73" s="1">
+      <c r="J73" s="2">
         <v>46436</v>
       </c>
       <c r="K73" t="b">
@@ -3712,7 +3738,7 @@
       <c r="H74">
         <v>221.2</v>
       </c>
-      <c r="J74" s="1">
+      <c r="J74" s="2">
         <v>46426</v>
       </c>
       <c r="K74" t="b">
@@ -3744,7 +3770,7 @@
       <c r="H75">
         <v>240.8</v>
       </c>
-      <c r="J75" s="1">
+      <c r="J75" s="2">
         <v>46450</v>
       </c>
       <c r="K75" t="b">
@@ -3776,7 +3802,7 @@
       <c r="H76">
         <v>245.8</v>
       </c>
-      <c r="J76" s="1">
+      <c r="J76" s="2">
         <v>46452</v>
       </c>
       <c r="K76" t="b">
@@ -3808,7 +3834,7 @@
       <c r="H77">
         <v>263.4</v>
       </c>
-      <c r="J77" s="1">
+      <c r="J77" s="2">
         <v>46322</v>
       </c>
       <c r="K77" t="b">
@@ -3840,7 +3866,7 @@
       <c r="H78">
         <v>275.2</v>
       </c>
-      <c r="J78" s="1">
+      <c r="J78" s="2">
         <v>46433</v>
       </c>
       <c r="K78" t="b">
@@ -3875,7 +3901,7 @@
       <c r="I79" t="s">
         <v>311</v>
       </c>
-      <c r="J79" s="1">
+      <c r="J79" s="2">
         <v>36557</v>
       </c>
       <c r="K79" t="b">
@@ -3910,7 +3936,7 @@
       <c r="I80" t="s">
         <v>312</v>
       </c>
-      <c r="J80" s="1">
+      <c r="J80" s="2">
         <v>41275</v>
       </c>
       <c r="K80" t="b">
@@ -3945,7 +3971,7 @@
       <c r="I81" t="s">
         <v>313</v>
       </c>
-      <c r="J81" s="1">
+      <c r="J81" s="2">
         <v>45380</v>
       </c>
       <c r="K81" t="b">
@@ -3980,7 +4006,7 @@
       <c r="I82" t="s">
         <v>314</v>
       </c>
-      <c r="J82" s="1">
+      <c r="J82" s="2">
         <v>45421</v>
       </c>
       <c r="K82" t="b">
@@ -4015,7 +4041,7 @@
       <c r="I83" t="s">
         <v>314</v>
       </c>
-      <c r="J83" s="1">
+      <c r="J83" s="2">
         <v>45428</v>
       </c>
       <c r="K83" t="b">
@@ -4050,7 +4076,7 @@
       <c r="I84" t="s">
         <v>315</v>
       </c>
-      <c r="J84" s="1">
+      <c r="J84" s="2">
         <v>45490</v>
       </c>
       <c r="K84" t="b">
@@ -4085,7 +4111,7 @@
       <c r="I85" t="s">
         <v>316</v>
       </c>
-      <c r="J85" s="1">
+      <c r="J85" s="2">
         <v>45566</v>
       </c>
       <c r="K85" t="b">
@@ -4120,7 +4146,7 @@
       <c r="I86" t="s">
         <v>317</v>
       </c>
-      <c r="J86" s="1">
+      <c r="J86" s="2">
         <v>45986</v>
       </c>
       <c r="K86" t="b">
@@ -4155,7 +4181,7 @@
       <c r="I87" t="s">
         <v>318</v>
       </c>
-      <c r="J87" s="1">
+      <c r="J87" s="2">
         <v>46284</v>
       </c>
       <c r="K87" t="b">
@@ -4190,7 +4216,7 @@
       <c r="I88" t="s">
         <v>319</v>
       </c>
-      <c r="J88" s="1">
+      <c r="J88" s="2">
         <v>46305</v>
       </c>
       <c r="K88" t="b">
@@ -4225,7 +4251,7 @@
       <c r="I89" t="s">
         <v>319</v>
       </c>
-      <c r="J89" s="1">
+      <c r="J89" s="2">
         <v>46310</v>
       </c>
       <c r="K89" t="b">
@@ -4260,7 +4286,7 @@
       <c r="I90" t="s">
         <v>319</v>
       </c>
-      <c r="J90" s="1">
+      <c r="J90" s="2">
         <v>46317</v>
       </c>
       <c r="K90" t="b">
@@ -4295,7 +4321,7 @@
       <c r="I91" t="s">
         <v>319</v>
       </c>
-      <c r="J91" s="1">
+      <c r="J91" s="2">
         <v>46319</v>
       </c>
       <c r="K91" t="b">
@@ -4330,7 +4356,7 @@
       <c r="I92" t="s">
         <v>320</v>
       </c>
-      <c r="J92" s="1">
+      <c r="J92" s="2">
         <v>46333</v>
       </c>
       <c r="K92" t="b">
@@ -4365,7 +4391,7 @@
       <c r="I93" t="s">
         <v>320</v>
       </c>
-      <c r="J93" s="1">
+      <c r="J93" s="2">
         <v>46338</v>
       </c>
       <c r="K93" t="b">
@@ -4400,7 +4426,7 @@
       <c r="I94" t="s">
         <v>320</v>
       </c>
-      <c r="J94" s="1">
+      <c r="J94" s="2">
         <v>46338</v>
       </c>
       <c r="K94" t="b">
@@ -4435,7 +4461,7 @@
       <c r="I95" t="s">
         <v>320</v>
       </c>
-      <c r="J95" s="1">
+      <c r="J95" s="2">
         <v>46341</v>
       </c>
       <c r="K95" t="b">
@@ -4470,7 +4496,7 @@
       <c r="I96" t="s">
         <v>320</v>
       </c>
-      <c r="J96" s="1">
+      <c r="J96" s="2">
         <v>46344</v>
       </c>
       <c r="K96" t="b">
@@ -4505,7 +4531,7 @@
       <c r="I97" t="s">
         <v>321</v>
       </c>
-      <c r="J97" s="1">
+      <c r="J97" s="2">
         <v>46360</v>
       </c>
       <c r="K97" t="b">
@@ -4540,7 +4566,7 @@
       <c r="I98" t="s">
         <v>321</v>
       </c>
-      <c r="J98" s="1">
+      <c r="J98" s="2">
         <v>46360</v>
       </c>
       <c r="K98" t="b">
@@ -4575,7 +4601,7 @@
       <c r="I99" t="s">
         <v>321</v>
       </c>
-      <c r="J99" s="1">
+      <c r="J99" s="2">
         <v>46367</v>
       </c>
       <c r="K99" t="b">
@@ -4610,7 +4636,7 @@
       <c r="I100" t="s">
         <v>321</v>
       </c>
-      <c r="J100" s="1">
+      <c r="J100" s="2">
         <v>46375</v>
       </c>
       <c r="K100" t="b">
@@ -4645,7 +4671,7 @@
       <c r="I101" t="s">
         <v>321</v>
       </c>
-      <c r="J101" s="1">
+      <c r="J101" s="2">
         <v>46387</v>
       </c>
       <c r="K101" t="b">
@@ -4680,7 +4706,7 @@
       <c r="I102" t="s">
         <v>321</v>
       </c>
-      <c r="J102" s="1">
+      <c r="J102" s="2">
         <v>46387</v>
       </c>
       <c r="K102" t="b">
@@ -4715,7 +4741,7 @@
       <c r="I103" t="s">
         <v>321</v>
       </c>
-      <c r="J103" s="1">
+      <c r="J103" s="2">
         <v>46387</v>
       </c>
       <c r="K103" t="b">
@@ -4750,7 +4776,7 @@
       <c r="I104" t="s">
         <v>321</v>
       </c>
-      <c r="J104" s="1">
+      <c r="J104" s="2">
         <v>46388</v>
       </c>
       <c r="K104" t="b">
@@ -4785,7 +4811,7 @@
       <c r="I105" t="s">
         <v>322</v>
       </c>
-      <c r="J105" s="1">
+      <c r="J105" s="2">
         <v>46401</v>
       </c>
       <c r="K105" t="b">
@@ -4820,7 +4846,7 @@
       <c r="I106" t="s">
         <v>322</v>
       </c>
-      <c r="J106" s="1">
+      <c r="J106" s="2">
         <v>46401</v>
       </c>
       <c r="K106" t="b">
@@ -4855,7 +4881,7 @@
       <c r="I107" t="s">
         <v>322</v>
       </c>
-      <c r="J107" s="1">
+      <c r="J107" s="2">
         <v>46401</v>
       </c>
       <c r="K107" t="b">
@@ -4890,7 +4916,7 @@
       <c r="I108" t="s">
         <v>322</v>
       </c>
-      <c r="J108" s="1">
+      <c r="J108" s="2">
         <v>46412</v>
       </c>
       <c r="K108" t="b">
@@ -4925,7 +4951,7 @@
       <c r="I109" t="s">
         <v>322</v>
       </c>
-      <c r="J109" s="1">
+      <c r="J109" s="2">
         <v>46412</v>
       </c>
       <c r="K109" t="b">
@@ -4960,7 +4986,7 @@
       <c r="I110" t="s">
         <v>322</v>
       </c>
-      <c r="J110" s="1">
+      <c r="J110" s="2">
         <v>46412</v>
       </c>
       <c r="K110" t="b">
@@ -4995,7 +5021,7 @@
       <c r="I111" t="s">
         <v>323</v>
       </c>
-      <c r="J111" s="1">
+      <c r="J111" s="2">
         <v>46424</v>
       </c>
       <c r="K111" t="b">
@@ -5030,7 +5056,7 @@
       <c r="I112" t="s">
         <v>323</v>
       </c>
-      <c r="J112" s="1">
+      <c r="J112" s="2">
         <v>46437</v>
       </c>
       <c r="K112" t="b">
@@ -5065,7 +5091,7 @@
       <c r="I113" t="s">
         <v>323</v>
       </c>
-      <c r="J113" s="1">
+      <c r="J113" s="2">
         <v>46451</v>
       </c>
       <c r="K113" t="b">
@@ -5100,7 +5126,7 @@
       <c r="I114" t="s">
         <v>323</v>
       </c>
-      <c r="J114" s="1">
+      <c r="J114" s="2">
         <v>46451</v>
       </c>
       <c r="K114" t="b">
@@ -5135,7 +5161,7 @@
       <c r="I115" t="s">
         <v>324</v>
       </c>
-      <c r="J115" s="1">
+      <c r="J115" s="2">
         <v>46455</v>
       </c>
       <c r="K115" t="b">
@@ -5170,7 +5196,7 @@
       <c r="I116" t="s">
         <v>324</v>
       </c>
-      <c r="J116" s="1">
+      <c r="J116" s="2">
         <v>46456</v>
       </c>
       <c r="K116" t="b">
@@ -5205,7 +5231,7 @@
       <c r="I117" t="s">
         <v>324</v>
       </c>
-      <c r="J117" s="1">
+      <c r="J117" s="2">
         <v>46457</v>
       </c>
       <c r="K117" t="b">
@@ -5240,7 +5266,7 @@
       <c r="I118" t="s">
         <v>324</v>
       </c>
-      <c r="J118" s="1">
+      <c r="J118" s="2">
         <v>46464</v>
       </c>
       <c r="K118" t="b">
@@ -5275,7 +5301,7 @@
       <c r="I119" t="s">
         <v>324</v>
       </c>
-      <c r="J119" s="1">
+      <c r="J119" s="2">
         <v>46470</v>
       </c>
       <c r="K119" t="b">
@@ -5310,7 +5336,7 @@
       <c r="I120" t="s">
         <v>325</v>
       </c>
-      <c r="J120" s="1">
+      <c r="J120" s="2">
         <v>46485</v>
       </c>
       <c r="K120" t="b">
@@ -5345,7 +5371,7 @@
       <c r="I121" t="s">
         <v>325</v>
       </c>
-      <c r="J121" s="1">
+      <c r="J121" s="2">
         <v>46499</v>
       </c>
       <c r="K121" t="b">
@@ -5380,7 +5406,7 @@
       <c r="I122" t="s">
         <v>325</v>
       </c>
-      <c r="J122" s="1">
+      <c r="J122" s="2">
         <v>46504</v>
       </c>
       <c r="K122" t="b">
@@ -5415,7 +5441,7 @@
       <c r="I123" t="s">
         <v>325</v>
       </c>
-      <c r="J123" s="1">
+      <c r="J123" s="2">
         <v>46504</v>
       </c>
       <c r="K123" t="b">
@@ -5450,7 +5476,7 @@
       <c r="I124" t="s">
         <v>325</v>
       </c>
-      <c r="J124" s="1">
+      <c r="J124" s="2">
         <v>46507</v>
       </c>
       <c r="K124" t="b">
@@ -5485,7 +5511,7 @@
       <c r="I125" t="s">
         <v>325</v>
       </c>
-      <c r="J125" s="1">
+      <c r="J125" s="2">
         <v>46508</v>
       </c>
       <c r="K125" t="b">
@@ -5520,7 +5546,7 @@
       <c r="I126" t="s">
         <v>325</v>
       </c>
-      <c r="J126" s="1">
+      <c r="J126" s="2">
         <v>46512</v>
       </c>
       <c r="K126" t="b">
@@ -5555,7 +5581,7 @@
       <c r="I127" t="s">
         <v>326</v>
       </c>
-      <c r="J127" s="1">
+      <c r="J127" s="2">
         <v>46512</v>
       </c>
       <c r="K127" t="b">
@@ -5590,7 +5616,7 @@
       <c r="I128" t="s">
         <v>326</v>
       </c>
-      <c r="J128" s="1">
+      <c r="J128" s="2">
         <v>46528</v>
       </c>
       <c r="K128" t="b">
@@ -5625,7 +5651,7 @@
       <c r="I129" t="s">
         <v>326</v>
       </c>
-      <c r="J129" s="1">
+      <c r="J129" s="2">
         <v>46529</v>
       </c>
       <c r="K129" t="b">
@@ -5660,7 +5686,7 @@
       <c r="I130" t="s">
         <v>326</v>
       </c>
-      <c r="J130" s="1">
+      <c r="J130" s="2">
         <v>46537</v>
       </c>
       <c r="K130" t="b">
@@ -5695,7 +5721,7 @@
       <c r="I131" t="s">
         <v>327</v>
       </c>
-      <c r="J131" s="1">
+      <c r="J131" s="2">
         <v>46546</v>
       </c>
       <c r="K131" t="b">
@@ -5730,7 +5756,7 @@
       <c r="I132" t="s">
         <v>327</v>
       </c>
-      <c r="J132" s="1">
+      <c r="J132" s="2">
         <v>46547</v>
       </c>
       <c r="K132" t="b">
@@ -5765,7 +5791,7 @@
       <c r="I133" t="s">
         <v>327</v>
       </c>
-      <c r="J133" s="1">
+      <c r="J133" s="2">
         <v>46547</v>
       </c>
       <c r="K133" t="b">
@@ -5800,7 +5826,7 @@
       <c r="I134" t="s">
         <v>327</v>
       </c>
-      <c r="J134" s="1">
+      <c r="J134" s="2">
         <v>46547</v>
       </c>
       <c r="K134" t="b">
@@ -5835,7 +5861,7 @@
       <c r="I135" t="s">
         <v>327</v>
       </c>
-      <c r="J135" s="1">
+      <c r="J135" s="2">
         <v>46551</v>
       </c>
       <c r="K135" t="b">
@@ -5870,7 +5896,7 @@
       <c r="I136" t="s">
         <v>327</v>
       </c>
-      <c r="J136" s="1">
+      <c r="J136" s="2">
         <v>46560</v>
       </c>
       <c r="K136" t="b">
@@ -5905,7 +5931,7 @@
       <c r="I137" t="s">
         <v>327</v>
       </c>
-      <c r="J137" s="1">
+      <c r="J137" s="2">
         <v>46564</v>
       </c>
       <c r="K137" t="b">
@@ -5940,7 +5966,7 @@
       <c r="I138" t="s">
         <v>327</v>
       </c>
-      <c r="J138" s="1">
+      <c r="J138" s="2">
         <v>46567</v>
       </c>
       <c r="K138" t="b">
@@ -5975,7 +6001,7 @@
       <c r="I139" t="s">
         <v>327</v>
       </c>
-      <c r="J139" s="1">
+      <c r="J139" s="2">
         <v>46568</v>
       </c>
       <c r="K139" t="b">
@@ -6010,7 +6036,7 @@
       <c r="I140" t="s">
         <v>328</v>
       </c>
-      <c r="J140" s="1">
+      <c r="J140" s="2">
         <v>46578</v>
       </c>
       <c r="K140" t="b">
@@ -6045,7 +6071,7 @@
       <c r="I141" t="s">
         <v>328</v>
       </c>
-      <c r="J141" s="1">
+      <c r="J141" s="2">
         <v>46592</v>
       </c>
       <c r="K141" t="b">
@@ -6080,7 +6106,7 @@
       <c r="I142" t="s">
         <v>328</v>
       </c>
-      <c r="J142" s="1">
+      <c r="J142" s="2">
         <v>46592</v>
       </c>
       <c r="K142" t="b">
@@ -6115,7 +6141,7 @@
       <c r="I143" t="s">
         <v>329</v>
       </c>
-      <c r="J143" s="1">
+      <c r="J143" s="2">
         <v>46212</v>
       </c>
       <c r="K143" t="b">
@@ -6150,7 +6176,7 @@
       <c r="I144" t="s">
         <v>330</v>
       </c>
-      <c r="J144" s="1">
+      <c r="J144" s="2">
         <v>46225</v>
       </c>
       <c r="K144" t="b">
@@ -6185,7 +6211,7 @@
       <c r="I145" t="s">
         <v>331</v>
       </c>
-      <c r="J145" s="1">
+      <c r="J145" s="2">
         <v>46263</v>
       </c>
       <c r="K145" t="b">
@@ -6217,7 +6243,7 @@
       <c r="H146">
         <v>-1476</v>
       </c>
-      <c r="J146" s="1">
+      <c r="J146" s="2">
         <v>43773</v>
       </c>
       <c r="K146" t="b">
@@ -6249,7 +6275,7 @@
       <c r="H147">
         <v>-1469</v>
       </c>
-      <c r="J147" s="1">
+      <c r="J147" s="2">
         <v>43773</v>
       </c>
       <c r="K147" t="b">
@@ -6281,7 +6307,7 @@
       <c r="H148">
         <v>-1186</v>
       </c>
-      <c r="J148" s="1">
+      <c r="J148" s="2">
         <v>45295</v>
       </c>
       <c r="K148" t="b">
@@ -6313,7 +6339,7 @@
       <c r="H149">
         <v>-1048</v>
       </c>
-      <c r="J149" s="1">
+      <c r="J149" s="2">
         <v>45617</v>
       </c>
       <c r="K149" t="b">
@@ -6345,7 +6371,7 @@
       <c r="H150">
         <v>-980</v>
       </c>
-      <c r="J150" s="1">
+      <c r="J150" s="2">
         <v>45677</v>
       </c>
       <c r="K150" t="b">
@@ -6377,7 +6403,7 @@
       <c r="H151">
         <v>-961</v>
       </c>
-      <c r="J151" s="1">
+      <c r="J151" s="2">
         <v>44944</v>
       </c>
       <c r="K151" t="b">
@@ -6409,7 +6435,7 @@
       <c r="H152">
         <v>-252</v>
       </c>
-      <c r="J152" s="1">
+      <c r="J152" s="2">
         <v>46092</v>
       </c>
       <c r="K152" t="b">
@@ -6441,7 +6467,7 @@
       <c r="H153">
         <v>3</v>
       </c>
-      <c r="J153" s="1">
+      <c r="J153" s="2">
         <v>46265</v>
       </c>
       <c r="K153" t="b">
@@ -6473,7 +6499,7 @@
       <c r="H154">
         <v>3</v>
       </c>
-      <c r="J154" s="1">
+      <c r="J154" s="2">
         <v>46265</v>
       </c>
       <c r="K154" t="b">
@@ -6505,7 +6531,7 @@
       <c r="H155">
         <v>43</v>
       </c>
-      <c r="J155" s="1">
+      <c r="J155" s="2">
         <v>46440</v>
       </c>
       <c r="K155" t="b">
@@ -6537,7 +6563,7 @@
       <c r="H156">
         <v>43</v>
       </c>
-      <c r="J156" s="1">
+      <c r="J156" s="2">
         <v>46440</v>
       </c>
       <c r="K156" t="b">
@@ -6569,7 +6595,7 @@
       <c r="H157">
         <v>72</v>
       </c>
-      <c r="J157" s="1">
+      <c r="J157" s="2">
         <v>46289</v>
       </c>
       <c r="K157" t="b">
@@ -6601,7 +6627,7 @@
       <c r="H158">
         <v>72</v>
       </c>
-      <c r="J158" s="1">
+      <c r="J158" s="2">
         <v>46289</v>
       </c>
       <c r="K158" t="b">
@@ -6633,7 +6659,7 @@
       <c r="H159">
         <v>81</v>
       </c>
-      <c r="J159" s="1">
+      <c r="J159" s="2">
         <v>46405</v>
       </c>
       <c r="K159" t="b">
@@ -6665,7 +6691,7 @@
       <c r="H160">
         <v>102</v>
       </c>
-      <c r="J160" s="1">
+      <c r="J160" s="2">
         <v>46463</v>
       </c>
       <c r="K160" t="b">
@@ -6697,7 +6723,7 @@
       <c r="H161">
         <v>109</v>
       </c>
-      <c r="J161" s="1">
+      <c r="J161" s="2">
         <v>46353</v>
       </c>
       <c r="K161" t="b">
@@ -6729,7 +6755,7 @@
       <c r="H162">
         <v>127</v>
       </c>
-      <c r="J162" s="1">
+      <c r="J162" s="2">
         <v>46417</v>
       </c>
       <c r="K162" t="b">
@@ -6761,7 +6787,7 @@
       <c r="H163">
         <v>152</v>
       </c>
-      <c r="J163" s="1">
+      <c r="J163" s="2">
         <v>46271</v>
       </c>
       <c r="K163" t="b">
@@ -6793,7 +6819,7 @@
       <c r="H164">
         <v>152</v>
       </c>
-      <c r="J164" s="1">
+      <c r="J164" s="2">
         <v>46271</v>
       </c>
       <c r="K164" t="b">
@@ -6825,7 +6851,7 @@
       <c r="H165">
         <v>153</v>
       </c>
-      <c r="J165" s="1">
+      <c r="J165" s="2">
         <v>46458</v>
       </c>
       <c r="K165" t="b">
@@ -6857,7 +6883,7 @@
       <c r="H166">
         <v>158</v>
       </c>
-      <c r="J166" s="1">
+      <c r="J166" s="2">
         <v>46381</v>
       </c>
       <c r="K166" t="b">
@@ -6889,7 +6915,7 @@
       <c r="H167">
         <v>163</v>
       </c>
-      <c r="J167" s="1">
+      <c r="J167" s="2">
         <v>46592</v>
       </c>
       <c r="K167" t="b">
@@ -6921,7 +6947,7 @@
       <c r="H168">
         <v>167</v>
       </c>
-      <c r="J168" s="1">
+      <c r="J168" s="2">
         <v>46441</v>
       </c>
       <c r="K168" t="b">
@@ -6953,7 +6979,7 @@
       <c r="H169">
         <v>169</v>
       </c>
-      <c r="J169" s="1">
+      <c r="J169" s="2">
         <v>46391</v>
       </c>
       <c r="K169" t="b">
@@ -6985,7 +7011,7 @@
       <c r="H170">
         <v>184</v>
       </c>
-      <c r="J170" s="1">
+      <c r="J170" s="2">
         <v>46385</v>
       </c>
       <c r="K170" t="b">
@@ -7017,7 +7043,7 @@
       <c r="H171">
         <v>186</v>
       </c>
-      <c r="J171" s="1">
+      <c r="J171" s="2">
         <v>46387</v>
       </c>
       <c r="K171" t="b">
@@ -7049,7 +7075,7 @@
       <c r="H172">
         <v>206</v>
       </c>
-      <c r="J172" s="1">
+      <c r="J172" s="2">
         <v>46399</v>
       </c>
       <c r="K172" t="b">
@@ -7081,7 +7107,7 @@
       <c r="H173">
         <v>206</v>
       </c>
-      <c r="J173" s="1">
+      <c r="J173" s="2">
         <v>46399</v>
       </c>
       <c r="K173" t="b">
@@ -7113,7 +7139,7 @@
       <c r="H174">
         <v>234</v>
       </c>
-      <c r="J174" s="1">
+      <c r="J174" s="2">
         <v>46458</v>
       </c>
       <c r="K174" t="b">
@@ -7145,7 +7171,7 @@
       <c r="H175">
         <v>248</v>
       </c>
-      <c r="J175" s="1">
+      <c r="J175" s="2">
         <v>46528</v>
       </c>
       <c r="K175" t="b">
@@ -7177,7 +7203,7 @@
       <c r="H176">
         <v>317</v>
       </c>
-      <c r="J176" s="1">
+      <c r="J176" s="2">
         <v>46540</v>
       </c>
       <c r="K176" t="b">
@@ -7209,7 +7235,7 @@
       <c r="H177">
         <v>340</v>
       </c>
-      <c r="J177" s="1">
+      <c r="J177" s="2">
         <v>46547</v>
       </c>
       <c r="K177" t="b">
@@ -7241,7 +7267,7 @@
       <c r="H178">
         <v>364</v>
       </c>
-      <c r="J178" s="1">
+      <c r="J178" s="2">
         <v>46557</v>
       </c>
       <c r="K178" t="b">
@@ -7273,7 +7299,7 @@
       <c r="H179">
         <v>368</v>
       </c>
-      <c r="J179" s="1">
+      <c r="J179" s="2">
         <v>46571</v>
       </c>
       <c r="K179" t="b">
@@ -7305,7 +7331,7 @@
       <c r="H180">
         <v>368</v>
       </c>
-      <c r="J180" s="1">
+      <c r="J180" s="2">
         <v>46571</v>
       </c>
       <c r="K180" t="b">
@@ -7337,7 +7363,7 @@
       <c r="H181">
         <v>370</v>
       </c>
-      <c r="J181" s="1">
+      <c r="J181" s="2">
         <v>46562</v>
       </c>
       <c r="K181" t="b">
@@ -7369,7 +7395,7 @@
       <c r="H182">
         <v>385</v>
       </c>
-      <c r="J182" s="1">
+      <c r="J182" s="2">
         <v>46574</v>
       </c>
       <c r="K182" t="b">
@@ -7401,7 +7427,7 @@
       <c r="H183">
         <v>385</v>
       </c>
-      <c r="J183" s="1">
+      <c r="J183" s="2">
         <v>46574</v>
       </c>
       <c r="K183" t="b">
@@ -7433,7 +7459,7 @@
       <c r="H184">
         <v>417</v>
       </c>
-      <c r="J184" s="1">
+      <c r="J184" s="2">
         <v>46578</v>
       </c>
       <c r="K184" t="b">
@@ -7465,7 +7491,7 @@
       <c r="H185">
         <v>721</v>
       </c>
-      <c r="J185" s="1">
+      <c r="J185" s="2">
         <v>46345</v>
       </c>
       <c r="K185" t="b">
@@ -7497,7 +7523,7 @@
       <c r="H186">
         <v>721</v>
       </c>
-      <c r="J186" s="1">
+      <c r="J186" s="2">
         <v>46345</v>
       </c>
       <c r="K186" t="b">
@@ -7529,7 +7555,7 @@
       <c r="H187">
         <v>850</v>
       </c>
-      <c r="J187" s="1">
+      <c r="J187" s="2">
         <v>46366</v>
       </c>
       <c r="K187" t="b">
@@ -7561,7 +7587,7 @@
       <c r="H188">
         <v>850</v>
       </c>
-      <c r="J188" s="1">
+      <c r="J188" s="2">
         <v>46366</v>
       </c>
       <c r="K188" t="b">
@@ -7593,7 +7619,7 @@
       <c r="H189">
         <v>1661</v>
       </c>
-      <c r="J189" s="1">
+      <c r="J189" s="2">
         <v>46524</v>
       </c>
       <c r="K189" t="b">
@@ -7625,7 +7651,7 @@
       <c r="H190">
         <v>1661</v>
       </c>
-      <c r="J190" s="1">
+      <c r="J190" s="2">
         <v>46524</v>
       </c>
       <c r="K190" t="b">
@@ -7657,7 +7683,7 @@
       <c r="H191">
         <v>488</v>
       </c>
-      <c r="J191" s="1">
+      <c r="J191" s="2">
         <v>46190</v>
       </c>
       <c r="K191" t="b">
@@ -7689,7 +7715,7 @@
       <c r="H192">
         <v>25565</v>
       </c>
-      <c r="J192" s="1">
+      <c r="J192" s="2">
         <v>46190</v>
       </c>
       <c r="K192" t="b">
@@ -7721,7 +7747,7 @@
       <c r="H193">
         <v>25567</v>
       </c>
-      <c r="J193" s="1">
+      <c r="J193" s="2">
         <v>46190</v>
       </c>
       <c r="K193" t="b">
@@ -7753,7 +7779,7 @@
       <c r="H194">
         <v>31293</v>
       </c>
-      <c r="J194" s="1">
+      <c r="J194" s="2">
         <v>46190</v>
       </c>
       <c r="K194" t="b">

</xml_diff>

<commit_message>
Atualização automática: vencimentos_tmot (02/09/2026 12:04)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
@@ -1019,16 +1019,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1044,7 +1036,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1052,30 +1044,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1375,37 +1349,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1434,7 +1408,7 @@
       <c r="H2">
         <v>-4300.3</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>39285</v>
       </c>
       <c r="K2" t="b">
@@ -1466,7 +1440,7 @@
       <c r="H3">
         <v>-2354.2</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>40669</v>
       </c>
       <c r="K3" t="b">
@@ -1498,7 +1472,7 @@
       <c r="H4">
         <v>-910.7</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>40669</v>
       </c>
       <c r="K4" t="b">
@@ -1530,7 +1504,7 @@
       <c r="H5">
         <v>-868</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>44884</v>
       </c>
       <c r="K5" t="b">
@@ -1562,7 +1536,7 @@
       <c r="H6">
         <v>-483.8</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>43855</v>
       </c>
       <c r="K6" t="b">
@@ -1594,7 +1568,7 @@
       <c r="H7">
         <v>-417</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>46014</v>
       </c>
       <c r="K7" t="b">
@@ -1626,7 +1600,7 @@
       <c r="H8">
         <v>-414.2</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>46014</v>
       </c>
       <c r="K8" t="b">
@@ -1658,7 +1632,7 @@
       <c r="H9">
         <v>-391.8</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>42769</v>
       </c>
       <c r="K9" t="b">
@@ -1690,7 +1664,7 @@
       <c r="H10">
         <v>-391.6</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>45804</v>
       </c>
       <c r="K10" t="b">
@@ -1722,7 +1696,7 @@
       <c r="H11">
         <v>-391.6</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>45804</v>
       </c>
       <c r="K11" t="b">
@@ -1754,7 +1728,7 @@
       <c r="H12">
         <v>-372.9</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>42821</v>
       </c>
       <c r="K12" t="b">
@@ -1786,7 +1760,7 @@
       <c r="H13">
         <v>-372.9</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>46014</v>
       </c>
       <c r="K13" t="b">
@@ -1818,7 +1792,7 @@
       <c r="H14">
         <v>-372.9</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>46014</v>
       </c>
       <c r="K14" t="b">
@@ -1850,7 +1824,7 @@
       <c r="H15">
         <v>-372.9</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <v>46014</v>
       </c>
       <c r="K15" t="b">
@@ -1882,7 +1856,7 @@
       <c r="H16">
         <v>-367.8</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <v>46017</v>
       </c>
       <c r="K16" t="b">
@@ -1914,7 +1888,7 @@
       <c r="H17">
         <v>-367.8</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="1">
         <v>46017</v>
       </c>
       <c r="K17" t="b">
@@ -1946,7 +1920,7 @@
       <c r="H18">
         <v>-347.2</v>
       </c>
-      <c r="J18" s="2">
+      <c r="J18" s="1">
         <v>40979</v>
       </c>
       <c r="K18" t="b">
@@ -1978,7 +1952,7 @@
       <c r="H19">
         <v>-293.8</v>
       </c>
-      <c r="J19" s="2">
+      <c r="J19" s="1">
         <v>45846</v>
       </c>
       <c r="K19" t="b">
@@ -2010,7 +1984,7 @@
       <c r="H20">
         <v>-206.4</v>
       </c>
-      <c r="J20" s="2">
+      <c r="J20" s="1">
         <v>36669</v>
       </c>
       <c r="K20" t="b">
@@ -2042,7 +2016,7 @@
       <c r="H21">
         <v>-131.6</v>
       </c>
-      <c r="J21" s="2">
+      <c r="J21" s="1">
         <v>46111</v>
       </c>
       <c r="K21" t="b">
@@ -2074,7 +2048,7 @@
       <c r="H22">
         <v>-131.6</v>
       </c>
-      <c r="J22" s="2">
+      <c r="J22" s="1">
         <v>46111</v>
       </c>
       <c r="K22" t="b">
@@ -2106,7 +2080,7 @@
       <c r="H23">
         <v>-131.6</v>
       </c>
-      <c r="J23" s="2">
+      <c r="J23" s="1">
         <v>46111</v>
       </c>
       <c r="K23" t="b">
@@ -2138,7 +2112,7 @@
       <c r="H24">
         <v>-131.6</v>
       </c>
-      <c r="J24" s="2">
+      <c r="J24" s="1">
         <v>46111</v>
       </c>
       <c r="K24" t="b">
@@ -2170,7 +2144,7 @@
       <c r="H25">
         <v>-131.6</v>
       </c>
-      <c r="J25" s="2">
+      <c r="J25" s="1">
         <v>46111</v>
       </c>
       <c r="K25" t="b">
@@ -2202,7 +2176,7 @@
       <c r="H26">
         <v>-98.3</v>
       </c>
-      <c r="J26" s="2">
+      <c r="J26" s="1">
         <v>41204</v>
       </c>
       <c r="K26" t="b">
@@ -2234,7 +2208,7 @@
       <c r="H27">
         <v>-47.2</v>
       </c>
-      <c r="J27" s="2">
+      <c r="J27" s="1">
         <v>44011</v>
       </c>
       <c r="K27" t="b">
@@ -2266,7 +2240,7 @@
       <c r="H28">
         <v>-22.3</v>
       </c>
-      <c r="J28" s="2">
+      <c r="J28" s="1">
         <v>46226</v>
       </c>
       <c r="K28" t="b">
@@ -2298,7 +2272,7 @@
       <c r="H29">
         <v>4.7</v>
       </c>
-      <c r="J29" s="2">
+      <c r="J29" s="1">
         <v>46265</v>
       </c>
       <c r="K29" t="b">
@@ -2330,7 +2304,7 @@
       <c r="H30">
         <v>7.5</v>
       </c>
-      <c r="J30" s="2">
+      <c r="J30" s="1">
         <v>46265</v>
       </c>
       <c r="K30" t="b">
@@ -2362,7 +2336,7 @@
       <c r="H31">
         <v>10</v>
       </c>
-      <c r="J31" s="2">
+      <c r="J31" s="1">
         <v>46265</v>
       </c>
       <c r="K31" t="b">
@@ -2394,7 +2368,7 @@
       <c r="H32">
         <v>12.8</v>
       </c>
-      <c r="J32" s="2">
+      <c r="J32" s="1">
         <v>46265</v>
       </c>
       <c r="K32" t="b">
@@ -2426,7 +2400,7 @@
       <c r="H33">
         <v>14</v>
       </c>
-      <c r="J33" s="2">
+      <c r="J33" s="1">
         <v>46265</v>
       </c>
       <c r="K33" t="b">
@@ -2458,7 +2432,7 @@
       <c r="H34">
         <v>17.8</v>
       </c>
-      <c r="J34" s="2">
+      <c r="J34" s="1">
         <v>46265</v>
       </c>
       <c r="K34" t="b">
@@ -2490,7 +2464,7 @@
       <c r="H35">
         <v>20.4</v>
       </c>
-      <c r="J35" s="2">
+      <c r="J35" s="1">
         <v>46265</v>
       </c>
       <c r="K35" t="b">
@@ -2522,7 +2496,7 @@
       <c r="H36">
         <v>21.2</v>
       </c>
-      <c r="J36" s="2">
+      <c r="J36" s="1">
         <v>46265</v>
       </c>
       <c r="K36" t="b">
@@ -2554,7 +2528,7 @@
       <c r="H37">
         <v>26.2</v>
       </c>
-      <c r="J37" s="2">
+      <c r="J37" s="1">
         <v>46265</v>
       </c>
       <c r="K37" t="b">
@@ -2586,7 +2560,7 @@
       <c r="H38">
         <v>33.6</v>
       </c>
-      <c r="J38" s="2">
+      <c r="J38" s="1">
         <v>46364</v>
       </c>
       <c r="K38" t="b">
@@ -2618,7 +2592,7 @@
       <c r="H39">
         <v>42.2</v>
       </c>
-      <c r="J39" s="2">
+      <c r="J39" s="1">
         <v>46269</v>
       </c>
       <c r="K39" t="b">
@@ -2650,7 +2624,7 @@
       <c r="H40">
         <v>42.8</v>
       </c>
-      <c r="J40" s="2">
+      <c r="J40" s="1">
         <v>46291</v>
       </c>
       <c r="K40" t="b">
@@ -2682,7 +2656,7 @@
       <c r="H41">
         <v>45.7</v>
       </c>
-      <c r="J41" s="2">
+      <c r="J41" s="1">
         <v>46395</v>
       </c>
       <c r="K41" t="b">
@@ -2714,7 +2688,7 @@
       <c r="H42">
         <v>47.2</v>
       </c>
-      <c r="J42" s="2">
+      <c r="J42" s="1">
         <v>46280</v>
       </c>
       <c r="K42" t="b">
@@ -2746,7 +2720,7 @@
       <c r="H43">
         <v>48.7</v>
       </c>
-      <c r="J43" s="2">
+      <c r="J43" s="1">
         <v>46281</v>
       </c>
       <c r="K43" t="b">
@@ -2778,7 +2752,7 @@
       <c r="H44">
         <v>60</v>
       </c>
-      <c r="J44" s="2">
+      <c r="J44" s="1">
         <v>46281</v>
       </c>
       <c r="K44" t="b">
@@ -2810,7 +2784,7 @@
       <c r="H45">
         <v>62.6</v>
       </c>
-      <c r="J45" s="2">
+      <c r="J45" s="1">
         <v>46265</v>
       </c>
       <c r="K45" t="b">
@@ -2842,7 +2816,7 @@
       <c r="H46">
         <v>64.59999999999999</v>
       </c>
-      <c r="J46" s="2">
+      <c r="J46" s="1">
         <v>46265</v>
       </c>
       <c r="K46" t="b">
@@ -2874,7 +2848,7 @@
       <c r="H47">
         <v>67.59999999999999</v>
       </c>
-      <c r="J47" s="2">
+      <c r="J47" s="1">
         <v>46267</v>
       </c>
       <c r="K47" t="b">
@@ -2906,7 +2880,7 @@
       <c r="H48">
         <v>68.3</v>
       </c>
-      <c r="J48" s="2">
+      <c r="J48" s="1">
         <v>46278</v>
       </c>
       <c r="K48" t="b">
@@ -2938,7 +2912,7 @@
       <c r="H49">
         <v>69.2</v>
       </c>
-      <c r="J49" s="2">
+      <c r="J49" s="1">
         <v>46453</v>
       </c>
       <c r="K49" t="b">
@@ -2970,7 +2944,7 @@
       <c r="H50">
         <v>69.8</v>
       </c>
-      <c r="J50" s="2">
+      <c r="J50" s="1">
         <v>46265</v>
       </c>
       <c r="K50" t="b">
@@ -3002,7 +2976,7 @@
       <c r="H51">
         <v>69.8</v>
       </c>
-      <c r="J51" s="2">
+      <c r="J51" s="1">
         <v>46265</v>
       </c>
       <c r="K51" t="b">
@@ -3034,7 +3008,7 @@
       <c r="H52">
         <v>72.2</v>
       </c>
-      <c r="J52" s="2">
+      <c r="J52" s="1">
         <v>46275</v>
       </c>
       <c r="K52" t="b">
@@ -3066,7 +3040,7 @@
       <c r="H53">
         <v>72.2</v>
       </c>
-      <c r="J53" s="2">
+      <c r="J53" s="1">
         <v>46275</v>
       </c>
       <c r="K53" t="b">
@@ -3098,7 +3072,7 @@
       <c r="H54">
         <v>78.09999999999999</v>
       </c>
-      <c r="J54" s="2">
+      <c r="J54" s="1">
         <v>46265</v>
       </c>
       <c r="K54" t="b">
@@ -3130,7 +3104,7 @@
       <c r="H55">
         <v>82.8</v>
       </c>
-      <c r="J55" s="2">
+      <c r="J55" s="1">
         <v>46487</v>
       </c>
       <c r="K55" t="b">
@@ -3162,7 +3136,7 @@
       <c r="H56">
         <v>83.09999999999999</v>
       </c>
-      <c r="J56" s="2">
+      <c r="J56" s="1">
         <v>46285</v>
       </c>
       <c r="K56" t="b">
@@ -3194,7 +3168,7 @@
       <c r="H57">
         <v>84.8</v>
       </c>
-      <c r="J57" s="2">
+      <c r="J57" s="1">
         <v>46492</v>
       </c>
       <c r="K57" t="b">
@@ -3226,7 +3200,7 @@
       <c r="H58">
         <v>104.9</v>
       </c>
-      <c r="J58" s="2">
+      <c r="J58" s="1">
         <v>46297</v>
       </c>
       <c r="K58" t="b">
@@ -3258,7 +3232,7 @@
       <c r="H59">
         <v>107.6</v>
       </c>
-      <c r="J59" s="2">
+      <c r="J59" s="1">
         <v>46283</v>
       </c>
       <c r="K59" t="b">
@@ -3290,7 +3264,7 @@
       <c r="H60">
         <v>111.9</v>
       </c>
-      <c r="J60" s="2">
+      <c r="J60" s="1">
         <v>46300</v>
       </c>
       <c r="K60" t="b">
@@ -3322,7 +3296,7 @@
       <c r="H61">
         <v>111.9</v>
       </c>
-      <c r="J61" s="2">
+      <c r="J61" s="1">
         <v>46300</v>
       </c>
       <c r="K61" t="b">
@@ -3354,7 +3328,7 @@
       <c r="H62">
         <v>111.9</v>
       </c>
-      <c r="J62" s="2">
+      <c r="J62" s="1">
         <v>46300</v>
       </c>
       <c r="K62" t="b">
@@ -3386,7 +3360,7 @@
       <c r="H63">
         <v>111.9</v>
       </c>
-      <c r="J63" s="2">
+      <c r="J63" s="1">
         <v>46300</v>
       </c>
       <c r="K63" t="b">
@@ -3418,7 +3392,7 @@
       <c r="H64">
         <v>111.9</v>
       </c>
-      <c r="J64" s="2">
+      <c r="J64" s="1">
         <v>46300</v>
       </c>
       <c r="K64" t="b">
@@ -3450,7 +3424,7 @@
       <c r="H65">
         <v>128.8</v>
       </c>
-      <c r="J65" s="2">
+      <c r="J65" s="1">
         <v>46308</v>
       </c>
       <c r="K65" t="b">
@@ -3482,7 +3456,7 @@
       <c r="H66">
         <v>131.1</v>
       </c>
-      <c r="J66" s="2">
+      <c r="J66" s="1">
         <v>46336</v>
       </c>
       <c r="K66" t="b">
@@ -3514,7 +3488,7 @@
       <c r="H67">
         <v>138.4</v>
       </c>
-      <c r="J67" s="2">
+      <c r="J67" s="1">
         <v>46343</v>
       </c>
       <c r="K67" t="b">
@@ -3546,7 +3520,7 @@
       <c r="H68">
         <v>141</v>
       </c>
-      <c r="J68" s="2">
+      <c r="J68" s="1">
         <v>46350</v>
       </c>
       <c r="K68" t="b">
@@ -3578,7 +3552,7 @@
       <c r="H69">
         <v>162</v>
       </c>
-      <c r="J69" s="2">
+      <c r="J69" s="1">
         <v>46391</v>
       </c>
       <c r="K69" t="b">
@@ -3610,7 +3584,7 @@
       <c r="H70">
         <v>167.2</v>
       </c>
-      <c r="J70" s="2">
+      <c r="J70" s="1">
         <v>46330</v>
       </c>
       <c r="K70" t="b">
@@ -3642,7 +3616,7 @@
       <c r="H71">
         <v>177.4</v>
       </c>
-      <c r="J71" s="2">
+      <c r="J71" s="1">
         <v>46418</v>
       </c>
       <c r="K71" t="b">
@@ -3674,7 +3648,7 @@
       <c r="H72">
         <v>200</v>
       </c>
-      <c r="J72" s="2">
+      <c r="J72" s="1">
         <v>46356</v>
       </c>
       <c r="K72" t="b">
@@ -3706,7 +3680,7 @@
       <c r="H73">
         <v>203.6</v>
       </c>
-      <c r="J73" s="2">
+      <c r="J73" s="1">
         <v>46436</v>
       </c>
       <c r="K73" t="b">
@@ -3738,7 +3712,7 @@
       <c r="H74">
         <v>221.2</v>
       </c>
-      <c r="J74" s="2">
+      <c r="J74" s="1">
         <v>46426</v>
       </c>
       <c r="K74" t="b">
@@ -3770,7 +3744,7 @@
       <c r="H75">
         <v>240.8</v>
       </c>
-      <c r="J75" s="2">
+      <c r="J75" s="1">
         <v>46450</v>
       </c>
       <c r="K75" t="b">
@@ -3802,7 +3776,7 @@
       <c r="H76">
         <v>245.8</v>
       </c>
-      <c r="J76" s="2">
+      <c r="J76" s="1">
         <v>46452</v>
       </c>
       <c r="K76" t="b">
@@ -3834,7 +3808,7 @@
       <c r="H77">
         <v>263.4</v>
       </c>
-      <c r="J77" s="2">
+      <c r="J77" s="1">
         <v>46322</v>
       </c>
       <c r="K77" t="b">
@@ -3866,7 +3840,7 @@
       <c r="H78">
         <v>275.2</v>
       </c>
-      <c r="J78" s="2">
+      <c r="J78" s="1">
         <v>46433</v>
       </c>
       <c r="K78" t="b">
@@ -3901,7 +3875,7 @@
       <c r="I79" t="s">
         <v>311</v>
       </c>
-      <c r="J79" s="2">
+      <c r="J79" s="1">
         <v>36557</v>
       </c>
       <c r="K79" t="b">
@@ -3936,7 +3910,7 @@
       <c r="I80" t="s">
         <v>312</v>
       </c>
-      <c r="J80" s="2">
+      <c r="J80" s="1">
         <v>41275</v>
       </c>
       <c r="K80" t="b">
@@ -3971,7 +3945,7 @@
       <c r="I81" t="s">
         <v>313</v>
       </c>
-      <c r="J81" s="2">
+      <c r="J81" s="1">
         <v>45380</v>
       </c>
       <c r="K81" t="b">
@@ -4006,7 +3980,7 @@
       <c r="I82" t="s">
         <v>314</v>
       </c>
-      <c r="J82" s="2">
+      <c r="J82" s="1">
         <v>45421</v>
       </c>
       <c r="K82" t="b">
@@ -4041,7 +4015,7 @@
       <c r="I83" t="s">
         <v>314</v>
       </c>
-      <c r="J83" s="2">
+      <c r="J83" s="1">
         <v>45428</v>
       </c>
       <c r="K83" t="b">
@@ -4076,7 +4050,7 @@
       <c r="I84" t="s">
         <v>315</v>
       </c>
-      <c r="J84" s="2">
+      <c r="J84" s="1">
         <v>45490</v>
       </c>
       <c r="K84" t="b">
@@ -4111,7 +4085,7 @@
       <c r="I85" t="s">
         <v>316</v>
       </c>
-      <c r="J85" s="2">
+      <c r="J85" s="1">
         <v>45566</v>
       </c>
       <c r="K85" t="b">
@@ -4146,7 +4120,7 @@
       <c r="I86" t="s">
         <v>317</v>
       </c>
-      <c r="J86" s="2">
+      <c r="J86" s="1">
         <v>45986</v>
       </c>
       <c r="K86" t="b">
@@ -4181,7 +4155,7 @@
       <c r="I87" t="s">
         <v>318</v>
       </c>
-      <c r="J87" s="2">
+      <c r="J87" s="1">
         <v>46284</v>
       </c>
       <c r="K87" t="b">
@@ -4216,7 +4190,7 @@
       <c r="I88" t="s">
         <v>319</v>
       </c>
-      <c r="J88" s="2">
+      <c r="J88" s="1">
         <v>46305</v>
       </c>
       <c r="K88" t="b">
@@ -4251,7 +4225,7 @@
       <c r="I89" t="s">
         <v>319</v>
       </c>
-      <c r="J89" s="2">
+      <c r="J89" s="1">
         <v>46310</v>
       </c>
       <c r="K89" t="b">
@@ -4286,7 +4260,7 @@
       <c r="I90" t="s">
         <v>319</v>
       </c>
-      <c r="J90" s="2">
+      <c r="J90" s="1">
         <v>46317</v>
       </c>
       <c r="K90" t="b">
@@ -4321,7 +4295,7 @@
       <c r="I91" t="s">
         <v>319</v>
       </c>
-      <c r="J91" s="2">
+      <c r="J91" s="1">
         <v>46319</v>
       </c>
       <c r="K91" t="b">
@@ -4356,7 +4330,7 @@
       <c r="I92" t="s">
         <v>320</v>
       </c>
-      <c r="J92" s="2">
+      <c r="J92" s="1">
         <v>46333</v>
       </c>
       <c r="K92" t="b">
@@ -4391,7 +4365,7 @@
       <c r="I93" t="s">
         <v>320</v>
       </c>
-      <c r="J93" s="2">
+      <c r="J93" s="1">
         <v>46338</v>
       </c>
       <c r="K93" t="b">
@@ -4426,7 +4400,7 @@
       <c r="I94" t="s">
         <v>320</v>
       </c>
-      <c r="J94" s="2">
+      <c r="J94" s="1">
         <v>46338</v>
       </c>
       <c r="K94" t="b">
@@ -4461,7 +4435,7 @@
       <c r="I95" t="s">
         <v>320</v>
       </c>
-      <c r="J95" s="2">
+      <c r="J95" s="1">
         <v>46341</v>
       </c>
       <c r="K95" t="b">
@@ -4496,7 +4470,7 @@
       <c r="I96" t="s">
         <v>320</v>
       </c>
-      <c r="J96" s="2">
+      <c r="J96" s="1">
         <v>46344</v>
       </c>
       <c r="K96" t="b">
@@ -4531,7 +4505,7 @@
       <c r="I97" t="s">
         <v>321</v>
       </c>
-      <c r="J97" s="2">
+      <c r="J97" s="1">
         <v>46360</v>
       </c>
       <c r="K97" t="b">
@@ -4566,7 +4540,7 @@
       <c r="I98" t="s">
         <v>321</v>
       </c>
-      <c r="J98" s="2">
+      <c r="J98" s="1">
         <v>46360</v>
       </c>
       <c r="K98" t="b">
@@ -4601,7 +4575,7 @@
       <c r="I99" t="s">
         <v>321</v>
       </c>
-      <c r="J99" s="2">
+      <c r="J99" s="1">
         <v>46367</v>
       </c>
       <c r="K99" t="b">
@@ -4636,7 +4610,7 @@
       <c r="I100" t="s">
         <v>321</v>
       </c>
-      <c r="J100" s="2">
+      <c r="J100" s="1">
         <v>46375</v>
       </c>
       <c r="K100" t="b">
@@ -4671,7 +4645,7 @@
       <c r="I101" t="s">
         <v>321</v>
       </c>
-      <c r="J101" s="2">
+      <c r="J101" s="1">
         <v>46387</v>
       </c>
       <c r="K101" t="b">
@@ -4706,7 +4680,7 @@
       <c r="I102" t="s">
         <v>321</v>
       </c>
-      <c r="J102" s="2">
+      <c r="J102" s="1">
         <v>46387</v>
       </c>
       <c r="K102" t="b">
@@ -4741,7 +4715,7 @@
       <c r="I103" t="s">
         <v>321</v>
       </c>
-      <c r="J103" s="2">
+      <c r="J103" s="1">
         <v>46387</v>
       </c>
       <c r="K103" t="b">
@@ -4776,7 +4750,7 @@
       <c r="I104" t="s">
         <v>321</v>
       </c>
-      <c r="J104" s="2">
+      <c r="J104" s="1">
         <v>46388</v>
       </c>
       <c r="K104" t="b">
@@ -4811,7 +4785,7 @@
       <c r="I105" t="s">
         <v>322</v>
       </c>
-      <c r="J105" s="2">
+      <c r="J105" s="1">
         <v>46401</v>
       </c>
       <c r="K105" t="b">
@@ -4846,7 +4820,7 @@
       <c r="I106" t="s">
         <v>322</v>
       </c>
-      <c r="J106" s="2">
+      <c r="J106" s="1">
         <v>46401</v>
       </c>
       <c r="K106" t="b">
@@ -4881,7 +4855,7 @@
       <c r="I107" t="s">
         <v>322</v>
       </c>
-      <c r="J107" s="2">
+      <c r="J107" s="1">
         <v>46401</v>
       </c>
       <c r="K107" t="b">
@@ -4916,7 +4890,7 @@
       <c r="I108" t="s">
         <v>322</v>
       </c>
-      <c r="J108" s="2">
+      <c r="J108" s="1">
         <v>46412</v>
       </c>
       <c r="K108" t="b">
@@ -4951,7 +4925,7 @@
       <c r="I109" t="s">
         <v>322</v>
       </c>
-      <c r="J109" s="2">
+      <c r="J109" s="1">
         <v>46412</v>
       </c>
       <c r="K109" t="b">
@@ -4986,7 +4960,7 @@
       <c r="I110" t="s">
         <v>322</v>
       </c>
-      <c r="J110" s="2">
+      <c r="J110" s="1">
         <v>46412</v>
       </c>
       <c r="K110" t="b">
@@ -5021,7 +4995,7 @@
       <c r="I111" t="s">
         <v>323</v>
       </c>
-      <c r="J111" s="2">
+      <c r="J111" s="1">
         <v>46424</v>
       </c>
       <c r="K111" t="b">
@@ -5056,7 +5030,7 @@
       <c r="I112" t="s">
         <v>323</v>
       </c>
-      <c r="J112" s="2">
+      <c r="J112" s="1">
         <v>46437</v>
       </c>
       <c r="K112" t="b">
@@ -5091,7 +5065,7 @@
       <c r="I113" t="s">
         <v>323</v>
       </c>
-      <c r="J113" s="2">
+      <c r="J113" s="1">
         <v>46451</v>
       </c>
       <c r="K113" t="b">
@@ -5126,7 +5100,7 @@
       <c r="I114" t="s">
         <v>323</v>
       </c>
-      <c r="J114" s="2">
+      <c r="J114" s="1">
         <v>46451</v>
       </c>
       <c r="K114" t="b">
@@ -5161,7 +5135,7 @@
       <c r="I115" t="s">
         <v>324</v>
       </c>
-      <c r="J115" s="2">
+      <c r="J115" s="1">
         <v>46455</v>
       </c>
       <c r="K115" t="b">
@@ -5196,7 +5170,7 @@
       <c r="I116" t="s">
         <v>324</v>
       </c>
-      <c r="J116" s="2">
+      <c r="J116" s="1">
         <v>46456</v>
       </c>
       <c r="K116" t="b">
@@ -5231,7 +5205,7 @@
       <c r="I117" t="s">
         <v>324</v>
       </c>
-      <c r="J117" s="2">
+      <c r="J117" s="1">
         <v>46457</v>
       </c>
       <c r="K117" t="b">
@@ -5266,7 +5240,7 @@
       <c r="I118" t="s">
         <v>324</v>
       </c>
-      <c r="J118" s="2">
+      <c r="J118" s="1">
         <v>46464</v>
       </c>
       <c r="K118" t="b">
@@ -5301,7 +5275,7 @@
       <c r="I119" t="s">
         <v>324</v>
       </c>
-      <c r="J119" s="2">
+      <c r="J119" s="1">
         <v>46470</v>
       </c>
       <c r="K119" t="b">
@@ -5336,7 +5310,7 @@
       <c r="I120" t="s">
         <v>325</v>
       </c>
-      <c r="J120" s="2">
+      <c r="J120" s="1">
         <v>46485</v>
       </c>
       <c r="K120" t="b">
@@ -5371,7 +5345,7 @@
       <c r="I121" t="s">
         <v>325</v>
       </c>
-      <c r="J121" s="2">
+      <c r="J121" s="1">
         <v>46499</v>
       </c>
       <c r="K121" t="b">
@@ -5406,7 +5380,7 @@
       <c r="I122" t="s">
         <v>325</v>
       </c>
-      <c r="J122" s="2">
+      <c r="J122" s="1">
         <v>46504</v>
       </c>
       <c r="K122" t="b">
@@ -5441,7 +5415,7 @@
       <c r="I123" t="s">
         <v>325</v>
       </c>
-      <c r="J123" s="2">
+      <c r="J123" s="1">
         <v>46504</v>
       </c>
       <c r="K123" t="b">
@@ -5476,7 +5450,7 @@
       <c r="I124" t="s">
         <v>325</v>
       </c>
-      <c r="J124" s="2">
+      <c r="J124" s="1">
         <v>46507</v>
       </c>
       <c r="K124" t="b">
@@ -5511,7 +5485,7 @@
       <c r="I125" t="s">
         <v>325</v>
       </c>
-      <c r="J125" s="2">
+      <c r="J125" s="1">
         <v>46508</v>
       </c>
       <c r="K125" t="b">
@@ -5546,7 +5520,7 @@
       <c r="I126" t="s">
         <v>325</v>
       </c>
-      <c r="J126" s="2">
+      <c r="J126" s="1">
         <v>46512</v>
       </c>
       <c r="K126" t="b">
@@ -5581,7 +5555,7 @@
       <c r="I127" t="s">
         <v>326</v>
       </c>
-      <c r="J127" s="2">
+      <c r="J127" s="1">
         <v>46512</v>
       </c>
       <c r="K127" t="b">
@@ -5616,7 +5590,7 @@
       <c r="I128" t="s">
         <v>326</v>
       </c>
-      <c r="J128" s="2">
+      <c r="J128" s="1">
         <v>46528</v>
       </c>
       <c r="K128" t="b">
@@ -5651,7 +5625,7 @@
       <c r="I129" t="s">
         <v>326</v>
       </c>
-      <c r="J129" s="2">
+      <c r="J129" s="1">
         <v>46529</v>
       </c>
       <c r="K129" t="b">
@@ -5686,7 +5660,7 @@
       <c r="I130" t="s">
         <v>326</v>
       </c>
-      <c r="J130" s="2">
+      <c r="J130" s="1">
         <v>46537</v>
       </c>
       <c r="K130" t="b">
@@ -5721,7 +5695,7 @@
       <c r="I131" t="s">
         <v>327</v>
       </c>
-      <c r="J131" s="2">
+      <c r="J131" s="1">
         <v>46546</v>
       </c>
       <c r="K131" t="b">
@@ -5756,7 +5730,7 @@
       <c r="I132" t="s">
         <v>327</v>
       </c>
-      <c r="J132" s="2">
+      <c r="J132" s="1">
         <v>46547</v>
       </c>
       <c r="K132" t="b">
@@ -5791,7 +5765,7 @@
       <c r="I133" t="s">
         <v>327</v>
       </c>
-      <c r="J133" s="2">
+      <c r="J133" s="1">
         <v>46547</v>
       </c>
       <c r="K133" t="b">
@@ -5826,7 +5800,7 @@
       <c r="I134" t="s">
         <v>327</v>
       </c>
-      <c r="J134" s="2">
+      <c r="J134" s="1">
         <v>46547</v>
       </c>
       <c r="K134" t="b">
@@ -5861,7 +5835,7 @@
       <c r="I135" t="s">
         <v>327</v>
       </c>
-      <c r="J135" s="2">
+      <c r="J135" s="1">
         <v>46551</v>
       </c>
       <c r="K135" t="b">
@@ -5896,7 +5870,7 @@
       <c r="I136" t="s">
         <v>327</v>
       </c>
-      <c r="J136" s="2">
+      <c r="J136" s="1">
         <v>46560</v>
       </c>
       <c r="K136" t="b">
@@ -5931,7 +5905,7 @@
       <c r="I137" t="s">
         <v>327</v>
       </c>
-      <c r="J137" s="2">
+      <c r="J137" s="1">
         <v>46564</v>
       </c>
       <c r="K137" t="b">
@@ -5966,7 +5940,7 @@
       <c r="I138" t="s">
         <v>327</v>
       </c>
-      <c r="J138" s="2">
+      <c r="J138" s="1">
         <v>46567</v>
       </c>
       <c r="K138" t="b">
@@ -6001,7 +5975,7 @@
       <c r="I139" t="s">
         <v>327</v>
       </c>
-      <c r="J139" s="2">
+      <c r="J139" s="1">
         <v>46568</v>
       </c>
       <c r="K139" t="b">
@@ -6036,7 +6010,7 @@
       <c r="I140" t="s">
         <v>328</v>
       </c>
-      <c r="J140" s="2">
+      <c r="J140" s="1">
         <v>46578</v>
       </c>
       <c r="K140" t="b">
@@ -6071,7 +6045,7 @@
       <c r="I141" t="s">
         <v>328</v>
       </c>
-      <c r="J141" s="2">
+      <c r="J141" s="1">
         <v>46592</v>
       </c>
       <c r="K141" t="b">
@@ -6106,7 +6080,7 @@
       <c r="I142" t="s">
         <v>328</v>
       </c>
-      <c r="J142" s="2">
+      <c r="J142" s="1">
         <v>46592</v>
       </c>
       <c r="K142" t="b">
@@ -6141,7 +6115,7 @@
       <c r="I143" t="s">
         <v>329</v>
       </c>
-      <c r="J143" s="2">
+      <c r="J143" s="1">
         <v>46212</v>
       </c>
       <c r="K143" t="b">
@@ -6176,7 +6150,7 @@
       <c r="I144" t="s">
         <v>330</v>
       </c>
-      <c r="J144" s="2">
+      <c r="J144" s="1">
         <v>46225</v>
       </c>
       <c r="K144" t="b">
@@ -6211,7 +6185,7 @@
       <c r="I145" t="s">
         <v>331</v>
       </c>
-      <c r="J145" s="2">
+      <c r="J145" s="1">
         <v>46263</v>
       </c>
       <c r="K145" t="b">
@@ -6243,7 +6217,7 @@
       <c r="H146">
         <v>-1476</v>
       </c>
-      <c r="J146" s="2">
+      <c r="J146" s="1">
         <v>43773</v>
       </c>
       <c r="K146" t="b">
@@ -6275,7 +6249,7 @@
       <c r="H147">
         <v>-1469</v>
       </c>
-      <c r="J147" s="2">
+      <c r="J147" s="1">
         <v>43773</v>
       </c>
       <c r="K147" t="b">
@@ -6307,7 +6281,7 @@
       <c r="H148">
         <v>-1186</v>
       </c>
-      <c r="J148" s="2">
+      <c r="J148" s="1">
         <v>45295</v>
       </c>
       <c r="K148" t="b">
@@ -6339,7 +6313,7 @@
       <c r="H149">
         <v>-1048</v>
       </c>
-      <c r="J149" s="2">
+      <c r="J149" s="1">
         <v>45617</v>
       </c>
       <c r="K149" t="b">
@@ -6371,7 +6345,7 @@
       <c r="H150">
         <v>-980</v>
       </c>
-      <c r="J150" s="2">
+      <c r="J150" s="1">
         <v>45677</v>
       </c>
       <c r="K150" t="b">
@@ -6403,7 +6377,7 @@
       <c r="H151">
         <v>-961</v>
       </c>
-      <c r="J151" s="2">
+      <c r="J151" s="1">
         <v>44944</v>
       </c>
       <c r="K151" t="b">
@@ -6435,7 +6409,7 @@
       <c r="H152">
         <v>-252</v>
       </c>
-      <c r="J152" s="2">
+      <c r="J152" s="1">
         <v>46092</v>
       </c>
       <c r="K152" t="b">
@@ -6467,7 +6441,7 @@
       <c r="H153">
         <v>3</v>
       </c>
-      <c r="J153" s="2">
+      <c r="J153" s="1">
         <v>46265</v>
       </c>
       <c r="K153" t="b">
@@ -6499,7 +6473,7 @@
       <c r="H154">
         <v>3</v>
       </c>
-      <c r="J154" s="2">
+      <c r="J154" s="1">
         <v>46265</v>
       </c>
       <c r="K154" t="b">
@@ -6531,7 +6505,7 @@
       <c r="H155">
         <v>43</v>
       </c>
-      <c r="J155" s="2">
+      <c r="J155" s="1">
         <v>46440</v>
       </c>
       <c r="K155" t="b">
@@ -6563,7 +6537,7 @@
       <c r="H156">
         <v>43</v>
       </c>
-      <c r="J156" s="2">
+      <c r="J156" s="1">
         <v>46440</v>
       </c>
       <c r="K156" t="b">
@@ -6595,7 +6569,7 @@
       <c r="H157">
         <v>72</v>
       </c>
-      <c r="J157" s="2">
+      <c r="J157" s="1">
         <v>46289</v>
       </c>
       <c r="K157" t="b">
@@ -6627,7 +6601,7 @@
       <c r="H158">
         <v>72</v>
       </c>
-      <c r="J158" s="2">
+      <c r="J158" s="1">
         <v>46289</v>
       </c>
       <c r="K158" t="b">
@@ -6659,7 +6633,7 @@
       <c r="H159">
         <v>81</v>
       </c>
-      <c r="J159" s="2">
+      <c r="J159" s="1">
         <v>46405</v>
       </c>
       <c r="K159" t="b">
@@ -6691,7 +6665,7 @@
       <c r="H160">
         <v>102</v>
       </c>
-      <c r="J160" s="2">
+      <c r="J160" s="1">
         <v>46463</v>
       </c>
       <c r="K160" t="b">
@@ -6723,7 +6697,7 @@
       <c r="H161">
         <v>109</v>
       </c>
-      <c r="J161" s="2">
+      <c r="J161" s="1">
         <v>46353</v>
       </c>
       <c r="K161" t="b">
@@ -6755,7 +6729,7 @@
       <c r="H162">
         <v>127</v>
       </c>
-      <c r="J162" s="2">
+      <c r="J162" s="1">
         <v>46417</v>
       </c>
       <c r="K162" t="b">
@@ -6787,7 +6761,7 @@
       <c r="H163">
         <v>152</v>
       </c>
-      <c r="J163" s="2">
+      <c r="J163" s="1">
         <v>46271</v>
       </c>
       <c r="K163" t="b">
@@ -6819,7 +6793,7 @@
       <c r="H164">
         <v>152</v>
       </c>
-      <c r="J164" s="2">
+      <c r="J164" s="1">
         <v>46271</v>
       </c>
       <c r="K164" t="b">
@@ -6851,7 +6825,7 @@
       <c r="H165">
         <v>153</v>
       </c>
-      <c r="J165" s="2">
+      <c r="J165" s="1">
         <v>46458</v>
       </c>
       <c r="K165" t="b">
@@ -6883,7 +6857,7 @@
       <c r="H166">
         <v>158</v>
       </c>
-      <c r="J166" s="2">
+      <c r="J166" s="1">
         <v>46381</v>
       </c>
       <c r="K166" t="b">
@@ -6915,7 +6889,7 @@
       <c r="H167">
         <v>163</v>
       </c>
-      <c r="J167" s="2">
+      <c r="J167" s="1">
         <v>46592</v>
       </c>
       <c r="K167" t="b">
@@ -6947,7 +6921,7 @@
       <c r="H168">
         <v>167</v>
       </c>
-      <c r="J168" s="2">
+      <c r="J168" s="1">
         <v>46441</v>
       </c>
       <c r="K168" t="b">
@@ -6979,7 +6953,7 @@
       <c r="H169">
         <v>169</v>
       </c>
-      <c r="J169" s="2">
+      <c r="J169" s="1">
         <v>46391</v>
       </c>
       <c r="K169" t="b">
@@ -7011,7 +6985,7 @@
       <c r="H170">
         <v>184</v>
       </c>
-      <c r="J170" s="2">
+      <c r="J170" s="1">
         <v>46385</v>
       </c>
       <c r="K170" t="b">
@@ -7043,7 +7017,7 @@
       <c r="H171">
         <v>186</v>
       </c>
-      <c r="J171" s="2">
+      <c r="J171" s="1">
         <v>46387</v>
       </c>
       <c r="K171" t="b">
@@ -7075,7 +7049,7 @@
       <c r="H172">
         <v>206</v>
       </c>
-      <c r="J172" s="2">
+      <c r="J172" s="1">
         <v>46399</v>
       </c>
       <c r="K172" t="b">
@@ -7107,7 +7081,7 @@
       <c r="H173">
         <v>206</v>
       </c>
-      <c r="J173" s="2">
+      <c r="J173" s="1">
         <v>46399</v>
       </c>
       <c r="K173" t="b">
@@ -7139,7 +7113,7 @@
       <c r="H174">
         <v>234</v>
       </c>
-      <c r="J174" s="2">
+      <c r="J174" s="1">
         <v>46458</v>
       </c>
       <c r="K174" t="b">
@@ -7171,7 +7145,7 @@
       <c r="H175">
         <v>248</v>
       </c>
-      <c r="J175" s="2">
+      <c r="J175" s="1">
         <v>46528</v>
       </c>
       <c r="K175" t="b">
@@ -7203,7 +7177,7 @@
       <c r="H176">
         <v>317</v>
       </c>
-      <c r="J176" s="2">
+      <c r="J176" s="1">
         <v>46540</v>
       </c>
       <c r="K176" t="b">
@@ -7235,7 +7209,7 @@
       <c r="H177">
         <v>340</v>
       </c>
-      <c r="J177" s="2">
+      <c r="J177" s="1">
         <v>46547</v>
       </c>
       <c r="K177" t="b">
@@ -7267,7 +7241,7 @@
       <c r="H178">
         <v>364</v>
       </c>
-      <c r="J178" s="2">
+      <c r="J178" s="1">
         <v>46557</v>
       </c>
       <c r="K178" t="b">
@@ -7299,7 +7273,7 @@
       <c r="H179">
         <v>368</v>
       </c>
-      <c r="J179" s="2">
+      <c r="J179" s="1">
         <v>46571</v>
       </c>
       <c r="K179" t="b">
@@ -7331,7 +7305,7 @@
       <c r="H180">
         <v>368</v>
       </c>
-      <c r="J180" s="2">
+      <c r="J180" s="1">
         <v>46571</v>
       </c>
       <c r="K180" t="b">
@@ -7363,7 +7337,7 @@
       <c r="H181">
         <v>370</v>
       </c>
-      <c r="J181" s="2">
+      <c r="J181" s="1">
         <v>46562</v>
       </c>
       <c r="K181" t="b">
@@ -7395,7 +7369,7 @@
       <c r="H182">
         <v>385</v>
       </c>
-      <c r="J182" s="2">
+      <c r="J182" s="1">
         <v>46574</v>
       </c>
       <c r="K182" t="b">
@@ -7427,7 +7401,7 @@
       <c r="H183">
         <v>385</v>
       </c>
-      <c r="J183" s="2">
+      <c r="J183" s="1">
         <v>46574</v>
       </c>
       <c r="K183" t="b">
@@ -7459,7 +7433,7 @@
       <c r="H184">
         <v>417</v>
       </c>
-      <c r="J184" s="2">
+      <c r="J184" s="1">
         <v>46578</v>
       </c>
       <c r="K184" t="b">
@@ -7491,7 +7465,7 @@
       <c r="H185">
         <v>721</v>
       </c>
-      <c r="J185" s="2">
+      <c r="J185" s="1">
         <v>46345</v>
       </c>
       <c r="K185" t="b">
@@ -7523,7 +7497,7 @@
       <c r="H186">
         <v>721</v>
       </c>
-      <c r="J186" s="2">
+      <c r="J186" s="1">
         <v>46345</v>
       </c>
       <c r="K186" t="b">
@@ -7555,7 +7529,7 @@
       <c r="H187">
         <v>850</v>
       </c>
-      <c r="J187" s="2">
+      <c r="J187" s="1">
         <v>46366</v>
       </c>
       <c r="K187" t="b">
@@ -7587,7 +7561,7 @@
       <c r="H188">
         <v>850</v>
       </c>
-      <c r="J188" s="2">
+      <c r="J188" s="1">
         <v>46366</v>
       </c>
       <c r="K188" t="b">
@@ -7619,7 +7593,7 @@
       <c r="H189">
         <v>1661</v>
       </c>
-      <c r="J189" s="2">
+      <c r="J189" s="1">
         <v>46524</v>
       </c>
       <c r="K189" t="b">
@@ -7651,7 +7625,7 @@
       <c r="H190">
         <v>1661</v>
       </c>
-      <c r="J190" s="2">
+      <c r="J190" s="1">
         <v>46524</v>
       </c>
       <c r="K190" t="b">
@@ -7683,7 +7657,7 @@
       <c r="H191">
         <v>488</v>
       </c>
-      <c r="J191" s="2">
+      <c r="J191" s="1">
         <v>46190</v>
       </c>
       <c r="K191" t="b">
@@ -7715,7 +7689,7 @@
       <c r="H192">
         <v>25565</v>
       </c>
-      <c r="J192" s="2">
+      <c r="J192" s="1">
         <v>46190</v>
       </c>
       <c r="K192" t="b">
@@ -7747,7 +7721,7 @@
       <c r="H193">
         <v>25567</v>
       </c>
-      <c r="J193" s="2">
+      <c r="J193" s="1">
         <v>46190</v>
       </c>
       <c r="K193" t="b">
@@ -7779,7 +7753,7 @@
       <c r="H194">
         <v>31293</v>
       </c>
-      <c r="J194" s="2">
+      <c r="J194" s="1">
         <v>46190</v>
       </c>
       <c r="K194" t="b">

</xml_diff>

<commit_message>
Atualização automática: vencimentos_tmot (03/09/2026 13:42)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
@@ -1019,8 +1019,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1036,7 +1044,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1044,12 +1052,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1349,37 +1375,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1408,7 +1434,7 @@
       <c r="H2">
         <v>-4300.3</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>39285</v>
       </c>
       <c r="K2" t="b">
@@ -1440,7 +1466,7 @@
       <c r="H3">
         <v>-2354.2</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>40669</v>
       </c>
       <c r="K3" t="b">
@@ -1472,7 +1498,7 @@
       <c r="H4">
         <v>-910.7</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>40669</v>
       </c>
       <c r="K4" t="b">
@@ -1504,7 +1530,7 @@
       <c r="H5">
         <v>-868</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>44884</v>
       </c>
       <c r="K5" t="b">
@@ -1536,7 +1562,7 @@
       <c r="H6">
         <v>-483.8</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>43855</v>
       </c>
       <c r="K6" t="b">
@@ -1568,7 +1594,7 @@
       <c r="H7">
         <v>-417</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>46014</v>
       </c>
       <c r="K7" t="b">
@@ -1600,7 +1626,7 @@
       <c r="H8">
         <v>-414.2</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>46014</v>
       </c>
       <c r="K8" t="b">
@@ -1632,7 +1658,7 @@
       <c r="H9">
         <v>-391.8</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>42769</v>
       </c>
       <c r="K9" t="b">
@@ -1664,7 +1690,7 @@
       <c r="H10">
         <v>-391.6</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>45804</v>
       </c>
       <c r="K10" t="b">
@@ -1696,7 +1722,7 @@
       <c r="H11">
         <v>-391.6</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>45804</v>
       </c>
       <c r="K11" t="b">
@@ -1728,7 +1754,7 @@
       <c r="H12">
         <v>-372.9</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>42821</v>
       </c>
       <c r="K12" t="b">
@@ -1760,7 +1786,7 @@
       <c r="H13">
         <v>-372.9</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>46014</v>
       </c>
       <c r="K13" t="b">
@@ -1792,7 +1818,7 @@
       <c r="H14">
         <v>-372.9</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>46014</v>
       </c>
       <c r="K14" t="b">
@@ -1824,7 +1850,7 @@
       <c r="H15">
         <v>-372.9</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>46014</v>
       </c>
       <c r="K15" t="b">
@@ -1856,7 +1882,7 @@
       <c r="H16">
         <v>-367.8</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="2">
         <v>46017</v>
       </c>
       <c r="K16" t="b">
@@ -1888,7 +1914,7 @@
       <c r="H17">
         <v>-367.8</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="2">
         <v>46017</v>
       </c>
       <c r="K17" t="b">
@@ -1920,7 +1946,7 @@
       <c r="H18">
         <v>-347.2</v>
       </c>
-      <c r="J18" s="1">
+      <c r="J18" s="2">
         <v>40979</v>
       </c>
       <c r="K18" t="b">
@@ -1952,7 +1978,7 @@
       <c r="H19">
         <v>-293.8</v>
       </c>
-      <c r="J19" s="1">
+      <c r="J19" s="2">
         <v>45846</v>
       </c>
       <c r="K19" t="b">
@@ -1984,7 +2010,7 @@
       <c r="H20">
         <v>-206.4</v>
       </c>
-      <c r="J20" s="1">
+      <c r="J20" s="2">
         <v>36669</v>
       </c>
       <c r="K20" t="b">
@@ -2016,7 +2042,7 @@
       <c r="H21">
         <v>-131.6</v>
       </c>
-      <c r="J21" s="1">
+      <c r="J21" s="2">
         <v>46111</v>
       </c>
       <c r="K21" t="b">
@@ -2048,7 +2074,7 @@
       <c r="H22">
         <v>-131.6</v>
       </c>
-      <c r="J22" s="1">
+      <c r="J22" s="2">
         <v>46111</v>
       </c>
       <c r="K22" t="b">
@@ -2080,7 +2106,7 @@
       <c r="H23">
         <v>-131.6</v>
       </c>
-      <c r="J23" s="1">
+      <c r="J23" s="2">
         <v>46111</v>
       </c>
       <c r="K23" t="b">
@@ -2112,7 +2138,7 @@
       <c r="H24">
         <v>-131.6</v>
       </c>
-      <c r="J24" s="1">
+      <c r="J24" s="2">
         <v>46111</v>
       </c>
       <c r="K24" t="b">
@@ -2144,7 +2170,7 @@
       <c r="H25">
         <v>-131.6</v>
       </c>
-      <c r="J25" s="1">
+      <c r="J25" s="2">
         <v>46111</v>
       </c>
       <c r="K25" t="b">
@@ -2176,7 +2202,7 @@
       <c r="H26">
         <v>-98.3</v>
       </c>
-      <c r="J26" s="1">
+      <c r="J26" s="2">
         <v>41204</v>
       </c>
       <c r="K26" t="b">
@@ -2208,7 +2234,7 @@
       <c r="H27">
         <v>-47.2</v>
       </c>
-      <c r="J27" s="1">
+      <c r="J27" s="2">
         <v>44011</v>
       </c>
       <c r="K27" t="b">
@@ -2240,7 +2266,7 @@
       <c r="H28">
         <v>-22.3</v>
       </c>
-      <c r="J28" s="1">
+      <c r="J28" s="2">
         <v>46226</v>
       </c>
       <c r="K28" t="b">
@@ -2272,7 +2298,7 @@
       <c r="H29">
         <v>4.7</v>
       </c>
-      <c r="J29" s="1">
+      <c r="J29" s="2">
         <v>46265</v>
       </c>
       <c r="K29" t="b">
@@ -2304,7 +2330,7 @@
       <c r="H30">
         <v>7.5</v>
       </c>
-      <c r="J30" s="1">
+      <c r="J30" s="2">
         <v>46265</v>
       </c>
       <c r="K30" t="b">
@@ -2336,7 +2362,7 @@
       <c r="H31">
         <v>10</v>
       </c>
-      <c r="J31" s="1">
+      <c r="J31" s="2">
         <v>46265</v>
       </c>
       <c r="K31" t="b">
@@ -2368,7 +2394,7 @@
       <c r="H32">
         <v>12.8</v>
       </c>
-      <c r="J32" s="1">
+      <c r="J32" s="2">
         <v>46265</v>
       </c>
       <c r="K32" t="b">
@@ -2400,7 +2426,7 @@
       <c r="H33">
         <v>14</v>
       </c>
-      <c r="J33" s="1">
+      <c r="J33" s="2">
         <v>46265</v>
       </c>
       <c r="K33" t="b">
@@ -2432,7 +2458,7 @@
       <c r="H34">
         <v>17.8</v>
       </c>
-      <c r="J34" s="1">
+      <c r="J34" s="2">
         <v>46265</v>
       </c>
       <c r="K34" t="b">
@@ -2464,7 +2490,7 @@
       <c r="H35">
         <v>20.4</v>
       </c>
-      <c r="J35" s="1">
+      <c r="J35" s="2">
         <v>46265</v>
       </c>
       <c r="K35" t="b">
@@ -2496,7 +2522,7 @@
       <c r="H36">
         <v>21.2</v>
       </c>
-      <c r="J36" s="1">
+      <c r="J36" s="2">
         <v>46265</v>
       </c>
       <c r="K36" t="b">
@@ -2528,7 +2554,7 @@
       <c r="H37">
         <v>26.2</v>
       </c>
-      <c r="J37" s="1">
+      <c r="J37" s="2">
         <v>46265</v>
       </c>
       <c r="K37" t="b">
@@ -2560,7 +2586,7 @@
       <c r="H38">
         <v>33.6</v>
       </c>
-      <c r="J38" s="1">
+      <c r="J38" s="2">
         <v>46364</v>
       </c>
       <c r="K38" t="b">
@@ -2592,7 +2618,7 @@
       <c r="H39">
         <v>42.2</v>
       </c>
-      <c r="J39" s="1">
+      <c r="J39" s="2">
         <v>46269</v>
       </c>
       <c r="K39" t="b">
@@ -2624,7 +2650,7 @@
       <c r="H40">
         <v>42.8</v>
       </c>
-      <c r="J40" s="1">
+      <c r="J40" s="2">
         <v>46291</v>
       </c>
       <c r="K40" t="b">
@@ -2656,7 +2682,7 @@
       <c r="H41">
         <v>45.7</v>
       </c>
-      <c r="J41" s="1">
+      <c r="J41" s="2">
         <v>46395</v>
       </c>
       <c r="K41" t="b">
@@ -2688,7 +2714,7 @@
       <c r="H42">
         <v>47.2</v>
       </c>
-      <c r="J42" s="1">
+      <c r="J42" s="2">
         <v>46280</v>
       </c>
       <c r="K42" t="b">
@@ -2720,7 +2746,7 @@
       <c r="H43">
         <v>48.7</v>
       </c>
-      <c r="J43" s="1">
+      <c r="J43" s="2">
         <v>46281</v>
       </c>
       <c r="K43" t="b">
@@ -2752,7 +2778,7 @@
       <c r="H44">
         <v>60</v>
       </c>
-      <c r="J44" s="1">
+      <c r="J44" s="2">
         <v>46281</v>
       </c>
       <c r="K44" t="b">
@@ -2784,7 +2810,7 @@
       <c r="H45">
         <v>62.6</v>
       </c>
-      <c r="J45" s="1">
+      <c r="J45" s="2">
         <v>46265</v>
       </c>
       <c r="K45" t="b">
@@ -2816,7 +2842,7 @@
       <c r="H46">
         <v>64.59999999999999</v>
       </c>
-      <c r="J46" s="1">
+      <c r="J46" s="2">
         <v>46265</v>
       </c>
       <c r="K46" t="b">
@@ -2848,7 +2874,7 @@
       <c r="H47">
         <v>67.59999999999999</v>
       </c>
-      <c r="J47" s="1">
+      <c r="J47" s="2">
         <v>46267</v>
       </c>
       <c r="K47" t="b">
@@ -2880,7 +2906,7 @@
       <c r="H48">
         <v>68.3</v>
       </c>
-      <c r="J48" s="1">
+      <c r="J48" s="2">
         <v>46278</v>
       </c>
       <c r="K48" t="b">
@@ -2912,7 +2938,7 @@
       <c r="H49">
         <v>69.2</v>
       </c>
-      <c r="J49" s="1">
+      <c r="J49" s="2">
         <v>46453</v>
       </c>
       <c r="K49" t="b">
@@ -2944,7 +2970,7 @@
       <c r="H50">
         <v>69.8</v>
       </c>
-      <c r="J50" s="1">
+      <c r="J50" s="2">
         <v>46265</v>
       </c>
       <c r="K50" t="b">
@@ -2976,7 +3002,7 @@
       <c r="H51">
         <v>69.8</v>
       </c>
-      <c r="J51" s="1">
+      <c r="J51" s="2">
         <v>46265</v>
       </c>
       <c r="K51" t="b">
@@ -3008,7 +3034,7 @@
       <c r="H52">
         <v>72.2</v>
       </c>
-      <c r="J52" s="1">
+      <c r="J52" s="2">
         <v>46275</v>
       </c>
       <c r="K52" t="b">
@@ -3040,7 +3066,7 @@
       <c r="H53">
         <v>72.2</v>
       </c>
-      <c r="J53" s="1">
+      <c r="J53" s="2">
         <v>46275</v>
       </c>
       <c r="K53" t="b">
@@ -3072,7 +3098,7 @@
       <c r="H54">
         <v>78.09999999999999</v>
       </c>
-      <c r="J54" s="1">
+      <c r="J54" s="2">
         <v>46265</v>
       </c>
       <c r="K54" t="b">
@@ -3104,7 +3130,7 @@
       <c r="H55">
         <v>82.8</v>
       </c>
-      <c r="J55" s="1">
+      <c r="J55" s="2">
         <v>46487</v>
       </c>
       <c r="K55" t="b">
@@ -3136,7 +3162,7 @@
       <c r="H56">
         <v>83.09999999999999</v>
       </c>
-      <c r="J56" s="1">
+      <c r="J56" s="2">
         <v>46285</v>
       </c>
       <c r="K56" t="b">
@@ -3168,7 +3194,7 @@
       <c r="H57">
         <v>84.8</v>
       </c>
-      <c r="J57" s="1">
+      <c r="J57" s="2">
         <v>46492</v>
       </c>
       <c r="K57" t="b">
@@ -3200,7 +3226,7 @@
       <c r="H58">
         <v>104.9</v>
       </c>
-      <c r="J58" s="1">
+      <c r="J58" s="2">
         <v>46297</v>
       </c>
       <c r="K58" t="b">
@@ -3232,7 +3258,7 @@
       <c r="H59">
         <v>107.6</v>
       </c>
-      <c r="J59" s="1">
+      <c r="J59" s="2">
         <v>46283</v>
       </c>
       <c r="K59" t="b">
@@ -3264,7 +3290,7 @@
       <c r="H60">
         <v>111.9</v>
       </c>
-      <c r="J60" s="1">
+      <c r="J60" s="2">
         <v>46300</v>
       </c>
       <c r="K60" t="b">
@@ -3296,7 +3322,7 @@
       <c r="H61">
         <v>111.9</v>
       </c>
-      <c r="J61" s="1">
+      <c r="J61" s="2">
         <v>46300</v>
       </c>
       <c r="K61" t="b">
@@ -3328,7 +3354,7 @@
       <c r="H62">
         <v>111.9</v>
       </c>
-      <c r="J62" s="1">
+      <c r="J62" s="2">
         <v>46300</v>
       </c>
       <c r="K62" t="b">
@@ -3360,7 +3386,7 @@
       <c r="H63">
         <v>111.9</v>
       </c>
-      <c r="J63" s="1">
+      <c r="J63" s="2">
         <v>46300</v>
       </c>
       <c r="K63" t="b">
@@ -3392,7 +3418,7 @@
       <c r="H64">
         <v>111.9</v>
       </c>
-      <c r="J64" s="1">
+      <c r="J64" s="2">
         <v>46300</v>
       </c>
       <c r="K64" t="b">
@@ -3424,7 +3450,7 @@
       <c r="H65">
         <v>128.8</v>
       </c>
-      <c r="J65" s="1">
+      <c r="J65" s="2">
         <v>46308</v>
       </c>
       <c r="K65" t="b">
@@ -3456,7 +3482,7 @@
       <c r="H66">
         <v>131.1</v>
       </c>
-      <c r="J66" s="1">
+      <c r="J66" s="2">
         <v>46336</v>
       </c>
       <c r="K66" t="b">
@@ -3488,7 +3514,7 @@
       <c r="H67">
         <v>138.4</v>
       </c>
-      <c r="J67" s="1">
+      <c r="J67" s="2">
         <v>46343</v>
       </c>
       <c r="K67" t="b">
@@ -3520,7 +3546,7 @@
       <c r="H68">
         <v>141</v>
       </c>
-      <c r="J68" s="1">
+      <c r="J68" s="2">
         <v>46350</v>
       </c>
       <c r="K68" t="b">
@@ -3552,7 +3578,7 @@
       <c r="H69">
         <v>162</v>
       </c>
-      <c r="J69" s="1">
+      <c r="J69" s="2">
         <v>46391</v>
       </c>
       <c r="K69" t="b">
@@ -3584,7 +3610,7 @@
       <c r="H70">
         <v>167.2</v>
       </c>
-      <c r="J70" s="1">
+      <c r="J70" s="2">
         <v>46330</v>
       </c>
       <c r="K70" t="b">
@@ -3616,7 +3642,7 @@
       <c r="H71">
         <v>177.4</v>
       </c>
-      <c r="J71" s="1">
+      <c r="J71" s="2">
         <v>46418</v>
       </c>
       <c r="K71" t="b">
@@ -3648,7 +3674,7 @@
       <c r="H72">
         <v>200</v>
       </c>
-      <c r="J72" s="1">
+      <c r="J72" s="2">
         <v>46356</v>
       </c>
       <c r="K72" t="b">
@@ -3680,7 +3706,7 @@
       <c r="H73">
         <v>203.6</v>
       </c>
-      <c r="J73" s="1">
+      <c r="J73" s="2">
         <v>46436</v>
       </c>
       <c r="K73" t="b">
@@ -3712,7 +3738,7 @@
       <c r="H74">
         <v>221.2</v>
       </c>
-      <c r="J74" s="1">
+      <c r="J74" s="2">
         <v>46426</v>
       </c>
       <c r="K74" t="b">
@@ -3744,7 +3770,7 @@
       <c r="H75">
         <v>240.8</v>
       </c>
-      <c r="J75" s="1">
+      <c r="J75" s="2">
         <v>46450</v>
       </c>
       <c r="K75" t="b">
@@ -3776,7 +3802,7 @@
       <c r="H76">
         <v>245.8</v>
       </c>
-      <c r="J76" s="1">
+      <c r="J76" s="2">
         <v>46452</v>
       </c>
       <c r="K76" t="b">
@@ -3808,7 +3834,7 @@
       <c r="H77">
         <v>263.4</v>
       </c>
-      <c r="J77" s="1">
+      <c r="J77" s="2">
         <v>46322</v>
       </c>
       <c r="K77" t="b">
@@ -3840,7 +3866,7 @@
       <c r="H78">
         <v>275.2</v>
       </c>
-      <c r="J78" s="1">
+      <c r="J78" s="2">
         <v>46433</v>
       </c>
       <c r="K78" t="b">
@@ -3875,7 +3901,7 @@
       <c r="I79" t="s">
         <v>311</v>
       </c>
-      <c r="J79" s="1">
+      <c r="J79" s="2">
         <v>36557</v>
       </c>
       <c r="K79" t="b">
@@ -3910,7 +3936,7 @@
       <c r="I80" t="s">
         <v>312</v>
       </c>
-      <c r="J80" s="1">
+      <c r="J80" s="2">
         <v>41275</v>
       </c>
       <c r="K80" t="b">
@@ -3945,7 +3971,7 @@
       <c r="I81" t="s">
         <v>313</v>
       </c>
-      <c r="J81" s="1">
+      <c r="J81" s="2">
         <v>45380</v>
       </c>
       <c r="K81" t="b">
@@ -3980,7 +4006,7 @@
       <c r="I82" t="s">
         <v>314</v>
       </c>
-      <c r="J82" s="1">
+      <c r="J82" s="2">
         <v>45421</v>
       </c>
       <c r="K82" t="b">
@@ -4015,7 +4041,7 @@
       <c r="I83" t="s">
         <v>314</v>
       </c>
-      <c r="J83" s="1">
+      <c r="J83" s="2">
         <v>45428</v>
       </c>
       <c r="K83" t="b">
@@ -4050,7 +4076,7 @@
       <c r="I84" t="s">
         <v>315</v>
       </c>
-      <c r="J84" s="1">
+      <c r="J84" s="2">
         <v>45490</v>
       </c>
       <c r="K84" t="b">
@@ -4085,7 +4111,7 @@
       <c r="I85" t="s">
         <v>316</v>
       </c>
-      <c r="J85" s="1">
+      <c r="J85" s="2">
         <v>45566</v>
       </c>
       <c r="K85" t="b">
@@ -4120,7 +4146,7 @@
       <c r="I86" t="s">
         <v>317</v>
       </c>
-      <c r="J86" s="1">
+      <c r="J86" s="2">
         <v>45986</v>
       </c>
       <c r="K86" t="b">
@@ -4155,7 +4181,7 @@
       <c r="I87" t="s">
         <v>318</v>
       </c>
-      <c r="J87" s="1">
+      <c r="J87" s="2">
         <v>46284</v>
       </c>
       <c r="K87" t="b">
@@ -4190,7 +4216,7 @@
       <c r="I88" t="s">
         <v>319</v>
       </c>
-      <c r="J88" s="1">
+      <c r="J88" s="2">
         <v>46305</v>
       </c>
       <c r="K88" t="b">
@@ -4225,7 +4251,7 @@
       <c r="I89" t="s">
         <v>319</v>
       </c>
-      <c r="J89" s="1">
+      <c r="J89" s="2">
         <v>46310</v>
       </c>
       <c r="K89" t="b">
@@ -4260,7 +4286,7 @@
       <c r="I90" t="s">
         <v>319</v>
       </c>
-      <c r="J90" s="1">
+      <c r="J90" s="2">
         <v>46317</v>
       </c>
       <c r="K90" t="b">
@@ -4295,7 +4321,7 @@
       <c r="I91" t="s">
         <v>319</v>
       </c>
-      <c r="J91" s="1">
+      <c r="J91" s="2">
         <v>46319</v>
       </c>
       <c r="K91" t="b">
@@ -4330,7 +4356,7 @@
       <c r="I92" t="s">
         <v>320</v>
       </c>
-      <c r="J92" s="1">
+      <c r="J92" s="2">
         <v>46333</v>
       </c>
       <c r="K92" t="b">
@@ -4365,7 +4391,7 @@
       <c r="I93" t="s">
         <v>320</v>
       </c>
-      <c r="J93" s="1">
+      <c r="J93" s="2">
         <v>46338</v>
       </c>
       <c r="K93" t="b">
@@ -4400,7 +4426,7 @@
       <c r="I94" t="s">
         <v>320</v>
       </c>
-      <c r="J94" s="1">
+      <c r="J94" s="2">
         <v>46338</v>
       </c>
       <c r="K94" t="b">
@@ -4435,7 +4461,7 @@
       <c r="I95" t="s">
         <v>320</v>
       </c>
-      <c r="J95" s="1">
+      <c r="J95" s="2">
         <v>46341</v>
       </c>
       <c r="K95" t="b">
@@ -4470,7 +4496,7 @@
       <c r="I96" t="s">
         <v>320</v>
       </c>
-      <c r="J96" s="1">
+      <c r="J96" s="2">
         <v>46344</v>
       </c>
       <c r="K96" t="b">
@@ -4505,7 +4531,7 @@
       <c r="I97" t="s">
         <v>321</v>
       </c>
-      <c r="J97" s="1">
+      <c r="J97" s="2">
         <v>46360</v>
       </c>
       <c r="K97" t="b">
@@ -4540,7 +4566,7 @@
       <c r="I98" t="s">
         <v>321</v>
       </c>
-      <c r="J98" s="1">
+      <c r="J98" s="2">
         <v>46360</v>
       </c>
       <c r="K98" t="b">
@@ -4575,7 +4601,7 @@
       <c r="I99" t="s">
         <v>321</v>
       </c>
-      <c r="J99" s="1">
+      <c r="J99" s="2">
         <v>46367</v>
       </c>
       <c r="K99" t="b">
@@ -4610,7 +4636,7 @@
       <c r="I100" t="s">
         <v>321</v>
       </c>
-      <c r="J100" s="1">
+      <c r="J100" s="2">
         <v>46375</v>
       </c>
       <c r="K100" t="b">
@@ -4645,7 +4671,7 @@
       <c r="I101" t="s">
         <v>321</v>
       </c>
-      <c r="J101" s="1">
+      <c r="J101" s="2">
         <v>46387</v>
       </c>
       <c r="K101" t="b">
@@ -4680,7 +4706,7 @@
       <c r="I102" t="s">
         <v>321</v>
       </c>
-      <c r="J102" s="1">
+      <c r="J102" s="2">
         <v>46387</v>
       </c>
       <c r="K102" t="b">
@@ -4715,7 +4741,7 @@
       <c r="I103" t="s">
         <v>321</v>
       </c>
-      <c r="J103" s="1">
+      <c r="J103" s="2">
         <v>46387</v>
       </c>
       <c r="K103" t="b">
@@ -4750,7 +4776,7 @@
       <c r="I104" t="s">
         <v>321</v>
       </c>
-      <c r="J104" s="1">
+      <c r="J104" s="2">
         <v>46388</v>
       </c>
       <c r="K104" t="b">
@@ -4785,7 +4811,7 @@
       <c r="I105" t="s">
         <v>322</v>
       </c>
-      <c r="J105" s="1">
+      <c r="J105" s="2">
         <v>46401</v>
       </c>
       <c r="K105" t="b">
@@ -4820,7 +4846,7 @@
       <c r="I106" t="s">
         <v>322</v>
       </c>
-      <c r="J106" s="1">
+      <c r="J106" s="2">
         <v>46401</v>
       </c>
       <c r="K106" t="b">
@@ -4855,7 +4881,7 @@
       <c r="I107" t="s">
         <v>322</v>
       </c>
-      <c r="J107" s="1">
+      <c r="J107" s="2">
         <v>46401</v>
       </c>
       <c r="K107" t="b">
@@ -4890,7 +4916,7 @@
       <c r="I108" t="s">
         <v>322</v>
       </c>
-      <c r="J108" s="1">
+      <c r="J108" s="2">
         <v>46412</v>
       </c>
       <c r="K108" t="b">
@@ -4925,7 +4951,7 @@
       <c r="I109" t="s">
         <v>322</v>
       </c>
-      <c r="J109" s="1">
+      <c r="J109" s="2">
         <v>46412</v>
       </c>
       <c r="K109" t="b">
@@ -4960,7 +4986,7 @@
       <c r="I110" t="s">
         <v>322</v>
       </c>
-      <c r="J110" s="1">
+      <c r="J110" s="2">
         <v>46412</v>
       </c>
       <c r="K110" t="b">
@@ -4995,7 +5021,7 @@
       <c r="I111" t="s">
         <v>323</v>
       </c>
-      <c r="J111" s="1">
+      <c r="J111" s="2">
         <v>46424</v>
       </c>
       <c r="K111" t="b">
@@ -5030,7 +5056,7 @@
       <c r="I112" t="s">
         <v>323</v>
       </c>
-      <c r="J112" s="1">
+      <c r="J112" s="2">
         <v>46437</v>
       </c>
       <c r="K112" t="b">
@@ -5065,7 +5091,7 @@
       <c r="I113" t="s">
         <v>323</v>
       </c>
-      <c r="J113" s="1">
+      <c r="J113" s="2">
         <v>46451</v>
       </c>
       <c r="K113" t="b">
@@ -5100,7 +5126,7 @@
       <c r="I114" t="s">
         <v>323</v>
       </c>
-      <c r="J114" s="1">
+      <c r="J114" s="2">
         <v>46451</v>
       </c>
       <c r="K114" t="b">
@@ -5135,7 +5161,7 @@
       <c r="I115" t="s">
         <v>324</v>
       </c>
-      <c r="J115" s="1">
+      <c r="J115" s="2">
         <v>46455</v>
       </c>
       <c r="K115" t="b">
@@ -5170,7 +5196,7 @@
       <c r="I116" t="s">
         <v>324</v>
       </c>
-      <c r="J116" s="1">
+      <c r="J116" s="2">
         <v>46456</v>
       </c>
       <c r="K116" t="b">
@@ -5205,7 +5231,7 @@
       <c r="I117" t="s">
         <v>324</v>
       </c>
-      <c r="J117" s="1">
+      <c r="J117" s="2">
         <v>46457</v>
       </c>
       <c r="K117" t="b">
@@ -5240,7 +5266,7 @@
       <c r="I118" t="s">
         <v>324</v>
       </c>
-      <c r="J118" s="1">
+      <c r="J118" s="2">
         <v>46464</v>
       </c>
       <c r="K118" t="b">
@@ -5275,7 +5301,7 @@
       <c r="I119" t="s">
         <v>324</v>
       </c>
-      <c r="J119" s="1">
+      <c r="J119" s="2">
         <v>46470</v>
       </c>
       <c r="K119" t="b">
@@ -5310,7 +5336,7 @@
       <c r="I120" t="s">
         <v>325</v>
       </c>
-      <c r="J120" s="1">
+      <c r="J120" s="2">
         <v>46485</v>
       </c>
       <c r="K120" t="b">
@@ -5345,7 +5371,7 @@
       <c r="I121" t="s">
         <v>325</v>
       </c>
-      <c r="J121" s="1">
+      <c r="J121" s="2">
         <v>46499</v>
       </c>
       <c r="K121" t="b">
@@ -5380,7 +5406,7 @@
       <c r="I122" t="s">
         <v>325</v>
       </c>
-      <c r="J122" s="1">
+      <c r="J122" s="2">
         <v>46504</v>
       </c>
       <c r="K122" t="b">
@@ -5415,7 +5441,7 @@
       <c r="I123" t="s">
         <v>325</v>
       </c>
-      <c r="J123" s="1">
+      <c r="J123" s="2">
         <v>46504</v>
       </c>
       <c r="K123" t="b">
@@ -5450,7 +5476,7 @@
       <c r="I124" t="s">
         <v>325</v>
       </c>
-      <c r="J124" s="1">
+      <c r="J124" s="2">
         <v>46507</v>
       </c>
       <c r="K124" t="b">
@@ -5485,7 +5511,7 @@
       <c r="I125" t="s">
         <v>325</v>
       </c>
-      <c r="J125" s="1">
+      <c r="J125" s="2">
         <v>46508</v>
       </c>
       <c r="K125" t="b">
@@ -5520,7 +5546,7 @@
       <c r="I126" t="s">
         <v>325</v>
       </c>
-      <c r="J126" s="1">
+      <c r="J126" s="2">
         <v>46512</v>
       </c>
       <c r="K126" t="b">
@@ -5555,7 +5581,7 @@
       <c r="I127" t="s">
         <v>326</v>
       </c>
-      <c r="J127" s="1">
+      <c r="J127" s="2">
         <v>46512</v>
       </c>
       <c r="K127" t="b">
@@ -5590,7 +5616,7 @@
       <c r="I128" t="s">
         <v>326</v>
       </c>
-      <c r="J128" s="1">
+      <c r="J128" s="2">
         <v>46528</v>
       </c>
       <c r="K128" t="b">
@@ -5625,7 +5651,7 @@
       <c r="I129" t="s">
         <v>326</v>
       </c>
-      <c r="J129" s="1">
+      <c r="J129" s="2">
         <v>46529</v>
       </c>
       <c r="K129" t="b">
@@ -5660,7 +5686,7 @@
       <c r="I130" t="s">
         <v>326</v>
       </c>
-      <c r="J130" s="1">
+      <c r="J130" s="2">
         <v>46537</v>
       </c>
       <c r="K130" t="b">
@@ -5695,7 +5721,7 @@
       <c r="I131" t="s">
         <v>327</v>
       </c>
-      <c r="J131" s="1">
+      <c r="J131" s="2">
         <v>46546</v>
       </c>
       <c r="K131" t="b">
@@ -5730,7 +5756,7 @@
       <c r="I132" t="s">
         <v>327</v>
       </c>
-      <c r="J132" s="1">
+      <c r="J132" s="2">
         <v>46547</v>
       </c>
       <c r="K132" t="b">
@@ -5765,7 +5791,7 @@
       <c r="I133" t="s">
         <v>327</v>
       </c>
-      <c r="J133" s="1">
+      <c r="J133" s="2">
         <v>46547</v>
       </c>
       <c r="K133" t="b">
@@ -5800,7 +5826,7 @@
       <c r="I134" t="s">
         <v>327</v>
       </c>
-      <c r="J134" s="1">
+      <c r="J134" s="2">
         <v>46547</v>
       </c>
       <c r="K134" t="b">
@@ -5835,7 +5861,7 @@
       <c r="I135" t="s">
         <v>327</v>
       </c>
-      <c r="J135" s="1">
+      <c r="J135" s="2">
         <v>46551</v>
       </c>
       <c r="K135" t="b">
@@ -5870,7 +5896,7 @@
       <c r="I136" t="s">
         <v>327</v>
       </c>
-      <c r="J136" s="1">
+      <c r="J136" s="2">
         <v>46560</v>
       </c>
       <c r="K136" t="b">
@@ -5905,7 +5931,7 @@
       <c r="I137" t="s">
         <v>327</v>
       </c>
-      <c r="J137" s="1">
+      <c r="J137" s="2">
         <v>46564</v>
       </c>
       <c r="K137" t="b">
@@ -5940,7 +5966,7 @@
       <c r="I138" t="s">
         <v>327</v>
       </c>
-      <c r="J138" s="1">
+      <c r="J138" s="2">
         <v>46567</v>
       </c>
       <c r="K138" t="b">
@@ -5975,7 +6001,7 @@
       <c r="I139" t="s">
         <v>327</v>
       </c>
-      <c r="J139" s="1">
+      <c r="J139" s="2">
         <v>46568</v>
       </c>
       <c r="K139" t="b">
@@ -6010,7 +6036,7 @@
       <c r="I140" t="s">
         <v>328</v>
       </c>
-      <c r="J140" s="1">
+      <c r="J140" s="2">
         <v>46578</v>
       </c>
       <c r="K140" t="b">
@@ -6045,7 +6071,7 @@
       <c r="I141" t="s">
         <v>328</v>
       </c>
-      <c r="J141" s="1">
+      <c r="J141" s="2">
         <v>46592</v>
       </c>
       <c r="K141" t="b">
@@ -6080,7 +6106,7 @@
       <c r="I142" t="s">
         <v>328</v>
       </c>
-      <c r="J142" s="1">
+      <c r="J142" s="2">
         <v>46592</v>
       </c>
       <c r="K142" t="b">
@@ -6115,7 +6141,7 @@
       <c r="I143" t="s">
         <v>329</v>
       </c>
-      <c r="J143" s="1">
+      <c r="J143" s="2">
         <v>46212</v>
       </c>
       <c r="K143" t="b">
@@ -6150,7 +6176,7 @@
       <c r="I144" t="s">
         <v>330</v>
       </c>
-      <c r="J144" s="1">
+      <c r="J144" s="2">
         <v>46225</v>
       </c>
       <c r="K144" t="b">
@@ -6185,7 +6211,7 @@
       <c r="I145" t="s">
         <v>331</v>
       </c>
-      <c r="J145" s="1">
+      <c r="J145" s="2">
         <v>46263</v>
       </c>
       <c r="K145" t="b">
@@ -6217,7 +6243,7 @@
       <c r="H146">
         <v>-1476</v>
       </c>
-      <c r="J146" s="1">
+      <c r="J146" s="2">
         <v>43773</v>
       </c>
       <c r="K146" t="b">
@@ -6249,7 +6275,7 @@
       <c r="H147">
         <v>-1469</v>
       </c>
-      <c r="J147" s="1">
+      <c r="J147" s="2">
         <v>43773</v>
       </c>
       <c r="K147" t="b">
@@ -6281,7 +6307,7 @@
       <c r="H148">
         <v>-1186</v>
       </c>
-      <c r="J148" s="1">
+      <c r="J148" s="2">
         <v>45295</v>
       </c>
       <c r="K148" t="b">
@@ -6313,7 +6339,7 @@
       <c r="H149">
         <v>-1048</v>
       </c>
-      <c r="J149" s="1">
+      <c r="J149" s="2">
         <v>45617</v>
       </c>
       <c r="K149" t="b">
@@ -6345,7 +6371,7 @@
       <c r="H150">
         <v>-980</v>
       </c>
-      <c r="J150" s="1">
+      <c r="J150" s="2">
         <v>45677</v>
       </c>
       <c r="K150" t="b">
@@ -6377,7 +6403,7 @@
       <c r="H151">
         <v>-961</v>
       </c>
-      <c r="J151" s="1">
+      <c r="J151" s="2">
         <v>44944</v>
       </c>
       <c r="K151" t="b">
@@ -6409,7 +6435,7 @@
       <c r="H152">
         <v>-252</v>
       </c>
-      <c r="J152" s="1">
+      <c r="J152" s="2">
         <v>46092</v>
       </c>
       <c r="K152" t="b">
@@ -6441,7 +6467,7 @@
       <c r="H153">
         <v>3</v>
       </c>
-      <c r="J153" s="1">
+      <c r="J153" s="2">
         <v>46265</v>
       </c>
       <c r="K153" t="b">
@@ -6473,7 +6499,7 @@
       <c r="H154">
         <v>3</v>
       </c>
-      <c r="J154" s="1">
+      <c r="J154" s="2">
         <v>46265</v>
       </c>
       <c r="K154" t="b">
@@ -6505,7 +6531,7 @@
       <c r="H155">
         <v>43</v>
       </c>
-      <c r="J155" s="1">
+      <c r="J155" s="2">
         <v>46440</v>
       </c>
       <c r="K155" t="b">
@@ -6537,7 +6563,7 @@
       <c r="H156">
         <v>43</v>
       </c>
-      <c r="J156" s="1">
+      <c r="J156" s="2">
         <v>46440</v>
       </c>
       <c r="K156" t="b">
@@ -6569,7 +6595,7 @@
       <c r="H157">
         <v>72</v>
       </c>
-      <c r="J157" s="1">
+      <c r="J157" s="2">
         <v>46289</v>
       </c>
       <c r="K157" t="b">
@@ -6601,7 +6627,7 @@
       <c r="H158">
         <v>72</v>
       </c>
-      <c r="J158" s="1">
+      <c r="J158" s="2">
         <v>46289</v>
       </c>
       <c r="K158" t="b">
@@ -6633,7 +6659,7 @@
       <c r="H159">
         <v>81</v>
       </c>
-      <c r="J159" s="1">
+      <c r="J159" s="2">
         <v>46405</v>
       </c>
       <c r="K159" t="b">
@@ -6665,7 +6691,7 @@
       <c r="H160">
         <v>102</v>
       </c>
-      <c r="J160" s="1">
+      <c r="J160" s="2">
         <v>46463</v>
       </c>
       <c r="K160" t="b">
@@ -6697,7 +6723,7 @@
       <c r="H161">
         <v>109</v>
       </c>
-      <c r="J161" s="1">
+      <c r="J161" s="2">
         <v>46353</v>
       </c>
       <c r="K161" t="b">
@@ -6729,7 +6755,7 @@
       <c r="H162">
         <v>127</v>
       </c>
-      <c r="J162" s="1">
+      <c r="J162" s="2">
         <v>46417</v>
       </c>
       <c r="K162" t="b">
@@ -6761,7 +6787,7 @@
       <c r="H163">
         <v>152</v>
       </c>
-      <c r="J163" s="1">
+      <c r="J163" s="2">
         <v>46271</v>
       </c>
       <c r="K163" t="b">
@@ -6793,7 +6819,7 @@
       <c r="H164">
         <v>152</v>
       </c>
-      <c r="J164" s="1">
+      <c r="J164" s="2">
         <v>46271</v>
       </c>
       <c r="K164" t="b">
@@ -6825,7 +6851,7 @@
       <c r="H165">
         <v>153</v>
       </c>
-      <c r="J165" s="1">
+      <c r="J165" s="2">
         <v>46458</v>
       </c>
       <c r="K165" t="b">
@@ -6857,7 +6883,7 @@
       <c r="H166">
         <v>158</v>
       </c>
-      <c r="J166" s="1">
+      <c r="J166" s="2">
         <v>46381</v>
       </c>
       <c r="K166" t="b">
@@ -6889,7 +6915,7 @@
       <c r="H167">
         <v>163</v>
       </c>
-      <c r="J167" s="1">
+      <c r="J167" s="2">
         <v>46592</v>
       </c>
       <c r="K167" t="b">
@@ -6921,7 +6947,7 @@
       <c r="H168">
         <v>167</v>
       </c>
-      <c r="J168" s="1">
+      <c r="J168" s="2">
         <v>46441</v>
       </c>
       <c r="K168" t="b">
@@ -6953,7 +6979,7 @@
       <c r="H169">
         <v>169</v>
       </c>
-      <c r="J169" s="1">
+      <c r="J169" s="2">
         <v>46391</v>
       </c>
       <c r="K169" t="b">
@@ -6985,7 +7011,7 @@
       <c r="H170">
         <v>184</v>
       </c>
-      <c r="J170" s="1">
+      <c r="J170" s="2">
         <v>46385</v>
       </c>
       <c r="K170" t="b">
@@ -7017,7 +7043,7 @@
       <c r="H171">
         <v>186</v>
       </c>
-      <c r="J171" s="1">
+      <c r="J171" s="2">
         <v>46387</v>
       </c>
       <c r="K171" t="b">
@@ -7049,7 +7075,7 @@
       <c r="H172">
         <v>206</v>
       </c>
-      <c r="J172" s="1">
+      <c r="J172" s="2">
         <v>46399</v>
       </c>
       <c r="K172" t="b">
@@ -7081,7 +7107,7 @@
       <c r="H173">
         <v>206</v>
       </c>
-      <c r="J173" s="1">
+      <c r="J173" s="2">
         <v>46399</v>
       </c>
       <c r="K173" t="b">
@@ -7113,7 +7139,7 @@
       <c r="H174">
         <v>234</v>
       </c>
-      <c r="J174" s="1">
+      <c r="J174" s="2">
         <v>46458</v>
       </c>
       <c r="K174" t="b">
@@ -7145,7 +7171,7 @@
       <c r="H175">
         <v>248</v>
       </c>
-      <c r="J175" s="1">
+      <c r="J175" s="2">
         <v>46528</v>
       </c>
       <c r="K175" t="b">
@@ -7177,7 +7203,7 @@
       <c r="H176">
         <v>317</v>
       </c>
-      <c r="J176" s="1">
+      <c r="J176" s="2">
         <v>46540</v>
       </c>
       <c r="K176" t="b">
@@ -7209,7 +7235,7 @@
       <c r="H177">
         <v>340</v>
       </c>
-      <c r="J177" s="1">
+      <c r="J177" s="2">
         <v>46547</v>
       </c>
       <c r="K177" t="b">
@@ -7241,7 +7267,7 @@
       <c r="H178">
         <v>364</v>
       </c>
-      <c r="J178" s="1">
+      <c r="J178" s="2">
         <v>46557</v>
       </c>
       <c r="K178" t="b">
@@ -7273,7 +7299,7 @@
       <c r="H179">
         <v>368</v>
       </c>
-      <c r="J179" s="1">
+      <c r="J179" s="2">
         <v>46571</v>
       </c>
       <c r="K179" t="b">
@@ -7305,7 +7331,7 @@
       <c r="H180">
         <v>368</v>
       </c>
-      <c r="J180" s="1">
+      <c r="J180" s="2">
         <v>46571</v>
       </c>
       <c r="K180" t="b">
@@ -7337,7 +7363,7 @@
       <c r="H181">
         <v>370</v>
       </c>
-      <c r="J181" s="1">
+      <c r="J181" s="2">
         <v>46562</v>
       </c>
       <c r="K181" t="b">
@@ -7369,7 +7395,7 @@
       <c r="H182">
         <v>385</v>
       </c>
-      <c r="J182" s="1">
+      <c r="J182" s="2">
         <v>46574</v>
       </c>
       <c r="K182" t="b">
@@ -7401,7 +7427,7 @@
       <c r="H183">
         <v>385</v>
       </c>
-      <c r="J183" s="1">
+      <c r="J183" s="2">
         <v>46574</v>
       </c>
       <c r="K183" t="b">
@@ -7433,7 +7459,7 @@
       <c r="H184">
         <v>417</v>
       </c>
-      <c r="J184" s="1">
+      <c r="J184" s="2">
         <v>46578</v>
       </c>
       <c r="K184" t="b">
@@ -7465,7 +7491,7 @@
       <c r="H185">
         <v>721</v>
       </c>
-      <c r="J185" s="1">
+      <c r="J185" s="2">
         <v>46345</v>
       </c>
       <c r="K185" t="b">
@@ -7497,7 +7523,7 @@
       <c r="H186">
         <v>721</v>
       </c>
-      <c r="J186" s="1">
+      <c r="J186" s="2">
         <v>46345</v>
       </c>
       <c r="K186" t="b">
@@ -7529,7 +7555,7 @@
       <c r="H187">
         <v>850</v>
       </c>
-      <c r="J187" s="1">
+      <c r="J187" s="2">
         <v>46366</v>
       </c>
       <c r="K187" t="b">
@@ -7561,7 +7587,7 @@
       <c r="H188">
         <v>850</v>
       </c>
-      <c r="J188" s="1">
+      <c r="J188" s="2">
         <v>46366</v>
       </c>
       <c r="K188" t="b">
@@ -7593,7 +7619,7 @@
       <c r="H189">
         <v>1661</v>
       </c>
-      <c r="J189" s="1">
+      <c r="J189" s="2">
         <v>46524</v>
       </c>
       <c r="K189" t="b">
@@ -7625,7 +7651,7 @@
       <c r="H190">
         <v>1661</v>
       </c>
-      <c r="J190" s="1">
+      <c r="J190" s="2">
         <v>46524</v>
       </c>
       <c r="K190" t="b">
@@ -7657,7 +7683,7 @@
       <c r="H191">
         <v>488</v>
       </c>
-      <c r="J191" s="1">
+      <c r="J191" s="2">
         <v>46190</v>
       </c>
       <c r="K191" t="b">
@@ -7689,7 +7715,7 @@
       <c r="H192">
         <v>25565</v>
       </c>
-      <c r="J192" s="1">
+      <c r="J192" s="2">
         <v>46190</v>
       </c>
       <c r="K192" t="b">
@@ -7721,7 +7747,7 @@
       <c r="H193">
         <v>25567</v>
       </c>
-      <c r="J193" s="1">
+      <c r="J193" s="2">
         <v>46190</v>
       </c>
       <c r="K193" t="b">
@@ -7753,7 +7779,7 @@
       <c r="H194">
         <v>31293</v>
       </c>
-      <c r="J194" s="1">
+      <c r="J194" s="2">
         <v>46190</v>
       </c>
       <c r="K194" t="b">

</xml_diff>

<commit_message>
Atualização automática: vencimentos_tmot (04/09/2026 11:55)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
@@ -1019,16 +1019,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1044,7 +1036,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1052,30 +1044,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1375,37 +1349,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1434,7 +1408,7 @@
       <c r="H2">
         <v>-4300.3</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>39285</v>
       </c>
       <c r="K2" t="b">
@@ -1466,7 +1440,7 @@
       <c r="H3">
         <v>-2354.2</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>40669</v>
       </c>
       <c r="K3" t="b">
@@ -1498,7 +1472,7 @@
       <c r="H4">
         <v>-910.7</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>40669</v>
       </c>
       <c r="K4" t="b">
@@ -1530,7 +1504,7 @@
       <c r="H5">
         <v>-868</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>44884</v>
       </c>
       <c r="K5" t="b">
@@ -1562,7 +1536,7 @@
       <c r="H6">
         <v>-483.8</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>43855</v>
       </c>
       <c r="K6" t="b">
@@ -1594,7 +1568,7 @@
       <c r="H7">
         <v>-417</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>46014</v>
       </c>
       <c r="K7" t="b">
@@ -1626,7 +1600,7 @@
       <c r="H8">
         <v>-414.2</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>46014</v>
       </c>
       <c r="K8" t="b">
@@ -1658,7 +1632,7 @@
       <c r="H9">
         <v>-391.8</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>42769</v>
       </c>
       <c r="K9" t="b">
@@ -1690,7 +1664,7 @@
       <c r="H10">
         <v>-391.6</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>45804</v>
       </c>
       <c r="K10" t="b">
@@ -1722,7 +1696,7 @@
       <c r="H11">
         <v>-391.6</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>45804</v>
       </c>
       <c r="K11" t="b">
@@ -1754,7 +1728,7 @@
       <c r="H12">
         <v>-372.9</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>42821</v>
       </c>
       <c r="K12" t="b">
@@ -1786,7 +1760,7 @@
       <c r="H13">
         <v>-372.9</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>46014</v>
       </c>
       <c r="K13" t="b">
@@ -1818,7 +1792,7 @@
       <c r="H14">
         <v>-372.9</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>46014</v>
       </c>
       <c r="K14" t="b">
@@ -1850,7 +1824,7 @@
       <c r="H15">
         <v>-372.9</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <v>46014</v>
       </c>
       <c r="K15" t="b">
@@ -1882,7 +1856,7 @@
       <c r="H16">
         <v>-367.8</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <v>46017</v>
       </c>
       <c r="K16" t="b">
@@ -1914,7 +1888,7 @@
       <c r="H17">
         <v>-367.8</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="1">
         <v>46017</v>
       </c>
       <c r="K17" t="b">
@@ -1946,7 +1920,7 @@
       <c r="H18">
         <v>-347.2</v>
       </c>
-      <c r="J18" s="2">
+      <c r="J18" s="1">
         <v>40979</v>
       </c>
       <c r="K18" t="b">
@@ -1978,7 +1952,7 @@
       <c r="H19">
         <v>-293.8</v>
       </c>
-      <c r="J19" s="2">
+      <c r="J19" s="1">
         <v>45846</v>
       </c>
       <c r="K19" t="b">
@@ -2010,7 +1984,7 @@
       <c r="H20">
         <v>-206.4</v>
       </c>
-      <c r="J20" s="2">
+      <c r="J20" s="1">
         <v>36669</v>
       </c>
       <c r="K20" t="b">
@@ -2042,7 +2016,7 @@
       <c r="H21">
         <v>-131.6</v>
       </c>
-      <c r="J21" s="2">
+      <c r="J21" s="1">
         <v>46111</v>
       </c>
       <c r="K21" t="b">
@@ -2074,7 +2048,7 @@
       <c r="H22">
         <v>-131.6</v>
       </c>
-      <c r="J22" s="2">
+      <c r="J22" s="1">
         <v>46111</v>
       </c>
       <c r="K22" t="b">
@@ -2106,7 +2080,7 @@
       <c r="H23">
         <v>-131.6</v>
       </c>
-      <c r="J23" s="2">
+      <c r="J23" s="1">
         <v>46111</v>
       </c>
       <c r="K23" t="b">
@@ -2138,7 +2112,7 @@
       <c r="H24">
         <v>-131.6</v>
       </c>
-      <c r="J24" s="2">
+      <c r="J24" s="1">
         <v>46111</v>
       </c>
       <c r="K24" t="b">
@@ -2170,7 +2144,7 @@
       <c r="H25">
         <v>-131.6</v>
       </c>
-      <c r="J25" s="2">
+      <c r="J25" s="1">
         <v>46111</v>
       </c>
       <c r="K25" t="b">
@@ -2202,7 +2176,7 @@
       <c r="H26">
         <v>-98.3</v>
       </c>
-      <c r="J26" s="2">
+      <c r="J26" s="1">
         <v>41204</v>
       </c>
       <c r="K26" t="b">
@@ -2234,7 +2208,7 @@
       <c r="H27">
         <v>-47.2</v>
       </c>
-      <c r="J27" s="2">
+      <c r="J27" s="1">
         <v>44011</v>
       </c>
       <c r="K27" t="b">
@@ -2266,7 +2240,7 @@
       <c r="H28">
         <v>-22.3</v>
       </c>
-      <c r="J28" s="2">
+      <c r="J28" s="1">
         <v>46226</v>
       </c>
       <c r="K28" t="b">
@@ -2298,7 +2272,7 @@
       <c r="H29">
         <v>4.7</v>
       </c>
-      <c r="J29" s="2">
+      <c r="J29" s="1">
         <v>46265</v>
       </c>
       <c r="K29" t="b">
@@ -2330,7 +2304,7 @@
       <c r="H30">
         <v>7.5</v>
       </c>
-      <c r="J30" s="2">
+      <c r="J30" s="1">
         <v>46265</v>
       </c>
       <c r="K30" t="b">
@@ -2362,7 +2336,7 @@
       <c r="H31">
         <v>10</v>
       </c>
-      <c r="J31" s="2">
+      <c r="J31" s="1">
         <v>46265</v>
       </c>
       <c r="K31" t="b">
@@ -2394,7 +2368,7 @@
       <c r="H32">
         <v>12.8</v>
       </c>
-      <c r="J32" s="2">
+      <c r="J32" s="1">
         <v>46265</v>
       </c>
       <c r="K32" t="b">
@@ -2426,7 +2400,7 @@
       <c r="H33">
         <v>14</v>
       </c>
-      <c r="J33" s="2">
+      <c r="J33" s="1">
         <v>46265</v>
       </c>
       <c r="K33" t="b">
@@ -2458,7 +2432,7 @@
       <c r="H34">
         <v>17.8</v>
       </c>
-      <c r="J34" s="2">
+      <c r="J34" s="1">
         <v>46265</v>
       </c>
       <c r="K34" t="b">
@@ -2490,7 +2464,7 @@
       <c r="H35">
         <v>20.4</v>
       </c>
-      <c r="J35" s="2">
+      <c r="J35" s="1">
         <v>46265</v>
       </c>
       <c r="K35" t="b">
@@ -2522,7 +2496,7 @@
       <c r="H36">
         <v>21.2</v>
       </c>
-      <c r="J36" s="2">
+      <c r="J36" s="1">
         <v>46265</v>
       </c>
       <c r="K36" t="b">
@@ -2554,7 +2528,7 @@
       <c r="H37">
         <v>26.2</v>
       </c>
-      <c r="J37" s="2">
+      <c r="J37" s="1">
         <v>46265</v>
       </c>
       <c r="K37" t="b">
@@ -2586,7 +2560,7 @@
       <c r="H38">
         <v>33.6</v>
       </c>
-      <c r="J38" s="2">
+      <c r="J38" s="1">
         <v>46364</v>
       </c>
       <c r="K38" t="b">
@@ -2618,7 +2592,7 @@
       <c r="H39">
         <v>42.2</v>
       </c>
-      <c r="J39" s="2">
+      <c r="J39" s="1">
         <v>46269</v>
       </c>
       <c r="K39" t="b">
@@ -2650,7 +2624,7 @@
       <c r="H40">
         <v>42.8</v>
       </c>
-      <c r="J40" s="2">
+      <c r="J40" s="1">
         <v>46291</v>
       </c>
       <c r="K40" t="b">
@@ -2682,7 +2656,7 @@
       <c r="H41">
         <v>45.7</v>
       </c>
-      <c r="J41" s="2">
+      <c r="J41" s="1">
         <v>46395</v>
       </c>
       <c r="K41" t="b">
@@ -2714,7 +2688,7 @@
       <c r="H42">
         <v>47.2</v>
       </c>
-      <c r="J42" s="2">
+      <c r="J42" s="1">
         <v>46280</v>
       </c>
       <c r="K42" t="b">
@@ -2746,7 +2720,7 @@
       <c r="H43">
         <v>48.7</v>
       </c>
-      <c r="J43" s="2">
+      <c r="J43" s="1">
         <v>46281</v>
       </c>
       <c r="K43" t="b">
@@ -2778,7 +2752,7 @@
       <c r="H44">
         <v>60</v>
       </c>
-      <c r="J44" s="2">
+      <c r="J44" s="1">
         <v>46281</v>
       </c>
       <c r="K44" t="b">
@@ -2810,7 +2784,7 @@
       <c r="H45">
         <v>62.6</v>
       </c>
-      <c r="J45" s="2">
+      <c r="J45" s="1">
         <v>46265</v>
       </c>
       <c r="K45" t="b">
@@ -2842,7 +2816,7 @@
       <c r="H46">
         <v>64.59999999999999</v>
       </c>
-      <c r="J46" s="2">
+      <c r="J46" s="1">
         <v>46265</v>
       </c>
       <c r="K46" t="b">
@@ -2874,7 +2848,7 @@
       <c r="H47">
         <v>67.59999999999999</v>
       </c>
-      <c r="J47" s="2">
+      <c r="J47" s="1">
         <v>46267</v>
       </c>
       <c r="K47" t="b">
@@ -2906,7 +2880,7 @@
       <c r="H48">
         <v>68.3</v>
       </c>
-      <c r="J48" s="2">
+      <c r="J48" s="1">
         <v>46278</v>
       </c>
       <c r="K48" t="b">
@@ -2938,7 +2912,7 @@
       <c r="H49">
         <v>69.2</v>
       </c>
-      <c r="J49" s="2">
+      <c r="J49" s="1">
         <v>46453</v>
       </c>
       <c r="K49" t="b">
@@ -2970,7 +2944,7 @@
       <c r="H50">
         <v>69.8</v>
       </c>
-      <c r="J50" s="2">
+      <c r="J50" s="1">
         <v>46265</v>
       </c>
       <c r="K50" t="b">
@@ -3002,7 +2976,7 @@
       <c r="H51">
         <v>69.8</v>
       </c>
-      <c r="J51" s="2">
+      <c r="J51" s="1">
         <v>46265</v>
       </c>
       <c r="K51" t="b">
@@ -3034,7 +3008,7 @@
       <c r="H52">
         <v>72.2</v>
       </c>
-      <c r="J52" s="2">
+      <c r="J52" s="1">
         <v>46275</v>
       </c>
       <c r="K52" t="b">
@@ -3066,7 +3040,7 @@
       <c r="H53">
         <v>72.2</v>
       </c>
-      <c r="J53" s="2">
+      <c r="J53" s="1">
         <v>46275</v>
       </c>
       <c r="K53" t="b">
@@ -3098,7 +3072,7 @@
       <c r="H54">
         <v>78.09999999999999</v>
       </c>
-      <c r="J54" s="2">
+      <c r="J54" s="1">
         <v>46265</v>
       </c>
       <c r="K54" t="b">
@@ -3130,7 +3104,7 @@
       <c r="H55">
         <v>82.8</v>
       </c>
-      <c r="J55" s="2">
+      <c r="J55" s="1">
         <v>46487</v>
       </c>
       <c r="K55" t="b">
@@ -3162,7 +3136,7 @@
       <c r="H56">
         <v>83.09999999999999</v>
       </c>
-      <c r="J56" s="2">
+      <c r="J56" s="1">
         <v>46285</v>
       </c>
       <c r="K56" t="b">
@@ -3194,7 +3168,7 @@
       <c r="H57">
         <v>84.8</v>
       </c>
-      <c r="J57" s="2">
+      <c r="J57" s="1">
         <v>46492</v>
       </c>
       <c r="K57" t="b">
@@ -3226,7 +3200,7 @@
       <c r="H58">
         <v>104.9</v>
       </c>
-      <c r="J58" s="2">
+      <c r="J58" s="1">
         <v>46297</v>
       </c>
       <c r="K58" t="b">
@@ -3258,7 +3232,7 @@
       <c r="H59">
         <v>107.6</v>
       </c>
-      <c r="J59" s="2">
+      <c r="J59" s="1">
         <v>46283</v>
       </c>
       <c r="K59" t="b">
@@ -3290,7 +3264,7 @@
       <c r="H60">
         <v>111.9</v>
       </c>
-      <c r="J60" s="2">
+      <c r="J60" s="1">
         <v>46300</v>
       </c>
       <c r="K60" t="b">
@@ -3322,7 +3296,7 @@
       <c r="H61">
         <v>111.9</v>
       </c>
-      <c r="J61" s="2">
+      <c r="J61" s="1">
         <v>46300</v>
       </c>
       <c r="K61" t="b">
@@ -3354,7 +3328,7 @@
       <c r="H62">
         <v>111.9</v>
       </c>
-      <c r="J62" s="2">
+      <c r="J62" s="1">
         <v>46300</v>
       </c>
       <c r="K62" t="b">
@@ -3386,7 +3360,7 @@
       <c r="H63">
         <v>111.9</v>
       </c>
-      <c r="J63" s="2">
+      <c r="J63" s="1">
         <v>46300</v>
       </c>
       <c r="K63" t="b">
@@ -3418,7 +3392,7 @@
       <c r="H64">
         <v>111.9</v>
       </c>
-      <c r="J64" s="2">
+      <c r="J64" s="1">
         <v>46300</v>
       </c>
       <c r="K64" t="b">
@@ -3450,7 +3424,7 @@
       <c r="H65">
         <v>128.8</v>
       </c>
-      <c r="J65" s="2">
+      <c r="J65" s="1">
         <v>46308</v>
       </c>
       <c r="K65" t="b">
@@ -3482,7 +3456,7 @@
       <c r="H66">
         <v>131.1</v>
       </c>
-      <c r="J66" s="2">
+      <c r="J66" s="1">
         <v>46336</v>
       </c>
       <c r="K66" t="b">
@@ -3514,7 +3488,7 @@
       <c r="H67">
         <v>138.4</v>
       </c>
-      <c r="J67" s="2">
+      <c r="J67" s="1">
         <v>46343</v>
       </c>
       <c r="K67" t="b">
@@ -3546,7 +3520,7 @@
       <c r="H68">
         <v>141</v>
       </c>
-      <c r="J68" s="2">
+      <c r="J68" s="1">
         <v>46350</v>
       </c>
       <c r="K68" t="b">
@@ -3578,7 +3552,7 @@
       <c r="H69">
         <v>162</v>
       </c>
-      <c r="J69" s="2">
+      <c r="J69" s="1">
         <v>46391</v>
       </c>
       <c r="K69" t="b">
@@ -3610,7 +3584,7 @@
       <c r="H70">
         <v>167.2</v>
       </c>
-      <c r="J70" s="2">
+      <c r="J70" s="1">
         <v>46330</v>
       </c>
       <c r="K70" t="b">
@@ -3642,7 +3616,7 @@
       <c r="H71">
         <v>177.4</v>
       </c>
-      <c r="J71" s="2">
+      <c r="J71" s="1">
         <v>46418</v>
       </c>
       <c r="K71" t="b">
@@ -3674,7 +3648,7 @@
       <c r="H72">
         <v>200</v>
       </c>
-      <c r="J72" s="2">
+      <c r="J72" s="1">
         <v>46356</v>
       </c>
       <c r="K72" t="b">
@@ -3706,7 +3680,7 @@
       <c r="H73">
         <v>203.6</v>
       </c>
-      <c r="J73" s="2">
+      <c r="J73" s="1">
         <v>46436</v>
       </c>
       <c r="K73" t="b">
@@ -3738,7 +3712,7 @@
       <c r="H74">
         <v>221.2</v>
       </c>
-      <c r="J74" s="2">
+      <c r="J74" s="1">
         <v>46426</v>
       </c>
       <c r="K74" t="b">
@@ -3770,7 +3744,7 @@
       <c r="H75">
         <v>240.8</v>
       </c>
-      <c r="J75" s="2">
+      <c r="J75" s="1">
         <v>46450</v>
       </c>
       <c r="K75" t="b">
@@ -3802,7 +3776,7 @@
       <c r="H76">
         <v>245.8</v>
       </c>
-      <c r="J76" s="2">
+      <c r="J76" s="1">
         <v>46452</v>
       </c>
       <c r="K76" t="b">
@@ -3834,7 +3808,7 @@
       <c r="H77">
         <v>263.4</v>
       </c>
-      <c r="J77" s="2">
+      <c r="J77" s="1">
         <v>46322</v>
       </c>
       <c r="K77" t="b">
@@ -3866,7 +3840,7 @@
       <c r="H78">
         <v>275.2</v>
       </c>
-      <c r="J78" s="2">
+      <c r="J78" s="1">
         <v>46433</v>
       </c>
       <c r="K78" t="b">
@@ -3901,7 +3875,7 @@
       <c r="I79" t="s">
         <v>311</v>
       </c>
-      <c r="J79" s="2">
+      <c r="J79" s="1">
         <v>36557</v>
       </c>
       <c r="K79" t="b">
@@ -3936,7 +3910,7 @@
       <c r="I80" t="s">
         <v>312</v>
       </c>
-      <c r="J80" s="2">
+      <c r="J80" s="1">
         <v>41275</v>
       </c>
       <c r="K80" t="b">
@@ -3971,7 +3945,7 @@
       <c r="I81" t="s">
         <v>313</v>
       </c>
-      <c r="J81" s="2">
+      <c r="J81" s="1">
         <v>45380</v>
       </c>
       <c r="K81" t="b">
@@ -4006,7 +3980,7 @@
       <c r="I82" t="s">
         <v>314</v>
       </c>
-      <c r="J82" s="2">
+      <c r="J82" s="1">
         <v>45421</v>
       </c>
       <c r="K82" t="b">
@@ -4041,7 +4015,7 @@
       <c r="I83" t="s">
         <v>314</v>
       </c>
-      <c r="J83" s="2">
+      <c r="J83" s="1">
         <v>45428</v>
       </c>
       <c r="K83" t="b">
@@ -4076,7 +4050,7 @@
       <c r="I84" t="s">
         <v>315</v>
       </c>
-      <c r="J84" s="2">
+      <c r="J84" s="1">
         <v>45490</v>
       </c>
       <c r="K84" t="b">
@@ -4111,7 +4085,7 @@
       <c r="I85" t="s">
         <v>316</v>
       </c>
-      <c r="J85" s="2">
+      <c r="J85" s="1">
         <v>45566</v>
       </c>
       <c r="K85" t="b">
@@ -4146,7 +4120,7 @@
       <c r="I86" t="s">
         <v>317</v>
       </c>
-      <c r="J86" s="2">
+      <c r="J86" s="1">
         <v>45986</v>
       </c>
       <c r="K86" t="b">
@@ -4181,7 +4155,7 @@
       <c r="I87" t="s">
         <v>318</v>
       </c>
-      <c r="J87" s="2">
+      <c r="J87" s="1">
         <v>46284</v>
       </c>
       <c r="K87" t="b">
@@ -4216,7 +4190,7 @@
       <c r="I88" t="s">
         <v>319</v>
       </c>
-      <c r="J88" s="2">
+      <c r="J88" s="1">
         <v>46305</v>
       </c>
       <c r="K88" t="b">
@@ -4251,7 +4225,7 @@
       <c r="I89" t="s">
         <v>319</v>
       </c>
-      <c r="J89" s="2">
+      <c r="J89" s="1">
         <v>46310</v>
       </c>
       <c r="K89" t="b">
@@ -4286,7 +4260,7 @@
       <c r="I90" t="s">
         <v>319</v>
       </c>
-      <c r="J90" s="2">
+      <c r="J90" s="1">
         <v>46317</v>
       </c>
       <c r="K90" t="b">
@@ -4321,7 +4295,7 @@
       <c r="I91" t="s">
         <v>319</v>
       </c>
-      <c r="J91" s="2">
+      <c r="J91" s="1">
         <v>46319</v>
       </c>
       <c r="K91" t="b">
@@ -4356,7 +4330,7 @@
       <c r="I92" t="s">
         <v>320</v>
       </c>
-      <c r="J92" s="2">
+      <c r="J92" s="1">
         <v>46333</v>
       </c>
       <c r="K92" t="b">
@@ -4391,7 +4365,7 @@
       <c r="I93" t="s">
         <v>320</v>
       </c>
-      <c r="J93" s="2">
+      <c r="J93" s="1">
         <v>46338</v>
       </c>
       <c r="K93" t="b">
@@ -4426,7 +4400,7 @@
       <c r="I94" t="s">
         <v>320</v>
       </c>
-      <c r="J94" s="2">
+      <c r="J94" s="1">
         <v>46338</v>
       </c>
       <c r="K94" t="b">
@@ -4461,7 +4435,7 @@
       <c r="I95" t="s">
         <v>320</v>
       </c>
-      <c r="J95" s="2">
+      <c r="J95" s="1">
         <v>46341</v>
       </c>
       <c r="K95" t="b">
@@ -4496,7 +4470,7 @@
       <c r="I96" t="s">
         <v>320</v>
       </c>
-      <c r="J96" s="2">
+      <c r="J96" s="1">
         <v>46344</v>
       </c>
       <c r="K96" t="b">
@@ -4531,7 +4505,7 @@
       <c r="I97" t="s">
         <v>321</v>
       </c>
-      <c r="J97" s="2">
+      <c r="J97" s="1">
         <v>46360</v>
       </c>
       <c r="K97" t="b">
@@ -4566,7 +4540,7 @@
       <c r="I98" t="s">
         <v>321</v>
       </c>
-      <c r="J98" s="2">
+      <c r="J98" s="1">
         <v>46360</v>
       </c>
       <c r="K98" t="b">
@@ -4601,7 +4575,7 @@
       <c r="I99" t="s">
         <v>321</v>
       </c>
-      <c r="J99" s="2">
+      <c r="J99" s="1">
         <v>46367</v>
       </c>
       <c r="K99" t="b">
@@ -4636,7 +4610,7 @@
       <c r="I100" t="s">
         <v>321</v>
       </c>
-      <c r="J100" s="2">
+      <c r="J100" s="1">
         <v>46375</v>
       </c>
       <c r="K100" t="b">
@@ -4671,7 +4645,7 @@
       <c r="I101" t="s">
         <v>321</v>
       </c>
-      <c r="J101" s="2">
+      <c r="J101" s="1">
         <v>46387</v>
       </c>
       <c r="K101" t="b">
@@ -4706,7 +4680,7 @@
       <c r="I102" t="s">
         <v>321</v>
       </c>
-      <c r="J102" s="2">
+      <c r="J102" s="1">
         <v>46387</v>
       </c>
       <c r="K102" t="b">
@@ -4741,7 +4715,7 @@
       <c r="I103" t="s">
         <v>321</v>
       </c>
-      <c r="J103" s="2">
+      <c r="J103" s="1">
         <v>46387</v>
       </c>
       <c r="K103" t="b">
@@ -4776,7 +4750,7 @@
       <c r="I104" t="s">
         <v>321</v>
       </c>
-      <c r="J104" s="2">
+      <c r="J104" s="1">
         <v>46388</v>
       </c>
       <c r="K104" t="b">
@@ -4811,7 +4785,7 @@
       <c r="I105" t="s">
         <v>322</v>
       </c>
-      <c r="J105" s="2">
+      <c r="J105" s="1">
         <v>46401</v>
       </c>
       <c r="K105" t="b">
@@ -4846,7 +4820,7 @@
       <c r="I106" t="s">
         <v>322</v>
       </c>
-      <c r="J106" s="2">
+      <c r="J106" s="1">
         <v>46401</v>
       </c>
       <c r="K106" t="b">
@@ -4881,7 +4855,7 @@
       <c r="I107" t="s">
         <v>322</v>
       </c>
-      <c r="J107" s="2">
+      <c r="J107" s="1">
         <v>46401</v>
       </c>
       <c r="K107" t="b">
@@ -4916,7 +4890,7 @@
       <c r="I108" t="s">
         <v>322</v>
       </c>
-      <c r="J108" s="2">
+      <c r="J108" s="1">
         <v>46412</v>
       </c>
       <c r="K108" t="b">
@@ -4951,7 +4925,7 @@
       <c r="I109" t="s">
         <v>322</v>
       </c>
-      <c r="J109" s="2">
+      <c r="J109" s="1">
         <v>46412</v>
       </c>
       <c r="K109" t="b">
@@ -4986,7 +4960,7 @@
       <c r="I110" t="s">
         <v>322</v>
       </c>
-      <c r="J110" s="2">
+      <c r="J110" s="1">
         <v>46412</v>
       </c>
       <c r="K110" t="b">
@@ -5021,7 +4995,7 @@
       <c r="I111" t="s">
         <v>323</v>
       </c>
-      <c r="J111" s="2">
+      <c r="J111" s="1">
         <v>46424</v>
       </c>
       <c r="K111" t="b">
@@ -5056,7 +5030,7 @@
       <c r="I112" t="s">
         <v>323</v>
       </c>
-      <c r="J112" s="2">
+      <c r="J112" s="1">
         <v>46437</v>
       </c>
       <c r="K112" t="b">
@@ -5091,7 +5065,7 @@
       <c r="I113" t="s">
         <v>323</v>
       </c>
-      <c r="J113" s="2">
+      <c r="J113" s="1">
         <v>46451</v>
       </c>
       <c r="K113" t="b">
@@ -5126,7 +5100,7 @@
       <c r="I114" t="s">
         <v>323</v>
       </c>
-      <c r="J114" s="2">
+      <c r="J114" s="1">
         <v>46451</v>
       </c>
       <c r="K114" t="b">
@@ -5161,7 +5135,7 @@
       <c r="I115" t="s">
         <v>324</v>
       </c>
-      <c r="J115" s="2">
+      <c r="J115" s="1">
         <v>46455</v>
       </c>
       <c r="K115" t="b">
@@ -5196,7 +5170,7 @@
       <c r="I116" t="s">
         <v>324</v>
       </c>
-      <c r="J116" s="2">
+      <c r="J116" s="1">
         <v>46456</v>
       </c>
       <c r="K116" t="b">
@@ -5231,7 +5205,7 @@
       <c r="I117" t="s">
         <v>324</v>
       </c>
-      <c r="J117" s="2">
+      <c r="J117" s="1">
         <v>46457</v>
       </c>
       <c r="K117" t="b">
@@ -5266,7 +5240,7 @@
       <c r="I118" t="s">
         <v>324</v>
       </c>
-      <c r="J118" s="2">
+      <c r="J118" s="1">
         <v>46464</v>
       </c>
       <c r="K118" t="b">
@@ -5301,7 +5275,7 @@
       <c r="I119" t="s">
         <v>324</v>
       </c>
-      <c r="J119" s="2">
+      <c r="J119" s="1">
         <v>46470</v>
       </c>
       <c r="K119" t="b">
@@ -5336,7 +5310,7 @@
       <c r="I120" t="s">
         <v>325</v>
       </c>
-      <c r="J120" s="2">
+      <c r="J120" s="1">
         <v>46485</v>
       </c>
       <c r="K120" t="b">
@@ -5371,7 +5345,7 @@
       <c r="I121" t="s">
         <v>325</v>
       </c>
-      <c r="J121" s="2">
+      <c r="J121" s="1">
         <v>46499</v>
       </c>
       <c r="K121" t="b">
@@ -5406,7 +5380,7 @@
       <c r="I122" t="s">
         <v>325</v>
       </c>
-      <c r="J122" s="2">
+      <c r="J122" s="1">
         <v>46504</v>
       </c>
       <c r="K122" t="b">
@@ -5441,7 +5415,7 @@
       <c r="I123" t="s">
         <v>325</v>
       </c>
-      <c r="J123" s="2">
+      <c r="J123" s="1">
         <v>46504</v>
       </c>
       <c r="K123" t="b">
@@ -5476,7 +5450,7 @@
       <c r="I124" t="s">
         <v>325</v>
       </c>
-      <c r="J124" s="2">
+      <c r="J124" s="1">
         <v>46507</v>
       </c>
       <c r="K124" t="b">
@@ -5511,7 +5485,7 @@
       <c r="I125" t="s">
         <v>325</v>
       </c>
-      <c r="J125" s="2">
+      <c r="J125" s="1">
         <v>46508</v>
       </c>
       <c r="K125" t="b">
@@ -5546,7 +5520,7 @@
       <c r="I126" t="s">
         <v>325</v>
       </c>
-      <c r="J126" s="2">
+      <c r="J126" s="1">
         <v>46512</v>
       </c>
       <c r="K126" t="b">
@@ -5581,7 +5555,7 @@
       <c r="I127" t="s">
         <v>326</v>
       </c>
-      <c r="J127" s="2">
+      <c r="J127" s="1">
         <v>46512</v>
       </c>
       <c r="K127" t="b">
@@ -5616,7 +5590,7 @@
       <c r="I128" t="s">
         <v>326</v>
       </c>
-      <c r="J128" s="2">
+      <c r="J128" s="1">
         <v>46528</v>
       </c>
       <c r="K128" t="b">
@@ -5651,7 +5625,7 @@
       <c r="I129" t="s">
         <v>326</v>
       </c>
-      <c r="J129" s="2">
+      <c r="J129" s="1">
         <v>46529</v>
       </c>
       <c r="K129" t="b">
@@ -5686,7 +5660,7 @@
       <c r="I130" t="s">
         <v>326</v>
       </c>
-      <c r="J130" s="2">
+      <c r="J130" s="1">
         <v>46537</v>
       </c>
       <c r="K130" t="b">
@@ -5721,7 +5695,7 @@
       <c r="I131" t="s">
         <v>327</v>
       </c>
-      <c r="J131" s="2">
+      <c r="J131" s="1">
         <v>46546</v>
       </c>
       <c r="K131" t="b">
@@ -5756,7 +5730,7 @@
       <c r="I132" t="s">
         <v>327</v>
       </c>
-      <c r="J132" s="2">
+      <c r="J132" s="1">
         <v>46547</v>
       </c>
       <c r="K132" t="b">
@@ -5791,7 +5765,7 @@
       <c r="I133" t="s">
         <v>327</v>
       </c>
-      <c r="J133" s="2">
+      <c r="J133" s="1">
         <v>46547</v>
       </c>
       <c r="K133" t="b">
@@ -5826,7 +5800,7 @@
       <c r="I134" t="s">
         <v>327</v>
       </c>
-      <c r="J134" s="2">
+      <c r="J134" s="1">
         <v>46547</v>
       </c>
       <c r="K134" t="b">
@@ -5861,7 +5835,7 @@
       <c r="I135" t="s">
         <v>327</v>
       </c>
-      <c r="J135" s="2">
+      <c r="J135" s="1">
         <v>46551</v>
       </c>
       <c r="K135" t="b">
@@ -5896,7 +5870,7 @@
       <c r="I136" t="s">
         <v>327</v>
       </c>
-      <c r="J136" s="2">
+      <c r="J136" s="1">
         <v>46560</v>
       </c>
       <c r="K136" t="b">
@@ -5931,7 +5905,7 @@
       <c r="I137" t="s">
         <v>327</v>
       </c>
-      <c r="J137" s="2">
+      <c r="J137" s="1">
         <v>46564</v>
       </c>
       <c r="K137" t="b">
@@ -5966,7 +5940,7 @@
       <c r="I138" t="s">
         <v>327</v>
       </c>
-      <c r="J138" s="2">
+      <c r="J138" s="1">
         <v>46567</v>
       </c>
       <c r="K138" t="b">
@@ -6001,7 +5975,7 @@
       <c r="I139" t="s">
         <v>327</v>
       </c>
-      <c r="J139" s="2">
+      <c r="J139" s="1">
         <v>46568</v>
       </c>
       <c r="K139" t="b">
@@ -6036,7 +6010,7 @@
       <c r="I140" t="s">
         <v>328</v>
       </c>
-      <c r="J140" s="2">
+      <c r="J140" s="1">
         <v>46578</v>
       </c>
       <c r="K140" t="b">
@@ -6071,7 +6045,7 @@
       <c r="I141" t="s">
         <v>328</v>
       </c>
-      <c r="J141" s="2">
+      <c r="J141" s="1">
         <v>46592</v>
       </c>
       <c r="K141" t="b">
@@ -6106,7 +6080,7 @@
       <c r="I142" t="s">
         <v>328</v>
       </c>
-      <c r="J142" s="2">
+      <c r="J142" s="1">
         <v>46592</v>
       </c>
       <c r="K142" t="b">
@@ -6141,7 +6115,7 @@
       <c r="I143" t="s">
         <v>329</v>
       </c>
-      <c r="J143" s="2">
+      <c r="J143" s="1">
         <v>46212</v>
       </c>
       <c r="K143" t="b">
@@ -6176,7 +6150,7 @@
       <c r="I144" t="s">
         <v>330</v>
       </c>
-      <c r="J144" s="2">
+      <c r="J144" s="1">
         <v>46225</v>
       </c>
       <c r="K144" t="b">
@@ -6211,7 +6185,7 @@
       <c r="I145" t="s">
         <v>331</v>
       </c>
-      <c r="J145" s="2">
+      <c r="J145" s="1">
         <v>46263</v>
       </c>
       <c r="K145" t="b">
@@ -6243,7 +6217,7 @@
       <c r="H146">
         <v>-1476</v>
       </c>
-      <c r="J146" s="2">
+      <c r="J146" s="1">
         <v>43773</v>
       </c>
       <c r="K146" t="b">
@@ -6275,7 +6249,7 @@
       <c r="H147">
         <v>-1469</v>
       </c>
-      <c r="J147" s="2">
+      <c r="J147" s="1">
         <v>43773</v>
       </c>
       <c r="K147" t="b">
@@ -6307,7 +6281,7 @@
       <c r="H148">
         <v>-1186</v>
       </c>
-      <c r="J148" s="2">
+      <c r="J148" s="1">
         <v>45295</v>
       </c>
       <c r="K148" t="b">
@@ -6339,7 +6313,7 @@
       <c r="H149">
         <v>-1048</v>
       </c>
-      <c r="J149" s="2">
+      <c r="J149" s="1">
         <v>45617</v>
       </c>
       <c r="K149" t="b">
@@ -6371,7 +6345,7 @@
       <c r="H150">
         <v>-980</v>
       </c>
-      <c r="J150" s="2">
+      <c r="J150" s="1">
         <v>45677</v>
       </c>
       <c r="K150" t="b">
@@ -6403,7 +6377,7 @@
       <c r="H151">
         <v>-961</v>
       </c>
-      <c r="J151" s="2">
+      <c r="J151" s="1">
         <v>44944</v>
       </c>
       <c r="K151" t="b">
@@ -6435,7 +6409,7 @@
       <c r="H152">
         <v>-252</v>
       </c>
-      <c r="J152" s="2">
+      <c r="J152" s="1">
         <v>46092</v>
       </c>
       <c r="K152" t="b">
@@ -6467,7 +6441,7 @@
       <c r="H153">
         <v>3</v>
       </c>
-      <c r="J153" s="2">
+      <c r="J153" s="1">
         <v>46265</v>
       </c>
       <c r="K153" t="b">
@@ -6499,7 +6473,7 @@
       <c r="H154">
         <v>3</v>
       </c>
-      <c r="J154" s="2">
+      <c r="J154" s="1">
         <v>46265</v>
       </c>
       <c r="K154" t="b">
@@ -6531,7 +6505,7 @@
       <c r="H155">
         <v>43</v>
       </c>
-      <c r="J155" s="2">
+      <c r="J155" s="1">
         <v>46440</v>
       </c>
       <c r="K155" t="b">
@@ -6563,7 +6537,7 @@
       <c r="H156">
         <v>43</v>
       </c>
-      <c r="J156" s="2">
+      <c r="J156" s="1">
         <v>46440</v>
       </c>
       <c r="K156" t="b">
@@ -6595,7 +6569,7 @@
       <c r="H157">
         <v>72</v>
       </c>
-      <c r="J157" s="2">
+      <c r="J157" s="1">
         <v>46289</v>
       </c>
       <c r="K157" t="b">
@@ -6627,7 +6601,7 @@
       <c r="H158">
         <v>72</v>
       </c>
-      <c r="J158" s="2">
+      <c r="J158" s="1">
         <v>46289</v>
       </c>
       <c r="K158" t="b">
@@ -6659,7 +6633,7 @@
       <c r="H159">
         <v>81</v>
       </c>
-      <c r="J159" s="2">
+      <c r="J159" s="1">
         <v>46405</v>
       </c>
       <c r="K159" t="b">
@@ -6691,7 +6665,7 @@
       <c r="H160">
         <v>102</v>
       </c>
-      <c r="J160" s="2">
+      <c r="J160" s="1">
         <v>46463</v>
       </c>
       <c r="K160" t="b">
@@ -6723,7 +6697,7 @@
       <c r="H161">
         <v>109</v>
       </c>
-      <c r="J161" s="2">
+      <c r="J161" s="1">
         <v>46353</v>
       </c>
       <c r="K161" t="b">
@@ -6755,7 +6729,7 @@
       <c r="H162">
         <v>127</v>
       </c>
-      <c r="J162" s="2">
+      <c r="J162" s="1">
         <v>46417</v>
       </c>
       <c r="K162" t="b">
@@ -6787,7 +6761,7 @@
       <c r="H163">
         <v>152</v>
       </c>
-      <c r="J163" s="2">
+      <c r="J163" s="1">
         <v>46271</v>
       </c>
       <c r="K163" t="b">
@@ -6819,7 +6793,7 @@
       <c r="H164">
         <v>152</v>
       </c>
-      <c r="J164" s="2">
+      <c r="J164" s="1">
         <v>46271</v>
       </c>
       <c r="K164" t="b">
@@ -6851,7 +6825,7 @@
       <c r="H165">
         <v>153</v>
       </c>
-      <c r="J165" s="2">
+      <c r="J165" s="1">
         <v>46458</v>
       </c>
       <c r="K165" t="b">
@@ -6883,7 +6857,7 @@
       <c r="H166">
         <v>158</v>
       </c>
-      <c r="J166" s="2">
+      <c r="J166" s="1">
         <v>46381</v>
       </c>
       <c r="K166" t="b">
@@ -6915,7 +6889,7 @@
       <c r="H167">
         <v>163</v>
       </c>
-      <c r="J167" s="2">
+      <c r="J167" s="1">
         <v>46592</v>
       </c>
       <c r="K167" t="b">
@@ -6947,7 +6921,7 @@
       <c r="H168">
         <v>167</v>
       </c>
-      <c r="J168" s="2">
+      <c r="J168" s="1">
         <v>46441</v>
       </c>
       <c r="K168" t="b">
@@ -6979,7 +6953,7 @@
       <c r="H169">
         <v>169</v>
       </c>
-      <c r="J169" s="2">
+      <c r="J169" s="1">
         <v>46391</v>
       </c>
       <c r="K169" t="b">
@@ -7011,7 +6985,7 @@
       <c r="H170">
         <v>184</v>
       </c>
-      <c r="J170" s="2">
+      <c r="J170" s="1">
         <v>46385</v>
       </c>
       <c r="K170" t="b">
@@ -7043,7 +7017,7 @@
       <c r="H171">
         <v>186</v>
       </c>
-      <c r="J171" s="2">
+      <c r="J171" s="1">
         <v>46387</v>
       </c>
       <c r="K171" t="b">
@@ -7075,7 +7049,7 @@
       <c r="H172">
         <v>206</v>
       </c>
-      <c r="J172" s="2">
+      <c r="J172" s="1">
         <v>46399</v>
       </c>
       <c r="K172" t="b">
@@ -7107,7 +7081,7 @@
       <c r="H173">
         <v>206</v>
       </c>
-      <c r="J173" s="2">
+      <c r="J173" s="1">
         <v>46399</v>
       </c>
       <c r="K173" t="b">
@@ -7139,7 +7113,7 @@
       <c r="H174">
         <v>234</v>
       </c>
-      <c r="J174" s="2">
+      <c r="J174" s="1">
         <v>46458</v>
       </c>
       <c r="K174" t="b">
@@ -7171,7 +7145,7 @@
       <c r="H175">
         <v>248</v>
       </c>
-      <c r="J175" s="2">
+      <c r="J175" s="1">
         <v>46528</v>
       </c>
       <c r="K175" t="b">
@@ -7203,7 +7177,7 @@
       <c r="H176">
         <v>317</v>
       </c>
-      <c r="J176" s="2">
+      <c r="J176" s="1">
         <v>46540</v>
       </c>
       <c r="K176" t="b">
@@ -7235,7 +7209,7 @@
       <c r="H177">
         <v>340</v>
       </c>
-      <c r="J177" s="2">
+      <c r="J177" s="1">
         <v>46547</v>
       </c>
       <c r="K177" t="b">
@@ -7267,7 +7241,7 @@
       <c r="H178">
         <v>364</v>
       </c>
-      <c r="J178" s="2">
+      <c r="J178" s="1">
         <v>46557</v>
       </c>
       <c r="K178" t="b">
@@ -7299,7 +7273,7 @@
       <c r="H179">
         <v>368</v>
       </c>
-      <c r="J179" s="2">
+      <c r="J179" s="1">
         <v>46571</v>
       </c>
       <c r="K179" t="b">
@@ -7331,7 +7305,7 @@
       <c r="H180">
         <v>368</v>
       </c>
-      <c r="J180" s="2">
+      <c r="J180" s="1">
         <v>46571</v>
       </c>
       <c r="K180" t="b">
@@ -7363,7 +7337,7 @@
       <c r="H181">
         <v>370</v>
       </c>
-      <c r="J181" s="2">
+      <c r="J181" s="1">
         <v>46562</v>
       </c>
       <c r="K181" t="b">
@@ -7395,7 +7369,7 @@
       <c r="H182">
         <v>385</v>
       </c>
-      <c r="J182" s="2">
+      <c r="J182" s="1">
         <v>46574</v>
       </c>
       <c r="K182" t="b">
@@ -7427,7 +7401,7 @@
       <c r="H183">
         <v>385</v>
       </c>
-      <c r="J183" s="2">
+      <c r="J183" s="1">
         <v>46574</v>
       </c>
       <c r="K183" t="b">
@@ -7459,7 +7433,7 @@
       <c r="H184">
         <v>417</v>
       </c>
-      <c r="J184" s="2">
+      <c r="J184" s="1">
         <v>46578</v>
       </c>
       <c r="K184" t="b">
@@ -7491,7 +7465,7 @@
       <c r="H185">
         <v>721</v>
       </c>
-      <c r="J185" s="2">
+      <c r="J185" s="1">
         <v>46345</v>
       </c>
       <c r="K185" t="b">
@@ -7523,7 +7497,7 @@
       <c r="H186">
         <v>721</v>
       </c>
-      <c r="J186" s="2">
+      <c r="J186" s="1">
         <v>46345</v>
       </c>
       <c r="K186" t="b">
@@ -7555,7 +7529,7 @@
       <c r="H187">
         <v>850</v>
       </c>
-      <c r="J187" s="2">
+      <c r="J187" s="1">
         <v>46366</v>
       </c>
       <c r="K187" t="b">
@@ -7587,7 +7561,7 @@
       <c r="H188">
         <v>850</v>
       </c>
-      <c r="J188" s="2">
+      <c r="J188" s="1">
         <v>46366</v>
       </c>
       <c r="K188" t="b">
@@ -7619,7 +7593,7 @@
       <c r="H189">
         <v>1661</v>
       </c>
-      <c r="J189" s="2">
+      <c r="J189" s="1">
         <v>46524</v>
       </c>
       <c r="K189" t="b">
@@ -7651,7 +7625,7 @@
       <c r="H190">
         <v>1661</v>
       </c>
-      <c r="J190" s="2">
+      <c r="J190" s="1">
         <v>46524</v>
       </c>
       <c r="K190" t="b">
@@ -7683,7 +7657,7 @@
       <c r="H191">
         <v>488</v>
       </c>
-      <c r="J191" s="2">
+      <c r="J191" s="1">
         <v>46190</v>
       </c>
       <c r="K191" t="b">
@@ -7715,7 +7689,7 @@
       <c r="H192">
         <v>25565</v>
       </c>
-      <c r="J192" s="2">
+      <c r="J192" s="1">
         <v>46190</v>
       </c>
       <c r="K192" t="b">
@@ -7747,7 +7721,7 @@
       <c r="H193">
         <v>25567</v>
       </c>
-      <c r="J193" s="2">
+      <c r="J193" s="1">
         <v>46190</v>
       </c>
       <c r="K193" t="b">
@@ -7779,7 +7753,7 @@
       <c r="H194">
         <v>31293</v>
       </c>
-      <c r="J194" s="2">
+      <c r="J194" s="1">
         <v>46190</v>
       </c>
       <c r="K194" t="b">

</xml_diff>

<commit_message>
Atualização automática: vencimentos_tmot (08/09/2026 08:22)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
@@ -1019,8 +1019,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1036,7 +1044,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1044,12 +1052,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1349,37 +1375,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1408,7 +1434,7 @@
       <c r="H2">
         <v>-4300.3</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>39285</v>
       </c>
       <c r="K2" t="b">
@@ -1440,7 +1466,7 @@
       <c r="H3">
         <v>-2354.2</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>40669</v>
       </c>
       <c r="K3" t="b">
@@ -1472,7 +1498,7 @@
       <c r="H4">
         <v>-910.7</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>40669</v>
       </c>
       <c r="K4" t="b">
@@ -1504,7 +1530,7 @@
       <c r="H5">
         <v>-868</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>44884</v>
       </c>
       <c r="K5" t="b">
@@ -1536,7 +1562,7 @@
       <c r="H6">
         <v>-483.8</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>43855</v>
       </c>
       <c r="K6" t="b">
@@ -1568,7 +1594,7 @@
       <c r="H7">
         <v>-417</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>46014</v>
       </c>
       <c r="K7" t="b">
@@ -1600,7 +1626,7 @@
       <c r="H8">
         <v>-414.2</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>46014</v>
       </c>
       <c r="K8" t="b">
@@ -1632,7 +1658,7 @@
       <c r="H9">
         <v>-391.8</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>42769</v>
       </c>
       <c r="K9" t="b">
@@ -1664,7 +1690,7 @@
       <c r="H10">
         <v>-391.6</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>45804</v>
       </c>
       <c r="K10" t="b">
@@ -1696,7 +1722,7 @@
       <c r="H11">
         <v>-391.6</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>45804</v>
       </c>
       <c r="K11" t="b">
@@ -1728,7 +1754,7 @@
       <c r="H12">
         <v>-372.9</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>42821</v>
       </c>
       <c r="K12" t="b">
@@ -1760,7 +1786,7 @@
       <c r="H13">
         <v>-372.9</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>46014</v>
       </c>
       <c r="K13" t="b">
@@ -1792,7 +1818,7 @@
       <c r="H14">
         <v>-372.9</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>46014</v>
       </c>
       <c r="K14" t="b">
@@ -1824,7 +1850,7 @@
       <c r="H15">
         <v>-372.9</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>46014</v>
       </c>
       <c r="K15" t="b">
@@ -1856,7 +1882,7 @@
       <c r="H16">
         <v>-367.8</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="2">
         <v>46017</v>
       </c>
       <c r="K16" t="b">
@@ -1888,7 +1914,7 @@
       <c r="H17">
         <v>-367.8</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="2">
         <v>46017</v>
       </c>
       <c r="K17" t="b">
@@ -1920,7 +1946,7 @@
       <c r="H18">
         <v>-347.2</v>
       </c>
-      <c r="J18" s="1">
+      <c r="J18" s="2">
         <v>40979</v>
       </c>
       <c r="K18" t="b">
@@ -1952,7 +1978,7 @@
       <c r="H19">
         <v>-293.8</v>
       </c>
-      <c r="J19" s="1">
+      <c r="J19" s="2">
         <v>45846</v>
       </c>
       <c r="K19" t="b">
@@ -1984,7 +2010,7 @@
       <c r="H20">
         <v>-206.4</v>
       </c>
-      <c r="J20" s="1">
+      <c r="J20" s="2">
         <v>36669</v>
       </c>
       <c r="K20" t="b">
@@ -2016,7 +2042,7 @@
       <c r="H21">
         <v>-131.6</v>
       </c>
-      <c r="J21" s="1">
+      <c r="J21" s="2">
         <v>46111</v>
       </c>
       <c r="K21" t="b">
@@ -2048,7 +2074,7 @@
       <c r="H22">
         <v>-131.6</v>
       </c>
-      <c r="J22" s="1">
+      <c r="J22" s="2">
         <v>46111</v>
       </c>
       <c r="K22" t="b">
@@ -2080,7 +2106,7 @@
       <c r="H23">
         <v>-131.6</v>
       </c>
-      <c r="J23" s="1">
+      <c r="J23" s="2">
         <v>46111</v>
       </c>
       <c r="K23" t="b">
@@ -2112,7 +2138,7 @@
       <c r="H24">
         <v>-131.6</v>
       </c>
-      <c r="J24" s="1">
+      <c r="J24" s="2">
         <v>46111</v>
       </c>
       <c r="K24" t="b">
@@ -2144,7 +2170,7 @@
       <c r="H25">
         <v>-131.6</v>
       </c>
-      <c r="J25" s="1">
+      <c r="J25" s="2">
         <v>46111</v>
       </c>
       <c r="K25" t="b">
@@ -2176,7 +2202,7 @@
       <c r="H26">
         <v>-98.3</v>
       </c>
-      <c r="J26" s="1">
+      <c r="J26" s="2">
         <v>41204</v>
       </c>
       <c r="K26" t="b">
@@ -2208,7 +2234,7 @@
       <c r="H27">
         <v>-47.2</v>
       </c>
-      <c r="J27" s="1">
+      <c r="J27" s="2">
         <v>44011</v>
       </c>
       <c r="K27" t="b">
@@ -2240,7 +2266,7 @@
       <c r="H28">
         <v>-22.3</v>
       </c>
-      <c r="J28" s="1">
+      <c r="J28" s="2">
         <v>46226</v>
       </c>
       <c r="K28" t="b">
@@ -2272,7 +2298,7 @@
       <c r="H29">
         <v>4.7</v>
       </c>
-      <c r="J29" s="1">
+      <c r="J29" s="2">
         <v>46265</v>
       </c>
       <c r="K29" t="b">
@@ -2304,7 +2330,7 @@
       <c r="H30">
         <v>7.5</v>
       </c>
-      <c r="J30" s="1">
+      <c r="J30" s="2">
         <v>46265</v>
       </c>
       <c r="K30" t="b">
@@ -2336,7 +2362,7 @@
       <c r="H31">
         <v>10</v>
       </c>
-      <c r="J31" s="1">
+      <c r="J31" s="2">
         <v>46265</v>
       </c>
       <c r="K31" t="b">
@@ -2368,7 +2394,7 @@
       <c r="H32">
         <v>12.8</v>
       </c>
-      <c r="J32" s="1">
+      <c r="J32" s="2">
         <v>46265</v>
       </c>
       <c r="K32" t="b">
@@ -2400,7 +2426,7 @@
       <c r="H33">
         <v>14</v>
       </c>
-      <c r="J33" s="1">
+      <c r="J33" s="2">
         <v>46265</v>
       </c>
       <c r="K33" t="b">
@@ -2432,7 +2458,7 @@
       <c r="H34">
         <v>17.8</v>
       </c>
-      <c r="J34" s="1">
+      <c r="J34" s="2">
         <v>46265</v>
       </c>
       <c r="K34" t="b">
@@ -2464,7 +2490,7 @@
       <c r="H35">
         <v>20.4</v>
       </c>
-      <c r="J35" s="1">
+      <c r="J35" s="2">
         <v>46265</v>
       </c>
       <c r="K35" t="b">
@@ -2496,7 +2522,7 @@
       <c r="H36">
         <v>21.2</v>
       </c>
-      <c r="J36" s="1">
+      <c r="J36" s="2">
         <v>46265</v>
       </c>
       <c r="K36" t="b">
@@ -2528,7 +2554,7 @@
       <c r="H37">
         <v>26.2</v>
       </c>
-      <c r="J37" s="1">
+      <c r="J37" s="2">
         <v>46265</v>
       </c>
       <c r="K37" t="b">
@@ -2560,7 +2586,7 @@
       <c r="H38">
         <v>33.6</v>
       </c>
-      <c r="J38" s="1">
+      <c r="J38" s="2">
         <v>46364</v>
       </c>
       <c r="K38" t="b">
@@ -2592,7 +2618,7 @@
       <c r="H39">
         <v>42.2</v>
       </c>
-      <c r="J39" s="1">
+      <c r="J39" s="2">
         <v>46269</v>
       </c>
       <c r="K39" t="b">
@@ -2624,7 +2650,7 @@
       <c r="H40">
         <v>42.8</v>
       </c>
-      <c r="J40" s="1">
+      <c r="J40" s="2">
         <v>46291</v>
       </c>
       <c r="K40" t="b">
@@ -2656,7 +2682,7 @@
       <c r="H41">
         <v>45.7</v>
       </c>
-      <c r="J41" s="1">
+      <c r="J41" s="2">
         <v>46395</v>
       </c>
       <c r="K41" t="b">
@@ -2688,7 +2714,7 @@
       <c r="H42">
         <v>47.2</v>
       </c>
-      <c r="J42" s="1">
+      <c r="J42" s="2">
         <v>46280</v>
       </c>
       <c r="K42" t="b">
@@ -2720,7 +2746,7 @@
       <c r="H43">
         <v>48.7</v>
       </c>
-      <c r="J43" s="1">
+      <c r="J43" s="2">
         <v>46281</v>
       </c>
       <c r="K43" t="b">
@@ -2752,7 +2778,7 @@
       <c r="H44">
         <v>60</v>
       </c>
-      <c r="J44" s="1">
+      <c r="J44" s="2">
         <v>46281</v>
       </c>
       <c r="K44" t="b">
@@ -2784,7 +2810,7 @@
       <c r="H45">
         <v>62.6</v>
       </c>
-      <c r="J45" s="1">
+      <c r="J45" s="2">
         <v>46265</v>
       </c>
       <c r="K45" t="b">
@@ -2816,7 +2842,7 @@
       <c r="H46">
         <v>64.59999999999999</v>
       </c>
-      <c r="J46" s="1">
+      <c r="J46" s="2">
         <v>46265</v>
       </c>
       <c r="K46" t="b">
@@ -2848,7 +2874,7 @@
       <c r="H47">
         <v>67.59999999999999</v>
       </c>
-      <c r="J47" s="1">
+      <c r="J47" s="2">
         <v>46267</v>
       </c>
       <c r="K47" t="b">
@@ -2880,7 +2906,7 @@
       <c r="H48">
         <v>68.3</v>
       </c>
-      <c r="J48" s="1">
+      <c r="J48" s="2">
         <v>46278</v>
       </c>
       <c r="K48" t="b">
@@ -2912,7 +2938,7 @@
       <c r="H49">
         <v>69.2</v>
       </c>
-      <c r="J49" s="1">
+      <c r="J49" s="2">
         <v>46453</v>
       </c>
       <c r="K49" t="b">
@@ -2944,7 +2970,7 @@
       <c r="H50">
         <v>69.8</v>
       </c>
-      <c r="J50" s="1">
+      <c r="J50" s="2">
         <v>46265</v>
       </c>
       <c r="K50" t="b">
@@ -2976,7 +3002,7 @@
       <c r="H51">
         <v>69.8</v>
       </c>
-      <c r="J51" s="1">
+      <c r="J51" s="2">
         <v>46265</v>
       </c>
       <c r="K51" t="b">
@@ -3008,7 +3034,7 @@
       <c r="H52">
         <v>72.2</v>
       </c>
-      <c r="J52" s="1">
+      <c r="J52" s="2">
         <v>46275</v>
       </c>
       <c r="K52" t="b">
@@ -3040,7 +3066,7 @@
       <c r="H53">
         <v>72.2</v>
       </c>
-      <c r="J53" s="1">
+      <c r="J53" s="2">
         <v>46275</v>
       </c>
       <c r="K53" t="b">
@@ -3072,7 +3098,7 @@
       <c r="H54">
         <v>78.09999999999999</v>
       </c>
-      <c r="J54" s="1">
+      <c r="J54" s="2">
         <v>46265</v>
       </c>
       <c r="K54" t="b">
@@ -3104,7 +3130,7 @@
       <c r="H55">
         <v>82.8</v>
       </c>
-      <c r="J55" s="1">
+      <c r="J55" s="2">
         <v>46487</v>
       </c>
       <c r="K55" t="b">
@@ -3136,7 +3162,7 @@
       <c r="H56">
         <v>83.09999999999999</v>
       </c>
-      <c r="J56" s="1">
+      <c r="J56" s="2">
         <v>46285</v>
       </c>
       <c r="K56" t="b">
@@ -3168,7 +3194,7 @@
       <c r="H57">
         <v>84.8</v>
       </c>
-      <c r="J57" s="1">
+      <c r="J57" s="2">
         <v>46492</v>
       </c>
       <c r="K57" t="b">
@@ -3200,7 +3226,7 @@
       <c r="H58">
         <v>104.9</v>
       </c>
-      <c r="J58" s="1">
+      <c r="J58" s="2">
         <v>46297</v>
       </c>
       <c r="K58" t="b">
@@ -3232,7 +3258,7 @@
       <c r="H59">
         <v>107.6</v>
       </c>
-      <c r="J59" s="1">
+      <c r="J59" s="2">
         <v>46283</v>
       </c>
       <c r="K59" t="b">
@@ -3264,7 +3290,7 @@
       <c r="H60">
         <v>111.9</v>
       </c>
-      <c r="J60" s="1">
+      <c r="J60" s="2">
         <v>46300</v>
       </c>
       <c r="K60" t="b">
@@ -3296,7 +3322,7 @@
       <c r="H61">
         <v>111.9</v>
       </c>
-      <c r="J61" s="1">
+      <c r="J61" s="2">
         <v>46300</v>
       </c>
       <c r="K61" t="b">
@@ -3328,7 +3354,7 @@
       <c r="H62">
         <v>111.9</v>
       </c>
-      <c r="J62" s="1">
+      <c r="J62" s="2">
         <v>46300</v>
       </c>
       <c r="K62" t="b">
@@ -3360,7 +3386,7 @@
       <c r="H63">
         <v>111.9</v>
       </c>
-      <c r="J63" s="1">
+      <c r="J63" s="2">
         <v>46300</v>
       </c>
       <c r="K63" t="b">
@@ -3392,7 +3418,7 @@
       <c r="H64">
         <v>111.9</v>
       </c>
-      <c r="J64" s="1">
+      <c r="J64" s="2">
         <v>46300</v>
       </c>
       <c r="K64" t="b">
@@ -3424,7 +3450,7 @@
       <c r="H65">
         <v>128.8</v>
       </c>
-      <c r="J65" s="1">
+      <c r="J65" s="2">
         <v>46308</v>
       </c>
       <c r="K65" t="b">
@@ -3456,7 +3482,7 @@
       <c r="H66">
         <v>131.1</v>
       </c>
-      <c r="J66" s="1">
+      <c r="J66" s="2">
         <v>46336</v>
       </c>
       <c r="K66" t="b">
@@ -3488,7 +3514,7 @@
       <c r="H67">
         <v>138.4</v>
       </c>
-      <c r="J67" s="1">
+      <c r="J67" s="2">
         <v>46343</v>
       </c>
       <c r="K67" t="b">
@@ -3520,7 +3546,7 @@
       <c r="H68">
         <v>141</v>
       </c>
-      <c r="J68" s="1">
+      <c r="J68" s="2">
         <v>46350</v>
       </c>
       <c r="K68" t="b">
@@ -3552,7 +3578,7 @@
       <c r="H69">
         <v>162</v>
       </c>
-      <c r="J69" s="1">
+      <c r="J69" s="2">
         <v>46391</v>
       </c>
       <c r="K69" t="b">
@@ -3584,7 +3610,7 @@
       <c r="H70">
         <v>167.2</v>
       </c>
-      <c r="J70" s="1">
+      <c r="J70" s="2">
         <v>46330</v>
       </c>
       <c r="K70" t="b">
@@ -3616,7 +3642,7 @@
       <c r="H71">
         <v>177.4</v>
       </c>
-      <c r="J71" s="1">
+      <c r="J71" s="2">
         <v>46418</v>
       </c>
       <c r="K71" t="b">
@@ -3648,7 +3674,7 @@
       <c r="H72">
         <v>200</v>
       </c>
-      <c r="J72" s="1">
+      <c r="J72" s="2">
         <v>46356</v>
       </c>
       <c r="K72" t="b">
@@ -3680,7 +3706,7 @@
       <c r="H73">
         <v>203.6</v>
       </c>
-      <c r="J73" s="1">
+      <c r="J73" s="2">
         <v>46436</v>
       </c>
       <c r="K73" t="b">
@@ -3712,7 +3738,7 @@
       <c r="H74">
         <v>221.2</v>
       </c>
-      <c r="J74" s="1">
+      <c r="J74" s="2">
         <v>46426</v>
       </c>
       <c r="K74" t="b">
@@ -3744,7 +3770,7 @@
       <c r="H75">
         <v>240.8</v>
       </c>
-      <c r="J75" s="1">
+      <c r="J75" s="2">
         <v>46450</v>
       </c>
       <c r="K75" t="b">
@@ -3776,7 +3802,7 @@
       <c r="H76">
         <v>245.8</v>
       </c>
-      <c r="J76" s="1">
+      <c r="J76" s="2">
         <v>46452</v>
       </c>
       <c r="K76" t="b">
@@ -3808,7 +3834,7 @@
       <c r="H77">
         <v>263.4</v>
       </c>
-      <c r="J77" s="1">
+      <c r="J77" s="2">
         <v>46322</v>
       </c>
       <c r="K77" t="b">
@@ -3840,7 +3866,7 @@
       <c r="H78">
         <v>275.2</v>
       </c>
-      <c r="J78" s="1">
+      <c r="J78" s="2">
         <v>46433</v>
       </c>
       <c r="K78" t="b">
@@ -3875,7 +3901,7 @@
       <c r="I79" t="s">
         <v>311</v>
       </c>
-      <c r="J79" s="1">
+      <c r="J79" s="2">
         <v>36557</v>
       </c>
       <c r="K79" t="b">
@@ -3910,7 +3936,7 @@
       <c r="I80" t="s">
         <v>312</v>
       </c>
-      <c r="J80" s="1">
+      <c r="J80" s="2">
         <v>41275</v>
       </c>
       <c r="K80" t="b">
@@ -3945,7 +3971,7 @@
       <c r="I81" t="s">
         <v>313</v>
       </c>
-      <c r="J81" s="1">
+      <c r="J81" s="2">
         <v>45380</v>
       </c>
       <c r="K81" t="b">
@@ -3980,7 +4006,7 @@
       <c r="I82" t="s">
         <v>314</v>
       </c>
-      <c r="J82" s="1">
+      <c r="J82" s="2">
         <v>45421</v>
       </c>
       <c r="K82" t="b">
@@ -4015,7 +4041,7 @@
       <c r="I83" t="s">
         <v>314</v>
       </c>
-      <c r="J83" s="1">
+      <c r="J83" s="2">
         <v>45428</v>
       </c>
       <c r="K83" t="b">
@@ -4050,7 +4076,7 @@
       <c r="I84" t="s">
         <v>315</v>
       </c>
-      <c r="J84" s="1">
+      <c r="J84" s="2">
         <v>45490</v>
       </c>
       <c r="K84" t="b">
@@ -4085,7 +4111,7 @@
       <c r="I85" t="s">
         <v>316</v>
       </c>
-      <c r="J85" s="1">
+      <c r="J85" s="2">
         <v>45566</v>
       </c>
       <c r="K85" t="b">
@@ -4120,7 +4146,7 @@
       <c r="I86" t="s">
         <v>317</v>
       </c>
-      <c r="J86" s="1">
+      <c r="J86" s="2">
         <v>45986</v>
       </c>
       <c r="K86" t="b">
@@ -4155,7 +4181,7 @@
       <c r="I87" t="s">
         <v>318</v>
       </c>
-      <c r="J87" s="1">
+      <c r="J87" s="2">
         <v>46284</v>
       </c>
       <c r="K87" t="b">
@@ -4190,7 +4216,7 @@
       <c r="I88" t="s">
         <v>319</v>
       </c>
-      <c r="J88" s="1">
+      <c r="J88" s="2">
         <v>46305</v>
       </c>
       <c r="K88" t="b">
@@ -4225,7 +4251,7 @@
       <c r="I89" t="s">
         <v>319</v>
       </c>
-      <c r="J89" s="1">
+      <c r="J89" s="2">
         <v>46310</v>
       </c>
       <c r="K89" t="b">
@@ -4260,7 +4286,7 @@
       <c r="I90" t="s">
         <v>319</v>
       </c>
-      <c r="J90" s="1">
+      <c r="J90" s="2">
         <v>46317</v>
       </c>
       <c r="K90" t="b">
@@ -4295,7 +4321,7 @@
       <c r="I91" t="s">
         <v>319</v>
       </c>
-      <c r="J91" s="1">
+      <c r="J91" s="2">
         <v>46319</v>
       </c>
       <c r="K91" t="b">
@@ -4330,7 +4356,7 @@
       <c r="I92" t="s">
         <v>320</v>
       </c>
-      <c r="J92" s="1">
+      <c r="J92" s="2">
         <v>46333</v>
       </c>
       <c r="K92" t="b">
@@ -4365,7 +4391,7 @@
       <c r="I93" t="s">
         <v>320</v>
       </c>
-      <c r="J93" s="1">
+      <c r="J93" s="2">
         <v>46338</v>
       </c>
       <c r="K93" t="b">
@@ -4400,7 +4426,7 @@
       <c r="I94" t="s">
         <v>320</v>
       </c>
-      <c r="J94" s="1">
+      <c r="J94" s="2">
         <v>46338</v>
       </c>
       <c r="K94" t="b">
@@ -4435,7 +4461,7 @@
       <c r="I95" t="s">
         <v>320</v>
       </c>
-      <c r="J95" s="1">
+      <c r="J95" s="2">
         <v>46341</v>
       </c>
       <c r="K95" t="b">
@@ -4470,7 +4496,7 @@
       <c r="I96" t="s">
         <v>320</v>
       </c>
-      <c r="J96" s="1">
+      <c r="J96" s="2">
         <v>46344</v>
       </c>
       <c r="K96" t="b">
@@ -4505,7 +4531,7 @@
       <c r="I97" t="s">
         <v>321</v>
       </c>
-      <c r="J97" s="1">
+      <c r="J97" s="2">
         <v>46360</v>
       </c>
       <c r="K97" t="b">
@@ -4540,7 +4566,7 @@
       <c r="I98" t="s">
         <v>321</v>
       </c>
-      <c r="J98" s="1">
+      <c r="J98" s="2">
         <v>46360</v>
       </c>
       <c r="K98" t="b">
@@ -4575,7 +4601,7 @@
       <c r="I99" t="s">
         <v>321</v>
       </c>
-      <c r="J99" s="1">
+      <c r="J99" s="2">
         <v>46367</v>
       </c>
       <c r="K99" t="b">
@@ -4610,7 +4636,7 @@
       <c r="I100" t="s">
         <v>321</v>
       </c>
-      <c r="J100" s="1">
+      <c r="J100" s="2">
         <v>46375</v>
       </c>
       <c r="K100" t="b">
@@ -4645,7 +4671,7 @@
       <c r="I101" t="s">
         <v>321</v>
       </c>
-      <c r="J101" s="1">
+      <c r="J101" s="2">
         <v>46387</v>
       </c>
       <c r="K101" t="b">
@@ -4680,7 +4706,7 @@
       <c r="I102" t="s">
         <v>321</v>
       </c>
-      <c r="J102" s="1">
+      <c r="J102" s="2">
         <v>46387</v>
       </c>
       <c r="K102" t="b">
@@ -4715,7 +4741,7 @@
       <c r="I103" t="s">
         <v>321</v>
       </c>
-      <c r="J103" s="1">
+      <c r="J103" s="2">
         <v>46387</v>
       </c>
       <c r="K103" t="b">
@@ -4750,7 +4776,7 @@
       <c r="I104" t="s">
         <v>321</v>
       </c>
-      <c r="J104" s="1">
+      <c r="J104" s="2">
         <v>46388</v>
       </c>
       <c r="K104" t="b">
@@ -4785,7 +4811,7 @@
       <c r="I105" t="s">
         <v>322</v>
       </c>
-      <c r="J105" s="1">
+      <c r="J105" s="2">
         <v>46401</v>
       </c>
       <c r="K105" t="b">
@@ -4820,7 +4846,7 @@
       <c r="I106" t="s">
         <v>322</v>
       </c>
-      <c r="J106" s="1">
+      <c r="J106" s="2">
         <v>46401</v>
       </c>
       <c r="K106" t="b">
@@ -4855,7 +4881,7 @@
       <c r="I107" t="s">
         <v>322</v>
       </c>
-      <c r="J107" s="1">
+      <c r="J107" s="2">
         <v>46401</v>
       </c>
       <c r="K107" t="b">
@@ -4890,7 +4916,7 @@
       <c r="I108" t="s">
         <v>322</v>
       </c>
-      <c r="J108" s="1">
+      <c r="J108" s="2">
         <v>46412</v>
       </c>
       <c r="K108" t="b">
@@ -4925,7 +4951,7 @@
       <c r="I109" t="s">
         <v>322</v>
       </c>
-      <c r="J109" s="1">
+      <c r="J109" s="2">
         <v>46412</v>
       </c>
       <c r="K109" t="b">
@@ -4960,7 +4986,7 @@
       <c r="I110" t="s">
         <v>322</v>
       </c>
-      <c r="J110" s="1">
+      <c r="J110" s="2">
         <v>46412</v>
       </c>
       <c r="K110" t="b">
@@ -4995,7 +5021,7 @@
       <c r="I111" t="s">
         <v>323</v>
       </c>
-      <c r="J111" s="1">
+      <c r="J111" s="2">
         <v>46424</v>
       </c>
       <c r="K111" t="b">
@@ -5030,7 +5056,7 @@
       <c r="I112" t="s">
         <v>323</v>
       </c>
-      <c r="J112" s="1">
+      <c r="J112" s="2">
         <v>46437</v>
       </c>
       <c r="K112" t="b">
@@ -5065,7 +5091,7 @@
       <c r="I113" t="s">
         <v>323</v>
       </c>
-      <c r="J113" s="1">
+      <c r="J113" s="2">
         <v>46451</v>
       </c>
       <c r="K113" t="b">
@@ -5100,7 +5126,7 @@
       <c r="I114" t="s">
         <v>323</v>
       </c>
-      <c r="J114" s="1">
+      <c r="J114" s="2">
         <v>46451</v>
       </c>
       <c r="K114" t="b">
@@ -5135,7 +5161,7 @@
       <c r="I115" t="s">
         <v>324</v>
       </c>
-      <c r="J115" s="1">
+      <c r="J115" s="2">
         <v>46455</v>
       </c>
       <c r="K115" t="b">
@@ -5170,7 +5196,7 @@
       <c r="I116" t="s">
         <v>324</v>
       </c>
-      <c r="J116" s="1">
+      <c r="J116" s="2">
         <v>46456</v>
       </c>
       <c r="K116" t="b">
@@ -5205,7 +5231,7 @@
       <c r="I117" t="s">
         <v>324</v>
       </c>
-      <c r="J117" s="1">
+      <c r="J117" s="2">
         <v>46457</v>
       </c>
       <c r="K117" t="b">
@@ -5240,7 +5266,7 @@
       <c r="I118" t="s">
         <v>324</v>
       </c>
-      <c r="J118" s="1">
+      <c r="J118" s="2">
         <v>46464</v>
       </c>
       <c r="K118" t="b">
@@ -5275,7 +5301,7 @@
       <c r="I119" t="s">
         <v>324</v>
       </c>
-      <c r="J119" s="1">
+      <c r="J119" s="2">
         <v>46470</v>
       </c>
       <c r="K119" t="b">
@@ -5310,7 +5336,7 @@
       <c r="I120" t="s">
         <v>325</v>
       </c>
-      <c r="J120" s="1">
+      <c r="J120" s="2">
         <v>46485</v>
       </c>
       <c r="K120" t="b">
@@ -5345,7 +5371,7 @@
       <c r="I121" t="s">
         <v>325</v>
       </c>
-      <c r="J121" s="1">
+      <c r="J121" s="2">
         <v>46499</v>
       </c>
       <c r="K121" t="b">
@@ -5380,7 +5406,7 @@
       <c r="I122" t="s">
         <v>325</v>
       </c>
-      <c r="J122" s="1">
+      <c r="J122" s="2">
         <v>46504</v>
       </c>
       <c r="K122" t="b">
@@ -5415,7 +5441,7 @@
       <c r="I123" t="s">
         <v>325</v>
       </c>
-      <c r="J123" s="1">
+      <c r="J123" s="2">
         <v>46504</v>
       </c>
       <c r="K123" t="b">
@@ -5450,7 +5476,7 @@
       <c r="I124" t="s">
         <v>325</v>
       </c>
-      <c r="J124" s="1">
+      <c r="J124" s="2">
         <v>46507</v>
       </c>
       <c r="K124" t="b">
@@ -5485,7 +5511,7 @@
       <c r="I125" t="s">
         <v>325</v>
       </c>
-      <c r="J125" s="1">
+      <c r="J125" s="2">
         <v>46508</v>
       </c>
       <c r="K125" t="b">
@@ -5520,7 +5546,7 @@
       <c r="I126" t="s">
         <v>325</v>
       </c>
-      <c r="J126" s="1">
+      <c r="J126" s="2">
         <v>46512</v>
       </c>
       <c r="K126" t="b">
@@ -5555,7 +5581,7 @@
       <c r="I127" t="s">
         <v>326</v>
       </c>
-      <c r="J127" s="1">
+      <c r="J127" s="2">
         <v>46512</v>
       </c>
       <c r="K127" t="b">
@@ -5590,7 +5616,7 @@
       <c r="I128" t="s">
         <v>326</v>
       </c>
-      <c r="J128" s="1">
+      <c r="J128" s="2">
         <v>46528</v>
       </c>
       <c r="K128" t="b">
@@ -5625,7 +5651,7 @@
       <c r="I129" t="s">
         <v>326</v>
       </c>
-      <c r="J129" s="1">
+      <c r="J129" s="2">
         <v>46529</v>
       </c>
       <c r="K129" t="b">
@@ -5660,7 +5686,7 @@
       <c r="I130" t="s">
         <v>326</v>
       </c>
-      <c r="J130" s="1">
+      <c r="J130" s="2">
         <v>46537</v>
       </c>
       <c r="K130" t="b">
@@ -5695,7 +5721,7 @@
       <c r="I131" t="s">
         <v>327</v>
       </c>
-      <c r="J131" s="1">
+      <c r="J131" s="2">
         <v>46546</v>
       </c>
       <c r="K131" t="b">
@@ -5730,7 +5756,7 @@
       <c r="I132" t="s">
         <v>327</v>
       </c>
-      <c r="J132" s="1">
+      <c r="J132" s="2">
         <v>46547</v>
       </c>
       <c r="K132" t="b">
@@ -5765,7 +5791,7 @@
       <c r="I133" t="s">
         <v>327</v>
       </c>
-      <c r="J133" s="1">
+      <c r="J133" s="2">
         <v>46547</v>
       </c>
       <c r="K133" t="b">
@@ -5800,7 +5826,7 @@
       <c r="I134" t="s">
         <v>327</v>
       </c>
-      <c r="J134" s="1">
+      <c r="J134" s="2">
         <v>46547</v>
       </c>
       <c r="K134" t="b">
@@ -5835,7 +5861,7 @@
       <c r="I135" t="s">
         <v>327</v>
       </c>
-      <c r="J135" s="1">
+      <c r="J135" s="2">
         <v>46551</v>
       </c>
       <c r="K135" t="b">
@@ -5870,7 +5896,7 @@
       <c r="I136" t="s">
         <v>327</v>
       </c>
-      <c r="J136" s="1">
+      <c r="J136" s="2">
         <v>46560</v>
       </c>
       <c r="K136" t="b">
@@ -5905,7 +5931,7 @@
       <c r="I137" t="s">
         <v>327</v>
       </c>
-      <c r="J137" s="1">
+      <c r="J137" s="2">
         <v>46564</v>
       </c>
       <c r="K137" t="b">
@@ -5940,7 +5966,7 @@
       <c r="I138" t="s">
         <v>327</v>
       </c>
-      <c r="J138" s="1">
+      <c r="J138" s="2">
         <v>46567</v>
       </c>
       <c r="K138" t="b">
@@ -5975,7 +6001,7 @@
       <c r="I139" t="s">
         <v>327</v>
       </c>
-      <c r="J139" s="1">
+      <c r="J139" s="2">
         <v>46568</v>
       </c>
       <c r="K139" t="b">
@@ -6010,7 +6036,7 @@
       <c r="I140" t="s">
         <v>328</v>
       </c>
-      <c r="J140" s="1">
+      <c r="J140" s="2">
         <v>46578</v>
       </c>
       <c r="K140" t="b">
@@ -6045,7 +6071,7 @@
       <c r="I141" t="s">
         <v>328</v>
       </c>
-      <c r="J141" s="1">
+      <c r="J141" s="2">
         <v>46592</v>
       </c>
       <c r="K141" t="b">
@@ -6080,7 +6106,7 @@
       <c r="I142" t="s">
         <v>328</v>
       </c>
-      <c r="J142" s="1">
+      <c r="J142" s="2">
         <v>46592</v>
       </c>
       <c r="K142" t="b">
@@ -6115,7 +6141,7 @@
       <c r="I143" t="s">
         <v>329</v>
       </c>
-      <c r="J143" s="1">
+      <c r="J143" s="2">
         <v>46212</v>
       </c>
       <c r="K143" t="b">
@@ -6150,7 +6176,7 @@
       <c r="I144" t="s">
         <v>330</v>
       </c>
-      <c r="J144" s="1">
+      <c r="J144" s="2">
         <v>46225</v>
       </c>
       <c r="K144" t="b">
@@ -6185,7 +6211,7 @@
       <c r="I145" t="s">
         <v>331</v>
       </c>
-      <c r="J145" s="1">
+      <c r="J145" s="2">
         <v>46263</v>
       </c>
       <c r="K145" t="b">
@@ -6217,7 +6243,7 @@
       <c r="H146">
         <v>-1476</v>
       </c>
-      <c r="J146" s="1">
+      <c r="J146" s="2">
         <v>43773</v>
       </c>
       <c r="K146" t="b">
@@ -6249,7 +6275,7 @@
       <c r="H147">
         <v>-1469</v>
       </c>
-      <c r="J147" s="1">
+      <c r="J147" s="2">
         <v>43773</v>
       </c>
       <c r="K147" t="b">
@@ -6281,7 +6307,7 @@
       <c r="H148">
         <v>-1186</v>
       </c>
-      <c r="J148" s="1">
+      <c r="J148" s="2">
         <v>45295</v>
       </c>
       <c r="K148" t="b">
@@ -6313,7 +6339,7 @@
       <c r="H149">
         <v>-1048</v>
       </c>
-      <c r="J149" s="1">
+      <c r="J149" s="2">
         <v>45617</v>
       </c>
       <c r="K149" t="b">
@@ -6345,7 +6371,7 @@
       <c r="H150">
         <v>-980</v>
       </c>
-      <c r="J150" s="1">
+      <c r="J150" s="2">
         <v>45677</v>
       </c>
       <c r="K150" t="b">
@@ -6377,7 +6403,7 @@
       <c r="H151">
         <v>-961</v>
       </c>
-      <c r="J151" s="1">
+      <c r="J151" s="2">
         <v>44944</v>
       </c>
       <c r="K151" t="b">
@@ -6409,7 +6435,7 @@
       <c r="H152">
         <v>-252</v>
       </c>
-      <c r="J152" s="1">
+      <c r="J152" s="2">
         <v>46092</v>
       </c>
       <c r="K152" t="b">
@@ -6441,7 +6467,7 @@
       <c r="H153">
         <v>3</v>
       </c>
-      <c r="J153" s="1">
+      <c r="J153" s="2">
         <v>46265</v>
       </c>
       <c r="K153" t="b">
@@ -6473,7 +6499,7 @@
       <c r="H154">
         <v>3</v>
       </c>
-      <c r="J154" s="1">
+      <c r="J154" s="2">
         <v>46265</v>
       </c>
       <c r="K154" t="b">
@@ -6505,7 +6531,7 @@
       <c r="H155">
         <v>43</v>
       </c>
-      <c r="J155" s="1">
+      <c r="J155" s="2">
         <v>46440</v>
       </c>
       <c r="K155" t="b">
@@ -6537,7 +6563,7 @@
       <c r="H156">
         <v>43</v>
       </c>
-      <c r="J156" s="1">
+      <c r="J156" s="2">
         <v>46440</v>
       </c>
       <c r="K156" t="b">
@@ -6569,7 +6595,7 @@
       <c r="H157">
         <v>72</v>
       </c>
-      <c r="J157" s="1">
+      <c r="J157" s="2">
         <v>46289</v>
       </c>
       <c r="K157" t="b">
@@ -6601,7 +6627,7 @@
       <c r="H158">
         <v>72</v>
       </c>
-      <c r="J158" s="1">
+      <c r="J158" s="2">
         <v>46289</v>
       </c>
       <c r="K158" t="b">
@@ -6633,7 +6659,7 @@
       <c r="H159">
         <v>81</v>
       </c>
-      <c r="J159" s="1">
+      <c r="J159" s="2">
         <v>46405</v>
       </c>
       <c r="K159" t="b">
@@ -6665,7 +6691,7 @@
       <c r="H160">
         <v>102</v>
       </c>
-      <c r="J160" s="1">
+      <c r="J160" s="2">
         <v>46463</v>
       </c>
       <c r="K160" t="b">
@@ -6697,7 +6723,7 @@
       <c r="H161">
         <v>109</v>
       </c>
-      <c r="J161" s="1">
+      <c r="J161" s="2">
         <v>46353</v>
       </c>
       <c r="K161" t="b">
@@ -6729,7 +6755,7 @@
       <c r="H162">
         <v>127</v>
       </c>
-      <c r="J162" s="1">
+      <c r="J162" s="2">
         <v>46417</v>
       </c>
       <c r="K162" t="b">
@@ -6761,7 +6787,7 @@
       <c r="H163">
         <v>152</v>
       </c>
-      <c r="J163" s="1">
+      <c r="J163" s="2">
         <v>46271</v>
       </c>
       <c r="K163" t="b">
@@ -6793,7 +6819,7 @@
       <c r="H164">
         <v>152</v>
       </c>
-      <c r="J164" s="1">
+      <c r="J164" s="2">
         <v>46271</v>
       </c>
       <c r="K164" t="b">
@@ -6825,7 +6851,7 @@
       <c r="H165">
         <v>153</v>
       </c>
-      <c r="J165" s="1">
+      <c r="J165" s="2">
         <v>46458</v>
       </c>
       <c r="K165" t="b">
@@ -6857,7 +6883,7 @@
       <c r="H166">
         <v>158</v>
       </c>
-      <c r="J166" s="1">
+      <c r="J166" s="2">
         <v>46381</v>
       </c>
       <c r="K166" t="b">
@@ -6889,7 +6915,7 @@
       <c r="H167">
         <v>163</v>
       </c>
-      <c r="J167" s="1">
+      <c r="J167" s="2">
         <v>46592</v>
       </c>
       <c r="K167" t="b">
@@ -6921,7 +6947,7 @@
       <c r="H168">
         <v>167</v>
       </c>
-      <c r="J168" s="1">
+      <c r="J168" s="2">
         <v>46441</v>
       </c>
       <c r="K168" t="b">
@@ -6953,7 +6979,7 @@
       <c r="H169">
         <v>169</v>
       </c>
-      <c r="J169" s="1">
+      <c r="J169" s="2">
         <v>46391</v>
       </c>
       <c r="K169" t="b">
@@ -6985,7 +7011,7 @@
       <c r="H170">
         <v>184</v>
       </c>
-      <c r="J170" s="1">
+      <c r="J170" s="2">
         <v>46385</v>
       </c>
       <c r="K170" t="b">
@@ -7017,7 +7043,7 @@
       <c r="H171">
         <v>186</v>
       </c>
-      <c r="J171" s="1">
+      <c r="J171" s="2">
         <v>46387</v>
       </c>
       <c r="K171" t="b">
@@ -7049,7 +7075,7 @@
       <c r="H172">
         <v>206</v>
       </c>
-      <c r="J172" s="1">
+      <c r="J172" s="2">
         <v>46399</v>
       </c>
       <c r="K172" t="b">
@@ -7081,7 +7107,7 @@
       <c r="H173">
         <v>206</v>
       </c>
-      <c r="J173" s="1">
+      <c r="J173" s="2">
         <v>46399</v>
       </c>
       <c r="K173" t="b">
@@ -7113,7 +7139,7 @@
       <c r="H174">
         <v>234</v>
       </c>
-      <c r="J174" s="1">
+      <c r="J174" s="2">
         <v>46458</v>
       </c>
       <c r="K174" t="b">
@@ -7145,7 +7171,7 @@
       <c r="H175">
         <v>248</v>
       </c>
-      <c r="J175" s="1">
+      <c r="J175" s="2">
         <v>46528</v>
       </c>
       <c r="K175" t="b">
@@ -7177,7 +7203,7 @@
       <c r="H176">
         <v>317</v>
       </c>
-      <c r="J176" s="1">
+      <c r="J176" s="2">
         <v>46540</v>
       </c>
       <c r="K176" t="b">
@@ -7209,7 +7235,7 @@
       <c r="H177">
         <v>340</v>
       </c>
-      <c r="J177" s="1">
+      <c r="J177" s="2">
         <v>46547</v>
       </c>
       <c r="K177" t="b">
@@ -7241,7 +7267,7 @@
       <c r="H178">
         <v>364</v>
       </c>
-      <c r="J178" s="1">
+      <c r="J178" s="2">
         <v>46557</v>
       </c>
       <c r="K178" t="b">
@@ -7273,7 +7299,7 @@
       <c r="H179">
         <v>368</v>
       </c>
-      <c r="J179" s="1">
+      <c r="J179" s="2">
         <v>46571</v>
       </c>
       <c r="K179" t="b">
@@ -7305,7 +7331,7 @@
       <c r="H180">
         <v>368</v>
       </c>
-      <c r="J180" s="1">
+      <c r="J180" s="2">
         <v>46571</v>
       </c>
       <c r="K180" t="b">
@@ -7337,7 +7363,7 @@
       <c r="H181">
         <v>370</v>
       </c>
-      <c r="J181" s="1">
+      <c r="J181" s="2">
         <v>46562</v>
       </c>
       <c r="K181" t="b">
@@ -7369,7 +7395,7 @@
       <c r="H182">
         <v>385</v>
       </c>
-      <c r="J182" s="1">
+      <c r="J182" s="2">
         <v>46574</v>
       </c>
       <c r="K182" t="b">
@@ -7401,7 +7427,7 @@
       <c r="H183">
         <v>385</v>
       </c>
-      <c r="J183" s="1">
+      <c r="J183" s="2">
         <v>46574</v>
       </c>
       <c r="K183" t="b">
@@ -7433,7 +7459,7 @@
       <c r="H184">
         <v>417</v>
       </c>
-      <c r="J184" s="1">
+      <c r="J184" s="2">
         <v>46578</v>
       </c>
       <c r="K184" t="b">
@@ -7465,7 +7491,7 @@
       <c r="H185">
         <v>721</v>
       </c>
-      <c r="J185" s="1">
+      <c r="J185" s="2">
         <v>46345</v>
       </c>
       <c r="K185" t="b">
@@ -7497,7 +7523,7 @@
       <c r="H186">
         <v>721</v>
       </c>
-      <c r="J186" s="1">
+      <c r="J186" s="2">
         <v>46345</v>
       </c>
       <c r="K186" t="b">
@@ -7529,7 +7555,7 @@
       <c r="H187">
         <v>850</v>
       </c>
-      <c r="J187" s="1">
+      <c r="J187" s="2">
         <v>46366</v>
       </c>
       <c r="K187" t="b">
@@ -7561,7 +7587,7 @@
       <c r="H188">
         <v>850</v>
       </c>
-      <c r="J188" s="1">
+      <c r="J188" s="2">
         <v>46366</v>
       </c>
       <c r="K188" t="b">
@@ -7593,7 +7619,7 @@
       <c r="H189">
         <v>1661</v>
       </c>
-      <c r="J189" s="1">
+      <c r="J189" s="2">
         <v>46524</v>
       </c>
       <c r="K189" t="b">
@@ -7625,7 +7651,7 @@
       <c r="H190">
         <v>1661</v>
       </c>
-      <c r="J190" s="1">
+      <c r="J190" s="2">
         <v>46524</v>
       </c>
       <c r="K190" t="b">
@@ -7657,7 +7683,7 @@
       <c r="H191">
         <v>488</v>
       </c>
-      <c r="J191" s="1">
+      <c r="J191" s="2">
         <v>46190</v>
       </c>
       <c r="K191" t="b">
@@ -7689,7 +7715,7 @@
       <c r="H192">
         <v>25565</v>
       </c>
-      <c r="J192" s="1">
+      <c r="J192" s="2">
         <v>46190</v>
       </c>
       <c r="K192" t="b">
@@ -7721,7 +7747,7 @@
       <c r="H193">
         <v>25567</v>
       </c>
-      <c r="J193" s="1">
+      <c r="J193" s="2">
         <v>46190</v>
       </c>
       <c r="K193" t="b">
@@ -7753,7 +7779,7 @@
       <c r="H194">
         <v>31293</v>
       </c>
-      <c r="J194" s="1">
+      <c r="J194" s="2">
         <v>46190</v>
       </c>
       <c r="K194" t="b">

</xml_diff>

<commit_message>
Atualização automática: vencimentos_tmot (08/09/2026 12:04)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
@@ -1019,16 +1019,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1044,7 +1036,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1052,30 +1044,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1375,37 +1349,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1434,7 +1408,7 @@
       <c r="H2">
         <v>-4300.3</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>39285</v>
       </c>
       <c r="K2" t="b">
@@ -1466,7 +1440,7 @@
       <c r="H3">
         <v>-2354.2</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>40669</v>
       </c>
       <c r="K3" t="b">
@@ -1498,7 +1472,7 @@
       <c r="H4">
         <v>-910.7</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>40669</v>
       </c>
       <c r="K4" t="b">
@@ -1530,7 +1504,7 @@
       <c r="H5">
         <v>-868</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>44884</v>
       </c>
       <c r="K5" t="b">
@@ -1562,7 +1536,7 @@
       <c r="H6">
         <v>-483.8</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>43855</v>
       </c>
       <c r="K6" t="b">
@@ -1594,7 +1568,7 @@
       <c r="H7">
         <v>-417</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>46014</v>
       </c>
       <c r="K7" t="b">
@@ -1626,7 +1600,7 @@
       <c r="H8">
         <v>-414.2</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>46014</v>
       </c>
       <c r="K8" t="b">
@@ -1658,7 +1632,7 @@
       <c r="H9">
         <v>-391.8</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>42769</v>
       </c>
       <c r="K9" t="b">
@@ -1690,7 +1664,7 @@
       <c r="H10">
         <v>-391.6</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>45804</v>
       </c>
       <c r="K10" t="b">
@@ -1722,7 +1696,7 @@
       <c r="H11">
         <v>-391.6</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>45804</v>
       </c>
       <c r="K11" t="b">
@@ -1754,7 +1728,7 @@
       <c r="H12">
         <v>-372.9</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>42821</v>
       </c>
       <c r="K12" t="b">
@@ -1786,7 +1760,7 @@
       <c r="H13">
         <v>-372.9</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>46014</v>
       </c>
       <c r="K13" t="b">
@@ -1818,7 +1792,7 @@
       <c r="H14">
         <v>-372.9</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>46014</v>
       </c>
       <c r="K14" t="b">
@@ -1850,7 +1824,7 @@
       <c r="H15">
         <v>-372.9</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <v>46014</v>
       </c>
       <c r="K15" t="b">
@@ -1882,7 +1856,7 @@
       <c r="H16">
         <v>-367.8</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <v>46017</v>
       </c>
       <c r="K16" t="b">
@@ -1914,7 +1888,7 @@
       <c r="H17">
         <v>-367.8</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="1">
         <v>46017</v>
       </c>
       <c r="K17" t="b">
@@ -1946,7 +1920,7 @@
       <c r="H18">
         <v>-347.2</v>
       </c>
-      <c r="J18" s="2">
+      <c r="J18" s="1">
         <v>40979</v>
       </c>
       <c r="K18" t="b">
@@ -1978,7 +1952,7 @@
       <c r="H19">
         <v>-293.8</v>
       </c>
-      <c r="J19" s="2">
+      <c r="J19" s="1">
         <v>45846</v>
       </c>
       <c r="K19" t="b">
@@ -2010,7 +1984,7 @@
       <c r="H20">
         <v>-206.4</v>
       </c>
-      <c r="J20" s="2">
+      <c r="J20" s="1">
         <v>36669</v>
       </c>
       <c r="K20" t="b">
@@ -2042,7 +2016,7 @@
       <c r="H21">
         <v>-131.6</v>
       </c>
-      <c r="J21" s="2">
+      <c r="J21" s="1">
         <v>46111</v>
       </c>
       <c r="K21" t="b">
@@ -2074,7 +2048,7 @@
       <c r="H22">
         <v>-131.6</v>
       </c>
-      <c r="J22" s="2">
+      <c r="J22" s="1">
         <v>46111</v>
       </c>
       <c r="K22" t="b">
@@ -2106,7 +2080,7 @@
       <c r="H23">
         <v>-131.6</v>
       </c>
-      <c r="J23" s="2">
+      <c r="J23" s="1">
         <v>46111</v>
       </c>
       <c r="K23" t="b">
@@ -2138,7 +2112,7 @@
       <c r="H24">
         <v>-131.6</v>
       </c>
-      <c r="J24" s="2">
+      <c r="J24" s="1">
         <v>46111</v>
       </c>
       <c r="K24" t="b">
@@ -2170,7 +2144,7 @@
       <c r="H25">
         <v>-131.6</v>
       </c>
-      <c r="J25" s="2">
+      <c r="J25" s="1">
         <v>46111</v>
       </c>
       <c r="K25" t="b">
@@ -2202,7 +2176,7 @@
       <c r="H26">
         <v>-98.3</v>
       </c>
-      <c r="J26" s="2">
+      <c r="J26" s="1">
         <v>41204</v>
       </c>
       <c r="K26" t="b">
@@ -2234,7 +2208,7 @@
       <c r="H27">
         <v>-47.2</v>
       </c>
-      <c r="J27" s="2">
+      <c r="J27" s="1">
         <v>44011</v>
       </c>
       <c r="K27" t="b">
@@ -2266,7 +2240,7 @@
       <c r="H28">
         <v>-22.3</v>
       </c>
-      <c r="J28" s="2">
+      <c r="J28" s="1">
         <v>46226</v>
       </c>
       <c r="K28" t="b">
@@ -2298,7 +2272,7 @@
       <c r="H29">
         <v>4.7</v>
       </c>
-      <c r="J29" s="2">
+      <c r="J29" s="1">
         <v>46265</v>
       </c>
       <c r="K29" t="b">
@@ -2330,7 +2304,7 @@
       <c r="H30">
         <v>7.5</v>
       </c>
-      <c r="J30" s="2">
+      <c r="J30" s="1">
         <v>46265</v>
       </c>
       <c r="K30" t="b">
@@ -2362,7 +2336,7 @@
       <c r="H31">
         <v>10</v>
       </c>
-      <c r="J31" s="2">
+      <c r="J31" s="1">
         <v>46265</v>
       </c>
       <c r="K31" t="b">
@@ -2394,7 +2368,7 @@
       <c r="H32">
         <v>12.8</v>
       </c>
-      <c r="J32" s="2">
+      <c r="J32" s="1">
         <v>46265</v>
       </c>
       <c r="K32" t="b">
@@ -2426,7 +2400,7 @@
       <c r="H33">
         <v>14</v>
       </c>
-      <c r="J33" s="2">
+      <c r="J33" s="1">
         <v>46265</v>
       </c>
       <c r="K33" t="b">
@@ -2458,7 +2432,7 @@
       <c r="H34">
         <v>17.8</v>
       </c>
-      <c r="J34" s="2">
+      <c r="J34" s="1">
         <v>46265</v>
       </c>
       <c r="K34" t="b">
@@ -2490,7 +2464,7 @@
       <c r="H35">
         <v>20.4</v>
       </c>
-      <c r="J35" s="2">
+      <c r="J35" s="1">
         <v>46265</v>
       </c>
       <c r="K35" t="b">
@@ -2522,7 +2496,7 @@
       <c r="H36">
         <v>21.2</v>
       </c>
-      <c r="J36" s="2">
+      <c r="J36" s="1">
         <v>46265</v>
       </c>
       <c r="K36" t="b">
@@ -2554,7 +2528,7 @@
       <c r="H37">
         <v>26.2</v>
       </c>
-      <c r="J37" s="2">
+      <c r="J37" s="1">
         <v>46265</v>
       </c>
       <c r="K37" t="b">
@@ -2586,7 +2560,7 @@
       <c r="H38">
         <v>33.6</v>
       </c>
-      <c r="J38" s="2">
+      <c r="J38" s="1">
         <v>46364</v>
       </c>
       <c r="K38" t="b">
@@ -2618,7 +2592,7 @@
       <c r="H39">
         <v>42.2</v>
       </c>
-      <c r="J39" s="2">
+      <c r="J39" s="1">
         <v>46269</v>
       </c>
       <c r="K39" t="b">
@@ -2650,7 +2624,7 @@
       <c r="H40">
         <v>42.8</v>
       </c>
-      <c r="J40" s="2">
+      <c r="J40" s="1">
         <v>46291</v>
       </c>
       <c r="K40" t="b">
@@ -2682,7 +2656,7 @@
       <c r="H41">
         <v>45.7</v>
       </c>
-      <c r="J41" s="2">
+      <c r="J41" s="1">
         <v>46395</v>
       </c>
       <c r="K41" t="b">
@@ -2714,7 +2688,7 @@
       <c r="H42">
         <v>47.2</v>
       </c>
-      <c r="J42" s="2">
+      <c r="J42" s="1">
         <v>46280</v>
       </c>
       <c r="K42" t="b">
@@ -2746,7 +2720,7 @@
       <c r="H43">
         <v>48.7</v>
       </c>
-      <c r="J43" s="2">
+      <c r="J43" s="1">
         <v>46281</v>
       </c>
       <c r="K43" t="b">
@@ -2778,7 +2752,7 @@
       <c r="H44">
         <v>60</v>
       </c>
-      <c r="J44" s="2">
+      <c r="J44" s="1">
         <v>46281</v>
       </c>
       <c r="K44" t="b">
@@ -2810,7 +2784,7 @@
       <c r="H45">
         <v>62.6</v>
       </c>
-      <c r="J45" s="2">
+      <c r="J45" s="1">
         <v>46265</v>
       </c>
       <c r="K45" t="b">
@@ -2842,7 +2816,7 @@
       <c r="H46">
         <v>64.59999999999999</v>
       </c>
-      <c r="J46" s="2">
+      <c r="J46" s="1">
         <v>46265</v>
       </c>
       <c r="K46" t="b">
@@ -2874,7 +2848,7 @@
       <c r="H47">
         <v>67.59999999999999</v>
       </c>
-      <c r="J47" s="2">
+      <c r="J47" s="1">
         <v>46267</v>
       </c>
       <c r="K47" t="b">
@@ -2906,7 +2880,7 @@
       <c r="H48">
         <v>68.3</v>
       </c>
-      <c r="J48" s="2">
+      <c r="J48" s="1">
         <v>46278</v>
       </c>
       <c r="K48" t="b">
@@ -2938,7 +2912,7 @@
       <c r="H49">
         <v>69.2</v>
       </c>
-      <c r="J49" s="2">
+      <c r="J49" s="1">
         <v>46453</v>
       </c>
       <c r="K49" t="b">
@@ -2970,7 +2944,7 @@
       <c r="H50">
         <v>69.8</v>
       </c>
-      <c r="J50" s="2">
+      <c r="J50" s="1">
         <v>46265</v>
       </c>
       <c r="K50" t="b">
@@ -3002,7 +2976,7 @@
       <c r="H51">
         <v>69.8</v>
       </c>
-      <c r="J51" s="2">
+      <c r="J51" s="1">
         <v>46265</v>
       </c>
       <c r="K51" t="b">
@@ -3034,7 +3008,7 @@
       <c r="H52">
         <v>72.2</v>
       </c>
-      <c r="J52" s="2">
+      <c r="J52" s="1">
         <v>46275</v>
       </c>
       <c r="K52" t="b">
@@ -3066,7 +3040,7 @@
       <c r="H53">
         <v>72.2</v>
       </c>
-      <c r="J53" s="2">
+      <c r="J53" s="1">
         <v>46275</v>
       </c>
       <c r="K53" t="b">
@@ -3098,7 +3072,7 @@
       <c r="H54">
         <v>78.09999999999999</v>
       </c>
-      <c r="J54" s="2">
+      <c r="J54" s="1">
         <v>46265</v>
       </c>
       <c r="K54" t="b">
@@ -3130,7 +3104,7 @@
       <c r="H55">
         <v>82.8</v>
       </c>
-      <c r="J55" s="2">
+      <c r="J55" s="1">
         <v>46487</v>
       </c>
       <c r="K55" t="b">
@@ -3162,7 +3136,7 @@
       <c r="H56">
         <v>83.09999999999999</v>
       </c>
-      <c r="J56" s="2">
+      <c r="J56" s="1">
         <v>46285</v>
       </c>
       <c r="K56" t="b">
@@ -3194,7 +3168,7 @@
       <c r="H57">
         <v>84.8</v>
       </c>
-      <c r="J57" s="2">
+      <c r="J57" s="1">
         <v>46492</v>
       </c>
       <c r="K57" t="b">
@@ -3226,7 +3200,7 @@
       <c r="H58">
         <v>104.9</v>
       </c>
-      <c r="J58" s="2">
+      <c r="J58" s="1">
         <v>46297</v>
       </c>
       <c r="K58" t="b">
@@ -3258,7 +3232,7 @@
       <c r="H59">
         <v>107.6</v>
       </c>
-      <c r="J59" s="2">
+      <c r="J59" s="1">
         <v>46283</v>
       </c>
       <c r="K59" t="b">
@@ -3290,7 +3264,7 @@
       <c r="H60">
         <v>111.9</v>
       </c>
-      <c r="J60" s="2">
+      <c r="J60" s="1">
         <v>46300</v>
       </c>
       <c r="K60" t="b">
@@ -3322,7 +3296,7 @@
       <c r="H61">
         <v>111.9</v>
       </c>
-      <c r="J61" s="2">
+      <c r="J61" s="1">
         <v>46300</v>
       </c>
       <c r="K61" t="b">
@@ -3354,7 +3328,7 @@
       <c r="H62">
         <v>111.9</v>
       </c>
-      <c r="J62" s="2">
+      <c r="J62" s="1">
         <v>46300</v>
       </c>
       <c r="K62" t="b">
@@ -3386,7 +3360,7 @@
       <c r="H63">
         <v>111.9</v>
       </c>
-      <c r="J63" s="2">
+      <c r="J63" s="1">
         <v>46300</v>
       </c>
       <c r="K63" t="b">
@@ -3418,7 +3392,7 @@
       <c r="H64">
         <v>111.9</v>
       </c>
-      <c r="J64" s="2">
+      <c r="J64" s="1">
         <v>46300</v>
       </c>
       <c r="K64" t="b">
@@ -3450,7 +3424,7 @@
       <c r="H65">
         <v>128.8</v>
       </c>
-      <c r="J65" s="2">
+      <c r="J65" s="1">
         <v>46308</v>
       </c>
       <c r="K65" t="b">
@@ -3482,7 +3456,7 @@
       <c r="H66">
         <v>131.1</v>
       </c>
-      <c r="J66" s="2">
+      <c r="J66" s="1">
         <v>46336</v>
       </c>
       <c r="K66" t="b">
@@ -3514,7 +3488,7 @@
       <c r="H67">
         <v>138.4</v>
       </c>
-      <c r="J67" s="2">
+      <c r="J67" s="1">
         <v>46343</v>
       </c>
       <c r="K67" t="b">
@@ -3546,7 +3520,7 @@
       <c r="H68">
         <v>141</v>
       </c>
-      <c r="J68" s="2">
+      <c r="J68" s="1">
         <v>46350</v>
       </c>
       <c r="K68" t="b">
@@ -3578,7 +3552,7 @@
       <c r="H69">
         <v>162</v>
       </c>
-      <c r="J69" s="2">
+      <c r="J69" s="1">
         <v>46391</v>
       </c>
       <c r="K69" t="b">
@@ -3610,7 +3584,7 @@
       <c r="H70">
         <v>167.2</v>
       </c>
-      <c r="J70" s="2">
+      <c r="J70" s="1">
         <v>46330</v>
       </c>
       <c r="K70" t="b">
@@ -3642,7 +3616,7 @@
       <c r="H71">
         <v>177.4</v>
       </c>
-      <c r="J71" s="2">
+      <c r="J71" s="1">
         <v>46418</v>
       </c>
       <c r="K71" t="b">
@@ -3674,7 +3648,7 @@
       <c r="H72">
         <v>200</v>
       </c>
-      <c r="J72" s="2">
+      <c r="J72" s="1">
         <v>46356</v>
       </c>
       <c r="K72" t="b">
@@ -3706,7 +3680,7 @@
       <c r="H73">
         <v>203.6</v>
       </c>
-      <c r="J73" s="2">
+      <c r="J73" s="1">
         <v>46436</v>
       </c>
       <c r="K73" t="b">
@@ -3738,7 +3712,7 @@
       <c r="H74">
         <v>221.2</v>
       </c>
-      <c r="J74" s="2">
+      <c r="J74" s="1">
         <v>46426</v>
       </c>
       <c r="K74" t="b">
@@ -3770,7 +3744,7 @@
       <c r="H75">
         <v>240.8</v>
       </c>
-      <c r="J75" s="2">
+      <c r="J75" s="1">
         <v>46450</v>
       </c>
       <c r="K75" t="b">
@@ -3802,7 +3776,7 @@
       <c r="H76">
         <v>245.8</v>
       </c>
-      <c r="J76" s="2">
+      <c r="J76" s="1">
         <v>46452</v>
       </c>
       <c r="K76" t="b">
@@ -3834,7 +3808,7 @@
       <c r="H77">
         <v>263.4</v>
       </c>
-      <c r="J77" s="2">
+      <c r="J77" s="1">
         <v>46322</v>
       </c>
       <c r="K77" t="b">
@@ -3866,7 +3840,7 @@
       <c r="H78">
         <v>275.2</v>
       </c>
-      <c r="J78" s="2">
+      <c r="J78" s="1">
         <v>46433</v>
       </c>
       <c r="K78" t="b">
@@ -3901,7 +3875,7 @@
       <c r="I79" t="s">
         <v>311</v>
       </c>
-      <c r="J79" s="2">
+      <c r="J79" s="1">
         <v>36557</v>
       </c>
       <c r="K79" t="b">
@@ -3936,7 +3910,7 @@
       <c r="I80" t="s">
         <v>312</v>
       </c>
-      <c r="J80" s="2">
+      <c r="J80" s="1">
         <v>41275</v>
       </c>
       <c r="K80" t="b">
@@ -3971,7 +3945,7 @@
       <c r="I81" t="s">
         <v>313</v>
       </c>
-      <c r="J81" s="2">
+      <c r="J81" s="1">
         <v>45380</v>
       </c>
       <c r="K81" t="b">
@@ -4006,7 +3980,7 @@
       <c r="I82" t="s">
         <v>314</v>
       </c>
-      <c r="J82" s="2">
+      <c r="J82" s="1">
         <v>45421</v>
       </c>
       <c r="K82" t="b">
@@ -4041,7 +4015,7 @@
       <c r="I83" t="s">
         <v>314</v>
       </c>
-      <c r="J83" s="2">
+      <c r="J83" s="1">
         <v>45428</v>
       </c>
       <c r="K83" t="b">
@@ -4076,7 +4050,7 @@
       <c r="I84" t="s">
         <v>315</v>
       </c>
-      <c r="J84" s="2">
+      <c r="J84" s="1">
         <v>45490</v>
       </c>
       <c r="K84" t="b">
@@ -4111,7 +4085,7 @@
       <c r="I85" t="s">
         <v>316</v>
       </c>
-      <c r="J85" s="2">
+      <c r="J85" s="1">
         <v>45566</v>
       </c>
       <c r="K85" t="b">
@@ -4146,7 +4120,7 @@
       <c r="I86" t="s">
         <v>317</v>
       </c>
-      <c r="J86" s="2">
+      <c r="J86" s="1">
         <v>45986</v>
       </c>
       <c r="K86" t="b">
@@ -4181,7 +4155,7 @@
       <c r="I87" t="s">
         <v>318</v>
       </c>
-      <c r="J87" s="2">
+      <c r="J87" s="1">
         <v>46284</v>
       </c>
       <c r="K87" t="b">
@@ -4216,7 +4190,7 @@
       <c r="I88" t="s">
         <v>319</v>
       </c>
-      <c r="J88" s="2">
+      <c r="J88" s="1">
         <v>46305</v>
       </c>
       <c r="K88" t="b">
@@ -4251,7 +4225,7 @@
       <c r="I89" t="s">
         <v>319</v>
       </c>
-      <c r="J89" s="2">
+      <c r="J89" s="1">
         <v>46310</v>
       </c>
       <c r="K89" t="b">
@@ -4286,7 +4260,7 @@
       <c r="I90" t="s">
         <v>319</v>
       </c>
-      <c r="J90" s="2">
+      <c r="J90" s="1">
         <v>46317</v>
       </c>
       <c r="K90" t="b">
@@ -4321,7 +4295,7 @@
       <c r="I91" t="s">
         <v>319</v>
       </c>
-      <c r="J91" s="2">
+      <c r="J91" s="1">
         <v>46319</v>
       </c>
       <c r="K91" t="b">
@@ -4356,7 +4330,7 @@
       <c r="I92" t="s">
         <v>320</v>
       </c>
-      <c r="J92" s="2">
+      <c r="J92" s="1">
         <v>46333</v>
       </c>
       <c r="K92" t="b">
@@ -4391,7 +4365,7 @@
       <c r="I93" t="s">
         <v>320</v>
       </c>
-      <c r="J93" s="2">
+      <c r="J93" s="1">
         <v>46338</v>
       </c>
       <c r="K93" t="b">
@@ -4426,7 +4400,7 @@
       <c r="I94" t="s">
         <v>320</v>
       </c>
-      <c r="J94" s="2">
+      <c r="J94" s="1">
         <v>46338</v>
       </c>
       <c r="K94" t="b">
@@ -4461,7 +4435,7 @@
       <c r="I95" t="s">
         <v>320</v>
       </c>
-      <c r="J95" s="2">
+      <c r="J95" s="1">
         <v>46341</v>
       </c>
       <c r="K95" t="b">
@@ -4496,7 +4470,7 @@
       <c r="I96" t="s">
         <v>320</v>
       </c>
-      <c r="J96" s="2">
+      <c r="J96" s="1">
         <v>46344</v>
       </c>
       <c r="K96" t="b">
@@ -4531,7 +4505,7 @@
       <c r="I97" t="s">
         <v>321</v>
       </c>
-      <c r="J97" s="2">
+      <c r="J97" s="1">
         <v>46360</v>
       </c>
       <c r="K97" t="b">
@@ -4566,7 +4540,7 @@
       <c r="I98" t="s">
         <v>321</v>
       </c>
-      <c r="J98" s="2">
+      <c r="J98" s="1">
         <v>46360</v>
       </c>
       <c r="K98" t="b">
@@ -4601,7 +4575,7 @@
       <c r="I99" t="s">
         <v>321</v>
       </c>
-      <c r="J99" s="2">
+      <c r="J99" s="1">
         <v>46367</v>
       </c>
       <c r="K99" t="b">
@@ -4636,7 +4610,7 @@
       <c r="I100" t="s">
         <v>321</v>
       </c>
-      <c r="J100" s="2">
+      <c r="J100" s="1">
         <v>46375</v>
       </c>
       <c r="K100" t="b">
@@ -4671,7 +4645,7 @@
       <c r="I101" t="s">
         <v>321</v>
       </c>
-      <c r="J101" s="2">
+      <c r="J101" s="1">
         <v>46387</v>
       </c>
       <c r="K101" t="b">
@@ -4706,7 +4680,7 @@
       <c r="I102" t="s">
         <v>321</v>
       </c>
-      <c r="J102" s="2">
+      <c r="J102" s="1">
         <v>46387</v>
       </c>
       <c r="K102" t="b">
@@ -4741,7 +4715,7 @@
       <c r="I103" t="s">
         <v>321</v>
       </c>
-      <c r="J103" s="2">
+      <c r="J103" s="1">
         <v>46387</v>
       </c>
       <c r="K103" t="b">
@@ -4776,7 +4750,7 @@
       <c r="I104" t="s">
         <v>321</v>
       </c>
-      <c r="J104" s="2">
+      <c r="J104" s="1">
         <v>46388</v>
       </c>
       <c r="K104" t="b">
@@ -4811,7 +4785,7 @@
       <c r="I105" t="s">
         <v>322</v>
       </c>
-      <c r="J105" s="2">
+      <c r="J105" s="1">
         <v>46401</v>
       </c>
       <c r="K105" t="b">
@@ -4846,7 +4820,7 @@
       <c r="I106" t="s">
         <v>322</v>
       </c>
-      <c r="J106" s="2">
+      <c r="J106" s="1">
         <v>46401</v>
       </c>
       <c r="K106" t="b">
@@ -4881,7 +4855,7 @@
       <c r="I107" t="s">
         <v>322</v>
       </c>
-      <c r="J107" s="2">
+      <c r="J107" s="1">
         <v>46401</v>
       </c>
       <c r="K107" t="b">
@@ -4916,7 +4890,7 @@
       <c r="I108" t="s">
         <v>322</v>
       </c>
-      <c r="J108" s="2">
+      <c r="J108" s="1">
         <v>46412</v>
       </c>
       <c r="K108" t="b">
@@ -4951,7 +4925,7 @@
       <c r="I109" t="s">
         <v>322</v>
       </c>
-      <c r="J109" s="2">
+      <c r="J109" s="1">
         <v>46412</v>
       </c>
       <c r="K109" t="b">
@@ -4986,7 +4960,7 @@
       <c r="I110" t="s">
         <v>322</v>
       </c>
-      <c r="J110" s="2">
+      <c r="J110" s="1">
         <v>46412</v>
       </c>
       <c r="K110" t="b">
@@ -5021,7 +4995,7 @@
       <c r="I111" t="s">
         <v>323</v>
       </c>
-      <c r="J111" s="2">
+      <c r="J111" s="1">
         <v>46424</v>
       </c>
       <c r="K111" t="b">
@@ -5056,7 +5030,7 @@
       <c r="I112" t="s">
         <v>323</v>
       </c>
-      <c r="J112" s="2">
+      <c r="J112" s="1">
         <v>46437</v>
       </c>
       <c r="K112" t="b">
@@ -5091,7 +5065,7 @@
       <c r="I113" t="s">
         <v>323</v>
       </c>
-      <c r="J113" s="2">
+      <c r="J113" s="1">
         <v>46451</v>
       </c>
       <c r="K113" t="b">
@@ -5126,7 +5100,7 @@
       <c r="I114" t="s">
         <v>323</v>
       </c>
-      <c r="J114" s="2">
+      <c r="J114" s="1">
         <v>46451</v>
       </c>
       <c r="K114" t="b">
@@ -5161,7 +5135,7 @@
       <c r="I115" t="s">
         <v>324</v>
       </c>
-      <c r="J115" s="2">
+      <c r="J115" s="1">
         <v>46455</v>
       </c>
       <c r="K115" t="b">
@@ -5196,7 +5170,7 @@
       <c r="I116" t="s">
         <v>324</v>
       </c>
-      <c r="J116" s="2">
+      <c r="J116" s="1">
         <v>46456</v>
       </c>
       <c r="K116" t="b">
@@ -5231,7 +5205,7 @@
       <c r="I117" t="s">
         <v>324</v>
       </c>
-      <c r="J117" s="2">
+      <c r="J117" s="1">
         <v>46457</v>
       </c>
       <c r="K117" t="b">
@@ -5266,7 +5240,7 @@
       <c r="I118" t="s">
         <v>324</v>
       </c>
-      <c r="J118" s="2">
+      <c r="J118" s="1">
         <v>46464</v>
       </c>
       <c r="K118" t="b">
@@ -5301,7 +5275,7 @@
       <c r="I119" t="s">
         <v>324</v>
       </c>
-      <c r="J119" s="2">
+      <c r="J119" s="1">
         <v>46470</v>
       </c>
       <c r="K119" t="b">
@@ -5336,7 +5310,7 @@
       <c r="I120" t="s">
         <v>325</v>
       </c>
-      <c r="J120" s="2">
+      <c r="J120" s="1">
         <v>46485</v>
       </c>
       <c r="K120" t="b">
@@ -5371,7 +5345,7 @@
       <c r="I121" t="s">
         <v>325</v>
       </c>
-      <c r="J121" s="2">
+      <c r="J121" s="1">
         <v>46499</v>
       </c>
       <c r="K121" t="b">
@@ -5406,7 +5380,7 @@
       <c r="I122" t="s">
         <v>325</v>
       </c>
-      <c r="J122" s="2">
+      <c r="J122" s="1">
         <v>46504</v>
       </c>
       <c r="K122" t="b">
@@ -5441,7 +5415,7 @@
       <c r="I123" t="s">
         <v>325</v>
       </c>
-      <c r="J123" s="2">
+      <c r="J123" s="1">
         <v>46504</v>
       </c>
       <c r="K123" t="b">
@@ -5476,7 +5450,7 @@
       <c r="I124" t="s">
         <v>325</v>
       </c>
-      <c r="J124" s="2">
+      <c r="J124" s="1">
         <v>46507</v>
       </c>
       <c r="K124" t="b">
@@ -5511,7 +5485,7 @@
       <c r="I125" t="s">
         <v>325</v>
       </c>
-      <c r="J125" s="2">
+      <c r="J125" s="1">
         <v>46508</v>
       </c>
       <c r="K125" t="b">
@@ -5546,7 +5520,7 @@
       <c r="I126" t="s">
         <v>325</v>
       </c>
-      <c r="J126" s="2">
+      <c r="J126" s="1">
         <v>46512</v>
       </c>
       <c r="K126" t="b">
@@ -5581,7 +5555,7 @@
       <c r="I127" t="s">
         <v>326</v>
       </c>
-      <c r="J127" s="2">
+      <c r="J127" s="1">
         <v>46512</v>
       </c>
       <c r="K127" t="b">
@@ -5616,7 +5590,7 @@
       <c r="I128" t="s">
         <v>326</v>
       </c>
-      <c r="J128" s="2">
+      <c r="J128" s="1">
         <v>46528</v>
       </c>
       <c r="K128" t="b">
@@ -5651,7 +5625,7 @@
       <c r="I129" t="s">
         <v>326</v>
       </c>
-      <c r="J129" s="2">
+      <c r="J129" s="1">
         <v>46529</v>
       </c>
       <c r="K129" t="b">
@@ -5686,7 +5660,7 @@
       <c r="I130" t="s">
         <v>326</v>
       </c>
-      <c r="J130" s="2">
+      <c r="J130" s="1">
         <v>46537</v>
       </c>
       <c r="K130" t="b">
@@ -5721,7 +5695,7 @@
       <c r="I131" t="s">
         <v>327</v>
       </c>
-      <c r="J131" s="2">
+      <c r="J131" s="1">
         <v>46546</v>
       </c>
       <c r="K131" t="b">
@@ -5756,7 +5730,7 @@
       <c r="I132" t="s">
         <v>327</v>
       </c>
-      <c r="J132" s="2">
+      <c r="J132" s="1">
         <v>46547</v>
       </c>
       <c r="K132" t="b">
@@ -5791,7 +5765,7 @@
       <c r="I133" t="s">
         <v>327</v>
       </c>
-      <c r="J133" s="2">
+      <c r="J133" s="1">
         <v>46547</v>
       </c>
       <c r="K133" t="b">
@@ -5826,7 +5800,7 @@
       <c r="I134" t="s">
         <v>327</v>
       </c>
-      <c r="J134" s="2">
+      <c r="J134" s="1">
         <v>46547</v>
       </c>
       <c r="K134" t="b">
@@ -5861,7 +5835,7 @@
       <c r="I135" t="s">
         <v>327</v>
       </c>
-      <c r="J135" s="2">
+      <c r="J135" s="1">
         <v>46551</v>
       </c>
       <c r="K135" t="b">
@@ -5896,7 +5870,7 @@
       <c r="I136" t="s">
         <v>327</v>
       </c>
-      <c r="J136" s="2">
+      <c r="J136" s="1">
         <v>46560</v>
       </c>
       <c r="K136" t="b">
@@ -5931,7 +5905,7 @@
       <c r="I137" t="s">
         <v>327</v>
       </c>
-      <c r="J137" s="2">
+      <c r="J137" s="1">
         <v>46564</v>
       </c>
       <c r="K137" t="b">
@@ -5966,7 +5940,7 @@
       <c r="I138" t="s">
         <v>327</v>
       </c>
-      <c r="J138" s="2">
+      <c r="J138" s="1">
         <v>46567</v>
       </c>
       <c r="K138" t="b">
@@ -6001,7 +5975,7 @@
       <c r="I139" t="s">
         <v>327</v>
       </c>
-      <c r="J139" s="2">
+      <c r="J139" s="1">
         <v>46568</v>
       </c>
       <c r="K139" t="b">
@@ -6036,7 +6010,7 @@
       <c r="I140" t="s">
         <v>328</v>
       </c>
-      <c r="J140" s="2">
+      <c r="J140" s="1">
         <v>46578</v>
       </c>
       <c r="K140" t="b">
@@ -6071,7 +6045,7 @@
       <c r="I141" t="s">
         <v>328</v>
       </c>
-      <c r="J141" s="2">
+      <c r="J141" s="1">
         <v>46592</v>
       </c>
       <c r="K141" t="b">
@@ -6106,7 +6080,7 @@
       <c r="I142" t="s">
         <v>328</v>
       </c>
-      <c r="J142" s="2">
+      <c r="J142" s="1">
         <v>46592</v>
       </c>
       <c r="K142" t="b">
@@ -6141,7 +6115,7 @@
       <c r="I143" t="s">
         <v>329</v>
       </c>
-      <c r="J143" s="2">
+      <c r="J143" s="1">
         <v>46212</v>
       </c>
       <c r="K143" t="b">
@@ -6176,7 +6150,7 @@
       <c r="I144" t="s">
         <v>330</v>
       </c>
-      <c r="J144" s="2">
+      <c r="J144" s="1">
         <v>46225</v>
       </c>
       <c r="K144" t="b">
@@ -6211,7 +6185,7 @@
       <c r="I145" t="s">
         <v>331</v>
       </c>
-      <c r="J145" s="2">
+      <c r="J145" s="1">
         <v>46263</v>
       </c>
       <c r="K145" t="b">
@@ -6243,7 +6217,7 @@
       <c r="H146">
         <v>-1476</v>
       </c>
-      <c r="J146" s="2">
+      <c r="J146" s="1">
         <v>43773</v>
       </c>
       <c r="K146" t="b">
@@ -6275,7 +6249,7 @@
       <c r="H147">
         <v>-1469</v>
       </c>
-      <c r="J147" s="2">
+      <c r="J147" s="1">
         <v>43773</v>
       </c>
       <c r="K147" t="b">
@@ -6307,7 +6281,7 @@
       <c r="H148">
         <v>-1186</v>
       </c>
-      <c r="J148" s="2">
+      <c r="J148" s="1">
         <v>45295</v>
       </c>
       <c r="K148" t="b">
@@ -6339,7 +6313,7 @@
       <c r="H149">
         <v>-1048</v>
       </c>
-      <c r="J149" s="2">
+      <c r="J149" s="1">
         <v>45617</v>
       </c>
       <c r="K149" t="b">
@@ -6371,7 +6345,7 @@
       <c r="H150">
         <v>-980</v>
       </c>
-      <c r="J150" s="2">
+      <c r="J150" s="1">
         <v>45677</v>
       </c>
       <c r="K150" t="b">
@@ -6403,7 +6377,7 @@
       <c r="H151">
         <v>-961</v>
       </c>
-      <c r="J151" s="2">
+      <c r="J151" s="1">
         <v>44944</v>
       </c>
       <c r="K151" t="b">
@@ -6435,7 +6409,7 @@
       <c r="H152">
         <v>-252</v>
       </c>
-      <c r="J152" s="2">
+      <c r="J152" s="1">
         <v>46092</v>
       </c>
       <c r="K152" t="b">
@@ -6467,7 +6441,7 @@
       <c r="H153">
         <v>3</v>
       </c>
-      <c r="J153" s="2">
+      <c r="J153" s="1">
         <v>46265</v>
       </c>
       <c r="K153" t="b">
@@ -6499,7 +6473,7 @@
       <c r="H154">
         <v>3</v>
       </c>
-      <c r="J154" s="2">
+      <c r="J154" s="1">
         <v>46265</v>
       </c>
       <c r="K154" t="b">
@@ -6531,7 +6505,7 @@
       <c r="H155">
         <v>43</v>
       </c>
-      <c r="J155" s="2">
+      <c r="J155" s="1">
         <v>46440</v>
       </c>
       <c r="K155" t="b">
@@ -6563,7 +6537,7 @@
       <c r="H156">
         <v>43</v>
       </c>
-      <c r="J156" s="2">
+      <c r="J156" s="1">
         <v>46440</v>
       </c>
       <c r="K156" t="b">
@@ -6595,7 +6569,7 @@
       <c r="H157">
         <v>72</v>
       </c>
-      <c r="J157" s="2">
+      <c r="J157" s="1">
         <v>46289</v>
       </c>
       <c r="K157" t="b">
@@ -6627,7 +6601,7 @@
       <c r="H158">
         <v>72</v>
       </c>
-      <c r="J158" s="2">
+      <c r="J158" s="1">
         <v>46289</v>
       </c>
       <c r="K158" t="b">
@@ -6659,7 +6633,7 @@
       <c r="H159">
         <v>81</v>
       </c>
-      <c r="J159" s="2">
+      <c r="J159" s="1">
         <v>46405</v>
       </c>
       <c r="K159" t="b">
@@ -6691,7 +6665,7 @@
       <c r="H160">
         <v>102</v>
       </c>
-      <c r="J160" s="2">
+      <c r="J160" s="1">
         <v>46463</v>
       </c>
       <c r="K160" t="b">
@@ -6723,7 +6697,7 @@
       <c r="H161">
         <v>109</v>
       </c>
-      <c r="J161" s="2">
+      <c r="J161" s="1">
         <v>46353</v>
       </c>
       <c r="K161" t="b">
@@ -6755,7 +6729,7 @@
       <c r="H162">
         <v>127</v>
       </c>
-      <c r="J162" s="2">
+      <c r="J162" s="1">
         <v>46417</v>
       </c>
       <c r="K162" t="b">
@@ -6787,7 +6761,7 @@
       <c r="H163">
         <v>152</v>
       </c>
-      <c r="J163" s="2">
+      <c r="J163" s="1">
         <v>46271</v>
       </c>
       <c r="K163" t="b">
@@ -6819,7 +6793,7 @@
       <c r="H164">
         <v>152</v>
       </c>
-      <c r="J164" s="2">
+      <c r="J164" s="1">
         <v>46271</v>
       </c>
       <c r="K164" t="b">
@@ -6851,7 +6825,7 @@
       <c r="H165">
         <v>153</v>
       </c>
-      <c r="J165" s="2">
+      <c r="J165" s="1">
         <v>46458</v>
       </c>
       <c r="K165" t="b">
@@ -6883,7 +6857,7 @@
       <c r="H166">
         <v>158</v>
       </c>
-      <c r="J166" s="2">
+      <c r="J166" s="1">
         <v>46381</v>
       </c>
       <c r="K166" t="b">
@@ -6915,7 +6889,7 @@
       <c r="H167">
         <v>163</v>
       </c>
-      <c r="J167" s="2">
+      <c r="J167" s="1">
         <v>46592</v>
       </c>
       <c r="K167" t="b">
@@ -6947,7 +6921,7 @@
       <c r="H168">
         <v>167</v>
       </c>
-      <c r="J168" s="2">
+      <c r="J168" s="1">
         <v>46441</v>
       </c>
       <c r="K168" t="b">
@@ -6979,7 +6953,7 @@
       <c r="H169">
         <v>169</v>
       </c>
-      <c r="J169" s="2">
+      <c r="J169" s="1">
         <v>46391</v>
       </c>
       <c r="K169" t="b">
@@ -7011,7 +6985,7 @@
       <c r="H170">
         <v>184</v>
       </c>
-      <c r="J170" s="2">
+      <c r="J170" s="1">
         <v>46385</v>
       </c>
       <c r="K170" t="b">
@@ -7043,7 +7017,7 @@
       <c r="H171">
         <v>186</v>
       </c>
-      <c r="J171" s="2">
+      <c r="J171" s="1">
         <v>46387</v>
       </c>
       <c r="K171" t="b">
@@ -7075,7 +7049,7 @@
       <c r="H172">
         <v>206</v>
       </c>
-      <c r="J172" s="2">
+      <c r="J172" s="1">
         <v>46399</v>
       </c>
       <c r="K172" t="b">
@@ -7107,7 +7081,7 @@
       <c r="H173">
         <v>206</v>
       </c>
-      <c r="J173" s="2">
+      <c r="J173" s="1">
         <v>46399</v>
       </c>
       <c r="K173" t="b">
@@ -7139,7 +7113,7 @@
       <c r="H174">
         <v>234</v>
       </c>
-      <c r="J174" s="2">
+      <c r="J174" s="1">
         <v>46458</v>
       </c>
       <c r="K174" t="b">
@@ -7171,7 +7145,7 @@
       <c r="H175">
         <v>248</v>
       </c>
-      <c r="J175" s="2">
+      <c r="J175" s="1">
         <v>46528</v>
       </c>
       <c r="K175" t="b">
@@ -7203,7 +7177,7 @@
       <c r="H176">
         <v>317</v>
       </c>
-      <c r="J176" s="2">
+      <c r="J176" s="1">
         <v>46540</v>
       </c>
       <c r="K176" t="b">
@@ -7235,7 +7209,7 @@
       <c r="H177">
         <v>340</v>
       </c>
-      <c r="J177" s="2">
+      <c r="J177" s="1">
         <v>46547</v>
       </c>
       <c r="K177" t="b">
@@ -7267,7 +7241,7 @@
       <c r="H178">
         <v>364</v>
       </c>
-      <c r="J178" s="2">
+      <c r="J178" s="1">
         <v>46557</v>
       </c>
       <c r="K178" t="b">
@@ -7299,7 +7273,7 @@
       <c r="H179">
         <v>368</v>
       </c>
-      <c r="J179" s="2">
+      <c r="J179" s="1">
         <v>46571</v>
       </c>
       <c r="K179" t="b">
@@ -7331,7 +7305,7 @@
       <c r="H180">
         <v>368</v>
       </c>
-      <c r="J180" s="2">
+      <c r="J180" s="1">
         <v>46571</v>
       </c>
       <c r="K180" t="b">
@@ -7363,7 +7337,7 @@
       <c r="H181">
         <v>370</v>
       </c>
-      <c r="J181" s="2">
+      <c r="J181" s="1">
         <v>46562</v>
       </c>
       <c r="K181" t="b">
@@ -7395,7 +7369,7 @@
       <c r="H182">
         <v>385</v>
       </c>
-      <c r="J182" s="2">
+      <c r="J182" s="1">
         <v>46574</v>
       </c>
       <c r="K182" t="b">
@@ -7427,7 +7401,7 @@
       <c r="H183">
         <v>385</v>
       </c>
-      <c r="J183" s="2">
+      <c r="J183" s="1">
         <v>46574</v>
       </c>
       <c r="K183" t="b">
@@ -7459,7 +7433,7 @@
       <c r="H184">
         <v>417</v>
       </c>
-      <c r="J184" s="2">
+      <c r="J184" s="1">
         <v>46578</v>
       </c>
       <c r="K184" t="b">
@@ -7491,7 +7465,7 @@
       <c r="H185">
         <v>721</v>
       </c>
-      <c r="J185" s="2">
+      <c r="J185" s="1">
         <v>46345</v>
       </c>
       <c r="K185" t="b">
@@ -7523,7 +7497,7 @@
       <c r="H186">
         <v>721</v>
       </c>
-      <c r="J186" s="2">
+      <c r="J186" s="1">
         <v>46345</v>
       </c>
       <c r="K186" t="b">
@@ -7555,7 +7529,7 @@
       <c r="H187">
         <v>850</v>
       </c>
-      <c r="J187" s="2">
+      <c r="J187" s="1">
         <v>46366</v>
       </c>
       <c r="K187" t="b">
@@ -7587,7 +7561,7 @@
       <c r="H188">
         <v>850</v>
       </c>
-      <c r="J188" s="2">
+      <c r="J188" s="1">
         <v>46366</v>
       </c>
       <c r="K188" t="b">
@@ -7619,7 +7593,7 @@
       <c r="H189">
         <v>1661</v>
       </c>
-      <c r="J189" s="2">
+      <c r="J189" s="1">
         <v>46524</v>
       </c>
       <c r="K189" t="b">
@@ -7651,7 +7625,7 @@
       <c r="H190">
         <v>1661</v>
       </c>
-      <c r="J190" s="2">
+      <c r="J190" s="1">
         <v>46524</v>
       </c>
       <c r="K190" t="b">
@@ -7683,7 +7657,7 @@
       <c r="H191">
         <v>488</v>
       </c>
-      <c r="J191" s="2">
+      <c r="J191" s="1">
         <v>46190</v>
       </c>
       <c r="K191" t="b">
@@ -7715,7 +7689,7 @@
       <c r="H192">
         <v>25565</v>
       </c>
-      <c r="J192" s="2">
+      <c r="J192" s="1">
         <v>46190</v>
       </c>
       <c r="K192" t="b">
@@ -7747,7 +7721,7 @@
       <c r="H193">
         <v>25567</v>
       </c>
-      <c r="J193" s="2">
+      <c r="J193" s="1">
         <v>46190</v>
       </c>
       <c r="K193" t="b">
@@ -7779,7 +7753,7 @@
       <c r="H194">
         <v>31293</v>
       </c>
-      <c r="J194" s="2">
+      <c r="J194" s="1">
         <v>46190</v>
       </c>
       <c r="K194" t="b">

</xml_diff>